<commit_message>
Thursday work and Evidence
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB593093-D12D-493B-9717-EB009CCD2877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B1612B-5330-4317-B286-5FAC546A606B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,9 +18,9 @@
     <sheet name="Drop-downs" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$23</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$106</definedName>
-    <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$115</definedName>
+    <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$32</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <customWorkbookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="102">
   <si>
     <t>Date</t>
   </si>
@@ -384,6 +384,30 @@
   </si>
   <si>
     <t>For some reason, GitHub refuses to show PDFs on my computer, but on other devices it does work. This is meant to try and fix that. POST-TASK EDIT: Seems to be  a problem with GitHub itself and not my device, and there does nto seem to be a solution.</t>
+  </si>
+  <si>
+    <t>0,5 so far</t>
+  </si>
+  <si>
+    <t>Organize block B and block A files</t>
+  </si>
+  <si>
+    <t>What is machine learning?</t>
+  </si>
+  <si>
+    <t>Introduction and overview</t>
+  </si>
+  <si>
+    <t>Types of Machine Learning Systems</t>
+  </si>
+  <si>
+    <t>Challenges of Machine Learning</t>
+  </si>
+  <si>
+    <t>Testing, Validating, and Model Selection</t>
+  </si>
+  <si>
+    <t>Complete “ML-quiz-W1” in brightspace</t>
   </si>
 </sst>
 </file>
@@ -1383,7 +1407,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:K130"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1509,7 +1533,7 @@
         <v>0.5</v>
       </c>
       <c r="I5" s="41">
-        <f t="shared" ref="I5:I23" si="0">H5-G5</f>
+        <f t="shared" ref="I5:I32" si="0">H5-G5</f>
         <v>0</v>
       </c>
       <c r="J5" s="42"/>
@@ -2020,19 +2044,40 @@
         <v>3</v>
       </c>
       <c r="H21" s="41"/>
-      <c r="I21" s="41"/>
+      <c r="I21" s="41">
+        <f t="shared" si="0"/>
+        <v>-3</v>
+      </c>
       <c r="J21" s="45"/>
-      <c r="K21" s="44"/>
+      <c r="K21" s="44" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="22" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A22" s="37"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="41"/>
+      <c r="A22" s="37">
+        <v>45615</v>
+      </c>
+      <c r="B22" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="E22" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F22" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G22" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H22" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I22" s="41">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2041,152 +2086,195 @@
       <c r="K22" s="44"/>
     </row>
     <row r="23" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A23" s="13"/>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F23" s="15"/>
-      <c r="G23" s="18">
-        <f>SUM(G5:G22)</f>
-        <v>16.100000000000001</v>
-      </c>
-      <c r="H23" s="18">
-        <f>SUM(H5:H22)</f>
-        <v>6.75</v>
-      </c>
-      <c r="I23" s="18">
+      <c r="A23" s="37">
+        <v>45617</v>
+      </c>
+      <c r="B23" s="38"/>
+      <c r="C23" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="41">
         <f t="shared" si="0"/>
-        <v>-9.3500000000000014</v>
-      </c>
-      <c r="J23" s="19"/>
-      <c r="K23" s="46"/>
-    </row>
-    <row r="24" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="69" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" s="66"/>
-      <c r="C24" s="66"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="66"/>
-      <c r="F24" s="66"/>
-      <c r="G24" s="66"/>
-      <c r="H24" s="66"/>
-      <c r="I24" s="66"/>
-      <c r="J24" s="66"/>
-      <c r="K24" s="67"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="45"/>
+      <c r="K23" s="44"/>
+    </row>
+    <row r="24" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A24" s="37">
+        <v>45617</v>
+      </c>
+      <c r="B24" s="38"/>
+      <c r="C24" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>97</v>
+      </c>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="41">
+        <v>1</v>
+      </c>
+      <c r="H24" s="41"/>
+      <c r="I24" s="41">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="J24" s="45"/>
+      <c r="K24" s="44"/>
     </row>
     <row r="25" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A25" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="B25" s="70" t="s">
-        <v>13</v>
-      </c>
-      <c r="C25" s="54"/>
-      <c r="D25" s="54"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="54"/>
-      <c r="J25" s="54"/>
-      <c r="K25" s="55"/>
-    </row>
-    <row r="26" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B26" s="70" t="s">
-        <v>20</v>
-      </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="54"/>
-      <c r="H26" s="54"/>
-      <c r="I26" s="54"/>
-      <c r="J26" s="54"/>
-      <c r="K26" s="55"/>
+      <c r="A25" s="37">
+        <v>45617</v>
+      </c>
+      <c r="B25" s="38"/>
+      <c r="C25" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="41">
+        <v>1</v>
+      </c>
+      <c r="H25" s="41"/>
+      <c r="I25" s="41">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="J25" s="45"/>
+      <c r="K25" s="44"/>
+    </row>
+    <row r="26" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A26" s="37">
+        <v>45617</v>
+      </c>
+      <c r="B26" s="38"/>
+      <c r="C26" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="41">
+        <v>2</v>
+      </c>
+      <c r="H26" s="41"/>
+      <c r="I26" s="41">
+        <f t="shared" si="0"/>
+        <v>-2</v>
+      </c>
+      <c r="J26" s="45"/>
+      <c r="K26" s="44"/>
     </row>
     <row r="27" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A27" s="47"/>
+      <c r="A27" s="37">
+        <v>45617</v>
+      </c>
       <c r="B27" s="38"/>
       <c r="C27" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D27" s="38"/>
+      <c r="D27" s="38" t="s">
+        <v>99</v>
+      </c>
       <c r="E27" s="40"/>
       <c r="F27" s="40"/>
-      <c r="G27" s="41"/>
+      <c r="G27" s="41">
+        <v>2</v>
+      </c>
       <c r="H27" s="41"/>
       <c r="I27" s="41">
-        <f t="shared" ref="I27:I37" si="1">H27-G27</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-2</v>
       </c>
       <c r="J27" s="45"/>
-      <c r="K27" s="43"/>
+      <c r="K27" s="44"/>
     </row>
     <row r="28" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A28" s="47"/>
+      <c r="A28" s="37">
+        <v>45617</v>
+      </c>
       <c r="B28" s="38"/>
       <c r="C28" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D28" s="38"/>
+      <c r="D28" s="38" t="s">
+        <v>100</v>
+      </c>
       <c r="E28" s="40"/>
       <c r="F28" s="40"/>
-      <c r="G28" s="41"/>
+      <c r="G28" s="41">
+        <v>1</v>
+      </c>
       <c r="H28" s="41"/>
       <c r="I28" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-1</v>
       </c>
       <c r="J28" s="45"/>
-      <c r="K28" s="43"/>
+      <c r="K28" s="44"/>
     </row>
     <row r="29" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A29" s="47"/>
+      <c r="A29" s="37">
+        <v>45617</v>
+      </c>
       <c r="B29" s="38"/>
       <c r="C29" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D29" s="38"/>
+      <c r="D29" s="38" t="s">
+        <v>101</v>
+      </c>
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
-      <c r="G29" s="41"/>
+      <c r="G29" s="41">
+        <v>1</v>
+      </c>
       <c r="H29" s="41"/>
       <c r="I29" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-1</v>
       </c>
       <c r="J29" s="45"/>
-      <c r="K29" s="43"/>
+      <c r="K29" s="44"/>
     </row>
     <row r="30" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A30" s="47"/>
+      <c r="A30" s="37">
+        <v>45617</v>
+      </c>
       <c r="B30" s="38"/>
       <c r="C30" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D30" s="38"/>
+      <c r="D30" s="38" t="s">
+        <v>64</v>
+      </c>
       <c r="E30" s="40"/>
       <c r="F30" s="40"/>
       <c r="G30" s="41"/>
       <c r="H30" s="41"/>
       <c r="I30" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J30" s="45"/>
-      <c r="K30" s="43"/>
+      <c r="K30" s="44"/>
     </row>
     <row r="31" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A31" s="47"/>
+      <c r="A31" s="37"/>
       <c r="B31" s="38"/>
       <c r="C31" s="39" t="s">
         <v>17</v>
@@ -2197,83 +2285,84 @@
       <c r="G31" s="41"/>
       <c r="H31" s="41"/>
       <c r="I31" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J31" s="45"/>
-      <c r="K31" s="43"/>
+      <c r="K31" s="44"/>
     </row>
     <row r="32" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A32" s="47"/>
-      <c r="B32" s="38"/>
-      <c r="C32" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D32" s="38"/>
-      <c r="E32" s="40"/>
-      <c r="F32" s="40"/>
-      <c r="G32" s="41"/>
-      <c r="H32" s="41"/>
-      <c r="I32" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J32" s="45"/>
-      <c r="K32" s="43"/>
-    </row>
-    <row r="33" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A33" s="47"/>
-      <c r="B33" s="38"/>
-      <c r="C33" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D33" s="38"/>
-      <c r="E33" s="40"/>
-      <c r="F33" s="40"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J33" s="45"/>
-      <c r="K33" s="43"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="15"/>
+      <c r="G32" s="18">
+        <f>SUM(G5:G31)</f>
+        <v>24.6</v>
+      </c>
+      <c r="H32" s="18">
+        <f>SUM(H5:H31)</f>
+        <v>7.25</v>
+      </c>
+      <c r="I32" s="18">
+        <f t="shared" si="0"/>
+        <v>-17.350000000000001</v>
+      </c>
+      <c r="J32" s="19"/>
+      <c r="K32" s="46"/>
+    </row>
+    <row r="33" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="69" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="66"/>
+      <c r="C33" s="66"/>
+      <c r="D33" s="66"/>
+      <c r="E33" s="66"/>
+      <c r="F33" s="66"/>
+      <c r="G33" s="66"/>
+      <c r="H33" s="66"/>
+      <c r="I33" s="66"/>
+      <c r="J33" s="66"/>
+      <c r="K33" s="67"/>
     </row>
     <row r="34" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A34" s="47"/>
-      <c r="B34" s="38"/>
-      <c r="C34" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D34" s="38"/>
-      <c r="E34" s="40"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="41"/>
-      <c r="H34" s="41"/>
-      <c r="I34" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J34" s="45"/>
-      <c r="K34" s="43"/>
-    </row>
-    <row r="35" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A35" s="47"/>
-      <c r="B35" s="38"/>
-      <c r="C35" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D35" s="38"/>
-      <c r="E35" s="40"/>
-      <c r="F35" s="40"/>
-      <c r="G35" s="41"/>
-      <c r="H35" s="41"/>
-      <c r="I35" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J35" s="45"/>
-      <c r="K35" s="43"/>
+      <c r="A34" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" s="54"/>
+      <c r="D34" s="54"/>
+      <c r="E34" s="54"/>
+      <c r="F34" s="54"/>
+      <c r="G34" s="54"/>
+      <c r="H34" s="54"/>
+      <c r="I34" s="54"/>
+      <c r="J34" s="54"/>
+      <c r="K34" s="55"/>
+    </row>
+    <row r="35" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="70" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="54"/>
+      <c r="D35" s="54"/>
+      <c r="E35" s="54"/>
+      <c r="F35" s="54"/>
+      <c r="G35" s="54"/>
+      <c r="H35" s="54"/>
+      <c r="I35" s="54"/>
+      <c r="J35" s="54"/>
+      <c r="K35" s="55"/>
     </row>
     <row r="36" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A36" s="47"/>
@@ -2287,87 +2376,86 @@
       <c r="G36" s="41"/>
       <c r="H36" s="41"/>
       <c r="I36" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="I36:I46" si="1">H36-G36</f>
         <v>0</v>
       </c>
       <c r="J36" s="45"/>
       <c r="K36" s="43"/>
     </row>
     <row r="37" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A37" s="13"/>
-      <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F37" s="15"/>
-      <c r="G37" s="18">
-        <f t="shared" ref="G37:H37" si="2">SUM(G25:G36)</f>
-        <v>0</v>
-      </c>
-      <c r="H37" s="18">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I37" s="18">
+      <c r="A37" s="47"/>
+      <c r="B37" s="38"/>
+      <c r="C37" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37" s="38"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="40"/>
+      <c r="G37" s="41"/>
+      <c r="H37" s="41"/>
+      <c r="I37" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J37" s="19"/>
-      <c r="K37" s="46"/>
-    </row>
-    <row r="38" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="B38" s="54"/>
-      <c r="C38" s="54"/>
-      <c r="D38" s="54"/>
-      <c r="E38" s="54"/>
-      <c r="F38" s="54"/>
-      <c r="G38" s="54"/>
-      <c r="H38" s="54"/>
-      <c r="I38" s="54"/>
-      <c r="J38" s="54"/>
-      <c r="K38" s="55"/>
+      <c r="J37" s="45"/>
+      <c r="K37" s="43"/>
+    </row>
+    <row r="38" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A38" s="47"/>
+      <c r="B38" s="38"/>
+      <c r="C38" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" s="38"/>
+      <c r="E38" s="40"/>
+      <c r="F38" s="40"/>
+      <c r="G38" s="41"/>
+      <c r="H38" s="41"/>
+      <c r="I38" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J38" s="45"/>
+      <c r="K38" s="43"/>
     </row>
     <row r="39" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A39" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B39" s="72" t="s">
-        <v>13</v>
-      </c>
-      <c r="C39" s="54"/>
-      <c r="D39" s="54"/>
-      <c r="E39" s="54"/>
-      <c r="F39" s="54"/>
-      <c r="G39" s="54"/>
-      <c r="H39" s="54"/>
-      <c r="I39" s="54"/>
-      <c r="J39" s="54"/>
-      <c r="K39" s="55"/>
-    </row>
-    <row r="40" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B40" s="72" t="s">
-        <v>15</v>
-      </c>
-      <c r="C40" s="54"/>
-      <c r="D40" s="54"/>
-      <c r="E40" s="54"/>
-      <c r="F40" s="54"/>
-      <c r="G40" s="54"/>
-      <c r="H40" s="54"/>
-      <c r="I40" s="54"/>
-      <c r="J40" s="54"/>
-      <c r="K40" s="55"/>
+      <c r="A39" s="47"/>
+      <c r="B39" s="38"/>
+      <c r="C39" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="38"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="41"/>
+      <c r="I39" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J39" s="45"/>
+      <c r="K39" s="43"/>
+    </row>
+    <row r="40" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A40" s="47"/>
+      <c r="B40" s="38"/>
+      <c r="C40" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="38"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="41"/>
+      <c r="H40" s="41"/>
+      <c r="I40" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J40" s="45"/>
+      <c r="K40" s="43"/>
     </row>
     <row r="41" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A41" s="37"/>
+      <c r="A41" s="47"/>
       <c r="B41" s="38"/>
       <c r="C41" s="39" t="s">
         <v>17</v>
@@ -2378,14 +2466,14 @@
       <c r="G41" s="41"/>
       <c r="H41" s="41"/>
       <c r="I41" s="41">
-        <f t="shared" ref="I41:I51" si="3">H41-G41</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J41" s="45"/>
       <c r="K41" s="43"/>
     </row>
     <row r="42" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A42" s="37"/>
+      <c r="A42" s="47"/>
       <c r="B42" s="38"/>
       <c r="C42" s="39" t="s">
         <v>17</v>
@@ -2396,14 +2484,14 @@
       <c r="G42" s="41"/>
       <c r="H42" s="41"/>
       <c r="I42" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J42" s="45"/>
       <c r="K42" s="43"/>
     </row>
     <row r="43" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A43" s="37"/>
+      <c r="A43" s="47"/>
       <c r="B43" s="38"/>
       <c r="C43" s="39" t="s">
         <v>17</v>
@@ -2414,14 +2502,14 @@
       <c r="G43" s="41"/>
       <c r="H43" s="41"/>
       <c r="I43" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J43" s="45"/>
       <c r="K43" s="43"/>
     </row>
     <row r="44" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A44" s="37"/>
+      <c r="A44" s="47"/>
       <c r="B44" s="38"/>
       <c r="C44" s="39" t="s">
         <v>17</v>
@@ -2432,14 +2520,14 @@
       <c r="G44" s="41"/>
       <c r="H44" s="41"/>
       <c r="I44" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J44" s="45"/>
       <c r="K44" s="43"/>
     </row>
     <row r="45" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A45" s="37"/>
+      <c r="A45" s="47"/>
       <c r="B45" s="38"/>
       <c r="C45" s="39" t="s">
         <v>17</v>
@@ -2450,83 +2538,84 @@
       <c r="G45" s="41"/>
       <c r="H45" s="41"/>
       <c r="I45" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J45" s="45"/>
       <c r="K45" s="43"/>
     </row>
     <row r="46" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A46" s="37"/>
-      <c r="B46" s="38"/>
-      <c r="C46" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D46" s="38"/>
-      <c r="E46" s="40"/>
-      <c r="F46" s="40"/>
-      <c r="G46" s="41"/>
-      <c r="H46" s="41"/>
-      <c r="I46" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J46" s="45"/>
-      <c r="K46" s="43"/>
-    </row>
-    <row r="47" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A47" s="37"/>
-      <c r="B47" s="38"/>
-      <c r="C47" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D47" s="38"/>
-      <c r="E47" s="40"/>
-      <c r="F47" s="40"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="41"/>
-      <c r="I47" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J47" s="45"/>
-      <c r="K47" s="43"/>
+      <c r="A46" s="13"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F46" s="15"/>
+      <c r="G46" s="18">
+        <f t="shared" ref="G46:H46" si="2">SUM(G34:G45)</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I46" s="18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J46" s="19"/>
+      <c r="K46" s="46"/>
+    </row>
+    <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="71" t="s">
+        <v>21</v>
+      </c>
+      <c r="B47" s="54"/>
+      <c r="C47" s="54"/>
+      <c r="D47" s="54"/>
+      <c r="E47" s="54"/>
+      <c r="F47" s="54"/>
+      <c r="G47" s="54"/>
+      <c r="H47" s="54"/>
+      <c r="I47" s="54"/>
+      <c r="J47" s="54"/>
+      <c r="K47" s="55"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A48" s="37"/>
-      <c r="B48" s="38"/>
-      <c r="C48" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D48" s="38"/>
-      <c r="E48" s="40"/>
-      <c r="F48" s="40"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="41"/>
-      <c r="I48" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J48" s="45"/>
-      <c r="K48" s="43"/>
-    </row>
-    <row r="49" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A49" s="37"/>
-      <c r="B49" s="38"/>
-      <c r="C49" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D49" s="38"/>
-      <c r="E49" s="40"/>
-      <c r="F49" s="40"/>
-      <c r="G49" s="41"/>
-      <c r="H49" s="41"/>
-      <c r="I49" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J49" s="45"/>
-      <c r="K49" s="43"/>
+      <c r="A48" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="C48" s="54"/>
+      <c r="D48" s="54"/>
+      <c r="E48" s="54"/>
+      <c r="F48" s="54"/>
+      <c r="G48" s="54"/>
+      <c r="H48" s="54"/>
+      <c r="I48" s="54"/>
+      <c r="J48" s="54"/>
+      <c r="K48" s="55"/>
+    </row>
+    <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B49" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="C49" s="54"/>
+      <c r="D49" s="54"/>
+      <c r="E49" s="54"/>
+      <c r="F49" s="54"/>
+      <c r="G49" s="54"/>
+      <c r="H49" s="54"/>
+      <c r="I49" s="54"/>
+      <c r="J49" s="54"/>
+      <c r="K49" s="55"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="37"/>
@@ -2540,84 +2629,83 @@
       <c r="G50" s="41"/>
       <c r="H50" s="41"/>
       <c r="I50" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="I50:I60" si="3">H50-G50</f>
         <v>0</v>
       </c>
       <c r="J50" s="45"/>
       <c r="K50" s="43"/>
     </row>
     <row r="51" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A51" s="13"/>
-      <c r="B51" s="15"/>
-      <c r="C51" s="15"/>
-      <c r="D51" s="15"/>
-      <c r="E51" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F51" s="15"/>
-      <c r="G51" s="18">
-        <f t="shared" ref="G51:H51" si="4">SUM(G41:G50)</f>
-        <v>0</v>
-      </c>
-      <c r="H51" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I51" s="18">
+      <c r="A51" s="37"/>
+      <c r="B51" s="38"/>
+      <c r="C51" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D51" s="38"/>
+      <c r="E51" s="40"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="41"/>
+      <c r="H51" s="41"/>
+      <c r="I51" s="41">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J51" s="19"/>
-      <c r="K51" s="46"/>
-    </row>
-    <row r="52" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="73" t="s">
-        <v>22</v>
-      </c>
-      <c r="B52" s="54"/>
-      <c r="C52" s="54"/>
-      <c r="D52" s="54"/>
-      <c r="E52" s="54"/>
-      <c r="F52" s="54"/>
-      <c r="G52" s="54"/>
-      <c r="H52" s="54"/>
-      <c r="I52" s="54"/>
-      <c r="J52" s="54"/>
-      <c r="K52" s="55"/>
+      <c r="J51" s="45"/>
+      <c r="K51" s="43"/>
+    </row>
+    <row r="52" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A52" s="37"/>
+      <c r="B52" s="38"/>
+      <c r="C52" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D52" s="38"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="40"/>
+      <c r="G52" s="41"/>
+      <c r="H52" s="41"/>
+      <c r="I52" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J52" s="45"/>
+      <c r="K52" s="43"/>
     </row>
     <row r="53" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A53" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B53" s="57" t="s">
-        <v>13</v>
-      </c>
-      <c r="C53" s="54"/>
-      <c r="D53" s="54"/>
-      <c r="E53" s="54"/>
-      <c r="F53" s="54"/>
-      <c r="G53" s="54"/>
-      <c r="H53" s="54"/>
-      <c r="I53" s="54"/>
-      <c r="J53" s="54"/>
-      <c r="K53" s="55"/>
-    </row>
-    <row r="54" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B54" s="57" t="s">
-        <v>15</v>
-      </c>
-      <c r="C54" s="54"/>
-      <c r="D54" s="54"/>
-      <c r="E54" s="54"/>
-      <c r="F54" s="54"/>
-      <c r="G54" s="54"/>
-      <c r="H54" s="54"/>
-      <c r="I54" s="54"/>
-      <c r="J54" s="54"/>
-      <c r="K54" s="55"/>
+      <c r="A53" s="37"/>
+      <c r="B53" s="38"/>
+      <c r="C53" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D53" s="38"/>
+      <c r="E53" s="40"/>
+      <c r="F53" s="40"/>
+      <c r="G53" s="41"/>
+      <c r="H53" s="41"/>
+      <c r="I53" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J53" s="45"/>
+      <c r="K53" s="43"/>
+    </row>
+    <row r="54" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A54" s="37"/>
+      <c r="B54" s="38"/>
+      <c r="C54" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D54" s="38"/>
+      <c r="E54" s="40"/>
+      <c r="F54" s="40"/>
+      <c r="G54" s="41"/>
+      <c r="H54" s="41"/>
+      <c r="I54" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J54" s="45"/>
+      <c r="K54" s="43"/>
     </row>
     <row r="55" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A55" s="37"/>
@@ -2631,7 +2719,7 @@
       <c r="G55" s="41"/>
       <c r="H55" s="41"/>
       <c r="I55" s="41">
-        <f t="shared" ref="I55:I65" si="5">H55-G55</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J55" s="45"/>
@@ -2649,7 +2737,7 @@
       <c r="G56" s="41"/>
       <c r="H56" s="41"/>
       <c r="I56" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J56" s="45"/>
@@ -2667,7 +2755,7 @@
       <c r="G57" s="41"/>
       <c r="H57" s="41"/>
       <c r="I57" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J57" s="45"/>
@@ -2685,7 +2773,7 @@
       <c r="G58" s="41"/>
       <c r="H58" s="41"/>
       <c r="I58" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J58" s="45"/>
@@ -2703,83 +2791,84 @@
       <c r="G59" s="41"/>
       <c r="H59" s="41"/>
       <c r="I59" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J59" s="45"/>
       <c r="K59" s="43"/>
     </row>
     <row r="60" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A60" s="37"/>
-      <c r="B60" s="38"/>
-      <c r="C60" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D60" s="38"/>
-      <c r="E60" s="40"/>
-      <c r="F60" s="40"/>
-      <c r="G60" s="41"/>
-      <c r="H60" s="41"/>
-      <c r="I60" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J60" s="45"/>
-      <c r="K60" s="43"/>
-    </row>
-    <row r="61" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A61" s="37"/>
-      <c r="B61" s="38"/>
-      <c r="C61" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D61" s="38"/>
-      <c r="E61" s="40"/>
-      <c r="F61" s="40"/>
-      <c r="G61" s="41"/>
-      <c r="H61" s="41"/>
-      <c r="I61" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J61" s="45"/>
-      <c r="K61" s="43"/>
+      <c r="A60" s="13"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F60" s="15"/>
+      <c r="G60" s="18">
+        <f t="shared" ref="G60:H60" si="4">SUM(G50:G59)</f>
+        <v>0</v>
+      </c>
+      <c r="H60" s="18">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I60" s="18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J60" s="19"/>
+      <c r="K60" s="46"/>
+    </row>
+    <row r="61" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="73" t="s">
+        <v>22</v>
+      </c>
+      <c r="B61" s="54"/>
+      <c r="C61" s="54"/>
+      <c r="D61" s="54"/>
+      <c r="E61" s="54"/>
+      <c r="F61" s="54"/>
+      <c r="G61" s="54"/>
+      <c r="H61" s="54"/>
+      <c r="I61" s="54"/>
+      <c r="J61" s="54"/>
+      <c r="K61" s="55"/>
     </row>
     <row r="62" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A62" s="37"/>
-      <c r="B62" s="38"/>
-      <c r="C62" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D62" s="38"/>
-      <c r="E62" s="40"/>
-      <c r="F62" s="40"/>
-      <c r="G62" s="41"/>
-      <c r="H62" s="41"/>
-      <c r="I62" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J62" s="45"/>
-      <c r="K62" s="43"/>
-    </row>
-    <row r="63" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A63" s="37"/>
-      <c r="B63" s="38"/>
-      <c r="C63" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D63" s="38"/>
-      <c r="E63" s="40"/>
-      <c r="F63" s="40"/>
-      <c r="G63" s="41"/>
-      <c r="H63" s="41"/>
-      <c r="I63" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J63" s="45"/>
-      <c r="K63" s="43"/>
+      <c r="A62" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B62" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" s="54"/>
+      <c r="D62" s="54"/>
+      <c r="E62" s="54"/>
+      <c r="F62" s="54"/>
+      <c r="G62" s="54"/>
+      <c r="H62" s="54"/>
+      <c r="I62" s="54"/>
+      <c r="J62" s="54"/>
+      <c r="K62" s="55"/>
+    </row>
+    <row r="63" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B63" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C63" s="54"/>
+      <c r="D63" s="54"/>
+      <c r="E63" s="54"/>
+      <c r="F63" s="54"/>
+      <c r="G63" s="54"/>
+      <c r="H63" s="54"/>
+      <c r="I63" s="54"/>
+      <c r="J63" s="54"/>
+      <c r="K63" s="55"/>
     </row>
     <row r="64" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A64" s="37"/>
@@ -2793,84 +2882,83 @@
       <c r="G64" s="41"/>
       <c r="H64" s="41"/>
       <c r="I64" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I64:I74" si="5">H64-G64</f>
         <v>0</v>
       </c>
       <c r="J64" s="45"/>
       <c r="K64" s="43"/>
     </row>
     <row r="65" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A65" s="13"/>
-      <c r="B65" s="15"/>
-      <c r="C65" s="15"/>
-      <c r="D65" s="15"/>
-      <c r="E65" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F65" s="15"/>
-      <c r="G65" s="18">
-        <f t="shared" ref="G65:H65" si="6">SUM(G55:G64)</f>
-        <v>0</v>
-      </c>
-      <c r="H65" s="18">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="I65" s="18">
+      <c r="A65" s="37"/>
+      <c r="B65" s="38"/>
+      <c r="C65" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D65" s="38"/>
+      <c r="E65" s="40"/>
+      <c r="F65" s="40"/>
+      <c r="G65" s="41"/>
+      <c r="H65" s="41"/>
+      <c r="I65" s="41">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J65" s="19"/>
-      <c r="K65" s="46"/>
-    </row>
-    <row r="66" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="58" t="s">
-        <v>23</v>
-      </c>
-      <c r="B66" s="54"/>
-      <c r="C66" s="54"/>
-      <c r="D66" s="54"/>
-      <c r="E66" s="54"/>
-      <c r="F66" s="54"/>
-      <c r="G66" s="54"/>
-      <c r="H66" s="54"/>
-      <c r="I66" s="54"/>
-      <c r="J66" s="54"/>
-      <c r="K66" s="55"/>
+      <c r="J65" s="45"/>
+      <c r="K65" s="43"/>
+    </row>
+    <row r="66" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A66" s="37"/>
+      <c r="B66" s="38"/>
+      <c r="C66" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D66" s="38"/>
+      <c r="E66" s="40"/>
+      <c r="F66" s="40"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="41"/>
+      <c r="I66" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J66" s="45"/>
+      <c r="K66" s="43"/>
     </row>
     <row r="67" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A67" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B67" s="59" t="s">
-        <v>13</v>
-      </c>
-      <c r="C67" s="54"/>
-      <c r="D67" s="54"/>
-      <c r="E67" s="54"/>
-      <c r="F67" s="54"/>
-      <c r="G67" s="54"/>
-      <c r="H67" s="54"/>
-      <c r="I67" s="54"/>
-      <c r="J67" s="54"/>
-      <c r="K67" s="55"/>
-    </row>
-    <row r="68" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="B68" s="59" t="s">
-        <v>15</v>
-      </c>
-      <c r="C68" s="54"/>
-      <c r="D68" s="54"/>
-      <c r="E68" s="54"/>
-      <c r="F68" s="54"/>
-      <c r="G68" s="54"/>
-      <c r="H68" s="54"/>
-      <c r="I68" s="54"/>
-      <c r="J68" s="54"/>
-      <c r="K68" s="55"/>
+      <c r="A67" s="37"/>
+      <c r="B67" s="38"/>
+      <c r="C67" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D67" s="38"/>
+      <c r="E67" s="40"/>
+      <c r="F67" s="40"/>
+      <c r="G67" s="41"/>
+      <c r="H67" s="41"/>
+      <c r="I67" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J67" s="45"/>
+      <c r="K67" s="43"/>
+    </row>
+    <row r="68" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A68" s="37"/>
+      <c r="B68" s="38"/>
+      <c r="C68" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D68" s="38"/>
+      <c r="E68" s="40"/>
+      <c r="F68" s="40"/>
+      <c r="G68" s="41"/>
+      <c r="H68" s="41"/>
+      <c r="I68" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J68" s="45"/>
+      <c r="K68" s="43"/>
     </row>
     <row r="69" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A69" s="37"/>
@@ -2884,7 +2972,7 @@
       <c r="G69" s="41"/>
       <c r="H69" s="41"/>
       <c r="I69" s="41">
-        <f t="shared" ref="I69:I79" si="7">H69-G69</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J69" s="45"/>
@@ -2902,7 +2990,7 @@
       <c r="G70" s="41"/>
       <c r="H70" s="41"/>
       <c r="I70" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J70" s="45"/>
@@ -2920,7 +3008,7 @@
       <c r="G71" s="41"/>
       <c r="H71" s="41"/>
       <c r="I71" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J71" s="45"/>
@@ -2938,7 +3026,7 @@
       <c r="G72" s="41"/>
       <c r="H72" s="41"/>
       <c r="I72" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J72" s="45"/>
@@ -2956,83 +3044,84 @@
       <c r="G73" s="41"/>
       <c r="H73" s="41"/>
       <c r="I73" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J73" s="45"/>
       <c r="K73" s="43"/>
     </row>
     <row r="74" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A74" s="37"/>
-      <c r="B74" s="38"/>
-      <c r="C74" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D74" s="38"/>
-      <c r="E74" s="40"/>
-      <c r="F74" s="40"/>
-      <c r="G74" s="41"/>
-      <c r="H74" s="41"/>
-      <c r="I74" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J74" s="45"/>
-      <c r="K74" s="43"/>
-    </row>
-    <row r="75" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A75" s="37"/>
-      <c r="B75" s="38"/>
-      <c r="C75" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D75" s="38"/>
-      <c r="E75" s="40"/>
-      <c r="F75" s="40"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="41"/>
-      <c r="I75" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J75" s="45"/>
-      <c r="K75" s="43"/>
+      <c r="A74" s="13"/>
+      <c r="B74" s="15"/>
+      <c r="C74" s="15"/>
+      <c r="D74" s="15"/>
+      <c r="E74" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F74" s="15"/>
+      <c r="G74" s="18">
+        <f t="shared" ref="G74:H74" si="6">SUM(G64:G73)</f>
+        <v>0</v>
+      </c>
+      <c r="H74" s="18">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I74" s="18">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J74" s="19"/>
+      <c r="K74" s="46"/>
+    </row>
+    <row r="75" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="B75" s="54"/>
+      <c r="C75" s="54"/>
+      <c r="D75" s="54"/>
+      <c r="E75" s="54"/>
+      <c r="F75" s="54"/>
+      <c r="G75" s="54"/>
+      <c r="H75" s="54"/>
+      <c r="I75" s="54"/>
+      <c r="J75" s="54"/>
+      <c r="K75" s="55"/>
     </row>
     <row r="76" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A76" s="37"/>
-      <c r="B76" s="38"/>
-      <c r="C76" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D76" s="38"/>
-      <c r="E76" s="40"/>
-      <c r="F76" s="40"/>
-      <c r="G76" s="41"/>
-      <c r="H76" s="41"/>
-      <c r="I76" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J76" s="45"/>
-      <c r="K76" s="43"/>
-    </row>
-    <row r="77" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A77" s="37"/>
-      <c r="B77" s="38"/>
-      <c r="C77" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D77" s="38"/>
-      <c r="E77" s="40"/>
-      <c r="F77" s="40"/>
-      <c r="G77" s="41"/>
-      <c r="H77" s="41"/>
-      <c r="I77" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J77" s="45"/>
-      <c r="K77" s="43"/>
+      <c r="A76" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B76" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C76" s="54"/>
+      <c r="D76" s="54"/>
+      <c r="E76" s="54"/>
+      <c r="F76" s="54"/>
+      <c r="G76" s="54"/>
+      <c r="H76" s="54"/>
+      <c r="I76" s="54"/>
+      <c r="J76" s="54"/>
+      <c r="K76" s="55"/>
+    </row>
+    <row r="77" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B77" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C77" s="54"/>
+      <c r="D77" s="54"/>
+      <c r="E77" s="54"/>
+      <c r="F77" s="54"/>
+      <c r="G77" s="54"/>
+      <c r="H77" s="54"/>
+      <c r="I77" s="54"/>
+      <c r="J77" s="54"/>
+      <c r="K77" s="55"/>
     </row>
     <row r="78" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A78" s="37"/>
@@ -3046,84 +3135,83 @@
       <c r="G78" s="41"/>
       <c r="H78" s="41"/>
       <c r="I78" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="I78:I88" si="7">H78-G78</f>
         <v>0</v>
       </c>
       <c r="J78" s="45"/>
       <c r="K78" s="43"/>
     </row>
     <row r="79" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A79" s="13"/>
-      <c r="B79" s="15"/>
-      <c r="C79" s="15"/>
-      <c r="D79" s="15"/>
-      <c r="E79" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F79" s="15"/>
-      <c r="G79" s="18">
-        <f t="shared" ref="G79:H79" si="8">SUM(G69:G78)</f>
-        <v>0</v>
-      </c>
-      <c r="H79" s="18">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I79" s="18">
+      <c r="A79" s="37"/>
+      <c r="B79" s="38"/>
+      <c r="C79" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D79" s="38"/>
+      <c r="E79" s="40"/>
+      <c r="F79" s="40"/>
+      <c r="G79" s="41"/>
+      <c r="H79" s="41"/>
+      <c r="I79" s="41">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J79" s="19"/>
-      <c r="K79" s="46"/>
-    </row>
-    <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="B80" s="54"/>
-      <c r="C80" s="54"/>
-      <c r="D80" s="54"/>
-      <c r="E80" s="54"/>
-      <c r="F80" s="54"/>
-      <c r="G80" s="54"/>
-      <c r="H80" s="54"/>
-      <c r="I80" s="54"/>
-      <c r="J80" s="54"/>
-      <c r="K80" s="55"/>
+      <c r="J79" s="45"/>
+      <c r="K79" s="43"/>
+    </row>
+    <row r="80" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A80" s="37"/>
+      <c r="B80" s="38"/>
+      <c r="C80" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D80" s="38"/>
+      <c r="E80" s="40"/>
+      <c r="F80" s="40"/>
+      <c r="G80" s="41"/>
+      <c r="H80" s="41"/>
+      <c r="I80" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J80" s="45"/>
+      <c r="K80" s="43"/>
     </row>
     <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A81" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B81" s="53" t="s">
-        <v>13</v>
-      </c>
-      <c r="C81" s="54"/>
-      <c r="D81" s="54"/>
-      <c r="E81" s="54"/>
-      <c r="F81" s="54"/>
-      <c r="G81" s="54"/>
-      <c r="H81" s="54"/>
-      <c r="I81" s="54"/>
-      <c r="J81" s="54"/>
-      <c r="K81" s="55"/>
-    </row>
-    <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B82" s="53" t="s">
-        <v>15</v>
-      </c>
-      <c r="C82" s="54"/>
-      <c r="D82" s="54"/>
-      <c r="E82" s="54"/>
-      <c r="F82" s="54"/>
-      <c r="G82" s="54"/>
-      <c r="H82" s="54"/>
-      <c r="I82" s="54"/>
-      <c r="J82" s="54"/>
-      <c r="K82" s="55"/>
+      <c r="A81" s="37"/>
+      <c r="B81" s="38"/>
+      <c r="C81" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D81" s="38"/>
+      <c r="E81" s="40"/>
+      <c r="F81" s="40"/>
+      <c r="G81" s="41"/>
+      <c r="H81" s="41"/>
+      <c r="I81" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J81" s="45"/>
+      <c r="K81" s="43"/>
+    </row>
+    <row r="82" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A82" s="37"/>
+      <c r="B82" s="38"/>
+      <c r="C82" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D82" s="38"/>
+      <c r="E82" s="40"/>
+      <c r="F82" s="40"/>
+      <c r="G82" s="41"/>
+      <c r="H82" s="41"/>
+      <c r="I82" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J82" s="45"/>
+      <c r="K82" s="43"/>
     </row>
     <row r="83" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A83" s="37"/>
@@ -3137,7 +3225,7 @@
       <c r="G83" s="41"/>
       <c r="H83" s="41"/>
       <c r="I83" s="41">
-        <f t="shared" ref="I83:I93" si="9">H83-G83</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J83" s="45"/>
@@ -3155,7 +3243,7 @@
       <c r="G84" s="41"/>
       <c r="H84" s="41"/>
       <c r="I84" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J84" s="45"/>
@@ -3173,13 +3261,11 @@
       <c r="G85" s="41"/>
       <c r="H85" s="41"/>
       <c r="I85" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J85" s="45"/>
-      <c r="K85" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K85" s="43"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="37"/>
@@ -3193,7 +3279,7 @@
       <c r="G86" s="41"/>
       <c r="H86" s="41"/>
       <c r="I86" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J86" s="45"/>
@@ -3211,83 +3297,84 @@
       <c r="G87" s="41"/>
       <c r="H87" s="41"/>
       <c r="I87" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J87" s="45"/>
       <c r="K87" s="43"/>
     </row>
     <row r="88" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A88" s="37"/>
-      <c r="B88" s="38"/>
-      <c r="C88" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D88" s="38"/>
-      <c r="E88" s="40"/>
-      <c r="F88" s="40"/>
-      <c r="G88" s="41"/>
-      <c r="H88" s="41"/>
-      <c r="I88" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J88" s="45"/>
-      <c r="K88" s="43"/>
-    </row>
-    <row r="89" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A89" s="37"/>
-      <c r="B89" s="38"/>
-      <c r="C89" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D89" s="38"/>
-      <c r="E89" s="40"/>
-      <c r="F89" s="40"/>
-      <c r="G89" s="41"/>
-      <c r="H89" s="41"/>
-      <c r="I89" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J89" s="45"/>
-      <c r="K89" s="43"/>
+      <c r="A88" s="13"/>
+      <c r="B88" s="15"/>
+      <c r="C88" s="15"/>
+      <c r="D88" s="15"/>
+      <c r="E88" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F88" s="15"/>
+      <c r="G88" s="18">
+        <f t="shared" ref="G88:H88" si="8">SUM(G78:G87)</f>
+        <v>0</v>
+      </c>
+      <c r="H88" s="18">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I88" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J88" s="19"/>
+      <c r="K88" s="46"/>
+    </row>
+    <row r="89" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="B89" s="54"/>
+      <c r="C89" s="54"/>
+      <c r="D89" s="54"/>
+      <c r="E89" s="54"/>
+      <c r="F89" s="54"/>
+      <c r="G89" s="54"/>
+      <c r="H89" s="54"/>
+      <c r="I89" s="54"/>
+      <c r="J89" s="54"/>
+      <c r="K89" s="55"/>
     </row>
     <row r="90" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A90" s="37"/>
-      <c r="B90" s="38"/>
-      <c r="C90" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D90" s="38"/>
-      <c r="E90" s="40"/>
-      <c r="F90" s="40"/>
-      <c r="G90" s="41"/>
-      <c r="H90" s="41"/>
-      <c r="I90" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J90" s="45"/>
-      <c r="K90" s="43"/>
-    </row>
-    <row r="91" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A91" s="37"/>
-      <c r="B91" s="38"/>
-      <c r="C91" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D91" s="38"/>
-      <c r="E91" s="40"/>
-      <c r="F91" s="40"/>
-      <c r="G91" s="41"/>
-      <c r="H91" s="41"/>
-      <c r="I91" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J91" s="45"/>
-      <c r="K91" s="43"/>
+      <c r="A90" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B90" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="C90" s="54"/>
+      <c r="D90" s="54"/>
+      <c r="E90" s="54"/>
+      <c r="F90" s="54"/>
+      <c r="G90" s="54"/>
+      <c r="H90" s="54"/>
+      <c r="I90" s="54"/>
+      <c r="J90" s="54"/>
+      <c r="K90" s="55"/>
+    </row>
+    <row r="91" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B91" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="C91" s="54"/>
+      <c r="D91" s="54"/>
+      <c r="E91" s="54"/>
+      <c r="F91" s="54"/>
+      <c r="G91" s="54"/>
+      <c r="H91" s="54"/>
+      <c r="I91" s="54"/>
+      <c r="J91" s="54"/>
+      <c r="K91" s="55"/>
     </row>
     <row r="92" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A92" s="37"/>
@@ -3301,84 +3388,85 @@
       <c r="G92" s="41"/>
       <c r="H92" s="41"/>
       <c r="I92" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I92:I102" si="9">H92-G92</f>
         <v>0</v>
       </c>
       <c r="J92" s="45"/>
       <c r="K92" s="43"/>
     </row>
     <row r="93" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A93" s="13"/>
-      <c r="B93" s="15"/>
-      <c r="C93" s="15"/>
-      <c r="D93" s="15"/>
-      <c r="E93" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F93" s="15"/>
-      <c r="G93" s="18">
-        <f t="shared" ref="G93:H93" si="10">SUM(G83:G92)</f>
-        <v>0</v>
-      </c>
-      <c r="H93" s="18">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="I93" s="18">
+      <c r="A93" s="37"/>
+      <c r="B93" s="38"/>
+      <c r="C93" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D93" s="38"/>
+      <c r="E93" s="40"/>
+      <c r="F93" s="40"/>
+      <c r="G93" s="41"/>
+      <c r="H93" s="41"/>
+      <c r="I93" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J93" s="19"/>
-      <c r="K93" s="46"/>
-    </row>
-    <row r="94" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="56" t="s">
-        <v>26</v>
-      </c>
-      <c r="B94" s="54"/>
-      <c r="C94" s="54"/>
-      <c r="D94" s="54"/>
-      <c r="E94" s="54"/>
-      <c r="F94" s="54"/>
-      <c r="G94" s="54"/>
-      <c r="H94" s="54"/>
-      <c r="I94" s="54"/>
-      <c r="J94" s="54"/>
-      <c r="K94" s="55"/>
+      <c r="J93" s="45"/>
+      <c r="K93" s="43"/>
+    </row>
+    <row r="94" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A94" s="37"/>
+      <c r="B94" s="38"/>
+      <c r="C94" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D94" s="38"/>
+      <c r="E94" s="40"/>
+      <c r="F94" s="40"/>
+      <c r="G94" s="41"/>
+      <c r="H94" s="41"/>
+      <c r="I94" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J94" s="45"/>
+      <c r="K94" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A95" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B95" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="C95" s="54"/>
-      <c r="D95" s="54"/>
-      <c r="E95" s="54"/>
-      <c r="F95" s="54"/>
-      <c r="G95" s="54"/>
-      <c r="H95" s="54"/>
-      <c r="I95" s="54"/>
-      <c r="J95" s="54"/>
-      <c r="K95" s="55"/>
-    </row>
-    <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B96" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="C96" s="54"/>
-      <c r="D96" s="54"/>
-      <c r="E96" s="54"/>
-      <c r="F96" s="54"/>
-      <c r="G96" s="54"/>
-      <c r="H96" s="54"/>
-      <c r="I96" s="54"/>
-      <c r="J96" s="54"/>
-      <c r="K96" s="55"/>
+      <c r="A95" s="37"/>
+      <c r="B95" s="38"/>
+      <c r="C95" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D95" s="38"/>
+      <c r="E95" s="40"/>
+      <c r="F95" s="40"/>
+      <c r="G95" s="41"/>
+      <c r="H95" s="41"/>
+      <c r="I95" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J95" s="45"/>
+      <c r="K95" s="43"/>
+    </row>
+    <row r="96" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A96" s="37"/>
+      <c r="B96" s="38"/>
+      <c r="C96" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D96" s="38"/>
+      <c r="E96" s="40"/>
+      <c r="F96" s="40"/>
+      <c r="G96" s="41"/>
+      <c r="H96" s="41"/>
+      <c r="I96" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J96" s="45"/>
+      <c r="K96" s="43"/>
     </row>
     <row r="97" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A97" s="37"/>
@@ -3392,7 +3480,7 @@
       <c r="G97" s="41"/>
       <c r="H97" s="41"/>
       <c r="I97" s="41">
-        <f t="shared" ref="I97:I107" si="11">H97-G97</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J97" s="45"/>
@@ -3410,7 +3498,7 @@
       <c r="G98" s="41"/>
       <c r="H98" s="41"/>
       <c r="I98" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J98" s="45"/>
@@ -3428,7 +3516,7 @@
       <c r="G99" s="41"/>
       <c r="H99" s="41"/>
       <c r="I99" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J99" s="45"/>
@@ -3446,7 +3534,7 @@
       <c r="G100" s="41"/>
       <c r="H100" s="41"/>
       <c r="I100" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J100" s="45"/>
@@ -3464,83 +3552,84 @@
       <c r="G101" s="41"/>
       <c r="H101" s="41"/>
       <c r="I101" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J101" s="45"/>
       <c r="K101" s="43"/>
     </row>
     <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A102" s="37"/>
-      <c r="B102" s="38"/>
-      <c r="C102" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D102" s="38"/>
-      <c r="E102" s="40"/>
-      <c r="F102" s="40"/>
-      <c r="G102" s="41"/>
-      <c r="H102" s="41"/>
-      <c r="I102" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J102" s="45"/>
-      <c r="K102" s="43"/>
-    </row>
-    <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A103" s="37"/>
-      <c r="B103" s="38"/>
-      <c r="C103" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D103" s="38"/>
-      <c r="E103" s="40"/>
-      <c r="F103" s="40"/>
-      <c r="G103" s="41"/>
-      <c r="H103" s="41"/>
-      <c r="I103" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J103" s="45"/>
-      <c r="K103" s="43"/>
+      <c r="A102" s="13"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="15"/>
+      <c r="D102" s="15"/>
+      <c r="E102" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F102" s="15"/>
+      <c r="G102" s="18">
+        <f t="shared" ref="G102:H102" si="10">SUM(G92:G101)</f>
+        <v>0</v>
+      </c>
+      <c r="H102" s="18">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="I102" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J102" s="19"/>
+      <c r="K102" s="46"/>
+    </row>
+    <row r="103" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="B103" s="54"/>
+      <c r="C103" s="54"/>
+      <c r="D103" s="54"/>
+      <c r="E103" s="54"/>
+      <c r="F103" s="54"/>
+      <c r="G103" s="54"/>
+      <c r="H103" s="54"/>
+      <c r="I103" s="54"/>
+      <c r="J103" s="54"/>
+      <c r="K103" s="55"/>
     </row>
     <row r="104" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A104" s="37"/>
-      <c r="B104" s="38"/>
-      <c r="C104" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D104" s="38"/>
-      <c r="E104" s="40"/>
-      <c r="F104" s="40"/>
-      <c r="G104" s="41"/>
-      <c r="H104" s="41"/>
-      <c r="I104" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J104" s="45"/>
-      <c r="K104" s="43"/>
-    </row>
-    <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A105" s="37"/>
-      <c r="B105" s="38"/>
-      <c r="C105" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D105" s="38"/>
-      <c r="E105" s="40"/>
-      <c r="F105" s="40"/>
-      <c r="G105" s="41"/>
-      <c r="H105" s="41"/>
-      <c r="I105" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J105" s="45"/>
-      <c r="K105" s="43"/>
+      <c r="A104" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B104" s="74" t="s">
+        <v>13</v>
+      </c>
+      <c r="C104" s="54"/>
+      <c r="D104" s="54"/>
+      <c r="E104" s="54"/>
+      <c r="F104" s="54"/>
+      <c r="G104" s="54"/>
+      <c r="H104" s="54"/>
+      <c r="I104" s="54"/>
+      <c r="J104" s="54"/>
+      <c r="K104" s="55"/>
+    </row>
+    <row r="105" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B105" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="C105" s="54"/>
+      <c r="D105" s="54"/>
+      <c r="E105" s="54"/>
+      <c r="F105" s="54"/>
+      <c r="G105" s="54"/>
+      <c r="H105" s="54"/>
+      <c r="I105" s="54"/>
+      <c r="J105" s="54"/>
+      <c r="K105" s="55"/>
     </row>
     <row r="106" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A106" s="37"/>
@@ -3554,84 +3643,83 @@
       <c r="G106" s="41"/>
       <c r="H106" s="41"/>
       <c r="I106" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="I106:I116" si="11">H106-G106</f>
         <v>0</v>
       </c>
       <c r="J106" s="45"/>
       <c r="K106" s="43"/>
     </row>
     <row r="107" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A107" s="13"/>
-      <c r="B107" s="15"/>
-      <c r="C107" s="15"/>
-      <c r="D107" s="15"/>
-      <c r="E107" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F107" s="15"/>
-      <c r="G107" s="18">
-        <f t="shared" ref="G107:H107" si="12">SUM(G97:G106)</f>
-        <v>0</v>
-      </c>
-      <c r="H107" s="18">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="I107" s="18">
+      <c r="A107" s="37"/>
+      <c r="B107" s="38"/>
+      <c r="C107" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D107" s="38"/>
+      <c r="E107" s="40"/>
+      <c r="F107" s="40"/>
+      <c r="G107" s="41"/>
+      <c r="H107" s="41"/>
+      <c r="I107" s="41">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J107" s="19"/>
-      <c r="K107" s="46"/>
-    </row>
-    <row r="108" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="B108" s="62"/>
-      <c r="C108" s="62"/>
-      <c r="D108" s="62"/>
-      <c r="E108" s="62"/>
-      <c r="F108" s="62"/>
-      <c r="G108" s="62"/>
-      <c r="H108" s="62"/>
-      <c r="I108" s="62"/>
-      <c r="J108" s="62"/>
-      <c r="K108" s="63"/>
+      <c r="J107" s="45"/>
+      <c r="K107" s="43"/>
+    </row>
+    <row r="108" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A108" s="37"/>
+      <c r="B108" s="38"/>
+      <c r="C108" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D108" s="38"/>
+      <c r="E108" s="40"/>
+      <c r="F108" s="40"/>
+      <c r="G108" s="41"/>
+      <c r="H108" s="41"/>
+      <c r="I108" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J108" s="45"/>
+      <c r="K108" s="43"/>
     </row>
     <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A109" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B109" s="64" t="s">
-        <v>13</v>
-      </c>
-      <c r="C109" s="62"/>
-      <c r="D109" s="62"/>
-      <c r="E109" s="62"/>
-      <c r="F109" s="62"/>
-      <c r="G109" s="62"/>
-      <c r="H109" s="62"/>
-      <c r="I109" s="62"/>
-      <c r="J109" s="62"/>
-      <c r="K109" s="63"/>
-    </row>
-    <row r="110" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B110" s="64" t="s">
-        <v>15</v>
-      </c>
-      <c r="C110" s="62"/>
-      <c r="D110" s="62"/>
-      <c r="E110" s="62"/>
-      <c r="F110" s="62"/>
-      <c r="G110" s="62"/>
-      <c r="H110" s="62"/>
-      <c r="I110" s="62"/>
-      <c r="J110" s="62"/>
-      <c r="K110" s="63"/>
+      <c r="A109" s="37"/>
+      <c r="B109" s="38"/>
+      <c r="C109" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D109" s="38"/>
+      <c r="E109" s="40"/>
+      <c r="F109" s="40"/>
+      <c r="G109" s="41"/>
+      <c r="H109" s="41"/>
+      <c r="I109" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J109" s="45"/>
+      <c r="K109" s="43"/>
+    </row>
+    <row r="110" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A110" s="37"/>
+      <c r="B110" s="38"/>
+      <c r="C110" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D110" s="38"/>
+      <c r="E110" s="40"/>
+      <c r="F110" s="40"/>
+      <c r="G110" s="41"/>
+      <c r="H110" s="41"/>
+      <c r="I110" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J110" s="45"/>
+      <c r="K110" s="43"/>
     </row>
     <row r="111" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A111" s="37"/>
@@ -3645,7 +3733,7 @@
       <c r="G111" s="41"/>
       <c r="H111" s="41"/>
       <c r="I111" s="41">
-        <f t="shared" ref="I111:I121" si="13">H111-G111</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J111" s="45"/>
@@ -3663,7 +3751,7 @@
       <c r="G112" s="41"/>
       <c r="H112" s="41"/>
       <c r="I112" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J112" s="45"/>
@@ -3681,7 +3769,7 @@
       <c r="G113" s="41"/>
       <c r="H113" s="41"/>
       <c r="I113" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J113" s="45"/>
@@ -3699,7 +3787,7 @@
       <c r="G114" s="41"/>
       <c r="H114" s="41"/>
       <c r="I114" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J114" s="45"/>
@@ -3717,83 +3805,84 @@
       <c r="G115" s="41"/>
       <c r="H115" s="41"/>
       <c r="I115" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J115" s="45"/>
       <c r="K115" s="43"/>
     </row>
     <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A116" s="37"/>
-      <c r="B116" s="38"/>
-      <c r="C116" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D116" s="38"/>
-      <c r="E116" s="40"/>
-      <c r="F116" s="40"/>
-      <c r="G116" s="41"/>
-      <c r="H116" s="41"/>
-      <c r="I116" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J116" s="45"/>
-      <c r="K116" s="43"/>
-    </row>
-    <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A117" s="37"/>
-      <c r="B117" s="38"/>
-      <c r="C117" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D117" s="38"/>
-      <c r="E117" s="40"/>
-      <c r="F117" s="40"/>
-      <c r="G117" s="41"/>
-      <c r="H117" s="41"/>
-      <c r="I117" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J117" s="45"/>
-      <c r="K117" s="43"/>
+      <c r="A116" s="13"/>
+      <c r="B116" s="15"/>
+      <c r="C116" s="15"/>
+      <c r="D116" s="15"/>
+      <c r="E116" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F116" s="15"/>
+      <c r="G116" s="18">
+        <f t="shared" ref="G116:H116" si="12">SUM(G106:G115)</f>
+        <v>0</v>
+      </c>
+      <c r="H116" s="18">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="I116" s="18">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J116" s="19"/>
+      <c r="K116" s="46"/>
+    </row>
+    <row r="117" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="61" t="s">
+        <v>27</v>
+      </c>
+      <c r="B117" s="62"/>
+      <c r="C117" s="62"/>
+      <c r="D117" s="62"/>
+      <c r="E117" s="62"/>
+      <c r="F117" s="62"/>
+      <c r="G117" s="62"/>
+      <c r="H117" s="62"/>
+      <c r="I117" s="62"/>
+      <c r="J117" s="62"/>
+      <c r="K117" s="63"/>
     </row>
     <row r="118" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A118" s="37"/>
-      <c r="B118" s="38"/>
-      <c r="C118" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D118" s="38"/>
-      <c r="E118" s="40"/>
-      <c r="F118" s="40"/>
-      <c r="G118" s="41"/>
-      <c r="H118" s="41"/>
-      <c r="I118" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J118" s="45"/>
-      <c r="K118" s="43"/>
-    </row>
-    <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A119" s="37"/>
-      <c r="B119" s="38"/>
-      <c r="C119" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D119" s="38"/>
-      <c r="E119" s="40"/>
-      <c r="F119" s="40"/>
-      <c r="G119" s="41"/>
-      <c r="H119" s="41"/>
-      <c r="I119" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J119" s="45"/>
-      <c r="K119" s="43"/>
+      <c r="A118" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B118" s="64" t="s">
+        <v>13</v>
+      </c>
+      <c r="C118" s="62"/>
+      <c r="D118" s="62"/>
+      <c r="E118" s="62"/>
+      <c r="F118" s="62"/>
+      <c r="G118" s="62"/>
+      <c r="H118" s="62"/>
+      <c r="I118" s="62"/>
+      <c r="J118" s="62"/>
+      <c r="K118" s="63"/>
+    </row>
+    <row r="119" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B119" s="64" t="s">
+        <v>15</v>
+      </c>
+      <c r="C119" s="62"/>
+      <c r="D119" s="62"/>
+      <c r="E119" s="62"/>
+      <c r="F119" s="62"/>
+      <c r="G119" s="62"/>
+      <c r="H119" s="62"/>
+      <c r="I119" s="62"/>
+      <c r="J119" s="62"/>
+      <c r="K119" s="63"/>
     </row>
     <row r="120" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A120" s="37"/>
@@ -3807,42 +3896,204 @@
       <c r="G120" s="41"/>
       <c r="H120" s="41"/>
       <c r="I120" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="I120:I130" si="13">H120-G120</f>
         <v>0</v>
       </c>
       <c r="J120" s="45"/>
       <c r="K120" s="43"/>
     </row>
     <row r="121" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A121" s="48"/>
-      <c r="B121" s="49"/>
-      <c r="C121" s="49"/>
-      <c r="D121" s="49"/>
-      <c r="E121" s="49" t="s">
+      <c r="A121" s="37"/>
+      <c r="B121" s="38"/>
+      <c r="C121" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D121" s="38"/>
+      <c r="E121" s="40"/>
+      <c r="F121" s="40"/>
+      <c r="G121" s="41"/>
+      <c r="H121" s="41"/>
+      <c r="I121" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J121" s="45"/>
+      <c r="K121" s="43"/>
+    </row>
+    <row r="122" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A122" s="37"/>
+      <c r="B122" s="38"/>
+      <c r="C122" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D122" s="38"/>
+      <c r="E122" s="40"/>
+      <c r="F122" s="40"/>
+      <c r="G122" s="41"/>
+      <c r="H122" s="41"/>
+      <c r="I122" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J122" s="45"/>
+      <c r="K122" s="43"/>
+    </row>
+    <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A123" s="37"/>
+      <c r="B123" s="38"/>
+      <c r="C123" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D123" s="38"/>
+      <c r="E123" s="40"/>
+      <c r="F123" s="40"/>
+      <c r="G123" s="41"/>
+      <c r="H123" s="41"/>
+      <c r="I123" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J123" s="45"/>
+      <c r="K123" s="43"/>
+    </row>
+    <row r="124" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A124" s="37"/>
+      <c r="B124" s="38"/>
+      <c r="C124" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D124" s="38"/>
+      <c r="E124" s="40"/>
+      <c r="F124" s="40"/>
+      <c r="G124" s="41"/>
+      <c r="H124" s="41"/>
+      <c r="I124" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J124" s="45"/>
+      <c r="K124" s="43"/>
+    </row>
+    <row r="125" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A125" s="37"/>
+      <c r="B125" s="38"/>
+      <c r="C125" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D125" s="38"/>
+      <c r="E125" s="40"/>
+      <c r="F125" s="40"/>
+      <c r="G125" s="41"/>
+      <c r="H125" s="41"/>
+      <c r="I125" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J125" s="45"/>
+      <c r="K125" s="43"/>
+    </row>
+    <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A126" s="37"/>
+      <c r="B126" s="38"/>
+      <c r="C126" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D126" s="38"/>
+      <c r="E126" s="40"/>
+      <c r="F126" s="40"/>
+      <c r="G126" s="41"/>
+      <c r="H126" s="41"/>
+      <c r="I126" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J126" s="45"/>
+      <c r="K126" s="43"/>
+    </row>
+    <row r="127" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A127" s="37"/>
+      <c r="B127" s="38"/>
+      <c r="C127" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D127" s="38"/>
+      <c r="E127" s="40"/>
+      <c r="F127" s="40"/>
+      <c r="G127" s="41"/>
+      <c r="H127" s="41"/>
+      <c r="I127" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J127" s="45"/>
+      <c r="K127" s="43"/>
+    </row>
+    <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A128" s="37"/>
+      <c r="B128" s="38"/>
+      <c r="C128" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D128" s="38"/>
+      <c r="E128" s="40"/>
+      <c r="F128" s="40"/>
+      <c r="G128" s="41"/>
+      <c r="H128" s="41"/>
+      <c r="I128" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J128" s="45"/>
+      <c r="K128" s="43"/>
+    </row>
+    <row r="129" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A129" s="37"/>
+      <c r="B129" s="38"/>
+      <c r="C129" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D129" s="38"/>
+      <c r="E129" s="40"/>
+      <c r="F129" s="40"/>
+      <c r="G129" s="41"/>
+      <c r="H129" s="41"/>
+      <c r="I129" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J129" s="45"/>
+      <c r="K129" s="43"/>
+    </row>
+    <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A130" s="48"/>
+      <c r="B130" s="49"/>
+      <c r="C130" s="49"/>
+      <c r="D130" s="49"/>
+      <c r="E130" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F121" s="49"/>
-      <c r="G121" s="50">
-        <f t="shared" ref="G121:H121" si="14">SUM(G111:G120)</f>
-        <v>0</v>
-      </c>
-      <c r="H121" s="50">
+      <c r="F130" s="49"/>
+      <c r="G130" s="50">
+        <f t="shared" ref="G130:H130" si="14">SUM(G120:G129)</f>
+        <v>0</v>
+      </c>
+      <c r="H130" s="50">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="I121" s="50">
+      <c r="I130" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J121" s="51"/>
-      <c r="K121" s="52"/>
+      <c r="J130" s="51"/>
+      <c r="K130" s="52"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K23" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{738C683C-EE2C-4CC2-9CA7-9A74D11B2546}">
+      <autoFilter ref="A1:K15" xr:uid="{37F66CFF-D3CB-4C05-B44C-28A7219A2FB3}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -3853,32 +4104,32 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A108:K108"/>
-    <mergeCell ref="B109:K109"/>
-    <mergeCell ref="B110:K110"/>
+    <mergeCell ref="A117:K117"/>
+    <mergeCell ref="B118:K118"/>
+    <mergeCell ref="B119:K119"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
-    <mergeCell ref="A24:K24"/>
-    <mergeCell ref="B25:K25"/>
-    <mergeCell ref="B26:K26"/>
-    <mergeCell ref="A38:K38"/>
-    <mergeCell ref="B39:K39"/>
-    <mergeCell ref="B40:K40"/>
-    <mergeCell ref="A52:K52"/>
-    <mergeCell ref="B95:K95"/>
-    <mergeCell ref="B96:K96"/>
-    <mergeCell ref="B53:K53"/>
-    <mergeCell ref="B81:K81"/>
-    <mergeCell ref="B82:K82"/>
-    <mergeCell ref="A94:K94"/>
-    <mergeCell ref="B54:K54"/>
-    <mergeCell ref="A66:K66"/>
-    <mergeCell ref="B67:K67"/>
-    <mergeCell ref="B68:K68"/>
-    <mergeCell ref="A80:K80"/>
+    <mergeCell ref="A33:K33"/>
+    <mergeCell ref="B34:K34"/>
+    <mergeCell ref="B35:K35"/>
+    <mergeCell ref="A47:K47"/>
+    <mergeCell ref="B48:K48"/>
+    <mergeCell ref="B49:K49"/>
+    <mergeCell ref="A61:K61"/>
+    <mergeCell ref="B104:K104"/>
+    <mergeCell ref="B105:K105"/>
+    <mergeCell ref="B62:K62"/>
+    <mergeCell ref="B90:K90"/>
+    <mergeCell ref="B91:K91"/>
+    <mergeCell ref="A103:K103"/>
+    <mergeCell ref="B63:K63"/>
+    <mergeCell ref="A75:K75"/>
+    <mergeCell ref="B76:K76"/>
+    <mergeCell ref="B77:K77"/>
+    <mergeCell ref="A89:K89"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B22 B25:B36 B41:B50 B55:B64 B69:B78 B83:B92 B97:B106">
+  <conditionalFormatting sqref="B5:B31 B34:B45 B50:B59 B64:B73 B78:B87 B92:B101 B106:B115">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -3895,7 +4146,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B23 B25:B37 B39:B51 B53:B65 B67:B79 B81:B93 B95:B107 B109:B121">
+  <conditionalFormatting sqref="B5:B32 B34:B46 B48:B60 B62:B74 B76:B88 B90:B102 B104:B116 B118:B130">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -3903,34 +4154,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B111:B120">
+  <conditionalFormatting sqref="B120:B129">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B111))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B120))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B111))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B120))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B111))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B120))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B111))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B120))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B111))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B120))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G23 G27:G37 G41:G51 G55:G65 G69:G79 G83:G93 G97:G107 G111:G121">
+  <conditionalFormatting sqref="G1 G3:G32 G36:G46 G50:G60 G64:G74 G78:G88 G92:G102 G106:G116 G120:G130">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H121">
+  <conditionalFormatting sqref="H1:H130">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I23 I27:I37 I41:I51 I55:I65 I69:I79 I83:I93 I97:I107 I111:I121">
+  <conditionalFormatting sqref="I36:I46 I50:I60 I64:I74 I78:I88 I92:I102 I106:I116 I120:I130 I5:I32">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -3939,7 +4190,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F111:F120 F97:F106 F27:F36 F41:F50 F55:F64 F69:F78 F83:F92 F5:F22" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F120:F129 F106:F115 F36:F45 F50:F59 F64:F73 F78:F87 F92:F101 F5:F31" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3952,13 +4203,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E22 E27:E36 E41:E50 E55:E64 E69:E78 E83:E92 E97:E106 E111:E120</xm:sqref>
+          <xm:sqref>E5:E31 E36:E45 E50:E59 E64:E73 E78:E87 E92:E101 E106:E115 E120:E129</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B22 B27:B36 B41:B50 B55:B64 B69:B78 B83:B92 B97:B106 B111:B120</xm:sqref>
+          <xm:sqref>B5:B31 B36:B45 B50:B59 B64:B73 B78:B87 B92:B101 B106:B115 B120:B129</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4038,7 +4289,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" cm="1">
-        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$27:$H$36,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
+        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$36:$H$45,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" cm="1">

</xml_diff>

<commit_message>
W1 D2 Work I (WorkLog)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B1612B-5330-4317-B286-5FAC546A606B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6D9703-2FEE-47C9-905B-19589D935185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,9 +18,9 @@
     <sheet name="Drop-downs" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$32</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$115</definedName>
-    <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$121</definedName>
+    <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$38</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <customWorkbookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="110">
   <si>
     <t>Date</t>
   </si>
@@ -408,6 +408,30 @@
   </si>
   <si>
     <t>Complete “ML-quiz-W1” in brightspace</t>
+  </si>
+  <si>
+    <t>Learn about SQL</t>
+  </si>
+  <si>
+    <t>Install SQL</t>
+  </si>
+  <si>
+    <t>Stand Up Meeting</t>
+  </si>
+  <si>
+    <t>Plan in WorkLog</t>
+  </si>
+  <si>
+    <t>Learn about basic SQL queries</t>
+  </si>
+  <si>
+    <t>Fill in Learning Log week 1</t>
+  </si>
+  <si>
+    <t>EDA with SQL</t>
+  </si>
+  <si>
+    <t>ILO 8.1</t>
   </si>
 </sst>
 </file>
@@ -883,26 +907,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -919,6 +923,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -936,6 +942,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1407,7 +1431,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K130"/>
+  <dimension ref="A1:K136"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1459,53 +1483,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="67"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="59"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="55"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="68" t="s">
+      <c r="B4" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="55"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="61"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="62"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -1533,7 +1557,7 @@
         <v>0.5</v>
       </c>
       <c r="I5" s="41">
-        <f t="shared" ref="I5:I32" si="0">H5-G5</f>
+        <f t="shared" ref="I5:I38" si="0">H5-G5</f>
         <v>0</v>
       </c>
       <c r="J5" s="42"/>
@@ -2089,17 +2113,27 @@
       <c r="A23" s="37">
         <v>45617</v>
       </c>
-      <c r="B23" s="38"/>
+      <c r="B23" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C23" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="38" t="s">
         <v>80</v>
       </c>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="41"/>
+      <c r="E23" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F23" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H23" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I23" s="41">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2111,22 +2145,30 @@
       <c r="A24" s="37">
         <v>45617</v>
       </c>
-      <c r="B24" s="38"/>
+      <c r="B24" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C24" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D24" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="E24" s="40"/>
-      <c r="F24" s="40"/>
+      <c r="E24" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" s="40" t="s">
+        <v>109</v>
+      </c>
       <c r="G24" s="41">
         <v>1</v>
       </c>
-      <c r="H24" s="41"/>
+      <c r="H24" s="41">
+        <v>1</v>
+      </c>
       <c r="I24" s="41">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="45"/>
       <c r="K24" s="44"/>
@@ -2135,22 +2177,30 @@
       <c r="A25" s="37">
         <v>45617</v>
       </c>
-      <c r="B25" s="38"/>
+      <c r="B25" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C25" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D25" s="38" t="s">
         <v>96</v>
       </c>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
+      <c r="E25" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25" s="40" t="s">
+        <v>109</v>
+      </c>
       <c r="G25" s="41">
         <v>1</v>
       </c>
-      <c r="H25" s="41"/>
+      <c r="H25" s="41">
+        <v>1</v>
+      </c>
       <c r="I25" s="41">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J25" s="45"/>
       <c r="K25" s="44"/>
@@ -2159,22 +2209,30 @@
       <c r="A26" s="37">
         <v>45617</v>
       </c>
-      <c r="B26" s="38"/>
+      <c r="B26" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C26" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D26" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="E26" s="40"/>
-      <c r="F26" s="40"/>
+      <c r="E26" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F26" s="40" t="s">
+        <v>109</v>
+      </c>
       <c r="G26" s="41">
         <v>2</v>
       </c>
-      <c r="H26" s="41"/>
+      <c r="H26" s="41">
+        <v>2</v>
+      </c>
       <c r="I26" s="41">
         <f t="shared" si="0"/>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="J26" s="45"/>
       <c r="K26" s="44"/>
@@ -2183,22 +2241,30 @@
       <c r="A27" s="37">
         <v>45617</v>
       </c>
-      <c r="B27" s="38"/>
+      <c r="B27" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C27" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D27" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
+      <c r="E27" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F27" s="40" t="s">
+        <v>109</v>
+      </c>
       <c r="G27" s="41">
         <v>2</v>
       </c>
-      <c r="H27" s="41"/>
+      <c r="H27" s="41">
+        <v>2</v>
+      </c>
       <c r="I27" s="41">
         <f t="shared" si="0"/>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="J27" s="45"/>
       <c r="K27" s="44"/>
@@ -2207,22 +2273,30 @@
       <c r="A28" s="37">
         <v>45617</v>
       </c>
-      <c r="B28" s="38"/>
+      <c r="B28" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C28" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
+      <c r="E28" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F28" s="40" t="s">
+        <v>109</v>
+      </c>
       <c r="G28" s="41">
         <v>1</v>
       </c>
-      <c r="H28" s="41"/>
+      <c r="H28" s="41">
+        <v>1</v>
+      </c>
       <c r="I28" s="41">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J28" s="45"/>
       <c r="K28" s="44"/>
@@ -2231,22 +2305,30 @@
       <c r="A29" s="37">
         <v>45617</v>
       </c>
-      <c r="B29" s="38"/>
+      <c r="B29" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C29" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D29" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
+      <c r="E29" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F29" s="40" t="s">
+        <v>109</v>
+      </c>
       <c r="G29" s="41">
         <v>1</v>
       </c>
-      <c r="H29" s="41"/>
+      <c r="H29" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I29" s="41">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="J29" s="45"/>
       <c r="K29" s="44"/>
@@ -2255,20 +2337,28 @@
       <c r="A30" s="37">
         <v>45617</v>
       </c>
-      <c r="B30" s="38"/>
+      <c r="B30" s="38" t="s">
+        <v>52</v>
+      </c>
       <c r="C30" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D30" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E30" s="40"/>
-      <c r="F30" s="40"/>
-      <c r="G30" s="41"/>
+      <c r="E30" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F30" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G30" s="41">
+        <v>0.5</v>
+      </c>
       <c r="H30" s="41"/>
       <c r="I30" s="41">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="J30" s="45"/>
       <c r="K30" s="44"/>
@@ -2276,14 +2366,22 @@
     <row r="31" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A31" s="37"/>
       <c r="B31" s="38"/>
-      <c r="C31" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D31" s="38"/>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40"/>
-      <c r="G31" s="41"/>
-      <c r="H31" s="41"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="E31" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F31" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G31" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H31" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I31" s="41">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2292,185 +2390,206 @@
       <c r="K31" s="44"/>
     </row>
     <row r="32" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A32" s="13"/>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F32" s="15"/>
-      <c r="G32" s="18">
-        <f>SUM(G5:G31)</f>
-        <v>24.6</v>
-      </c>
-      <c r="H32" s="18">
-        <f>SUM(H5:H31)</f>
-        <v>7.25</v>
-      </c>
-      <c r="I32" s="18">
-        <f t="shared" si="0"/>
-        <v>-17.350000000000001</v>
-      </c>
-      <c r="J32" s="19"/>
-      <c r="K32" s="46"/>
-    </row>
-    <row r="33" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="69" t="s">
-        <v>19</v>
-      </c>
-      <c r="B33" s="66"/>
-      <c r="C33" s="66"/>
-      <c r="D33" s="66"/>
-      <c r="E33" s="66"/>
-      <c r="F33" s="66"/>
-      <c r="G33" s="66"/>
-      <c r="H33" s="66"/>
-      <c r="I33" s="66"/>
-      <c r="J33" s="66"/>
-      <c r="K33" s="67"/>
+      <c r="A32" s="37"/>
+      <c r="B32" s="38"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="E32" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F32" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G32" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H32" s="41"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="45"/>
+      <c r="K32" s="44"/>
+    </row>
+    <row r="33" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A33" s="37"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="E33" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F33" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G33" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="45"/>
+      <c r="K33" s="44"/>
     </row>
     <row r="34" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A34" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="B34" s="70" t="s">
-        <v>13</v>
-      </c>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="54"/>
-      <c r="H34" s="54"/>
-      <c r="I34" s="54"/>
-      <c r="J34" s="54"/>
-      <c r="K34" s="55"/>
-    </row>
-    <row r="35" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B35" s="70" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="54"/>
-      <c r="D35" s="54"/>
-      <c r="E35" s="54"/>
-      <c r="F35" s="54"/>
-      <c r="G35" s="54"/>
-      <c r="H35" s="54"/>
-      <c r="I35" s="54"/>
-      <c r="J35" s="54"/>
-      <c r="K35" s="55"/>
+      <c r="A34" s="37"/>
+      <c r="B34" s="38"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="E34" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F34" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G34" s="41">
+        <v>2</v>
+      </c>
+      <c r="H34" s="41"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="45"/>
+      <c r="K34" s="44"/>
+    </row>
+    <row r="35" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A35" s="37"/>
+      <c r="B35" s="38"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="E35" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F35" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G35" s="41">
+        <v>2</v>
+      </c>
+      <c r="H35" s="41"/>
+      <c r="I35" s="41"/>
+      <c r="J35" s="45"/>
+      <c r="K35" s="44"/>
     </row>
     <row r="36" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A36" s="47"/>
+      <c r="A36" s="37"/>
       <c r="B36" s="38"/>
-      <c r="C36" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" s="38"/>
-      <c r="E36" s="40"/>
-      <c r="F36" s="40"/>
-      <c r="G36" s="41"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="E36" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F36" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G36" s="41">
+        <v>4</v>
+      </c>
       <c r="H36" s="41"/>
-      <c r="I36" s="41">
-        <f t="shared" ref="I36:I46" si="1">H36-G36</f>
-        <v>0</v>
-      </c>
+      <c r="I36" s="41"/>
       <c r="J36" s="45"/>
-      <c r="K36" s="43"/>
+      <c r="K36" s="44"/>
     </row>
     <row r="37" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A37" s="47"/>
+      <c r="A37" s="37"/>
       <c r="B37" s="38"/>
       <c r="C37" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D37" s="38"/>
+      <c r="D37" s="38" t="s">
+        <v>107</v>
+      </c>
       <c r="E37" s="40"/>
-      <c r="F37" s="40"/>
-      <c r="G37" s="41"/>
+      <c r="F37" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G37" s="41">
+        <v>0.5</v>
+      </c>
       <c r="H37" s="41"/>
       <c r="I37" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
       </c>
       <c r="J37" s="45"/>
-      <c r="K37" s="43"/>
+      <c r="K37" s="44"/>
     </row>
     <row r="38" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A38" s="47"/>
-      <c r="B38" s="38"/>
-      <c r="C38" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D38" s="38"/>
-      <c r="E38" s="40"/>
-      <c r="F38" s="40"/>
-      <c r="G38" s="41"/>
-      <c r="H38" s="41"/>
-      <c r="I38" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J38" s="45"/>
-      <c r="K38" s="43"/>
-    </row>
-    <row r="39" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A39" s="47"/>
-      <c r="B39" s="38"/>
-      <c r="C39" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D39" s="38"/>
-      <c r="E39" s="40"/>
-      <c r="F39" s="40"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="41"/>
-      <c r="I39" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J39" s="45"/>
-      <c r="K39" s="43"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="15"/>
+      <c r="G38" s="18">
+        <f>SUM(G5:G37)</f>
+        <v>34.85</v>
+      </c>
+      <c r="H38" s="18">
+        <f>SUM(H5:H37)</f>
+        <v>15.25</v>
+      </c>
+      <c r="I38" s="18">
+        <f t="shared" si="0"/>
+        <v>-19.600000000000001</v>
+      </c>
+      <c r="J38" s="19"/>
+      <c r="K38" s="46"/>
+    </row>
+    <row r="39" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="63" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39" s="58"/>
+      <c r="C39" s="58"/>
+      <c r="D39" s="58"/>
+      <c r="E39" s="58"/>
+      <c r="F39" s="58"/>
+      <c r="G39" s="58"/>
+      <c r="H39" s="58"/>
+      <c r="I39" s="58"/>
+      <c r="J39" s="58"/>
+      <c r="K39" s="59"/>
     </row>
     <row r="40" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A40" s="47"/>
-      <c r="B40" s="38"/>
-      <c r="C40" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D40" s="38"/>
-      <c r="E40" s="40"/>
-      <c r="F40" s="40"/>
-      <c r="G40" s="41"/>
-      <c r="H40" s="41"/>
-      <c r="I40" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J40" s="45"/>
-      <c r="K40" s="43"/>
-    </row>
-    <row r="41" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A41" s="47"/>
-      <c r="B41" s="38"/>
-      <c r="C41" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D41" s="38"/>
-      <c r="E41" s="40"/>
-      <c r="F41" s="40"/>
-      <c r="G41" s="41"/>
-      <c r="H41" s="41"/>
-      <c r="I41" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J41" s="45"/>
-      <c r="K41" s="43"/>
+      <c r="A40" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" s="64" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="61"/>
+      <c r="D40" s="61"/>
+      <c r="E40" s="61"/>
+      <c r="F40" s="61"/>
+      <c r="G40" s="61"/>
+      <c r="H40" s="61"/>
+      <c r="I40" s="61"/>
+      <c r="J40" s="61"/>
+      <c r="K40" s="62"/>
+    </row>
+    <row r="41" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B41" s="64" t="s">
+        <v>20</v>
+      </c>
+      <c r="C41" s="61"/>
+      <c r="D41" s="61"/>
+      <c r="E41" s="61"/>
+      <c r="F41" s="61"/>
+      <c r="G41" s="61"/>
+      <c r="H41" s="61"/>
+      <c r="I41" s="61"/>
+      <c r="J41" s="61"/>
+      <c r="K41" s="62"/>
     </row>
     <row r="42" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A42" s="47"/>
@@ -2484,7 +2603,7 @@
       <c r="G42" s="41"/>
       <c r="H42" s="41"/>
       <c r="I42" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="I42:I52" si="1">H42-G42</f>
         <v>0</v>
       </c>
       <c r="J42" s="45"/>
@@ -2545,80 +2664,79 @@
       <c r="K45" s="43"/>
     </row>
     <row r="46" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A46" s="13"/>
-      <c r="B46" s="15"/>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F46" s="15"/>
-      <c r="G46" s="18">
-        <f t="shared" ref="G46:H46" si="2">SUM(G34:G45)</f>
-        <v>0</v>
-      </c>
-      <c r="H46" s="18">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I46" s="18">
+      <c r="A46" s="47"/>
+      <c r="B46" s="38"/>
+      <c r="C46" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" s="38"/>
+      <c r="E46" s="40"/>
+      <c r="F46" s="40"/>
+      <c r="G46" s="41"/>
+      <c r="H46" s="41"/>
+      <c r="I46" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J46" s="19"/>
-      <c r="K46" s="46"/>
-    </row>
-    <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="B47" s="54"/>
-      <c r="C47" s="54"/>
-      <c r="D47" s="54"/>
-      <c r="E47" s="54"/>
-      <c r="F47" s="54"/>
-      <c r="G47" s="54"/>
-      <c r="H47" s="54"/>
-      <c r="I47" s="54"/>
-      <c r="J47" s="54"/>
-      <c r="K47" s="55"/>
+      <c r="J46" s="45"/>
+      <c r="K46" s="43"/>
+    </row>
+    <row r="47" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A47" s="47"/>
+      <c r="B47" s="38"/>
+      <c r="C47" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="38"/>
+      <c r="E47" s="40"/>
+      <c r="F47" s="40"/>
+      <c r="G47" s="41"/>
+      <c r="H47" s="41"/>
+      <c r="I47" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J47" s="45"/>
+      <c r="K47" s="43"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A48" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B48" s="72" t="s">
-        <v>13</v>
-      </c>
-      <c r="C48" s="54"/>
-      <c r="D48" s="54"/>
-      <c r="E48" s="54"/>
-      <c r="F48" s="54"/>
-      <c r="G48" s="54"/>
-      <c r="H48" s="54"/>
-      <c r="I48" s="54"/>
-      <c r="J48" s="54"/>
-      <c r="K48" s="55"/>
-    </row>
-    <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B49" s="72" t="s">
-        <v>15</v>
-      </c>
-      <c r="C49" s="54"/>
-      <c r="D49" s="54"/>
-      <c r="E49" s="54"/>
-      <c r="F49" s="54"/>
-      <c r="G49" s="54"/>
-      <c r="H49" s="54"/>
-      <c r="I49" s="54"/>
-      <c r="J49" s="54"/>
-      <c r="K49" s="55"/>
+      <c r="A48" s="47"/>
+      <c r="B48" s="38"/>
+      <c r="C48" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" s="38"/>
+      <c r="E48" s="40"/>
+      <c r="F48" s="40"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="41"/>
+      <c r="I48" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J48" s="45"/>
+      <c r="K48" s="43"/>
+    </row>
+    <row r="49" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A49" s="47"/>
+      <c r="B49" s="38"/>
+      <c r="C49" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D49" s="38"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
+      <c r="G49" s="41"/>
+      <c r="H49" s="41"/>
+      <c r="I49" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J49" s="45"/>
+      <c r="K49" s="43"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A50" s="37"/>
+      <c r="A50" s="47"/>
       <c r="B50" s="38"/>
       <c r="C50" s="39" t="s">
         <v>17</v>
@@ -2629,14 +2747,14 @@
       <c r="G50" s="41"/>
       <c r="H50" s="41"/>
       <c r="I50" s="41">
-        <f t="shared" ref="I50:I60" si="3">H50-G50</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J50" s="45"/>
       <c r="K50" s="43"/>
     </row>
     <row r="51" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A51" s="37"/>
+      <c r="A51" s="47"/>
       <c r="B51" s="38"/>
       <c r="C51" s="39" t="s">
         <v>17</v>
@@ -2647,83 +2765,84 @@
       <c r="G51" s="41"/>
       <c r="H51" s="41"/>
       <c r="I51" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J51" s="45"/>
       <c r="K51" s="43"/>
     </row>
     <row r="52" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A52" s="37"/>
-      <c r="B52" s="38"/>
-      <c r="C52" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D52" s="38"/>
-      <c r="E52" s="40"/>
-      <c r="F52" s="40"/>
-      <c r="G52" s="41"/>
-      <c r="H52" s="41"/>
-      <c r="I52" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J52" s="45"/>
-      <c r="K52" s="43"/>
-    </row>
-    <row r="53" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A53" s="37"/>
-      <c r="B53" s="38"/>
-      <c r="C53" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D53" s="38"/>
-      <c r="E53" s="40"/>
-      <c r="F53" s="40"/>
-      <c r="G53" s="41"/>
-      <c r="H53" s="41"/>
-      <c r="I53" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J53" s="45"/>
-      <c r="K53" s="43"/>
+      <c r="A52" s="13"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F52" s="15"/>
+      <c r="G52" s="18">
+        <f t="shared" ref="G52:H52" si="2">SUM(G40:G51)</f>
+        <v>0</v>
+      </c>
+      <c r="H52" s="18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I52" s="18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J52" s="19"/>
+      <c r="K52" s="46"/>
+    </row>
+    <row r="53" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="B53" s="61"/>
+      <c r="C53" s="61"/>
+      <c r="D53" s="61"/>
+      <c r="E53" s="61"/>
+      <c r="F53" s="61"/>
+      <c r="G53" s="61"/>
+      <c r="H53" s="61"/>
+      <c r="I53" s="61"/>
+      <c r="J53" s="61"/>
+      <c r="K53" s="62"/>
     </row>
     <row r="54" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A54" s="37"/>
-      <c r="B54" s="38"/>
-      <c r="C54" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D54" s="38"/>
-      <c r="E54" s="40"/>
-      <c r="F54" s="40"/>
-      <c r="G54" s="41"/>
-      <c r="H54" s="41"/>
-      <c r="I54" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J54" s="45"/>
-      <c r="K54" s="43"/>
-    </row>
-    <row r="55" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A55" s="37"/>
-      <c r="B55" s="38"/>
-      <c r="C55" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D55" s="38"/>
-      <c r="E55" s="40"/>
-      <c r="F55" s="40"/>
-      <c r="G55" s="41"/>
-      <c r="H55" s="41"/>
-      <c r="I55" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J55" s="45"/>
-      <c r="K55" s="43"/>
+      <c r="A54" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B54" s="66" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" s="61"/>
+      <c r="D54" s="61"/>
+      <c r="E54" s="61"/>
+      <c r="F54" s="61"/>
+      <c r="G54" s="61"/>
+      <c r="H54" s="61"/>
+      <c r="I54" s="61"/>
+      <c r="J54" s="61"/>
+      <c r="K54" s="62"/>
+    </row>
+    <row r="55" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B55" s="66" t="s">
+        <v>15</v>
+      </c>
+      <c r="C55" s="61"/>
+      <c r="D55" s="61"/>
+      <c r="E55" s="61"/>
+      <c r="F55" s="61"/>
+      <c r="G55" s="61"/>
+      <c r="H55" s="61"/>
+      <c r="I55" s="61"/>
+      <c r="J55" s="61"/>
+      <c r="K55" s="62"/>
     </row>
     <row r="56" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A56" s="37"/>
@@ -2737,7 +2856,7 @@
       <c r="G56" s="41"/>
       <c r="H56" s="41"/>
       <c r="I56" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="I56:I66" si="3">H56-G56</f>
         <v>0</v>
       </c>
       <c r="J56" s="45"/>
@@ -2798,77 +2917,76 @@
       <c r="K59" s="43"/>
     </row>
     <row r="60" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A60" s="13"/>
-      <c r="B60" s="15"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F60" s="15"/>
-      <c r="G60" s="18">
-        <f t="shared" ref="G60:H60" si="4">SUM(G50:G59)</f>
-        <v>0</v>
-      </c>
-      <c r="H60" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I60" s="18">
+      <c r="A60" s="37"/>
+      <c r="B60" s="38"/>
+      <c r="C60" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D60" s="38"/>
+      <c r="E60" s="40"/>
+      <c r="F60" s="40"/>
+      <c r="G60" s="41"/>
+      <c r="H60" s="41"/>
+      <c r="I60" s="41">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J60" s="19"/>
-      <c r="K60" s="46"/>
-    </row>
-    <row r="61" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="73" t="s">
-        <v>22</v>
-      </c>
-      <c r="B61" s="54"/>
-      <c r="C61" s="54"/>
-      <c r="D61" s="54"/>
-      <c r="E61" s="54"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="54"/>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="54"/>
-      <c r="K61" s="55"/>
+      <c r="J60" s="45"/>
+      <c r="K60" s="43"/>
+    </row>
+    <row r="61" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A61" s="37"/>
+      <c r="B61" s="38"/>
+      <c r="C61" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D61" s="38"/>
+      <c r="E61" s="40"/>
+      <c r="F61" s="40"/>
+      <c r="G61" s="41"/>
+      <c r="H61" s="41"/>
+      <c r="I61" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J61" s="45"/>
+      <c r="K61" s="43"/>
     </row>
     <row r="62" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A62" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B62" s="57" t="s">
-        <v>13</v>
-      </c>
-      <c r="C62" s="54"/>
-      <c r="D62" s="54"/>
-      <c r="E62" s="54"/>
-      <c r="F62" s="54"/>
-      <c r="G62" s="54"/>
-      <c r="H62" s="54"/>
-      <c r="I62" s="54"/>
-      <c r="J62" s="54"/>
-      <c r="K62" s="55"/>
-    </row>
-    <row r="63" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B63" s="57" t="s">
-        <v>15</v>
-      </c>
-      <c r="C63" s="54"/>
-      <c r="D63" s="54"/>
-      <c r="E63" s="54"/>
-      <c r="F63" s="54"/>
-      <c r="G63" s="54"/>
-      <c r="H63" s="54"/>
-      <c r="I63" s="54"/>
-      <c r="J63" s="54"/>
-      <c r="K63" s="55"/>
+      <c r="A62" s="37"/>
+      <c r="B62" s="38"/>
+      <c r="C62" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D62" s="38"/>
+      <c r="E62" s="40"/>
+      <c r="F62" s="40"/>
+      <c r="G62" s="41"/>
+      <c r="H62" s="41"/>
+      <c r="I62" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J62" s="45"/>
+      <c r="K62" s="43"/>
+    </row>
+    <row r="63" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A63" s="37"/>
+      <c r="B63" s="38"/>
+      <c r="C63" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D63" s="38"/>
+      <c r="E63" s="40"/>
+      <c r="F63" s="40"/>
+      <c r="G63" s="41"/>
+      <c r="H63" s="41"/>
+      <c r="I63" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J63" s="45"/>
+      <c r="K63" s="43"/>
     </row>
     <row r="64" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A64" s="37"/>
@@ -2882,7 +3000,7 @@
       <c r="G64" s="41"/>
       <c r="H64" s="41"/>
       <c r="I64" s="41">
-        <f t="shared" ref="I64:I74" si="5">H64-G64</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J64" s="45"/>
@@ -2900,83 +3018,84 @@
       <c r="G65" s="41"/>
       <c r="H65" s="41"/>
       <c r="I65" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J65" s="45"/>
       <c r="K65" s="43"/>
     </row>
     <row r="66" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A66" s="37"/>
-      <c r="B66" s="38"/>
-      <c r="C66" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D66" s="38"/>
-      <c r="E66" s="40"/>
-      <c r="F66" s="40"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="41"/>
-      <c r="I66" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J66" s="45"/>
-      <c r="K66" s="43"/>
-    </row>
-    <row r="67" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A67" s="37"/>
-      <c r="B67" s="38"/>
-      <c r="C67" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D67" s="38"/>
-      <c r="E67" s="40"/>
-      <c r="F67" s="40"/>
-      <c r="G67" s="41"/>
-      <c r="H67" s="41"/>
-      <c r="I67" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J67" s="45"/>
-      <c r="K67" s="43"/>
+      <c r="A66" s="13"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="15"/>
+      <c r="E66" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F66" s="15"/>
+      <c r="G66" s="18">
+        <f t="shared" ref="G66:H66" si="4">SUM(G56:G65)</f>
+        <v>0</v>
+      </c>
+      <c r="H66" s="18">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I66" s="18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J66" s="19"/>
+      <c r="K66" s="46"/>
+    </row>
+    <row r="67" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="67" t="s">
+        <v>22</v>
+      </c>
+      <c r="B67" s="61"/>
+      <c r="C67" s="61"/>
+      <c r="D67" s="61"/>
+      <c r="E67" s="61"/>
+      <c r="F67" s="61"/>
+      <c r="G67" s="61"/>
+      <c r="H67" s="61"/>
+      <c r="I67" s="61"/>
+      <c r="J67" s="61"/>
+      <c r="K67" s="62"/>
     </row>
     <row r="68" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A68" s="37"/>
-      <c r="B68" s="38"/>
-      <c r="C68" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D68" s="38"/>
-      <c r="E68" s="40"/>
-      <c r="F68" s="40"/>
-      <c r="G68" s="41"/>
-      <c r="H68" s="41"/>
-      <c r="I68" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J68" s="45"/>
-      <c r="K68" s="43"/>
-    </row>
-    <row r="69" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A69" s="37"/>
-      <c r="B69" s="38"/>
-      <c r="C69" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D69" s="38"/>
-      <c r="E69" s="40"/>
-      <c r="F69" s="40"/>
-      <c r="G69" s="41"/>
-      <c r="H69" s="41"/>
-      <c r="I69" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J69" s="45"/>
-      <c r="K69" s="43"/>
+      <c r="A68" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B68" s="69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C68" s="61"/>
+      <c r="D68" s="61"/>
+      <c r="E68" s="61"/>
+      <c r="F68" s="61"/>
+      <c r="G68" s="61"/>
+      <c r="H68" s="61"/>
+      <c r="I68" s="61"/>
+      <c r="J68" s="61"/>
+      <c r="K68" s="62"/>
+    </row>
+    <row r="69" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B69" s="69" t="s">
+        <v>15</v>
+      </c>
+      <c r="C69" s="61"/>
+      <c r="D69" s="61"/>
+      <c r="E69" s="61"/>
+      <c r="F69" s="61"/>
+      <c r="G69" s="61"/>
+      <c r="H69" s="61"/>
+      <c r="I69" s="61"/>
+      <c r="J69" s="61"/>
+      <c r="K69" s="62"/>
     </row>
     <row r="70" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A70" s="37"/>
@@ -2990,7 +3109,7 @@
       <c r="G70" s="41"/>
       <c r="H70" s="41"/>
       <c r="I70" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I70:I80" si="5">H70-G70</f>
         <v>0</v>
       </c>
       <c r="J70" s="45"/>
@@ -3051,77 +3170,76 @@
       <c r="K73" s="43"/>
     </row>
     <row r="74" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A74" s="13"/>
-      <c r="B74" s="15"/>
-      <c r="C74" s="15"/>
-      <c r="D74" s="15"/>
-      <c r="E74" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F74" s="15"/>
-      <c r="G74" s="18">
-        <f t="shared" ref="G74:H74" si="6">SUM(G64:G73)</f>
-        <v>0</v>
-      </c>
-      <c r="H74" s="18">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="I74" s="18">
+      <c r="A74" s="37"/>
+      <c r="B74" s="38"/>
+      <c r="C74" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D74" s="38"/>
+      <c r="E74" s="40"/>
+      <c r="F74" s="40"/>
+      <c r="G74" s="41"/>
+      <c r="H74" s="41"/>
+      <c r="I74" s="41">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J74" s="19"/>
-      <c r="K74" s="46"/>
-    </row>
-    <row r="75" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="58" t="s">
-        <v>23</v>
-      </c>
-      <c r="B75" s="54"/>
-      <c r="C75" s="54"/>
-      <c r="D75" s="54"/>
-      <c r="E75" s="54"/>
-      <c r="F75" s="54"/>
-      <c r="G75" s="54"/>
-      <c r="H75" s="54"/>
-      <c r="I75" s="54"/>
-      <c r="J75" s="54"/>
-      <c r="K75" s="55"/>
+      <c r="J74" s="45"/>
+      <c r="K74" s="43"/>
+    </row>
+    <row r="75" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A75" s="37"/>
+      <c r="B75" s="38"/>
+      <c r="C75" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D75" s="38"/>
+      <c r="E75" s="40"/>
+      <c r="F75" s="40"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="41"/>
+      <c r="I75" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J75" s="45"/>
+      <c r="K75" s="43"/>
     </row>
     <row r="76" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A76" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B76" s="59" t="s">
-        <v>13</v>
-      </c>
-      <c r="C76" s="54"/>
-      <c r="D76" s="54"/>
-      <c r="E76" s="54"/>
-      <c r="F76" s="54"/>
-      <c r="G76" s="54"/>
-      <c r="H76" s="54"/>
-      <c r="I76" s="54"/>
-      <c r="J76" s="54"/>
-      <c r="K76" s="55"/>
-    </row>
-    <row r="77" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="B77" s="59" t="s">
-        <v>15</v>
-      </c>
-      <c r="C77" s="54"/>
-      <c r="D77" s="54"/>
-      <c r="E77" s="54"/>
-      <c r="F77" s="54"/>
-      <c r="G77" s="54"/>
-      <c r="H77" s="54"/>
-      <c r="I77" s="54"/>
-      <c r="J77" s="54"/>
-      <c r="K77" s="55"/>
+      <c r="A76" s="37"/>
+      <c r="B76" s="38"/>
+      <c r="C76" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D76" s="38"/>
+      <c r="E76" s="40"/>
+      <c r="F76" s="40"/>
+      <c r="G76" s="41"/>
+      <c r="H76" s="41"/>
+      <c r="I76" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J76" s="45"/>
+      <c r="K76" s="43"/>
+    </row>
+    <row r="77" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A77" s="37"/>
+      <c r="B77" s="38"/>
+      <c r="C77" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D77" s="38"/>
+      <c r="E77" s="40"/>
+      <c r="F77" s="40"/>
+      <c r="G77" s="41"/>
+      <c r="H77" s="41"/>
+      <c r="I77" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J77" s="45"/>
+      <c r="K77" s="43"/>
     </row>
     <row r="78" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A78" s="37"/>
@@ -3135,7 +3253,7 @@
       <c r="G78" s="41"/>
       <c r="H78" s="41"/>
       <c r="I78" s="41">
-        <f t="shared" ref="I78:I88" si="7">H78-G78</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J78" s="45"/>
@@ -3153,83 +3271,84 @@
       <c r="G79" s="41"/>
       <c r="H79" s="41"/>
       <c r="I79" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J79" s="45"/>
       <c r="K79" s="43"/>
     </row>
     <row r="80" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A80" s="37"/>
-      <c r="B80" s="38"/>
-      <c r="C80" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D80" s="38"/>
-      <c r="E80" s="40"/>
-      <c r="F80" s="40"/>
-      <c r="G80" s="41"/>
-      <c r="H80" s="41"/>
-      <c r="I80" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J80" s="45"/>
-      <c r="K80" s="43"/>
-    </row>
-    <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A81" s="37"/>
-      <c r="B81" s="38"/>
-      <c r="C81" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D81" s="38"/>
-      <c r="E81" s="40"/>
-      <c r="F81" s="40"/>
-      <c r="G81" s="41"/>
-      <c r="H81" s="41"/>
-      <c r="I81" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J81" s="45"/>
-      <c r="K81" s="43"/>
+      <c r="A80" s="13"/>
+      <c r="B80" s="15"/>
+      <c r="C80" s="15"/>
+      <c r="D80" s="15"/>
+      <c r="E80" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F80" s="15"/>
+      <c r="G80" s="18">
+        <f t="shared" ref="G80:H80" si="6">SUM(G70:G79)</f>
+        <v>0</v>
+      </c>
+      <c r="H80" s="18">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I80" s="18">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J80" s="19"/>
+      <c r="K80" s="46"/>
+    </row>
+    <row r="81" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="72" t="s">
+        <v>23</v>
+      </c>
+      <c r="B81" s="61"/>
+      <c r="C81" s="61"/>
+      <c r="D81" s="61"/>
+      <c r="E81" s="61"/>
+      <c r="F81" s="61"/>
+      <c r="G81" s="61"/>
+      <c r="H81" s="61"/>
+      <c r="I81" s="61"/>
+      <c r="J81" s="61"/>
+      <c r="K81" s="62"/>
     </row>
     <row r="82" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A82" s="37"/>
-      <c r="B82" s="38"/>
-      <c r="C82" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D82" s="38"/>
-      <c r="E82" s="40"/>
-      <c r="F82" s="40"/>
-      <c r="G82" s="41"/>
-      <c r="H82" s="41"/>
-      <c r="I82" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J82" s="45"/>
-      <c r="K82" s="43"/>
-    </row>
-    <row r="83" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A83" s="37"/>
-      <c r="B83" s="38"/>
-      <c r="C83" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D83" s="38"/>
-      <c r="E83" s="40"/>
-      <c r="F83" s="40"/>
-      <c r="G83" s="41"/>
-      <c r="H83" s="41"/>
-      <c r="I83" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J83" s="45"/>
-      <c r="K83" s="43"/>
+      <c r="A82" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B82" s="73" t="s">
+        <v>13</v>
+      </c>
+      <c r="C82" s="61"/>
+      <c r="D82" s="61"/>
+      <c r="E82" s="61"/>
+      <c r="F82" s="61"/>
+      <c r="G82" s="61"/>
+      <c r="H82" s="61"/>
+      <c r="I82" s="61"/>
+      <c r="J82" s="61"/>
+      <c r="K82" s="62"/>
+    </row>
+    <row r="83" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B83" s="73" t="s">
+        <v>15</v>
+      </c>
+      <c r="C83" s="61"/>
+      <c r="D83" s="61"/>
+      <c r="E83" s="61"/>
+      <c r="F83" s="61"/>
+      <c r="G83" s="61"/>
+      <c r="H83" s="61"/>
+      <c r="I83" s="61"/>
+      <c r="J83" s="61"/>
+      <c r="K83" s="62"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="37"/>
@@ -3243,7 +3362,7 @@
       <c r="G84" s="41"/>
       <c r="H84" s="41"/>
       <c r="I84" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="I84:I94" si="7">H84-G84</f>
         <v>0</v>
       </c>
       <c r="J84" s="45"/>
@@ -3304,77 +3423,76 @@
       <c r="K87" s="43"/>
     </row>
     <row r="88" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A88" s="13"/>
-      <c r="B88" s="15"/>
-      <c r="C88" s="15"/>
-      <c r="D88" s="15"/>
-      <c r="E88" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F88" s="15"/>
-      <c r="G88" s="18">
-        <f t="shared" ref="G88:H88" si="8">SUM(G78:G87)</f>
-        <v>0</v>
-      </c>
-      <c r="H88" s="18">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I88" s="18">
+      <c r="A88" s="37"/>
+      <c r="B88" s="38"/>
+      <c r="C88" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D88" s="38"/>
+      <c r="E88" s="40"/>
+      <c r="F88" s="40"/>
+      <c r="G88" s="41"/>
+      <c r="H88" s="41"/>
+      <c r="I88" s="41">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J88" s="19"/>
-      <c r="K88" s="46"/>
-    </row>
-    <row r="89" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="B89" s="54"/>
-      <c r="C89" s="54"/>
-      <c r="D89" s="54"/>
-      <c r="E89" s="54"/>
-      <c r="F89" s="54"/>
-      <c r="G89" s="54"/>
-      <c r="H89" s="54"/>
-      <c r="I89" s="54"/>
-      <c r="J89" s="54"/>
-      <c r="K89" s="55"/>
+      <c r="J88" s="45"/>
+      <c r="K88" s="43"/>
+    </row>
+    <row r="89" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A89" s="37"/>
+      <c r="B89" s="38"/>
+      <c r="C89" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D89" s="38"/>
+      <c r="E89" s="40"/>
+      <c r="F89" s="40"/>
+      <c r="G89" s="41"/>
+      <c r="H89" s="41"/>
+      <c r="I89" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J89" s="45"/>
+      <c r="K89" s="43"/>
     </row>
     <row r="90" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A90" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B90" s="53" t="s">
-        <v>13</v>
-      </c>
-      <c r="C90" s="54"/>
-      <c r="D90" s="54"/>
-      <c r="E90" s="54"/>
-      <c r="F90" s="54"/>
-      <c r="G90" s="54"/>
-      <c r="H90" s="54"/>
-      <c r="I90" s="54"/>
-      <c r="J90" s="54"/>
-      <c r="K90" s="55"/>
-    </row>
-    <row r="91" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B91" s="53" t="s">
-        <v>15</v>
-      </c>
-      <c r="C91" s="54"/>
-      <c r="D91" s="54"/>
-      <c r="E91" s="54"/>
-      <c r="F91" s="54"/>
-      <c r="G91" s="54"/>
-      <c r="H91" s="54"/>
-      <c r="I91" s="54"/>
-      <c r="J91" s="54"/>
-      <c r="K91" s="55"/>
+      <c r="A90" s="37"/>
+      <c r="B90" s="38"/>
+      <c r="C90" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D90" s="38"/>
+      <c r="E90" s="40"/>
+      <c r="F90" s="40"/>
+      <c r="G90" s="41"/>
+      <c r="H90" s="41"/>
+      <c r="I90" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J90" s="45"/>
+      <c r="K90" s="43"/>
+    </row>
+    <row r="91" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A91" s="37"/>
+      <c r="B91" s="38"/>
+      <c r="C91" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D91" s="38"/>
+      <c r="E91" s="40"/>
+      <c r="F91" s="40"/>
+      <c r="G91" s="41"/>
+      <c r="H91" s="41"/>
+      <c r="I91" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J91" s="45"/>
+      <c r="K91" s="43"/>
     </row>
     <row r="92" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A92" s="37"/>
@@ -3388,7 +3506,7 @@
       <c r="G92" s="41"/>
       <c r="H92" s="41"/>
       <c r="I92" s="41">
-        <f t="shared" ref="I92:I102" si="9">H92-G92</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J92" s="45"/>
@@ -3406,85 +3524,84 @@
       <c r="G93" s="41"/>
       <c r="H93" s="41"/>
       <c r="I93" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J93" s="45"/>
       <c r="K93" s="43"/>
     </row>
     <row r="94" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A94" s="37"/>
-      <c r="B94" s="38"/>
-      <c r="C94" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D94" s="38"/>
-      <c r="E94" s="40"/>
-      <c r="F94" s="40"/>
-      <c r="G94" s="41"/>
-      <c r="H94" s="41"/>
-      <c r="I94" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J94" s="45"/>
-      <c r="K94" s="43" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A95" s="37"/>
-      <c r="B95" s="38"/>
-      <c r="C95" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D95" s="38"/>
-      <c r="E95" s="40"/>
-      <c r="F95" s="40"/>
-      <c r="G95" s="41"/>
-      <c r="H95" s="41"/>
-      <c r="I95" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J95" s="45"/>
-      <c r="K95" s="43"/>
+      <c r="A94" s="13"/>
+      <c r="B94" s="15"/>
+      <c r="C94" s="15"/>
+      <c r="D94" s="15"/>
+      <c r="E94" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F94" s="15"/>
+      <c r="G94" s="18">
+        <f t="shared" ref="G94:H94" si="8">SUM(G84:G93)</f>
+        <v>0</v>
+      </c>
+      <c r="H94" s="18">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I94" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J94" s="19"/>
+      <c r="K94" s="46"/>
+    </row>
+    <row r="95" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="74" t="s">
+        <v>24</v>
+      </c>
+      <c r="B95" s="61"/>
+      <c r="C95" s="61"/>
+      <c r="D95" s="61"/>
+      <c r="E95" s="61"/>
+      <c r="F95" s="61"/>
+      <c r="G95" s="61"/>
+      <c r="H95" s="61"/>
+      <c r="I95" s="61"/>
+      <c r="J95" s="61"/>
+      <c r="K95" s="62"/>
     </row>
     <row r="96" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A96" s="37"/>
-      <c r="B96" s="38"/>
-      <c r="C96" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D96" s="38"/>
-      <c r="E96" s="40"/>
-      <c r="F96" s="40"/>
-      <c r="G96" s="41"/>
-      <c r="H96" s="41"/>
-      <c r="I96" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J96" s="45"/>
-      <c r="K96" s="43"/>
-    </row>
-    <row r="97" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A97" s="37"/>
-      <c r="B97" s="38"/>
-      <c r="C97" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D97" s="38"/>
-      <c r="E97" s="40"/>
-      <c r="F97" s="40"/>
-      <c r="G97" s="41"/>
-      <c r="H97" s="41"/>
-      <c r="I97" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J97" s="45"/>
-      <c r="K97" s="43"/>
+      <c r="A96" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B96" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="C96" s="61"/>
+      <c r="D96" s="61"/>
+      <c r="E96" s="61"/>
+      <c r="F96" s="61"/>
+      <c r="G96" s="61"/>
+      <c r="H96" s="61"/>
+      <c r="I96" s="61"/>
+      <c r="J96" s="61"/>
+      <c r="K96" s="62"/>
+    </row>
+    <row r="97" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B97" s="70" t="s">
+        <v>15</v>
+      </c>
+      <c r="C97" s="61"/>
+      <c r="D97" s="61"/>
+      <c r="E97" s="61"/>
+      <c r="F97" s="61"/>
+      <c r="G97" s="61"/>
+      <c r="H97" s="61"/>
+      <c r="I97" s="61"/>
+      <c r="J97" s="61"/>
+      <c r="K97" s="62"/>
     </row>
     <row r="98" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A98" s="37"/>
@@ -3498,7 +3615,7 @@
       <c r="G98" s="41"/>
       <c r="H98" s="41"/>
       <c r="I98" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I98:I108" si="9">H98-G98</f>
         <v>0</v>
       </c>
       <c r="J98" s="45"/>
@@ -3538,7 +3655,9 @@
         <v>0</v>
       </c>
       <c r="J100" s="45"/>
-      <c r="K100" s="43"/>
+      <c r="K100" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="101" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A101" s="37"/>
@@ -3559,77 +3678,76 @@
       <c r="K101" s="43"/>
     </row>
     <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A102" s="13"/>
-      <c r="B102" s="15"/>
-      <c r="C102" s="15"/>
-      <c r="D102" s="15"/>
-      <c r="E102" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F102" s="15"/>
-      <c r="G102" s="18">
-        <f t="shared" ref="G102:H102" si="10">SUM(G92:G101)</f>
-        <v>0</v>
-      </c>
-      <c r="H102" s="18">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="I102" s="18">
+      <c r="A102" s="37"/>
+      <c r="B102" s="38"/>
+      <c r="C102" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D102" s="38"/>
+      <c r="E102" s="40"/>
+      <c r="F102" s="40"/>
+      <c r="G102" s="41"/>
+      <c r="H102" s="41"/>
+      <c r="I102" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J102" s="19"/>
-      <c r="K102" s="46"/>
-    </row>
-    <row r="103" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="56" t="s">
-        <v>26</v>
-      </c>
-      <c r="B103" s="54"/>
-      <c r="C103" s="54"/>
-      <c r="D103" s="54"/>
-      <c r="E103" s="54"/>
-      <c r="F103" s="54"/>
-      <c r="G103" s="54"/>
-      <c r="H103" s="54"/>
-      <c r="I103" s="54"/>
-      <c r="J103" s="54"/>
-      <c r="K103" s="55"/>
+      <c r="J102" s="45"/>
+      <c r="K102" s="43"/>
+    </row>
+    <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A103" s="37"/>
+      <c r="B103" s="38"/>
+      <c r="C103" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D103" s="38"/>
+      <c r="E103" s="40"/>
+      <c r="F103" s="40"/>
+      <c r="G103" s="41"/>
+      <c r="H103" s="41"/>
+      <c r="I103" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J103" s="45"/>
+      <c r="K103" s="43"/>
     </row>
     <row r="104" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A104" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B104" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="C104" s="54"/>
-      <c r="D104" s="54"/>
-      <c r="E104" s="54"/>
-      <c r="F104" s="54"/>
-      <c r="G104" s="54"/>
-      <c r="H104" s="54"/>
-      <c r="I104" s="54"/>
-      <c r="J104" s="54"/>
-      <c r="K104" s="55"/>
-    </row>
-    <row r="105" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B105" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="C105" s="54"/>
-      <c r="D105" s="54"/>
-      <c r="E105" s="54"/>
-      <c r="F105" s="54"/>
-      <c r="G105" s="54"/>
-      <c r="H105" s="54"/>
-      <c r="I105" s="54"/>
-      <c r="J105" s="54"/>
-      <c r="K105" s="55"/>
+      <c r="A104" s="37"/>
+      <c r="B104" s="38"/>
+      <c r="C104" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D104" s="38"/>
+      <c r="E104" s="40"/>
+      <c r="F104" s="40"/>
+      <c r="G104" s="41"/>
+      <c r="H104" s="41"/>
+      <c r="I104" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J104" s="45"/>
+      <c r="K104" s="43"/>
+    </row>
+    <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A105" s="37"/>
+      <c r="B105" s="38"/>
+      <c r="C105" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D105" s="38"/>
+      <c r="E105" s="40"/>
+      <c r="F105" s="40"/>
+      <c r="G105" s="41"/>
+      <c r="H105" s="41"/>
+      <c r="I105" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J105" s="45"/>
+      <c r="K105" s="43"/>
     </row>
     <row r="106" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A106" s="37"/>
@@ -3643,7 +3761,7 @@
       <c r="G106" s="41"/>
       <c r="H106" s="41"/>
       <c r="I106" s="41">
-        <f t="shared" ref="I106:I116" si="11">H106-G106</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J106" s="45"/>
@@ -3661,83 +3779,84 @@
       <c r="G107" s="41"/>
       <c r="H107" s="41"/>
       <c r="I107" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J107" s="45"/>
       <c r="K107" s="43"/>
     </row>
     <row r="108" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A108" s="37"/>
-      <c r="B108" s="38"/>
-      <c r="C108" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D108" s="38"/>
-      <c r="E108" s="40"/>
-      <c r="F108" s="40"/>
-      <c r="G108" s="41"/>
-      <c r="H108" s="41"/>
-      <c r="I108" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J108" s="45"/>
-      <c r="K108" s="43"/>
-    </row>
-    <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A109" s="37"/>
-      <c r="B109" s="38"/>
-      <c r="C109" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D109" s="38"/>
-      <c r="E109" s="40"/>
-      <c r="F109" s="40"/>
-      <c r="G109" s="41"/>
-      <c r="H109" s="41"/>
-      <c r="I109" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J109" s="45"/>
-      <c r="K109" s="43"/>
+      <c r="A108" s="13"/>
+      <c r="B108" s="15"/>
+      <c r="C108" s="15"/>
+      <c r="D108" s="15"/>
+      <c r="E108" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F108" s="15"/>
+      <c r="G108" s="18">
+        <f t="shared" ref="G108:H108" si="10">SUM(G98:G107)</f>
+        <v>0</v>
+      </c>
+      <c r="H108" s="18">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="I108" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J108" s="19"/>
+      <c r="K108" s="46"/>
+    </row>
+    <row r="109" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="71" t="s">
+        <v>26</v>
+      </c>
+      <c r="B109" s="61"/>
+      <c r="C109" s="61"/>
+      <c r="D109" s="61"/>
+      <c r="E109" s="61"/>
+      <c r="F109" s="61"/>
+      <c r="G109" s="61"/>
+      <c r="H109" s="61"/>
+      <c r="I109" s="61"/>
+      <c r="J109" s="61"/>
+      <c r="K109" s="62"/>
     </row>
     <row r="110" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A110" s="37"/>
-      <c r="B110" s="38"/>
-      <c r="C110" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D110" s="38"/>
-      <c r="E110" s="40"/>
-      <c r="F110" s="40"/>
-      <c r="G110" s="41"/>
-      <c r="H110" s="41"/>
-      <c r="I110" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J110" s="45"/>
-      <c r="K110" s="43"/>
-    </row>
-    <row r="111" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A111" s="37"/>
-      <c r="B111" s="38"/>
-      <c r="C111" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D111" s="38"/>
-      <c r="E111" s="40"/>
-      <c r="F111" s="40"/>
-      <c r="G111" s="41"/>
-      <c r="H111" s="41"/>
-      <c r="I111" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J111" s="45"/>
-      <c r="K111" s="43"/>
+      <c r="A110" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B110" s="68" t="s">
+        <v>13</v>
+      </c>
+      <c r="C110" s="61"/>
+      <c r="D110" s="61"/>
+      <c r="E110" s="61"/>
+      <c r="F110" s="61"/>
+      <c r="G110" s="61"/>
+      <c r="H110" s="61"/>
+      <c r="I110" s="61"/>
+      <c r="J110" s="61"/>
+      <c r="K110" s="62"/>
+    </row>
+    <row r="111" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B111" s="68" t="s">
+        <v>15</v>
+      </c>
+      <c r="C111" s="61"/>
+      <c r="D111" s="61"/>
+      <c r="E111" s="61"/>
+      <c r="F111" s="61"/>
+      <c r="G111" s="61"/>
+      <c r="H111" s="61"/>
+      <c r="I111" s="61"/>
+      <c r="J111" s="61"/>
+      <c r="K111" s="62"/>
     </row>
     <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A112" s="37"/>
@@ -3751,7 +3870,7 @@
       <c r="G112" s="41"/>
       <c r="H112" s="41"/>
       <c r="I112" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="I112:I122" si="11">H112-G112</f>
         <v>0</v>
       </c>
       <c r="J112" s="45"/>
@@ -3812,77 +3931,76 @@
       <c r="K115" s="43"/>
     </row>
     <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A116" s="13"/>
-      <c r="B116" s="15"/>
-      <c r="C116" s="15"/>
-      <c r="D116" s="15"/>
-      <c r="E116" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F116" s="15"/>
-      <c r="G116" s="18">
-        <f t="shared" ref="G116:H116" si="12">SUM(G106:G115)</f>
-        <v>0</v>
-      </c>
-      <c r="H116" s="18">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="I116" s="18">
+      <c r="A116" s="37"/>
+      <c r="B116" s="38"/>
+      <c r="C116" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D116" s="38"/>
+      <c r="E116" s="40"/>
+      <c r="F116" s="40"/>
+      <c r="G116" s="41"/>
+      <c r="H116" s="41"/>
+      <c r="I116" s="41">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J116" s="19"/>
-      <c r="K116" s="46"/>
-    </row>
-    <row r="117" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="B117" s="62"/>
-      <c r="C117" s="62"/>
-      <c r="D117" s="62"/>
-      <c r="E117" s="62"/>
-      <c r="F117" s="62"/>
-      <c r="G117" s="62"/>
-      <c r="H117" s="62"/>
-      <c r="I117" s="62"/>
-      <c r="J117" s="62"/>
-      <c r="K117" s="63"/>
+      <c r="J116" s="45"/>
+      <c r="K116" s="43"/>
+    </row>
+    <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A117" s="37"/>
+      <c r="B117" s="38"/>
+      <c r="C117" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D117" s="38"/>
+      <c r="E117" s="40"/>
+      <c r="F117" s="40"/>
+      <c r="G117" s="41"/>
+      <c r="H117" s="41"/>
+      <c r="I117" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J117" s="45"/>
+      <c r="K117" s="43"/>
     </row>
     <row r="118" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A118" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B118" s="64" t="s">
-        <v>13</v>
-      </c>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
-    </row>
-    <row r="119" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B119" s="64" t="s">
-        <v>15</v>
-      </c>
-      <c r="C119" s="62"/>
-      <c r="D119" s="62"/>
-      <c r="E119" s="62"/>
-      <c r="F119" s="62"/>
-      <c r="G119" s="62"/>
-      <c r="H119" s="62"/>
-      <c r="I119" s="62"/>
-      <c r="J119" s="62"/>
-      <c r="K119" s="63"/>
+      <c r="A118" s="37"/>
+      <c r="B118" s="38"/>
+      <c r="C118" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D118" s="38"/>
+      <c r="E118" s="40"/>
+      <c r="F118" s="40"/>
+      <c r="G118" s="41"/>
+      <c r="H118" s="41"/>
+      <c r="I118" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J118" s="45"/>
+      <c r="K118" s="43"/>
+    </row>
+    <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A119" s="37"/>
+      <c r="B119" s="38"/>
+      <c r="C119" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D119" s="38"/>
+      <c r="E119" s="40"/>
+      <c r="F119" s="40"/>
+      <c r="G119" s="41"/>
+      <c r="H119" s="41"/>
+      <c r="I119" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J119" s="45"/>
+      <c r="K119" s="43"/>
     </row>
     <row r="120" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A120" s="37"/>
@@ -3896,7 +4014,7 @@
       <c r="G120" s="41"/>
       <c r="H120" s="41"/>
       <c r="I120" s="41">
-        <f t="shared" ref="I120:I130" si="13">H120-G120</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J120" s="45"/>
@@ -3914,83 +4032,84 @@
       <c r="G121" s="41"/>
       <c r="H121" s="41"/>
       <c r="I121" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J121" s="45"/>
       <c r="K121" s="43"/>
     </row>
     <row r="122" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A122" s="37"/>
-      <c r="B122" s="38"/>
-      <c r="C122" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D122" s="38"/>
-      <c r="E122" s="40"/>
-      <c r="F122" s="40"/>
-      <c r="G122" s="41"/>
-      <c r="H122" s="41"/>
-      <c r="I122" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J122" s="45"/>
-      <c r="K122" s="43"/>
-    </row>
-    <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A123" s="37"/>
-      <c r="B123" s="38"/>
-      <c r="C123" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D123" s="38"/>
-      <c r="E123" s="40"/>
-      <c r="F123" s="40"/>
-      <c r="G123" s="41"/>
-      <c r="H123" s="41"/>
-      <c r="I123" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J123" s="45"/>
-      <c r="K123" s="43"/>
+      <c r="A122" s="13"/>
+      <c r="B122" s="15"/>
+      <c r="C122" s="15"/>
+      <c r="D122" s="15"/>
+      <c r="E122" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F122" s="15"/>
+      <c r="G122" s="18">
+        <f t="shared" ref="G122:H122" si="12">SUM(G112:G121)</f>
+        <v>0</v>
+      </c>
+      <c r="H122" s="18">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="I122" s="18">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J122" s="19"/>
+      <c r="K122" s="46"/>
+    </row>
+    <row r="123" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="53" t="s">
+        <v>27</v>
+      </c>
+      <c r="B123" s="54"/>
+      <c r="C123" s="54"/>
+      <c r="D123" s="54"/>
+      <c r="E123" s="54"/>
+      <c r="F123" s="54"/>
+      <c r="G123" s="54"/>
+      <c r="H123" s="54"/>
+      <c r="I123" s="54"/>
+      <c r="J123" s="54"/>
+      <c r="K123" s="55"/>
     </row>
     <row r="124" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A124" s="37"/>
-      <c r="B124" s="38"/>
-      <c r="C124" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D124" s="38"/>
-      <c r="E124" s="40"/>
-      <c r="F124" s="40"/>
-      <c r="G124" s="41"/>
-      <c r="H124" s="41"/>
-      <c r="I124" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J124" s="45"/>
-      <c r="K124" s="43"/>
-    </row>
-    <row r="125" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A125" s="37"/>
-      <c r="B125" s="38"/>
-      <c r="C125" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D125" s="38"/>
-      <c r="E125" s="40"/>
-      <c r="F125" s="40"/>
-      <c r="G125" s="41"/>
-      <c r="H125" s="41"/>
-      <c r="I125" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J125" s="45"/>
-      <c r="K125" s="43"/>
+      <c r="A124" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B124" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="C124" s="54"/>
+      <c r="D124" s="54"/>
+      <c r="E124" s="54"/>
+      <c r="F124" s="54"/>
+      <c r="G124" s="54"/>
+      <c r="H124" s="54"/>
+      <c r="I124" s="54"/>
+      <c r="J124" s="54"/>
+      <c r="K124" s="55"/>
+    </row>
+    <row r="125" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B125" s="56" t="s">
+        <v>15</v>
+      </c>
+      <c r="C125" s="54"/>
+      <c r="D125" s="54"/>
+      <c r="E125" s="54"/>
+      <c r="F125" s="54"/>
+      <c r="G125" s="54"/>
+      <c r="H125" s="54"/>
+      <c r="I125" s="54"/>
+      <c r="J125" s="54"/>
+      <c r="K125" s="55"/>
     </row>
     <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A126" s="37"/>
@@ -4004,7 +4123,7 @@
       <c r="G126" s="41"/>
       <c r="H126" s="41"/>
       <c r="I126" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="I126:I136" si="13">H126-G126</f>
         <v>0</v>
       </c>
       <c r="J126" s="45"/>
@@ -4065,35 +4184,143 @@
       <c r="K129" s="43"/>
     </row>
     <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A130" s="48"/>
-      <c r="B130" s="49"/>
-      <c r="C130" s="49"/>
-      <c r="D130" s="49"/>
-      <c r="E130" s="49" t="s">
+      <c r="A130" s="37"/>
+      <c r="B130" s="38"/>
+      <c r="C130" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D130" s="38"/>
+      <c r="E130" s="40"/>
+      <c r="F130" s="40"/>
+      <c r="G130" s="41"/>
+      <c r="H130" s="41"/>
+      <c r="I130" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J130" s="45"/>
+      <c r="K130" s="43"/>
+    </row>
+    <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A131" s="37"/>
+      <c r="B131" s="38"/>
+      <c r="C131" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D131" s="38"/>
+      <c r="E131" s="40"/>
+      <c r="F131" s="40"/>
+      <c r="G131" s="41"/>
+      <c r="H131" s="41"/>
+      <c r="I131" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J131" s="45"/>
+      <c r="K131" s="43"/>
+    </row>
+    <row r="132" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A132" s="37"/>
+      <c r="B132" s="38"/>
+      <c r="C132" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D132" s="38"/>
+      <c r="E132" s="40"/>
+      <c r="F132" s="40"/>
+      <c r="G132" s="41"/>
+      <c r="H132" s="41"/>
+      <c r="I132" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J132" s="45"/>
+      <c r="K132" s="43"/>
+    </row>
+    <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A133" s="37"/>
+      <c r="B133" s="38"/>
+      <c r="C133" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D133" s="38"/>
+      <c r="E133" s="40"/>
+      <c r="F133" s="40"/>
+      <c r="G133" s="41"/>
+      <c r="H133" s="41"/>
+      <c r="I133" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J133" s="45"/>
+      <c r="K133" s="43"/>
+    </row>
+    <row r="134" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A134" s="37"/>
+      <c r="B134" s="38"/>
+      <c r="C134" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D134" s="38"/>
+      <c r="E134" s="40"/>
+      <c r="F134" s="40"/>
+      <c r="G134" s="41"/>
+      <c r="H134" s="41"/>
+      <c r="I134" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J134" s="45"/>
+      <c r="K134" s="43"/>
+    </row>
+    <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A135" s="37"/>
+      <c r="B135" s="38"/>
+      <c r="C135" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D135" s="38"/>
+      <c r="E135" s="40"/>
+      <c r="F135" s="40"/>
+      <c r="G135" s="41"/>
+      <c r="H135" s="41"/>
+      <c r="I135" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J135" s="45"/>
+      <c r="K135" s="43"/>
+    </row>
+    <row r="136" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A136" s="48"/>
+      <c r="B136" s="49"/>
+      <c r="C136" s="49"/>
+      <c r="D136" s="49"/>
+      <c r="E136" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F130" s="49"/>
-      <c r="G130" s="50">
-        <f t="shared" ref="G130:H130" si="14">SUM(G120:G129)</f>
-        <v>0</v>
-      </c>
-      <c r="H130" s="50">
+      <c r="F136" s="49"/>
+      <c r="G136" s="50">
+        <f t="shared" ref="G136:H136" si="14">SUM(G126:G135)</f>
+        <v>0</v>
+      </c>
+      <c r="H136" s="50">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="I130" s="50">
+      <c r="I136" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J130" s="51"/>
-      <c r="K130" s="52"/>
+      <c r="J136" s="51"/>
+      <c r="K136" s="52"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K38" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{37F66CFF-D3CB-4C05-B44C-28A7219A2FB3}">
+      <autoFilter ref="A1:K15" xr:uid="{E701863D-E635-476F-BEE7-EDA0E07C86C2}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -4104,32 +4331,32 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A117:K117"/>
-    <mergeCell ref="B118:K118"/>
-    <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B96:K96"/>
+    <mergeCell ref="B97:K97"/>
+    <mergeCell ref="A109:K109"/>
+    <mergeCell ref="B69:K69"/>
+    <mergeCell ref="A81:K81"/>
+    <mergeCell ref="B82:K82"/>
+    <mergeCell ref="B83:K83"/>
+    <mergeCell ref="A95:K95"/>
+    <mergeCell ref="A123:K123"/>
+    <mergeCell ref="B124:K124"/>
+    <mergeCell ref="B125:K125"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
-    <mergeCell ref="A33:K33"/>
-    <mergeCell ref="B34:K34"/>
-    <mergeCell ref="B35:K35"/>
-    <mergeCell ref="A47:K47"/>
-    <mergeCell ref="B48:K48"/>
-    <mergeCell ref="B49:K49"/>
-    <mergeCell ref="A61:K61"/>
-    <mergeCell ref="B104:K104"/>
-    <mergeCell ref="B105:K105"/>
-    <mergeCell ref="B62:K62"/>
-    <mergeCell ref="B90:K90"/>
-    <mergeCell ref="B91:K91"/>
-    <mergeCell ref="A103:K103"/>
-    <mergeCell ref="B63:K63"/>
-    <mergeCell ref="A75:K75"/>
-    <mergeCell ref="B76:K76"/>
-    <mergeCell ref="B77:K77"/>
-    <mergeCell ref="A89:K89"/>
+    <mergeCell ref="A39:K39"/>
+    <mergeCell ref="B40:K40"/>
+    <mergeCell ref="B41:K41"/>
+    <mergeCell ref="A53:K53"/>
+    <mergeCell ref="B54:K54"/>
+    <mergeCell ref="B55:K55"/>
+    <mergeCell ref="A67:K67"/>
+    <mergeCell ref="B110:K110"/>
+    <mergeCell ref="B111:K111"/>
+    <mergeCell ref="B68:K68"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B31 B34:B45 B50:B59 B64:B73 B78:B87 B92:B101 B106:B115">
+  <conditionalFormatting sqref="B5:B37 B40:B51 B56:B65 B70:B79 B84:B93 B98:B107 B112:B121">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -4146,7 +4373,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B32 B34:B46 B48:B60 B62:B74 B76:B88 B90:B102 B104:B116 B118:B130">
+  <conditionalFormatting sqref="B5:B38 B40:B52 B54:B66 B68:B80 B82:B94 B96:B108 B110:B122 B124:B136">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -4154,34 +4381,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B120:B129">
+  <conditionalFormatting sqref="B126:B135">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B120))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B126))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B120))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B126))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B120))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B126))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B120))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B126))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B120))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B126))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G32 G36:G46 G50:G60 G64:G74 G78:G88 G92:G102 G106:G116 G120:G130">
+  <conditionalFormatting sqref="G1 G3:G38 G42:G52 G56:G66 G70:G80 G84:G94 G98:G108 G112:G122 G126:G136">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H130">
+  <conditionalFormatting sqref="H1:H136">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I36:I46 I50:I60 I64:I74 I78:I88 I92:I102 I106:I116 I120:I130 I5:I32">
+  <conditionalFormatting sqref="I5:I38 I42:I52 I56:I66 I70:I80 I84:I94 I98:I108 I112:I122 I126:I136">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -4190,7 +4417,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F120:F129 F106:F115 F36:F45 F50:F59 F64:F73 F78:F87 F92:F101 F5:F31" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F126:F135 F112:F121 F42:F51 F56:F65 F70:F79 F84:F93 F98:F107 F5:F37" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4203,13 +4430,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E31 E36:E45 E50:E59 E64:E73 E78:E87 E92:E101 E106:E115 E120:E129</xm:sqref>
+          <xm:sqref>E5:E37 E42:E51 E56:E65 E70:E79 E84:E93 E98:E107 E112:E121 E126:E135</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B31 B36:B45 B50:B59 B64:B73 B78:B87 B92:B101 B106:B115 B120:B129</xm:sqref>
+          <xm:sqref>B5:B37 B42:B51 B56:B65 B70:B79 B84:B93 B98:B107 B112:B121 B126:B135</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4289,7 +4516,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" cm="1">
-        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$36:$H$45,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
+        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$42:$H$51,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" cm="1">
@@ -5850,26 +6077,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -6104,10 +6311,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6124,20 +6362,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W1 D2 Work II (End of day)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6D9703-2FEE-47C9-905B-19589D935185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D50D50-5697-4EA3-B456-67D04EA8C759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,9 +18,9 @@
     <sheet name="Drop-downs" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$38</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$121</definedName>
-    <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$128</definedName>
+    <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$45</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <customWorkbookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="121">
   <si>
     <t>Date</t>
   </si>
@@ -433,6 +433,39 @@
   <si>
     <t>ILO 8.1</t>
   </si>
+  <si>
+    <t>https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/3b3d71a66f4e9950bc4b200f6428d8d3c5793552/Block%20B/2024-11-21.png</t>
+  </si>
+  <si>
+    <t>Upload files to GitHub for evidencing</t>
+  </si>
+  <si>
+    <t>Evidence week 1</t>
+  </si>
+  <si>
+    <t>SQL Content review session</t>
+  </si>
+  <si>
+    <t>Figure out how to connect to postgres</t>
+  </si>
+  <si>
+    <t>Re-install PostgreSQL to fix problem</t>
+  </si>
+  <si>
+    <t>Was not able to figure out how to fix the problem.</t>
+  </si>
+  <si>
+    <t>Do DataCamp course "Intermediate SQL course"</t>
+  </si>
+  <si>
+    <t>Do DataCamp course "Joining Data in SQL"</t>
+  </si>
+  <si>
+    <t>Set up VPN</t>
+  </si>
+  <si>
+    <t>Does not work at school, have to set up at home.</t>
+  </si>
 </sst>
 </file>
 
@@ -443,7 +476,7 @@
     <numFmt numFmtId="165" formatCode="d&quot;-&quot;mmm&quot;-&quot;yyyy"/>
     <numFmt numFmtId="166" formatCode="d/m/yy"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -523,6 +556,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="15">
@@ -756,10 +795,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -907,6 +947,26 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -923,8 +983,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -943,24 +1001,6 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -968,11 +1008,31 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="18">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE8B2"/>
+          <bgColor rgb="FFFCE8B2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4C7C3"/>
+          <bgColor rgb="FFF4C7C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1431,7 +1491,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K136"/>
+  <dimension ref="A1:K143"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1483,53 +1543,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="59"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="67"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="60" t="s">
+      <c r="B3" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="55"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="60" t="s">
+      <c r="B4" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="61"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
-      <c r="G4" s="61"/>
-      <c r="H4" s="61"/>
-      <c r="I4" s="61"/>
-      <c r="J4" s="61"/>
-      <c r="K4" s="62"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+      <c r="K4" s="55"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -1557,7 +1617,7 @@
         <v>0.5</v>
       </c>
       <c r="I5" s="41">
-        <f t="shared" ref="I5:I38" si="0">H5-G5</f>
+        <f t="shared" ref="I5:I45" si="0">H5-G5</f>
         <v>0</v>
       </c>
       <c r="J5" s="42"/>
@@ -2330,7 +2390,9 @@
         <f t="shared" si="0"/>
         <v>-0.5</v>
       </c>
-      <c r="J29" s="45"/>
+      <c r="J29" s="78" t="s">
+        <v>110</v>
+      </c>
       <c r="K29" s="44"/>
     </row>
     <row r="30" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -2338,13 +2400,13 @@
         <v>45617</v>
       </c>
       <c r="B30" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C30" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D30" s="38" t="s">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="E30" s="40" t="s">
         <v>64</v>
@@ -2355,18 +2417,26 @@
       <c r="G30" s="41">
         <v>0.5</v>
       </c>
-      <c r="H30" s="41"/>
+      <c r="H30" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I30" s="41">
         <f t="shared" si="0"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J30" s="45"/>
       <c r="K30" s="44"/>
     </row>
     <row r="31" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A31" s="37"/>
-      <c r="B31" s="38"/>
-      <c r="C31" s="39"/>
+      <c r="A31" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B31" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="39" t="s">
+        <v>17</v>
+      </c>
       <c r="D31" s="38" t="s">
         <v>105</v>
       </c>
@@ -2390,9 +2460,15 @@
       <c r="K31" s="44"/>
     </row>
     <row r="32" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A32" s="37"/>
-      <c r="B32" s="38"/>
-      <c r="C32" s="39"/>
+      <c r="A32" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B32" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" s="39" t="s">
+        <v>17</v>
+      </c>
       <c r="D32" s="38" t="s">
         <v>104</v>
       </c>
@@ -2405,59 +2481,92 @@
       <c r="G32" s="41">
         <v>0.25</v>
       </c>
-      <c r="H32" s="41"/>
-      <c r="I32" s="41"/>
+      <c r="H32" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="I32" s="41">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="J32" s="45"/>
       <c r="K32" s="44"/>
     </row>
     <row r="33" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A33" s="37"/>
-      <c r="B33" s="38"/>
-      <c r="C33" s="39"/>
+      <c r="A33" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B33" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="39" t="s">
+        <v>17</v>
+      </c>
       <c r="D33" s="38" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="E33" s="40" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="F33" s="40" t="s">
         <v>109</v>
       </c>
       <c r="G33" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
+        <v>1</v>
+      </c>
+      <c r="H33" s="41">
+        <v>1</v>
+      </c>
+      <c r="I33" s="41">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="J33" s="45"/>
       <c r="K33" s="44"/>
     </row>
     <row r="34" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A34" s="37"/>
-      <c r="B34" s="38"/>
-      <c r="C34" s="39"/>
+      <c r="A34" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B34" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C34" s="39" t="s">
+        <v>17</v>
+      </c>
       <c r="D34" s="38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E34" s="40" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="F34" s="40" t="s">
         <v>109</v>
       </c>
       <c r="G34" s="41">
-        <v>2</v>
-      </c>
-      <c r="H34" s="41"/>
-      <c r="I34" s="41"/>
+        <v>0.5</v>
+      </c>
+      <c r="H34" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="I34" s="41">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="J34" s="45"/>
       <c r="K34" s="44"/>
     </row>
     <row r="35" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A35" s="37"/>
-      <c r="B35" s="38"/>
-      <c r="C35" s="39"/>
+      <c r="A35" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B35" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C35" s="39" t="s">
+        <v>17</v>
+      </c>
       <c r="D35" s="38" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E35" s="40" t="s">
         <v>50</v>
@@ -2466,256 +2575,362 @@
         <v>109</v>
       </c>
       <c r="G35" s="41">
-        <v>2</v>
-      </c>
-      <c r="H35" s="41"/>
-      <c r="I35" s="41"/>
+        <v>1</v>
+      </c>
+      <c r="H35" s="41">
+        <v>1</v>
+      </c>
+      <c r="I35" s="41">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="J35" s="45"/>
       <c r="K35" s="44"/>
     </row>
     <row r="36" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A36" s="37"/>
-      <c r="B36" s="38"/>
-      <c r="C36" s="39"/>
+      <c r="A36" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B36" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="39" t="s">
+        <v>17</v>
+      </c>
       <c r="D36" s="38" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="E36" s="40" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F36" s="40" t="s">
         <v>109</v>
       </c>
       <c r="G36" s="41">
-        <v>4</v>
-      </c>
-      <c r="H36" s="41"/>
-      <c r="I36" s="41"/>
+        <v>0.5</v>
+      </c>
+      <c r="H36" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="I36" s="41">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="J36" s="45"/>
-      <c r="K36" s="44"/>
+      <c r="K36" s="44" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="37" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A37" s="37"/>
-      <c r="B37" s="38"/>
+      <c r="A37" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B37" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C37" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D37" s="38" t="s">
-        <v>107</v>
-      </c>
-      <c r="E37" s="40"/>
+        <v>115</v>
+      </c>
+      <c r="E37" s="40" t="s">
+        <v>50</v>
+      </c>
       <c r="F37" s="40" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="G37" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="H37" s="41"/>
+        <v>1</v>
+      </c>
+      <c r="H37" s="41">
+        <v>1</v>
+      </c>
       <c r="I37" s="41">
         <f t="shared" si="0"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J37" s="45"/>
       <c r="K37" s="44"/>
     </row>
     <row r="38" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A38" s="13"/>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F38" s="15"/>
-      <c r="G38" s="18">
-        <f>SUM(G5:G37)</f>
-        <v>34.85</v>
-      </c>
-      <c r="H38" s="18">
-        <f>SUM(H5:H37)</f>
-        <v>15.25</v>
-      </c>
-      <c r="I38" s="18">
+      <c r="A38" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B38" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="E38" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F38" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G38" s="41">
+        <v>1</v>
+      </c>
+      <c r="H38" s="41">
+        <v>1</v>
+      </c>
+      <c r="I38" s="41">
         <f t="shared" si="0"/>
-        <v>-19.600000000000001</v>
-      </c>
-      <c r="J38" s="19"/>
-      <c r="K38" s="46"/>
-    </row>
-    <row r="39" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="63" t="s">
-        <v>19</v>
-      </c>
-      <c r="B39" s="58"/>
-      <c r="C39" s="58"/>
-      <c r="D39" s="58"/>
-      <c r="E39" s="58"/>
-      <c r="F39" s="58"/>
-      <c r="G39" s="58"/>
-      <c r="H39" s="58"/>
-      <c r="I39" s="58"/>
-      <c r="J39" s="58"/>
-      <c r="K39" s="59"/>
+        <v>0</v>
+      </c>
+      <c r="J38" s="45"/>
+      <c r="K38" s="44"/>
+    </row>
+    <row r="39" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A39" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B39" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="E39" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F39" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G39" s="41">
+        <v>1</v>
+      </c>
+      <c r="H39" s="41"/>
+      <c r="I39" s="41">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="J39" s="45"/>
+      <c r="K39" s="44" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="40" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A40" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="B40" s="64" t="s">
-        <v>13</v>
-      </c>
-      <c r="C40" s="61"/>
-      <c r="D40" s="61"/>
-      <c r="E40" s="61"/>
-      <c r="F40" s="61"/>
-      <c r="G40" s="61"/>
-      <c r="H40" s="61"/>
-      <c r="I40" s="61"/>
-      <c r="J40" s="61"/>
-      <c r="K40" s="62"/>
-    </row>
-    <row r="41" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B41" s="64" t="s">
-        <v>20</v>
-      </c>
-      <c r="C41" s="61"/>
-      <c r="D41" s="61"/>
-      <c r="E41" s="61"/>
-      <c r="F41" s="61"/>
-      <c r="G41" s="61"/>
-      <c r="H41" s="61"/>
-      <c r="I41" s="61"/>
-      <c r="J41" s="61"/>
-      <c r="K41" s="62"/>
+      <c r="A40" s="37">
+        <v>45618</v>
+      </c>
+      <c r="B40" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C40" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="E40" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F40" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G40" s="41">
+        <v>4</v>
+      </c>
+      <c r="H40" s="41"/>
+      <c r="I40" s="41">
+        <f t="shared" si="0"/>
+        <v>-4</v>
+      </c>
+      <c r="J40" s="45"/>
+      <c r="K40" s="44"/>
+    </row>
+    <row r="41" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A41" s="37"/>
+      <c r="B41" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C41" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="E41" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="F41" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G41" s="41">
+        <v>4</v>
+      </c>
+      <c r="H41" s="41"/>
+      <c r="I41" s="41">
+        <f t="shared" si="0"/>
+        <v>-4</v>
+      </c>
+      <c r="J41" s="45"/>
+      <c r="K41" s="44"/>
     </row>
     <row r="42" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A42" s="47"/>
-      <c r="B42" s="38"/>
+      <c r="A42" s="37"/>
+      <c r="B42" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C42" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D42" s="38"/>
-      <c r="E42" s="40"/>
-      <c r="F42" s="40"/>
-      <c r="G42" s="41"/>
+      <c r="D42" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="E42" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="F42" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G42" s="41">
+        <v>4</v>
+      </c>
       <c r="H42" s="41"/>
       <c r="I42" s="41">
-        <f t="shared" ref="I42:I52" si="1">H42-G42</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-4</v>
       </c>
       <c r="J42" s="45"/>
-      <c r="K42" s="43"/>
+      <c r="K42" s="44"/>
     </row>
     <row r="43" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A43" s="47"/>
-      <c r="B43" s="38"/>
+      <c r="A43" s="37"/>
+      <c r="B43" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C43" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D43" s="38"/>
-      <c r="E43" s="40"/>
-      <c r="F43" s="40"/>
-      <c r="G43" s="41"/>
+      <c r="D43" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="E43" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F43" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G43" s="41">
+        <v>0.5</v>
+      </c>
       <c r="H43" s="41"/>
       <c r="I43" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
       </c>
       <c r="J43" s="45"/>
-      <c r="K43" s="43"/>
+      <c r="K43" s="44"/>
     </row>
     <row r="44" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A44" s="47"/>
-      <c r="B44" s="38"/>
+      <c r="A44" s="37"/>
+      <c r="B44" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C44" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D44" s="38"/>
-      <c r="E44" s="40"/>
-      <c r="F44" s="40"/>
-      <c r="G44" s="41"/>
+      <c r="D44" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="E44" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F44" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G44" s="41">
+        <v>0.5</v>
+      </c>
       <c r="H44" s="41"/>
       <c r="I44" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
       </c>
       <c r="J44" s="45"/>
-      <c r="K44" s="43"/>
+      <c r="K44" s="44"/>
     </row>
     <row r="45" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A45" s="47"/>
-      <c r="B45" s="38"/>
-      <c r="C45" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D45" s="38"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="41"/>
-      <c r="H45" s="41"/>
-      <c r="I45" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J45" s="45"/>
-      <c r="K45" s="43"/>
-    </row>
-    <row r="46" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A46" s="47"/>
-      <c r="B46" s="38"/>
-      <c r="C46" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D46" s="38"/>
-      <c r="E46" s="40"/>
-      <c r="F46" s="40"/>
-      <c r="G46" s="41"/>
-      <c r="H46" s="41"/>
-      <c r="I46" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J46" s="45"/>
-      <c r="K46" s="43"/>
+      <c r="A45" s="13"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F45" s="15"/>
+      <c r="G45" s="18">
+        <f>SUM(G5:G44)</f>
+        <v>44.85</v>
+      </c>
+      <c r="H45" s="18">
+        <f>SUM(H5:H44)</f>
+        <v>21</v>
+      </c>
+      <c r="I45" s="18">
+        <f t="shared" si="0"/>
+        <v>-23.85</v>
+      </c>
+      <c r="J45" s="19"/>
+      <c r="K45" s="46"/>
+    </row>
+    <row r="46" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="69" t="s">
+        <v>19</v>
+      </c>
+      <c r="B46" s="66"/>
+      <c r="C46" s="66"/>
+      <c r="D46" s="66"/>
+      <c r="E46" s="66"/>
+      <c r="F46" s="66"/>
+      <c r="G46" s="66"/>
+      <c r="H46" s="66"/>
+      <c r="I46" s="66"/>
+      <c r="J46" s="66"/>
+      <c r="K46" s="67"/>
     </row>
     <row r="47" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A47" s="47"/>
-      <c r="B47" s="38"/>
-      <c r="C47" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D47" s="38"/>
-      <c r="E47" s="40"/>
-      <c r="F47" s="40"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="41"/>
-      <c r="I47" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J47" s="45"/>
-      <c r="K47" s="43"/>
-    </row>
-    <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A48" s="47"/>
-      <c r="B48" s="38"/>
-      <c r="C48" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D48" s="38"/>
-      <c r="E48" s="40"/>
-      <c r="F48" s="40"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="41"/>
-      <c r="I48" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J48" s="45"/>
-      <c r="K48" s="43"/>
+      <c r="A47" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="C47" s="54"/>
+      <c r="D47" s="54"/>
+      <c r="E47" s="54"/>
+      <c r="F47" s="54"/>
+      <c r="G47" s="54"/>
+      <c r="H47" s="54"/>
+      <c r="I47" s="54"/>
+      <c r="J47" s="54"/>
+      <c r="K47" s="55"/>
+    </row>
+    <row r="48" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B48" s="70" t="s">
+        <v>20</v>
+      </c>
+      <c r="C48" s="54"/>
+      <c r="D48" s="54"/>
+      <c r="E48" s="54"/>
+      <c r="F48" s="54"/>
+      <c r="G48" s="54"/>
+      <c r="H48" s="54"/>
+      <c r="I48" s="54"/>
+      <c r="J48" s="54"/>
+      <c r="K48" s="55"/>
     </row>
     <row r="49" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A49" s="47"/>
@@ -2729,7 +2944,7 @@
       <c r="G49" s="41"/>
       <c r="H49" s="41"/>
       <c r="I49" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="I49:I59" si="1">H49-G49</f>
         <v>0</v>
       </c>
       <c r="J49" s="45"/>
@@ -2772,80 +2987,79 @@
       <c r="K51" s="43"/>
     </row>
     <row r="52" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A52" s="13"/>
-      <c r="B52" s="15"/>
-      <c r="C52" s="15"/>
-      <c r="D52" s="15"/>
-      <c r="E52" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F52" s="15"/>
-      <c r="G52" s="18">
-        <f t="shared" ref="G52:H52" si="2">SUM(G40:G51)</f>
-        <v>0</v>
-      </c>
-      <c r="H52" s="18">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I52" s="18">
+      <c r="A52" s="47"/>
+      <c r="B52" s="38"/>
+      <c r="C52" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D52" s="38"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="40"/>
+      <c r="G52" s="41"/>
+      <c r="H52" s="41"/>
+      <c r="I52" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J52" s="19"/>
-      <c r="K52" s="46"/>
-    </row>
-    <row r="53" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="65" t="s">
-        <v>21</v>
-      </c>
-      <c r="B53" s="61"/>
-      <c r="C53" s="61"/>
-      <c r="D53" s="61"/>
-      <c r="E53" s="61"/>
-      <c r="F53" s="61"/>
-      <c r="G53" s="61"/>
-      <c r="H53" s="61"/>
-      <c r="I53" s="61"/>
-      <c r="J53" s="61"/>
-      <c r="K53" s="62"/>
+      <c r="J52" s="45"/>
+      <c r="K52" s="43"/>
+    </row>
+    <row r="53" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A53" s="47"/>
+      <c r="B53" s="38"/>
+      <c r="C53" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D53" s="38"/>
+      <c r="E53" s="40"/>
+      <c r="F53" s="40"/>
+      <c r="G53" s="41"/>
+      <c r="H53" s="41"/>
+      <c r="I53" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J53" s="45"/>
+      <c r="K53" s="43"/>
     </row>
     <row r="54" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A54" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B54" s="66" t="s">
-        <v>13</v>
-      </c>
-      <c r="C54" s="61"/>
-      <c r="D54" s="61"/>
-      <c r="E54" s="61"/>
-      <c r="F54" s="61"/>
-      <c r="G54" s="61"/>
-      <c r="H54" s="61"/>
-      <c r="I54" s="61"/>
-      <c r="J54" s="61"/>
-      <c r="K54" s="62"/>
-    </row>
-    <row r="55" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B55" s="66" t="s">
-        <v>15</v>
-      </c>
-      <c r="C55" s="61"/>
-      <c r="D55" s="61"/>
-      <c r="E55" s="61"/>
-      <c r="F55" s="61"/>
-      <c r="G55" s="61"/>
-      <c r="H55" s="61"/>
-      <c r="I55" s="61"/>
-      <c r="J55" s="61"/>
-      <c r="K55" s="62"/>
+      <c r="A54" s="47"/>
+      <c r="B54" s="38"/>
+      <c r="C54" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D54" s="38"/>
+      <c r="E54" s="40"/>
+      <c r="F54" s="40"/>
+      <c r="G54" s="41"/>
+      <c r="H54" s="41"/>
+      <c r="I54" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J54" s="45"/>
+      <c r="K54" s="43"/>
+    </row>
+    <row r="55" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A55" s="47"/>
+      <c r="B55" s="38"/>
+      <c r="C55" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D55" s="38"/>
+      <c r="E55" s="40"/>
+      <c r="F55" s="40"/>
+      <c r="G55" s="41"/>
+      <c r="H55" s="41"/>
+      <c r="I55" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J55" s="45"/>
+      <c r="K55" s="43"/>
     </row>
     <row r="56" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A56" s="37"/>
+      <c r="A56" s="47"/>
       <c r="B56" s="38"/>
       <c r="C56" s="39" t="s">
         <v>17</v>
@@ -2856,14 +3070,14 @@
       <c r="G56" s="41"/>
       <c r="H56" s="41"/>
       <c r="I56" s="41">
-        <f t="shared" ref="I56:I66" si="3">H56-G56</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J56" s="45"/>
       <c r="K56" s="43"/>
     </row>
     <row r="57" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A57" s="37"/>
+      <c r="A57" s="47"/>
       <c r="B57" s="38"/>
       <c r="C57" s="39" t="s">
         <v>17</v>
@@ -2874,14 +3088,14 @@
       <c r="G57" s="41"/>
       <c r="H57" s="41"/>
       <c r="I57" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J57" s="45"/>
       <c r="K57" s="43"/>
     </row>
     <row r="58" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A58" s="37"/>
+      <c r="A58" s="47"/>
       <c r="B58" s="38"/>
       <c r="C58" s="39" t="s">
         <v>17</v>
@@ -2892,83 +3106,84 @@
       <c r="G58" s="41"/>
       <c r="H58" s="41"/>
       <c r="I58" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J58" s="45"/>
       <c r="K58" s="43"/>
     </row>
     <row r="59" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A59" s="37"/>
-      <c r="B59" s="38"/>
-      <c r="C59" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D59" s="38"/>
-      <c r="E59" s="40"/>
-      <c r="F59" s="40"/>
-      <c r="G59" s="41"/>
-      <c r="H59" s="41"/>
-      <c r="I59" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J59" s="45"/>
-      <c r="K59" s="43"/>
-    </row>
-    <row r="60" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A60" s="37"/>
-      <c r="B60" s="38"/>
-      <c r="C60" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D60" s="38"/>
-      <c r="E60" s="40"/>
-      <c r="F60" s="40"/>
-      <c r="G60" s="41"/>
-      <c r="H60" s="41"/>
-      <c r="I60" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J60" s="45"/>
-      <c r="K60" s="43"/>
+      <c r="A59" s="13"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F59" s="15"/>
+      <c r="G59" s="18">
+        <f t="shared" ref="G59:H59" si="2">SUM(G47:G58)</f>
+        <v>0</v>
+      </c>
+      <c r="H59" s="18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I59" s="18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J59" s="19"/>
+      <c r="K59" s="46"/>
+    </row>
+    <row r="60" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="71" t="s">
+        <v>21</v>
+      </c>
+      <c r="B60" s="54"/>
+      <c r="C60" s="54"/>
+      <c r="D60" s="54"/>
+      <c r="E60" s="54"/>
+      <c r="F60" s="54"/>
+      <c r="G60" s="54"/>
+      <c r="H60" s="54"/>
+      <c r="I60" s="54"/>
+      <c r="J60" s="54"/>
+      <c r="K60" s="55"/>
     </row>
     <row r="61" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A61" s="37"/>
-      <c r="B61" s="38"/>
-      <c r="C61" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D61" s="38"/>
-      <c r="E61" s="40"/>
-      <c r="F61" s="40"/>
-      <c r="G61" s="41"/>
-      <c r="H61" s="41"/>
-      <c r="I61" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J61" s="45"/>
-      <c r="K61" s="43"/>
-    </row>
-    <row r="62" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A62" s="37"/>
-      <c r="B62" s="38"/>
-      <c r="C62" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D62" s="38"/>
-      <c r="E62" s="40"/>
-      <c r="F62" s="40"/>
-      <c r="G62" s="41"/>
-      <c r="H62" s="41"/>
-      <c r="I62" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J62" s="45"/>
-      <c r="K62" s="43"/>
+      <c r="A61" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B61" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="C61" s="54"/>
+      <c r="D61" s="54"/>
+      <c r="E61" s="54"/>
+      <c r="F61" s="54"/>
+      <c r="G61" s="54"/>
+      <c r="H61" s="54"/>
+      <c r="I61" s="54"/>
+      <c r="J61" s="54"/>
+      <c r="K61" s="55"/>
+    </row>
+    <row r="62" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B62" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="C62" s="54"/>
+      <c r="D62" s="54"/>
+      <c r="E62" s="54"/>
+      <c r="F62" s="54"/>
+      <c r="G62" s="54"/>
+      <c r="H62" s="54"/>
+      <c r="I62" s="54"/>
+      <c r="J62" s="54"/>
+      <c r="K62" s="55"/>
     </row>
     <row r="63" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A63" s="37"/>
@@ -2982,7 +3197,7 @@
       <c r="G63" s="41"/>
       <c r="H63" s="41"/>
       <c r="I63" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="I63:I73" si="3">H63-G63</f>
         <v>0</v>
       </c>
       <c r="J63" s="45"/>
@@ -3025,77 +3240,76 @@
       <c r="K65" s="43"/>
     </row>
     <row r="66" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A66" s="13"/>
-      <c r="B66" s="15"/>
-      <c r="C66" s="15"/>
-      <c r="D66" s="15"/>
-      <c r="E66" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F66" s="15"/>
-      <c r="G66" s="18">
-        <f t="shared" ref="G66:H66" si="4">SUM(G56:G65)</f>
-        <v>0</v>
-      </c>
-      <c r="H66" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I66" s="18">
+      <c r="A66" s="37"/>
+      <c r="B66" s="38"/>
+      <c r="C66" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D66" s="38"/>
+      <c r="E66" s="40"/>
+      <c r="F66" s="40"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="41"/>
+      <c r="I66" s="41">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J66" s="19"/>
-      <c r="K66" s="46"/>
-    </row>
-    <row r="67" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="67" t="s">
-        <v>22</v>
-      </c>
-      <c r="B67" s="61"/>
-      <c r="C67" s="61"/>
-      <c r="D67" s="61"/>
-      <c r="E67" s="61"/>
-      <c r="F67" s="61"/>
-      <c r="G67" s="61"/>
-      <c r="H67" s="61"/>
-      <c r="I67" s="61"/>
-      <c r="J67" s="61"/>
-      <c r="K67" s="62"/>
+      <c r="J66" s="45"/>
+      <c r="K66" s="43"/>
+    </row>
+    <row r="67" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A67" s="37"/>
+      <c r="B67" s="38"/>
+      <c r="C67" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D67" s="38"/>
+      <c r="E67" s="40"/>
+      <c r="F67" s="40"/>
+      <c r="G67" s="41"/>
+      <c r="H67" s="41"/>
+      <c r="I67" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J67" s="45"/>
+      <c r="K67" s="43"/>
     </row>
     <row r="68" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A68" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B68" s="69" t="s">
-        <v>13</v>
-      </c>
-      <c r="C68" s="61"/>
-      <c r="D68" s="61"/>
-      <c r="E68" s="61"/>
-      <c r="F68" s="61"/>
-      <c r="G68" s="61"/>
-      <c r="H68" s="61"/>
-      <c r="I68" s="61"/>
-      <c r="J68" s="61"/>
-      <c r="K68" s="62"/>
-    </row>
-    <row r="69" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B69" s="69" t="s">
-        <v>15</v>
-      </c>
-      <c r="C69" s="61"/>
-      <c r="D69" s="61"/>
-      <c r="E69" s="61"/>
-      <c r="F69" s="61"/>
-      <c r="G69" s="61"/>
-      <c r="H69" s="61"/>
-      <c r="I69" s="61"/>
-      <c r="J69" s="61"/>
-      <c r="K69" s="62"/>
+      <c r="A68" s="37"/>
+      <c r="B68" s="38"/>
+      <c r="C68" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D68" s="38"/>
+      <c r="E68" s="40"/>
+      <c r="F68" s="40"/>
+      <c r="G68" s="41"/>
+      <c r="H68" s="41"/>
+      <c r="I68" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J68" s="45"/>
+      <c r="K68" s="43"/>
+    </row>
+    <row r="69" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A69" s="37"/>
+      <c r="B69" s="38"/>
+      <c r="C69" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D69" s="38"/>
+      <c r="E69" s="40"/>
+      <c r="F69" s="40"/>
+      <c r="G69" s="41"/>
+      <c r="H69" s="41"/>
+      <c r="I69" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J69" s="45"/>
+      <c r="K69" s="43"/>
     </row>
     <row r="70" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A70" s="37"/>
@@ -3109,7 +3323,7 @@
       <c r="G70" s="41"/>
       <c r="H70" s="41"/>
       <c r="I70" s="41">
-        <f t="shared" ref="I70:I80" si="5">H70-G70</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J70" s="45"/>
@@ -3127,7 +3341,7 @@
       <c r="G71" s="41"/>
       <c r="H71" s="41"/>
       <c r="I71" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J71" s="45"/>
@@ -3145,83 +3359,84 @@
       <c r="G72" s="41"/>
       <c r="H72" s="41"/>
       <c r="I72" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J72" s="45"/>
       <c r="K72" s="43"/>
     </row>
     <row r="73" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A73" s="37"/>
-      <c r="B73" s="38"/>
-      <c r="C73" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D73" s="38"/>
-      <c r="E73" s="40"/>
-      <c r="F73" s="40"/>
-      <c r="G73" s="41"/>
-      <c r="H73" s="41"/>
-      <c r="I73" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J73" s="45"/>
-      <c r="K73" s="43"/>
-    </row>
-    <row r="74" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A74" s="37"/>
-      <c r="B74" s="38"/>
-      <c r="C74" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D74" s="38"/>
-      <c r="E74" s="40"/>
-      <c r="F74" s="40"/>
-      <c r="G74" s="41"/>
-      <c r="H74" s="41"/>
-      <c r="I74" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J74" s="45"/>
-      <c r="K74" s="43"/>
+      <c r="A73" s="13"/>
+      <c r="B73" s="15"/>
+      <c r="C73" s="15"/>
+      <c r="D73" s="15"/>
+      <c r="E73" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F73" s="15"/>
+      <c r="G73" s="18">
+        <f t="shared" ref="G73:H73" si="4">SUM(G63:G72)</f>
+        <v>0</v>
+      </c>
+      <c r="H73" s="18">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I73" s="18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J73" s="19"/>
+      <c r="K73" s="46"/>
+    </row>
+    <row r="74" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="73" t="s">
+        <v>22</v>
+      </c>
+      <c r="B74" s="54"/>
+      <c r="C74" s="54"/>
+      <c r="D74" s="54"/>
+      <c r="E74" s="54"/>
+      <c r="F74" s="54"/>
+      <c r="G74" s="54"/>
+      <c r="H74" s="54"/>
+      <c r="I74" s="54"/>
+      <c r="J74" s="54"/>
+      <c r="K74" s="55"/>
     </row>
     <row r="75" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A75" s="37"/>
-      <c r="B75" s="38"/>
-      <c r="C75" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D75" s="38"/>
-      <c r="E75" s="40"/>
-      <c r="F75" s="40"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="41"/>
-      <c r="I75" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J75" s="45"/>
-      <c r="K75" s="43"/>
-    </row>
-    <row r="76" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A76" s="37"/>
-      <c r="B76" s="38"/>
-      <c r="C76" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D76" s="38"/>
-      <c r="E76" s="40"/>
-      <c r="F76" s="40"/>
-      <c r="G76" s="41"/>
-      <c r="H76" s="41"/>
-      <c r="I76" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J76" s="45"/>
-      <c r="K76" s="43"/>
+      <c r="A75" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B75" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C75" s="54"/>
+      <c r="D75" s="54"/>
+      <c r="E75" s="54"/>
+      <c r="F75" s="54"/>
+      <c r="G75" s="54"/>
+      <c r="H75" s="54"/>
+      <c r="I75" s="54"/>
+      <c r="J75" s="54"/>
+      <c r="K75" s="55"/>
+    </row>
+    <row r="76" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B76" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C76" s="54"/>
+      <c r="D76" s="54"/>
+      <c r="E76" s="54"/>
+      <c r="F76" s="54"/>
+      <c r="G76" s="54"/>
+      <c r="H76" s="54"/>
+      <c r="I76" s="54"/>
+      <c r="J76" s="54"/>
+      <c r="K76" s="55"/>
     </row>
     <row r="77" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A77" s="37"/>
@@ -3235,7 +3450,7 @@
       <c r="G77" s="41"/>
       <c r="H77" s="41"/>
       <c r="I77" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I77:I87" si="5">H77-G77</f>
         <v>0</v>
       </c>
       <c r="J77" s="45"/>
@@ -3278,77 +3493,76 @@
       <c r="K79" s="43"/>
     </row>
     <row r="80" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A80" s="13"/>
-      <c r="B80" s="15"/>
-      <c r="C80" s="15"/>
-      <c r="D80" s="15"/>
-      <c r="E80" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F80" s="15"/>
-      <c r="G80" s="18">
-        <f t="shared" ref="G80:H80" si="6">SUM(G70:G79)</f>
-        <v>0</v>
-      </c>
-      <c r="H80" s="18">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="I80" s="18">
+      <c r="A80" s="37"/>
+      <c r="B80" s="38"/>
+      <c r="C80" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D80" s="38"/>
+      <c r="E80" s="40"/>
+      <c r="F80" s="40"/>
+      <c r="G80" s="41"/>
+      <c r="H80" s="41"/>
+      <c r="I80" s="41">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J80" s="19"/>
-      <c r="K80" s="46"/>
-    </row>
-    <row r="81" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="72" t="s">
-        <v>23</v>
-      </c>
-      <c r="B81" s="61"/>
-      <c r="C81" s="61"/>
-      <c r="D81" s="61"/>
-      <c r="E81" s="61"/>
-      <c r="F81" s="61"/>
-      <c r="G81" s="61"/>
-      <c r="H81" s="61"/>
-      <c r="I81" s="61"/>
-      <c r="J81" s="61"/>
-      <c r="K81" s="62"/>
+      <c r="J80" s="45"/>
+      <c r="K80" s="43"/>
+    </row>
+    <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A81" s="37"/>
+      <c r="B81" s="38"/>
+      <c r="C81" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D81" s="38"/>
+      <c r="E81" s="40"/>
+      <c r="F81" s="40"/>
+      <c r="G81" s="41"/>
+      <c r="H81" s="41"/>
+      <c r="I81" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J81" s="45"/>
+      <c r="K81" s="43"/>
     </row>
     <row r="82" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A82" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B82" s="73" t="s">
-        <v>13</v>
-      </c>
-      <c r="C82" s="61"/>
-      <c r="D82" s="61"/>
-      <c r="E82" s="61"/>
-      <c r="F82" s="61"/>
-      <c r="G82" s="61"/>
-      <c r="H82" s="61"/>
-      <c r="I82" s="61"/>
-      <c r="J82" s="61"/>
-      <c r="K82" s="62"/>
-    </row>
-    <row r="83" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="B83" s="73" t="s">
-        <v>15</v>
-      </c>
-      <c r="C83" s="61"/>
-      <c r="D83" s="61"/>
-      <c r="E83" s="61"/>
-      <c r="F83" s="61"/>
-      <c r="G83" s="61"/>
-      <c r="H83" s="61"/>
-      <c r="I83" s="61"/>
-      <c r="J83" s="61"/>
-      <c r="K83" s="62"/>
+      <c r="A82" s="37"/>
+      <c r="B82" s="38"/>
+      <c r="C82" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D82" s="38"/>
+      <c r="E82" s="40"/>
+      <c r="F82" s="40"/>
+      <c r="G82" s="41"/>
+      <c r="H82" s="41"/>
+      <c r="I82" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J82" s="45"/>
+      <c r="K82" s="43"/>
+    </row>
+    <row r="83" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A83" s="37"/>
+      <c r="B83" s="38"/>
+      <c r="C83" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D83" s="38"/>
+      <c r="E83" s="40"/>
+      <c r="F83" s="40"/>
+      <c r="G83" s="41"/>
+      <c r="H83" s="41"/>
+      <c r="I83" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J83" s="45"/>
+      <c r="K83" s="43"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="37"/>
@@ -3362,7 +3576,7 @@
       <c r="G84" s="41"/>
       <c r="H84" s="41"/>
       <c r="I84" s="41">
-        <f t="shared" ref="I84:I94" si="7">H84-G84</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J84" s="45"/>
@@ -3380,7 +3594,7 @@
       <c r="G85" s="41"/>
       <c r="H85" s="41"/>
       <c r="I85" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J85" s="45"/>
@@ -3398,83 +3612,84 @@
       <c r="G86" s="41"/>
       <c r="H86" s="41"/>
       <c r="I86" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J86" s="45"/>
       <c r="K86" s="43"/>
     </row>
     <row r="87" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A87" s="37"/>
-      <c r="B87" s="38"/>
-      <c r="C87" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D87" s="38"/>
-      <c r="E87" s="40"/>
-      <c r="F87" s="40"/>
-      <c r="G87" s="41"/>
-      <c r="H87" s="41"/>
-      <c r="I87" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J87" s="45"/>
-      <c r="K87" s="43"/>
-    </row>
-    <row r="88" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A88" s="37"/>
-      <c r="B88" s="38"/>
-      <c r="C88" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D88" s="38"/>
-      <c r="E88" s="40"/>
-      <c r="F88" s="40"/>
-      <c r="G88" s="41"/>
-      <c r="H88" s="41"/>
-      <c r="I88" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J88" s="45"/>
-      <c r="K88" s="43"/>
+      <c r="A87" s="13"/>
+      <c r="B87" s="15"/>
+      <c r="C87" s="15"/>
+      <c r="D87" s="15"/>
+      <c r="E87" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F87" s="15"/>
+      <c r="G87" s="18">
+        <f t="shared" ref="G87:H87" si="6">SUM(G77:G86)</f>
+        <v>0</v>
+      </c>
+      <c r="H87" s="18">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I87" s="18">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J87" s="19"/>
+      <c r="K87" s="46"/>
+    </row>
+    <row r="88" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="B88" s="54"/>
+      <c r="C88" s="54"/>
+      <c r="D88" s="54"/>
+      <c r="E88" s="54"/>
+      <c r="F88" s="54"/>
+      <c r="G88" s="54"/>
+      <c r="H88" s="54"/>
+      <c r="I88" s="54"/>
+      <c r="J88" s="54"/>
+      <c r="K88" s="55"/>
     </row>
     <row r="89" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A89" s="37"/>
-      <c r="B89" s="38"/>
-      <c r="C89" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D89" s="38"/>
-      <c r="E89" s="40"/>
-      <c r="F89" s="40"/>
-      <c r="G89" s="41"/>
-      <c r="H89" s="41"/>
-      <c r="I89" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J89" s="45"/>
-      <c r="K89" s="43"/>
-    </row>
-    <row r="90" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A90" s="37"/>
-      <c r="B90" s="38"/>
-      <c r="C90" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D90" s="38"/>
-      <c r="E90" s="40"/>
-      <c r="F90" s="40"/>
-      <c r="G90" s="41"/>
-      <c r="H90" s="41"/>
-      <c r="I90" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J90" s="45"/>
-      <c r="K90" s="43"/>
+      <c r="A89" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B89" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C89" s="54"/>
+      <c r="D89" s="54"/>
+      <c r="E89" s="54"/>
+      <c r="F89" s="54"/>
+      <c r="G89" s="54"/>
+      <c r="H89" s="54"/>
+      <c r="I89" s="54"/>
+      <c r="J89" s="54"/>
+      <c r="K89" s="55"/>
+    </row>
+    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B90" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C90" s="54"/>
+      <c r="D90" s="54"/>
+      <c r="E90" s="54"/>
+      <c r="F90" s="54"/>
+      <c r="G90" s="54"/>
+      <c r="H90" s="54"/>
+      <c r="I90" s="54"/>
+      <c r="J90" s="54"/>
+      <c r="K90" s="55"/>
     </row>
     <row r="91" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A91" s="37"/>
@@ -3488,7 +3703,7 @@
       <c r="G91" s="41"/>
       <c r="H91" s="41"/>
       <c r="I91" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="I91:I101" si="7">H91-G91</f>
         <v>0</v>
       </c>
       <c r="J91" s="45"/>
@@ -3531,77 +3746,76 @@
       <c r="K93" s="43"/>
     </row>
     <row r="94" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A94" s="13"/>
-      <c r="B94" s="15"/>
-      <c r="C94" s="15"/>
-      <c r="D94" s="15"/>
-      <c r="E94" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F94" s="15"/>
-      <c r="G94" s="18">
-        <f t="shared" ref="G94:H94" si="8">SUM(G84:G93)</f>
-        <v>0</v>
-      </c>
-      <c r="H94" s="18">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I94" s="18">
+      <c r="A94" s="37"/>
+      <c r="B94" s="38"/>
+      <c r="C94" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D94" s="38"/>
+      <c r="E94" s="40"/>
+      <c r="F94" s="40"/>
+      <c r="G94" s="41"/>
+      <c r="H94" s="41"/>
+      <c r="I94" s="41">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J94" s="19"/>
-      <c r="K94" s="46"/>
-    </row>
-    <row r="95" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="74" t="s">
-        <v>24</v>
-      </c>
-      <c r="B95" s="61"/>
-      <c r="C95" s="61"/>
-      <c r="D95" s="61"/>
-      <c r="E95" s="61"/>
-      <c r="F95" s="61"/>
-      <c r="G95" s="61"/>
-      <c r="H95" s="61"/>
-      <c r="I95" s="61"/>
-      <c r="J95" s="61"/>
-      <c r="K95" s="62"/>
+      <c r="J94" s="45"/>
+      <c r="K94" s="43"/>
+    </row>
+    <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A95" s="37"/>
+      <c r="B95" s="38"/>
+      <c r="C95" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D95" s="38"/>
+      <c r="E95" s="40"/>
+      <c r="F95" s="40"/>
+      <c r="G95" s="41"/>
+      <c r="H95" s="41"/>
+      <c r="I95" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J95" s="45"/>
+      <c r="K95" s="43"/>
     </row>
     <row r="96" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A96" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B96" s="70" t="s">
-        <v>13</v>
-      </c>
-      <c r="C96" s="61"/>
-      <c r="D96" s="61"/>
-      <c r="E96" s="61"/>
-      <c r="F96" s="61"/>
-      <c r="G96" s="61"/>
-      <c r="H96" s="61"/>
-      <c r="I96" s="61"/>
-      <c r="J96" s="61"/>
-      <c r="K96" s="62"/>
-    </row>
-    <row r="97" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B97" s="70" t="s">
-        <v>15</v>
-      </c>
-      <c r="C97" s="61"/>
-      <c r="D97" s="61"/>
-      <c r="E97" s="61"/>
-      <c r="F97" s="61"/>
-      <c r="G97" s="61"/>
-      <c r="H97" s="61"/>
-      <c r="I97" s="61"/>
-      <c r="J97" s="61"/>
-      <c r="K97" s="62"/>
+      <c r="A96" s="37"/>
+      <c r="B96" s="38"/>
+      <c r="C96" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D96" s="38"/>
+      <c r="E96" s="40"/>
+      <c r="F96" s="40"/>
+      <c r="G96" s="41"/>
+      <c r="H96" s="41"/>
+      <c r="I96" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J96" s="45"/>
+      <c r="K96" s="43"/>
+    </row>
+    <row r="97" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A97" s="37"/>
+      <c r="B97" s="38"/>
+      <c r="C97" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D97" s="38"/>
+      <c r="E97" s="40"/>
+      <c r="F97" s="40"/>
+      <c r="G97" s="41"/>
+      <c r="H97" s="41"/>
+      <c r="I97" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J97" s="45"/>
+      <c r="K97" s="43"/>
     </row>
     <row r="98" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A98" s="37"/>
@@ -3615,7 +3829,7 @@
       <c r="G98" s="41"/>
       <c r="H98" s="41"/>
       <c r="I98" s="41">
-        <f t="shared" ref="I98:I108" si="9">H98-G98</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J98" s="45"/>
@@ -3633,7 +3847,7 @@
       <c r="G99" s="41"/>
       <c r="H99" s="41"/>
       <c r="I99" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J99" s="45"/>
@@ -3651,85 +3865,84 @@
       <c r="G100" s="41"/>
       <c r="H100" s="41"/>
       <c r="I100" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J100" s="45"/>
-      <c r="K100" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K100" s="43"/>
     </row>
     <row r="101" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A101" s="37"/>
-      <c r="B101" s="38"/>
-      <c r="C101" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D101" s="38"/>
-      <c r="E101" s="40"/>
-      <c r="F101" s="40"/>
-      <c r="G101" s="41"/>
-      <c r="H101" s="41"/>
-      <c r="I101" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J101" s="45"/>
-      <c r="K101" s="43"/>
-    </row>
-    <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A102" s="37"/>
-      <c r="B102" s="38"/>
-      <c r="C102" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D102" s="38"/>
-      <c r="E102" s="40"/>
-      <c r="F102" s="40"/>
-      <c r="G102" s="41"/>
-      <c r="H102" s="41"/>
-      <c r="I102" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J102" s="45"/>
-      <c r="K102" s="43"/>
+      <c r="A101" s="13"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="15"/>
+      <c r="D101" s="15"/>
+      <c r="E101" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F101" s="15"/>
+      <c r="G101" s="18">
+        <f t="shared" ref="G101:H101" si="8">SUM(G91:G100)</f>
+        <v>0</v>
+      </c>
+      <c r="H101" s="18">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I101" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J101" s="19"/>
+      <c r="K101" s="46"/>
+    </row>
+    <row r="102" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="B102" s="54"/>
+      <c r="C102" s="54"/>
+      <c r="D102" s="54"/>
+      <c r="E102" s="54"/>
+      <c r="F102" s="54"/>
+      <c r="G102" s="54"/>
+      <c r="H102" s="54"/>
+      <c r="I102" s="54"/>
+      <c r="J102" s="54"/>
+      <c r="K102" s="55"/>
     </row>
     <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A103" s="37"/>
-      <c r="B103" s="38"/>
-      <c r="C103" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D103" s="38"/>
-      <c r="E103" s="40"/>
-      <c r="F103" s="40"/>
-      <c r="G103" s="41"/>
-      <c r="H103" s="41"/>
-      <c r="I103" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J103" s="45"/>
-      <c r="K103" s="43"/>
-    </row>
-    <row r="104" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A104" s="37"/>
-      <c r="B104" s="38"/>
-      <c r="C104" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D104" s="38"/>
-      <c r="E104" s="40"/>
-      <c r="F104" s="40"/>
-      <c r="G104" s="41"/>
-      <c r="H104" s="41"/>
-      <c r="I104" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J104" s="45"/>
-      <c r="K104" s="43"/>
+      <c r="A103" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B103" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="C103" s="54"/>
+      <c r="D103" s="54"/>
+      <c r="E103" s="54"/>
+      <c r="F103" s="54"/>
+      <c r="G103" s="54"/>
+      <c r="H103" s="54"/>
+      <c r="I103" s="54"/>
+      <c r="J103" s="54"/>
+      <c r="K103" s="55"/>
+    </row>
+    <row r="104" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B104" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="C104" s="54"/>
+      <c r="D104" s="54"/>
+      <c r="E104" s="54"/>
+      <c r="F104" s="54"/>
+      <c r="G104" s="54"/>
+      <c r="H104" s="54"/>
+      <c r="I104" s="54"/>
+      <c r="J104" s="54"/>
+      <c r="K104" s="55"/>
     </row>
     <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A105" s="37"/>
@@ -3743,7 +3956,7 @@
       <c r="G105" s="41"/>
       <c r="H105" s="41"/>
       <c r="I105" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I105:I115" si="9">H105-G105</f>
         <v>0</v>
       </c>
       <c r="J105" s="45"/>
@@ -3783,80 +3996,81 @@
         <v>0</v>
       </c>
       <c r="J107" s="45"/>
-      <c r="K107" s="43"/>
+      <c r="K107" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="108" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A108" s="13"/>
-      <c r="B108" s="15"/>
-      <c r="C108" s="15"/>
-      <c r="D108" s="15"/>
-      <c r="E108" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F108" s="15"/>
-      <c r="G108" s="18">
-        <f t="shared" ref="G108:H108" si="10">SUM(G98:G107)</f>
-        <v>0</v>
-      </c>
-      <c r="H108" s="18">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="I108" s="18">
+      <c r="A108" s="37"/>
+      <c r="B108" s="38"/>
+      <c r="C108" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D108" s="38"/>
+      <c r="E108" s="40"/>
+      <c r="F108" s="40"/>
+      <c r="G108" s="41"/>
+      <c r="H108" s="41"/>
+      <c r="I108" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J108" s="19"/>
-      <c r="K108" s="46"/>
-    </row>
-    <row r="109" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="71" t="s">
-        <v>26</v>
-      </c>
-      <c r="B109" s="61"/>
-      <c r="C109" s="61"/>
-      <c r="D109" s="61"/>
-      <c r="E109" s="61"/>
-      <c r="F109" s="61"/>
-      <c r="G109" s="61"/>
-      <c r="H109" s="61"/>
-      <c r="I109" s="61"/>
-      <c r="J109" s="61"/>
-      <c r="K109" s="62"/>
+      <c r="J108" s="45"/>
+      <c r="K108" s="43"/>
+    </row>
+    <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A109" s="37"/>
+      <c r="B109" s="38"/>
+      <c r="C109" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D109" s="38"/>
+      <c r="E109" s="40"/>
+      <c r="F109" s="40"/>
+      <c r="G109" s="41"/>
+      <c r="H109" s="41"/>
+      <c r="I109" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J109" s="45"/>
+      <c r="K109" s="43"/>
     </row>
     <row r="110" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A110" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B110" s="68" t="s">
-        <v>13</v>
-      </c>
-      <c r="C110" s="61"/>
-      <c r="D110" s="61"/>
-      <c r="E110" s="61"/>
-      <c r="F110" s="61"/>
-      <c r="G110" s="61"/>
-      <c r="H110" s="61"/>
-      <c r="I110" s="61"/>
-      <c r="J110" s="61"/>
-      <c r="K110" s="62"/>
-    </row>
-    <row r="111" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B111" s="68" t="s">
-        <v>15</v>
-      </c>
-      <c r="C111" s="61"/>
-      <c r="D111" s="61"/>
-      <c r="E111" s="61"/>
-      <c r="F111" s="61"/>
-      <c r="G111" s="61"/>
-      <c r="H111" s="61"/>
-      <c r="I111" s="61"/>
-      <c r="J111" s="61"/>
-      <c r="K111" s="62"/>
+      <c r="A110" s="37"/>
+      <c r="B110" s="38"/>
+      <c r="C110" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D110" s="38"/>
+      <c r="E110" s="40"/>
+      <c r="F110" s="40"/>
+      <c r="G110" s="41"/>
+      <c r="H110" s="41"/>
+      <c r="I110" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J110" s="45"/>
+      <c r="K110" s="43"/>
+    </row>
+    <row r="111" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A111" s="37"/>
+      <c r="B111" s="38"/>
+      <c r="C111" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D111" s="38"/>
+      <c r="E111" s="40"/>
+      <c r="F111" s="40"/>
+      <c r="G111" s="41"/>
+      <c r="H111" s="41"/>
+      <c r="I111" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J111" s="45"/>
+      <c r="K111" s="43"/>
     </row>
     <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A112" s="37"/>
@@ -3870,7 +4084,7 @@
       <c r="G112" s="41"/>
       <c r="H112" s="41"/>
       <c r="I112" s="41">
-        <f t="shared" ref="I112:I122" si="11">H112-G112</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J112" s="45"/>
@@ -3888,7 +4102,7 @@
       <c r="G113" s="41"/>
       <c r="H113" s="41"/>
       <c r="I113" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J113" s="45"/>
@@ -3906,83 +4120,84 @@
       <c r="G114" s="41"/>
       <c r="H114" s="41"/>
       <c r="I114" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J114" s="45"/>
       <c r="K114" s="43"/>
     </row>
     <row r="115" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A115" s="37"/>
-      <c r="B115" s="38"/>
-      <c r="C115" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D115" s="38"/>
-      <c r="E115" s="40"/>
-      <c r="F115" s="40"/>
-      <c r="G115" s="41"/>
-      <c r="H115" s="41"/>
-      <c r="I115" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J115" s="45"/>
-      <c r="K115" s="43"/>
-    </row>
-    <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A116" s="37"/>
-      <c r="B116" s="38"/>
-      <c r="C116" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D116" s="38"/>
-      <c r="E116" s="40"/>
-      <c r="F116" s="40"/>
-      <c r="G116" s="41"/>
-      <c r="H116" s="41"/>
-      <c r="I116" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J116" s="45"/>
-      <c r="K116" s="43"/>
+      <c r="A115" s="13"/>
+      <c r="B115" s="15"/>
+      <c r="C115" s="15"/>
+      <c r="D115" s="15"/>
+      <c r="E115" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F115" s="15"/>
+      <c r="G115" s="18">
+        <f t="shared" ref="G115:H115" si="10">SUM(G105:G114)</f>
+        <v>0</v>
+      </c>
+      <c r="H115" s="18">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="I115" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J115" s="19"/>
+      <c r="K115" s="46"/>
+    </row>
+    <row r="116" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="B116" s="54"/>
+      <c r="C116" s="54"/>
+      <c r="D116" s="54"/>
+      <c r="E116" s="54"/>
+      <c r="F116" s="54"/>
+      <c r="G116" s="54"/>
+      <c r="H116" s="54"/>
+      <c r="I116" s="54"/>
+      <c r="J116" s="54"/>
+      <c r="K116" s="55"/>
     </row>
     <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A117" s="37"/>
-      <c r="B117" s="38"/>
-      <c r="C117" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D117" s="38"/>
-      <c r="E117" s="40"/>
-      <c r="F117" s="40"/>
-      <c r="G117" s="41"/>
-      <c r="H117" s="41"/>
-      <c r="I117" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J117" s="45"/>
-      <c r="K117" s="43"/>
-    </row>
-    <row r="118" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A118" s="37"/>
-      <c r="B118" s="38"/>
-      <c r="C118" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D118" s="38"/>
-      <c r="E118" s="40"/>
-      <c r="F118" s="40"/>
-      <c r="G118" s="41"/>
-      <c r="H118" s="41"/>
-      <c r="I118" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J118" s="45"/>
-      <c r="K118" s="43"/>
+      <c r="A117" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B117" s="74" t="s">
+        <v>13</v>
+      </c>
+      <c r="C117" s="54"/>
+      <c r="D117" s="54"/>
+      <c r="E117" s="54"/>
+      <c r="F117" s="54"/>
+      <c r="G117" s="54"/>
+      <c r="H117" s="54"/>
+      <c r="I117" s="54"/>
+      <c r="J117" s="54"/>
+      <c r="K117" s="55"/>
+    </row>
+    <row r="118" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B118" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="C118" s="54"/>
+      <c r="D118" s="54"/>
+      <c r="E118" s="54"/>
+      <c r="F118" s="54"/>
+      <c r="G118" s="54"/>
+      <c r="H118" s="54"/>
+      <c r="I118" s="54"/>
+      <c r="J118" s="54"/>
+      <c r="K118" s="55"/>
     </row>
     <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A119" s="37"/>
@@ -3996,7 +4211,7 @@
       <c r="G119" s="41"/>
       <c r="H119" s="41"/>
       <c r="I119" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="I119:I129" si="11">H119-G119</f>
         <v>0</v>
       </c>
       <c r="J119" s="45"/>
@@ -4039,77 +4254,76 @@
       <c r="K121" s="43"/>
     </row>
     <row r="122" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A122" s="13"/>
-      <c r="B122" s="15"/>
-      <c r="C122" s="15"/>
-      <c r="D122" s="15"/>
-      <c r="E122" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F122" s="15"/>
-      <c r="G122" s="18">
-        <f t="shared" ref="G122:H122" si="12">SUM(G112:G121)</f>
-        <v>0</v>
-      </c>
-      <c r="H122" s="18">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="I122" s="18">
+      <c r="A122" s="37"/>
+      <c r="B122" s="38"/>
+      <c r="C122" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D122" s="38"/>
+      <c r="E122" s="40"/>
+      <c r="F122" s="40"/>
+      <c r="G122" s="41"/>
+      <c r="H122" s="41"/>
+      <c r="I122" s="41">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J122" s="19"/>
-      <c r="K122" s="46"/>
-    </row>
-    <row r="123" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="53" t="s">
-        <v>27</v>
-      </c>
-      <c r="B123" s="54"/>
-      <c r="C123" s="54"/>
-      <c r="D123" s="54"/>
-      <c r="E123" s="54"/>
-      <c r="F123" s="54"/>
-      <c r="G123" s="54"/>
-      <c r="H123" s="54"/>
-      <c r="I123" s="54"/>
-      <c r="J123" s="54"/>
-      <c r="K123" s="55"/>
+      <c r="J122" s="45"/>
+      <c r="K122" s="43"/>
+    </row>
+    <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A123" s="37"/>
+      <c r="B123" s="38"/>
+      <c r="C123" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D123" s="38"/>
+      <c r="E123" s="40"/>
+      <c r="F123" s="40"/>
+      <c r="G123" s="41"/>
+      <c r="H123" s="41"/>
+      <c r="I123" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J123" s="45"/>
+      <c r="K123" s="43"/>
     </row>
     <row r="124" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A124" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B124" s="56" t="s">
-        <v>13</v>
-      </c>
-      <c r="C124" s="54"/>
-      <c r="D124" s="54"/>
-      <c r="E124" s="54"/>
-      <c r="F124" s="54"/>
-      <c r="G124" s="54"/>
-      <c r="H124" s="54"/>
-      <c r="I124" s="54"/>
-      <c r="J124" s="54"/>
-      <c r="K124" s="55"/>
-    </row>
-    <row r="125" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B125" s="56" t="s">
-        <v>15</v>
-      </c>
-      <c r="C125" s="54"/>
-      <c r="D125" s="54"/>
-      <c r="E125" s="54"/>
-      <c r="F125" s="54"/>
-      <c r="G125" s="54"/>
-      <c r="H125" s="54"/>
-      <c r="I125" s="54"/>
-      <c r="J125" s="54"/>
-      <c r="K125" s="55"/>
+      <c r="A124" s="37"/>
+      <c r="B124" s="38"/>
+      <c r="C124" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D124" s="38"/>
+      <c r="E124" s="40"/>
+      <c r="F124" s="40"/>
+      <c r="G124" s="41"/>
+      <c r="H124" s="41"/>
+      <c r="I124" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J124" s="45"/>
+      <c r="K124" s="43"/>
+    </row>
+    <row r="125" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A125" s="37"/>
+      <c r="B125" s="38"/>
+      <c r="C125" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D125" s="38"/>
+      <c r="E125" s="40"/>
+      <c r="F125" s="40"/>
+      <c r="G125" s="41"/>
+      <c r="H125" s="41"/>
+      <c r="I125" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J125" s="45"/>
+      <c r="K125" s="43"/>
     </row>
     <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A126" s="37"/>
@@ -4123,7 +4337,7 @@
       <c r="G126" s="41"/>
       <c r="H126" s="41"/>
       <c r="I126" s="41">
-        <f t="shared" ref="I126:I136" si="13">H126-G126</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J126" s="45"/>
@@ -4141,7 +4355,7 @@
       <c r="G127" s="41"/>
       <c r="H127" s="41"/>
       <c r="I127" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J127" s="45"/>
@@ -4159,83 +4373,84 @@
       <c r="G128" s="41"/>
       <c r="H128" s="41"/>
       <c r="I128" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J128" s="45"/>
       <c r="K128" s="43"/>
     </row>
     <row r="129" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A129" s="37"/>
-      <c r="B129" s="38"/>
-      <c r="C129" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D129" s="38"/>
-      <c r="E129" s="40"/>
-      <c r="F129" s="40"/>
-      <c r="G129" s="41"/>
-      <c r="H129" s="41"/>
-      <c r="I129" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J129" s="45"/>
-      <c r="K129" s="43"/>
-    </row>
-    <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A130" s="37"/>
-      <c r="B130" s="38"/>
-      <c r="C130" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D130" s="38"/>
-      <c r="E130" s="40"/>
-      <c r="F130" s="40"/>
-      <c r="G130" s="41"/>
-      <c r="H130" s="41"/>
-      <c r="I130" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J130" s="45"/>
-      <c r="K130" s="43"/>
+      <c r="A129" s="13"/>
+      <c r="B129" s="15"/>
+      <c r="C129" s="15"/>
+      <c r="D129" s="15"/>
+      <c r="E129" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F129" s="15"/>
+      <c r="G129" s="18">
+        <f t="shared" ref="G129:H129" si="12">SUM(G119:G128)</f>
+        <v>0</v>
+      </c>
+      <c r="H129" s="18">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="I129" s="18">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J129" s="19"/>
+      <c r="K129" s="46"/>
+    </row>
+    <row r="130" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="61" t="s">
+        <v>27</v>
+      </c>
+      <c r="B130" s="62"/>
+      <c r="C130" s="62"/>
+      <c r="D130" s="62"/>
+      <c r="E130" s="62"/>
+      <c r="F130" s="62"/>
+      <c r="G130" s="62"/>
+      <c r="H130" s="62"/>
+      <c r="I130" s="62"/>
+      <c r="J130" s="62"/>
+      <c r="K130" s="63"/>
     </row>
     <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A131" s="37"/>
-      <c r="B131" s="38"/>
-      <c r="C131" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D131" s="38"/>
-      <c r="E131" s="40"/>
-      <c r="F131" s="40"/>
-      <c r="G131" s="41"/>
-      <c r="H131" s="41"/>
-      <c r="I131" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J131" s="45"/>
-      <c r="K131" s="43"/>
-    </row>
-    <row r="132" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A132" s="37"/>
-      <c r="B132" s="38"/>
-      <c r="C132" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D132" s="38"/>
-      <c r="E132" s="40"/>
-      <c r="F132" s="40"/>
-      <c r="G132" s="41"/>
-      <c r="H132" s="41"/>
-      <c r="I132" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J132" s="45"/>
-      <c r="K132" s="43"/>
+      <c r="A131" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B131" s="64" t="s">
+        <v>13</v>
+      </c>
+      <c r="C131" s="62"/>
+      <c r="D131" s="62"/>
+      <c r="E131" s="62"/>
+      <c r="F131" s="62"/>
+      <c r="G131" s="62"/>
+      <c r="H131" s="62"/>
+      <c r="I131" s="62"/>
+      <c r="J131" s="62"/>
+      <c r="K131" s="63"/>
+    </row>
+    <row r="132" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B132" s="64" t="s">
+        <v>15</v>
+      </c>
+      <c r="C132" s="62"/>
+      <c r="D132" s="62"/>
+      <c r="E132" s="62"/>
+      <c r="F132" s="62"/>
+      <c r="G132" s="62"/>
+      <c r="H132" s="62"/>
+      <c r="I132" s="62"/>
+      <c r="J132" s="62"/>
+      <c r="K132" s="63"/>
     </row>
     <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A133" s="37"/>
@@ -4249,7 +4464,7 @@
       <c r="G133" s="41"/>
       <c r="H133" s="41"/>
       <c r="I133" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="I133:I143" si="13">H133-G133</f>
         <v>0</v>
       </c>
       <c r="J133" s="45"/>
@@ -4292,35 +4507,161 @@
       <c r="K135" s="43"/>
     </row>
     <row r="136" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A136" s="48"/>
-      <c r="B136" s="49"/>
-      <c r="C136" s="49"/>
-      <c r="D136" s="49"/>
-      <c r="E136" s="49" t="s">
+      <c r="A136" s="37"/>
+      <c r="B136" s="38"/>
+      <c r="C136" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D136" s="38"/>
+      <c r="E136" s="40"/>
+      <c r="F136" s="40"/>
+      <c r="G136" s="41"/>
+      <c r="H136" s="41"/>
+      <c r="I136" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J136" s="45"/>
+      <c r="K136" s="43"/>
+    </row>
+    <row r="137" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A137" s="37"/>
+      <c r="B137" s="38"/>
+      <c r="C137" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D137" s="38"/>
+      <c r="E137" s="40"/>
+      <c r="F137" s="40"/>
+      <c r="G137" s="41"/>
+      <c r="H137" s="41"/>
+      <c r="I137" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J137" s="45"/>
+      <c r="K137" s="43"/>
+    </row>
+    <row r="138" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A138" s="37"/>
+      <c r="B138" s="38"/>
+      <c r="C138" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D138" s="38"/>
+      <c r="E138" s="40"/>
+      <c r="F138" s="40"/>
+      <c r="G138" s="41"/>
+      <c r="H138" s="41"/>
+      <c r="I138" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J138" s="45"/>
+      <c r="K138" s="43"/>
+    </row>
+    <row r="139" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A139" s="37"/>
+      <c r="B139" s="38"/>
+      <c r="C139" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D139" s="38"/>
+      <c r="E139" s="40"/>
+      <c r="F139" s="40"/>
+      <c r="G139" s="41"/>
+      <c r="H139" s="41"/>
+      <c r="I139" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J139" s="45"/>
+      <c r="K139" s="43"/>
+    </row>
+    <row r="140" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A140" s="37"/>
+      <c r="B140" s="38"/>
+      <c r="C140" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D140" s="38"/>
+      <c r="E140" s="40"/>
+      <c r="F140" s="40"/>
+      <c r="G140" s="41"/>
+      <c r="H140" s="41"/>
+      <c r="I140" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J140" s="45"/>
+      <c r="K140" s="43"/>
+    </row>
+    <row r="141" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A141" s="37"/>
+      <c r="B141" s="38"/>
+      <c r="C141" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D141" s="38"/>
+      <c r="E141" s="40"/>
+      <c r="F141" s="40"/>
+      <c r="G141" s="41"/>
+      <c r="H141" s="41"/>
+      <c r="I141" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J141" s="45"/>
+      <c r="K141" s="43"/>
+    </row>
+    <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A142" s="37"/>
+      <c r="B142" s="38"/>
+      <c r="C142" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D142" s="38"/>
+      <c r="E142" s="40"/>
+      <c r="F142" s="40"/>
+      <c r="G142" s="41"/>
+      <c r="H142" s="41"/>
+      <c r="I142" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J142" s="45"/>
+      <c r="K142" s="43"/>
+    </row>
+    <row r="143" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A143" s="48"/>
+      <c r="B143" s="49"/>
+      <c r="C143" s="49"/>
+      <c r="D143" s="49"/>
+      <c r="E143" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F136" s="49"/>
-      <c r="G136" s="50">
-        <f t="shared" ref="G136:H136" si="14">SUM(G126:G135)</f>
-        <v>0</v>
-      </c>
-      <c r="H136" s="50">
+      <c r="F143" s="49"/>
+      <c r="G143" s="50">
+        <f t="shared" ref="G143:H143" si="14">SUM(G133:G142)</f>
+        <v>0</v>
+      </c>
+      <c r="H143" s="50">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="I136" s="50">
+      <c r="I143" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J136" s="51"/>
-      <c r="K136" s="52"/>
+      <c r="J143" s="51"/>
+      <c r="K143" s="52"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K38" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{E701863D-E635-476F-BEE7-EDA0E07C86C2}">
+      <autoFilter ref="A1:K15" xr:uid="{9400C8B7-216F-46C1-9400-EC89A2528798}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -4331,98 +4672,101 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B96:K96"/>
-    <mergeCell ref="B97:K97"/>
-    <mergeCell ref="A109:K109"/>
-    <mergeCell ref="B69:K69"/>
-    <mergeCell ref="A81:K81"/>
-    <mergeCell ref="B82:K82"/>
-    <mergeCell ref="B83:K83"/>
-    <mergeCell ref="A95:K95"/>
-    <mergeCell ref="A123:K123"/>
-    <mergeCell ref="B124:K124"/>
-    <mergeCell ref="B125:K125"/>
+    <mergeCell ref="A130:K130"/>
+    <mergeCell ref="B131:K131"/>
+    <mergeCell ref="B132:K132"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
-    <mergeCell ref="A39:K39"/>
-    <mergeCell ref="B40:K40"/>
-    <mergeCell ref="B41:K41"/>
-    <mergeCell ref="A53:K53"/>
-    <mergeCell ref="B54:K54"/>
-    <mergeCell ref="B55:K55"/>
-    <mergeCell ref="A67:K67"/>
-    <mergeCell ref="B110:K110"/>
-    <mergeCell ref="B111:K111"/>
-    <mergeCell ref="B68:K68"/>
+    <mergeCell ref="A46:K46"/>
+    <mergeCell ref="B47:K47"/>
+    <mergeCell ref="B48:K48"/>
+    <mergeCell ref="A60:K60"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="B62:K62"/>
+    <mergeCell ref="A74:K74"/>
+    <mergeCell ref="B117:K117"/>
+    <mergeCell ref="B118:K118"/>
+    <mergeCell ref="B75:K75"/>
+    <mergeCell ref="B103:K103"/>
+    <mergeCell ref="B104:K104"/>
+    <mergeCell ref="A116:K116"/>
+    <mergeCell ref="B76:K76"/>
+    <mergeCell ref="A88:K88"/>
+    <mergeCell ref="B89:K89"/>
+    <mergeCell ref="B90:K90"/>
+    <mergeCell ref="A102:K102"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B37 B40:B51 B56:B65 B70:B79 B84:B93 B98:B107 B112:B121">
-    <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
+  <conditionalFormatting sqref="B5:B44 B47:B58 B63:B72 B77:B86 B91:B100 B105:B114 B119:B128">
+    <cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="7" operator="containsText" text="Planned">
+    <cfRule type="containsText" dxfId="16" priority="7" operator="containsText" text="Planned">
       <formula>NOT(ISERROR(SEARCH(("Planned"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="8" operator="containsText" text="In-Progress">
+    <cfRule type="containsText" dxfId="15" priority="8" operator="containsText" text="In-Progress">
       <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="9" operator="containsText" text="Blocked">
+    <cfRule type="containsText" dxfId="14" priority="9" operator="containsText" text="Blocked">
       <formula>NOT(ISERROR(SEARCH(("Blocked"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="10" operator="containsText" text="Done">
+    <cfRule type="containsText" dxfId="13" priority="10" operator="containsText" text="Done">
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B38 B40:B52 B54:B66 B68:B80 B82:B94 B96:B108 B110:B122 B124:B136">
-    <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
+  <conditionalFormatting sqref="B5:B45 B47:B59 B61:B73 B75:B87 B89:B101 B103:B115 B117:B129 B131:B143">
+    <cfRule type="containsText" dxfId="12" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="Cancelled">
+    <cfRule type="containsText" dxfId="11" priority="12" operator="containsText" text="Cancelled">
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B126:B135">
-    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B126))))</formula>
+  <conditionalFormatting sqref="B133:B142">
+    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Unplanned">
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B133))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B126))))</formula>
+    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="Planned">
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B133))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B126))))</formula>
+    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In-Progress">
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B133))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B126))))</formula>
+    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="Blocked">
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B133))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B126))))</formula>
+    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="Done">
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B133))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G38 G42:G52 G56:G66 G70:G80 G84:G94 G98:G108 G112:G122 G126:G136">
-    <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
+  <conditionalFormatting sqref="G1 G3:G45 G49:G59 G63:G73 G77:G87 G91:G101 G105:G115 G119:G129 G133:G143">
+    <cfRule type="cellIs" dxfId="5" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H136">
-    <cfRule type="containsBlanks" dxfId="2" priority="16">
+  <conditionalFormatting sqref="H1:H143">
+    <cfRule type="containsBlanks" dxfId="4" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I38 I42:I52 I56:I66 I70:I80 I84:I94 I98:I108 I112:I122 I126:I136">
-    <cfRule type="expression" dxfId="1" priority="13">
+  <conditionalFormatting sqref="I49:I59 I63:I73 I77:I87 I91:I101 I105:I115 I119:I129 I133:I143 I5:I45">
+    <cfRule type="expression" dxfId="3" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="14">
+    <cfRule type="expression" dxfId="2" priority="14">
       <formula>H5/G5&lt;=0.5</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F126:F135 F112:F121 F42:F51 F56:F65 F70:F79 F84:F93 F98:F107 F5:F37" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F133:F142 F119:F128 F49:F58 F63:F72 F77:F86 F91:F100 F105:F114 F5:F44" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J29" r:id="rId1" xr:uid="{0999D960-5356-4EE8-BA28-70F36BB764AC}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -4430,13 +4774,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E37 E42:E51 E56:E65 E70:E79 E84:E93 E98:E107 E112:E121 E126:E135</xm:sqref>
+          <xm:sqref>E5:E44 E49:E58 E63:E72 E77:E86 E91:E100 E105:E114 E119:E128 E133:E142</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B37 B42:B51 B56:B65 B70:B79 B84:B93 B98:B107 B112:B121 B126:B135</xm:sqref>
+          <xm:sqref>B5:B44 B49:B58 B63:B72 B77:B86 B91:B100 B105:B114 B119:B128 B133:B142</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4516,7 +4860,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" cm="1">
-        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$42:$H$51,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
+        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$49:$H$58,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" cm="1">
@@ -6077,6 +6421,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -6311,27 +6675,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6348,23 +6711,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W2 Datalab 1 Work I
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D50D50-5697-4EA3-B456-67D04EA8C759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4891ABE2-D5A5-4345-8106-B6EF0DE7CD63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$45</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$128</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$132</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$45</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="134">
   <si>
     <t>Date</t>
   </si>
@@ -465,6 +465,45 @@
   </si>
   <si>
     <t>Does not work at school, have to set up at home.</t>
+  </si>
+  <si>
+    <t>Introduction and Understanding the Problem</t>
+  </si>
+  <si>
+    <t>Data Exploration and Visualization</t>
+  </si>
+  <si>
+    <t>Data Preparation and Feature Engineering</t>
+  </si>
+  <si>
+    <t>Model Selection, Training and Tuning</t>
+  </si>
+  <si>
+    <t>Evaluation, Testing and Deliverables</t>
+  </si>
+  <si>
+    <t>Complete “ML-quiz-W2_1” in brightspace</t>
+  </si>
+  <si>
+    <t>Fill in Learning Log week 2</t>
+  </si>
+  <si>
+    <t>Stand-up meeting Week 2 Datalab 1</t>
+  </si>
+  <si>
+    <t>EDA with Python (split this up)</t>
+  </si>
+  <si>
+    <t>Re-Install all the Python packages</t>
+  </si>
+  <si>
+    <t>For some reason, VSC didn't see the environment I created last week, so I had to go through the process again.</t>
+  </si>
+  <si>
+    <t>Learn MatPlotLib</t>
+  </si>
+  <si>
+    <t>Learn Seaborn</t>
   </si>
 </sst>
 </file>
@@ -947,25 +986,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -983,6 +1005,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1001,6 +1025,24 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1008,31 +1050,12 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE8B2"/>
-          <bgColor rgb="FFFCE8B2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF4C7C3"/>
-          <bgColor rgb="FFF4C7C3"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1491,7 +1514,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K143"/>
+  <dimension ref="A1:K147"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1543,53 +1566,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="67"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="55"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="68" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="55"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -2390,7 +2413,7 @@
         <f t="shared" si="0"/>
         <v>-0.5</v>
       </c>
-      <c r="J29" s="78" t="s">
+      <c r="J29" s="53" t="s">
         <v>110</v>
       </c>
       <c r="K29" s="44"/>
@@ -2884,83 +2907,111 @@
       <c r="K45" s="46"/>
     </row>
     <row r="46" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="69" t="s">
+      <c r="A46" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="66"/>
-      <c r="C46" s="66"/>
-      <c r="D46" s="66"/>
-      <c r="E46" s="66"/>
-      <c r="F46" s="66"/>
-      <c r="G46" s="66"/>
-      <c r="H46" s="66"/>
-      <c r="I46" s="66"/>
-      <c r="J46" s="66"/>
-      <c r="K46" s="67"/>
+      <c r="B46" s="59"/>
+      <c r="C46" s="59"/>
+      <c r="D46" s="59"/>
+      <c r="E46" s="59"/>
+      <c r="F46" s="59"/>
+      <c r="G46" s="59"/>
+      <c r="H46" s="59"/>
+      <c r="I46" s="59"/>
+      <c r="J46" s="59"/>
+      <c r="K46" s="60"/>
     </row>
     <row r="47" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A47" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B47" s="70" t="s">
+      <c r="B47" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C47" s="54"/>
-      <c r="D47" s="54"/>
-      <c r="E47" s="54"/>
-      <c r="F47" s="54"/>
-      <c r="G47" s="54"/>
-      <c r="H47" s="54"/>
-      <c r="I47" s="54"/>
-      <c r="J47" s="54"/>
-      <c r="K47" s="55"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="62"/>
+      <c r="E47" s="62"/>
+      <c r="F47" s="62"/>
+      <c r="G47" s="62"/>
+      <c r="H47" s="62"/>
+      <c r="I47" s="62"/>
+      <c r="J47" s="62"/>
+      <c r="K47" s="63"/>
     </row>
     <row r="48" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="70" t="s">
+      <c r="B48" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C48" s="54"/>
-      <c r="D48" s="54"/>
-      <c r="E48" s="54"/>
-      <c r="F48" s="54"/>
-      <c r="G48" s="54"/>
-      <c r="H48" s="54"/>
-      <c r="I48" s="54"/>
-      <c r="J48" s="54"/>
-      <c r="K48" s="55"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A49" s="47"/>
-      <c r="B49" s="38"/>
+      <c r="A49" s="47">
+        <v>45621</v>
+      </c>
+      <c r="B49" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C49" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D49" s="38"/>
-      <c r="E49" s="40"/>
-      <c r="F49" s="40"/>
-      <c r="G49" s="41"/>
-      <c r="H49" s="41"/>
+      <c r="D49" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="E49" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F49" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G49" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H49" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I49" s="41">
-        <f t="shared" ref="I49:I59" si="1">H49-G49</f>
+        <f t="shared" ref="I49:I63" si="1">H49-G49</f>
         <v>0</v>
       </c>
       <c r="J49" s="45"/>
       <c r="K49" s="43"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A50" s="47"/>
-      <c r="B50" s="38"/>
+      <c r="A50" s="47">
+        <v>45621</v>
+      </c>
+      <c r="B50" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C50" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D50" s="38"/>
-      <c r="E50" s="40"/>
-      <c r="F50" s="40"/>
-      <c r="G50" s="41"/>
-      <c r="H50" s="41"/>
+      <c r="D50" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="E50" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F50" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G50" s="41">
+        <v>1</v>
+      </c>
+      <c r="H50" s="41">
+        <v>1</v>
+      </c>
       <c r="I50" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2969,16 +3020,30 @@
       <c r="K50" s="43"/>
     </row>
     <row r="51" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A51" s="47"/>
-      <c r="B51" s="38"/>
+      <c r="A51" s="47">
+        <v>45621</v>
+      </c>
+      <c r="B51" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C51" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D51" s="38"/>
-      <c r="E51" s="40"/>
-      <c r="F51" s="40"/>
-      <c r="G51" s="41"/>
-      <c r="H51" s="41"/>
+      <c r="D51" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="E51" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F51" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G51" s="41">
+        <v>2</v>
+      </c>
+      <c r="H51" s="41">
+        <v>2</v>
+      </c>
       <c r="I51" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2987,16 +3052,30 @@
       <c r="K51" s="43"/>
     </row>
     <row r="52" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A52" s="47"/>
-      <c r="B52" s="38"/>
+      <c r="A52" s="47">
+        <v>45621</v>
+      </c>
+      <c r="B52" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C52" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D52" s="38"/>
-      <c r="E52" s="40"/>
-      <c r="F52" s="40"/>
-      <c r="G52" s="41"/>
-      <c r="H52" s="41"/>
+      <c r="D52" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="E52" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F52" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G52" s="41">
+        <v>2</v>
+      </c>
+      <c r="H52" s="41">
+        <v>2</v>
+      </c>
       <c r="I52" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3005,16 +3084,30 @@
       <c r="K52" s="43"/>
     </row>
     <row r="53" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A53" s="47"/>
-      <c r="B53" s="38"/>
+      <c r="A53" s="47">
+        <v>45621</v>
+      </c>
+      <c r="B53" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C53" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D53" s="38"/>
-      <c r="E53" s="40"/>
-      <c r="F53" s="40"/>
-      <c r="G53" s="41"/>
-      <c r="H53" s="41"/>
+      <c r="D53" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="E53" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F53" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G53" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H53" s="41">
+        <v>1.5</v>
+      </c>
       <c r="I53" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3023,16 +3116,30 @@
       <c r="K53" s="43"/>
     </row>
     <row r="54" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A54" s="47"/>
-      <c r="B54" s="38"/>
+      <c r="A54" s="47">
+        <v>45621</v>
+      </c>
+      <c r="B54" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C54" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D54" s="38"/>
-      <c r="E54" s="40"/>
-      <c r="F54" s="40"/>
-      <c r="G54" s="41"/>
-      <c r="H54" s="41"/>
+      <c r="D54" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="E54" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F54" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G54" s="41">
+        <v>1</v>
+      </c>
+      <c r="H54" s="41">
+        <v>1</v>
+      </c>
       <c r="I54" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3041,16 +3148,30 @@
       <c r="K54" s="43"/>
     </row>
     <row r="55" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A55" s="47"/>
-      <c r="B55" s="38"/>
+      <c r="A55" s="47">
+        <v>45621</v>
+      </c>
+      <c r="B55" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C55" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D55" s="38"/>
-      <c r="E55" s="40"/>
-      <c r="F55" s="40"/>
-      <c r="G55" s="41"/>
-      <c r="H55" s="41"/>
+      <c r="D55" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="E55" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F55" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G55" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H55" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I55" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3059,16 +3180,30 @@
       <c r="K55" s="43"/>
     </row>
     <row r="56" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A56" s="47"/>
-      <c r="B56" s="38"/>
+      <c r="A56" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B56" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C56" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D56" s="38"/>
-      <c r="E56" s="40"/>
-      <c r="F56" s="40"/>
-      <c r="G56" s="41"/>
-      <c r="H56" s="41"/>
+      <c r="D56" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="E56" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F56" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G56" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H56" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I56" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3077,16 +3212,30 @@
       <c r="K56" s="43"/>
     </row>
     <row r="57" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A57" s="47"/>
-      <c r="B57" s="38"/>
+      <c r="A57" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B57" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C57" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D57" s="38"/>
-      <c r="E57" s="40"/>
-      <c r="F57" s="40"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="41"/>
+      <c r="D57" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="E57" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F57" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G57" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H57" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I57" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3095,167 +3244,219 @@
       <c r="K57" s="43"/>
     </row>
     <row r="58" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A58" s="47"/>
-      <c r="B58" s="38"/>
+      <c r="A58" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B58" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C58" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D58" s="38"/>
-      <c r="E58" s="40"/>
-      <c r="F58" s="40"/>
-      <c r="G58" s="41"/>
-      <c r="H58" s="41"/>
+      <c r="D58" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="E58" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F58" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G58" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H58" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I58" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J58" s="45"/>
-      <c r="K58" s="43"/>
+      <c r="K58" s="43" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="59" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A59" s="13"/>
-      <c r="B59" s="15"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15" t="s">
+      <c r="A59" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B59" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C59" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D59" s="38" t="s">
+        <v>132</v>
+      </c>
+      <c r="E59" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F59" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G59" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H59" s="41"/>
+      <c r="I59" s="41">
+        <f t="shared" si="1"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J59" s="45"/>
+      <c r="K59" s="43"/>
+    </row>
+    <row r="60" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A60" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B60" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C60" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D60" s="38" t="s">
+        <v>133</v>
+      </c>
+      <c r="E60" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F60" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G60" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H60" s="41"/>
+      <c r="I60" s="41">
+        <f t="shared" si="1"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J60" s="45"/>
+      <c r="K60" s="43"/>
+    </row>
+    <row r="61" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A61" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B61" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C61" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D61" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="E61" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F61" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G61" s="41">
+        <v>6.5</v>
+      </c>
+      <c r="H61" s="41"/>
+      <c r="I61" s="41">
+        <f t="shared" si="1"/>
+        <v>-6.5</v>
+      </c>
+      <c r="J61" s="45"/>
+      <c r="K61" s="43"/>
+    </row>
+    <row r="62" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A62" s="47"/>
+      <c r="B62" s="38"/>
+      <c r="C62" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D62" s="38"/>
+      <c r="E62" s="40"/>
+      <c r="F62" s="40"/>
+      <c r="G62" s="41"/>
+      <c r="H62" s="41"/>
+      <c r="I62" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J62" s="45"/>
+      <c r="K62" s="43"/>
+    </row>
+    <row r="63" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A63" s="13"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F59" s="15"/>
-      <c r="G59" s="18">
-        <f t="shared" ref="G59:H59" si="2">SUM(G47:G58)</f>
-        <v>0</v>
-      </c>
-      <c r="H59" s="18">
+      <c r="F63" s="15"/>
+      <c r="G63" s="18">
+        <f t="shared" ref="G63:H63" si="2">SUM(G47:G62)</f>
+        <v>17.25</v>
+      </c>
+      <c r="H63" s="18">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I59" s="18">
+        <v>9.75</v>
+      </c>
+      <c r="I63" s="18">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J59" s="19"/>
-      <c r="K59" s="46"/>
-    </row>
-    <row r="60" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="71" t="s">
+        <v>-7.5</v>
+      </c>
+      <c r="J63" s="19"/>
+      <c r="K63" s="46"/>
+    </row>
+    <row r="64" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B60" s="54"/>
-      <c r="C60" s="54"/>
-      <c r="D60" s="54"/>
-      <c r="E60" s="54"/>
-      <c r="F60" s="54"/>
-      <c r="G60" s="54"/>
-      <c r="H60" s="54"/>
-      <c r="I60" s="54"/>
-      <c r="J60" s="54"/>
-      <c r="K60" s="55"/>
-    </row>
-    <row r="61" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A61" s="21" t="s">
+      <c r="B64" s="62"/>
+      <c r="C64" s="62"/>
+      <c r="D64" s="62"/>
+      <c r="E64" s="62"/>
+      <c r="F64" s="62"/>
+      <c r="G64" s="62"/>
+      <c r="H64" s="62"/>
+      <c r="I64" s="62"/>
+      <c r="J64" s="62"/>
+      <c r="K64" s="63"/>
+    </row>
+    <row r="65" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A65" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B61" s="72" t="s">
+      <c r="B65" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C61" s="54"/>
-      <c r="D61" s="54"/>
-      <c r="E61" s="54"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="54"/>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="54"/>
-      <c r="K61" s="55"/>
-    </row>
-    <row r="62" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="22" t="s">
+      <c r="C65" s="62"/>
+      <c r="D65" s="62"/>
+      <c r="E65" s="62"/>
+      <c r="F65" s="62"/>
+      <c r="G65" s="62"/>
+      <c r="H65" s="62"/>
+      <c r="I65" s="62"/>
+      <c r="J65" s="62"/>
+      <c r="K65" s="63"/>
+    </row>
+    <row r="66" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B62" s="72" t="s">
+      <c r="B66" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C62" s="54"/>
-      <c r="D62" s="54"/>
-      <c r="E62" s="54"/>
-      <c r="F62" s="54"/>
-      <c r="G62" s="54"/>
-      <c r="H62" s="54"/>
-      <c r="I62" s="54"/>
-      <c r="J62" s="54"/>
-      <c r="K62" s="55"/>
-    </row>
-    <row r="63" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A63" s="37"/>
-      <c r="B63" s="38"/>
-      <c r="C63" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D63" s="38"/>
-      <c r="E63" s="40"/>
-      <c r="F63" s="40"/>
-      <c r="G63" s="41"/>
-      <c r="H63" s="41"/>
-      <c r="I63" s="41">
-        <f t="shared" ref="I63:I73" si="3">H63-G63</f>
-        <v>0</v>
-      </c>
-      <c r="J63" s="45"/>
-      <c r="K63" s="43"/>
-    </row>
-    <row r="64" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A64" s="37"/>
-      <c r="B64" s="38"/>
-      <c r="C64" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D64" s="38"/>
-      <c r="E64" s="40"/>
-      <c r="F64" s="40"/>
-      <c r="G64" s="41"/>
-      <c r="H64" s="41"/>
-      <c r="I64" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J64" s="45"/>
-      <c r="K64" s="43"/>
-    </row>
-    <row r="65" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A65" s="37"/>
-      <c r="B65" s="38"/>
-      <c r="C65" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D65" s="38"/>
-      <c r="E65" s="40"/>
-      <c r="F65" s="40"/>
-      <c r="G65" s="41"/>
-      <c r="H65" s="41"/>
-      <c r="I65" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J65" s="45"/>
-      <c r="K65" s="43"/>
-    </row>
-    <row r="66" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A66" s="37"/>
-      <c r="B66" s="38"/>
-      <c r="C66" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D66" s="38"/>
-      <c r="E66" s="40"/>
-      <c r="F66" s="40"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="41"/>
-      <c r="I66" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J66" s="45"/>
-      <c r="K66" s="43"/>
+      <c r="C66" s="62"/>
+      <c r="D66" s="62"/>
+      <c r="E66" s="62"/>
+      <c r="F66" s="62"/>
+      <c r="G66" s="62"/>
+      <c r="H66" s="62"/>
+      <c r="I66" s="62"/>
+      <c r="J66" s="62"/>
+      <c r="K66" s="63"/>
     </row>
     <row r="67" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A67" s="37"/>
@@ -3269,7 +3470,7 @@
       <c r="G67" s="41"/>
       <c r="H67" s="41"/>
       <c r="I67" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="I67:I77" si="3">H67-G67</f>
         <v>0</v>
       </c>
       <c r="J67" s="45"/>
@@ -3366,149 +3567,149 @@
       <c r="K72" s="43"/>
     </row>
     <row r="73" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A73" s="13"/>
-      <c r="B73" s="15"/>
-      <c r="C73" s="15"/>
-      <c r="D73" s="15"/>
-      <c r="E73" s="15" t="s">
+      <c r="A73" s="37"/>
+      <c r="B73" s="38"/>
+      <c r="C73" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D73" s="38"/>
+      <c r="E73" s="40"/>
+      <c r="F73" s="40"/>
+      <c r="G73" s="41"/>
+      <c r="H73" s="41"/>
+      <c r="I73" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J73" s="45"/>
+      <c r="K73" s="43"/>
+    </row>
+    <row r="74" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A74" s="37"/>
+      <c r="B74" s="38"/>
+      <c r="C74" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D74" s="38"/>
+      <c r="E74" s="40"/>
+      <c r="F74" s="40"/>
+      <c r="G74" s="41"/>
+      <c r="H74" s="41"/>
+      <c r="I74" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J74" s="45"/>
+      <c r="K74" s="43"/>
+    </row>
+    <row r="75" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A75" s="37"/>
+      <c r="B75" s="38"/>
+      <c r="C75" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D75" s="38"/>
+      <c r="E75" s="40"/>
+      <c r="F75" s="40"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="41"/>
+      <c r="I75" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J75" s="45"/>
+      <c r="K75" s="43"/>
+    </row>
+    <row r="76" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A76" s="37"/>
+      <c r="B76" s="38"/>
+      <c r="C76" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D76" s="38"/>
+      <c r="E76" s="40"/>
+      <c r="F76" s="40"/>
+      <c r="G76" s="41"/>
+      <c r="H76" s="41"/>
+      <c r="I76" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J76" s="45"/>
+      <c r="K76" s="43"/>
+    </row>
+    <row r="77" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A77" s="13"/>
+      <c r="B77" s="15"/>
+      <c r="C77" s="15"/>
+      <c r="D77" s="15"/>
+      <c r="E77" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F73" s="15"/>
-      <c r="G73" s="18">
-        <f t="shared" ref="G73:H73" si="4">SUM(G63:G72)</f>
-        <v>0</v>
-      </c>
-      <c r="H73" s="18">
+      <c r="F77" s="15"/>
+      <c r="G77" s="18">
+        <f t="shared" ref="G77:H77" si="4">SUM(G67:G76)</f>
+        <v>0</v>
+      </c>
+      <c r="H77" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="I73" s="18">
+      <c r="I77" s="18">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J73" s="19"/>
-      <c r="K73" s="46"/>
-    </row>
-    <row r="74" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="73" t="s">
+      <c r="J77" s="19"/>
+      <c r="K77" s="46"/>
+    </row>
+    <row r="78" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B74" s="54"/>
-      <c r="C74" s="54"/>
-      <c r="D74" s="54"/>
-      <c r="E74" s="54"/>
-      <c r="F74" s="54"/>
-      <c r="G74" s="54"/>
-      <c r="H74" s="54"/>
-      <c r="I74" s="54"/>
-      <c r="J74" s="54"/>
-      <c r="K74" s="55"/>
-    </row>
-    <row r="75" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A75" s="23" t="s">
+      <c r="B78" s="62"/>
+      <c r="C78" s="62"/>
+      <c r="D78" s="62"/>
+      <c r="E78" s="62"/>
+      <c r="F78" s="62"/>
+      <c r="G78" s="62"/>
+      <c r="H78" s="62"/>
+      <c r="I78" s="62"/>
+      <c r="J78" s="62"/>
+      <c r="K78" s="63"/>
+    </row>
+    <row r="79" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A79" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B75" s="57" t="s">
+      <c r="B79" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C75" s="54"/>
-      <c r="D75" s="54"/>
-      <c r="E75" s="54"/>
-      <c r="F75" s="54"/>
-      <c r="G75" s="54"/>
-      <c r="H75" s="54"/>
-      <c r="I75" s="54"/>
-      <c r="J75" s="54"/>
-      <c r="K75" s="55"/>
-    </row>
-    <row r="76" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="24" t="s">
+      <c r="C79" s="62"/>
+      <c r="D79" s="62"/>
+      <c r="E79" s="62"/>
+      <c r="F79" s="62"/>
+      <c r="G79" s="62"/>
+      <c r="H79" s="62"/>
+      <c r="I79" s="62"/>
+      <c r="J79" s="62"/>
+      <c r="K79" s="63"/>
+    </row>
+    <row r="80" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B76" s="57" t="s">
+      <c r="B80" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C76" s="54"/>
-      <c r="D76" s="54"/>
-      <c r="E76" s="54"/>
-      <c r="F76" s="54"/>
-      <c r="G76" s="54"/>
-      <c r="H76" s="54"/>
-      <c r="I76" s="54"/>
-      <c r="J76" s="54"/>
-      <c r="K76" s="55"/>
-    </row>
-    <row r="77" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A77" s="37"/>
-      <c r="B77" s="38"/>
-      <c r="C77" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D77" s="38"/>
-      <c r="E77" s="40"/>
-      <c r="F77" s="40"/>
-      <c r="G77" s="41"/>
-      <c r="H77" s="41"/>
-      <c r="I77" s="41">
-        <f t="shared" ref="I77:I87" si="5">H77-G77</f>
-        <v>0</v>
-      </c>
-      <c r="J77" s="45"/>
-      <c r="K77" s="43"/>
-    </row>
-    <row r="78" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A78" s="37"/>
-      <c r="B78" s="38"/>
-      <c r="C78" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D78" s="38"/>
-      <c r="E78" s="40"/>
-      <c r="F78" s="40"/>
-      <c r="G78" s="41"/>
-      <c r="H78" s="41"/>
-      <c r="I78" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J78" s="45"/>
-      <c r="K78" s="43"/>
-    </row>
-    <row r="79" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A79" s="37"/>
-      <c r="B79" s="38"/>
-      <c r="C79" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D79" s="38"/>
-      <c r="E79" s="40"/>
-      <c r="F79" s="40"/>
-      <c r="G79" s="41"/>
-      <c r="H79" s="41"/>
-      <c r="I79" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J79" s="45"/>
-      <c r="K79" s="43"/>
-    </row>
-    <row r="80" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A80" s="37"/>
-      <c r="B80" s="38"/>
-      <c r="C80" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D80" s="38"/>
-      <c r="E80" s="40"/>
-      <c r="F80" s="40"/>
-      <c r="G80" s="41"/>
-      <c r="H80" s="41"/>
-      <c r="I80" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J80" s="45"/>
-      <c r="K80" s="43"/>
+      <c r="C80" s="62"/>
+      <c r="D80" s="62"/>
+      <c r="E80" s="62"/>
+      <c r="F80" s="62"/>
+      <c r="G80" s="62"/>
+      <c r="H80" s="62"/>
+      <c r="I80" s="62"/>
+      <c r="J80" s="62"/>
+      <c r="K80" s="63"/>
     </row>
     <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A81" s="37"/>
@@ -3522,7 +3723,7 @@
       <c r="G81" s="41"/>
       <c r="H81" s="41"/>
       <c r="I81" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I81:I91" si="5">H81-G81</f>
         <v>0</v>
       </c>
       <c r="J81" s="45"/>
@@ -3619,149 +3820,149 @@
       <c r="K86" s="43"/>
     </row>
     <row r="87" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A87" s="13"/>
-      <c r="B87" s="15"/>
-      <c r="C87" s="15"/>
-      <c r="D87" s="15"/>
-      <c r="E87" s="15" t="s">
+      <c r="A87" s="37"/>
+      <c r="B87" s="38"/>
+      <c r="C87" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D87" s="38"/>
+      <c r="E87" s="40"/>
+      <c r="F87" s="40"/>
+      <c r="G87" s="41"/>
+      <c r="H87" s="41"/>
+      <c r="I87" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J87" s="45"/>
+      <c r="K87" s="43"/>
+    </row>
+    <row r="88" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A88" s="37"/>
+      <c r="B88" s="38"/>
+      <c r="C88" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D88" s="38"/>
+      <c r="E88" s="40"/>
+      <c r="F88" s="40"/>
+      <c r="G88" s="41"/>
+      <c r="H88" s="41"/>
+      <c r="I88" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J88" s="45"/>
+      <c r="K88" s="43"/>
+    </row>
+    <row r="89" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A89" s="37"/>
+      <c r="B89" s="38"/>
+      <c r="C89" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D89" s="38"/>
+      <c r="E89" s="40"/>
+      <c r="F89" s="40"/>
+      <c r="G89" s="41"/>
+      <c r="H89" s="41"/>
+      <c r="I89" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J89" s="45"/>
+      <c r="K89" s="43"/>
+    </row>
+    <row r="90" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A90" s="37"/>
+      <c r="B90" s="38"/>
+      <c r="C90" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D90" s="38"/>
+      <c r="E90" s="40"/>
+      <c r="F90" s="40"/>
+      <c r="G90" s="41"/>
+      <c r="H90" s="41"/>
+      <c r="I90" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J90" s="45"/>
+      <c r="K90" s="43"/>
+    </row>
+    <row r="91" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A91" s="13"/>
+      <c r="B91" s="15"/>
+      <c r="C91" s="15"/>
+      <c r="D91" s="15"/>
+      <c r="E91" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F87" s="15"/>
-      <c r="G87" s="18">
-        <f t="shared" ref="G87:H87" si="6">SUM(G77:G86)</f>
-        <v>0</v>
-      </c>
-      <c r="H87" s="18">
+      <c r="F91" s="15"/>
+      <c r="G91" s="18">
+        <f t="shared" ref="G91:H91" si="6">SUM(G81:G90)</f>
+        <v>0</v>
+      </c>
+      <c r="H91" s="18">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="I87" s="18">
+      <c r="I91" s="18">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J87" s="19"/>
-      <c r="K87" s="46"/>
-    </row>
-    <row r="88" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="58" t="s">
+      <c r="J91" s="19"/>
+      <c r="K91" s="46"/>
+    </row>
+    <row r="92" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B88" s="54"/>
-      <c r="C88" s="54"/>
-      <c r="D88" s="54"/>
-      <c r="E88" s="54"/>
-      <c r="F88" s="54"/>
-      <c r="G88" s="54"/>
-      <c r="H88" s="54"/>
-      <c r="I88" s="54"/>
-      <c r="J88" s="54"/>
-      <c r="K88" s="55"/>
-    </row>
-    <row r="89" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A89" s="25" t="s">
+      <c r="B92" s="62"/>
+      <c r="C92" s="62"/>
+      <c r="D92" s="62"/>
+      <c r="E92" s="62"/>
+      <c r="F92" s="62"/>
+      <c r="G92" s="62"/>
+      <c r="H92" s="62"/>
+      <c r="I92" s="62"/>
+      <c r="J92" s="62"/>
+      <c r="K92" s="63"/>
+    </row>
+    <row r="93" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A93" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B89" s="59" t="s">
+      <c r="B93" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C89" s="54"/>
-      <c r="D89" s="54"/>
-      <c r="E89" s="54"/>
-      <c r="F89" s="54"/>
-      <c r="G89" s="54"/>
-      <c r="H89" s="54"/>
-      <c r="I89" s="54"/>
-      <c r="J89" s="54"/>
-      <c r="K89" s="55"/>
-    </row>
-    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="26" t="s">
+      <c r="C93" s="62"/>
+      <c r="D93" s="62"/>
+      <c r="E93" s="62"/>
+      <c r="F93" s="62"/>
+      <c r="G93" s="62"/>
+      <c r="H93" s="62"/>
+      <c r="I93" s="62"/>
+      <c r="J93" s="62"/>
+      <c r="K93" s="63"/>
+    </row>
+    <row r="94" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="59" t="s">
+      <c r="B94" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C90" s="54"/>
-      <c r="D90" s="54"/>
-      <c r="E90" s="54"/>
-      <c r="F90" s="54"/>
-      <c r="G90" s="54"/>
-      <c r="H90" s="54"/>
-      <c r="I90" s="54"/>
-      <c r="J90" s="54"/>
-      <c r="K90" s="55"/>
-    </row>
-    <row r="91" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A91" s="37"/>
-      <c r="B91" s="38"/>
-      <c r="C91" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D91" s="38"/>
-      <c r="E91" s="40"/>
-      <c r="F91" s="40"/>
-      <c r="G91" s="41"/>
-      <c r="H91" s="41"/>
-      <c r="I91" s="41">
-        <f t="shared" ref="I91:I101" si="7">H91-G91</f>
-        <v>0</v>
-      </c>
-      <c r="J91" s="45"/>
-      <c r="K91" s="43"/>
-    </row>
-    <row r="92" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A92" s="37"/>
-      <c r="B92" s="38"/>
-      <c r="C92" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D92" s="38"/>
-      <c r="E92" s="40"/>
-      <c r="F92" s="40"/>
-      <c r="G92" s="41"/>
-      <c r="H92" s="41"/>
-      <c r="I92" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J92" s="45"/>
-      <c r="K92" s="43"/>
-    </row>
-    <row r="93" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A93" s="37"/>
-      <c r="B93" s="38"/>
-      <c r="C93" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D93" s="38"/>
-      <c r="E93" s="40"/>
-      <c r="F93" s="40"/>
-      <c r="G93" s="41"/>
-      <c r="H93" s="41"/>
-      <c r="I93" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J93" s="45"/>
-      <c r="K93" s="43"/>
-    </row>
-    <row r="94" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A94" s="37"/>
-      <c r="B94" s="38"/>
-      <c r="C94" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D94" s="38"/>
-      <c r="E94" s="40"/>
-      <c r="F94" s="40"/>
-      <c r="G94" s="41"/>
-      <c r="H94" s="41"/>
-      <c r="I94" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J94" s="45"/>
-      <c r="K94" s="43"/>
+      <c r="C94" s="62"/>
+      <c r="D94" s="62"/>
+      <c r="E94" s="62"/>
+      <c r="F94" s="62"/>
+      <c r="G94" s="62"/>
+      <c r="H94" s="62"/>
+      <c r="I94" s="62"/>
+      <c r="J94" s="62"/>
+      <c r="K94" s="63"/>
     </row>
     <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A95" s="37"/>
@@ -3775,7 +3976,7 @@
       <c r="G95" s="41"/>
       <c r="H95" s="41"/>
       <c r="I95" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="I95:I105" si="7">H95-G95</f>
         <v>0</v>
       </c>
       <c r="J95" s="45"/>
@@ -3872,151 +4073,149 @@
       <c r="K100" s="43"/>
     </row>
     <row r="101" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A101" s="13"/>
-      <c r="B101" s="15"/>
-      <c r="C101" s="15"/>
-      <c r="D101" s="15"/>
-      <c r="E101" s="15" t="s">
+      <c r="A101" s="37"/>
+      <c r="B101" s="38"/>
+      <c r="C101" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D101" s="38"/>
+      <c r="E101" s="40"/>
+      <c r="F101" s="40"/>
+      <c r="G101" s="41"/>
+      <c r="H101" s="41"/>
+      <c r="I101" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J101" s="45"/>
+      <c r="K101" s="43"/>
+    </row>
+    <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A102" s="37"/>
+      <c r="B102" s="38"/>
+      <c r="C102" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D102" s="38"/>
+      <c r="E102" s="40"/>
+      <c r="F102" s="40"/>
+      <c r="G102" s="41"/>
+      <c r="H102" s="41"/>
+      <c r="I102" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J102" s="45"/>
+      <c r="K102" s="43"/>
+    </row>
+    <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A103" s="37"/>
+      <c r="B103" s="38"/>
+      <c r="C103" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D103" s="38"/>
+      <c r="E103" s="40"/>
+      <c r="F103" s="40"/>
+      <c r="G103" s="41"/>
+      <c r="H103" s="41"/>
+      <c r="I103" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J103" s="45"/>
+      <c r="K103" s="43"/>
+    </row>
+    <row r="104" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A104" s="37"/>
+      <c r="B104" s="38"/>
+      <c r="C104" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D104" s="38"/>
+      <c r="E104" s="40"/>
+      <c r="F104" s="40"/>
+      <c r="G104" s="41"/>
+      <c r="H104" s="41"/>
+      <c r="I104" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J104" s="45"/>
+      <c r="K104" s="43"/>
+    </row>
+    <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A105" s="13"/>
+      <c r="B105" s="15"/>
+      <c r="C105" s="15"/>
+      <c r="D105" s="15"/>
+      <c r="E105" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F101" s="15"/>
-      <c r="G101" s="18">
-        <f t="shared" ref="G101:H101" si="8">SUM(G91:G100)</f>
-        <v>0</v>
-      </c>
-      <c r="H101" s="18">
+      <c r="F105" s="15"/>
+      <c r="G105" s="18">
+        <f t="shared" ref="G105:H105" si="8">SUM(G95:G104)</f>
+        <v>0</v>
+      </c>
+      <c r="H105" s="18">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="I101" s="18">
+      <c r="I105" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J101" s="19"/>
-      <c r="K101" s="46"/>
-    </row>
-    <row r="102" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="60" t="s">
+      <c r="J105" s="19"/>
+      <c r="K105" s="46"/>
+    </row>
+    <row r="106" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B102" s="54"/>
-      <c r="C102" s="54"/>
-      <c r="D102" s="54"/>
-      <c r="E102" s="54"/>
-      <c r="F102" s="54"/>
-      <c r="G102" s="54"/>
-      <c r="H102" s="54"/>
-      <c r="I102" s="54"/>
-      <c r="J102" s="54"/>
-      <c r="K102" s="55"/>
-    </row>
-    <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A103" s="27" t="s">
+      <c r="B106" s="62"/>
+      <c r="C106" s="62"/>
+      <c r="D106" s="62"/>
+      <c r="E106" s="62"/>
+      <c r="F106" s="62"/>
+      <c r="G106" s="62"/>
+      <c r="H106" s="62"/>
+      <c r="I106" s="62"/>
+      <c r="J106" s="62"/>
+      <c r="K106" s="63"/>
+    </row>
+    <row r="107" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A107" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B103" s="53" t="s">
+      <c r="B107" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C103" s="54"/>
-      <c r="D103" s="54"/>
-      <c r="E103" s="54"/>
-      <c r="F103" s="54"/>
-      <c r="G103" s="54"/>
-      <c r="H103" s="54"/>
-      <c r="I103" s="54"/>
-      <c r="J103" s="54"/>
-      <c r="K103" s="55"/>
-    </row>
-    <row r="104" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="28" t="s">
+      <c r="C107" s="62"/>
+      <c r="D107" s="62"/>
+      <c r="E107" s="62"/>
+      <c r="F107" s="62"/>
+      <c r="G107" s="62"/>
+      <c r="H107" s="62"/>
+      <c r="I107" s="62"/>
+      <c r="J107" s="62"/>
+      <c r="K107" s="63"/>
+    </row>
+    <row r="108" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B104" s="53" t="s">
+      <c r="B108" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C104" s="54"/>
-      <c r="D104" s="54"/>
-      <c r="E104" s="54"/>
-      <c r="F104" s="54"/>
-      <c r="G104" s="54"/>
-      <c r="H104" s="54"/>
-      <c r="I104" s="54"/>
-      <c r="J104" s="54"/>
-      <c r="K104" s="55"/>
-    </row>
-    <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A105" s="37"/>
-      <c r="B105" s="38"/>
-      <c r="C105" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D105" s="38"/>
-      <c r="E105" s="40"/>
-      <c r="F105" s="40"/>
-      <c r="G105" s="41"/>
-      <c r="H105" s="41"/>
-      <c r="I105" s="41">
-        <f t="shared" ref="I105:I115" si="9">H105-G105</f>
-        <v>0</v>
-      </c>
-      <c r="J105" s="45"/>
-      <c r="K105" s="43"/>
-    </row>
-    <row r="106" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A106" s="37"/>
-      <c r="B106" s="38"/>
-      <c r="C106" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D106" s="38"/>
-      <c r="E106" s="40"/>
-      <c r="F106" s="40"/>
-      <c r="G106" s="41"/>
-      <c r="H106" s="41"/>
-      <c r="I106" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J106" s="45"/>
-      <c r="K106" s="43"/>
-    </row>
-    <row r="107" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A107" s="37"/>
-      <c r="B107" s="38"/>
-      <c r="C107" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D107" s="38"/>
-      <c r="E107" s="40"/>
-      <c r="F107" s="40"/>
-      <c r="G107" s="41"/>
-      <c r="H107" s="41"/>
-      <c r="I107" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J107" s="45"/>
-      <c r="K107" s="43" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="108" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A108" s="37"/>
-      <c r="B108" s="38"/>
-      <c r="C108" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D108" s="38"/>
-      <c r="E108" s="40"/>
-      <c r="F108" s="40"/>
-      <c r="G108" s="41"/>
-      <c r="H108" s="41"/>
-      <c r="I108" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J108" s="45"/>
-      <c r="K108" s="43"/>
+      <c r="C108" s="62"/>
+      <c r="D108" s="62"/>
+      <c r="E108" s="62"/>
+      <c r="F108" s="62"/>
+      <c r="G108" s="62"/>
+      <c r="H108" s="62"/>
+      <c r="I108" s="62"/>
+      <c r="J108" s="62"/>
+      <c r="K108" s="63"/>
     </row>
     <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A109" s="37"/>
@@ -4030,7 +4229,7 @@
       <c r="G109" s="41"/>
       <c r="H109" s="41"/>
       <c r="I109" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I109:I119" si="9">H109-G109</f>
         <v>0</v>
       </c>
       <c r="J109" s="45"/>
@@ -4070,7 +4269,9 @@
         <v>0</v>
       </c>
       <c r="J111" s="45"/>
-      <c r="K111" s="43"/>
+      <c r="K111" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A112" s="37"/>
@@ -4127,149 +4328,149 @@
       <c r="K114" s="43"/>
     </row>
     <row r="115" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A115" s="13"/>
-      <c r="B115" s="15"/>
-      <c r="C115" s="15"/>
-      <c r="D115" s="15"/>
-      <c r="E115" s="15" t="s">
+      <c r="A115" s="37"/>
+      <c r="B115" s="38"/>
+      <c r="C115" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D115" s="38"/>
+      <c r="E115" s="40"/>
+      <c r="F115" s="40"/>
+      <c r="G115" s="41"/>
+      <c r="H115" s="41"/>
+      <c r="I115" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J115" s="45"/>
+      <c r="K115" s="43"/>
+    </row>
+    <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A116" s="37"/>
+      <c r="B116" s="38"/>
+      <c r="C116" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D116" s="38"/>
+      <c r="E116" s="40"/>
+      <c r="F116" s="40"/>
+      <c r="G116" s="41"/>
+      <c r="H116" s="41"/>
+      <c r="I116" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J116" s="45"/>
+      <c r="K116" s="43"/>
+    </row>
+    <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A117" s="37"/>
+      <c r="B117" s="38"/>
+      <c r="C117" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D117" s="38"/>
+      <c r="E117" s="40"/>
+      <c r="F117" s="40"/>
+      <c r="G117" s="41"/>
+      <c r="H117" s="41"/>
+      <c r="I117" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J117" s="45"/>
+      <c r="K117" s="43"/>
+    </row>
+    <row r="118" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A118" s="37"/>
+      <c r="B118" s="38"/>
+      <c r="C118" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D118" s="38"/>
+      <c r="E118" s="40"/>
+      <c r="F118" s="40"/>
+      <c r="G118" s="41"/>
+      <c r="H118" s="41"/>
+      <c r="I118" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J118" s="45"/>
+      <c r="K118" s="43"/>
+    </row>
+    <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A119" s="13"/>
+      <c r="B119" s="15"/>
+      <c r="C119" s="15"/>
+      <c r="D119" s="15"/>
+      <c r="E119" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F115" s="15"/>
-      <c r="G115" s="18">
-        <f t="shared" ref="G115:H115" si="10">SUM(G105:G114)</f>
-        <v>0</v>
-      </c>
-      <c r="H115" s="18">
+      <c r="F119" s="15"/>
+      <c r="G119" s="18">
+        <f t="shared" ref="G119:H119" si="10">SUM(G109:G118)</f>
+        <v>0</v>
+      </c>
+      <c r="H119" s="18">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="I115" s="18">
+      <c r="I119" s="18">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J115" s="19"/>
-      <c r="K115" s="46"/>
-    </row>
-    <row r="116" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="56" t="s">
+      <c r="J119" s="19"/>
+      <c r="K119" s="46"/>
+    </row>
+    <row r="120" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="B116" s="54"/>
-      <c r="C116" s="54"/>
-      <c r="D116" s="54"/>
-      <c r="E116" s="54"/>
-      <c r="F116" s="54"/>
-      <c r="G116" s="54"/>
-      <c r="H116" s="54"/>
-      <c r="I116" s="54"/>
-      <c r="J116" s="54"/>
-      <c r="K116" s="55"/>
-    </row>
-    <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A117" s="29" t="s">
+      <c r="B120" s="62"/>
+      <c r="C120" s="62"/>
+      <c r="D120" s="62"/>
+      <c r="E120" s="62"/>
+      <c r="F120" s="62"/>
+      <c r="G120" s="62"/>
+      <c r="H120" s="62"/>
+      <c r="I120" s="62"/>
+      <c r="J120" s="62"/>
+      <c r="K120" s="63"/>
+    </row>
+    <row r="121" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A121" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B117" s="74" t="s">
+      <c r="B121" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C117" s="54"/>
-      <c r="D117" s="54"/>
-      <c r="E117" s="54"/>
-      <c r="F117" s="54"/>
-      <c r="G117" s="54"/>
-      <c r="H117" s="54"/>
-      <c r="I117" s="54"/>
-      <c r="J117" s="54"/>
-      <c r="K117" s="55"/>
-    </row>
-    <row r="118" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="30" t="s">
+      <c r="C121" s="62"/>
+      <c r="D121" s="62"/>
+      <c r="E121" s="62"/>
+      <c r="F121" s="62"/>
+      <c r="G121" s="62"/>
+      <c r="H121" s="62"/>
+      <c r="I121" s="62"/>
+      <c r="J121" s="62"/>
+      <c r="K121" s="63"/>
+    </row>
+    <row r="122" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B118" s="74" t="s">
+      <c r="B122" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C118" s="54"/>
-      <c r="D118" s="54"/>
-      <c r="E118" s="54"/>
-      <c r="F118" s="54"/>
-      <c r="G118" s="54"/>
-      <c r="H118" s="54"/>
-      <c r="I118" s="54"/>
-      <c r="J118" s="54"/>
-      <c r="K118" s="55"/>
-    </row>
-    <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A119" s="37"/>
-      <c r="B119" s="38"/>
-      <c r="C119" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D119" s="38"/>
-      <c r="E119" s="40"/>
-      <c r="F119" s="40"/>
-      <c r="G119" s="41"/>
-      <c r="H119" s="41"/>
-      <c r="I119" s="41">
-        <f t="shared" ref="I119:I129" si="11">H119-G119</f>
-        <v>0</v>
-      </c>
-      <c r="J119" s="45"/>
-      <c r="K119" s="43"/>
-    </row>
-    <row r="120" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A120" s="37"/>
-      <c r="B120" s="38"/>
-      <c r="C120" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D120" s="38"/>
-      <c r="E120" s="40"/>
-      <c r="F120" s="40"/>
-      <c r="G120" s="41"/>
-      <c r="H120" s="41"/>
-      <c r="I120" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J120" s="45"/>
-      <c r="K120" s="43"/>
-    </row>
-    <row r="121" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A121" s="37"/>
-      <c r="B121" s="38"/>
-      <c r="C121" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D121" s="38"/>
-      <c r="E121" s="40"/>
-      <c r="F121" s="40"/>
-      <c r="G121" s="41"/>
-      <c r="H121" s="41"/>
-      <c r="I121" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J121" s="45"/>
-      <c r="K121" s="43"/>
-    </row>
-    <row r="122" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A122" s="37"/>
-      <c r="B122" s="38"/>
-      <c r="C122" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D122" s="38"/>
-      <c r="E122" s="40"/>
-      <c r="F122" s="40"/>
-      <c r="G122" s="41"/>
-      <c r="H122" s="41"/>
-      <c r="I122" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J122" s="45"/>
-      <c r="K122" s="43"/>
+      <c r="C122" s="62"/>
+      <c r="D122" s="62"/>
+      <c r="E122" s="62"/>
+      <c r="F122" s="62"/>
+      <c r="G122" s="62"/>
+      <c r="H122" s="62"/>
+      <c r="I122" s="62"/>
+      <c r="J122" s="62"/>
+      <c r="K122" s="63"/>
     </row>
     <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A123" s="37"/>
@@ -4283,7 +4484,7 @@
       <c r="G123" s="41"/>
       <c r="H123" s="41"/>
       <c r="I123" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="I123:I133" si="11">H123-G123</f>
         <v>0</v>
       </c>
       <c r="J123" s="45"/>
@@ -4380,149 +4581,149 @@
       <c r="K128" s="43"/>
     </row>
     <row r="129" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A129" s="13"/>
-      <c r="B129" s="15"/>
-      <c r="C129" s="15"/>
-      <c r="D129" s="15"/>
-      <c r="E129" s="15" t="s">
+      <c r="A129" s="37"/>
+      <c r="B129" s="38"/>
+      <c r="C129" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D129" s="38"/>
+      <c r="E129" s="40"/>
+      <c r="F129" s="40"/>
+      <c r="G129" s="41"/>
+      <c r="H129" s="41"/>
+      <c r="I129" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J129" s="45"/>
+      <c r="K129" s="43"/>
+    </row>
+    <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A130" s="37"/>
+      <c r="B130" s="38"/>
+      <c r="C130" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D130" s="38"/>
+      <c r="E130" s="40"/>
+      <c r="F130" s="40"/>
+      <c r="G130" s="41"/>
+      <c r="H130" s="41"/>
+      <c r="I130" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J130" s="45"/>
+      <c r="K130" s="43"/>
+    </row>
+    <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A131" s="37"/>
+      <c r="B131" s="38"/>
+      <c r="C131" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D131" s="38"/>
+      <c r="E131" s="40"/>
+      <c r="F131" s="40"/>
+      <c r="G131" s="41"/>
+      <c r="H131" s="41"/>
+      <c r="I131" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J131" s="45"/>
+      <c r="K131" s="43"/>
+    </row>
+    <row r="132" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A132" s="37"/>
+      <c r="B132" s="38"/>
+      <c r="C132" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D132" s="38"/>
+      <c r="E132" s="40"/>
+      <c r="F132" s="40"/>
+      <c r="G132" s="41"/>
+      <c r="H132" s="41"/>
+      <c r="I132" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J132" s="45"/>
+      <c r="K132" s="43"/>
+    </row>
+    <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A133" s="13"/>
+      <c r="B133" s="15"/>
+      <c r="C133" s="15"/>
+      <c r="D133" s="15"/>
+      <c r="E133" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F129" s="15"/>
-      <c r="G129" s="18">
-        <f t="shared" ref="G129:H129" si="12">SUM(G119:G128)</f>
-        <v>0</v>
-      </c>
-      <c r="H129" s="18">
+      <c r="F133" s="15"/>
+      <c r="G133" s="18">
+        <f t="shared" ref="G133:H133" si="12">SUM(G123:G132)</f>
+        <v>0</v>
+      </c>
+      <c r="H133" s="18">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="I129" s="18">
+      <c r="I133" s="18">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J129" s="19"/>
-      <c r="K129" s="46"/>
-    </row>
-    <row r="130" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="61" t="s">
+      <c r="J133" s="19"/>
+      <c r="K133" s="46"/>
+    </row>
+    <row r="134" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B130" s="62"/>
-      <c r="C130" s="62"/>
-      <c r="D130" s="62"/>
-      <c r="E130" s="62"/>
-      <c r="F130" s="62"/>
-      <c r="G130" s="62"/>
-      <c r="H130" s="62"/>
-      <c r="I130" s="62"/>
-      <c r="J130" s="62"/>
-      <c r="K130" s="63"/>
-    </row>
-    <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A131" s="32" t="s">
+      <c r="B134" s="55"/>
+      <c r="C134" s="55"/>
+      <c r="D134" s="55"/>
+      <c r="E134" s="55"/>
+      <c r="F134" s="55"/>
+      <c r="G134" s="55"/>
+      <c r="H134" s="55"/>
+      <c r="I134" s="55"/>
+      <c r="J134" s="55"/>
+      <c r="K134" s="56"/>
+    </row>
+    <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A135" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B131" s="64" t="s">
+      <c r="B135" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C131" s="62"/>
-      <c r="D131" s="62"/>
-      <c r="E131" s="62"/>
-      <c r="F131" s="62"/>
-      <c r="G131" s="62"/>
-      <c r="H131" s="62"/>
-      <c r="I131" s="62"/>
-      <c r="J131" s="62"/>
-      <c r="K131" s="63"/>
-    </row>
-    <row r="132" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="33" t="s">
+      <c r="C135" s="55"/>
+      <c r="D135" s="55"/>
+      <c r="E135" s="55"/>
+      <c r="F135" s="55"/>
+      <c r="G135" s="55"/>
+      <c r="H135" s="55"/>
+      <c r="I135" s="55"/>
+      <c r="J135" s="55"/>
+      <c r="K135" s="56"/>
+    </row>
+    <row r="136" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B132" s="64" t="s">
+      <c r="B136" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C132" s="62"/>
-      <c r="D132" s="62"/>
-      <c r="E132" s="62"/>
-      <c r="F132" s="62"/>
-      <c r="G132" s="62"/>
-      <c r="H132" s="62"/>
-      <c r="I132" s="62"/>
-      <c r="J132" s="62"/>
-      <c r="K132" s="63"/>
-    </row>
-    <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A133" s="37"/>
-      <c r="B133" s="38"/>
-      <c r="C133" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D133" s="38"/>
-      <c r="E133" s="40"/>
-      <c r="F133" s="40"/>
-      <c r="G133" s="41"/>
-      <c r="H133" s="41"/>
-      <c r="I133" s="41">
-        <f t="shared" ref="I133:I143" si="13">H133-G133</f>
-        <v>0</v>
-      </c>
-      <c r="J133" s="45"/>
-      <c r="K133" s="43"/>
-    </row>
-    <row r="134" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A134" s="37"/>
-      <c r="B134" s="38"/>
-      <c r="C134" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D134" s="38"/>
-      <c r="E134" s="40"/>
-      <c r="F134" s="40"/>
-      <c r="G134" s="41"/>
-      <c r="H134" s="41"/>
-      <c r="I134" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J134" s="45"/>
-      <c r="K134" s="43"/>
-    </row>
-    <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A135" s="37"/>
-      <c r="B135" s="38"/>
-      <c r="C135" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D135" s="38"/>
-      <c r="E135" s="40"/>
-      <c r="F135" s="40"/>
-      <c r="G135" s="41"/>
-      <c r="H135" s="41"/>
-      <c r="I135" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J135" s="45"/>
-      <c r="K135" s="43"/>
-    </row>
-    <row r="136" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A136" s="37"/>
-      <c r="B136" s="38"/>
-      <c r="C136" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D136" s="38"/>
-      <c r="E136" s="40"/>
-      <c r="F136" s="40"/>
-      <c r="G136" s="41"/>
-      <c r="H136" s="41"/>
-      <c r="I136" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J136" s="45"/>
-      <c r="K136" s="43"/>
+      <c r="C136" s="55"/>
+      <c r="D136" s="55"/>
+      <c r="E136" s="55"/>
+      <c r="F136" s="55"/>
+      <c r="G136" s="55"/>
+      <c r="H136" s="55"/>
+      <c r="I136" s="55"/>
+      <c r="J136" s="55"/>
+      <c r="K136" s="56"/>
     </row>
     <row r="137" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A137" s="37"/>
@@ -4536,7 +4737,7 @@
       <c r="G137" s="41"/>
       <c r="H137" s="41"/>
       <c r="I137" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="I137:I147" si="13">H137-G137</f>
         <v>0</v>
       </c>
       <c r="J137" s="45"/>
@@ -4633,35 +4834,107 @@
       <c r="K142" s="43"/>
     </row>
     <row r="143" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A143" s="48"/>
-      <c r="B143" s="49"/>
-      <c r="C143" s="49"/>
-      <c r="D143" s="49"/>
-      <c r="E143" s="49" t="s">
+      <c r="A143" s="37"/>
+      <c r="B143" s="38"/>
+      <c r="C143" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D143" s="38"/>
+      <c r="E143" s="40"/>
+      <c r="F143" s="40"/>
+      <c r="G143" s="41"/>
+      <c r="H143" s="41"/>
+      <c r="I143" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J143" s="45"/>
+      <c r="K143" s="43"/>
+    </row>
+    <row r="144" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A144" s="37"/>
+      <c r="B144" s="38"/>
+      <c r="C144" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D144" s="38"/>
+      <c r="E144" s="40"/>
+      <c r="F144" s="40"/>
+      <c r="G144" s="41"/>
+      <c r="H144" s="41"/>
+      <c r="I144" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J144" s="45"/>
+      <c r="K144" s="43"/>
+    </row>
+    <row r="145" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A145" s="37"/>
+      <c r="B145" s="38"/>
+      <c r="C145" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D145" s="38"/>
+      <c r="E145" s="40"/>
+      <c r="F145" s="40"/>
+      <c r="G145" s="41"/>
+      <c r="H145" s="41"/>
+      <c r="I145" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J145" s="45"/>
+      <c r="K145" s="43"/>
+    </row>
+    <row r="146" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A146" s="37"/>
+      <c r="B146" s="38"/>
+      <c r="C146" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D146" s="38"/>
+      <c r="E146" s="40"/>
+      <c r="F146" s="40"/>
+      <c r="G146" s="41"/>
+      <c r="H146" s="41"/>
+      <c r="I146" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J146" s="45"/>
+      <c r="K146" s="43"/>
+    </row>
+    <row r="147" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A147" s="48"/>
+      <c r="B147" s="49"/>
+      <c r="C147" s="49"/>
+      <c r="D147" s="49"/>
+      <c r="E147" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F143" s="49"/>
-      <c r="G143" s="50">
-        <f t="shared" ref="G143:H143" si="14">SUM(G133:G142)</f>
-        <v>0</v>
-      </c>
-      <c r="H143" s="50">
+      <c r="F147" s="49"/>
+      <c r="G147" s="50">
+        <f t="shared" ref="G147:H147" si="14">SUM(G137:G146)</f>
+        <v>0</v>
+      </c>
+      <c r="H147" s="50">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="I143" s="50">
+      <c r="I147" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J143" s="51"/>
-      <c r="K143" s="52"/>
+      <c r="J147" s="51"/>
+      <c r="K147" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{9400C8B7-216F-46C1-9400-EC89A2528798}">
+      <autoFilter ref="A1:K15" xr:uid="{636BFA57-7D4A-4230-A823-E879218B7A26}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -4672,93 +4945,93 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A130:K130"/>
-    <mergeCell ref="B131:K131"/>
-    <mergeCell ref="B132:K132"/>
+    <mergeCell ref="B107:K107"/>
+    <mergeCell ref="B108:K108"/>
+    <mergeCell ref="A120:K120"/>
+    <mergeCell ref="B80:K80"/>
+    <mergeCell ref="A92:K92"/>
+    <mergeCell ref="B93:K93"/>
+    <mergeCell ref="B94:K94"/>
+    <mergeCell ref="A106:K106"/>
+    <mergeCell ref="A134:K134"/>
+    <mergeCell ref="B135:K135"/>
+    <mergeCell ref="B136:K136"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="A46:K46"/>
     <mergeCell ref="B47:K47"/>
     <mergeCell ref="B48:K48"/>
-    <mergeCell ref="A60:K60"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="B62:K62"/>
-    <mergeCell ref="A74:K74"/>
-    <mergeCell ref="B117:K117"/>
-    <mergeCell ref="B118:K118"/>
-    <mergeCell ref="B75:K75"/>
-    <mergeCell ref="B103:K103"/>
-    <mergeCell ref="B104:K104"/>
-    <mergeCell ref="A116:K116"/>
-    <mergeCell ref="B76:K76"/>
-    <mergeCell ref="A88:K88"/>
-    <mergeCell ref="B89:K89"/>
-    <mergeCell ref="B90:K90"/>
-    <mergeCell ref="A102:K102"/>
+    <mergeCell ref="A64:K64"/>
+    <mergeCell ref="B65:K65"/>
+    <mergeCell ref="B66:K66"/>
+    <mergeCell ref="A78:K78"/>
+    <mergeCell ref="B121:K121"/>
+    <mergeCell ref="B122:K122"/>
+    <mergeCell ref="B79:K79"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B44 B47:B58 B63:B72 B77:B86 B91:B100 B105:B114 B119:B128">
-    <cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="Unplanned">
+  <conditionalFormatting sqref="B5:B44 B47:B62 B67:B76 B81:B90 B95:B104 B109:B118 B123:B132">
+    <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="7" operator="containsText" text="Planned">
+    <cfRule type="containsText" dxfId="14" priority="7" operator="containsText" text="Planned">
       <formula>NOT(ISERROR(SEARCH(("Planned"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="8" operator="containsText" text="In-Progress">
+    <cfRule type="containsText" dxfId="13" priority="8" operator="containsText" text="In-Progress">
       <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="9" operator="containsText" text="Blocked">
+    <cfRule type="containsText" dxfId="12" priority="9" operator="containsText" text="Blocked">
       <formula>NOT(ISERROR(SEARCH(("Blocked"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="10" operator="containsText" text="Done">
+    <cfRule type="containsText" dxfId="11" priority="10" operator="containsText" text="Done">
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B45 B47:B59 B61:B73 B75:B87 B89:B101 B103:B115 B117:B129 B131:B143">
-    <cfRule type="containsText" dxfId="12" priority="11" operator="containsText" text="Unplanned">
+  <conditionalFormatting sqref="B5:B45 B47:B63 B65:B77 B79:B91 B93:B105 B107:B119 B121:B133 B135:B147">
+    <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="12" operator="containsText" text="Cancelled">
+    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="Cancelled">
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B133:B142">
-    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B133))))</formula>
+  <conditionalFormatting sqref="B137:B146">
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B137))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B133))))</formula>
+    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B137))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B133))))</formula>
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B137))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B133))))</formula>
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B137))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B133))))</formula>
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B137))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G45 G49:G59 G63:G73 G77:G87 G91:G101 G105:G115 G119:G129 G133:G143">
-    <cfRule type="cellIs" dxfId="5" priority="15" operator="greaterThan">
+  <conditionalFormatting sqref="G1 G3:G45 G49:G63 G67:G77 G81:G91 G95:G105 G109:G119 G123:G133 G137:G147">
+    <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H143">
-    <cfRule type="containsBlanks" dxfId="4" priority="16">
+  <conditionalFormatting sqref="H1:H147">
+    <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I49:I59 I63:I73 I77:I87 I91:I101 I105:I115 I119:I129 I133:I143 I5:I45">
-    <cfRule type="expression" dxfId="3" priority="13">
+  <conditionalFormatting sqref="I5:I45 I67:I77 I81:I91 I95:I105 I109:I119 I123:I133 I137:I147 I49:I63">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="14">
+    <cfRule type="expression" dxfId="0" priority="14">
       <formula>H5/G5&lt;=0.5</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F133:F142 F119:F128 F49:F58 F63:F72 F77:F86 F91:F100 F105:F114 F5:F44" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F137:F146 F123:F132 F49:F62 F67:F76 F81:F90 F95:F104 F109:F118 F5:F44" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4774,13 +5047,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E44 E49:E58 E63:E72 E77:E86 E91:E100 E105:E114 E119:E128 E133:E142</xm:sqref>
+          <xm:sqref>E5:E44 E49:E62 E67:E76 E81:E90 E95:E104 E109:E118 E123:E132 E137:E146</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B44 B49:B58 B63:B72 B77:B86 B91:B100 B105:B114 B119:B128 B133:B142</xm:sqref>
+          <xm:sqref>B5:B44 B49:B62 B67:B76 B81:B90 B95:B104 B109:B118 B123:B132 B137:B146</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4860,7 +5133,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" cm="1">
-        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$49:$H$58,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
+        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$49:$H$62,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" cm="1">
@@ -5213,58 +5486,58 @@
       <c r="K13" s="17"/>
     </row>
     <row r="14" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="75" t="s">
+      <c r="B14" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="76"/>
-      <c r="D14" s="76"/>
-      <c r="E14" s="76"/>
-      <c r="F14" s="76"/>
-      <c r="G14" s="76"/>
-      <c r="H14" s="76"/>
-      <c r="I14" s="76"/>
-      <c r="J14" s="76"/>
-      <c r="K14" s="76"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="77"/>
+      <c r="K14" s="77"/>
     </row>
     <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="9"/>
     </row>
     <row r="19" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="77" t="s">
+      <c r="B19" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="77"/>
-      <c r="D19" s="77"/>
-      <c r="E19" s="77"/>
-      <c r="F19" s="77"/>
+      <c r="C19" s="78"/>
+      <c r="D19" s="78"/>
+      <c r="E19" s="78"/>
+      <c r="F19" s="78"/>
     </row>
     <row r="20" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="77"/>
-      <c r="C20" s="77"/>
-      <c r="D20" s="77"/>
-      <c r="E20" s="77"/>
-      <c r="F20" s="77"/>
+      <c r="B20" s="78"/>
+      <c r="C20" s="78"/>
+      <c r="D20" s="78"/>
+      <c r="E20" s="78"/>
+      <c r="F20" s="78"/>
     </row>
     <row r="21" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="77"/>
-      <c r="C21" s="77"/>
-      <c r="D21" s="77"/>
-      <c r="E21" s="77"/>
-      <c r="F21" s="77"/>
+      <c r="B21" s="78"/>
+      <c r="C21" s="78"/>
+      <c r="D21" s="78"/>
+      <c r="E21" s="78"/>
+      <c r="F21" s="78"/>
     </row>
     <row r="22" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="77"/>
-      <c r="C22" s="77"/>
-      <c r="D22" s="77"/>
-      <c r="E22" s="77"/>
-      <c r="F22" s="77"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="78"/>
+      <c r="D22" s="78"/>
+      <c r="E22" s="78"/>
+      <c r="F22" s="78"/>
     </row>
     <row r="23" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="77"/>
-      <c r="C23" s="77"/>
-      <c r="D23" s="77"/>
-      <c r="E23" s="77"/>
-      <c r="F23" s="77"/>
+      <c r="B23" s="78"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6421,26 +6694,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -6675,10 +6928,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6695,20 +6979,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W2 Datalab 1 Work II
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4891ABE2-D5A5-4345-8106-B6EF0DE7CD63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{049651C3-8AE2-40D4-8B72-08F808D3B87B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$45</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$132</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$134</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$45</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="139">
   <si>
     <t>Date</t>
   </si>
@@ -491,9 +491,6 @@
     <t>Stand-up meeting Week 2 Datalab 1</t>
   </si>
   <si>
-    <t>EDA with Python (split this up)</t>
-  </si>
-  <si>
     <t>Re-Install all the Python packages</t>
   </si>
   <si>
@@ -504,6 +501,24 @@
   </si>
   <si>
     <t>Learn Seaborn</t>
+  </si>
+  <si>
+    <t>Install Seaborn for a 3rd time</t>
+  </si>
+  <si>
+    <t>Despite installing the package twice already, VSC could not import it.</t>
+  </si>
+  <si>
+    <t>Restart Laptop due to issues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some features of my laptop were acting up a bit, so I restarted my pc to fix them. </t>
+  </si>
+  <si>
+    <t>Unfortunately, during this task the annoucement came in, which threw me off my focus and caused this task to take so long.</t>
+  </si>
+  <si>
+    <t>EDA with Python</t>
   </si>
 </sst>
 </file>
@@ -1514,7 +1529,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K147"/>
+  <dimension ref="A1:K149"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -2981,7 +2996,7 @@
         <v>0.5</v>
       </c>
       <c r="I49" s="41">
-        <f t="shared" ref="I49:I63" si="1">H49-G49</f>
+        <f t="shared" ref="I49:I65" si="1">H49-G49</f>
         <v>0</v>
       </c>
       <c r="J49" s="45"/>
@@ -3254,7 +3269,7 @@
         <v>17</v>
       </c>
       <c r="D58" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E58" s="40" t="s">
         <v>50</v>
@@ -3274,7 +3289,7 @@
       </c>
       <c r="J58" s="45"/>
       <c r="K58" s="43" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -3282,13 +3297,13 @@
         <v>45622</v>
       </c>
       <c r="B59" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C59" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D59" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E59" s="40" t="s">
         <v>67</v>
@@ -3299,10 +3314,12 @@
       <c r="G59" s="41">
         <v>0.5</v>
       </c>
-      <c r="H59" s="41"/>
+      <c r="H59" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I59" s="41">
         <f t="shared" si="1"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J59" s="45"/>
       <c r="K59" s="43"/>
@@ -3312,13 +3329,13 @@
         <v>45622</v>
       </c>
       <c r="B60" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C60" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D60" s="38" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E60" s="40" t="s">
         <v>67</v>
@@ -3329,26 +3346,30 @@
       <c r="G60" s="41">
         <v>0.5</v>
       </c>
-      <c r="H60" s="41"/>
+      <c r="H60" s="41">
+        <v>2.35</v>
+      </c>
       <c r="I60" s="41">
         <f t="shared" si="1"/>
-        <v>-0.5</v>
+        <v>1.85</v>
       </c>
       <c r="J60" s="45"/>
-      <c r="K60" s="43"/>
+      <c r="K60" s="43" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="61" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A61" s="47">
         <v>45622</v>
       </c>
       <c r="B61" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C61" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D61" s="38" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E61" s="40" t="s">
         <v>50</v>
@@ -3357,97 +3378,133 @@
         <v>109</v>
       </c>
       <c r="G61" s="41">
-        <v>6.5</v>
-      </c>
-      <c r="H61" s="41"/>
+        <v>0.1</v>
+      </c>
+      <c r="H61" s="41">
+        <v>0.1</v>
+      </c>
       <c r="I61" s="41">
         <f t="shared" si="1"/>
-        <v>-6.5</v>
+        <v>0</v>
       </c>
       <c r="J61" s="45"/>
-      <c r="K61" s="43"/>
+      <c r="K61" s="43" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="62" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A62" s="47"/>
-      <c r="B62" s="38"/>
+      <c r="A62" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B62" s="38" t="s">
+        <v>46</v>
+      </c>
       <c r="C62" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D62" s="38"/>
-      <c r="E62" s="40"/>
-      <c r="F62" s="40"/>
-      <c r="G62" s="41"/>
-      <c r="H62" s="41"/>
+      <c r="D62" s="38" t="s">
+        <v>135</v>
+      </c>
+      <c r="E62" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="F62" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G62" s="41">
+        <v>0</v>
+      </c>
+      <c r="H62" s="41">
+        <v>0.1</v>
+      </c>
       <c r="I62" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J62" s="45"/>
-      <c r="K62" s="43"/>
+      <c r="K62" s="43" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="63" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A63" s="13"/>
-      <c r="B63" s="15"/>
-      <c r="C63" s="15"/>
-      <c r="D63" s="15"/>
-      <c r="E63" s="15" t="s">
+      <c r="A63" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B63" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C63" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D63" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="E63" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F63" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G63" s="41">
+        <v>4</v>
+      </c>
+      <c r="H63" s="41">
+        <v>3.55</v>
+      </c>
+      <c r="I63" s="41">
+        <f t="shared" si="1"/>
+        <v>-0.45000000000000018</v>
+      </c>
+      <c r="J63" s="45"/>
+      <c r="K63" s="43"/>
+    </row>
+    <row r="64" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A64" s="47"/>
+      <c r="B64" s="38"/>
+      <c r="C64" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D64" s="38"/>
+      <c r="E64" s="40"/>
+      <c r="F64" s="40"/>
+      <c r="G64" s="41"/>
+      <c r="H64" s="41"/>
+      <c r="I64" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J64" s="45"/>
+      <c r="K64" s="43"/>
+    </row>
+    <row r="65" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A65" s="13"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F63" s="15"/>
-      <c r="G63" s="18">
-        <f t="shared" ref="G63:H63" si="2">SUM(G47:G62)</f>
-        <v>17.25</v>
-      </c>
-      <c r="H63" s="18">
+      <c r="F65" s="15"/>
+      <c r="G65" s="18">
+        <f t="shared" ref="G65:H65" si="2">SUM(G47:G64)</f>
+        <v>14.85</v>
+      </c>
+      <c r="H65" s="18">
         <f t="shared" si="2"/>
-        <v>9.75</v>
-      </c>
-      <c r="I63" s="18">
+        <v>16.349999999999998</v>
+      </c>
+      <c r="I65" s="18">
         <f t="shared" si="1"/>
-        <v>-7.5</v>
-      </c>
-      <c r="J63" s="19"/>
-      <c r="K63" s="46"/>
-    </row>
-    <row r="64" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="66" t="s">
+        <v>1.4999999999999982</v>
+      </c>
+      <c r="J65" s="19"/>
+      <c r="K65" s="46"/>
+    </row>
+    <row r="66" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B64" s="62"/>
-      <c r="C64" s="62"/>
-      <c r="D64" s="62"/>
-      <c r="E64" s="62"/>
-      <c r="F64" s="62"/>
-      <c r="G64" s="62"/>
-      <c r="H64" s="62"/>
-      <c r="I64" s="62"/>
-      <c r="J64" s="62"/>
-      <c r="K64" s="63"/>
-    </row>
-    <row r="65" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A65" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B65" s="67" t="s">
-        <v>13</v>
-      </c>
-      <c r="C65" s="62"/>
-      <c r="D65" s="62"/>
-      <c r="E65" s="62"/>
-      <c r="F65" s="62"/>
-      <c r="G65" s="62"/>
-      <c r="H65" s="62"/>
-      <c r="I65" s="62"/>
-      <c r="J65" s="62"/>
-      <c r="K65" s="63"/>
-    </row>
-    <row r="66" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B66" s="67" t="s">
-        <v>15</v>
-      </c>
+      <c r="B66" s="62"/>
       <c r="C66" s="62"/>
       <c r="D66" s="62"/>
       <c r="E66" s="62"/>
@@ -3459,40 +3516,38 @@
       <c r="K66" s="63"/>
     </row>
     <row r="67" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A67" s="37"/>
-      <c r="B67" s="38"/>
-      <c r="C67" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D67" s="38"/>
-      <c r="E67" s="40"/>
-      <c r="F67" s="40"/>
-      <c r="G67" s="41"/>
-      <c r="H67" s="41"/>
-      <c r="I67" s="41">
-        <f t="shared" ref="I67:I77" si="3">H67-G67</f>
-        <v>0</v>
-      </c>
-      <c r="J67" s="45"/>
-      <c r="K67" s="43"/>
-    </row>
-    <row r="68" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A68" s="37"/>
-      <c r="B68" s="38"/>
-      <c r="C68" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D68" s="38"/>
-      <c r="E68" s="40"/>
-      <c r="F68" s="40"/>
-      <c r="G68" s="41"/>
-      <c r="H68" s="41"/>
-      <c r="I68" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J68" s="45"/>
-      <c r="K68" s="43"/>
+      <c r="A67" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B67" s="67" t="s">
+        <v>13</v>
+      </c>
+      <c r="C67" s="62"/>
+      <c r="D67" s="62"/>
+      <c r="E67" s="62"/>
+      <c r="F67" s="62"/>
+      <c r="G67" s="62"/>
+      <c r="H67" s="62"/>
+      <c r="I67" s="62"/>
+      <c r="J67" s="62"/>
+      <c r="K67" s="63"/>
+    </row>
+    <row r="68" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B68" s="67" t="s">
+        <v>15</v>
+      </c>
+      <c r="C68" s="62"/>
+      <c r="D68" s="62"/>
+      <c r="E68" s="62"/>
+      <c r="F68" s="62"/>
+      <c r="G68" s="62"/>
+      <c r="H68" s="62"/>
+      <c r="I68" s="62"/>
+      <c r="J68" s="62"/>
+      <c r="K68" s="63"/>
     </row>
     <row r="69" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A69" s="37"/>
@@ -3506,7 +3561,7 @@
       <c r="G69" s="41"/>
       <c r="H69" s="41"/>
       <c r="I69" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="I69:I79" si="3">H69-G69</f>
         <v>0</v>
       </c>
       <c r="J69" s="45"/>
@@ -3639,68 +3694,70 @@
       <c r="K76" s="43"/>
     </row>
     <row r="77" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A77" s="13"/>
-      <c r="B77" s="15"/>
-      <c r="C77" s="15"/>
-      <c r="D77" s="15"/>
-      <c r="E77" s="15" t="s">
+      <c r="A77" s="37"/>
+      <c r="B77" s="38"/>
+      <c r="C77" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D77" s="38"/>
+      <c r="E77" s="40"/>
+      <c r="F77" s="40"/>
+      <c r="G77" s="41"/>
+      <c r="H77" s="41"/>
+      <c r="I77" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J77" s="45"/>
+      <c r="K77" s="43"/>
+    </row>
+    <row r="78" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A78" s="37"/>
+      <c r="B78" s="38"/>
+      <c r="C78" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D78" s="38"/>
+      <c r="E78" s="40"/>
+      <c r="F78" s="40"/>
+      <c r="G78" s="41"/>
+      <c r="H78" s="41"/>
+      <c r="I78" s="41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J78" s="45"/>
+      <c r="K78" s="43"/>
+    </row>
+    <row r="79" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A79" s="13"/>
+      <c r="B79" s="15"/>
+      <c r="C79" s="15"/>
+      <c r="D79" s="15"/>
+      <c r="E79" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F77" s="15"/>
-      <c r="G77" s="18">
-        <f t="shared" ref="G77:H77" si="4">SUM(G67:G76)</f>
-        <v>0</v>
-      </c>
-      <c r="H77" s="18">
+      <c r="F79" s="15"/>
+      <c r="G79" s="18">
+        <f t="shared" ref="G79:H79" si="4">SUM(G69:G78)</f>
+        <v>0</v>
+      </c>
+      <c r="H79" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="I77" s="18">
+      <c r="I79" s="18">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J77" s="19"/>
-      <c r="K77" s="46"/>
-    </row>
-    <row r="78" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="68" t="s">
+      <c r="J79" s="19"/>
+      <c r="K79" s="46"/>
+    </row>
+    <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B78" s="62"/>
-      <c r="C78" s="62"/>
-      <c r="D78" s="62"/>
-      <c r="E78" s="62"/>
-      <c r="F78" s="62"/>
-      <c r="G78" s="62"/>
-      <c r="H78" s="62"/>
-      <c r="I78" s="62"/>
-      <c r="J78" s="62"/>
-      <c r="K78" s="63"/>
-    </row>
-    <row r="79" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A79" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B79" s="70" t="s">
-        <v>13</v>
-      </c>
-      <c r="C79" s="62"/>
-      <c r="D79" s="62"/>
-      <c r="E79" s="62"/>
-      <c r="F79" s="62"/>
-      <c r="G79" s="62"/>
-      <c r="H79" s="62"/>
-      <c r="I79" s="62"/>
-      <c r="J79" s="62"/>
-      <c r="K79" s="63"/>
-    </row>
-    <row r="80" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B80" s="70" t="s">
-        <v>15</v>
-      </c>
+      <c r="B80" s="62"/>
       <c r="C80" s="62"/>
       <c r="D80" s="62"/>
       <c r="E80" s="62"/>
@@ -3712,40 +3769,38 @@
       <c r="K80" s="63"/>
     </row>
     <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A81" s="37"/>
-      <c r="B81" s="38"/>
-      <c r="C81" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D81" s="38"/>
-      <c r="E81" s="40"/>
-      <c r="F81" s="40"/>
-      <c r="G81" s="41"/>
-      <c r="H81" s="41"/>
-      <c r="I81" s="41">
-        <f t="shared" ref="I81:I91" si="5">H81-G81</f>
-        <v>0</v>
-      </c>
-      <c r="J81" s="45"/>
-      <c r="K81" s="43"/>
-    </row>
-    <row r="82" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A82" s="37"/>
-      <c r="B82" s="38"/>
-      <c r="C82" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D82" s="38"/>
-      <c r="E82" s="40"/>
-      <c r="F82" s="40"/>
-      <c r="G82" s="41"/>
-      <c r="H82" s="41"/>
-      <c r="I82" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J82" s="45"/>
-      <c r="K82" s="43"/>
+      <c r="A81" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B81" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="C81" s="62"/>
+      <c r="D81" s="62"/>
+      <c r="E81" s="62"/>
+      <c r="F81" s="62"/>
+      <c r="G81" s="62"/>
+      <c r="H81" s="62"/>
+      <c r="I81" s="62"/>
+      <c r="J81" s="62"/>
+      <c r="K81" s="63"/>
+    </row>
+    <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B82" s="70" t="s">
+        <v>15</v>
+      </c>
+      <c r="C82" s="62"/>
+      <c r="D82" s="62"/>
+      <c r="E82" s="62"/>
+      <c r="F82" s="62"/>
+      <c r="G82" s="62"/>
+      <c r="H82" s="62"/>
+      <c r="I82" s="62"/>
+      <c r="J82" s="62"/>
+      <c r="K82" s="63"/>
     </row>
     <row r="83" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A83" s="37"/>
@@ -3759,7 +3814,7 @@
       <c r="G83" s="41"/>
       <c r="H83" s="41"/>
       <c r="I83" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I83:I93" si="5">H83-G83</f>
         <v>0</v>
       </c>
       <c r="J83" s="45"/>
@@ -3892,68 +3947,70 @@
       <c r="K90" s="43"/>
     </row>
     <row r="91" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A91" s="13"/>
-      <c r="B91" s="15"/>
-      <c r="C91" s="15"/>
-      <c r="D91" s="15"/>
-      <c r="E91" s="15" t="s">
+      <c r="A91" s="37"/>
+      <c r="B91" s="38"/>
+      <c r="C91" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D91" s="38"/>
+      <c r="E91" s="40"/>
+      <c r="F91" s="40"/>
+      <c r="G91" s="41"/>
+      <c r="H91" s="41"/>
+      <c r="I91" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J91" s="45"/>
+      <c r="K91" s="43"/>
+    </row>
+    <row r="92" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A92" s="37"/>
+      <c r="B92" s="38"/>
+      <c r="C92" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D92" s="38"/>
+      <c r="E92" s="40"/>
+      <c r="F92" s="40"/>
+      <c r="G92" s="41"/>
+      <c r="H92" s="41"/>
+      <c r="I92" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J92" s="45"/>
+      <c r="K92" s="43"/>
+    </row>
+    <row r="93" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A93" s="13"/>
+      <c r="B93" s="15"/>
+      <c r="C93" s="15"/>
+      <c r="D93" s="15"/>
+      <c r="E93" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F91" s="15"/>
-      <c r="G91" s="18">
-        <f t="shared" ref="G91:H91" si="6">SUM(G81:G90)</f>
-        <v>0</v>
-      </c>
-      <c r="H91" s="18">
+      <c r="F93" s="15"/>
+      <c r="G93" s="18">
+        <f t="shared" ref="G93:H93" si="6">SUM(G83:G92)</f>
+        <v>0</v>
+      </c>
+      <c r="H93" s="18">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="I91" s="18">
+      <c r="I93" s="18">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J91" s="19"/>
-      <c r="K91" s="46"/>
-    </row>
-    <row r="92" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="73" t="s">
+      <c r="J93" s="19"/>
+      <c r="K93" s="46"/>
+    </row>
+    <row r="94" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B92" s="62"/>
-      <c r="C92" s="62"/>
-      <c r="D92" s="62"/>
-      <c r="E92" s="62"/>
-      <c r="F92" s="62"/>
-      <c r="G92" s="62"/>
-      <c r="H92" s="62"/>
-      <c r="I92" s="62"/>
-      <c r="J92" s="62"/>
-      <c r="K92" s="63"/>
-    </row>
-    <row r="93" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A93" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B93" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="C93" s="62"/>
-      <c r="D93" s="62"/>
-      <c r="E93" s="62"/>
-      <c r="F93" s="62"/>
-      <c r="G93" s="62"/>
-      <c r="H93" s="62"/>
-      <c r="I93" s="62"/>
-      <c r="J93" s="62"/>
-      <c r="K93" s="63"/>
-    </row>
-    <row r="94" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="B94" s="74" t="s">
-        <v>15</v>
-      </c>
+      <c r="B94" s="62"/>
       <c r="C94" s="62"/>
       <c r="D94" s="62"/>
       <c r="E94" s="62"/>
@@ -3965,40 +4022,38 @@
       <c r="K94" s="63"/>
     </row>
     <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A95" s="37"/>
-      <c r="B95" s="38"/>
-      <c r="C95" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D95" s="38"/>
-      <c r="E95" s="40"/>
-      <c r="F95" s="40"/>
-      <c r="G95" s="41"/>
-      <c r="H95" s="41"/>
-      <c r="I95" s="41">
-        <f t="shared" ref="I95:I105" si="7">H95-G95</f>
-        <v>0</v>
-      </c>
-      <c r="J95" s="45"/>
-      <c r="K95" s="43"/>
-    </row>
-    <row r="96" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A96" s="37"/>
-      <c r="B96" s="38"/>
-      <c r="C96" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D96" s="38"/>
-      <c r="E96" s="40"/>
-      <c r="F96" s="40"/>
-      <c r="G96" s="41"/>
-      <c r="H96" s="41"/>
-      <c r="I96" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J96" s="45"/>
-      <c r="K96" s="43"/>
+      <c r="A95" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B95" s="74" t="s">
+        <v>13</v>
+      </c>
+      <c r="C95" s="62"/>
+      <c r="D95" s="62"/>
+      <c r="E95" s="62"/>
+      <c r="F95" s="62"/>
+      <c r="G95" s="62"/>
+      <c r="H95" s="62"/>
+      <c r="I95" s="62"/>
+      <c r="J95" s="62"/>
+      <c r="K95" s="63"/>
+    </row>
+    <row r="96" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B96" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="C96" s="62"/>
+      <c r="D96" s="62"/>
+      <c r="E96" s="62"/>
+      <c r="F96" s="62"/>
+      <c r="G96" s="62"/>
+      <c r="H96" s="62"/>
+      <c r="I96" s="62"/>
+      <c r="J96" s="62"/>
+      <c r="K96" s="63"/>
     </row>
     <row r="97" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A97" s="37"/>
@@ -4012,7 +4067,7 @@
       <c r="G97" s="41"/>
       <c r="H97" s="41"/>
       <c r="I97" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="I97:I107" si="7">H97-G97</f>
         <v>0</v>
       </c>
       <c r="J97" s="45"/>
@@ -4145,68 +4200,70 @@
       <c r="K104" s="43"/>
     </row>
     <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A105" s="13"/>
-      <c r="B105" s="15"/>
-      <c r="C105" s="15"/>
-      <c r="D105" s="15"/>
-      <c r="E105" s="15" t="s">
+      <c r="A105" s="37"/>
+      <c r="B105" s="38"/>
+      <c r="C105" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D105" s="38"/>
+      <c r="E105" s="40"/>
+      <c r="F105" s="40"/>
+      <c r="G105" s="41"/>
+      <c r="H105" s="41"/>
+      <c r="I105" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J105" s="45"/>
+      <c r="K105" s="43"/>
+    </row>
+    <row r="106" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A106" s="37"/>
+      <c r="B106" s="38"/>
+      <c r="C106" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D106" s="38"/>
+      <c r="E106" s="40"/>
+      <c r="F106" s="40"/>
+      <c r="G106" s="41"/>
+      <c r="H106" s="41"/>
+      <c r="I106" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J106" s="45"/>
+      <c r="K106" s="43"/>
+    </row>
+    <row r="107" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A107" s="13"/>
+      <c r="B107" s="15"/>
+      <c r="C107" s="15"/>
+      <c r="D107" s="15"/>
+      <c r="E107" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F105" s="15"/>
-      <c r="G105" s="18">
-        <f t="shared" ref="G105:H105" si="8">SUM(G95:G104)</f>
-        <v>0</v>
-      </c>
-      <c r="H105" s="18">
+      <c r="F107" s="15"/>
+      <c r="G107" s="18">
+        <f t="shared" ref="G107:H107" si="8">SUM(G97:G106)</f>
+        <v>0</v>
+      </c>
+      <c r="H107" s="18">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="I105" s="18">
+      <c r="I107" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J105" s="19"/>
-      <c r="K105" s="46"/>
-    </row>
-    <row r="106" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="75" t="s">
+      <c r="J107" s="19"/>
+      <c r="K107" s="46"/>
+    </row>
+    <row r="108" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B106" s="62"/>
-      <c r="C106" s="62"/>
-      <c r="D106" s="62"/>
-      <c r="E106" s="62"/>
-      <c r="F106" s="62"/>
-      <c r="G106" s="62"/>
-      <c r="H106" s="62"/>
-      <c r="I106" s="62"/>
-      <c r="J106" s="62"/>
-      <c r="K106" s="63"/>
-    </row>
-    <row r="107" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A107" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B107" s="71" t="s">
-        <v>13</v>
-      </c>
-      <c r="C107" s="62"/>
-      <c r="D107" s="62"/>
-      <c r="E107" s="62"/>
-      <c r="F107" s="62"/>
-      <c r="G107" s="62"/>
-      <c r="H107" s="62"/>
-      <c r="I107" s="62"/>
-      <c r="J107" s="62"/>
-      <c r="K107" s="63"/>
-    </row>
-    <row r="108" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B108" s="71" t="s">
-        <v>15</v>
-      </c>
+      <c r="B108" s="62"/>
       <c r="C108" s="62"/>
       <c r="D108" s="62"/>
       <c r="E108" s="62"/>
@@ -4218,40 +4275,38 @@
       <c r="K108" s="63"/>
     </row>
     <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A109" s="37"/>
-      <c r="B109" s="38"/>
-      <c r="C109" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D109" s="38"/>
-      <c r="E109" s="40"/>
-      <c r="F109" s="40"/>
-      <c r="G109" s="41"/>
-      <c r="H109" s="41"/>
-      <c r="I109" s="41">
-        <f t="shared" ref="I109:I119" si="9">H109-G109</f>
-        <v>0</v>
-      </c>
-      <c r="J109" s="45"/>
-      <c r="K109" s="43"/>
-    </row>
-    <row r="110" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A110" s="37"/>
-      <c r="B110" s="38"/>
-      <c r="C110" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D110" s="38"/>
-      <c r="E110" s="40"/>
-      <c r="F110" s="40"/>
-      <c r="G110" s="41"/>
-      <c r="H110" s="41"/>
-      <c r="I110" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J110" s="45"/>
-      <c r="K110" s="43"/>
+      <c r="A109" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B109" s="71" t="s">
+        <v>13</v>
+      </c>
+      <c r="C109" s="62"/>
+      <c r="D109" s="62"/>
+      <c r="E109" s="62"/>
+      <c r="F109" s="62"/>
+      <c r="G109" s="62"/>
+      <c r="H109" s="62"/>
+      <c r="I109" s="62"/>
+      <c r="J109" s="62"/>
+      <c r="K109" s="63"/>
+    </row>
+    <row r="110" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B110" s="71" t="s">
+        <v>15</v>
+      </c>
+      <c r="C110" s="62"/>
+      <c r="D110" s="62"/>
+      <c r="E110" s="62"/>
+      <c r="F110" s="62"/>
+      <c r="G110" s="62"/>
+      <c r="H110" s="62"/>
+      <c r="I110" s="62"/>
+      <c r="J110" s="62"/>
+      <c r="K110" s="63"/>
     </row>
     <row r="111" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A111" s="37"/>
@@ -4265,13 +4320,11 @@
       <c r="G111" s="41"/>
       <c r="H111" s="41"/>
       <c r="I111" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I111:I121" si="9">H111-G111</f>
         <v>0</v>
       </c>
       <c r="J111" s="45"/>
-      <c r="K111" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K111" s="43"/>
     </row>
     <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A112" s="37"/>
@@ -4307,7 +4360,9 @@
         <v>0</v>
       </c>
       <c r="J113" s="45"/>
-      <c r="K113" s="43"/>
+      <c r="K113" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A114" s="37"/>
@@ -4400,68 +4455,70 @@
       <c r="K118" s="43"/>
     </row>
     <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A119" s="13"/>
-      <c r="B119" s="15"/>
-      <c r="C119" s="15"/>
-      <c r="D119" s="15"/>
-      <c r="E119" s="15" t="s">
+      <c r="A119" s="37"/>
+      <c r="B119" s="38"/>
+      <c r="C119" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D119" s="38"/>
+      <c r="E119" s="40"/>
+      <c r="F119" s="40"/>
+      <c r="G119" s="41"/>
+      <c r="H119" s="41"/>
+      <c r="I119" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J119" s="45"/>
+      <c r="K119" s="43"/>
+    </row>
+    <row r="120" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A120" s="37"/>
+      <c r="B120" s="38"/>
+      <c r="C120" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D120" s="38"/>
+      <c r="E120" s="40"/>
+      <c r="F120" s="40"/>
+      <c r="G120" s="41"/>
+      <c r="H120" s="41"/>
+      <c r="I120" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J120" s="45"/>
+      <c r="K120" s="43"/>
+    </row>
+    <row r="121" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A121" s="13"/>
+      <c r="B121" s="15"/>
+      <c r="C121" s="15"/>
+      <c r="D121" s="15"/>
+      <c r="E121" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F119" s="15"/>
-      <c r="G119" s="18">
-        <f t="shared" ref="G119:H119" si="10">SUM(G109:G118)</f>
-        <v>0</v>
-      </c>
-      <c r="H119" s="18">
+      <c r="F121" s="15"/>
+      <c r="G121" s="18">
+        <f t="shared" ref="G121:H121" si="10">SUM(G111:G120)</f>
+        <v>0</v>
+      </c>
+      <c r="H121" s="18">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="I119" s="18">
+      <c r="I121" s="18">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J119" s="19"/>
-      <c r="K119" s="46"/>
-    </row>
-    <row r="120" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="72" t="s">
+      <c r="J121" s="19"/>
+      <c r="K121" s="46"/>
+    </row>
+    <row r="122" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="B120" s="62"/>
-      <c r="C120" s="62"/>
-      <c r="D120" s="62"/>
-      <c r="E120" s="62"/>
-      <c r="F120" s="62"/>
-      <c r="G120" s="62"/>
-      <c r="H120" s="62"/>
-      <c r="I120" s="62"/>
-      <c r="J120" s="62"/>
-      <c r="K120" s="63"/>
-    </row>
-    <row r="121" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A121" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B121" s="69" t="s">
-        <v>13</v>
-      </c>
-      <c r="C121" s="62"/>
-      <c r="D121" s="62"/>
-      <c r="E121" s="62"/>
-      <c r="F121" s="62"/>
-      <c r="G121" s="62"/>
-      <c r="H121" s="62"/>
-      <c r="I121" s="62"/>
-      <c r="J121" s="62"/>
-      <c r="K121" s="63"/>
-    </row>
-    <row r="122" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B122" s="69" t="s">
-        <v>15</v>
-      </c>
+      <c r="B122" s="62"/>
       <c r="C122" s="62"/>
       <c r="D122" s="62"/>
       <c r="E122" s="62"/>
@@ -4473,40 +4530,38 @@
       <c r="K122" s="63"/>
     </row>
     <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A123" s="37"/>
-      <c r="B123" s="38"/>
-      <c r="C123" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D123" s="38"/>
-      <c r="E123" s="40"/>
-      <c r="F123" s="40"/>
-      <c r="G123" s="41"/>
-      <c r="H123" s="41"/>
-      <c r="I123" s="41">
-        <f t="shared" ref="I123:I133" si="11">H123-G123</f>
-        <v>0</v>
-      </c>
-      <c r="J123" s="45"/>
-      <c r="K123" s="43"/>
-    </row>
-    <row r="124" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A124" s="37"/>
-      <c r="B124" s="38"/>
-      <c r="C124" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D124" s="38"/>
-      <c r="E124" s="40"/>
-      <c r="F124" s="40"/>
-      <c r="G124" s="41"/>
-      <c r="H124" s="41"/>
-      <c r="I124" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J124" s="45"/>
-      <c r="K124" s="43"/>
+      <c r="A123" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B123" s="69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C123" s="62"/>
+      <c r="D123" s="62"/>
+      <c r="E123" s="62"/>
+      <c r="F123" s="62"/>
+      <c r="G123" s="62"/>
+      <c r="H123" s="62"/>
+      <c r="I123" s="62"/>
+      <c r="J123" s="62"/>
+      <c r="K123" s="63"/>
+    </row>
+    <row r="124" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B124" s="69" t="s">
+        <v>15</v>
+      </c>
+      <c r="C124" s="62"/>
+      <c r="D124" s="62"/>
+      <c r="E124" s="62"/>
+      <c r="F124" s="62"/>
+      <c r="G124" s="62"/>
+      <c r="H124" s="62"/>
+      <c r="I124" s="62"/>
+      <c r="J124" s="62"/>
+      <c r="K124" s="63"/>
     </row>
     <row r="125" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A125" s="37"/>
@@ -4520,7 +4575,7 @@
       <c r="G125" s="41"/>
       <c r="H125" s="41"/>
       <c r="I125" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="I125:I135" si="11">H125-G125</f>
         <v>0</v>
       </c>
       <c r="J125" s="45"/>
@@ -4653,68 +4708,70 @@
       <c r="K132" s="43"/>
     </row>
     <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A133" s="13"/>
-      <c r="B133" s="15"/>
-      <c r="C133" s="15"/>
-      <c r="D133" s="15"/>
-      <c r="E133" s="15" t="s">
+      <c r="A133" s="37"/>
+      <c r="B133" s="38"/>
+      <c r="C133" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D133" s="38"/>
+      <c r="E133" s="40"/>
+      <c r="F133" s="40"/>
+      <c r="G133" s="41"/>
+      <c r="H133" s="41"/>
+      <c r="I133" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J133" s="45"/>
+      <c r="K133" s="43"/>
+    </row>
+    <row r="134" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A134" s="37"/>
+      <c r="B134" s="38"/>
+      <c r="C134" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D134" s="38"/>
+      <c r="E134" s="40"/>
+      <c r="F134" s="40"/>
+      <c r="G134" s="41"/>
+      <c r="H134" s="41"/>
+      <c r="I134" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J134" s="45"/>
+      <c r="K134" s="43"/>
+    </row>
+    <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A135" s="13"/>
+      <c r="B135" s="15"/>
+      <c r="C135" s="15"/>
+      <c r="D135" s="15"/>
+      <c r="E135" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F133" s="15"/>
-      <c r="G133" s="18">
-        <f t="shared" ref="G133:H133" si="12">SUM(G123:G132)</f>
-        <v>0</v>
-      </c>
-      <c r="H133" s="18">
+      <c r="F135" s="15"/>
+      <c r="G135" s="18">
+        <f t="shared" ref="G135:H135" si="12">SUM(G125:G134)</f>
+        <v>0</v>
+      </c>
+      <c r="H135" s="18">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="I133" s="18">
+      <c r="I135" s="18">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J133" s="19"/>
-      <c r="K133" s="46"/>
-    </row>
-    <row r="134" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="54" t="s">
+      <c r="J135" s="19"/>
+      <c r="K135" s="46"/>
+    </row>
+    <row r="136" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B134" s="55"/>
-      <c r="C134" s="55"/>
-      <c r="D134" s="55"/>
-      <c r="E134" s="55"/>
-      <c r="F134" s="55"/>
-      <c r="G134" s="55"/>
-      <c r="H134" s="55"/>
-      <c r="I134" s="55"/>
-      <c r="J134" s="55"/>
-      <c r="K134" s="56"/>
-    </row>
-    <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A135" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B135" s="57" t="s">
-        <v>13</v>
-      </c>
-      <c r="C135" s="55"/>
-      <c r="D135" s="55"/>
-      <c r="E135" s="55"/>
-      <c r="F135" s="55"/>
-      <c r="G135" s="55"/>
-      <c r="H135" s="55"/>
-      <c r="I135" s="55"/>
-      <c r="J135" s="55"/>
-      <c r="K135" s="56"/>
-    </row>
-    <row r="136" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B136" s="57" t="s">
-        <v>15</v>
-      </c>
+      <c r="B136" s="55"/>
       <c r="C136" s="55"/>
       <c r="D136" s="55"/>
       <c r="E136" s="55"/>
@@ -4726,40 +4783,38 @@
       <c r="K136" s="56"/>
     </row>
     <row r="137" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A137" s="37"/>
-      <c r="B137" s="38"/>
-      <c r="C137" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D137" s="38"/>
-      <c r="E137" s="40"/>
-      <c r="F137" s="40"/>
-      <c r="G137" s="41"/>
-      <c r="H137" s="41"/>
-      <c r="I137" s="41">
-        <f t="shared" ref="I137:I147" si="13">H137-G137</f>
-        <v>0</v>
-      </c>
-      <c r="J137" s="45"/>
-      <c r="K137" s="43"/>
-    </row>
-    <row r="138" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A138" s="37"/>
-      <c r="B138" s="38"/>
-      <c r="C138" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D138" s="38"/>
-      <c r="E138" s="40"/>
-      <c r="F138" s="40"/>
-      <c r="G138" s="41"/>
-      <c r="H138" s="41"/>
-      <c r="I138" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J138" s="45"/>
-      <c r="K138" s="43"/>
+      <c r="A137" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B137" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C137" s="55"/>
+      <c r="D137" s="55"/>
+      <c r="E137" s="55"/>
+      <c r="F137" s="55"/>
+      <c r="G137" s="55"/>
+      <c r="H137" s="55"/>
+      <c r="I137" s="55"/>
+      <c r="J137" s="55"/>
+      <c r="K137" s="56"/>
+    </row>
+    <row r="138" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B138" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C138" s="55"/>
+      <c r="D138" s="55"/>
+      <c r="E138" s="55"/>
+      <c r="F138" s="55"/>
+      <c r="G138" s="55"/>
+      <c r="H138" s="55"/>
+      <c r="I138" s="55"/>
+      <c r="J138" s="55"/>
+      <c r="K138" s="56"/>
     </row>
     <row r="139" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A139" s="37"/>
@@ -4773,7 +4828,7 @@
       <c r="G139" s="41"/>
       <c r="H139" s="41"/>
       <c r="I139" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="I139:I149" si="13">H139-G139</f>
         <v>0</v>
       </c>
       <c r="J139" s="45"/>
@@ -4906,35 +4961,71 @@
       <c r="K146" s="43"/>
     </row>
     <row r="147" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A147" s="48"/>
-      <c r="B147" s="49"/>
-      <c r="C147" s="49"/>
-      <c r="D147" s="49"/>
-      <c r="E147" s="49" t="s">
+      <c r="A147" s="37"/>
+      <c r="B147" s="38"/>
+      <c r="C147" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D147" s="38"/>
+      <c r="E147" s="40"/>
+      <c r="F147" s="40"/>
+      <c r="G147" s="41"/>
+      <c r="H147" s="41"/>
+      <c r="I147" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J147" s="45"/>
+      <c r="K147" s="43"/>
+    </row>
+    <row r="148" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A148" s="37"/>
+      <c r="B148" s="38"/>
+      <c r="C148" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D148" s="38"/>
+      <c r="E148" s="40"/>
+      <c r="F148" s="40"/>
+      <c r="G148" s="41"/>
+      <c r="H148" s="41"/>
+      <c r="I148" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J148" s="45"/>
+      <c r="K148" s="43"/>
+    </row>
+    <row r="149" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A149" s="48"/>
+      <c r="B149" s="49"/>
+      <c r="C149" s="49"/>
+      <c r="D149" s="49"/>
+      <c r="E149" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F147" s="49"/>
-      <c r="G147" s="50">
-        <f t="shared" ref="G147:H147" si="14">SUM(G137:G146)</f>
-        <v>0</v>
-      </c>
-      <c r="H147" s="50">
+      <c r="F149" s="49"/>
+      <c r="G149" s="50">
+        <f t="shared" ref="G149:H149" si="14">SUM(G139:G148)</f>
+        <v>0</v>
+      </c>
+      <c r="H149" s="50">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="I147" s="50">
+      <c r="I149" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J147" s="51"/>
-      <c r="K147" s="52"/>
+      <c r="J149" s="51"/>
+      <c r="K149" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{636BFA57-7D4A-4230-A823-E879218B7A26}">
+      <autoFilter ref="A1:K15" xr:uid="{E618F7EC-EE6C-4EC9-803D-CB7D6E0706F7}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -4945,32 +5036,32 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B107:K107"/>
-    <mergeCell ref="B108:K108"/>
-    <mergeCell ref="A120:K120"/>
-    <mergeCell ref="B80:K80"/>
-    <mergeCell ref="A92:K92"/>
-    <mergeCell ref="B93:K93"/>
-    <mergeCell ref="B94:K94"/>
-    <mergeCell ref="A106:K106"/>
-    <mergeCell ref="A134:K134"/>
-    <mergeCell ref="B135:K135"/>
-    <mergeCell ref="B136:K136"/>
+    <mergeCell ref="B109:K109"/>
+    <mergeCell ref="B110:K110"/>
+    <mergeCell ref="A122:K122"/>
+    <mergeCell ref="B82:K82"/>
+    <mergeCell ref="A94:K94"/>
+    <mergeCell ref="B95:K95"/>
+    <mergeCell ref="B96:K96"/>
+    <mergeCell ref="A108:K108"/>
+    <mergeCell ref="A136:K136"/>
+    <mergeCell ref="B137:K137"/>
+    <mergeCell ref="B138:K138"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="A46:K46"/>
     <mergeCell ref="B47:K47"/>
     <mergeCell ref="B48:K48"/>
-    <mergeCell ref="A64:K64"/>
-    <mergeCell ref="B65:K65"/>
-    <mergeCell ref="B66:K66"/>
-    <mergeCell ref="A78:K78"/>
-    <mergeCell ref="B121:K121"/>
-    <mergeCell ref="B122:K122"/>
-    <mergeCell ref="B79:K79"/>
+    <mergeCell ref="A66:K66"/>
+    <mergeCell ref="B67:K67"/>
+    <mergeCell ref="B68:K68"/>
+    <mergeCell ref="A80:K80"/>
+    <mergeCell ref="B123:K123"/>
+    <mergeCell ref="B124:K124"/>
+    <mergeCell ref="B81:K81"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B44 B47:B62 B67:B76 B81:B90 B95:B104 B109:B118 B123:B132">
+  <conditionalFormatting sqref="B5:B44 B47:B64 B69:B78 B83:B92 B97:B106 B111:B120 B125:B134">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -4987,7 +5078,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B45 B47:B63 B65:B77 B79:B91 B93:B105 B107:B119 B121:B133 B135:B147">
+  <conditionalFormatting sqref="B5:B45 B47:B65 B67:B79 B81:B93 B95:B107 B109:B121 B123:B135 B137:B149">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -4995,34 +5086,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B137:B146">
+  <conditionalFormatting sqref="B139:B148">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B137))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B139))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B137))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B139))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B137))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B139))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B137))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B139))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B137))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B139))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G45 G49:G63 G67:G77 G81:G91 G95:G105 G109:G119 G123:G133 G137:G147">
+  <conditionalFormatting sqref="G1 G3:G45 G49:G65 G69:G79 G83:G93 G97:G107 G111:G121 G125:G135 G139:G149">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H147">
+  <conditionalFormatting sqref="H1:H149">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I45 I67:I77 I81:I91 I95:I105 I109:I119 I123:I133 I137:I147 I49:I63">
+  <conditionalFormatting sqref="I5:I45 I49:I65 I69:I79 I83:I93 I97:I107 I111:I121 I125:I135 I139:I149">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -5031,7 +5122,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F137:F146 F123:F132 F49:F62 F67:F76 F81:F90 F95:F104 F109:F118 F5:F44" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F139:F148 F125:F134 F49:F64 F69:F78 F83:F92 F97:F106 F111:F120 F5:F44" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5047,13 +5138,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E44 E49:E62 E67:E76 E81:E90 E95:E104 E109:E118 E123:E132 E137:E146</xm:sqref>
+          <xm:sqref>E5:E44 E49:E64 E69:E78 E83:E92 E97:E106 E111:E120 E125:E134 E139:E148</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B44 B49:B62 B67:B76 B81:B90 B95:B104 B109:B118 B123:B132 B137:B146</xm:sqref>
+          <xm:sqref>B5:B44 B49:B64 B69:B78 B83:B92 B97:B106 B111:B120 B125:B134 B139:B148</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5133,7 +5224,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" cm="1">
-        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$49:$H$62,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
+        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$49:$H$64,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" cm="1">

</xml_diff>

<commit_message>
Update Worklog - Y1B-2024-25_ADSAI.xlsx
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{049651C3-8AE2-40D4-8B72-08F808D3B87B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC7FDAE-BB9F-4E4C-B0A9-314263192696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1004,6 +1004,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1020,8 +1040,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1039,24 +1057,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1581,53 +1581,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -2922,53 +2922,53 @@
       <c r="K45" s="46"/>
     </row>
     <row r="46" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="64" t="s">
+      <c r="A46" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="59"/>
-      <c r="C46" s="59"/>
-      <c r="D46" s="59"/>
-      <c r="E46" s="59"/>
-      <c r="F46" s="59"/>
-      <c r="G46" s="59"/>
-      <c r="H46" s="59"/>
-      <c r="I46" s="59"/>
-      <c r="J46" s="59"/>
-      <c r="K46" s="60"/>
+      <c r="B46" s="67"/>
+      <c r="C46" s="67"/>
+      <c r="D46" s="67"/>
+      <c r="E46" s="67"/>
+      <c r="F46" s="67"/>
+      <c r="G46" s="67"/>
+      <c r="H46" s="67"/>
+      <c r="I46" s="67"/>
+      <c r="J46" s="67"/>
+      <c r="K46" s="68"/>
     </row>
     <row r="47" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A47" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B47" s="65" t="s">
+      <c r="B47" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C47" s="62"/>
-      <c r="D47" s="62"/>
-      <c r="E47" s="62"/>
-      <c r="F47" s="62"/>
-      <c r="G47" s="62"/>
-      <c r="H47" s="62"/>
-      <c r="I47" s="62"/>
-      <c r="J47" s="62"/>
-      <c r="K47" s="63"/>
+      <c r="C47" s="55"/>
+      <c r="D47" s="55"/>
+      <c r="E47" s="55"/>
+      <c r="F47" s="55"/>
+      <c r="G47" s="55"/>
+      <c r="H47" s="55"/>
+      <c r="I47" s="55"/>
+      <c r="J47" s="55"/>
+      <c r="K47" s="56"/>
     </row>
     <row r="48" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A49" s="47">
@@ -3501,53 +3501,53 @@
       <c r="K65" s="46"/>
     </row>
     <row r="66" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="66" t="s">
+      <c r="A66" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B66" s="62"/>
-      <c r="C66" s="62"/>
-      <c r="D66" s="62"/>
-      <c r="E66" s="62"/>
-      <c r="F66" s="62"/>
-      <c r="G66" s="62"/>
-      <c r="H66" s="62"/>
-      <c r="I66" s="62"/>
-      <c r="J66" s="62"/>
-      <c r="K66" s="63"/>
+      <c r="B66" s="55"/>
+      <c r="C66" s="55"/>
+      <c r="D66" s="55"/>
+      <c r="E66" s="55"/>
+      <c r="F66" s="55"/>
+      <c r="G66" s="55"/>
+      <c r="H66" s="55"/>
+      <c r="I66" s="55"/>
+      <c r="J66" s="55"/>
+      <c r="K66" s="56"/>
     </row>
     <row r="67" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A67" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="67" t="s">
+      <c r="B67" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C67" s="62"/>
-      <c r="D67" s="62"/>
-      <c r="E67" s="62"/>
-      <c r="F67" s="62"/>
-      <c r="G67" s="62"/>
-      <c r="H67" s="62"/>
-      <c r="I67" s="62"/>
-      <c r="J67" s="62"/>
-      <c r="K67" s="63"/>
+      <c r="C67" s="55"/>
+      <c r="D67" s="55"/>
+      <c r="E67" s="55"/>
+      <c r="F67" s="55"/>
+      <c r="G67" s="55"/>
+      <c r="H67" s="55"/>
+      <c r="I67" s="55"/>
+      <c r="J67" s="55"/>
+      <c r="K67" s="56"/>
     </row>
     <row r="68" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B68" s="67" t="s">
+      <c r="B68" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C68" s="62"/>
-      <c r="D68" s="62"/>
-      <c r="E68" s="62"/>
-      <c r="F68" s="62"/>
-      <c r="G68" s="62"/>
-      <c r="H68" s="62"/>
-      <c r="I68" s="62"/>
-      <c r="J68" s="62"/>
-      <c r="K68" s="63"/>
+      <c r="C68" s="55"/>
+      <c r="D68" s="55"/>
+      <c r="E68" s="55"/>
+      <c r="F68" s="55"/>
+      <c r="G68" s="55"/>
+      <c r="H68" s="55"/>
+      <c r="I68" s="55"/>
+      <c r="J68" s="55"/>
+      <c r="K68" s="56"/>
     </row>
     <row r="69" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A69" s="37"/>
@@ -3754,53 +3754,53 @@
       <c r="K79" s="46"/>
     </row>
     <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="68" t="s">
+      <c r="A80" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B80" s="62"/>
-      <c r="C80" s="62"/>
-      <c r="D80" s="62"/>
-      <c r="E80" s="62"/>
-      <c r="F80" s="62"/>
-      <c r="G80" s="62"/>
-      <c r="H80" s="62"/>
-      <c r="I80" s="62"/>
-      <c r="J80" s="62"/>
-      <c r="K80" s="63"/>
+      <c r="B80" s="55"/>
+      <c r="C80" s="55"/>
+      <c r="D80" s="55"/>
+      <c r="E80" s="55"/>
+      <c r="F80" s="55"/>
+      <c r="G80" s="55"/>
+      <c r="H80" s="55"/>
+      <c r="I80" s="55"/>
+      <c r="J80" s="55"/>
+      <c r="K80" s="56"/>
     </row>
     <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A81" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B81" s="70" t="s">
+      <c r="B81" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C81" s="62"/>
-      <c r="D81" s="62"/>
-      <c r="E81" s="62"/>
-      <c r="F81" s="62"/>
-      <c r="G81" s="62"/>
-      <c r="H81" s="62"/>
-      <c r="I81" s="62"/>
-      <c r="J81" s="62"/>
-      <c r="K81" s="63"/>
+      <c r="C81" s="55"/>
+      <c r="D81" s="55"/>
+      <c r="E81" s="55"/>
+      <c r="F81" s="55"/>
+      <c r="G81" s="55"/>
+      <c r="H81" s="55"/>
+      <c r="I81" s="55"/>
+      <c r="J81" s="55"/>
+      <c r="K81" s="56"/>
     </row>
     <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="70" t="s">
+      <c r="B82" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C82" s="62"/>
-      <c r="D82" s="62"/>
-      <c r="E82" s="62"/>
-      <c r="F82" s="62"/>
-      <c r="G82" s="62"/>
-      <c r="H82" s="62"/>
-      <c r="I82" s="62"/>
-      <c r="J82" s="62"/>
-      <c r="K82" s="63"/>
+      <c r="C82" s="55"/>
+      <c r="D82" s="55"/>
+      <c r="E82" s="55"/>
+      <c r="F82" s="55"/>
+      <c r="G82" s="55"/>
+      <c r="H82" s="55"/>
+      <c r="I82" s="55"/>
+      <c r="J82" s="55"/>
+      <c r="K82" s="56"/>
     </row>
     <row r="83" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A83" s="37"/>
@@ -4007,53 +4007,53 @@
       <c r="K93" s="46"/>
     </row>
     <row r="94" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="73" t="s">
+      <c r="A94" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B94" s="62"/>
-      <c r="C94" s="62"/>
-      <c r="D94" s="62"/>
-      <c r="E94" s="62"/>
-      <c r="F94" s="62"/>
-      <c r="G94" s="62"/>
-      <c r="H94" s="62"/>
-      <c r="I94" s="62"/>
-      <c r="J94" s="62"/>
-      <c r="K94" s="63"/>
+      <c r="B94" s="55"/>
+      <c r="C94" s="55"/>
+      <c r="D94" s="55"/>
+      <c r="E94" s="55"/>
+      <c r="F94" s="55"/>
+      <c r="G94" s="55"/>
+      <c r="H94" s="55"/>
+      <c r="I94" s="55"/>
+      <c r="J94" s="55"/>
+      <c r="K94" s="56"/>
     </row>
     <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A95" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B95" s="74" t="s">
+      <c r="B95" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C95" s="62"/>
-      <c r="D95" s="62"/>
-      <c r="E95" s="62"/>
-      <c r="F95" s="62"/>
-      <c r="G95" s="62"/>
-      <c r="H95" s="62"/>
-      <c r="I95" s="62"/>
-      <c r="J95" s="62"/>
-      <c r="K95" s="63"/>
+      <c r="C95" s="55"/>
+      <c r="D95" s="55"/>
+      <c r="E95" s="55"/>
+      <c r="F95" s="55"/>
+      <c r="G95" s="55"/>
+      <c r="H95" s="55"/>
+      <c r="I95" s="55"/>
+      <c r="J95" s="55"/>
+      <c r="K95" s="56"/>
     </row>
     <row r="96" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B96" s="74" t="s">
+      <c r="B96" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C96" s="62"/>
-      <c r="D96" s="62"/>
-      <c r="E96" s="62"/>
-      <c r="F96" s="62"/>
-      <c r="G96" s="62"/>
-      <c r="H96" s="62"/>
-      <c r="I96" s="62"/>
-      <c r="J96" s="62"/>
-      <c r="K96" s="63"/>
+      <c r="C96" s="55"/>
+      <c r="D96" s="55"/>
+      <c r="E96" s="55"/>
+      <c r="F96" s="55"/>
+      <c r="G96" s="55"/>
+      <c r="H96" s="55"/>
+      <c r="I96" s="55"/>
+      <c r="J96" s="55"/>
+      <c r="K96" s="56"/>
     </row>
     <row r="97" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A97" s="37"/>
@@ -4260,53 +4260,53 @@
       <c r="K107" s="46"/>
     </row>
     <row r="108" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="75" t="s">
+      <c r="A108" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B108" s="62"/>
-      <c r="C108" s="62"/>
-      <c r="D108" s="62"/>
-      <c r="E108" s="62"/>
-      <c r="F108" s="62"/>
-      <c r="G108" s="62"/>
-      <c r="H108" s="62"/>
-      <c r="I108" s="62"/>
-      <c r="J108" s="62"/>
-      <c r="K108" s="63"/>
+      <c r="B108" s="55"/>
+      <c r="C108" s="55"/>
+      <c r="D108" s="55"/>
+      <c r="E108" s="55"/>
+      <c r="F108" s="55"/>
+      <c r="G108" s="55"/>
+      <c r="H108" s="55"/>
+      <c r="I108" s="55"/>
+      <c r="J108" s="55"/>
+      <c r="K108" s="56"/>
     </row>
     <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A109" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B109" s="71" t="s">
+      <c r="B109" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C109" s="62"/>
-      <c r="D109" s="62"/>
-      <c r="E109" s="62"/>
-      <c r="F109" s="62"/>
-      <c r="G109" s="62"/>
-      <c r="H109" s="62"/>
-      <c r="I109" s="62"/>
-      <c r="J109" s="62"/>
-      <c r="K109" s="63"/>
+      <c r="C109" s="55"/>
+      <c r="D109" s="55"/>
+      <c r="E109" s="55"/>
+      <c r="F109" s="55"/>
+      <c r="G109" s="55"/>
+      <c r="H109" s="55"/>
+      <c r="I109" s="55"/>
+      <c r="J109" s="55"/>
+      <c r="K109" s="56"/>
     </row>
     <row r="110" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B110" s="71" t="s">
+      <c r="B110" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C110" s="62"/>
-      <c r="D110" s="62"/>
-      <c r="E110" s="62"/>
-      <c r="F110" s="62"/>
-      <c r="G110" s="62"/>
-      <c r="H110" s="62"/>
-      <c r="I110" s="62"/>
-      <c r="J110" s="62"/>
-      <c r="K110" s="63"/>
+      <c r="C110" s="55"/>
+      <c r="D110" s="55"/>
+      <c r="E110" s="55"/>
+      <c r="F110" s="55"/>
+      <c r="G110" s="55"/>
+      <c r="H110" s="55"/>
+      <c r="I110" s="55"/>
+      <c r="J110" s="55"/>
+      <c r="K110" s="56"/>
     </row>
     <row r="111" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A111" s="37"/>
@@ -4515,53 +4515,53 @@
       <c r="K121" s="46"/>
     </row>
     <row r="122" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="72" t="s">
+      <c r="A122" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B122" s="62"/>
-      <c r="C122" s="62"/>
-      <c r="D122" s="62"/>
-      <c r="E122" s="62"/>
-      <c r="F122" s="62"/>
-      <c r="G122" s="62"/>
-      <c r="H122" s="62"/>
-      <c r="I122" s="62"/>
-      <c r="J122" s="62"/>
-      <c r="K122" s="63"/>
+      <c r="B122" s="55"/>
+      <c r="C122" s="55"/>
+      <c r="D122" s="55"/>
+      <c r="E122" s="55"/>
+      <c r="F122" s="55"/>
+      <c r="G122" s="55"/>
+      <c r="H122" s="55"/>
+      <c r="I122" s="55"/>
+      <c r="J122" s="55"/>
+      <c r="K122" s="56"/>
     </row>
     <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A123" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B123" s="69" t="s">
+      <c r="B123" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C123" s="62"/>
-      <c r="D123" s="62"/>
-      <c r="E123" s="62"/>
-      <c r="F123" s="62"/>
-      <c r="G123" s="62"/>
-      <c r="H123" s="62"/>
-      <c r="I123" s="62"/>
-      <c r="J123" s="62"/>
-      <c r="K123" s="63"/>
+      <c r="C123" s="55"/>
+      <c r="D123" s="55"/>
+      <c r="E123" s="55"/>
+      <c r="F123" s="55"/>
+      <c r="G123" s="55"/>
+      <c r="H123" s="55"/>
+      <c r="I123" s="55"/>
+      <c r="J123" s="55"/>
+      <c r="K123" s="56"/>
     </row>
     <row r="124" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B124" s="69" t="s">
+      <c r="B124" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C124" s="62"/>
-      <c r="D124" s="62"/>
-      <c r="E124" s="62"/>
-      <c r="F124" s="62"/>
-      <c r="G124" s="62"/>
-      <c r="H124" s="62"/>
-      <c r="I124" s="62"/>
-      <c r="J124" s="62"/>
-      <c r="K124" s="63"/>
+      <c r="C124" s="55"/>
+      <c r="D124" s="55"/>
+      <c r="E124" s="55"/>
+      <c r="F124" s="55"/>
+      <c r="G124" s="55"/>
+      <c r="H124" s="55"/>
+      <c r="I124" s="55"/>
+      <c r="J124" s="55"/>
+      <c r="K124" s="56"/>
     </row>
     <row r="125" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A125" s="37"/>
@@ -4768,53 +4768,53 @@
       <c r="K135" s="46"/>
     </row>
     <row r="136" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="54" t="s">
+      <c r="A136" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B136" s="55"/>
-      <c r="C136" s="55"/>
-      <c r="D136" s="55"/>
-      <c r="E136" s="55"/>
-      <c r="F136" s="55"/>
-      <c r="G136" s="55"/>
-      <c r="H136" s="55"/>
-      <c r="I136" s="55"/>
-      <c r="J136" s="55"/>
-      <c r="K136" s="56"/>
+      <c r="B136" s="63"/>
+      <c r="C136" s="63"/>
+      <c r="D136" s="63"/>
+      <c r="E136" s="63"/>
+      <c r="F136" s="63"/>
+      <c r="G136" s="63"/>
+      <c r="H136" s="63"/>
+      <c r="I136" s="63"/>
+      <c r="J136" s="63"/>
+      <c r="K136" s="64"/>
     </row>
     <row r="137" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A137" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B137" s="57" t="s">
+      <c r="B137" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C137" s="55"/>
-      <c r="D137" s="55"/>
-      <c r="E137" s="55"/>
-      <c r="F137" s="55"/>
-      <c r="G137" s="55"/>
-      <c r="H137" s="55"/>
-      <c r="I137" s="55"/>
-      <c r="J137" s="55"/>
-      <c r="K137" s="56"/>
+      <c r="C137" s="63"/>
+      <c r="D137" s="63"/>
+      <c r="E137" s="63"/>
+      <c r="F137" s="63"/>
+      <c r="G137" s="63"/>
+      <c r="H137" s="63"/>
+      <c r="I137" s="63"/>
+      <c r="J137" s="63"/>
+      <c r="K137" s="64"/>
     </row>
     <row r="138" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B138" s="57" t="s">
+      <c r="B138" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C138" s="55"/>
-      <c r="D138" s="55"/>
-      <c r="E138" s="55"/>
-      <c r="F138" s="55"/>
-      <c r="G138" s="55"/>
-      <c r="H138" s="55"/>
-      <c r="I138" s="55"/>
-      <c r="J138" s="55"/>
-      <c r="K138" s="56"/>
+      <c r="C138" s="63"/>
+      <c r="D138" s="63"/>
+      <c r="E138" s="63"/>
+      <c r="F138" s="63"/>
+      <c r="G138" s="63"/>
+      <c r="H138" s="63"/>
+      <c r="I138" s="63"/>
+      <c r="J138" s="63"/>
+      <c r="K138" s="64"/>
     </row>
     <row r="139" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A139" s="37"/>
@@ -5025,7 +5025,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{E618F7EC-EE6C-4EC9-803D-CB7D6E0706F7}">
+      <autoFilter ref="A1:K15" xr:uid="{ABCA17DA-9000-40D6-9FD8-97574B35A77E}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5036,14 +5036,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B109:K109"/>
-    <mergeCell ref="B110:K110"/>
-    <mergeCell ref="A122:K122"/>
-    <mergeCell ref="B82:K82"/>
-    <mergeCell ref="A94:K94"/>
-    <mergeCell ref="B95:K95"/>
-    <mergeCell ref="B96:K96"/>
-    <mergeCell ref="A108:K108"/>
     <mergeCell ref="A136:K136"/>
     <mergeCell ref="B137:K137"/>
     <mergeCell ref="B138:K138"/>
@@ -5060,6 +5052,14 @@
     <mergeCell ref="B123:K123"/>
     <mergeCell ref="B124:K124"/>
     <mergeCell ref="B81:K81"/>
+    <mergeCell ref="B109:K109"/>
+    <mergeCell ref="B110:K110"/>
+    <mergeCell ref="A122:K122"/>
+    <mergeCell ref="B82:K82"/>
+    <mergeCell ref="A94:K94"/>
+    <mergeCell ref="B95:K95"/>
+    <mergeCell ref="B96:K96"/>
+    <mergeCell ref="A108:K108"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B44 B47:B64 B69:B78 B83:B92 B97:B106 B111:B120 B125:B134">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -6785,6 +6785,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -7019,27 +7039,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7056,23 +7075,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W2 Datalab 2 Work I (Startup and pre-datalab work)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC7FDAE-BB9F-4E4C-B0A9-314263192696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36866D89-51B8-4503-BC92-3B7574B7C72B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,9 +18,9 @@
     <sheet name="Drop-downs" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$45</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$134</definedName>
-    <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$148</definedName>
+    <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <customWorkbookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="156">
   <si>
     <t>Date</t>
   </si>
@@ -464,9 +464,6 @@
     <t>Set up VPN</t>
   </si>
   <si>
-    <t>Does not work at school, have to set up at home.</t>
-  </si>
-  <si>
     <t>Introduction and Understanding the Problem</t>
   </si>
   <si>
@@ -519,6 +516,60 @@
   </si>
   <si>
     <t>EDA with Python</t>
+  </si>
+  <si>
+    <t>Do the DataCamp course "Exploratory Data Analysis In Python"</t>
+  </si>
+  <si>
+    <t>Analyze the state of Creative Brief Project</t>
+  </si>
+  <si>
+    <t>Prepare for Friday DataLab</t>
+  </si>
+  <si>
+    <t>28&amp;29-11-2024</t>
+  </si>
+  <si>
+    <t>DataLab 2 Stand-up meeting</t>
+  </si>
+  <si>
+    <t>Friday Content Review Session</t>
+  </si>
+  <si>
+    <t>Guest Lecture</t>
+  </si>
+  <si>
+    <t>EDA with Kaggle dataset</t>
+  </si>
+  <si>
+    <t>You do not have to do it after finishing the SQL part.</t>
+  </si>
+  <si>
+    <t>Evidence in Learning Log week 1</t>
+  </si>
+  <si>
+    <t>I am not certain what has to be done with the "SMARTER" goals</t>
+  </si>
+  <si>
+    <t>Evidence in WorkLog</t>
+  </si>
+  <si>
+    <t>Evidence Week 2 Learning Log</t>
+  </si>
+  <si>
+    <t>Fill in Week 2 Learning Log</t>
+  </si>
+  <si>
+    <t>Do Vector quiz in Brightspace</t>
+  </si>
+  <si>
+    <t>Learn about Vectors</t>
+  </si>
+  <si>
+    <t>Search for old Vector materials from High School</t>
+  </si>
+  <si>
+    <t>Attempt to apply for retake of Python Exam</t>
   </si>
 </sst>
 </file>
@@ -1529,7 +1580,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K149"/>
+  <dimension ref="A1:K163"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1655,7 +1706,7 @@
         <v>0.5</v>
       </c>
       <c r="I5" s="41">
-        <f t="shared" ref="I5:I45" si="0">H5-G5</f>
+        <f t="shared" ref="I5:I46" si="0">H5-G5</f>
         <v>0</v>
       </c>
       <c r="J5" s="42"/>
@@ -1732,7 +1783,7 @@
         <v>45614</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C8" s="39" t="s">
         <v>17</v>
@@ -1749,10 +1800,12 @@
       <c r="G8" s="41">
         <v>1.5</v>
       </c>
-      <c r="H8" s="41"/>
+      <c r="H8" s="41">
+        <v>1</v>
+      </c>
       <c r="I8" s="41">
         <f t="shared" si="0"/>
-        <v>-1.5</v>
+        <v>-0.5</v>
       </c>
       <c r="J8" s="42"/>
       <c r="K8" s="44"/>
@@ -1762,7 +1815,7 @@
         <v>45614</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C9" s="39" t="s">
         <v>17</v>
@@ -1779,10 +1832,12 @@
       <c r="G9" s="41">
         <v>4</v>
       </c>
-      <c r="H9" s="41"/>
+      <c r="H9" s="41">
+        <v>4</v>
+      </c>
       <c r="I9" s="41">
         <f t="shared" si="0"/>
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="J9" s="42"/>
       <c r="K9" s="44"/>
@@ -2020,7 +2075,7 @@
         <v>45615</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C17" s="39" t="s">
         <v>17</v>
@@ -2037,13 +2092,17 @@
       <c r="G17" s="41">
         <v>0.5</v>
       </c>
-      <c r="H17" s="41"/>
+      <c r="H17" s="41">
+        <v>0.75</v>
+      </c>
       <c r="I17" s="41">
         <f t="shared" si="0"/>
-        <v>-0.5</v>
+        <v>0.25</v>
       </c>
       <c r="J17" s="45"/>
-      <c r="K17" s="44"/>
+      <c r="K17" s="44" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="18" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A18" s="37">
@@ -2148,7 +2207,7 @@
         <v>45615</v>
       </c>
       <c r="B21" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C21" s="39" t="s">
         <v>17</v>
@@ -2165,10 +2224,12 @@
       <c r="G21" s="41">
         <v>3</v>
       </c>
-      <c r="H21" s="41"/>
+      <c r="H21" s="41">
+        <v>3</v>
+      </c>
       <c r="I21" s="41">
         <f t="shared" si="0"/>
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="J21" s="45"/>
       <c r="K21" s="44" t="s">
@@ -2566,7 +2627,7 @@
         <v>45618</v>
       </c>
       <c r="B34" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C34" s="39" t="s">
         <v>17</v>
@@ -2728,7 +2789,7 @@
         <v>45618</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C39" s="39" t="s">
         <v>17</v>
@@ -2745,14 +2806,16 @@
       <c r="G39" s="41">
         <v>1</v>
       </c>
-      <c r="H39" s="41"/>
+      <c r="H39" s="41">
+        <v>1</v>
+      </c>
       <c r="I39" s="41">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J39" s="45"/>
       <c r="K39" s="44" t="s">
-        <v>120</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -2760,7 +2823,7 @@
         <v>45618</v>
       </c>
       <c r="B40" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C40" s="39" t="s">
         <v>17</v>
@@ -2777,10 +2840,12 @@
       <c r="G40" s="41">
         <v>4</v>
       </c>
-      <c r="H40" s="41"/>
+      <c r="H40" s="41">
+        <v>4</v>
+      </c>
       <c r="I40" s="41">
         <f t="shared" si="0"/>
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="J40" s="45"/>
       <c r="K40" s="44"/>
@@ -2870,9 +2935,11 @@
       <c r="K43" s="44"/>
     </row>
     <row r="44" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A44" s="37"/>
+      <c r="A44" s="37">
+        <v>45618</v>
+      </c>
       <c r="B44" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C44" s="39" t="s">
         <v>17</v>
@@ -2889,76 +2956,89 @@
       <c r="G44" s="41">
         <v>0.5</v>
       </c>
-      <c r="H44" s="41"/>
+      <c r="H44" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I44" s="41">
         <f t="shared" si="0"/>
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="J44" s="45"/>
       <c r="K44" s="44"/>
     </row>
     <row r="45" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A45" s="13"/>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
-      <c r="E45" s="15" t="s">
+      <c r="A45" s="37"/>
+      <c r="B45" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="E45" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F45" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G45" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H45" s="41"/>
+      <c r="I45" s="41">
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J45" s="45"/>
+      <c r="K45" s="44"/>
+    </row>
+    <row r="46" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A46" s="13"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F45" s="15"/>
-      <c r="G45" s="18">
-        <f>SUM(G5:G44)</f>
-        <v>44.85</v>
-      </c>
-      <c r="H45" s="18">
+      <c r="F46" s="15"/>
+      <c r="G46" s="18">
+        <f>SUM(G5:G45)</f>
+        <v>45.35</v>
+      </c>
+      <c r="H46" s="18">
         <f>SUM(H5:H44)</f>
-        <v>21</v>
-      </c>
-      <c r="I45" s="18">
+        <v>35</v>
+      </c>
+      <c r="I46" s="18">
         <f t="shared" si="0"/>
-        <v>-23.85</v>
-      </c>
-      <c r="J45" s="19"/>
-      <c r="K45" s="46"/>
-    </row>
-    <row r="46" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="70" t="s">
+        <v>-10.350000000000001</v>
+      </c>
+      <c r="J46" s="19"/>
+      <c r="K46" s="46"/>
+    </row>
+    <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="67"/>
-      <c r="C46" s="67"/>
-      <c r="D46" s="67"/>
-      <c r="E46" s="67"/>
-      <c r="F46" s="67"/>
-      <c r="G46" s="67"/>
-      <c r="H46" s="67"/>
-      <c r="I46" s="67"/>
-      <c r="J46" s="67"/>
-      <c r="K46" s="68"/>
-    </row>
-    <row r="47" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A47" s="31" t="s">
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
+    </row>
+    <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B47" s="71" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
-      </c>
-      <c r="C47" s="55"/>
-      <c r="D47" s="55"/>
-      <c r="E47" s="55"/>
-      <c r="F47" s="55"/>
-      <c r="G47" s="55"/>
-      <c r="H47" s="55"/>
-      <c r="I47" s="55"/>
-      <c r="J47" s="55"/>
-      <c r="K47" s="56"/>
-    </row>
-    <row r="48" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B48" s="71" t="s">
-        <v>20</v>
       </c>
       <c r="C48" s="55"/>
       <c r="D48" s="55"/>
@@ -2970,37 +3050,22 @@
       <c r="J48" s="55"/>
       <c r="K48" s="56"/>
     </row>
-    <row r="49" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A49" s="47">
-        <v>45621</v>
-      </c>
-      <c r="B49" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="C49" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D49" s="38" t="s">
-        <v>80</v>
-      </c>
-      <c r="E49" s="40" t="s">
-        <v>64</v>
-      </c>
-      <c r="F49" s="40" t="s">
-        <v>87</v>
-      </c>
-      <c r="G49" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="H49" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="I49" s="41">
-        <f t="shared" ref="I49:I65" si="1">H49-G49</f>
-        <v>0</v>
-      </c>
-      <c r="J49" s="45"/>
-      <c r="K49" s="43"/>
+    <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B49" s="71" t="s">
+        <v>20</v>
+      </c>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -3013,22 +3078,22 @@
         <v>17</v>
       </c>
       <c r="D50" s="38" t="s">
-        <v>121</v>
+        <v>80</v>
       </c>
       <c r="E50" s="40" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F50" s="40" t="s">
-        <v>109</v>
+        <v>87</v>
       </c>
       <c r="G50" s="41">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H50" s="41">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I50" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="I50:I79" si="1">H50-G50</f>
         <v>0</v>
       </c>
       <c r="J50" s="45"/>
@@ -3045,7 +3110,7 @@
         <v>17</v>
       </c>
       <c r="D51" s="38" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E51" s="40" t="s">
         <v>67</v>
@@ -3054,10 +3119,10 @@
         <v>109</v>
       </c>
       <c r="G51" s="41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H51" s="41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I51" s="41">
         <f t="shared" si="1"/>
@@ -3077,7 +3142,7 @@
         <v>17</v>
       </c>
       <c r="D52" s="38" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E52" s="40" t="s">
         <v>67</v>
@@ -3109,7 +3174,7 @@
         <v>17</v>
       </c>
       <c r="D53" s="38" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E53" s="40" t="s">
         <v>67</v>
@@ -3118,10 +3183,10 @@
         <v>109</v>
       </c>
       <c r="G53" s="41">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H53" s="41">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="I53" s="41">
         <f t="shared" si="1"/>
@@ -3141,7 +3206,7 @@
         <v>17</v>
       </c>
       <c r="D54" s="38" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E54" s="40" t="s">
         <v>67</v>
@@ -3150,10 +3215,10 @@
         <v>109</v>
       </c>
       <c r="G54" s="41">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H54" s="41">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I54" s="41">
         <f t="shared" si="1"/>
@@ -3173,19 +3238,19 @@
         <v>17</v>
       </c>
       <c r="D55" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E55" s="40" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="F55" s="40" t="s">
         <v>109</v>
       </c>
       <c r="G55" s="41">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H55" s="41">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I55" s="41">
         <f t="shared" si="1"/>
@@ -3196,7 +3261,7 @@
     </row>
     <row r="56" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A56" s="47">
-        <v>45622</v>
+        <v>45621</v>
       </c>
       <c r="B56" s="38" t="s">
         <v>55</v>
@@ -3205,13 +3270,13 @@
         <v>17</v>
       </c>
       <c r="D56" s="38" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E56" s="40" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F56" s="40" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="G56" s="41">
         <v>0.5</v>
@@ -3237,19 +3302,19 @@
         <v>17</v>
       </c>
       <c r="D57" s="38" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E57" s="40" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="F57" s="40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G57" s="41">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="H57" s="41">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I57" s="41">
         <f t="shared" si="1"/>
@@ -3269,28 +3334,26 @@
         <v>17</v>
       </c>
       <c r="D58" s="38" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E58" s="40" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F58" s="40" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="G58" s="41">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="H58" s="41">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="I58" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J58" s="45"/>
-      <c r="K58" s="43" t="s">
-        <v>130</v>
-      </c>
+      <c r="K58" s="43"/>
     </row>
     <row r="59" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A59" s="47">
@@ -3303,10 +3366,10 @@
         <v>17</v>
       </c>
       <c r="D59" s="38" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E59" s="40" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="F59" s="40" t="s">
         <v>109</v>
@@ -3322,7 +3385,9 @@
         <v>0</v>
       </c>
       <c r="J59" s="45"/>
-      <c r="K59" s="43"/>
+      <c r="K59" s="43" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="60" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A60" s="47">
@@ -3335,7 +3400,7 @@
         <v>17</v>
       </c>
       <c r="D60" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E60" s="40" t="s">
         <v>67</v>
@@ -3347,16 +3412,14 @@
         <v>0.5</v>
       </c>
       <c r="H60" s="41">
-        <v>2.35</v>
+        <v>0.5</v>
       </c>
       <c r="I60" s="41">
         <f t="shared" si="1"/>
-        <v>1.85</v>
+        <v>0</v>
       </c>
       <c r="J60" s="45"/>
-      <c r="K60" s="43" t="s">
-        <v>137</v>
-      </c>
+      <c r="K60" s="43"/>
     </row>
     <row r="61" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A61" s="47">
@@ -3369,27 +3432,27 @@
         <v>17</v>
       </c>
       <c r="D61" s="38" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E61" s="40" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="F61" s="40" t="s">
         <v>109</v>
       </c>
       <c r="G61" s="41">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="H61" s="41">
-        <v>0.1</v>
+        <v>2.35</v>
       </c>
       <c r="I61" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.85</v>
       </c>
       <c r="J61" s="45"/>
       <c r="K61" s="43" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -3397,33 +3460,33 @@
         <v>45622</v>
       </c>
       <c r="B62" s="38" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C62" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D62" s="38" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E62" s="40" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F62" s="40" t="s">
         <v>109</v>
       </c>
       <c r="G62" s="41">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H62" s="41">
         <v>0.1</v>
       </c>
       <c r="I62" s="41">
         <f t="shared" si="1"/>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J62" s="45"/>
       <c r="K62" s="43" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -3431,299 +3494,492 @@
         <v>45622</v>
       </c>
       <c r="B63" s="38" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C63" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D63" s="38" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E63" s="40" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F63" s="40" t="s">
         <v>109</v>
       </c>
       <c r="G63" s="41">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H63" s="41">
-        <v>3.55</v>
+        <v>0.1</v>
       </c>
       <c r="I63" s="41">
         <f t="shared" si="1"/>
-        <v>-0.45000000000000018</v>
+        <v>0.1</v>
       </c>
       <c r="J63" s="45"/>
-      <c r="K63" s="43"/>
+      <c r="K63" s="43" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="64" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A64" s="47"/>
-      <c r="B64" s="38"/>
+      <c r="A64" s="47">
+        <v>45622</v>
+      </c>
+      <c r="B64" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C64" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D64" s="38"/>
-      <c r="E64" s="40"/>
-      <c r="F64" s="40"/>
-      <c r="G64" s="41"/>
-      <c r="H64" s="41"/>
+      <c r="D64" s="38" t="s">
+        <v>137</v>
+      </c>
+      <c r="E64" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F64" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G64" s="41">
+        <v>4</v>
+      </c>
+      <c r="H64" s="41">
+        <v>3.55</v>
+      </c>
       <c r="I64" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.45000000000000018</v>
       </c>
       <c r="J64" s="45"/>
       <c r="K64" s="43"/>
     </row>
     <row r="65" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A65" s="13"/>
-      <c r="B65" s="15"/>
-      <c r="C65" s="15"/>
-      <c r="D65" s="15"/>
-      <c r="E65" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F65" s="15"/>
-      <c r="G65" s="18">
-        <f t="shared" ref="G65:H65" si="2">SUM(G47:G64)</f>
-        <v>14.85</v>
-      </c>
-      <c r="H65" s="18">
-        <f t="shared" si="2"/>
-        <v>16.349999999999998</v>
-      </c>
-      <c r="I65" s="18">
+      <c r="A65" s="47">
+        <v>45623</v>
+      </c>
+      <c r="B65" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C65" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D65" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="E65" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F65" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G65" s="41">
+        <v>3</v>
+      </c>
+      <c r="H65" s="41">
+        <v>3</v>
+      </c>
+      <c r="I65" s="41">
         <f t="shared" si="1"/>
-        <v>1.4999999999999982</v>
-      </c>
-      <c r="J65" s="19"/>
-      <c r="K65" s="46"/>
-    </row>
-    <row r="66" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="72" t="s">
-        <v>21</v>
-      </c>
-      <c r="B66" s="55"/>
-      <c r="C66" s="55"/>
-      <c r="D66" s="55"/>
-      <c r="E66" s="55"/>
-      <c r="F66" s="55"/>
-      <c r="G66" s="55"/>
-      <c r="H66" s="55"/>
-      <c r="I66" s="55"/>
-      <c r="J66" s="55"/>
-      <c r="K66" s="56"/>
+        <v>0</v>
+      </c>
+      <c r="J65" s="45"/>
+      <c r="K65" s="43"/>
+    </row>
+    <row r="66" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A66" s="47">
+        <v>45623</v>
+      </c>
+      <c r="B66" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C66" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D66" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="E66" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F66" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G66" s="41">
+        <v>2</v>
+      </c>
+      <c r="H66" s="41">
+        <v>2</v>
+      </c>
+      <c r="I66" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J66" s="45"/>
+      <c r="K66" s="43"/>
     </row>
     <row r="67" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A67" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B67" s="73" t="s">
-        <v>13</v>
-      </c>
-      <c r="C67" s="55"/>
-      <c r="D67" s="55"/>
-      <c r="E67" s="55"/>
-      <c r="F67" s="55"/>
-      <c r="G67" s="55"/>
-      <c r="H67" s="55"/>
-      <c r="I67" s="55"/>
-      <c r="J67" s="55"/>
-      <c r="K67" s="56"/>
-    </row>
-    <row r="68" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B68" s="73" t="s">
-        <v>15</v>
-      </c>
-      <c r="C68" s="55"/>
-      <c r="D68" s="55"/>
-      <c r="E68" s="55"/>
-      <c r="F68" s="55"/>
-      <c r="G68" s="55"/>
-      <c r="H68" s="55"/>
-      <c r="I68" s="55"/>
-      <c r="J68" s="55"/>
-      <c r="K68" s="56"/>
+      <c r="A67" s="47">
+        <v>45623</v>
+      </c>
+      <c r="B67" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C67" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D67" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="E67" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F67" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G67" s="41">
+        <v>1</v>
+      </c>
+      <c r="H67" s="41"/>
+      <c r="I67" s="41">
+        <f t="shared" si="1"/>
+        <v>-1</v>
+      </c>
+      <c r="J67" s="45"/>
+      <c r="K67" s="43"/>
+    </row>
+    <row r="68" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A68" s="47">
+        <v>45624</v>
+      </c>
+      <c r="B68" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C68" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D68" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="E68" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="F68" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G68" s="41">
+        <v>4</v>
+      </c>
+      <c r="H68" s="41">
+        <v>4</v>
+      </c>
+      <c r="I68" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J68" s="45"/>
+      <c r="K68" s="43"/>
     </row>
     <row r="69" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A69" s="37"/>
-      <c r="B69" s="38"/>
+      <c r="A69" s="47">
+        <v>45624</v>
+      </c>
+      <c r="B69" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C69" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D69" s="38"/>
-      <c r="E69" s="40"/>
-      <c r="F69" s="40"/>
-      <c r="G69" s="41"/>
-      <c r="H69" s="41"/>
+      <c r="D69" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="E69" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F69" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G69" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H69" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I69" s="41">
-        <f t="shared" ref="I69:I79" si="3">H69-G69</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J69" s="45"/>
       <c r="K69" s="43"/>
     </row>
     <row r="70" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A70" s="37"/>
-      <c r="B70" s="38"/>
+      <c r="A70" s="47" t="s">
+        <v>141</v>
+      </c>
+      <c r="B70" s="38" t="s">
+        <v>52</v>
+      </c>
       <c r="C70" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D70" s="38"/>
-      <c r="E70" s="40"/>
-      <c r="F70" s="40"/>
-      <c r="G70" s="41"/>
+      <c r="D70" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="E70" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F70" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G70" s="41">
+        <v>1</v>
+      </c>
       <c r="H70" s="41"/>
       <c r="I70" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>-1</v>
       </c>
       <c r="J70" s="45"/>
-      <c r="K70" s="43"/>
+      <c r="K70" s="43" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="71" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A71" s="37"/>
-      <c r="B71" s="38"/>
+      <c r="A71" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B71" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C71" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D71" s="38"/>
-      <c r="E71" s="40"/>
-      <c r="F71" s="40"/>
-      <c r="G71" s="41"/>
-      <c r="H71" s="41"/>
+      <c r="D71" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="E71" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F71" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G71" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H71" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I71" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J71" s="45"/>
       <c r="K71" s="43"/>
     </row>
     <row r="72" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A72" s="37"/>
-      <c r="B72" s="38"/>
+      <c r="A72" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B72" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C72" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D72" s="38"/>
-      <c r="E72" s="40"/>
-      <c r="F72" s="40"/>
-      <c r="G72" s="41"/>
-      <c r="H72" s="41"/>
+      <c r="D72" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="E72" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F72" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G72" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H72" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I72" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J72" s="45"/>
       <c r="K72" s="43"/>
     </row>
     <row r="73" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A73" s="37"/>
-      <c r="B73" s="38"/>
+      <c r="A73" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B73" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C73" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D73" s="38"/>
-      <c r="E73" s="40"/>
-      <c r="F73" s="40"/>
-      <c r="G73" s="41"/>
+      <c r="D73" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="E73" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F73" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G73" s="41">
+        <v>1</v>
+      </c>
       <c r="H73" s="41"/>
       <c r="I73" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>-1</v>
       </c>
       <c r="J73" s="45"/>
       <c r="K73" s="43"/>
     </row>
     <row r="74" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A74" s="37"/>
-      <c r="B74" s="38"/>
+      <c r="A74" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B74" s="38" t="s">
+        <v>46</v>
+      </c>
       <c r="C74" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D74" s="38"/>
-      <c r="E74" s="40"/>
-      <c r="F74" s="40"/>
-      <c r="G74" s="41"/>
-      <c r="H74" s="41"/>
+      <c r="D74" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="E74" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="F74" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="G74" s="41">
+        <v>0</v>
+      </c>
+      <c r="H74" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I74" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>0.25</v>
       </c>
       <c r="J74" s="45"/>
       <c r="K74" s="43"/>
     </row>
     <row r="75" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A75" s="37"/>
-      <c r="B75" s="38"/>
+      <c r="A75" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B75" s="38" t="s">
+        <v>52</v>
+      </c>
       <c r="C75" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D75" s="38"/>
-      <c r="E75" s="40"/>
-      <c r="F75" s="40"/>
-      <c r="G75" s="41"/>
+      <c r="D75" s="38" t="s">
+        <v>145</v>
+      </c>
+      <c r="E75" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F75" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G75" s="41">
+        <v>4</v>
+      </c>
       <c r="H75" s="41"/>
       <c r="I75" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>-4</v>
       </c>
       <c r="J75" s="45"/>
       <c r="K75" s="43"/>
     </row>
     <row r="76" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A76" s="37"/>
-      <c r="B76" s="38"/>
+      <c r="A76" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B76" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C76" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D76" s="38"/>
-      <c r="E76" s="40"/>
-      <c r="F76" s="40"/>
+      <c r="D76" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E76" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F76" s="40" t="s">
+        <v>87</v>
+      </c>
       <c r="G76" s="41"/>
       <c r="H76" s="41"/>
       <c r="I76" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J76" s="45"/>
       <c r="K76" s="43"/>
     </row>
     <row r="77" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A77" s="37"/>
-      <c r="B77" s="38"/>
+      <c r="A77" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B77" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C77" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D77" s="38"/>
-      <c r="E77" s="40"/>
-      <c r="F77" s="40"/>
+      <c r="D77" s="38" t="s">
+        <v>151</v>
+      </c>
+      <c r="E77" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F77" s="40" t="s">
+        <v>88</v>
+      </c>
       <c r="G77" s="41"/>
       <c r="H77" s="41"/>
       <c r="I77" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J77" s="45"/>
       <c r="K77" s="43"/>
     </row>
     <row r="78" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A78" s="37"/>
-      <c r="B78" s="38"/>
+      <c r="A78" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B78" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C78" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D78" s="38"/>
-      <c r="E78" s="40"/>
-      <c r="F78" s="40"/>
+      <c r="D78" s="38" t="s">
+        <v>150</v>
+      </c>
+      <c r="E78" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F78" s="40" t="s">
+        <v>88</v>
+      </c>
       <c r="G78" s="41"/>
       <c r="H78" s="41"/>
       <c r="I78" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J78" s="45"/>
@@ -3739,23 +3995,23 @@
       </c>
       <c r="F79" s="15"/>
       <c r="G79" s="18">
-        <f t="shared" ref="G79:H79" si="4">SUM(G69:G78)</f>
-        <v>0</v>
+        <f t="shared" ref="G79:H79" si="2">SUM(G48:G77)</f>
+        <v>31.85</v>
       </c>
       <c r="H79" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>26.599999999999998</v>
       </c>
       <c r="I79" s="18">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>-5.2500000000000036</v>
       </c>
       <c r="J79" s="19"/>
       <c r="K79" s="46"/>
     </row>
     <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="74" t="s">
-        <v>22</v>
+      <c r="A80" s="72" t="s">
+        <v>21</v>
       </c>
       <c r="B80" s="55"/>
       <c r="C80" s="55"/>
@@ -3769,10 +4025,10 @@
       <c r="K80" s="56"/>
     </row>
     <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A81" s="23" t="s">
+      <c r="A81" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B81" s="58" t="s">
+      <c r="B81" s="73" t="s">
         <v>13</v>
       </c>
       <c r="C81" s="55"/>
@@ -3786,10 +4042,10 @@
       <c r="K81" s="56"/>
     </row>
     <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="24" t="s">
+      <c r="A82" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="58" t="s">
+      <c r="B82" s="73" t="s">
         <v>15</v>
       </c>
       <c r="C82" s="55"/>
@@ -3814,7 +4070,7 @@
       <c r="G83" s="41"/>
       <c r="H83" s="41"/>
       <c r="I83" s="41">
-        <f t="shared" ref="I83:I93" si="5">H83-G83</f>
+        <f t="shared" ref="I83:I93" si="3">H83-G83</f>
         <v>0</v>
       </c>
       <c r="J83" s="45"/>
@@ -3832,7 +4088,7 @@
       <c r="G84" s="41"/>
       <c r="H84" s="41"/>
       <c r="I84" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J84" s="45"/>
@@ -3850,7 +4106,7 @@
       <c r="G85" s="41"/>
       <c r="H85" s="41"/>
       <c r="I85" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J85" s="45"/>
@@ -3868,7 +4124,7 @@
       <c r="G86" s="41"/>
       <c r="H86" s="41"/>
       <c r="I86" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J86" s="45"/>
@@ -3886,7 +4142,7 @@
       <c r="G87" s="41"/>
       <c r="H87" s="41"/>
       <c r="I87" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J87" s="45"/>
@@ -3904,7 +4160,7 @@
       <c r="G88" s="41"/>
       <c r="H88" s="41"/>
       <c r="I88" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J88" s="45"/>
@@ -3922,7 +4178,7 @@
       <c r="G89" s="41"/>
       <c r="H89" s="41"/>
       <c r="I89" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J89" s="45"/>
@@ -3940,7 +4196,7 @@
       <c r="G90" s="41"/>
       <c r="H90" s="41"/>
       <c r="I90" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J90" s="45"/>
@@ -3958,7 +4214,7 @@
       <c r="G91" s="41"/>
       <c r="H91" s="41"/>
       <c r="I91" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J91" s="45"/>
@@ -3976,7 +4232,7 @@
       <c r="G92" s="41"/>
       <c r="H92" s="41"/>
       <c r="I92" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J92" s="45"/>
@@ -3992,23 +4248,23 @@
       </c>
       <c r="F93" s="15"/>
       <c r="G93" s="18">
-        <f t="shared" ref="G93:H93" si="6">SUM(G83:G92)</f>
+        <f t="shared" ref="G93:H93" si="4">SUM(G83:G92)</f>
         <v>0</v>
       </c>
       <c r="H93" s="18">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I93" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J93" s="19"/>
       <c r="K93" s="46"/>
     </row>
     <row r="94" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="59" t="s">
-        <v>23</v>
+      <c r="A94" s="74" t="s">
+        <v>22</v>
       </c>
       <c r="B94" s="55"/>
       <c r="C94" s="55"/>
@@ -4022,10 +4278,10 @@
       <c r="K94" s="56"/>
     </row>
     <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A95" s="25" t="s">
+      <c r="A95" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B95" s="60" t="s">
+      <c r="B95" s="58" t="s">
         <v>13</v>
       </c>
       <c r="C95" s="55"/>
@@ -4039,10 +4295,10 @@
       <c r="K95" s="56"/>
     </row>
     <row r="96" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="26" t="s">
+      <c r="A96" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B96" s="60" t="s">
+      <c r="B96" s="58" t="s">
         <v>15</v>
       </c>
       <c r="C96" s="55"/>
@@ -4067,7 +4323,7 @@
       <c r="G97" s="41"/>
       <c r="H97" s="41"/>
       <c r="I97" s="41">
-        <f t="shared" ref="I97:I107" si="7">H97-G97</f>
+        <f t="shared" ref="I97:I107" si="5">H97-G97</f>
         <v>0</v>
       </c>
       <c r="J97" s="45"/>
@@ -4085,7 +4341,7 @@
       <c r="G98" s="41"/>
       <c r="H98" s="41"/>
       <c r="I98" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J98" s="45"/>
@@ -4103,7 +4359,7 @@
       <c r="G99" s="41"/>
       <c r="H99" s="41"/>
       <c r="I99" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J99" s="45"/>
@@ -4121,7 +4377,7 @@
       <c r="G100" s="41"/>
       <c r="H100" s="41"/>
       <c r="I100" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J100" s="45"/>
@@ -4139,7 +4395,7 @@
       <c r="G101" s="41"/>
       <c r="H101" s="41"/>
       <c r="I101" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J101" s="45"/>
@@ -4157,7 +4413,7 @@
       <c r="G102" s="41"/>
       <c r="H102" s="41"/>
       <c r="I102" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J102" s="45"/>
@@ -4175,7 +4431,7 @@
       <c r="G103" s="41"/>
       <c r="H103" s="41"/>
       <c r="I103" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J103" s="45"/>
@@ -4193,7 +4449,7 @@
       <c r="G104" s="41"/>
       <c r="H104" s="41"/>
       <c r="I104" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J104" s="45"/>
@@ -4211,7 +4467,7 @@
       <c r="G105" s="41"/>
       <c r="H105" s="41"/>
       <c r="I105" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J105" s="45"/>
@@ -4229,7 +4485,7 @@
       <c r="G106" s="41"/>
       <c r="H106" s="41"/>
       <c r="I106" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J106" s="45"/>
@@ -4245,23 +4501,23 @@
       </c>
       <c r="F107" s="15"/>
       <c r="G107" s="18">
-        <f t="shared" ref="G107:H107" si="8">SUM(G97:G106)</f>
+        <f t="shared" ref="G107:H107" si="6">SUM(G97:G106)</f>
         <v>0</v>
       </c>
       <c r="H107" s="18">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="I107" s="18">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J107" s="19"/>
       <c r="K107" s="46"/>
     </row>
     <row r="108" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="61" t="s">
-        <v>24</v>
+      <c r="A108" s="59" t="s">
+        <v>23</v>
       </c>
       <c r="B108" s="55"/>
       <c r="C108" s="55"/>
@@ -4275,10 +4531,10 @@
       <c r="K108" s="56"/>
     </row>
     <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A109" s="27" t="s">
+      <c r="A109" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B109" s="54" t="s">
+      <c r="B109" s="60" t="s">
         <v>13</v>
       </c>
       <c r="C109" s="55"/>
@@ -4292,10 +4548,10 @@
       <c r="K109" s="56"/>
     </row>
     <row r="110" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="28" t="s">
+      <c r="A110" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B110" s="54" t="s">
+      <c r="B110" s="60" t="s">
         <v>15</v>
       </c>
       <c r="C110" s="55"/>
@@ -4320,7 +4576,7 @@
       <c r="G111" s="41"/>
       <c r="H111" s="41"/>
       <c r="I111" s="41">
-        <f t="shared" ref="I111:I121" si="9">H111-G111</f>
+        <f t="shared" ref="I111:I121" si="7">H111-G111</f>
         <v>0</v>
       </c>
       <c r="J111" s="45"/>
@@ -4338,7 +4594,7 @@
       <c r="G112" s="41"/>
       <c r="H112" s="41"/>
       <c r="I112" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J112" s="45"/>
@@ -4356,13 +4612,11 @@
       <c r="G113" s="41"/>
       <c r="H113" s="41"/>
       <c r="I113" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J113" s="45"/>
-      <c r="K113" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K113" s="43"/>
     </row>
     <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A114" s="37"/>
@@ -4376,7 +4630,7 @@
       <c r="G114" s="41"/>
       <c r="H114" s="41"/>
       <c r="I114" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J114" s="45"/>
@@ -4394,7 +4648,7 @@
       <c r="G115" s="41"/>
       <c r="H115" s="41"/>
       <c r="I115" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J115" s="45"/>
@@ -4412,7 +4666,7 @@
       <c r="G116" s="41"/>
       <c r="H116" s="41"/>
       <c r="I116" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J116" s="45"/>
@@ -4430,7 +4684,7 @@
       <c r="G117" s="41"/>
       <c r="H117" s="41"/>
       <c r="I117" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J117" s="45"/>
@@ -4448,7 +4702,7 @@
       <c r="G118" s="41"/>
       <c r="H118" s="41"/>
       <c r="I118" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J118" s="45"/>
@@ -4466,7 +4720,7 @@
       <c r="G119" s="41"/>
       <c r="H119" s="41"/>
       <c r="I119" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J119" s="45"/>
@@ -4484,7 +4738,7 @@
       <c r="G120" s="41"/>
       <c r="H120" s="41"/>
       <c r="I120" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J120" s="45"/>
@@ -4500,23 +4754,23 @@
       </c>
       <c r="F121" s="15"/>
       <c r="G121" s="18">
-        <f t="shared" ref="G121:H121" si="10">SUM(G111:G120)</f>
+        <f t="shared" ref="G121:H121" si="8">SUM(G111:G120)</f>
         <v>0</v>
       </c>
       <c r="H121" s="18">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I121" s="18">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J121" s="19"/>
       <c r="K121" s="46"/>
     </row>
     <row r="122" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="57" t="s">
-        <v>26</v>
+      <c r="A122" s="61" t="s">
+        <v>24</v>
       </c>
       <c r="B122" s="55"/>
       <c r="C122" s="55"/>
@@ -4530,10 +4784,10 @@
       <c r="K122" s="56"/>
     </row>
     <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A123" s="29" t="s">
+      <c r="A123" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B123" s="75" t="s">
+      <c r="B123" s="54" t="s">
         <v>13</v>
       </c>
       <c r="C123" s="55"/>
@@ -4546,11 +4800,11 @@
       <c r="J123" s="55"/>
       <c r="K123" s="56"/>
     </row>
-    <row r="124" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="30" t="s">
+    <row r="124" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B124" s="75" t="s">
+      <c r="B124" s="54" t="s">
         <v>15</v>
       </c>
       <c r="C124" s="55"/>
@@ -4575,7 +4829,7 @@
       <c r="G125" s="41"/>
       <c r="H125" s="41"/>
       <c r="I125" s="41">
-        <f t="shared" ref="I125:I135" si="11">H125-G125</f>
+        <f t="shared" ref="I125:I135" si="9">H125-G125</f>
         <v>0</v>
       </c>
       <c r="J125" s="45"/>
@@ -4593,7 +4847,7 @@
       <c r="G126" s="41"/>
       <c r="H126" s="41"/>
       <c r="I126" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J126" s="45"/>
@@ -4611,11 +4865,13 @@
       <c r="G127" s="41"/>
       <c r="H127" s="41"/>
       <c r="I127" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J127" s="45"/>
-      <c r="K127" s="43"/>
+      <c r="K127" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A128" s="37"/>
@@ -4629,7 +4885,7 @@
       <c r="G128" s="41"/>
       <c r="H128" s="41"/>
       <c r="I128" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J128" s="45"/>
@@ -4647,7 +4903,7 @@
       <c r="G129" s="41"/>
       <c r="H129" s="41"/>
       <c r="I129" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J129" s="45"/>
@@ -4665,7 +4921,7 @@
       <c r="G130" s="41"/>
       <c r="H130" s="41"/>
       <c r="I130" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J130" s="45"/>
@@ -4683,7 +4939,7 @@
       <c r="G131" s="41"/>
       <c r="H131" s="41"/>
       <c r="I131" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J131" s="45"/>
@@ -4701,7 +4957,7 @@
       <c r="G132" s="41"/>
       <c r="H132" s="41"/>
       <c r="I132" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J132" s="45"/>
@@ -4719,7 +4975,7 @@
       <c r="G133" s="41"/>
       <c r="H133" s="41"/>
       <c r="I133" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J133" s="45"/>
@@ -4737,7 +4993,7 @@
       <c r="G134" s="41"/>
       <c r="H134" s="41"/>
       <c r="I134" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J134" s="45"/>
@@ -4753,68 +5009,68 @@
       </c>
       <c r="F135" s="15"/>
       <c r="G135" s="18">
-        <f t="shared" ref="G135:H135" si="12">SUM(G125:G134)</f>
+        <f t="shared" ref="G135:H135" si="10">SUM(G125:G134)</f>
         <v>0</v>
       </c>
       <c r="H135" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="I135" s="18">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J135" s="19"/>
       <c r="K135" s="46"/>
     </row>
     <row r="136" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="62" t="s">
-        <v>27</v>
-      </c>
-      <c r="B136" s="63"/>
-      <c r="C136" s="63"/>
-      <c r="D136" s="63"/>
-      <c r="E136" s="63"/>
-      <c r="F136" s="63"/>
-      <c r="G136" s="63"/>
-      <c r="H136" s="63"/>
-      <c r="I136" s="63"/>
-      <c r="J136" s="63"/>
-      <c r="K136" s="64"/>
+      <c r="A136" s="57" t="s">
+        <v>26</v>
+      </c>
+      <c r="B136" s="55"/>
+      <c r="C136" s="55"/>
+      <c r="D136" s="55"/>
+      <c r="E136" s="55"/>
+      <c r="F136" s="55"/>
+      <c r="G136" s="55"/>
+      <c r="H136" s="55"/>
+      <c r="I136" s="55"/>
+      <c r="J136" s="55"/>
+      <c r="K136" s="56"/>
     </row>
     <row r="137" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A137" s="32" t="s">
+      <c r="A137" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B137" s="65" t="s">
+      <c r="B137" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C137" s="63"/>
-      <c r="D137" s="63"/>
-      <c r="E137" s="63"/>
-      <c r="F137" s="63"/>
-      <c r="G137" s="63"/>
-      <c r="H137" s="63"/>
-      <c r="I137" s="63"/>
-      <c r="J137" s="63"/>
-      <c r="K137" s="64"/>
+      <c r="C137" s="55"/>
+      <c r="D137" s="55"/>
+      <c r="E137" s="55"/>
+      <c r="F137" s="55"/>
+      <c r="G137" s="55"/>
+      <c r="H137" s="55"/>
+      <c r="I137" s="55"/>
+      <c r="J137" s="55"/>
+      <c r="K137" s="56"/>
     </row>
     <row r="138" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="33" t="s">
+      <c r="A138" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B138" s="65" t="s">
+      <c r="B138" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C138" s="63"/>
-      <c r="D138" s="63"/>
-      <c r="E138" s="63"/>
-      <c r="F138" s="63"/>
-      <c r="G138" s="63"/>
-      <c r="H138" s="63"/>
-      <c r="I138" s="63"/>
-      <c r="J138" s="63"/>
-      <c r="K138" s="64"/>
+      <c r="C138" s="55"/>
+      <c r="D138" s="55"/>
+      <c r="E138" s="55"/>
+      <c r="F138" s="55"/>
+      <c r="G138" s="55"/>
+      <c r="H138" s="55"/>
+      <c r="I138" s="55"/>
+      <c r="J138" s="55"/>
+      <c r="K138" s="56"/>
     </row>
     <row r="139" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A139" s="37"/>
@@ -4828,7 +5084,7 @@
       <c r="G139" s="41"/>
       <c r="H139" s="41"/>
       <c r="I139" s="41">
-        <f t="shared" ref="I139:I149" si="13">H139-G139</f>
+        <f t="shared" ref="I139:I149" si="11">H139-G139</f>
         <v>0</v>
       </c>
       <c r="J139" s="45"/>
@@ -4846,7 +5102,7 @@
       <c r="G140" s="41"/>
       <c r="H140" s="41"/>
       <c r="I140" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J140" s="45"/>
@@ -4864,7 +5120,7 @@
       <c r="G141" s="41"/>
       <c r="H141" s="41"/>
       <c r="I141" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J141" s="45"/>
@@ -4882,7 +5138,7 @@
       <c r="G142" s="41"/>
       <c r="H142" s="41"/>
       <c r="I142" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J142" s="45"/>
@@ -4900,7 +5156,7 @@
       <c r="G143" s="41"/>
       <c r="H143" s="41"/>
       <c r="I143" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J143" s="45"/>
@@ -4918,7 +5174,7 @@
       <c r="G144" s="41"/>
       <c r="H144" s="41"/>
       <c r="I144" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J144" s="45"/>
@@ -4936,7 +5192,7 @@
       <c r="G145" s="41"/>
       <c r="H145" s="41"/>
       <c r="I145" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J145" s="45"/>
@@ -4954,7 +5210,7 @@
       <c r="G146" s="41"/>
       <c r="H146" s="41"/>
       <c r="I146" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J146" s="45"/>
@@ -4972,7 +5228,7 @@
       <c r="G147" s="41"/>
       <c r="H147" s="41"/>
       <c r="I147" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J147" s="45"/>
@@ -4990,42 +5246,295 @@
       <c r="G148" s="41"/>
       <c r="H148" s="41"/>
       <c r="I148" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J148" s="45"/>
       <c r="K148" s="43"/>
     </row>
     <row r="149" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A149" s="48"/>
-      <c r="B149" s="49"/>
-      <c r="C149" s="49"/>
-      <c r="D149" s="49"/>
-      <c r="E149" s="49" t="s">
+      <c r="A149" s="13"/>
+      <c r="B149" s="15"/>
+      <c r="C149" s="15"/>
+      <c r="D149" s="15"/>
+      <c r="E149" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F149" s="49"/>
-      <c r="G149" s="50">
-        <f t="shared" ref="G149:H149" si="14">SUM(G139:G148)</f>
-        <v>0</v>
-      </c>
-      <c r="H149" s="50">
+      <c r="F149" s="15"/>
+      <c r="G149" s="18">
+        <f t="shared" ref="G149:H149" si="12">SUM(G139:G148)</f>
+        <v>0</v>
+      </c>
+      <c r="H149" s="18">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="I149" s="18">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J149" s="19"/>
+      <c r="K149" s="46"/>
+    </row>
+    <row r="150" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="62" t="s">
+        <v>27</v>
+      </c>
+      <c r="B150" s="63"/>
+      <c r="C150" s="63"/>
+      <c r="D150" s="63"/>
+      <c r="E150" s="63"/>
+      <c r="F150" s="63"/>
+      <c r="G150" s="63"/>
+      <c r="H150" s="63"/>
+      <c r="I150" s="63"/>
+      <c r="J150" s="63"/>
+      <c r="K150" s="64"/>
+    </row>
+    <row r="151" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A151" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B151" s="65" t="s">
+        <v>13</v>
+      </c>
+      <c r="C151" s="63"/>
+      <c r="D151" s="63"/>
+      <c r="E151" s="63"/>
+      <c r="F151" s="63"/>
+      <c r="G151" s="63"/>
+      <c r="H151" s="63"/>
+      <c r="I151" s="63"/>
+      <c r="J151" s="63"/>
+      <c r="K151" s="64"/>
+    </row>
+    <row r="152" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B152" s="65" t="s">
+        <v>15</v>
+      </c>
+      <c r="C152" s="63"/>
+      <c r="D152" s="63"/>
+      <c r="E152" s="63"/>
+      <c r="F152" s="63"/>
+      <c r="G152" s="63"/>
+      <c r="H152" s="63"/>
+      <c r="I152" s="63"/>
+      <c r="J152" s="63"/>
+      <c r="K152" s="64"/>
+    </row>
+    <row r="153" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A153" s="37"/>
+      <c r="B153" s="38"/>
+      <c r="C153" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D153" s="38"/>
+      <c r="E153" s="40"/>
+      <c r="F153" s="40"/>
+      <c r="G153" s="41"/>
+      <c r="H153" s="41"/>
+      <c r="I153" s="41">
+        <f t="shared" ref="I153:I163" si="13">H153-G153</f>
+        <v>0</v>
+      </c>
+      <c r="J153" s="45"/>
+      <c r="K153" s="43"/>
+    </row>
+    <row r="154" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A154" s="37"/>
+      <c r="B154" s="38"/>
+      <c r="C154" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D154" s="38"/>
+      <c r="E154" s="40"/>
+      <c r="F154" s="40"/>
+      <c r="G154" s="41"/>
+      <c r="H154" s="41"/>
+      <c r="I154" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J154" s="45"/>
+      <c r="K154" s="43"/>
+    </row>
+    <row r="155" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A155" s="37"/>
+      <c r="B155" s="38"/>
+      <c r="C155" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D155" s="38"/>
+      <c r="E155" s="40"/>
+      <c r="F155" s="40"/>
+      <c r="G155" s="41"/>
+      <c r="H155" s="41"/>
+      <c r="I155" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J155" s="45"/>
+      <c r="K155" s="43"/>
+    </row>
+    <row r="156" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A156" s="37"/>
+      <c r="B156" s="38"/>
+      <c r="C156" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D156" s="38"/>
+      <c r="E156" s="40"/>
+      <c r="F156" s="40"/>
+      <c r="G156" s="41"/>
+      <c r="H156" s="41"/>
+      <c r="I156" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J156" s="45"/>
+      <c r="K156" s="43"/>
+    </row>
+    <row r="157" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A157" s="37"/>
+      <c r="B157" s="38"/>
+      <c r="C157" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D157" s="38"/>
+      <c r="E157" s="40"/>
+      <c r="F157" s="40"/>
+      <c r="G157" s="41"/>
+      <c r="H157" s="41"/>
+      <c r="I157" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J157" s="45"/>
+      <c r="K157" s="43"/>
+    </row>
+    <row r="158" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A158" s="37"/>
+      <c r="B158" s="38"/>
+      <c r="C158" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D158" s="38"/>
+      <c r="E158" s="40"/>
+      <c r="F158" s="40"/>
+      <c r="G158" s="41"/>
+      <c r="H158" s="41"/>
+      <c r="I158" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J158" s="45"/>
+      <c r="K158" s="43"/>
+    </row>
+    <row r="159" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A159" s="37"/>
+      <c r="B159" s="38"/>
+      <c r="C159" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D159" s="38"/>
+      <c r="E159" s="40"/>
+      <c r="F159" s="40"/>
+      <c r="G159" s="41"/>
+      <c r="H159" s="41"/>
+      <c r="I159" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J159" s="45"/>
+      <c r="K159" s="43"/>
+    </row>
+    <row r="160" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A160" s="37"/>
+      <c r="B160" s="38"/>
+      <c r="C160" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D160" s="38"/>
+      <c r="E160" s="40"/>
+      <c r="F160" s="40"/>
+      <c r="G160" s="41"/>
+      <c r="H160" s="41"/>
+      <c r="I160" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J160" s="45"/>
+      <c r="K160" s="43"/>
+    </row>
+    <row r="161" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A161" s="37"/>
+      <c r="B161" s="38"/>
+      <c r="C161" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D161" s="38"/>
+      <c r="E161" s="40"/>
+      <c r="F161" s="40"/>
+      <c r="G161" s="41"/>
+      <c r="H161" s="41"/>
+      <c r="I161" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J161" s="45"/>
+      <c r="K161" s="43"/>
+    </row>
+    <row r="162" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A162" s="37"/>
+      <c r="B162" s="38"/>
+      <c r="C162" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D162" s="38"/>
+      <c r="E162" s="40"/>
+      <c r="F162" s="40"/>
+      <c r="G162" s="41"/>
+      <c r="H162" s="41"/>
+      <c r="I162" s="41">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="J162" s="45"/>
+      <c r="K162" s="43"/>
+    </row>
+    <row r="163" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A163" s="48"/>
+      <c r="B163" s="49"/>
+      <c r="C163" s="49"/>
+      <c r="D163" s="49"/>
+      <c r="E163" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="F163" s="49"/>
+      <c r="G163" s="50">
+        <f t="shared" ref="G163:H163" si="14">SUM(G153:G162)</f>
+        <v>0</v>
+      </c>
+      <c r="H163" s="50">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="I149" s="50">
+      <c r="I163" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J149" s="51"/>
-      <c r="K149" s="52"/>
+      <c r="J163" s="51"/>
+      <c r="K163" s="52"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{ABCA17DA-9000-40D6-9FD8-97574B35A77E}">
+      <autoFilter ref="A1:K15" xr:uid="{21B2745E-3BE8-45F1-A565-B45E72302408}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5036,32 +5545,32 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A136:K136"/>
-    <mergeCell ref="B137:K137"/>
-    <mergeCell ref="B138:K138"/>
+    <mergeCell ref="A150:K150"/>
+    <mergeCell ref="B151:K151"/>
+    <mergeCell ref="B152:K152"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
-    <mergeCell ref="A46:K46"/>
-    <mergeCell ref="B47:K47"/>
+    <mergeCell ref="A47:K47"/>
     <mergeCell ref="B48:K48"/>
-    <mergeCell ref="A66:K66"/>
-    <mergeCell ref="B67:K67"/>
-    <mergeCell ref="B68:K68"/>
+    <mergeCell ref="B49:K49"/>
     <mergeCell ref="A80:K80"/>
+    <mergeCell ref="B81:K81"/>
+    <mergeCell ref="B82:K82"/>
+    <mergeCell ref="A94:K94"/>
+    <mergeCell ref="B137:K137"/>
+    <mergeCell ref="B138:K138"/>
+    <mergeCell ref="B95:K95"/>
     <mergeCell ref="B123:K123"/>
     <mergeCell ref="B124:K124"/>
-    <mergeCell ref="B81:K81"/>
+    <mergeCell ref="A136:K136"/>
+    <mergeCell ref="B96:K96"/>
+    <mergeCell ref="A108:K108"/>
     <mergeCell ref="B109:K109"/>
     <mergeCell ref="B110:K110"/>
     <mergeCell ref="A122:K122"/>
-    <mergeCell ref="B82:K82"/>
-    <mergeCell ref="A94:K94"/>
-    <mergeCell ref="B95:K95"/>
-    <mergeCell ref="B96:K96"/>
-    <mergeCell ref="A108:K108"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B44 B47:B64 B69:B78 B83:B92 B97:B106 B111:B120 B125:B134">
+  <conditionalFormatting sqref="B5:B45 B48:B78 B83:B92 B97:B106 B111:B120 B125:B134 B139:B148">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5078,7 +5587,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B45 B47:B65 B67:B79 B81:B93 B95:B107 B109:B121 B123:B135 B137:B149">
+  <conditionalFormatting sqref="B5:B46 B48:B79 B81:B93 B95:B107 B109:B121 B123:B135 B137:B149 B151:B163">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5086,34 +5595,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B139:B148">
+  <conditionalFormatting sqref="B153:B162">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B139))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B153))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B139))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B153))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B139))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B153))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B139))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B153))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B139))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B153))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G45 G49:G65 G69:G79 G83:G93 G97:G107 G111:G121 G125:G135 G139:G149">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G79 G83:G93 G97:G107 G111:G121 G125:G135 G139:G149 G153:G163">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H149">
+  <conditionalFormatting sqref="H1:H163">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I45 I49:I65 I69:I79 I83:I93 I97:I107 I111:I121 I125:I135 I139:I149">
+  <conditionalFormatting sqref="I83:I93 I97:I107 I111:I121 I125:I135 I139:I149 I153:I163 I5:I46 I50:I79">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -5122,7 +5631,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F139:F148 F125:F134 F49:F64 F69:F78 F83:F92 F97:F106 F111:F120 F5:F44" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F153:F162 F139:F148 F50:F78 F83:F92 F97:F106 F111:F120 F125:F134 F5:F45" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5138,13 +5647,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E44 E49:E64 E69:E78 E83:E92 E97:E106 E111:E120 E125:E134 E139:E148</xm:sqref>
+          <xm:sqref>E5:E45 E50:E78 E83:E92 E97:E106 E111:E120 E125:E134 E139:E148 E153:E162</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B44 B49:B64 B69:B78 B83:B92 B97:B106 B111:B120 B125:B134 B139:B148</xm:sqref>
+          <xm:sqref>B5:B45 B50:B78 B83:B92 B97:B106 B111:B120 B125:B134 B139:B148 B153:B162</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5224,7 +5733,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" cm="1">
-        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$49:$H$64,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
+        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$50:$H$77,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" cm="1">

</xml_diff>

<commit_message>
W2 Datalab 2 Work II (Post-datalab)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36866D89-51B8-4503-BC92-3B7574B7C72B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{093DA171-1404-43AB-AD4A-10387CF7CE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$148</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$151</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="160">
   <si>
     <t>Date</t>
   </si>
@@ -570,6 +570,18 @@
   </si>
   <si>
     <t>Attempt to apply for retake of Python Exam</t>
+  </si>
+  <si>
+    <t>0,75 at 13:00</t>
+  </si>
+  <si>
+    <t>1-on-1 feedback session with mentor</t>
+  </si>
+  <si>
+    <t>Re-write Learning Log Section A and SMARTER Goals</t>
+  </si>
+  <si>
+    <t>Re-write Week 1 and 2 reflection and feedback</t>
   </si>
 </sst>
 </file>
@@ -1055,26 +1067,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1091,6 +1083,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1108,6 +1102,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1580,7 +1592,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K163"/>
+  <dimension ref="A1:K166"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1632,53 +1644,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -1881,7 +1893,7 @@
         <v>45614</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C11" s="39" t="s">
         <v>17</v>
@@ -2232,9 +2244,7 @@
         <v>0</v>
       </c>
       <c r="J21" s="45"/>
-      <c r="K21" s="44" t="s">
-        <v>94</v>
-      </c>
+      <c r="K21" s="44"/>
     </row>
     <row r="22" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A22" s="37">
@@ -3019,53 +3029,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="62"/>
+      <c r="K49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -3093,7 +3103,7 @@
         <v>0.5</v>
       </c>
       <c r="I50" s="41">
-        <f t="shared" ref="I50:I79" si="1">H50-G50</f>
+        <f t="shared" ref="I50:I82" si="1">H50-G50</f>
         <v>0</v>
       </c>
       <c r="J50" s="45"/>
@@ -3814,7 +3824,7 @@
         <v>45625</v>
       </c>
       <c r="B73" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C73" s="39" t="s">
         <v>17</v>
@@ -3831,10 +3841,12 @@
       <c r="G73" s="41">
         <v>1</v>
       </c>
-      <c r="H73" s="41"/>
+      <c r="H73" s="41">
+        <v>0.75</v>
+      </c>
       <c r="I73" s="41">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>-0.25</v>
       </c>
       <c r="J73" s="45"/>
       <c r="K73" s="43"/>
@@ -3899,32 +3911,38 @@
         <v>-4</v>
       </c>
       <c r="J75" s="45"/>
-      <c r="K75" s="43"/>
+      <c r="K75" s="43" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="76" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A76" s="47">
         <v>45625</v>
       </c>
       <c r="B76" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C76" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D76" s="38" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="E76" s="40" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="F76" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="G76" s="41"/>
-      <c r="H76" s="41"/>
+      <c r="G76" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H76" s="41">
+        <v>0.33</v>
+      </c>
       <c r="I76" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8.0000000000000016E-2</v>
       </c>
       <c r="J76" s="45"/>
       <c r="K76" s="43"/>
@@ -3934,16 +3952,16 @@
         <v>45625</v>
       </c>
       <c r="B77" s="38" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="C77" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D77" s="38" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="E77" s="40" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F77" s="40" t="s">
         <v>88</v>
@@ -3962,16 +3980,16 @@
         <v>45625</v>
       </c>
       <c r="B78" s="38" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="C78" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D78" s="38" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="E78" s="40" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F78" s="40" t="s">
         <v>88</v>
@@ -3986,131 +4004,167 @@
       <c r="K78" s="43"/>
     </row>
     <row r="79" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A79" s="13"/>
-      <c r="B79" s="15"/>
-      <c r="C79" s="15"/>
-      <c r="D79" s="15"/>
-      <c r="E79" s="15" t="s">
+      <c r="A79" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B79" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C79" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D79" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E79" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F79" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G79" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H79" s="41"/>
+      <c r="I79" s="41">
+        <f t="shared" si="1"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J79" s="45"/>
+      <c r="K79" s="43"/>
+    </row>
+    <row r="80" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A80" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B80" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C80" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D80" s="38" t="s">
+        <v>151</v>
+      </c>
+      <c r="E80" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F80" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G80" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H80" s="41"/>
+      <c r="I80" s="41">
+        <f t="shared" si="1"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J80" s="45"/>
+      <c r="K80" s="43"/>
+    </row>
+    <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A81" s="47">
+        <v>45625</v>
+      </c>
+      <c r="B81" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C81" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D81" s="38" t="s">
+        <v>150</v>
+      </c>
+      <c r="E81" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F81" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G81" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H81" s="41"/>
+      <c r="I81" s="41">
+        <f t="shared" si="1"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J81" s="45"/>
+      <c r="K81" s="43"/>
+    </row>
+    <row r="82" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A82" s="13"/>
+      <c r="B82" s="15"/>
+      <c r="C82" s="15"/>
+      <c r="D82" s="15"/>
+      <c r="E82" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F79" s="15"/>
-      <c r="G79" s="18">
-        <f t="shared" ref="G79:H79" si="2">SUM(G48:G77)</f>
-        <v>31.85</v>
-      </c>
-      <c r="H79" s="18">
-        <f t="shared" si="2"/>
-        <v>26.599999999999998</v>
-      </c>
-      <c r="I79" s="18">
+      <c r="F82" s="15"/>
+      <c r="G82" s="18">
+        <f>SUM(G48:G81)</f>
+        <v>32.85</v>
+      </c>
+      <c r="H82" s="18">
+        <f>SUM(H48:H81)</f>
+        <v>27.679999999999996</v>
+      </c>
+      <c r="I82" s="18">
         <f t="shared" si="1"/>
-        <v>-5.2500000000000036</v>
-      </c>
-      <c r="J79" s="19"/>
-      <c r="K79" s="46"/>
-    </row>
-    <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="72" t="s">
+        <v>-5.1700000000000053</v>
+      </c>
+      <c r="J82" s="19"/>
+      <c r="K82" s="46"/>
+    </row>
+    <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B80" s="55"/>
-      <c r="C80" s="55"/>
-      <c r="D80" s="55"/>
-      <c r="E80" s="55"/>
-      <c r="F80" s="55"/>
-      <c r="G80" s="55"/>
-      <c r="H80" s="55"/>
-      <c r="I80" s="55"/>
-      <c r="J80" s="55"/>
-      <c r="K80" s="56"/>
-    </row>
-    <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A81" s="21" t="s">
+      <c r="B83" s="62"/>
+      <c r="C83" s="62"/>
+      <c r="D83" s="62"/>
+      <c r="E83" s="62"/>
+      <c r="F83" s="62"/>
+      <c r="G83" s="62"/>
+      <c r="H83" s="62"/>
+      <c r="I83" s="62"/>
+      <c r="J83" s="62"/>
+      <c r="K83" s="63"/>
+    </row>
+    <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B81" s="73" t="s">
+      <c r="B84" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C81" s="55"/>
-      <c r="D81" s="55"/>
-      <c r="E81" s="55"/>
-      <c r="F81" s="55"/>
-      <c r="G81" s="55"/>
-      <c r="H81" s="55"/>
-      <c r="I81" s="55"/>
-      <c r="J81" s="55"/>
-      <c r="K81" s="56"/>
-    </row>
-    <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="22" t="s">
+      <c r="C84" s="62"/>
+      <c r="D84" s="62"/>
+      <c r="E84" s="62"/>
+      <c r="F84" s="62"/>
+      <c r="G84" s="62"/>
+      <c r="H84" s="62"/>
+      <c r="I84" s="62"/>
+      <c r="J84" s="62"/>
+      <c r="K84" s="63"/>
+    </row>
+    <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="73" t="s">
+      <c r="B85" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C82" s="55"/>
-      <c r="D82" s="55"/>
-      <c r="E82" s="55"/>
-      <c r="F82" s="55"/>
-      <c r="G82" s="55"/>
-      <c r="H82" s="55"/>
-      <c r="I82" s="55"/>
-      <c r="J82" s="55"/>
-      <c r="K82" s="56"/>
-    </row>
-    <row r="83" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A83" s="37"/>
-      <c r="B83" s="38"/>
-      <c r="C83" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D83" s="38"/>
-      <c r="E83" s="40"/>
-      <c r="F83" s="40"/>
-      <c r="G83" s="41"/>
-      <c r="H83" s="41"/>
-      <c r="I83" s="41">
-        <f t="shared" ref="I83:I93" si="3">H83-G83</f>
-        <v>0</v>
-      </c>
-      <c r="J83" s="45"/>
-      <c r="K83" s="43"/>
-    </row>
-    <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A84" s="37"/>
-      <c r="B84" s="38"/>
-      <c r="C84" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D84" s="38"/>
-      <c r="E84" s="40"/>
-      <c r="F84" s="40"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="41"/>
-      <c r="I84" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J84" s="45"/>
-      <c r="K84" s="43"/>
-    </row>
-    <row r="85" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A85" s="37"/>
-      <c r="B85" s="38"/>
-      <c r="C85" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D85" s="38"/>
-      <c r="E85" s="40"/>
-      <c r="F85" s="40"/>
-      <c r="G85" s="41"/>
-      <c r="H85" s="41"/>
-      <c r="I85" s="41">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J85" s="45"/>
-      <c r="K85" s="43"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="62"/>
+      <c r="G85" s="62"/>
+      <c r="H85" s="62"/>
+      <c r="I85" s="62"/>
+      <c r="J85" s="62"/>
+      <c r="K85" s="63"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="37"/>
@@ -4124,7 +4178,7 @@
       <c r="G86" s="41"/>
       <c r="H86" s="41"/>
       <c r="I86" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="I86:I96" si="2">H86-G86</f>
         <v>0</v>
       </c>
       <c r="J86" s="45"/>
@@ -4142,7 +4196,7 @@
       <c r="G87" s="41"/>
       <c r="H87" s="41"/>
       <c r="I87" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J87" s="45"/>
@@ -4160,7 +4214,7 @@
       <c r="G88" s="41"/>
       <c r="H88" s="41"/>
       <c r="I88" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J88" s="45"/>
@@ -4178,7 +4232,7 @@
       <c r="G89" s="41"/>
       <c r="H89" s="41"/>
       <c r="I89" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J89" s="45"/>
@@ -4196,7 +4250,7 @@
       <c r="G90" s="41"/>
       <c r="H90" s="41"/>
       <c r="I90" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J90" s="45"/>
@@ -4214,7 +4268,7 @@
       <c r="G91" s="41"/>
       <c r="H91" s="41"/>
       <c r="I91" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J91" s="45"/>
@@ -4232,138 +4286,138 @@
       <c r="G92" s="41"/>
       <c r="H92" s="41"/>
       <c r="I92" s="41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J92" s="45"/>
       <c r="K92" s="43"/>
     </row>
     <row r="93" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A93" s="13"/>
-      <c r="B93" s="15"/>
-      <c r="C93" s="15"/>
-      <c r="D93" s="15"/>
-      <c r="E93" s="15" t="s">
+      <c r="A93" s="37"/>
+      <c r="B93" s="38"/>
+      <c r="C93" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D93" s="38"/>
+      <c r="E93" s="40"/>
+      <c r="F93" s="40"/>
+      <c r="G93" s="41"/>
+      <c r="H93" s="41"/>
+      <c r="I93" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J93" s="45"/>
+      <c r="K93" s="43"/>
+    </row>
+    <row r="94" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A94" s="37"/>
+      <c r="B94" s="38"/>
+      <c r="C94" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D94" s="38"/>
+      <c r="E94" s="40"/>
+      <c r="F94" s="40"/>
+      <c r="G94" s="41"/>
+      <c r="H94" s="41"/>
+      <c r="I94" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J94" s="45"/>
+      <c r="K94" s="43"/>
+    </row>
+    <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A95" s="37"/>
+      <c r="B95" s="38"/>
+      <c r="C95" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D95" s="38"/>
+      <c r="E95" s="40"/>
+      <c r="F95" s="40"/>
+      <c r="G95" s="41"/>
+      <c r="H95" s="41"/>
+      <c r="I95" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J95" s="45"/>
+      <c r="K95" s="43"/>
+    </row>
+    <row r="96" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A96" s="13"/>
+      <c r="B96" s="15"/>
+      <c r="C96" s="15"/>
+      <c r="D96" s="15"/>
+      <c r="E96" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F93" s="15"/>
-      <c r="G93" s="18">
-        <f t="shared" ref="G93:H93" si="4">SUM(G83:G92)</f>
-        <v>0</v>
-      </c>
-      <c r="H93" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I93" s="18">
+      <c r="F96" s="15"/>
+      <c r="G96" s="18">
+        <f t="shared" ref="G96:H96" si="3">SUM(G86:G95)</f>
+        <v>0</v>
+      </c>
+      <c r="H96" s="18">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J93" s="19"/>
-      <c r="K93" s="46"/>
-    </row>
-    <row r="94" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="74" t="s">
+      <c r="I96" s="18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J96" s="19"/>
+      <c r="K96" s="46"/>
+    </row>
+    <row r="97" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B94" s="55"/>
-      <c r="C94" s="55"/>
-      <c r="D94" s="55"/>
-      <c r="E94" s="55"/>
-      <c r="F94" s="55"/>
-      <c r="G94" s="55"/>
-      <c r="H94" s="55"/>
-      <c r="I94" s="55"/>
-      <c r="J94" s="55"/>
-      <c r="K94" s="56"/>
-    </row>
-    <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A95" s="23" t="s">
+      <c r="B97" s="62"/>
+      <c r="C97" s="62"/>
+      <c r="D97" s="62"/>
+      <c r="E97" s="62"/>
+      <c r="F97" s="62"/>
+      <c r="G97" s="62"/>
+      <c r="H97" s="62"/>
+      <c r="I97" s="62"/>
+      <c r="J97" s="62"/>
+      <c r="K97" s="63"/>
+    </row>
+    <row r="98" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A98" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B95" s="58" t="s">
+      <c r="B98" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C95" s="55"/>
-      <c r="D95" s="55"/>
-      <c r="E95" s="55"/>
-      <c r="F95" s="55"/>
-      <c r="G95" s="55"/>
-      <c r="H95" s="55"/>
-      <c r="I95" s="55"/>
-      <c r="J95" s="55"/>
-      <c r="K95" s="56"/>
-    </row>
-    <row r="96" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="24" t="s">
+      <c r="C98" s="62"/>
+      <c r="D98" s="62"/>
+      <c r="E98" s="62"/>
+      <c r="F98" s="62"/>
+      <c r="G98" s="62"/>
+      <c r="H98" s="62"/>
+      <c r="I98" s="62"/>
+      <c r="J98" s="62"/>
+      <c r="K98" s="63"/>
+    </row>
+    <row r="99" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B96" s="58" t="s">
+      <c r="B99" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C96" s="55"/>
-      <c r="D96" s="55"/>
-      <c r="E96" s="55"/>
-      <c r="F96" s="55"/>
-      <c r="G96" s="55"/>
-      <c r="H96" s="55"/>
-      <c r="I96" s="55"/>
-      <c r="J96" s="55"/>
-      <c r="K96" s="56"/>
-    </row>
-    <row r="97" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A97" s="37"/>
-      <c r="B97" s="38"/>
-      <c r="C97" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D97" s="38"/>
-      <c r="E97" s="40"/>
-      <c r="F97" s="40"/>
-      <c r="G97" s="41"/>
-      <c r="H97" s="41"/>
-      <c r="I97" s="41">
-        <f t="shared" ref="I97:I107" si="5">H97-G97</f>
-        <v>0</v>
-      </c>
-      <c r="J97" s="45"/>
-      <c r="K97" s="43"/>
-    </row>
-    <row r="98" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A98" s="37"/>
-      <c r="B98" s="38"/>
-      <c r="C98" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D98" s="38"/>
-      <c r="E98" s="40"/>
-      <c r="F98" s="40"/>
-      <c r="G98" s="41"/>
-      <c r="H98" s="41"/>
-      <c r="I98" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J98" s="45"/>
-      <c r="K98" s="43"/>
-    </row>
-    <row r="99" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A99" s="37"/>
-      <c r="B99" s="38"/>
-      <c r="C99" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D99" s="38"/>
-      <c r="E99" s="40"/>
-      <c r="F99" s="40"/>
-      <c r="G99" s="41"/>
-      <c r="H99" s="41"/>
-      <c r="I99" s="41">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J99" s="45"/>
-      <c r="K99" s="43"/>
+      <c r="C99" s="62"/>
+      <c r="D99" s="62"/>
+      <c r="E99" s="62"/>
+      <c r="F99" s="62"/>
+      <c r="G99" s="62"/>
+      <c r="H99" s="62"/>
+      <c r="I99" s="62"/>
+      <c r="J99" s="62"/>
+      <c r="K99" s="63"/>
     </row>
     <row r="100" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A100" s="37"/>
@@ -4377,7 +4431,7 @@
       <c r="G100" s="41"/>
       <c r="H100" s="41"/>
       <c r="I100" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I100:I110" si="4">H100-G100</f>
         <v>0</v>
       </c>
       <c r="J100" s="45"/>
@@ -4395,7 +4449,7 @@
       <c r="G101" s="41"/>
       <c r="H101" s="41"/>
       <c r="I101" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J101" s="45"/>
@@ -4413,7 +4467,7 @@
       <c r="G102" s="41"/>
       <c r="H102" s="41"/>
       <c r="I102" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J102" s="45"/>
@@ -4431,7 +4485,7 @@
       <c r="G103" s="41"/>
       <c r="H103" s="41"/>
       <c r="I103" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J103" s="45"/>
@@ -4449,7 +4503,7 @@
       <c r="G104" s="41"/>
       <c r="H104" s="41"/>
       <c r="I104" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J104" s="45"/>
@@ -4467,7 +4521,7 @@
       <c r="G105" s="41"/>
       <c r="H105" s="41"/>
       <c r="I105" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J105" s="45"/>
@@ -4485,138 +4539,138 @@
       <c r="G106" s="41"/>
       <c r="H106" s="41"/>
       <c r="I106" s="41">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J106" s="45"/>
       <c r="K106" s="43"/>
     </row>
     <row r="107" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A107" s="13"/>
-      <c r="B107" s="15"/>
-      <c r="C107" s="15"/>
-      <c r="D107" s="15"/>
-      <c r="E107" s="15" t="s">
+      <c r="A107" s="37"/>
+      <c r="B107" s="38"/>
+      <c r="C107" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D107" s="38"/>
+      <c r="E107" s="40"/>
+      <c r="F107" s="40"/>
+      <c r="G107" s="41"/>
+      <c r="H107" s="41"/>
+      <c r="I107" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J107" s="45"/>
+      <c r="K107" s="43"/>
+    </row>
+    <row r="108" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A108" s="37"/>
+      <c r="B108" s="38"/>
+      <c r="C108" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D108" s="38"/>
+      <c r="E108" s="40"/>
+      <c r="F108" s="40"/>
+      <c r="G108" s="41"/>
+      <c r="H108" s="41"/>
+      <c r="I108" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J108" s="45"/>
+      <c r="K108" s="43"/>
+    </row>
+    <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A109" s="37"/>
+      <c r="B109" s="38"/>
+      <c r="C109" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D109" s="38"/>
+      <c r="E109" s="40"/>
+      <c r="F109" s="40"/>
+      <c r="G109" s="41"/>
+      <c r="H109" s="41"/>
+      <c r="I109" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J109" s="45"/>
+      <c r="K109" s="43"/>
+    </row>
+    <row r="110" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A110" s="13"/>
+      <c r="B110" s="15"/>
+      <c r="C110" s="15"/>
+      <c r="D110" s="15"/>
+      <c r="E110" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F107" s="15"/>
-      <c r="G107" s="18">
-        <f t="shared" ref="G107:H107" si="6">SUM(G97:G106)</f>
-        <v>0</v>
-      </c>
-      <c r="H107" s="18">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="I107" s="18">
+      <c r="F110" s="15"/>
+      <c r="G110" s="18">
+        <f t="shared" ref="G110:H110" si="5">SUM(G100:G109)</f>
+        <v>0</v>
+      </c>
+      <c r="H110" s="18">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J107" s="19"/>
-      <c r="K107" s="46"/>
-    </row>
-    <row r="108" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="59" t="s">
+      <c r="I110" s="18">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J110" s="19"/>
+      <c r="K110" s="46"/>
+    </row>
+    <row r="111" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B108" s="55"/>
-      <c r="C108" s="55"/>
-      <c r="D108" s="55"/>
-      <c r="E108" s="55"/>
-      <c r="F108" s="55"/>
-      <c r="G108" s="55"/>
-      <c r="H108" s="55"/>
-      <c r="I108" s="55"/>
-      <c r="J108" s="55"/>
-      <c r="K108" s="56"/>
-    </row>
-    <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A109" s="25" t="s">
+      <c r="B111" s="62"/>
+      <c r="C111" s="62"/>
+      <c r="D111" s="62"/>
+      <c r="E111" s="62"/>
+      <c r="F111" s="62"/>
+      <c r="G111" s="62"/>
+      <c r="H111" s="62"/>
+      <c r="I111" s="62"/>
+      <c r="J111" s="62"/>
+      <c r="K111" s="63"/>
+    </row>
+    <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A112" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B109" s="60" t="s">
+      <c r="B112" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C109" s="55"/>
-      <c r="D109" s="55"/>
-      <c r="E109" s="55"/>
-      <c r="F109" s="55"/>
-      <c r="G109" s="55"/>
-      <c r="H109" s="55"/>
-      <c r="I109" s="55"/>
-      <c r="J109" s="55"/>
-      <c r="K109" s="56"/>
-    </row>
-    <row r="110" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="26" t="s">
+      <c r="C112" s="62"/>
+      <c r="D112" s="62"/>
+      <c r="E112" s="62"/>
+      <c r="F112" s="62"/>
+      <c r="G112" s="62"/>
+      <c r="H112" s="62"/>
+      <c r="I112" s="62"/>
+      <c r="J112" s="62"/>
+      <c r="K112" s="63"/>
+    </row>
+    <row r="113" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B110" s="60" t="s">
+      <c r="B113" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C110" s="55"/>
-      <c r="D110" s="55"/>
-      <c r="E110" s="55"/>
-      <c r="F110" s="55"/>
-      <c r="G110" s="55"/>
-      <c r="H110" s="55"/>
-      <c r="I110" s="55"/>
-      <c r="J110" s="55"/>
-      <c r="K110" s="56"/>
-    </row>
-    <row r="111" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A111" s="37"/>
-      <c r="B111" s="38"/>
-      <c r="C111" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D111" s="38"/>
-      <c r="E111" s="40"/>
-      <c r="F111" s="40"/>
-      <c r="G111" s="41"/>
-      <c r="H111" s="41"/>
-      <c r="I111" s="41">
-        <f t="shared" ref="I111:I121" si="7">H111-G111</f>
-        <v>0</v>
-      </c>
-      <c r="J111" s="45"/>
-      <c r="K111" s="43"/>
-    </row>
-    <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A112" s="37"/>
-      <c r="B112" s="38"/>
-      <c r="C112" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D112" s="38"/>
-      <c r="E112" s="40"/>
-      <c r="F112" s="40"/>
-      <c r="G112" s="41"/>
-      <c r="H112" s="41"/>
-      <c r="I112" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J112" s="45"/>
-      <c r="K112" s="43"/>
-    </row>
-    <row r="113" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A113" s="37"/>
-      <c r="B113" s="38"/>
-      <c r="C113" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D113" s="38"/>
-      <c r="E113" s="40"/>
-      <c r="F113" s="40"/>
-      <c r="G113" s="41"/>
-      <c r="H113" s="41"/>
-      <c r="I113" s="41">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J113" s="45"/>
-      <c r="K113" s="43"/>
+      <c r="C113" s="62"/>
+      <c r="D113" s="62"/>
+      <c r="E113" s="62"/>
+      <c r="F113" s="62"/>
+      <c r="G113" s="62"/>
+      <c r="H113" s="62"/>
+      <c r="I113" s="62"/>
+      <c r="J113" s="62"/>
+      <c r="K113" s="63"/>
     </row>
     <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A114" s="37"/>
@@ -4630,7 +4684,7 @@
       <c r="G114" s="41"/>
       <c r="H114" s="41"/>
       <c r="I114" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="I114:I124" si="6">H114-G114</f>
         <v>0</v>
       </c>
       <c r="J114" s="45"/>
@@ -4648,7 +4702,7 @@
       <c r="G115" s="41"/>
       <c r="H115" s="41"/>
       <c r="I115" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J115" s="45"/>
@@ -4666,7 +4720,7 @@
       <c r="G116" s="41"/>
       <c r="H116" s="41"/>
       <c r="I116" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J116" s="45"/>
@@ -4684,7 +4738,7 @@
       <c r="G117" s="41"/>
       <c r="H117" s="41"/>
       <c r="I117" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J117" s="45"/>
@@ -4702,7 +4756,7 @@
       <c r="G118" s="41"/>
       <c r="H118" s="41"/>
       <c r="I118" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J118" s="45"/>
@@ -4720,7 +4774,7 @@
       <c r="G119" s="41"/>
       <c r="H119" s="41"/>
       <c r="I119" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J119" s="45"/>
@@ -4738,140 +4792,138 @@
       <c r="G120" s="41"/>
       <c r="H120" s="41"/>
       <c r="I120" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J120" s="45"/>
       <c r="K120" s="43"/>
     </row>
     <row r="121" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A121" s="13"/>
-      <c r="B121" s="15"/>
-      <c r="C121" s="15"/>
-      <c r="D121" s="15"/>
-      <c r="E121" s="15" t="s">
+      <c r="A121" s="37"/>
+      <c r="B121" s="38"/>
+      <c r="C121" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D121" s="38"/>
+      <c r="E121" s="40"/>
+      <c r="F121" s="40"/>
+      <c r="G121" s="41"/>
+      <c r="H121" s="41"/>
+      <c r="I121" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J121" s="45"/>
+      <c r="K121" s="43"/>
+    </row>
+    <row r="122" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A122" s="37"/>
+      <c r="B122" s="38"/>
+      <c r="C122" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D122" s="38"/>
+      <c r="E122" s="40"/>
+      <c r="F122" s="40"/>
+      <c r="G122" s="41"/>
+      <c r="H122" s="41"/>
+      <c r="I122" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J122" s="45"/>
+      <c r="K122" s="43"/>
+    </row>
+    <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A123" s="37"/>
+      <c r="B123" s="38"/>
+      <c r="C123" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D123" s="38"/>
+      <c r="E123" s="40"/>
+      <c r="F123" s="40"/>
+      <c r="G123" s="41"/>
+      <c r="H123" s="41"/>
+      <c r="I123" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J123" s="45"/>
+      <c r="K123" s="43"/>
+    </row>
+    <row r="124" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A124" s="13"/>
+      <c r="B124" s="15"/>
+      <c r="C124" s="15"/>
+      <c r="D124" s="15"/>
+      <c r="E124" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F121" s="15"/>
-      <c r="G121" s="18">
-        <f t="shared" ref="G121:H121" si="8">SUM(G111:G120)</f>
-        <v>0</v>
-      </c>
-      <c r="H121" s="18">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I121" s="18">
+      <c r="F124" s="15"/>
+      <c r="G124" s="18">
+        <f t="shared" ref="G124:H124" si="7">SUM(G114:G123)</f>
+        <v>0</v>
+      </c>
+      <c r="H124" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J121" s="19"/>
-      <c r="K121" s="46"/>
-    </row>
-    <row r="122" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="61" t="s">
+      <c r="I124" s="18">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J124" s="19"/>
+      <c r="K124" s="46"/>
+    </row>
+    <row r="125" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B122" s="55"/>
-      <c r="C122" s="55"/>
-      <c r="D122" s="55"/>
-      <c r="E122" s="55"/>
-      <c r="F122" s="55"/>
-      <c r="G122" s="55"/>
-      <c r="H122" s="55"/>
-      <c r="I122" s="55"/>
-      <c r="J122" s="55"/>
-      <c r="K122" s="56"/>
-    </row>
-    <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A123" s="27" t="s">
+      <c r="B125" s="62"/>
+      <c r="C125" s="62"/>
+      <c r="D125" s="62"/>
+      <c r="E125" s="62"/>
+      <c r="F125" s="62"/>
+      <c r="G125" s="62"/>
+      <c r="H125" s="62"/>
+      <c r="I125" s="62"/>
+      <c r="J125" s="62"/>
+      <c r="K125" s="63"/>
+    </row>
+    <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A126" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B123" s="54" t="s">
+      <c r="B126" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C123" s="55"/>
-      <c r="D123" s="55"/>
-      <c r="E123" s="55"/>
-      <c r="F123" s="55"/>
-      <c r="G123" s="55"/>
-      <c r="H123" s="55"/>
-      <c r="I123" s="55"/>
-      <c r="J123" s="55"/>
-      <c r="K123" s="56"/>
-    </row>
-    <row r="124" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="28" t="s">
+      <c r="C126" s="62"/>
+      <c r="D126" s="62"/>
+      <c r="E126" s="62"/>
+      <c r="F126" s="62"/>
+      <c r="G126" s="62"/>
+      <c r="H126" s="62"/>
+      <c r="I126" s="62"/>
+      <c r="J126" s="62"/>
+      <c r="K126" s="63"/>
+    </row>
+    <row r="127" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B124" s="54" t="s">
+      <c r="B127" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C124" s="55"/>
-      <c r="D124" s="55"/>
-      <c r="E124" s="55"/>
-      <c r="F124" s="55"/>
-      <c r="G124" s="55"/>
-      <c r="H124" s="55"/>
-      <c r="I124" s="55"/>
-      <c r="J124" s="55"/>
-      <c r="K124" s="56"/>
-    </row>
-    <row r="125" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A125" s="37"/>
-      <c r="B125" s="38"/>
-      <c r="C125" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D125" s="38"/>
-      <c r="E125" s="40"/>
-      <c r="F125" s="40"/>
-      <c r="G125" s="41"/>
-      <c r="H125" s="41"/>
-      <c r="I125" s="41">
-        <f t="shared" ref="I125:I135" si="9">H125-G125</f>
-        <v>0</v>
-      </c>
-      <c r="J125" s="45"/>
-      <c r="K125" s="43"/>
-    </row>
-    <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A126" s="37"/>
-      <c r="B126" s="38"/>
-      <c r="C126" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D126" s="38"/>
-      <c r="E126" s="40"/>
-      <c r="F126" s="40"/>
-      <c r="G126" s="41"/>
-      <c r="H126" s="41"/>
-      <c r="I126" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J126" s="45"/>
-      <c r="K126" s="43"/>
-    </row>
-    <row r="127" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A127" s="37"/>
-      <c r="B127" s="38"/>
-      <c r="C127" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D127" s="38"/>
-      <c r="E127" s="40"/>
-      <c r="F127" s="40"/>
-      <c r="G127" s="41"/>
-      <c r="H127" s="41"/>
-      <c r="I127" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J127" s="45"/>
-      <c r="K127" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="C127" s="62"/>
+      <c r="D127" s="62"/>
+      <c r="E127" s="62"/>
+      <c r="F127" s="62"/>
+      <c r="G127" s="62"/>
+      <c r="H127" s="62"/>
+      <c r="I127" s="62"/>
+      <c r="J127" s="62"/>
+      <c r="K127" s="63"/>
     </row>
     <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A128" s="37"/>
@@ -4885,7 +4937,7 @@
       <c r="G128" s="41"/>
       <c r="H128" s="41"/>
       <c r="I128" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I128:I138" si="8">H128-G128</f>
         <v>0</v>
       </c>
       <c r="J128" s="45"/>
@@ -4903,7 +4955,7 @@
       <c r="G129" s="41"/>
       <c r="H129" s="41"/>
       <c r="I129" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J129" s="45"/>
@@ -4921,11 +4973,13 @@
       <c r="G130" s="41"/>
       <c r="H130" s="41"/>
       <c r="I130" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J130" s="45"/>
-      <c r="K130" s="43"/>
+      <c r="K130" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A131" s="37"/>
@@ -4939,7 +4993,7 @@
       <c r="G131" s="41"/>
       <c r="H131" s="41"/>
       <c r="I131" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J131" s="45"/>
@@ -4957,7 +5011,7 @@
       <c r="G132" s="41"/>
       <c r="H132" s="41"/>
       <c r="I132" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J132" s="45"/>
@@ -4975,7 +5029,7 @@
       <c r="G133" s="41"/>
       <c r="H133" s="41"/>
       <c r="I133" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J133" s="45"/>
@@ -4993,138 +5047,138 @@
       <c r="G134" s="41"/>
       <c r="H134" s="41"/>
       <c r="I134" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J134" s="45"/>
       <c r="K134" s="43"/>
     </row>
     <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A135" s="13"/>
-      <c r="B135" s="15"/>
-      <c r="C135" s="15"/>
-      <c r="D135" s="15"/>
-      <c r="E135" s="15" t="s">
+      <c r="A135" s="37"/>
+      <c r="B135" s="38"/>
+      <c r="C135" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D135" s="38"/>
+      <c r="E135" s="40"/>
+      <c r="F135" s="40"/>
+      <c r="G135" s="41"/>
+      <c r="H135" s="41"/>
+      <c r="I135" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J135" s="45"/>
+      <c r="K135" s="43"/>
+    </row>
+    <row r="136" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A136" s="37"/>
+      <c r="B136" s="38"/>
+      <c r="C136" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D136" s="38"/>
+      <c r="E136" s="40"/>
+      <c r="F136" s="40"/>
+      <c r="G136" s="41"/>
+      <c r="H136" s="41"/>
+      <c r="I136" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J136" s="45"/>
+      <c r="K136" s="43"/>
+    </row>
+    <row r="137" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A137" s="37"/>
+      <c r="B137" s="38"/>
+      <c r="C137" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D137" s="38"/>
+      <c r="E137" s="40"/>
+      <c r="F137" s="40"/>
+      <c r="G137" s="41"/>
+      <c r="H137" s="41"/>
+      <c r="I137" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J137" s="45"/>
+      <c r="K137" s="43"/>
+    </row>
+    <row r="138" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A138" s="13"/>
+      <c r="B138" s="15"/>
+      <c r="C138" s="15"/>
+      <c r="D138" s="15"/>
+      <c r="E138" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F135" s="15"/>
-      <c r="G135" s="18">
-        <f t="shared" ref="G135:H135" si="10">SUM(G125:G134)</f>
-        <v>0</v>
-      </c>
-      <c r="H135" s="18">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="I135" s="18">
+      <c r="F138" s="15"/>
+      <c r="G138" s="18">
+        <f t="shared" ref="G138:H138" si="9">SUM(G128:G137)</f>
+        <v>0</v>
+      </c>
+      <c r="H138" s="18">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J135" s="19"/>
-      <c r="K135" s="46"/>
-    </row>
-    <row r="136" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="57" t="s">
+      <c r="I138" s="18">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J138" s="19"/>
+      <c r="K138" s="46"/>
+    </row>
+    <row r="139" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="B136" s="55"/>
-      <c r="C136" s="55"/>
-      <c r="D136" s="55"/>
-      <c r="E136" s="55"/>
-      <c r="F136" s="55"/>
-      <c r="G136" s="55"/>
-      <c r="H136" s="55"/>
-      <c r="I136" s="55"/>
-      <c r="J136" s="55"/>
-      <c r="K136" s="56"/>
-    </row>
-    <row r="137" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A137" s="29" t="s">
+      <c r="B139" s="62"/>
+      <c r="C139" s="62"/>
+      <c r="D139" s="62"/>
+      <c r="E139" s="62"/>
+      <c r="F139" s="62"/>
+      <c r="G139" s="62"/>
+      <c r="H139" s="62"/>
+      <c r="I139" s="62"/>
+      <c r="J139" s="62"/>
+      <c r="K139" s="63"/>
+    </row>
+    <row r="140" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A140" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B137" s="75" t="s">
+      <c r="B140" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C137" s="55"/>
-      <c r="D137" s="55"/>
-      <c r="E137" s="55"/>
-      <c r="F137" s="55"/>
-      <c r="G137" s="55"/>
-      <c r="H137" s="55"/>
-      <c r="I137" s="55"/>
-      <c r="J137" s="55"/>
-      <c r="K137" s="56"/>
-    </row>
-    <row r="138" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="30" t="s">
+      <c r="C140" s="62"/>
+      <c r="D140" s="62"/>
+      <c r="E140" s="62"/>
+      <c r="F140" s="62"/>
+      <c r="G140" s="62"/>
+      <c r="H140" s="62"/>
+      <c r="I140" s="62"/>
+      <c r="J140" s="62"/>
+      <c r="K140" s="63"/>
+    </row>
+    <row r="141" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B138" s="75" t="s">
+      <c r="B141" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C138" s="55"/>
-      <c r="D138" s="55"/>
-      <c r="E138" s="55"/>
-      <c r="F138" s="55"/>
-      <c r="G138" s="55"/>
-      <c r="H138" s="55"/>
-      <c r="I138" s="55"/>
-      <c r="J138" s="55"/>
-      <c r="K138" s="56"/>
-    </row>
-    <row r="139" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A139" s="37"/>
-      <c r="B139" s="38"/>
-      <c r="C139" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D139" s="38"/>
-      <c r="E139" s="40"/>
-      <c r="F139" s="40"/>
-      <c r="G139" s="41"/>
-      <c r="H139" s="41"/>
-      <c r="I139" s="41">
-        <f t="shared" ref="I139:I149" si="11">H139-G139</f>
-        <v>0</v>
-      </c>
-      <c r="J139" s="45"/>
-      <c r="K139" s="43"/>
-    </row>
-    <row r="140" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A140" s="37"/>
-      <c r="B140" s="38"/>
-      <c r="C140" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D140" s="38"/>
-      <c r="E140" s="40"/>
-      <c r="F140" s="40"/>
-      <c r="G140" s="41"/>
-      <c r="H140" s="41"/>
-      <c r="I140" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J140" s="45"/>
-      <c r="K140" s="43"/>
-    </row>
-    <row r="141" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A141" s="37"/>
-      <c r="B141" s="38"/>
-      <c r="C141" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D141" s="38"/>
-      <c r="E141" s="40"/>
-      <c r="F141" s="40"/>
-      <c r="G141" s="41"/>
-      <c r="H141" s="41"/>
-      <c r="I141" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J141" s="45"/>
-      <c r="K141" s="43"/>
+      <c r="C141" s="62"/>
+      <c r="D141" s="62"/>
+      <c r="E141" s="62"/>
+      <c r="F141" s="62"/>
+      <c r="G141" s="62"/>
+      <c r="H141" s="62"/>
+      <c r="I141" s="62"/>
+      <c r="J141" s="62"/>
+      <c r="K141" s="63"/>
     </row>
     <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A142" s="37"/>
@@ -5138,7 +5192,7 @@
       <c r="G142" s="41"/>
       <c r="H142" s="41"/>
       <c r="I142" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="I142:I152" si="10">H142-G142</f>
         <v>0</v>
       </c>
       <c r="J142" s="45"/>
@@ -5156,7 +5210,7 @@
       <c r="G143" s="41"/>
       <c r="H143" s="41"/>
       <c r="I143" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J143" s="45"/>
@@ -5174,7 +5228,7 @@
       <c r="G144" s="41"/>
       <c r="H144" s="41"/>
       <c r="I144" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J144" s="45"/>
@@ -5192,7 +5246,7 @@
       <c r="G145" s="41"/>
       <c r="H145" s="41"/>
       <c r="I145" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J145" s="45"/>
@@ -5210,7 +5264,7 @@
       <c r="G146" s="41"/>
       <c r="H146" s="41"/>
       <c r="I146" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J146" s="45"/>
@@ -5228,7 +5282,7 @@
       <c r="G147" s="41"/>
       <c r="H147" s="41"/>
       <c r="I147" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J147" s="45"/>
@@ -5246,138 +5300,138 @@
       <c r="G148" s="41"/>
       <c r="H148" s="41"/>
       <c r="I148" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J148" s="45"/>
       <c r="K148" s="43"/>
     </row>
     <row r="149" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A149" s="13"/>
-      <c r="B149" s="15"/>
-      <c r="C149" s="15"/>
-      <c r="D149" s="15"/>
-      <c r="E149" s="15" t="s">
+      <c r="A149" s="37"/>
+      <c r="B149" s="38"/>
+      <c r="C149" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D149" s="38"/>
+      <c r="E149" s="40"/>
+      <c r="F149" s="40"/>
+      <c r="G149" s="41"/>
+      <c r="H149" s="41"/>
+      <c r="I149" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J149" s="45"/>
+      <c r="K149" s="43"/>
+    </row>
+    <row r="150" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A150" s="37"/>
+      <c r="B150" s="38"/>
+      <c r="C150" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D150" s="38"/>
+      <c r="E150" s="40"/>
+      <c r="F150" s="40"/>
+      <c r="G150" s="41"/>
+      <c r="H150" s="41"/>
+      <c r="I150" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J150" s="45"/>
+      <c r="K150" s="43"/>
+    </row>
+    <row r="151" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A151" s="37"/>
+      <c r="B151" s="38"/>
+      <c r="C151" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D151" s="38"/>
+      <c r="E151" s="40"/>
+      <c r="F151" s="40"/>
+      <c r="G151" s="41"/>
+      <c r="H151" s="41"/>
+      <c r="I151" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J151" s="45"/>
+      <c r="K151" s="43"/>
+    </row>
+    <row r="152" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A152" s="13"/>
+      <c r="B152" s="15"/>
+      <c r="C152" s="15"/>
+      <c r="D152" s="15"/>
+      <c r="E152" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F149" s="15"/>
-      <c r="G149" s="18">
-        <f t="shared" ref="G149:H149" si="12">SUM(G139:G148)</f>
-        <v>0</v>
-      </c>
-      <c r="H149" s="18">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="I149" s="18">
+      <c r="F152" s="15"/>
+      <c r="G152" s="18">
+        <f t="shared" ref="G152:H152" si="11">SUM(G142:G151)</f>
+        <v>0</v>
+      </c>
+      <c r="H152" s="18">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J149" s="19"/>
-      <c r="K149" s="46"/>
-    </row>
-    <row r="150" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="62" t="s">
+      <c r="I152" s="18">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J152" s="19"/>
+      <c r="K152" s="46"/>
+    </row>
+    <row r="153" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B150" s="63"/>
-      <c r="C150" s="63"/>
-      <c r="D150" s="63"/>
-      <c r="E150" s="63"/>
-      <c r="F150" s="63"/>
-      <c r="G150" s="63"/>
-      <c r="H150" s="63"/>
-      <c r="I150" s="63"/>
-      <c r="J150" s="63"/>
-      <c r="K150" s="64"/>
-    </row>
-    <row r="151" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A151" s="32" t="s">
+      <c r="B153" s="55"/>
+      <c r="C153" s="55"/>
+      <c r="D153" s="55"/>
+      <c r="E153" s="55"/>
+      <c r="F153" s="55"/>
+      <c r="G153" s="55"/>
+      <c r="H153" s="55"/>
+      <c r="I153" s="55"/>
+      <c r="J153" s="55"/>
+      <c r="K153" s="56"/>
+    </row>
+    <row r="154" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A154" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B151" s="65" t="s">
+      <c r="B154" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C151" s="63"/>
-      <c r="D151" s="63"/>
-      <c r="E151" s="63"/>
-      <c r="F151" s="63"/>
-      <c r="G151" s="63"/>
-      <c r="H151" s="63"/>
-      <c r="I151" s="63"/>
-      <c r="J151" s="63"/>
-      <c r="K151" s="64"/>
-    </row>
-    <row r="152" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="33" t="s">
+      <c r="C154" s="55"/>
+      <c r="D154" s="55"/>
+      <c r="E154" s="55"/>
+      <c r="F154" s="55"/>
+      <c r="G154" s="55"/>
+      <c r="H154" s="55"/>
+      <c r="I154" s="55"/>
+      <c r="J154" s="55"/>
+      <c r="K154" s="56"/>
+    </row>
+    <row r="155" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B152" s="65" t="s">
+      <c r="B155" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C152" s="63"/>
-      <c r="D152" s="63"/>
-      <c r="E152" s="63"/>
-      <c r="F152" s="63"/>
-      <c r="G152" s="63"/>
-      <c r="H152" s="63"/>
-      <c r="I152" s="63"/>
-      <c r="J152" s="63"/>
-      <c r="K152" s="64"/>
-    </row>
-    <row r="153" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A153" s="37"/>
-      <c r="B153" s="38"/>
-      <c r="C153" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D153" s="38"/>
-      <c r="E153" s="40"/>
-      <c r="F153" s="40"/>
-      <c r="G153" s="41"/>
-      <c r="H153" s="41"/>
-      <c r="I153" s="41">
-        <f t="shared" ref="I153:I163" si="13">H153-G153</f>
-        <v>0</v>
-      </c>
-      <c r="J153" s="45"/>
-      <c r="K153" s="43"/>
-    </row>
-    <row r="154" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A154" s="37"/>
-      <c r="B154" s="38"/>
-      <c r="C154" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D154" s="38"/>
-      <c r="E154" s="40"/>
-      <c r="F154" s="40"/>
-      <c r="G154" s="41"/>
-      <c r="H154" s="41"/>
-      <c r="I154" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J154" s="45"/>
-      <c r="K154" s="43"/>
-    </row>
-    <row r="155" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A155" s="37"/>
-      <c r="B155" s="38"/>
-      <c r="C155" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D155" s="38"/>
-      <c r="E155" s="40"/>
-      <c r="F155" s="40"/>
-      <c r="G155" s="41"/>
-      <c r="H155" s="41"/>
-      <c r="I155" s="41">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J155" s="45"/>
-      <c r="K155" s="43"/>
+      <c r="C155" s="55"/>
+      <c r="D155" s="55"/>
+      <c r="E155" s="55"/>
+      <c r="F155" s="55"/>
+      <c r="G155" s="55"/>
+      <c r="H155" s="55"/>
+      <c r="I155" s="55"/>
+      <c r="J155" s="55"/>
+      <c r="K155" s="56"/>
     </row>
     <row r="156" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A156" s="37"/>
@@ -5391,7 +5445,7 @@
       <c r="G156" s="41"/>
       <c r="H156" s="41"/>
       <c r="I156" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="I156:I166" si="12">H156-G156</f>
         <v>0</v>
       </c>
       <c r="J156" s="45"/>
@@ -5409,7 +5463,7 @@
       <c r="G157" s="41"/>
       <c r="H157" s="41"/>
       <c r="I157" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J157" s="45"/>
@@ -5427,7 +5481,7 @@
       <c r="G158" s="41"/>
       <c r="H158" s="41"/>
       <c r="I158" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J158" s="45"/>
@@ -5445,7 +5499,7 @@
       <c r="G159" s="41"/>
       <c r="H159" s="41"/>
       <c r="I159" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J159" s="45"/>
@@ -5463,7 +5517,7 @@
       <c r="G160" s="41"/>
       <c r="H160" s="41"/>
       <c r="I160" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J160" s="45"/>
@@ -5481,7 +5535,7 @@
       <c r="G161" s="41"/>
       <c r="H161" s="41"/>
       <c r="I161" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J161" s="45"/>
@@ -5499,42 +5553,96 @@
       <c r="G162" s="41"/>
       <c r="H162" s="41"/>
       <c r="I162" s="41">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J162" s="45"/>
       <c r="K162" s="43"/>
     </row>
     <row r="163" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A163" s="48"/>
-      <c r="B163" s="49"/>
-      <c r="C163" s="49"/>
-      <c r="D163" s="49"/>
-      <c r="E163" s="49" t="s">
+      <c r="A163" s="37"/>
+      <c r="B163" s="38"/>
+      <c r="C163" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D163" s="38"/>
+      <c r="E163" s="40"/>
+      <c r="F163" s="40"/>
+      <c r="G163" s="41"/>
+      <c r="H163" s="41"/>
+      <c r="I163" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J163" s="45"/>
+      <c r="K163" s="43"/>
+    </row>
+    <row r="164" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A164" s="37"/>
+      <c r="B164" s="38"/>
+      <c r="C164" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D164" s="38"/>
+      <c r="E164" s="40"/>
+      <c r="F164" s="40"/>
+      <c r="G164" s="41"/>
+      <c r="H164" s="41"/>
+      <c r="I164" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J164" s="45"/>
+      <c r="K164" s="43"/>
+    </row>
+    <row r="165" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A165" s="37"/>
+      <c r="B165" s="38"/>
+      <c r="C165" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D165" s="38"/>
+      <c r="E165" s="40"/>
+      <c r="F165" s="40"/>
+      <c r="G165" s="41"/>
+      <c r="H165" s="41"/>
+      <c r="I165" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J165" s="45"/>
+      <c r="K165" s="43"/>
+    </row>
+    <row r="166" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A166" s="48"/>
+      <c r="B166" s="49"/>
+      <c r="C166" s="49"/>
+      <c r="D166" s="49"/>
+      <c r="E166" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F163" s="49"/>
-      <c r="G163" s="50">
-        <f t="shared" ref="G163:H163" si="14">SUM(G153:G162)</f>
-        <v>0</v>
-      </c>
-      <c r="H163" s="50">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="I163" s="50">
+      <c r="F166" s="49"/>
+      <c r="G166" s="50">
+        <f t="shared" ref="G166:H166" si="13">SUM(G156:G165)</f>
+        <v>0</v>
+      </c>
+      <c r="H166" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J163" s="51"/>
-      <c r="K163" s="52"/>
+      <c r="I166" s="50">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J166" s="51"/>
+      <c r="K166" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{21B2745E-3BE8-45F1-A565-B45E72302408}">
+      <autoFilter ref="A1:K15" xr:uid="{4455D6ED-FAC2-488E-BD29-41FCE24FB687}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5545,32 +5653,32 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A150:K150"/>
-    <mergeCell ref="B151:K151"/>
-    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B126:K126"/>
+    <mergeCell ref="B127:K127"/>
+    <mergeCell ref="A139:K139"/>
+    <mergeCell ref="B99:K99"/>
+    <mergeCell ref="A111:K111"/>
+    <mergeCell ref="B112:K112"/>
+    <mergeCell ref="B113:K113"/>
+    <mergeCell ref="A125:K125"/>
+    <mergeCell ref="A153:K153"/>
+    <mergeCell ref="B154:K154"/>
+    <mergeCell ref="B155:K155"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="A47:K47"/>
     <mergeCell ref="B48:K48"/>
     <mergeCell ref="B49:K49"/>
-    <mergeCell ref="A80:K80"/>
-    <mergeCell ref="B81:K81"/>
-    <mergeCell ref="B82:K82"/>
-    <mergeCell ref="A94:K94"/>
-    <mergeCell ref="B137:K137"/>
-    <mergeCell ref="B138:K138"/>
-    <mergeCell ref="B95:K95"/>
-    <mergeCell ref="B123:K123"/>
-    <mergeCell ref="B124:K124"/>
-    <mergeCell ref="A136:K136"/>
-    <mergeCell ref="B96:K96"/>
-    <mergeCell ref="A108:K108"/>
-    <mergeCell ref="B109:K109"/>
-    <mergeCell ref="B110:K110"/>
-    <mergeCell ref="A122:K122"/>
+    <mergeCell ref="A83:K83"/>
+    <mergeCell ref="B84:K84"/>
+    <mergeCell ref="B85:K85"/>
+    <mergeCell ref="A97:K97"/>
+    <mergeCell ref="B140:K140"/>
+    <mergeCell ref="B141:K141"/>
+    <mergeCell ref="B98:K98"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B78 B83:B92 B97:B106 B111:B120 B125:B134 B139:B148">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B95 B100:B109 B114:B123 B128:B137 B142:B151">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5587,7 +5695,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B79 B81:B93 B95:B107 B109:B121 B123:B135 B137:B149 B151:B163">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B96 B98:B110 B112:B124 B126:B138 B140:B152 B154:B166">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5595,34 +5703,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B153:B162">
+  <conditionalFormatting sqref="B156:B165">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B153))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B156))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B153))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B156))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B153))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B156))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B153))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B156))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B153))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B156))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G79 G83:G93 G97:G107 G111:G121 G125:G135 G139:G149 G153:G163">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G96 G100:G110 G114:G124 G128:G138 G142:G152 G156:G166">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H163">
+  <conditionalFormatting sqref="H1:H166">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I83:I93 I97:I107 I111:I121 I125:I135 I139:I149 I153:I163 I5:I46 I50:I79">
+  <conditionalFormatting sqref="I5:I46 I86:I96 I100:I110 I114:I124 I128:I138 I142:I152 I156:I166 I50:I82">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -5631,7 +5739,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F153:F162 F139:F148 F50:F78 F83:F92 F97:F106 F111:F120 F125:F134 F5:F45" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F156:F165 F142:F151 F50:F81 F86:F95 F100:F109 F114:F123 F128:F137 F5:F45" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5647,13 +5755,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E50:E78 E83:E92 E97:E106 E111:E120 E125:E134 E139:E148 E153:E162</xm:sqref>
+          <xm:sqref>E5:E45 E50:E81 E86:E95 E100:E109 E114:E123 E128:E137 E142:E151 E156:E165</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B50:B78 B83:B92 B97:B106 B111:B120 B125:B134 B139:B148 B153:B162</xm:sqref>
+          <xm:sqref>B5:B45 B50:B81 B86:B95 B100:B109 B114:B123 B128:B137 B142:B151 B156:B165</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5733,7 +5841,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" cm="1">
-        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$50:$H$77,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
+        <f t="array" ref="D4">IFERROR(SUM(_xlfn._xlws.FILTER('Worklog_Tasks&amp;Times'!$H$50:$H$80,'Worklog_Tasks&amp;Times'!$F$5:$F$17=$B4)),0)</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" cm="1">
@@ -7294,26 +7402,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -7548,10 +7636,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7568,20 +7687,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Week 2 finish and week 3 start.
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{093DA171-1404-43AB-AD4A-10387CF7CE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A542D92-A685-4C29-BCD6-35756D4E2CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$151</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$153</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="169">
   <si>
     <t>Date</t>
   </si>
@@ -386,9 +386,6 @@
     <t>For some reason, GitHub refuses to show PDFs on my computer, but on other devices it does work. This is meant to try and fix that. POST-TASK EDIT: Seems to be  a problem with GitHub itself and not my device, and there does nto seem to be a solution.</t>
   </si>
   <si>
-    <t>0,5 so far</t>
-  </si>
-  <si>
     <t>Organize block B and block A files</t>
   </si>
   <si>
@@ -551,9 +548,6 @@
     <t>I am not certain what has to be done with the "SMARTER" goals</t>
   </si>
   <si>
-    <t>Evidence in WorkLog</t>
-  </si>
-  <si>
     <t>Evidence Week 2 Learning Log</t>
   </si>
   <si>
@@ -582,6 +576,39 @@
   </si>
   <si>
     <t>Re-write Week 1 and 2 reflection and feedback</t>
+  </si>
+  <si>
+    <t>Fill in Learning Log Week 3</t>
+  </si>
+  <si>
+    <t>Read chapter 3</t>
+  </si>
+  <si>
+    <t>Complete “ML-quiz-W3_1” in brightspace</t>
+  </si>
+  <si>
+    <t>Read chapter 4</t>
+  </si>
+  <si>
+    <t>Complete “ML-quiz-W3_2” in brightspace</t>
+  </si>
+  <si>
+    <t>Read summary of chapter 4</t>
+  </si>
+  <si>
+    <t>Read summary of chapter 3</t>
+  </si>
+  <si>
+    <t>Had to help my sister with her school work intermittently while I was doing this quiz.</t>
+  </si>
+  <si>
+    <t>Evidence week 2 in WorkLog</t>
+  </si>
+  <si>
+    <t>I'm still not too sure about the SMATER goals.</t>
+  </si>
+  <si>
+    <t>Look ahead at the Tuesday DataLab</t>
   </si>
 </sst>
 </file>
@@ -1067,6 +1094,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1083,8 +1130,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1102,24 +1147,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1592,7 +1619,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K166"/>
+  <dimension ref="A1:K168"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1644,53 +1671,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -2113,7 +2140,7 @@
       </c>
       <c r="J17" s="45"/>
       <c r="K17" s="44" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -2257,7 +2284,7 @@
         <v>17</v>
       </c>
       <c r="D22" s="38" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E22" s="40" t="s">
         <v>64</v>
@@ -2321,13 +2348,13 @@
         <v>17</v>
       </c>
       <c r="D24" s="38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E24" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F24" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G24" s="41">
         <v>1</v>
@@ -2353,13 +2380,13 @@
         <v>17</v>
       </c>
       <c r="D25" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E25" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F25" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G25" s="41">
         <v>1</v>
@@ -2385,13 +2412,13 @@
         <v>17</v>
       </c>
       <c r="D26" s="38" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E26" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F26" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G26" s="41">
         <v>2</v>
@@ -2417,13 +2444,13 @@
         <v>17</v>
       </c>
       <c r="D27" s="38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E27" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F27" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G27" s="41">
         <v>2</v>
@@ -2449,13 +2476,13 @@
         <v>17</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E28" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F28" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G28" s="41">
         <v>1</v>
@@ -2481,13 +2508,13 @@
         <v>17</v>
       </c>
       <c r="D29" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E29" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F29" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G29" s="41">
         <v>1</v>
@@ -2500,7 +2527,7 @@
         <v>-0.5</v>
       </c>
       <c r="J29" s="53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K29" s="44"/>
     </row>
@@ -2515,7 +2542,7 @@
         <v>17</v>
       </c>
       <c r="D30" s="38" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E30" s="40" t="s">
         <v>64</v>
@@ -2547,7 +2574,7 @@
         <v>17</v>
       </c>
       <c r="D31" s="38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E31" s="40" t="s">
         <v>62</v>
@@ -2579,7 +2606,7 @@
         <v>17</v>
       </c>
       <c r="D32" s="38" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E32" s="40" t="s">
         <v>47</v>
@@ -2611,13 +2638,13 @@
         <v>17</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E33" s="40" t="s">
         <v>47</v>
       </c>
       <c r="F33" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G33" s="41">
         <v>1</v>
@@ -2643,13 +2670,13 @@
         <v>17</v>
       </c>
       <c r="D34" s="38" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E34" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F34" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G34" s="41">
         <v>0.5</v>
@@ -2675,13 +2702,13 @@
         <v>17</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E35" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F35" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G35" s="41">
         <v>1</v>
@@ -2707,13 +2734,13 @@
         <v>17</v>
       </c>
       <c r="D36" s="38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E36" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F36" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G36" s="41">
         <v>0.5</v>
@@ -2727,7 +2754,7 @@
       </c>
       <c r="J36" s="45"/>
       <c r="K36" s="44" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -2741,13 +2768,13 @@
         <v>17</v>
       </c>
       <c r="D37" s="38" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E37" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F37" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G37" s="41">
         <v>1</v>
@@ -2773,13 +2800,13 @@
         <v>17</v>
       </c>
       <c r="D38" s="38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E38" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F38" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G38" s="41">
         <v>1</v>
@@ -2805,13 +2832,13 @@
         <v>17</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E39" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F39" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G39" s="41">
         <v>1</v>
@@ -2825,7 +2852,7 @@
       </c>
       <c r="J39" s="45"/>
       <c r="K39" s="44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -2839,13 +2866,13 @@
         <v>17</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E40" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F40" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G40" s="41">
         <v>4</v>
@@ -2869,13 +2896,13 @@
         <v>17</v>
       </c>
       <c r="D41" s="38" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E41" s="40" t="s">
         <v>59</v>
       </c>
       <c r="F41" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G41" s="41">
         <v>4</v>
@@ -2897,13 +2924,13 @@
         <v>17</v>
       </c>
       <c r="D42" s="38" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E42" s="40" t="s">
         <v>59</v>
       </c>
       <c r="F42" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G42" s="41">
         <v>4</v>
@@ -2925,7 +2952,7 @@
         <v>17</v>
       </c>
       <c r="D43" s="38" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E43" s="40" t="s">
         <v>64</v>
@@ -2955,7 +2982,7 @@
         <v>17</v>
       </c>
       <c r="D44" s="38" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E44" s="40" t="s">
         <v>64</v>
@@ -2985,7 +3012,7 @@
         <v>17</v>
       </c>
       <c r="D45" s="38" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E45" s="40" t="s">
         <v>64</v>
@@ -3029,53 +3056,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -3120,13 +3147,13 @@
         <v>17</v>
       </c>
       <c r="D51" s="38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E51" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F51" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G51" s="41">
         <v>1</v>
@@ -3152,13 +3179,13 @@
         <v>17</v>
       </c>
       <c r="D52" s="38" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E52" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F52" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G52" s="41">
         <v>2</v>
@@ -3184,13 +3211,13 @@
         <v>17</v>
       </c>
       <c r="D53" s="38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E53" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F53" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G53" s="41">
         <v>2</v>
@@ -3216,13 +3243,13 @@
         <v>17</v>
       </c>
       <c r="D54" s="38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E54" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F54" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G54" s="41">
         <v>1.5</v>
@@ -3248,13 +3275,13 @@
         <v>17</v>
       </c>
       <c r="D55" s="38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E55" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F55" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G55" s="41">
         <v>1</v>
@@ -3280,13 +3307,13 @@
         <v>17</v>
       </c>
       <c r="D56" s="38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E56" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F56" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G56" s="41">
         <v>0.5</v>
@@ -3312,7 +3339,7 @@
         <v>17</v>
       </c>
       <c r="D57" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E57" s="40" t="s">
         <v>62</v>
@@ -3344,7 +3371,7 @@
         <v>17</v>
       </c>
       <c r="D58" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E58" s="40" t="s">
         <v>47</v>
@@ -3376,13 +3403,13 @@
         <v>17</v>
       </c>
       <c r="D59" s="38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E59" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F59" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G59" s="41">
         <v>0.5</v>
@@ -3396,7 +3423,7 @@
       </c>
       <c r="J59" s="45"/>
       <c r="K59" s="43" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -3410,13 +3437,13 @@
         <v>17</v>
       </c>
       <c r="D60" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E60" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F60" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G60" s="41">
         <v>0.5</v>
@@ -3442,13 +3469,13 @@
         <v>17</v>
       </c>
       <c r="D61" s="38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E61" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F61" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G61" s="41">
         <v>0.5</v>
@@ -3462,7 +3489,7 @@
       </c>
       <c r="J61" s="45"/>
       <c r="K61" s="43" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -3476,13 +3503,13 @@
         <v>17</v>
       </c>
       <c r="D62" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E62" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F62" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G62" s="41">
         <v>0.1</v>
@@ -3496,7 +3523,7 @@
       </c>
       <c r="J62" s="45"/>
       <c r="K62" s="43" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -3510,13 +3537,13 @@
         <v>17</v>
       </c>
       <c r="D63" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E63" s="40" t="s">
         <v>46</v>
       </c>
       <c r="F63" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G63" s="41">
         <v>0</v>
@@ -3530,7 +3557,7 @@
       </c>
       <c r="J63" s="45"/>
       <c r="K63" s="43" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -3544,13 +3571,13 @@
         <v>17</v>
       </c>
       <c r="D64" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E64" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F64" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G64" s="41">
         <v>4</v>
@@ -3576,13 +3603,13 @@
         <v>17</v>
       </c>
       <c r="D65" s="38" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E65" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F65" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G65" s="41">
         <v>3</v>
@@ -3608,13 +3635,13 @@
         <v>17</v>
       </c>
       <c r="D66" s="38" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E66" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F66" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G66" s="41">
         <v>2</v>
@@ -3640,13 +3667,13 @@
         <v>17</v>
       </c>
       <c r="D67" s="38" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E67" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F67" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G67" s="41">
         <v>1</v>
@@ -3670,13 +3697,13 @@
         <v>17</v>
       </c>
       <c r="D68" s="38" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E68" s="40" t="s">
         <v>59</v>
       </c>
       <c r="F68" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G68" s="41">
         <v>4</v>
@@ -3702,13 +3729,13 @@
         <v>17</v>
       </c>
       <c r="D69" s="38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E69" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F69" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G69" s="41">
         <v>0.25</v>
@@ -3725,35 +3752,35 @@
     </row>
     <row r="70" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A70" s="47" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B70" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C70" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D70" s="38" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E70" s="40" t="s">
         <v>64</v>
       </c>
       <c r="F70" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G70" s="41">
         <v>1</v>
       </c>
-      <c r="H70" s="41"/>
+      <c r="H70" s="41">
+        <v>0.75</v>
+      </c>
       <c r="I70" s="41">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>-0.25</v>
       </c>
       <c r="J70" s="45"/>
-      <c r="K70" s="43" t="s">
-        <v>94</v>
-      </c>
+      <c r="K70" s="43"/>
     </row>
     <row r="71" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A71" s="47">
@@ -3766,7 +3793,7 @@
         <v>17</v>
       </c>
       <c r="D71" s="38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E71" s="40" t="s">
         <v>47</v>
@@ -3798,13 +3825,13 @@
         <v>17</v>
       </c>
       <c r="D72" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E72" s="40" t="s">
         <v>47</v>
       </c>
       <c r="F72" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G72" s="41">
         <v>0.5</v>
@@ -3830,7 +3857,7 @@
         <v>17</v>
       </c>
       <c r="D73" s="38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E73" s="40" t="s">
         <v>66</v>
@@ -3862,7 +3889,7 @@
         <v>17</v>
       </c>
       <c r="D74" s="38" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E74" s="40" t="s">
         <v>46</v>
@@ -3888,31 +3915,33 @@
         <v>45625</v>
       </c>
       <c r="B75" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C75" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D75" s="38" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E75" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F75" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G75" s="41">
         <v>4</v>
       </c>
-      <c r="H75" s="41"/>
+      <c r="H75" s="41">
+        <v>3.5</v>
+      </c>
       <c r="I75" s="41">
         <f t="shared" si="1"/>
-        <v>-4</v>
+        <v>-0.5</v>
       </c>
       <c r="J75" s="45"/>
       <c r="K75" s="43" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="76" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
@@ -3926,7 +3955,7 @@
         <v>17</v>
       </c>
       <c r="D76" s="38" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E76" s="40" t="s">
         <v>47</v>
@@ -3952,24 +3981,28 @@
         <v>45625</v>
       </c>
       <c r="B77" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C77" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D77" s="38" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="E77" s="40" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F77" s="40" t="s">
         <v>88</v>
       </c>
-      <c r="G77" s="41"/>
-      <c r="H77" s="41"/>
+      <c r="G77" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H77" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I77" s="41">
-        <f t="shared" si="1"/>
+        <f>H77-G77</f>
         <v>0</v>
       </c>
       <c r="J77" s="45"/>
@@ -3980,13 +4013,13 @@
         <v>45625</v>
       </c>
       <c r="B78" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C78" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D78" s="38" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E78" s="40" t="s">
         <v>62</v>
@@ -3994,49 +4027,55 @@
       <c r="F78" s="40" t="s">
         <v>88</v>
       </c>
-      <c r="G78" s="41"/>
-      <c r="H78" s="41"/>
+      <c r="G78" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H78" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I78" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J78" s="45"/>
-      <c r="K78" s="43"/>
+      <c r="K78" s="43" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="79" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A79" s="47">
         <v>45625</v>
       </c>
       <c r="B79" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C79" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D79" s="38" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="E79" s="40" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F79" s="40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G79" s="41">
-        <v>0.25</v>
-      </c>
-      <c r="H79" s="41"/>
+        <v>0.5</v>
+      </c>
+      <c r="H79" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I79" s="41">
         <f t="shared" si="1"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J79" s="45"/>
       <c r="K79" s="43"/>
     </row>
     <row r="80" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A80" s="47">
-        <v>45625</v>
-      </c>
+      <c r="A80" s="47"/>
       <c r="B80" s="38" t="s">
         <v>43</v>
       </c>
@@ -4044,13 +4083,13 @@
         <v>17</v>
       </c>
       <c r="D80" s="38" t="s">
-        <v>151</v>
+        <v>166</v>
       </c>
       <c r="E80" s="40" t="s">
         <v>64</v>
       </c>
       <c r="F80" s="40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G80" s="41">
         <v>0.25</v>
@@ -4064,9 +4103,7 @@
       <c r="K80" s="43"/>
     </row>
     <row r="81" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A81" s="47">
-        <v>45625</v>
-      </c>
+      <c r="A81" s="47"/>
       <c r="B81" s="38" t="s">
         <v>43</v>
       </c>
@@ -4074,7 +4111,7 @@
         <v>17</v>
       </c>
       <c r="D81" s="38" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E81" s="40" t="s">
         <v>64</v>
@@ -4104,97 +4141,125 @@
       <c r="F82" s="15"/>
       <c r="G82" s="18">
         <f>SUM(G48:G81)</f>
-        <v>32.85</v>
+        <v>33.85</v>
       </c>
       <c r="H82" s="18">
         <f>SUM(H48:H81)</f>
-        <v>27.679999999999996</v>
+        <v>33.179999999999993</v>
       </c>
       <c r="I82" s="18">
         <f t="shared" si="1"/>
-        <v>-5.1700000000000053</v>
+        <v>-0.67000000000000881</v>
       </c>
       <c r="J82" s="19"/>
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A86" s="37"/>
-      <c r="B86" s="38"/>
+      <c r="A86" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B86" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C86" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D86" s="38"/>
-      <c r="E86" s="40"/>
-      <c r="F86" s="40"/>
-      <c r="G86" s="41"/>
-      <c r="H86" s="41"/>
+      <c r="D86" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="E86" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F86" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G86" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H86" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I86" s="41">
-        <f t="shared" ref="I86:I96" si="2">H86-G86</f>
+        <f t="shared" ref="I86:I98" si="2">H86-G86</f>
         <v>0</v>
       </c>
       <c r="J86" s="45"/>
       <c r="K86" s="43"/>
     </row>
     <row r="87" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A87" s="37"/>
-      <c r="B87" s="38"/>
+      <c r="A87" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B87" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C87" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D87" s="38"/>
-      <c r="E87" s="40"/>
-      <c r="F87" s="40"/>
-      <c r="G87" s="41"/>
-      <c r="H87" s="41"/>
+      <c r="D87" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="E87" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F87" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G87" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H87" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I87" s="41">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4203,34 +4268,62 @@
       <c r="K87" s="43"/>
     </row>
     <row r="88" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A88" s="37"/>
-      <c r="B88" s="38"/>
+      <c r="A88" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B88" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C88" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D88" s="38"/>
-      <c r="E88" s="40"/>
-      <c r="F88" s="40"/>
-      <c r="G88" s="41"/>
-      <c r="H88" s="41"/>
+      <c r="D88" s="38" t="s">
+        <v>159</v>
+      </c>
+      <c r="E88" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F88" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G88" s="41">
+        <v>2</v>
+      </c>
+      <c r="H88" s="41">
+        <v>1.5</v>
+      </c>
       <c r="I88" s="41">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="J88" s="45"/>
       <c r="K88" s="43"/>
     </row>
     <row r="89" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A89" s="37"/>
-      <c r="B89" s="38"/>
+      <c r="A89" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B89" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C89" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D89" s="38"/>
-      <c r="E89" s="40"/>
-      <c r="F89" s="40"/>
-      <c r="G89" s="41"/>
-      <c r="H89" s="41"/>
+      <c r="D89" s="38" t="s">
+        <v>164</v>
+      </c>
+      <c r="E89" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F89" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G89" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H89" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I89" s="41">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4239,52 +4332,94 @@
       <c r="K89" s="43"/>
     </row>
     <row r="90" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A90" s="37"/>
-      <c r="B90" s="38"/>
+      <c r="A90" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B90" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C90" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D90" s="38"/>
-      <c r="E90" s="40"/>
-      <c r="F90" s="40"/>
-      <c r="G90" s="41"/>
-      <c r="H90" s="41"/>
+      <c r="D90" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="E90" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F90" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G90" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H90" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I90" s="41">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-0.25</v>
       </c>
       <c r="J90" s="45"/>
       <c r="K90" s="43"/>
     </row>
     <row r="91" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A91" s="37"/>
-      <c r="B91" s="38"/>
+      <c r="A91" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B91" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C91" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D91" s="38"/>
-      <c r="E91" s="40"/>
-      <c r="F91" s="40"/>
-      <c r="G91" s="41"/>
-      <c r="H91" s="41"/>
+      <c r="D91" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="E91" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F91" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G91" s="41">
+        <v>4</v>
+      </c>
+      <c r="H91" s="41">
+        <v>2.5</v>
+      </c>
       <c r="I91" s="41">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1.5</v>
       </c>
       <c r="J91" s="45"/>
       <c r="K91" s="43"/>
     </row>
     <row r="92" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A92" s="37"/>
-      <c r="B92" s="38"/>
+      <c r="A92" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B92" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C92" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D92" s="38"/>
-      <c r="E92" s="40"/>
-      <c r="F92" s="40"/>
-      <c r="G92" s="41"/>
-      <c r="H92" s="41"/>
+      <c r="D92" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="E92" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F92" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G92" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H92" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I92" s="41">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4293,34 +4428,64 @@
       <c r="K92" s="43"/>
     </row>
     <row r="93" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A93" s="37"/>
-      <c r="B93" s="38"/>
+      <c r="A93" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B93" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C93" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D93" s="38"/>
-      <c r="E93" s="40"/>
-      <c r="F93" s="40"/>
-      <c r="G93" s="41"/>
-      <c r="H93" s="41"/>
+      <c r="D93" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="E93" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F93" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G93" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H93" s="41">
+        <v>1</v>
+      </c>
       <c r="I93" s="41">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J93" s="45"/>
-      <c r="K93" s="43"/>
+      <c r="K93" s="43" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="94" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A94" s="37"/>
-      <c r="B94" s="38"/>
+      <c r="A94" s="37">
+        <v>45628</v>
+      </c>
+      <c r="B94" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C94" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D94" s="38"/>
-      <c r="E94" s="40"/>
-      <c r="F94" s="40"/>
-      <c r="G94" s="41"/>
-      <c r="H94" s="41"/>
+      <c r="D94" s="38" t="s">
+        <v>168</v>
+      </c>
+      <c r="E94" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F94" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G94" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H94" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I94" s="41">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4347,113 +4512,113 @@
       <c r="K95" s="43"/>
     </row>
     <row r="96" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A96" s="13"/>
-      <c r="B96" s="15"/>
-      <c r="C96" s="15"/>
-      <c r="D96" s="15"/>
-      <c r="E96" s="15" t="s">
+      <c r="A96" s="37"/>
+      <c r="B96" s="38"/>
+      <c r="C96" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D96" s="38"/>
+      <c r="E96" s="40"/>
+      <c r="F96" s="40"/>
+      <c r="G96" s="41"/>
+      <c r="H96" s="41"/>
+      <c r="I96" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J96" s="45"/>
+      <c r="K96" s="43"/>
+    </row>
+    <row r="97" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A97" s="37"/>
+      <c r="B97" s="38"/>
+      <c r="C97" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D97" s="38"/>
+      <c r="E97" s="40"/>
+      <c r="F97" s="40"/>
+      <c r="G97" s="41"/>
+      <c r="H97" s="41"/>
+      <c r="I97" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J97" s="45"/>
+      <c r="K97" s="43"/>
+    </row>
+    <row r="98" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A98" s="13"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="15"/>
+      <c r="D98" s="15"/>
+      <c r="E98" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F96" s="15"/>
-      <c r="G96" s="18">
-        <f t="shared" ref="G96:H96" si="3">SUM(G86:G95)</f>
-        <v>0</v>
-      </c>
-      <c r="H96" s="18">
+      <c r="F98" s="15"/>
+      <c r="G98" s="18">
+        <f t="shared" ref="G98:H98" si="3">SUM(G86:G97)</f>
+        <v>9.25</v>
+      </c>
+      <c r="H98" s="18">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="I96" s="18">
+        <v>7.5</v>
+      </c>
+      <c r="I98" s="18">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J96" s="19"/>
-      <c r="K96" s="46"/>
-    </row>
-    <row r="97" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="68" t="s">
+        <v>-1.75</v>
+      </c>
+      <c r="J98" s="19"/>
+      <c r="K98" s="46"/>
+    </row>
+    <row r="99" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B97" s="62"/>
-      <c r="C97" s="62"/>
-      <c r="D97" s="62"/>
-      <c r="E97" s="62"/>
-      <c r="F97" s="62"/>
-      <c r="G97" s="62"/>
-      <c r="H97" s="62"/>
-      <c r="I97" s="62"/>
-      <c r="J97" s="62"/>
-      <c r="K97" s="63"/>
-    </row>
-    <row r="98" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A98" s="23" t="s">
+      <c r="B99" s="55"/>
+      <c r="C99" s="55"/>
+      <c r="D99" s="55"/>
+      <c r="E99" s="55"/>
+      <c r="F99" s="55"/>
+      <c r="G99" s="55"/>
+      <c r="H99" s="55"/>
+      <c r="I99" s="55"/>
+      <c r="J99" s="55"/>
+      <c r="K99" s="56"/>
+    </row>
+    <row r="100" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A100" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B98" s="70" t="s">
+      <c r="B100" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C98" s="62"/>
-      <c r="D98" s="62"/>
-      <c r="E98" s="62"/>
-      <c r="F98" s="62"/>
-      <c r="G98" s="62"/>
-      <c r="H98" s="62"/>
-      <c r="I98" s="62"/>
-      <c r="J98" s="62"/>
-      <c r="K98" s="63"/>
-    </row>
-    <row r="99" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="24" t="s">
+      <c r="C100" s="55"/>
+      <c r="D100" s="55"/>
+      <c r="E100" s="55"/>
+      <c r="F100" s="55"/>
+      <c r="G100" s="55"/>
+      <c r="H100" s="55"/>
+      <c r="I100" s="55"/>
+      <c r="J100" s="55"/>
+      <c r="K100" s="56"/>
+    </row>
+    <row r="101" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B99" s="70" t="s">
+      <c r="B101" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C99" s="62"/>
-      <c r="D99" s="62"/>
-      <c r="E99" s="62"/>
-      <c r="F99" s="62"/>
-      <c r="G99" s="62"/>
-      <c r="H99" s="62"/>
-      <c r="I99" s="62"/>
-      <c r="J99" s="62"/>
-      <c r="K99" s="63"/>
-    </row>
-    <row r="100" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A100" s="37"/>
-      <c r="B100" s="38"/>
-      <c r="C100" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D100" s="38"/>
-      <c r="E100" s="40"/>
-      <c r="F100" s="40"/>
-      <c r="G100" s="41"/>
-      <c r="H100" s="41"/>
-      <c r="I100" s="41">
-        <f t="shared" ref="I100:I110" si="4">H100-G100</f>
-        <v>0</v>
-      </c>
-      <c r="J100" s="45"/>
-      <c r="K100" s="43"/>
-    </row>
-    <row r="101" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A101" s="37"/>
-      <c r="B101" s="38"/>
-      <c r="C101" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D101" s="38"/>
-      <c r="E101" s="40"/>
-      <c r="F101" s="40"/>
-      <c r="G101" s="41"/>
-      <c r="H101" s="41"/>
-      <c r="I101" s="41">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="J101" s="45"/>
-      <c r="K101" s="43"/>
+      <c r="C101" s="55"/>
+      <c r="D101" s="55"/>
+      <c r="E101" s="55"/>
+      <c r="F101" s="55"/>
+      <c r="G101" s="55"/>
+      <c r="H101" s="55"/>
+      <c r="I101" s="55"/>
+      <c r="J101" s="55"/>
+      <c r="K101" s="56"/>
     </row>
     <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A102" s="37"/>
@@ -4467,7 +4632,7 @@
       <c r="G102" s="41"/>
       <c r="H102" s="41"/>
       <c r="I102" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I102:I112" si="4">H102-G102</f>
         <v>0</v>
       </c>
       <c r="J102" s="45"/>
@@ -4600,113 +4765,113 @@
       <c r="K109" s="43"/>
     </row>
     <row r="110" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A110" s="13"/>
-      <c r="B110" s="15"/>
-      <c r="C110" s="15"/>
-      <c r="D110" s="15"/>
-      <c r="E110" s="15" t="s">
+      <c r="A110" s="37"/>
+      <c r="B110" s="38"/>
+      <c r="C110" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D110" s="38"/>
+      <c r="E110" s="40"/>
+      <c r="F110" s="40"/>
+      <c r="G110" s="41"/>
+      <c r="H110" s="41"/>
+      <c r="I110" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J110" s="45"/>
+      <c r="K110" s="43"/>
+    </row>
+    <row r="111" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A111" s="37"/>
+      <c r="B111" s="38"/>
+      <c r="C111" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D111" s="38"/>
+      <c r="E111" s="40"/>
+      <c r="F111" s="40"/>
+      <c r="G111" s="41"/>
+      <c r="H111" s="41"/>
+      <c r="I111" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J111" s="45"/>
+      <c r="K111" s="43"/>
+    </row>
+    <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A112" s="13"/>
+      <c r="B112" s="15"/>
+      <c r="C112" s="15"/>
+      <c r="D112" s="15"/>
+      <c r="E112" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F110" s="15"/>
-      <c r="G110" s="18">
-        <f t="shared" ref="G110:H110" si="5">SUM(G100:G109)</f>
-        <v>0</v>
-      </c>
-      <c r="H110" s="18">
+      <c r="F112" s="15"/>
+      <c r="G112" s="18">
+        <f t="shared" ref="G112:H112" si="5">SUM(G102:G111)</f>
+        <v>0</v>
+      </c>
+      <c r="H112" s="18">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I110" s="18">
+      <c r="I112" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J110" s="19"/>
-      <c r="K110" s="46"/>
-    </row>
-    <row r="111" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="73" t="s">
+      <c r="J112" s="19"/>
+      <c r="K112" s="46"/>
+    </row>
+    <row r="113" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B111" s="62"/>
-      <c r="C111" s="62"/>
-      <c r="D111" s="62"/>
-      <c r="E111" s="62"/>
-      <c r="F111" s="62"/>
-      <c r="G111" s="62"/>
-      <c r="H111" s="62"/>
-      <c r="I111" s="62"/>
-      <c r="J111" s="62"/>
-      <c r="K111" s="63"/>
-    </row>
-    <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A112" s="25" t="s">
+      <c r="B113" s="55"/>
+      <c r="C113" s="55"/>
+      <c r="D113" s="55"/>
+      <c r="E113" s="55"/>
+      <c r="F113" s="55"/>
+      <c r="G113" s="55"/>
+      <c r="H113" s="55"/>
+      <c r="I113" s="55"/>
+      <c r="J113" s="55"/>
+      <c r="K113" s="56"/>
+    </row>
+    <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A114" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B112" s="74" t="s">
+      <c r="B114" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C112" s="62"/>
-      <c r="D112" s="62"/>
-      <c r="E112" s="62"/>
-      <c r="F112" s="62"/>
-      <c r="G112" s="62"/>
-      <c r="H112" s="62"/>
-      <c r="I112" s="62"/>
-      <c r="J112" s="62"/>
-      <c r="K112" s="63"/>
-    </row>
-    <row r="113" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="26" t="s">
+      <c r="C114" s="55"/>
+      <c r="D114" s="55"/>
+      <c r="E114" s="55"/>
+      <c r="F114" s="55"/>
+      <c r="G114" s="55"/>
+      <c r="H114" s="55"/>
+      <c r="I114" s="55"/>
+      <c r="J114" s="55"/>
+      <c r="K114" s="56"/>
+    </row>
+    <row r="115" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B113" s="74" t="s">
+      <c r="B115" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C113" s="62"/>
-      <c r="D113" s="62"/>
-      <c r="E113" s="62"/>
-      <c r="F113" s="62"/>
-      <c r="G113" s="62"/>
-      <c r="H113" s="62"/>
-      <c r="I113" s="62"/>
-      <c r="J113" s="62"/>
-      <c r="K113" s="63"/>
-    </row>
-    <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A114" s="37"/>
-      <c r="B114" s="38"/>
-      <c r="C114" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D114" s="38"/>
-      <c r="E114" s="40"/>
-      <c r="F114" s="40"/>
-      <c r="G114" s="41"/>
-      <c r="H114" s="41"/>
-      <c r="I114" s="41">
-        <f t="shared" ref="I114:I124" si="6">H114-G114</f>
-        <v>0</v>
-      </c>
-      <c r="J114" s="45"/>
-      <c r="K114" s="43"/>
-    </row>
-    <row r="115" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A115" s="37"/>
-      <c r="B115" s="38"/>
-      <c r="C115" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D115" s="38"/>
-      <c r="E115" s="40"/>
-      <c r="F115" s="40"/>
-      <c r="G115" s="41"/>
-      <c r="H115" s="41"/>
-      <c r="I115" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J115" s="45"/>
-      <c r="K115" s="43"/>
+      <c r="C115" s="55"/>
+      <c r="D115" s="55"/>
+      <c r="E115" s="55"/>
+      <c r="F115" s="55"/>
+      <c r="G115" s="55"/>
+      <c r="H115" s="55"/>
+      <c r="I115" s="55"/>
+      <c r="J115" s="55"/>
+      <c r="K115" s="56"/>
     </row>
     <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A116" s="37"/>
@@ -4720,7 +4885,7 @@
       <c r="G116" s="41"/>
       <c r="H116" s="41"/>
       <c r="I116" s="41">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="I116:I126" si="6">H116-G116</f>
         <v>0</v>
       </c>
       <c r="J116" s="45"/>
@@ -4853,113 +5018,113 @@
       <c r="K123" s="43"/>
     </row>
     <row r="124" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A124" s="13"/>
-      <c r="B124" s="15"/>
-      <c r="C124" s="15"/>
-      <c r="D124" s="15"/>
-      <c r="E124" s="15" t="s">
+      <c r="A124" s="37"/>
+      <c r="B124" s="38"/>
+      <c r="C124" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D124" s="38"/>
+      <c r="E124" s="40"/>
+      <c r="F124" s="40"/>
+      <c r="G124" s="41"/>
+      <c r="H124" s="41"/>
+      <c r="I124" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J124" s="45"/>
+      <c r="K124" s="43"/>
+    </row>
+    <row r="125" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A125" s="37"/>
+      <c r="B125" s="38"/>
+      <c r="C125" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D125" s="38"/>
+      <c r="E125" s="40"/>
+      <c r="F125" s="40"/>
+      <c r="G125" s="41"/>
+      <c r="H125" s="41"/>
+      <c r="I125" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J125" s="45"/>
+      <c r="K125" s="43"/>
+    </row>
+    <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A126" s="13"/>
+      <c r="B126" s="15"/>
+      <c r="C126" s="15"/>
+      <c r="D126" s="15"/>
+      <c r="E126" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F124" s="15"/>
-      <c r="G124" s="18">
-        <f t="shared" ref="G124:H124" si="7">SUM(G114:G123)</f>
-        <v>0</v>
-      </c>
-      <c r="H124" s="18">
+      <c r="F126" s="15"/>
+      <c r="G126" s="18">
+        <f t="shared" ref="G126:H126" si="7">SUM(G116:G125)</f>
+        <v>0</v>
+      </c>
+      <c r="H126" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I124" s="18">
+      <c r="I126" s="18">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J124" s="19"/>
-      <c r="K124" s="46"/>
-    </row>
-    <row r="125" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="75" t="s">
+      <c r="J126" s="19"/>
+      <c r="K126" s="46"/>
+    </row>
+    <row r="127" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B125" s="62"/>
-      <c r="C125" s="62"/>
-      <c r="D125" s="62"/>
-      <c r="E125" s="62"/>
-      <c r="F125" s="62"/>
-      <c r="G125" s="62"/>
-      <c r="H125" s="62"/>
-      <c r="I125" s="62"/>
-      <c r="J125" s="62"/>
-      <c r="K125" s="63"/>
-    </row>
-    <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A126" s="27" t="s">
+      <c r="B127" s="55"/>
+      <c r="C127" s="55"/>
+      <c r="D127" s="55"/>
+      <c r="E127" s="55"/>
+      <c r="F127" s="55"/>
+      <c r="G127" s="55"/>
+      <c r="H127" s="55"/>
+      <c r="I127" s="55"/>
+      <c r="J127" s="55"/>
+      <c r="K127" s="56"/>
+    </row>
+    <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A128" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B126" s="71" t="s">
+      <c r="B128" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C126" s="62"/>
-      <c r="D126" s="62"/>
-      <c r="E126" s="62"/>
-      <c r="F126" s="62"/>
-      <c r="G126" s="62"/>
-      <c r="H126" s="62"/>
-      <c r="I126" s="62"/>
-      <c r="J126" s="62"/>
-      <c r="K126" s="63"/>
-    </row>
-    <row r="127" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="28" t="s">
+      <c r="C128" s="55"/>
+      <c r="D128" s="55"/>
+      <c r="E128" s="55"/>
+      <c r="F128" s="55"/>
+      <c r="G128" s="55"/>
+      <c r="H128" s="55"/>
+      <c r="I128" s="55"/>
+      <c r="J128" s="55"/>
+      <c r="K128" s="56"/>
+    </row>
+    <row r="129" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B127" s="71" t="s">
+      <c r="B129" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C127" s="62"/>
-      <c r="D127" s="62"/>
-      <c r="E127" s="62"/>
-      <c r="F127" s="62"/>
-      <c r="G127" s="62"/>
-      <c r="H127" s="62"/>
-      <c r="I127" s="62"/>
-      <c r="J127" s="62"/>
-      <c r="K127" s="63"/>
-    </row>
-    <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A128" s="37"/>
-      <c r="B128" s="38"/>
-      <c r="C128" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D128" s="38"/>
-      <c r="E128" s="40"/>
-      <c r="F128" s="40"/>
-      <c r="G128" s="41"/>
-      <c r="H128" s="41"/>
-      <c r="I128" s="41">
-        <f t="shared" ref="I128:I138" si="8">H128-G128</f>
-        <v>0</v>
-      </c>
-      <c r="J128" s="45"/>
-      <c r="K128" s="43"/>
-    </row>
-    <row r="129" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A129" s="37"/>
-      <c r="B129" s="38"/>
-      <c r="C129" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D129" s="38"/>
-      <c r="E129" s="40"/>
-      <c r="F129" s="40"/>
-      <c r="G129" s="41"/>
-      <c r="H129" s="41"/>
-      <c r="I129" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J129" s="45"/>
-      <c r="K129" s="43"/>
+      <c r="C129" s="55"/>
+      <c r="D129" s="55"/>
+      <c r="E129" s="55"/>
+      <c r="F129" s="55"/>
+      <c r="G129" s="55"/>
+      <c r="H129" s="55"/>
+      <c r="I129" s="55"/>
+      <c r="J129" s="55"/>
+      <c r="K129" s="56"/>
     </row>
     <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A130" s="37"/>
@@ -4973,13 +5138,11 @@
       <c r="G130" s="41"/>
       <c r="H130" s="41"/>
       <c r="I130" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I130:I140" si="8">H130-G130</f>
         <v>0</v>
       </c>
       <c r="J130" s="45"/>
-      <c r="K130" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K130" s="43"/>
     </row>
     <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A131" s="37"/>
@@ -5015,7 +5178,9 @@
         <v>0</v>
       </c>
       <c r="J132" s="45"/>
-      <c r="K132" s="43"/>
+      <c r="K132" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A133" s="37"/>
@@ -5108,113 +5273,113 @@
       <c r="K137" s="43"/>
     </row>
     <row r="138" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A138" s="13"/>
-      <c r="B138" s="15"/>
-      <c r="C138" s="15"/>
-      <c r="D138" s="15"/>
-      <c r="E138" s="15" t="s">
+      <c r="A138" s="37"/>
+      <c r="B138" s="38"/>
+      <c r="C138" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D138" s="38"/>
+      <c r="E138" s="40"/>
+      <c r="F138" s="40"/>
+      <c r="G138" s="41"/>
+      <c r="H138" s="41"/>
+      <c r="I138" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J138" s="45"/>
+      <c r="K138" s="43"/>
+    </row>
+    <row r="139" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A139" s="37"/>
+      <c r="B139" s="38"/>
+      <c r="C139" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D139" s="38"/>
+      <c r="E139" s="40"/>
+      <c r="F139" s="40"/>
+      <c r="G139" s="41"/>
+      <c r="H139" s="41"/>
+      <c r="I139" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J139" s="45"/>
+      <c r="K139" s="43"/>
+    </row>
+    <row r="140" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A140" s="13"/>
+      <c r="B140" s="15"/>
+      <c r="C140" s="15"/>
+      <c r="D140" s="15"/>
+      <c r="E140" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F138" s="15"/>
-      <c r="G138" s="18">
-        <f t="shared" ref="G138:H138" si="9">SUM(G128:G137)</f>
-        <v>0</v>
-      </c>
-      <c r="H138" s="18">
+      <c r="F140" s="15"/>
+      <c r="G140" s="18">
+        <f t="shared" ref="G140:H140" si="9">SUM(G130:G139)</f>
+        <v>0</v>
+      </c>
+      <c r="H140" s="18">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="I138" s="18">
+      <c r="I140" s="18">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J138" s="19"/>
-      <c r="K138" s="46"/>
-    </row>
-    <row r="139" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="72" t="s">
+      <c r="J140" s="19"/>
+      <c r="K140" s="46"/>
+    </row>
+    <row r="141" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B139" s="62"/>
-      <c r="C139" s="62"/>
-      <c r="D139" s="62"/>
-      <c r="E139" s="62"/>
-      <c r="F139" s="62"/>
-      <c r="G139" s="62"/>
-      <c r="H139" s="62"/>
-      <c r="I139" s="62"/>
-      <c r="J139" s="62"/>
-      <c r="K139" s="63"/>
-    </row>
-    <row r="140" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A140" s="29" t="s">
+      <c r="B141" s="55"/>
+      <c r="C141" s="55"/>
+      <c r="D141" s="55"/>
+      <c r="E141" s="55"/>
+      <c r="F141" s="55"/>
+      <c r="G141" s="55"/>
+      <c r="H141" s="55"/>
+      <c r="I141" s="55"/>
+      <c r="J141" s="55"/>
+      <c r="K141" s="56"/>
+    </row>
+    <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A142" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B140" s="69" t="s">
+      <c r="B142" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C140" s="62"/>
-      <c r="D140" s="62"/>
-      <c r="E140" s="62"/>
-      <c r="F140" s="62"/>
-      <c r="G140" s="62"/>
-      <c r="H140" s="62"/>
-      <c r="I140" s="62"/>
-      <c r="J140" s="62"/>
-      <c r="K140" s="63"/>
-    </row>
-    <row r="141" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="30" t="s">
+      <c r="C142" s="55"/>
+      <c r="D142" s="55"/>
+      <c r="E142" s="55"/>
+      <c r="F142" s="55"/>
+      <c r="G142" s="55"/>
+      <c r="H142" s="55"/>
+      <c r="I142" s="55"/>
+      <c r="J142" s="55"/>
+      <c r="K142" s="56"/>
+    </row>
+    <row r="143" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B141" s="69" t="s">
+      <c r="B143" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C141" s="62"/>
-      <c r="D141" s="62"/>
-      <c r="E141" s="62"/>
-      <c r="F141" s="62"/>
-      <c r="G141" s="62"/>
-      <c r="H141" s="62"/>
-      <c r="I141" s="62"/>
-      <c r="J141" s="62"/>
-      <c r="K141" s="63"/>
-    </row>
-    <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A142" s="37"/>
-      <c r="B142" s="38"/>
-      <c r="C142" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D142" s="38"/>
-      <c r="E142" s="40"/>
-      <c r="F142" s="40"/>
-      <c r="G142" s="41"/>
-      <c r="H142" s="41"/>
-      <c r="I142" s="41">
-        <f t="shared" ref="I142:I152" si="10">H142-G142</f>
-        <v>0</v>
-      </c>
-      <c r="J142" s="45"/>
-      <c r="K142" s="43"/>
-    </row>
-    <row r="143" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A143" s="37"/>
-      <c r="B143" s="38"/>
-      <c r="C143" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D143" s="38"/>
-      <c r="E143" s="40"/>
-      <c r="F143" s="40"/>
-      <c r="G143" s="41"/>
-      <c r="H143" s="41"/>
-      <c r="I143" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J143" s="45"/>
-      <c r="K143" s="43"/>
+      <c r="C143" s="55"/>
+      <c r="D143" s="55"/>
+      <c r="E143" s="55"/>
+      <c r="F143" s="55"/>
+      <c r="G143" s="55"/>
+      <c r="H143" s="55"/>
+      <c r="I143" s="55"/>
+      <c r="J143" s="55"/>
+      <c r="K143" s="56"/>
     </row>
     <row r="144" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A144" s="37"/>
@@ -5228,7 +5393,7 @@
       <c r="G144" s="41"/>
       <c r="H144" s="41"/>
       <c r="I144" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I144:I154" si="10">H144-G144</f>
         <v>0</v>
       </c>
       <c r="J144" s="45"/>
@@ -5361,113 +5526,113 @@
       <c r="K151" s="43"/>
     </row>
     <row r="152" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A152" s="13"/>
-      <c r="B152" s="15"/>
-      <c r="C152" s="15"/>
-      <c r="D152" s="15"/>
-      <c r="E152" s="15" t="s">
+      <c r="A152" s="37"/>
+      <c r="B152" s="38"/>
+      <c r="C152" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D152" s="38"/>
+      <c r="E152" s="40"/>
+      <c r="F152" s="40"/>
+      <c r="G152" s="41"/>
+      <c r="H152" s="41"/>
+      <c r="I152" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J152" s="45"/>
+      <c r="K152" s="43"/>
+    </row>
+    <row r="153" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A153" s="37"/>
+      <c r="B153" s="38"/>
+      <c r="C153" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D153" s="38"/>
+      <c r="E153" s="40"/>
+      <c r="F153" s="40"/>
+      <c r="G153" s="41"/>
+      <c r="H153" s="41"/>
+      <c r="I153" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J153" s="45"/>
+      <c r="K153" s="43"/>
+    </row>
+    <row r="154" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A154" s="13"/>
+      <c r="B154" s="15"/>
+      <c r="C154" s="15"/>
+      <c r="D154" s="15"/>
+      <c r="E154" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F152" s="15"/>
-      <c r="G152" s="18">
-        <f t="shared" ref="G152:H152" si="11">SUM(G142:G151)</f>
-        <v>0</v>
-      </c>
-      <c r="H152" s="18">
+      <c r="F154" s="15"/>
+      <c r="G154" s="18">
+        <f t="shared" ref="G154:H154" si="11">SUM(G144:G153)</f>
+        <v>0</v>
+      </c>
+      <c r="H154" s="18">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="I152" s="18">
+      <c r="I154" s="18">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J152" s="19"/>
-      <c r="K152" s="46"/>
-    </row>
-    <row r="153" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="54" t="s">
+      <c r="J154" s="19"/>
+      <c r="K154" s="46"/>
+    </row>
+    <row r="155" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B153" s="55"/>
-      <c r="C153" s="55"/>
-      <c r="D153" s="55"/>
-      <c r="E153" s="55"/>
-      <c r="F153" s="55"/>
-      <c r="G153" s="55"/>
-      <c r="H153" s="55"/>
-      <c r="I153" s="55"/>
-      <c r="J153" s="55"/>
-      <c r="K153" s="56"/>
-    </row>
-    <row r="154" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A154" s="32" t="s">
+      <c r="B155" s="63"/>
+      <c r="C155" s="63"/>
+      <c r="D155" s="63"/>
+      <c r="E155" s="63"/>
+      <c r="F155" s="63"/>
+      <c r="G155" s="63"/>
+      <c r="H155" s="63"/>
+      <c r="I155" s="63"/>
+      <c r="J155" s="63"/>
+      <c r="K155" s="64"/>
+    </row>
+    <row r="156" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A156" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B154" s="57" t="s">
+      <c r="B156" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C154" s="55"/>
-      <c r="D154" s="55"/>
-      <c r="E154" s="55"/>
-      <c r="F154" s="55"/>
-      <c r="G154" s="55"/>
-      <c r="H154" s="55"/>
-      <c r="I154" s="55"/>
-      <c r="J154" s="55"/>
-      <c r="K154" s="56"/>
-    </row>
-    <row r="155" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="33" t="s">
+      <c r="C156" s="63"/>
+      <c r="D156" s="63"/>
+      <c r="E156" s="63"/>
+      <c r="F156" s="63"/>
+      <c r="G156" s="63"/>
+      <c r="H156" s="63"/>
+      <c r="I156" s="63"/>
+      <c r="J156" s="63"/>
+      <c r="K156" s="64"/>
+    </row>
+    <row r="157" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B155" s="57" t="s">
+      <c r="B157" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C155" s="55"/>
-      <c r="D155" s="55"/>
-      <c r="E155" s="55"/>
-      <c r="F155" s="55"/>
-      <c r="G155" s="55"/>
-      <c r="H155" s="55"/>
-      <c r="I155" s="55"/>
-      <c r="J155" s="55"/>
-      <c r="K155" s="56"/>
-    </row>
-    <row r="156" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A156" s="37"/>
-      <c r="B156" s="38"/>
-      <c r="C156" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D156" s="38"/>
-      <c r="E156" s="40"/>
-      <c r="F156" s="40"/>
-      <c r="G156" s="41"/>
-      <c r="H156" s="41"/>
-      <c r="I156" s="41">
-        <f t="shared" ref="I156:I166" si="12">H156-G156</f>
-        <v>0</v>
-      </c>
-      <c r="J156" s="45"/>
-      <c r="K156" s="43"/>
-    </row>
-    <row r="157" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A157" s="37"/>
-      <c r="B157" s="38"/>
-      <c r="C157" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D157" s="38"/>
-      <c r="E157" s="40"/>
-      <c r="F157" s="40"/>
-      <c r="G157" s="41"/>
-      <c r="H157" s="41"/>
-      <c r="I157" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J157" s="45"/>
-      <c r="K157" s="43"/>
+      <c r="C157" s="63"/>
+      <c r="D157" s="63"/>
+      <c r="E157" s="63"/>
+      <c r="F157" s="63"/>
+      <c r="G157" s="63"/>
+      <c r="H157" s="63"/>
+      <c r="I157" s="63"/>
+      <c r="J157" s="63"/>
+      <c r="K157" s="64"/>
     </row>
     <row r="158" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A158" s="37"/>
@@ -5481,7 +5646,7 @@
       <c r="G158" s="41"/>
       <c r="H158" s="41"/>
       <c r="I158" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="I158:I168" si="12">H158-G158</f>
         <v>0</v>
       </c>
       <c r="J158" s="45"/>
@@ -5614,35 +5779,71 @@
       <c r="K165" s="43"/>
     </row>
     <row r="166" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A166" s="48"/>
-      <c r="B166" s="49"/>
-      <c r="C166" s="49"/>
-      <c r="D166" s="49"/>
-      <c r="E166" s="49" t="s">
+      <c r="A166" s="37"/>
+      <c r="B166" s="38"/>
+      <c r="C166" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D166" s="38"/>
+      <c r="E166" s="40"/>
+      <c r="F166" s="40"/>
+      <c r="G166" s="41"/>
+      <c r="H166" s="41"/>
+      <c r="I166" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J166" s="45"/>
+      <c r="K166" s="43"/>
+    </row>
+    <row r="167" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A167" s="37"/>
+      <c r="B167" s="38"/>
+      <c r="C167" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D167" s="38"/>
+      <c r="E167" s="40"/>
+      <c r="F167" s="40"/>
+      <c r="G167" s="41"/>
+      <c r="H167" s="41"/>
+      <c r="I167" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J167" s="45"/>
+      <c r="K167" s="43"/>
+    </row>
+    <row r="168" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A168" s="48"/>
+      <c r="B168" s="49"/>
+      <c r="C168" s="49"/>
+      <c r="D168" s="49"/>
+      <c r="E168" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F166" s="49"/>
-      <c r="G166" s="50">
-        <f t="shared" ref="G166:H166" si="13">SUM(G156:G165)</f>
-        <v>0</v>
-      </c>
-      <c r="H166" s="50">
+      <c r="F168" s="49"/>
+      <c r="G168" s="50">
+        <f t="shared" ref="G168:H168" si="13">SUM(G158:G167)</f>
+        <v>0</v>
+      </c>
+      <c r="H168" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="I166" s="50">
+      <c r="I168" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J166" s="51"/>
-      <c r="K166" s="52"/>
+      <c r="J168" s="51"/>
+      <c r="K168" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{4455D6ED-FAC2-488E-BD29-41FCE24FB687}">
+      <autoFilter ref="A1:K15" xr:uid="{5FA84217-2540-41CB-8206-F264705ECBC8}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5653,17 +5854,9 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B126:K126"/>
-    <mergeCell ref="B127:K127"/>
-    <mergeCell ref="A139:K139"/>
-    <mergeCell ref="B99:K99"/>
-    <mergeCell ref="A111:K111"/>
-    <mergeCell ref="B112:K112"/>
-    <mergeCell ref="B113:K113"/>
-    <mergeCell ref="A125:K125"/>
-    <mergeCell ref="A153:K153"/>
-    <mergeCell ref="B154:K154"/>
-    <mergeCell ref="B155:K155"/>
+    <mergeCell ref="A155:K155"/>
+    <mergeCell ref="B156:K156"/>
+    <mergeCell ref="B157:K157"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -5673,12 +5866,20 @@
     <mergeCell ref="A83:K83"/>
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
-    <mergeCell ref="A97:K97"/>
-    <mergeCell ref="B140:K140"/>
-    <mergeCell ref="B141:K141"/>
-    <mergeCell ref="B98:K98"/>
+    <mergeCell ref="A99:K99"/>
+    <mergeCell ref="B142:K142"/>
+    <mergeCell ref="B143:K143"/>
+    <mergeCell ref="B100:K100"/>
+    <mergeCell ref="B128:K128"/>
+    <mergeCell ref="B129:K129"/>
+    <mergeCell ref="A141:K141"/>
+    <mergeCell ref="B101:K101"/>
+    <mergeCell ref="A113:K113"/>
+    <mergeCell ref="B114:K114"/>
+    <mergeCell ref="B115:K115"/>
+    <mergeCell ref="A127:K127"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B95 B100:B109 B114:B123 B128:B137 B142:B151">
+  <conditionalFormatting sqref="B5:B45 B86:B97 B102:B111 B116:B125 B130:B139 B144:B153 B48:B81">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5695,7 +5896,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B96 B98:B110 B112:B124 B126:B138 B140:B152 B154:B166">
+  <conditionalFormatting sqref="B5:B46 B84:B98 B100:B112 B114:B126 B128:B140 B142:B154 B156:B168 B48:B82">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5703,34 +5904,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B156:B165">
+  <conditionalFormatting sqref="B158:B167">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B156))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B158))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B156))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B158))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B156))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B158))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B156))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B158))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B156))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B158))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G96 G100:G110 G114:G124 G128:G138 G142:G152 G156:G166">
+  <conditionalFormatting sqref="G1 G3:G46 G86:G98 G102:G112 G116:G126 G130:G140 G144:G154 G158:G168 G50:G82">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H166">
+  <conditionalFormatting sqref="H1:H168">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I86:I96 I100:I110 I114:I124 I128:I138 I142:I152 I156:I166 I50:I82">
+  <conditionalFormatting sqref="I5:I46 I102:I112 I116:I126 I130:I140 I144:I154 I158:I168 I86:I98 I50:I82">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -5739,7 +5940,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F156:F165 F142:F151 F50:F81 F86:F95 F100:F109 F114:F123 F128:F137 F5:F45" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F158:F167 F144:F153 F86:F97 F102:F111 F116:F125 F130:F139 F5:F45 F81 F50:F80" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5755,13 +5956,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E50:E81 E86:E95 E100:E109 E114:E123 E128:E137 E142:E151 E156:E165</xm:sqref>
+          <xm:sqref>E5:E45 E86:E97 E102:E111 E116:E125 E130:E139 E144:E153 E158:E167 E81 E50:E80</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B50:B81 B86:B95 B100:B109 B114:B123 B128:B137 B142:B151 B156:B165</xm:sqref>
+          <xm:sqref>B5:B45 B86:B97 B102:B111 B116:B125 B130:B139 B144:B153 B158:B167 B81 B50:B80</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7402,6 +7603,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -7636,27 +7857,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7673,23 +7893,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W3 Datalab 1 Work I
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A542D92-A685-4C29-BCD6-35756D4E2CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BF0BC81-1E36-4791-A38F-85A32A89C15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1094,26 +1094,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1130,6 +1110,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1147,6 +1129,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1671,53 +1671,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3056,53 +3056,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="62"/>
+      <c r="K49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4155,53 +4155,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72" t="s">
+      <c r="A83" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="55"/>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="55"/>
-      <c r="I83" s="55"/>
-      <c r="J83" s="55"/>
-      <c r="K83" s="56"/>
+      <c r="B83" s="62"/>
+      <c r="C83" s="62"/>
+      <c r="D83" s="62"/>
+      <c r="E83" s="62"/>
+      <c r="F83" s="62"/>
+      <c r="G83" s="62"/>
+      <c r="H83" s="62"/>
+      <c r="I83" s="62"/>
+      <c r="J83" s="62"/>
+      <c r="K83" s="63"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="73" t="s">
+      <c r="B84" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="55"/>
-      <c r="D84" s="55"/>
-      <c r="E84" s="55"/>
-      <c r="F84" s="55"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="55"/>
-      <c r="I84" s="55"/>
-      <c r="J84" s="55"/>
-      <c r="K84" s="56"/>
+      <c r="C84" s="62"/>
+      <c r="D84" s="62"/>
+      <c r="E84" s="62"/>
+      <c r="F84" s="62"/>
+      <c r="G84" s="62"/>
+      <c r="H84" s="62"/>
+      <c r="I84" s="62"/>
+      <c r="J84" s="62"/>
+      <c r="K84" s="63"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="73" t="s">
+      <c r="B85" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="55"/>
-      <c r="D85" s="55"/>
-      <c r="E85" s="55"/>
-      <c r="F85" s="55"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="55"/>
-      <c r="I85" s="55"/>
-      <c r="J85" s="55"/>
-      <c r="K85" s="56"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="62"/>
+      <c r="G85" s="62"/>
+      <c r="H85" s="62"/>
+      <c r="I85" s="62"/>
+      <c r="J85" s="62"/>
+      <c r="K85" s="63"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -4572,53 +4572,53 @@
       <c r="K98" s="46"/>
     </row>
     <row r="99" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="74" t="s">
+      <c r="A99" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B99" s="55"/>
-      <c r="C99" s="55"/>
-      <c r="D99" s="55"/>
-      <c r="E99" s="55"/>
-      <c r="F99" s="55"/>
-      <c r="G99" s="55"/>
-      <c r="H99" s="55"/>
-      <c r="I99" s="55"/>
-      <c r="J99" s="55"/>
-      <c r="K99" s="56"/>
+      <c r="B99" s="62"/>
+      <c r="C99" s="62"/>
+      <c r="D99" s="62"/>
+      <c r="E99" s="62"/>
+      <c r="F99" s="62"/>
+      <c r="G99" s="62"/>
+      <c r="H99" s="62"/>
+      <c r="I99" s="62"/>
+      <c r="J99" s="62"/>
+      <c r="K99" s="63"/>
     </row>
     <row r="100" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A100" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B100" s="58" t="s">
+      <c r="B100" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C100" s="55"/>
-      <c r="D100" s="55"/>
-      <c r="E100" s="55"/>
-      <c r="F100" s="55"/>
-      <c r="G100" s="55"/>
-      <c r="H100" s="55"/>
-      <c r="I100" s="55"/>
-      <c r="J100" s="55"/>
-      <c r="K100" s="56"/>
+      <c r="C100" s="62"/>
+      <c r="D100" s="62"/>
+      <c r="E100" s="62"/>
+      <c r="F100" s="62"/>
+      <c r="G100" s="62"/>
+      <c r="H100" s="62"/>
+      <c r="I100" s="62"/>
+      <c r="J100" s="62"/>
+      <c r="K100" s="63"/>
     </row>
     <row r="101" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B101" s="58" t="s">
+      <c r="B101" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C101" s="55"/>
-      <c r="D101" s="55"/>
-      <c r="E101" s="55"/>
-      <c r="F101" s="55"/>
-      <c r="G101" s="55"/>
-      <c r="H101" s="55"/>
-      <c r="I101" s="55"/>
-      <c r="J101" s="55"/>
-      <c r="K101" s="56"/>
+      <c r="C101" s="62"/>
+      <c r="D101" s="62"/>
+      <c r="E101" s="62"/>
+      <c r="F101" s="62"/>
+      <c r="G101" s="62"/>
+      <c r="H101" s="62"/>
+      <c r="I101" s="62"/>
+      <c r="J101" s="62"/>
+      <c r="K101" s="63"/>
     </row>
     <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A102" s="37"/>
@@ -4825,53 +4825,53 @@
       <c r="K112" s="46"/>
     </row>
     <row r="113" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="59" t="s">
+      <c r="A113" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B113" s="55"/>
-      <c r="C113" s="55"/>
-      <c r="D113" s="55"/>
-      <c r="E113" s="55"/>
-      <c r="F113" s="55"/>
-      <c r="G113" s="55"/>
-      <c r="H113" s="55"/>
-      <c r="I113" s="55"/>
-      <c r="J113" s="55"/>
-      <c r="K113" s="56"/>
+      <c r="B113" s="62"/>
+      <c r="C113" s="62"/>
+      <c r="D113" s="62"/>
+      <c r="E113" s="62"/>
+      <c r="F113" s="62"/>
+      <c r="G113" s="62"/>
+      <c r="H113" s="62"/>
+      <c r="I113" s="62"/>
+      <c r="J113" s="62"/>
+      <c r="K113" s="63"/>
     </row>
     <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A114" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B114" s="60" t="s">
+      <c r="B114" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C114" s="55"/>
-      <c r="D114" s="55"/>
-      <c r="E114" s="55"/>
-      <c r="F114" s="55"/>
-      <c r="G114" s="55"/>
-      <c r="H114" s="55"/>
-      <c r="I114" s="55"/>
-      <c r="J114" s="55"/>
-      <c r="K114" s="56"/>
+      <c r="C114" s="62"/>
+      <c r="D114" s="62"/>
+      <c r="E114" s="62"/>
+      <c r="F114" s="62"/>
+      <c r="G114" s="62"/>
+      <c r="H114" s="62"/>
+      <c r="I114" s="62"/>
+      <c r="J114" s="62"/>
+      <c r="K114" s="63"/>
     </row>
     <row r="115" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B115" s="60" t="s">
+      <c r="B115" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C115" s="55"/>
-      <c r="D115" s="55"/>
-      <c r="E115" s="55"/>
-      <c r="F115" s="55"/>
-      <c r="G115" s="55"/>
-      <c r="H115" s="55"/>
-      <c r="I115" s="55"/>
-      <c r="J115" s="55"/>
-      <c r="K115" s="56"/>
+      <c r="C115" s="62"/>
+      <c r="D115" s="62"/>
+      <c r="E115" s="62"/>
+      <c r="F115" s="62"/>
+      <c r="G115" s="62"/>
+      <c r="H115" s="62"/>
+      <c r="I115" s="62"/>
+      <c r="J115" s="62"/>
+      <c r="K115" s="63"/>
     </row>
     <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A116" s="37"/>
@@ -5078,53 +5078,53 @@
       <c r="K126" s="46"/>
     </row>
     <row r="127" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="61" t="s">
+      <c r="A127" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B127" s="55"/>
-      <c r="C127" s="55"/>
-      <c r="D127" s="55"/>
-      <c r="E127" s="55"/>
-      <c r="F127" s="55"/>
-      <c r="G127" s="55"/>
-      <c r="H127" s="55"/>
-      <c r="I127" s="55"/>
-      <c r="J127" s="55"/>
-      <c r="K127" s="56"/>
+      <c r="B127" s="62"/>
+      <c r="C127" s="62"/>
+      <c r="D127" s="62"/>
+      <c r="E127" s="62"/>
+      <c r="F127" s="62"/>
+      <c r="G127" s="62"/>
+      <c r="H127" s="62"/>
+      <c r="I127" s="62"/>
+      <c r="J127" s="62"/>
+      <c r="K127" s="63"/>
     </row>
     <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A128" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B128" s="54" t="s">
+      <c r="B128" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C128" s="55"/>
-      <c r="D128" s="55"/>
-      <c r="E128" s="55"/>
-      <c r="F128" s="55"/>
-      <c r="G128" s="55"/>
-      <c r="H128" s="55"/>
-      <c r="I128" s="55"/>
-      <c r="J128" s="55"/>
-      <c r="K128" s="56"/>
+      <c r="C128" s="62"/>
+      <c r="D128" s="62"/>
+      <c r="E128" s="62"/>
+      <c r="F128" s="62"/>
+      <c r="G128" s="62"/>
+      <c r="H128" s="62"/>
+      <c r="I128" s="62"/>
+      <c r="J128" s="62"/>
+      <c r="K128" s="63"/>
     </row>
     <row r="129" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B129" s="54" t="s">
+      <c r="B129" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C129" s="55"/>
-      <c r="D129" s="55"/>
-      <c r="E129" s="55"/>
-      <c r="F129" s="55"/>
-      <c r="G129" s="55"/>
-      <c r="H129" s="55"/>
-      <c r="I129" s="55"/>
-      <c r="J129" s="55"/>
-      <c r="K129" s="56"/>
+      <c r="C129" s="62"/>
+      <c r="D129" s="62"/>
+      <c r="E129" s="62"/>
+      <c r="F129" s="62"/>
+      <c r="G129" s="62"/>
+      <c r="H129" s="62"/>
+      <c r="I129" s="62"/>
+      <c r="J129" s="62"/>
+      <c r="K129" s="63"/>
     </row>
     <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A130" s="37"/>
@@ -5333,53 +5333,53 @@
       <c r="K140" s="46"/>
     </row>
     <row r="141" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="57" t="s">
+      <c r="A141" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="B141" s="55"/>
-      <c r="C141" s="55"/>
-      <c r="D141" s="55"/>
-      <c r="E141" s="55"/>
-      <c r="F141" s="55"/>
-      <c r="G141" s="55"/>
-      <c r="H141" s="55"/>
-      <c r="I141" s="55"/>
-      <c r="J141" s="55"/>
-      <c r="K141" s="56"/>
+      <c r="B141" s="62"/>
+      <c r="C141" s="62"/>
+      <c r="D141" s="62"/>
+      <c r="E141" s="62"/>
+      <c r="F141" s="62"/>
+      <c r="G141" s="62"/>
+      <c r="H141" s="62"/>
+      <c r="I141" s="62"/>
+      <c r="J141" s="62"/>
+      <c r="K141" s="63"/>
     </row>
     <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A142" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B142" s="75" t="s">
+      <c r="B142" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C142" s="55"/>
-      <c r="D142" s="55"/>
-      <c r="E142" s="55"/>
-      <c r="F142" s="55"/>
-      <c r="G142" s="55"/>
-      <c r="H142" s="55"/>
-      <c r="I142" s="55"/>
-      <c r="J142" s="55"/>
-      <c r="K142" s="56"/>
+      <c r="C142" s="62"/>
+      <c r="D142" s="62"/>
+      <c r="E142" s="62"/>
+      <c r="F142" s="62"/>
+      <c r="G142" s="62"/>
+      <c r="H142" s="62"/>
+      <c r="I142" s="62"/>
+      <c r="J142" s="62"/>
+      <c r="K142" s="63"/>
     </row>
     <row r="143" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B143" s="75" t="s">
+      <c r="B143" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C143" s="55"/>
-      <c r="D143" s="55"/>
-      <c r="E143" s="55"/>
-      <c r="F143" s="55"/>
-      <c r="G143" s="55"/>
-      <c r="H143" s="55"/>
-      <c r="I143" s="55"/>
-      <c r="J143" s="55"/>
-      <c r="K143" s="56"/>
+      <c r="C143" s="62"/>
+      <c r="D143" s="62"/>
+      <c r="E143" s="62"/>
+      <c r="F143" s="62"/>
+      <c r="G143" s="62"/>
+      <c r="H143" s="62"/>
+      <c r="I143" s="62"/>
+      <c r="J143" s="62"/>
+      <c r="K143" s="63"/>
     </row>
     <row r="144" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A144" s="37"/>
@@ -5586,53 +5586,53 @@
       <c r="K154" s="46"/>
     </row>
     <row r="155" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="62" t="s">
+      <c r="A155" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B155" s="63"/>
-      <c r="C155" s="63"/>
-      <c r="D155" s="63"/>
-      <c r="E155" s="63"/>
-      <c r="F155" s="63"/>
-      <c r="G155" s="63"/>
-      <c r="H155" s="63"/>
-      <c r="I155" s="63"/>
-      <c r="J155" s="63"/>
-      <c r="K155" s="64"/>
+      <c r="B155" s="55"/>
+      <c r="C155" s="55"/>
+      <c r="D155" s="55"/>
+      <c r="E155" s="55"/>
+      <c r="F155" s="55"/>
+      <c r="G155" s="55"/>
+      <c r="H155" s="55"/>
+      <c r="I155" s="55"/>
+      <c r="J155" s="55"/>
+      <c r="K155" s="56"/>
     </row>
     <row r="156" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A156" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B156" s="65" t="s">
+      <c r="B156" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C156" s="63"/>
-      <c r="D156" s="63"/>
-      <c r="E156" s="63"/>
-      <c r="F156" s="63"/>
-      <c r="G156" s="63"/>
-      <c r="H156" s="63"/>
-      <c r="I156" s="63"/>
-      <c r="J156" s="63"/>
-      <c r="K156" s="64"/>
+      <c r="C156" s="55"/>
+      <c r="D156" s="55"/>
+      <c r="E156" s="55"/>
+      <c r="F156" s="55"/>
+      <c r="G156" s="55"/>
+      <c r="H156" s="55"/>
+      <c r="I156" s="55"/>
+      <c r="J156" s="55"/>
+      <c r="K156" s="56"/>
     </row>
     <row r="157" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B157" s="65" t="s">
+      <c r="B157" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C157" s="63"/>
-      <c r="D157" s="63"/>
-      <c r="E157" s="63"/>
-      <c r="F157" s="63"/>
-      <c r="G157" s="63"/>
-      <c r="H157" s="63"/>
-      <c r="I157" s="63"/>
-      <c r="J157" s="63"/>
-      <c r="K157" s="64"/>
+      <c r="C157" s="55"/>
+      <c r="D157" s="55"/>
+      <c r="E157" s="55"/>
+      <c r="F157" s="55"/>
+      <c r="G157" s="55"/>
+      <c r="H157" s="55"/>
+      <c r="I157" s="55"/>
+      <c r="J157" s="55"/>
+      <c r="K157" s="56"/>
     </row>
     <row r="158" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A158" s="37"/>
@@ -5843,7 +5843,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{5FA84217-2540-41CB-8206-F264705ECBC8}">
+      <autoFilter ref="A1:K15" xr:uid="{47F12E79-EA31-4F9C-A76A-23D0ED283334}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5854,6 +5854,14 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
+    <mergeCell ref="B128:K128"/>
+    <mergeCell ref="B129:K129"/>
+    <mergeCell ref="A141:K141"/>
+    <mergeCell ref="B101:K101"/>
+    <mergeCell ref="A113:K113"/>
+    <mergeCell ref="B114:K114"/>
+    <mergeCell ref="B115:K115"/>
+    <mergeCell ref="A127:K127"/>
     <mergeCell ref="A155:K155"/>
     <mergeCell ref="B156:K156"/>
     <mergeCell ref="B157:K157"/>
@@ -5870,16 +5878,8 @@
     <mergeCell ref="B142:K142"/>
     <mergeCell ref="B143:K143"/>
     <mergeCell ref="B100:K100"/>
-    <mergeCell ref="B128:K128"/>
-    <mergeCell ref="B129:K129"/>
-    <mergeCell ref="A141:K141"/>
-    <mergeCell ref="B101:K101"/>
-    <mergeCell ref="A113:K113"/>
-    <mergeCell ref="B114:K114"/>
-    <mergeCell ref="B115:K115"/>
-    <mergeCell ref="A127:K127"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B86:B97 B102:B111 B116:B125 B130:B139 B144:B153 B48:B81">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B97 B102:B111 B116:B125 B130:B139 B144:B153">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5896,7 +5896,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B84:B98 B100:B112 B114:B126 B128:B140 B142:B154 B156:B168 B48:B82">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B98 B100:B112 B114:B126 B128:B140 B142:B154 B156:B168">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5921,7 +5921,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B158))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G86:G98 G102:G112 G116:G126 G130:G140 G144:G154 G158:G168 G50:G82">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G98 G102:G112 G116:G126 G130:G140 G144:G154 G158:G168">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
@@ -5931,7 +5931,7 @@
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I102:I112 I116:I126 I130:I140 I144:I154 I158:I168 I86:I98 I50:I82">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I98 I102:I112 I116:I126 I130:I140 I144:I154 I158:I168">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -7603,26 +7603,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -7857,10 +7837,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7877,20 +7888,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W3 Datalab 1 Work II (pre-break)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BF0BC81-1E36-4791-A38F-85A32A89C15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E6DB97-A59D-4CE8-8310-0862A4DE3F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$153</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$155</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="172">
   <si>
     <t>Date</t>
   </si>
@@ -609,6 +609,15 @@
   </si>
   <si>
     <t>Look ahead at the Tuesday DataLab</t>
+  </si>
+  <si>
+    <t>DataLab 1 stand-up meeting</t>
+  </si>
+  <si>
+    <t>Implement Linear Regression</t>
+  </si>
+  <si>
+    <t>Implement Decision Tree Regression</t>
   </si>
 </sst>
 </file>
@@ -1094,6 +1103,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1110,8 +1139,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1129,24 +1156,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1619,7 +1628,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K168"/>
+  <dimension ref="A1:K170"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1671,53 +1680,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3056,53 +3065,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4155,53 +4164,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -4229,7 +4238,7 @@
         <v>0.5</v>
       </c>
       <c r="I86" s="41">
-        <f t="shared" ref="I86:I98" si="2">H86-G86</f>
+        <f t="shared" ref="I86:I100" si="2">H86-G86</f>
         <v>0</v>
       </c>
       <c r="J86" s="45"/>
@@ -4494,16 +4503,30 @@
       <c r="K94" s="43"/>
     </row>
     <row r="95" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A95" s="37"/>
-      <c r="B95" s="38"/>
+      <c r="A95" s="37">
+        <v>45629</v>
+      </c>
+      <c r="B95" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C95" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D95" s="38"/>
-      <c r="E95" s="40"/>
-      <c r="F95" s="40"/>
-      <c r="G95" s="41"/>
-      <c r="H95" s="41"/>
+      <c r="D95" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="E95" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F95" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G95" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H95" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I95" s="41">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4512,16 +4535,30 @@
       <c r="K95" s="43"/>
     </row>
     <row r="96" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A96" s="37"/>
-      <c r="B96" s="38"/>
+      <c r="A96" s="37">
+        <v>45629</v>
+      </c>
+      <c r="B96" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C96" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D96" s="38"/>
-      <c r="E96" s="40"/>
-      <c r="F96" s="40"/>
-      <c r="G96" s="41"/>
-      <c r="H96" s="41"/>
+      <c r="D96" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="E96" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F96" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G96" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H96" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I96" s="41">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4530,131 +4567,155 @@
       <c r="K96" s="43"/>
     </row>
     <row r="97" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A97" s="37"/>
-      <c r="B97" s="38"/>
+      <c r="A97" s="37">
+        <v>45629</v>
+      </c>
+      <c r="B97" s="38" t="s">
+        <v>52</v>
+      </c>
       <c r="C97" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D97" s="38"/>
-      <c r="E97" s="40"/>
-      <c r="F97" s="40"/>
-      <c r="G97" s="41"/>
+      <c r="D97" s="38" t="s">
+        <v>170</v>
+      </c>
+      <c r="E97" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F97" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G97" s="41">
+        <v>4</v>
+      </c>
       <c r="H97" s="41"/>
       <c r="I97" s="41">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="J97" s="45"/>
       <c r="K97" s="43"/>
     </row>
     <row r="98" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A98" s="13"/>
-      <c r="B98" s="15"/>
-      <c r="C98" s="15"/>
-      <c r="D98" s="15"/>
-      <c r="E98" s="15" t="s">
+      <c r="A98" s="37">
+        <v>45629</v>
+      </c>
+      <c r="B98" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C98" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D98" s="38" t="s">
+        <v>171</v>
+      </c>
+      <c r="E98" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F98" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G98" s="41">
+        <v>2.5</v>
+      </c>
+      <c r="H98" s="41"/>
+      <c r="I98" s="41">
+        <f t="shared" si="2"/>
+        <v>-2.5</v>
+      </c>
+      <c r="J98" s="45"/>
+      <c r="K98" s="43"/>
+    </row>
+    <row r="99" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A99" s="37"/>
+      <c r="B99" s="38"/>
+      <c r="C99" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D99" s="38"/>
+      <c r="E99" s="40"/>
+      <c r="F99" s="40"/>
+      <c r="G99" s="41"/>
+      <c r="H99" s="41"/>
+      <c r="I99" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J99" s="45"/>
+      <c r="K99" s="43"/>
+    </row>
+    <row r="100" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A100" s="13"/>
+      <c r="B100" s="15"/>
+      <c r="C100" s="15"/>
+      <c r="D100" s="15"/>
+      <c r="E100" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F98" s="15"/>
-      <c r="G98" s="18">
-        <f t="shared" ref="G98:H98" si="3">SUM(G86:G97)</f>
-        <v>9.25</v>
-      </c>
-      <c r="H98" s="18">
+      <c r="F100" s="15"/>
+      <c r="G100" s="18">
+        <f t="shared" ref="G100:H100" si="3">SUM(G86:G99)</f>
+        <v>16.5</v>
+      </c>
+      <c r="H100" s="18">
         <f t="shared" si="3"/>
-        <v>7.5</v>
-      </c>
-      <c r="I98" s="18">
+        <v>8.25</v>
+      </c>
+      <c r="I100" s="18">
         <f t="shared" si="2"/>
-        <v>-1.75</v>
-      </c>
-      <c r="J98" s="19"/>
-      <c r="K98" s="46"/>
-    </row>
-    <row r="99" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="68" t="s">
+        <v>-8.25</v>
+      </c>
+      <c r="J100" s="19"/>
+      <c r="K100" s="46"/>
+    </row>
+    <row r="101" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B99" s="62"/>
-      <c r="C99" s="62"/>
-      <c r="D99" s="62"/>
-      <c r="E99" s="62"/>
-      <c r="F99" s="62"/>
-      <c r="G99" s="62"/>
-      <c r="H99" s="62"/>
-      <c r="I99" s="62"/>
-      <c r="J99" s="62"/>
-      <c r="K99" s="63"/>
-    </row>
-    <row r="100" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A100" s="23" t="s">
+      <c r="B101" s="55"/>
+      <c r="C101" s="55"/>
+      <c r="D101" s="55"/>
+      <c r="E101" s="55"/>
+      <c r="F101" s="55"/>
+      <c r="G101" s="55"/>
+      <c r="H101" s="55"/>
+      <c r="I101" s="55"/>
+      <c r="J101" s="55"/>
+      <c r="K101" s="56"/>
+    </row>
+    <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A102" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B100" s="70" t="s">
+      <c r="B102" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C100" s="62"/>
-      <c r="D100" s="62"/>
-      <c r="E100" s="62"/>
-      <c r="F100" s="62"/>
-      <c r="G100" s="62"/>
-      <c r="H100" s="62"/>
-      <c r="I100" s="62"/>
-      <c r="J100" s="62"/>
-      <c r="K100" s="63"/>
-    </row>
-    <row r="101" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="24" t="s">
+      <c r="C102" s="55"/>
+      <c r="D102" s="55"/>
+      <c r="E102" s="55"/>
+      <c r="F102" s="55"/>
+      <c r="G102" s="55"/>
+      <c r="H102" s="55"/>
+      <c r="I102" s="55"/>
+      <c r="J102" s="55"/>
+      <c r="K102" s="56"/>
+    </row>
+    <row r="103" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B101" s="70" t="s">
+      <c r="B103" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C101" s="62"/>
-      <c r="D101" s="62"/>
-      <c r="E101" s="62"/>
-      <c r="F101" s="62"/>
-      <c r="G101" s="62"/>
-      <c r="H101" s="62"/>
-      <c r="I101" s="62"/>
-      <c r="J101" s="62"/>
-      <c r="K101" s="63"/>
-    </row>
-    <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A102" s="37"/>
-      <c r="B102" s="38"/>
-      <c r="C102" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D102" s="38"/>
-      <c r="E102" s="40"/>
-      <c r="F102" s="40"/>
-      <c r="G102" s="41"/>
-      <c r="H102" s="41"/>
-      <c r="I102" s="41">
-        <f t="shared" ref="I102:I112" si="4">H102-G102</f>
-        <v>0</v>
-      </c>
-      <c r="J102" s="45"/>
-      <c r="K102" s="43"/>
-    </row>
-    <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A103" s="37"/>
-      <c r="B103" s="38"/>
-      <c r="C103" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D103" s="38"/>
-      <c r="E103" s="40"/>
-      <c r="F103" s="40"/>
-      <c r="G103" s="41"/>
-      <c r="H103" s="41"/>
-      <c r="I103" s="41">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="J103" s="45"/>
-      <c r="K103" s="43"/>
+      <c r="C103" s="55"/>
+      <c r="D103" s="55"/>
+      <c r="E103" s="55"/>
+      <c r="F103" s="55"/>
+      <c r="G103" s="55"/>
+      <c r="H103" s="55"/>
+      <c r="I103" s="55"/>
+      <c r="J103" s="55"/>
+      <c r="K103" s="56"/>
     </row>
     <row r="104" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A104" s="37"/>
@@ -4668,7 +4729,7 @@
       <c r="G104" s="41"/>
       <c r="H104" s="41"/>
       <c r="I104" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I104:I114" si="4">H104-G104</f>
         <v>0</v>
       </c>
       <c r="J104" s="45"/>
@@ -4801,113 +4862,113 @@
       <c r="K111" s="43"/>
     </row>
     <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A112" s="13"/>
-      <c r="B112" s="15"/>
-      <c r="C112" s="15"/>
-      <c r="D112" s="15"/>
-      <c r="E112" s="15" t="s">
+      <c r="A112" s="37"/>
+      <c r="B112" s="38"/>
+      <c r="C112" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D112" s="38"/>
+      <c r="E112" s="40"/>
+      <c r="F112" s="40"/>
+      <c r="G112" s="41"/>
+      <c r="H112" s="41"/>
+      <c r="I112" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J112" s="45"/>
+      <c r="K112" s="43"/>
+    </row>
+    <row r="113" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A113" s="37"/>
+      <c r="B113" s="38"/>
+      <c r="C113" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D113" s="38"/>
+      <c r="E113" s="40"/>
+      <c r="F113" s="40"/>
+      <c r="G113" s="41"/>
+      <c r="H113" s="41"/>
+      <c r="I113" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J113" s="45"/>
+      <c r="K113" s="43"/>
+    </row>
+    <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A114" s="13"/>
+      <c r="B114" s="15"/>
+      <c r="C114" s="15"/>
+      <c r="D114" s="15"/>
+      <c r="E114" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F112" s="15"/>
-      <c r="G112" s="18">
-        <f t="shared" ref="G112:H112" si="5">SUM(G102:G111)</f>
-        <v>0</v>
-      </c>
-      <c r="H112" s="18">
+      <c r="F114" s="15"/>
+      <c r="G114" s="18">
+        <f t="shared" ref="G114:H114" si="5">SUM(G104:G113)</f>
+        <v>0</v>
+      </c>
+      <c r="H114" s="18">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I112" s="18">
+      <c r="I114" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J112" s="19"/>
-      <c r="K112" s="46"/>
-    </row>
-    <row r="113" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="73" t="s">
+      <c r="J114" s="19"/>
+      <c r="K114" s="46"/>
+    </row>
+    <row r="115" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B113" s="62"/>
-      <c r="C113" s="62"/>
-      <c r="D113" s="62"/>
-      <c r="E113" s="62"/>
-      <c r="F113" s="62"/>
-      <c r="G113" s="62"/>
-      <c r="H113" s="62"/>
-      <c r="I113" s="62"/>
-      <c r="J113" s="62"/>
-      <c r="K113" s="63"/>
-    </row>
-    <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A114" s="25" t="s">
+      <c r="B115" s="55"/>
+      <c r="C115" s="55"/>
+      <c r="D115" s="55"/>
+      <c r="E115" s="55"/>
+      <c r="F115" s="55"/>
+      <c r="G115" s="55"/>
+      <c r="H115" s="55"/>
+      <c r="I115" s="55"/>
+      <c r="J115" s="55"/>
+      <c r="K115" s="56"/>
+    </row>
+    <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A116" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B114" s="74" t="s">
+      <c r="B116" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C114" s="62"/>
-      <c r="D114" s="62"/>
-      <c r="E114" s="62"/>
-      <c r="F114" s="62"/>
-      <c r="G114" s="62"/>
-      <c r="H114" s="62"/>
-      <c r="I114" s="62"/>
-      <c r="J114" s="62"/>
-      <c r="K114" s="63"/>
-    </row>
-    <row r="115" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="26" t="s">
+      <c r="C116" s="55"/>
+      <c r="D116" s="55"/>
+      <c r="E116" s="55"/>
+      <c r="F116" s="55"/>
+      <c r="G116" s="55"/>
+      <c r="H116" s="55"/>
+      <c r="I116" s="55"/>
+      <c r="J116" s="55"/>
+      <c r="K116" s="56"/>
+    </row>
+    <row r="117" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B115" s="74" t="s">
+      <c r="B117" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C115" s="62"/>
-      <c r="D115" s="62"/>
-      <c r="E115" s="62"/>
-      <c r="F115" s="62"/>
-      <c r="G115" s="62"/>
-      <c r="H115" s="62"/>
-      <c r="I115" s="62"/>
-      <c r="J115" s="62"/>
-      <c r="K115" s="63"/>
-    </row>
-    <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A116" s="37"/>
-      <c r="B116" s="38"/>
-      <c r="C116" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D116" s="38"/>
-      <c r="E116" s="40"/>
-      <c r="F116" s="40"/>
-      <c r="G116" s="41"/>
-      <c r="H116" s="41"/>
-      <c r="I116" s="41">
-        <f t="shared" ref="I116:I126" si="6">H116-G116</f>
-        <v>0</v>
-      </c>
-      <c r="J116" s="45"/>
-      <c r="K116" s="43"/>
-    </row>
-    <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A117" s="37"/>
-      <c r="B117" s="38"/>
-      <c r="C117" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D117" s="38"/>
-      <c r="E117" s="40"/>
-      <c r="F117" s="40"/>
-      <c r="G117" s="41"/>
-      <c r="H117" s="41"/>
-      <c r="I117" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J117" s="45"/>
-      <c r="K117" s="43"/>
+      <c r="C117" s="55"/>
+      <c r="D117" s="55"/>
+      <c r="E117" s="55"/>
+      <c r="F117" s="55"/>
+      <c r="G117" s="55"/>
+      <c r="H117" s="55"/>
+      <c r="I117" s="55"/>
+      <c r="J117" s="55"/>
+      <c r="K117" s="56"/>
     </row>
     <row r="118" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A118" s="37"/>
@@ -4921,7 +4982,7 @@
       <c r="G118" s="41"/>
       <c r="H118" s="41"/>
       <c r="I118" s="41">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="I118:I128" si="6">H118-G118</f>
         <v>0</v>
       </c>
       <c r="J118" s="45"/>
@@ -5054,113 +5115,113 @@
       <c r="K125" s="43"/>
     </row>
     <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A126" s="13"/>
-      <c r="B126" s="15"/>
-      <c r="C126" s="15"/>
-      <c r="D126" s="15"/>
-      <c r="E126" s="15" t="s">
+      <c r="A126" s="37"/>
+      <c r="B126" s="38"/>
+      <c r="C126" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D126" s="38"/>
+      <c r="E126" s="40"/>
+      <c r="F126" s="40"/>
+      <c r="G126" s="41"/>
+      <c r="H126" s="41"/>
+      <c r="I126" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J126" s="45"/>
+      <c r="K126" s="43"/>
+    </row>
+    <row r="127" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A127" s="37"/>
+      <c r="B127" s="38"/>
+      <c r="C127" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D127" s="38"/>
+      <c r="E127" s="40"/>
+      <c r="F127" s="40"/>
+      <c r="G127" s="41"/>
+      <c r="H127" s="41"/>
+      <c r="I127" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J127" s="45"/>
+      <c r="K127" s="43"/>
+    </row>
+    <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A128" s="13"/>
+      <c r="B128" s="15"/>
+      <c r="C128" s="15"/>
+      <c r="D128" s="15"/>
+      <c r="E128" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F126" s="15"/>
-      <c r="G126" s="18">
-        <f t="shared" ref="G126:H126" si="7">SUM(G116:G125)</f>
-        <v>0</v>
-      </c>
-      <c r="H126" s="18">
+      <c r="F128" s="15"/>
+      <c r="G128" s="18">
+        <f t="shared" ref="G128:H128" si="7">SUM(G118:G127)</f>
+        <v>0</v>
+      </c>
+      <c r="H128" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I126" s="18">
+      <c r="I128" s="18">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J126" s="19"/>
-      <c r="K126" s="46"/>
-    </row>
-    <row r="127" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="75" t="s">
+      <c r="J128" s="19"/>
+      <c r="K128" s="46"/>
+    </row>
+    <row r="129" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B127" s="62"/>
-      <c r="C127" s="62"/>
-      <c r="D127" s="62"/>
-      <c r="E127" s="62"/>
-      <c r="F127" s="62"/>
-      <c r="G127" s="62"/>
-      <c r="H127" s="62"/>
-      <c r="I127" s="62"/>
-      <c r="J127" s="62"/>
-      <c r="K127" s="63"/>
-    </row>
-    <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A128" s="27" t="s">
+      <c r="B129" s="55"/>
+      <c r="C129" s="55"/>
+      <c r="D129" s="55"/>
+      <c r="E129" s="55"/>
+      <c r="F129" s="55"/>
+      <c r="G129" s="55"/>
+      <c r="H129" s="55"/>
+      <c r="I129" s="55"/>
+      <c r="J129" s="55"/>
+      <c r="K129" s="56"/>
+    </row>
+    <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A130" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B128" s="71" t="s">
+      <c r="B130" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C128" s="62"/>
-      <c r="D128" s="62"/>
-      <c r="E128" s="62"/>
-      <c r="F128" s="62"/>
-      <c r="G128" s="62"/>
-      <c r="H128" s="62"/>
-      <c r="I128" s="62"/>
-      <c r="J128" s="62"/>
-      <c r="K128" s="63"/>
-    </row>
-    <row r="129" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="28" t="s">
+      <c r="C130" s="55"/>
+      <c r="D130" s="55"/>
+      <c r="E130" s="55"/>
+      <c r="F130" s="55"/>
+      <c r="G130" s="55"/>
+      <c r="H130" s="55"/>
+      <c r="I130" s="55"/>
+      <c r="J130" s="55"/>
+      <c r="K130" s="56"/>
+    </row>
+    <row r="131" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B129" s="71" t="s">
+      <c r="B131" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C129" s="62"/>
-      <c r="D129" s="62"/>
-      <c r="E129" s="62"/>
-      <c r="F129" s="62"/>
-      <c r="G129" s="62"/>
-      <c r="H129" s="62"/>
-      <c r="I129" s="62"/>
-      <c r="J129" s="62"/>
-      <c r="K129" s="63"/>
-    </row>
-    <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A130" s="37"/>
-      <c r="B130" s="38"/>
-      <c r="C130" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D130" s="38"/>
-      <c r="E130" s="40"/>
-      <c r="F130" s="40"/>
-      <c r="G130" s="41"/>
-      <c r="H130" s="41"/>
-      <c r="I130" s="41">
-        <f t="shared" ref="I130:I140" si="8">H130-G130</f>
-        <v>0</v>
-      </c>
-      <c r="J130" s="45"/>
-      <c r="K130" s="43"/>
-    </row>
-    <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A131" s="37"/>
-      <c r="B131" s="38"/>
-      <c r="C131" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D131" s="38"/>
-      <c r="E131" s="40"/>
-      <c r="F131" s="40"/>
-      <c r="G131" s="41"/>
-      <c r="H131" s="41"/>
-      <c r="I131" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J131" s="45"/>
-      <c r="K131" s="43"/>
+      <c r="C131" s="55"/>
+      <c r="D131" s="55"/>
+      <c r="E131" s="55"/>
+      <c r="F131" s="55"/>
+      <c r="G131" s="55"/>
+      <c r="H131" s="55"/>
+      <c r="I131" s="55"/>
+      <c r="J131" s="55"/>
+      <c r="K131" s="56"/>
     </row>
     <row r="132" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A132" s="37"/>
@@ -5174,13 +5235,11 @@
       <c r="G132" s="41"/>
       <c r="H132" s="41"/>
       <c r="I132" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I132:I142" si="8">H132-G132</f>
         <v>0</v>
       </c>
       <c r="J132" s="45"/>
-      <c r="K132" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K132" s="43"/>
     </row>
     <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A133" s="37"/>
@@ -5216,7 +5275,9 @@
         <v>0</v>
       </c>
       <c r="J134" s="45"/>
-      <c r="K134" s="43"/>
+      <c r="K134" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A135" s="37"/>
@@ -5309,113 +5370,113 @@
       <c r="K139" s="43"/>
     </row>
     <row r="140" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A140" s="13"/>
-      <c r="B140" s="15"/>
-      <c r="C140" s="15"/>
-      <c r="D140" s="15"/>
-      <c r="E140" s="15" t="s">
+      <c r="A140" s="37"/>
+      <c r="B140" s="38"/>
+      <c r="C140" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D140" s="38"/>
+      <c r="E140" s="40"/>
+      <c r="F140" s="40"/>
+      <c r="G140" s="41"/>
+      <c r="H140" s="41"/>
+      <c r="I140" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J140" s="45"/>
+      <c r="K140" s="43"/>
+    </row>
+    <row r="141" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A141" s="37"/>
+      <c r="B141" s="38"/>
+      <c r="C141" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D141" s="38"/>
+      <c r="E141" s="40"/>
+      <c r="F141" s="40"/>
+      <c r="G141" s="41"/>
+      <c r="H141" s="41"/>
+      <c r="I141" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J141" s="45"/>
+      <c r="K141" s="43"/>
+    </row>
+    <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A142" s="13"/>
+      <c r="B142" s="15"/>
+      <c r="C142" s="15"/>
+      <c r="D142" s="15"/>
+      <c r="E142" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F140" s="15"/>
-      <c r="G140" s="18">
-        <f t="shared" ref="G140:H140" si="9">SUM(G130:G139)</f>
-        <v>0</v>
-      </c>
-      <c r="H140" s="18">
+      <c r="F142" s="15"/>
+      <c r="G142" s="18">
+        <f t="shared" ref="G142:H142" si="9">SUM(G132:G141)</f>
+        <v>0</v>
+      </c>
+      <c r="H142" s="18">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="I140" s="18">
+      <c r="I142" s="18">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J140" s="19"/>
-      <c r="K140" s="46"/>
-    </row>
-    <row r="141" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="72" t="s">
+      <c r="J142" s="19"/>
+      <c r="K142" s="46"/>
+    </row>
+    <row r="143" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B141" s="62"/>
-      <c r="C141" s="62"/>
-      <c r="D141" s="62"/>
-      <c r="E141" s="62"/>
-      <c r="F141" s="62"/>
-      <c r="G141" s="62"/>
-      <c r="H141" s="62"/>
-      <c r="I141" s="62"/>
-      <c r="J141" s="62"/>
-      <c r="K141" s="63"/>
-    </row>
-    <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A142" s="29" t="s">
+      <c r="B143" s="55"/>
+      <c r="C143" s="55"/>
+      <c r="D143" s="55"/>
+      <c r="E143" s="55"/>
+      <c r="F143" s="55"/>
+      <c r="G143" s="55"/>
+      <c r="H143" s="55"/>
+      <c r="I143" s="55"/>
+      <c r="J143" s="55"/>
+      <c r="K143" s="56"/>
+    </row>
+    <row r="144" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A144" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B142" s="69" t="s">
+      <c r="B144" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C142" s="62"/>
-      <c r="D142" s="62"/>
-      <c r="E142" s="62"/>
-      <c r="F142" s="62"/>
-      <c r="G142" s="62"/>
-      <c r="H142" s="62"/>
-      <c r="I142" s="62"/>
-      <c r="J142" s="62"/>
-      <c r="K142" s="63"/>
-    </row>
-    <row r="143" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="30" t="s">
+      <c r="C144" s="55"/>
+      <c r="D144" s="55"/>
+      <c r="E144" s="55"/>
+      <c r="F144" s="55"/>
+      <c r="G144" s="55"/>
+      <c r="H144" s="55"/>
+      <c r="I144" s="55"/>
+      <c r="J144" s="55"/>
+      <c r="K144" s="56"/>
+    </row>
+    <row r="145" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B143" s="69" t="s">
+      <c r="B145" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C143" s="62"/>
-      <c r="D143" s="62"/>
-      <c r="E143" s="62"/>
-      <c r="F143" s="62"/>
-      <c r="G143" s="62"/>
-      <c r="H143" s="62"/>
-      <c r="I143" s="62"/>
-      <c r="J143" s="62"/>
-      <c r="K143" s="63"/>
-    </row>
-    <row r="144" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A144" s="37"/>
-      <c r="B144" s="38"/>
-      <c r="C144" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D144" s="38"/>
-      <c r="E144" s="40"/>
-      <c r="F144" s="40"/>
-      <c r="G144" s="41"/>
-      <c r="H144" s="41"/>
-      <c r="I144" s="41">
-        <f t="shared" ref="I144:I154" si="10">H144-G144</f>
-        <v>0</v>
-      </c>
-      <c r="J144" s="45"/>
-      <c r="K144" s="43"/>
-    </row>
-    <row r="145" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A145" s="37"/>
-      <c r="B145" s="38"/>
-      <c r="C145" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D145" s="38"/>
-      <c r="E145" s="40"/>
-      <c r="F145" s="40"/>
-      <c r="G145" s="41"/>
-      <c r="H145" s="41"/>
-      <c r="I145" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J145" s="45"/>
-      <c r="K145" s="43"/>
+      <c r="C145" s="55"/>
+      <c r="D145" s="55"/>
+      <c r="E145" s="55"/>
+      <c r="F145" s="55"/>
+      <c r="G145" s="55"/>
+      <c r="H145" s="55"/>
+      <c r="I145" s="55"/>
+      <c r="J145" s="55"/>
+      <c r="K145" s="56"/>
     </row>
     <row r="146" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A146" s="37"/>
@@ -5429,7 +5490,7 @@
       <c r="G146" s="41"/>
       <c r="H146" s="41"/>
       <c r="I146" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I146:I156" si="10">H146-G146</f>
         <v>0</v>
       </c>
       <c r="J146" s="45"/>
@@ -5562,113 +5623,113 @@
       <c r="K153" s="43"/>
     </row>
     <row r="154" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A154" s="13"/>
-      <c r="B154" s="15"/>
-      <c r="C154" s="15"/>
-      <c r="D154" s="15"/>
-      <c r="E154" s="15" t="s">
+      <c r="A154" s="37"/>
+      <c r="B154" s="38"/>
+      <c r="C154" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D154" s="38"/>
+      <c r="E154" s="40"/>
+      <c r="F154" s="40"/>
+      <c r="G154" s="41"/>
+      <c r="H154" s="41"/>
+      <c r="I154" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J154" s="45"/>
+      <c r="K154" s="43"/>
+    </row>
+    <row r="155" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A155" s="37"/>
+      <c r="B155" s="38"/>
+      <c r="C155" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D155" s="38"/>
+      <c r="E155" s="40"/>
+      <c r="F155" s="40"/>
+      <c r="G155" s="41"/>
+      <c r="H155" s="41"/>
+      <c r="I155" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J155" s="45"/>
+      <c r="K155" s="43"/>
+    </row>
+    <row r="156" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A156" s="13"/>
+      <c r="B156" s="15"/>
+      <c r="C156" s="15"/>
+      <c r="D156" s="15"/>
+      <c r="E156" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F154" s="15"/>
-      <c r="G154" s="18">
-        <f t="shared" ref="G154:H154" si="11">SUM(G144:G153)</f>
-        <v>0</v>
-      </c>
-      <c r="H154" s="18">
+      <c r="F156" s="15"/>
+      <c r="G156" s="18">
+        <f t="shared" ref="G156:H156" si="11">SUM(G146:G155)</f>
+        <v>0</v>
+      </c>
+      <c r="H156" s="18">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="I154" s="18">
+      <c r="I156" s="18">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J154" s="19"/>
-      <c r="K154" s="46"/>
-    </row>
-    <row r="155" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="54" t="s">
+      <c r="J156" s="19"/>
+      <c r="K156" s="46"/>
+    </row>
+    <row r="157" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B155" s="55"/>
-      <c r="C155" s="55"/>
-      <c r="D155" s="55"/>
-      <c r="E155" s="55"/>
-      <c r="F155" s="55"/>
-      <c r="G155" s="55"/>
-      <c r="H155" s="55"/>
-      <c r="I155" s="55"/>
-      <c r="J155" s="55"/>
-      <c r="K155" s="56"/>
-    </row>
-    <row r="156" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A156" s="32" t="s">
+      <c r="B157" s="63"/>
+      <c r="C157" s="63"/>
+      <c r="D157" s="63"/>
+      <c r="E157" s="63"/>
+      <c r="F157" s="63"/>
+      <c r="G157" s="63"/>
+      <c r="H157" s="63"/>
+      <c r="I157" s="63"/>
+      <c r="J157" s="63"/>
+      <c r="K157" s="64"/>
+    </row>
+    <row r="158" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A158" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B156" s="57" t="s">
+      <c r="B158" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C156" s="55"/>
-      <c r="D156" s="55"/>
-      <c r="E156" s="55"/>
-      <c r="F156" s="55"/>
-      <c r="G156" s="55"/>
-      <c r="H156" s="55"/>
-      <c r="I156" s="55"/>
-      <c r="J156" s="55"/>
-      <c r="K156" s="56"/>
-    </row>
-    <row r="157" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="33" t="s">
+      <c r="C158" s="63"/>
+      <c r="D158" s="63"/>
+      <c r="E158" s="63"/>
+      <c r="F158" s="63"/>
+      <c r="G158" s="63"/>
+      <c r="H158" s="63"/>
+      <c r="I158" s="63"/>
+      <c r="J158" s="63"/>
+      <c r="K158" s="64"/>
+    </row>
+    <row r="159" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B157" s="57" t="s">
+      <c r="B159" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C157" s="55"/>
-      <c r="D157" s="55"/>
-      <c r="E157" s="55"/>
-      <c r="F157" s="55"/>
-      <c r="G157" s="55"/>
-      <c r="H157" s="55"/>
-      <c r="I157" s="55"/>
-      <c r="J157" s="55"/>
-      <c r="K157" s="56"/>
-    </row>
-    <row r="158" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A158" s="37"/>
-      <c r="B158" s="38"/>
-      <c r="C158" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D158" s="38"/>
-      <c r="E158" s="40"/>
-      <c r="F158" s="40"/>
-      <c r="G158" s="41"/>
-      <c r="H158" s="41"/>
-      <c r="I158" s="41">
-        <f t="shared" ref="I158:I168" si="12">H158-G158</f>
-        <v>0</v>
-      </c>
-      <c r="J158" s="45"/>
-      <c r="K158" s="43"/>
-    </row>
-    <row r="159" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A159" s="37"/>
-      <c r="B159" s="38"/>
-      <c r="C159" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D159" s="38"/>
-      <c r="E159" s="40"/>
-      <c r="F159" s="40"/>
-      <c r="G159" s="41"/>
-      <c r="H159" s="41"/>
-      <c r="I159" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J159" s="45"/>
-      <c r="K159" s="43"/>
+      <c r="C159" s="63"/>
+      <c r="D159" s="63"/>
+      <c r="E159" s="63"/>
+      <c r="F159" s="63"/>
+      <c r="G159" s="63"/>
+      <c r="H159" s="63"/>
+      <c r="I159" s="63"/>
+      <c r="J159" s="63"/>
+      <c r="K159" s="64"/>
     </row>
     <row r="160" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A160" s="37"/>
@@ -5682,7 +5743,7 @@
       <c r="G160" s="41"/>
       <c r="H160" s="41"/>
       <c r="I160" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="I160:I170" si="12">H160-G160</f>
         <v>0</v>
       </c>
       <c r="J160" s="45"/>
@@ -5815,35 +5876,71 @@
       <c r="K167" s="43"/>
     </row>
     <row r="168" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A168" s="48"/>
-      <c r="B168" s="49"/>
-      <c r="C168" s="49"/>
-      <c r="D168" s="49"/>
-      <c r="E168" s="49" t="s">
+      <c r="A168" s="37"/>
+      <c r="B168" s="38"/>
+      <c r="C168" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D168" s="38"/>
+      <c r="E168" s="40"/>
+      <c r="F168" s="40"/>
+      <c r="G168" s="41"/>
+      <c r="H168" s="41"/>
+      <c r="I168" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J168" s="45"/>
+      <c r="K168" s="43"/>
+    </row>
+    <row r="169" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A169" s="37"/>
+      <c r="B169" s="38"/>
+      <c r="C169" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D169" s="38"/>
+      <c r="E169" s="40"/>
+      <c r="F169" s="40"/>
+      <c r="G169" s="41"/>
+      <c r="H169" s="41"/>
+      <c r="I169" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J169" s="45"/>
+      <c r="K169" s="43"/>
+    </row>
+    <row r="170" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A170" s="48"/>
+      <c r="B170" s="49"/>
+      <c r="C170" s="49"/>
+      <c r="D170" s="49"/>
+      <c r="E170" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F168" s="49"/>
-      <c r="G168" s="50">
-        <f t="shared" ref="G168:H168" si="13">SUM(G158:G167)</f>
-        <v>0</v>
-      </c>
-      <c r="H168" s="50">
+      <c r="F170" s="49"/>
+      <c r="G170" s="50">
+        <f t="shared" ref="G170:H170" si="13">SUM(G160:G169)</f>
+        <v>0</v>
+      </c>
+      <c r="H170" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="I168" s="50">
+      <c r="I170" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J168" s="51"/>
-      <c r="K168" s="52"/>
+      <c r="J170" s="51"/>
+      <c r="K170" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{47F12E79-EA31-4F9C-A76A-23D0ED283334}">
+      <autoFilter ref="A1:K15" xr:uid="{148386E4-773C-4965-B2FA-BF62B2CF7AA1}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5854,17 +5951,9 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B128:K128"/>
-    <mergeCell ref="B129:K129"/>
-    <mergeCell ref="A141:K141"/>
-    <mergeCell ref="B101:K101"/>
-    <mergeCell ref="A113:K113"/>
-    <mergeCell ref="B114:K114"/>
-    <mergeCell ref="B115:K115"/>
-    <mergeCell ref="A127:K127"/>
-    <mergeCell ref="A155:K155"/>
-    <mergeCell ref="B156:K156"/>
-    <mergeCell ref="B157:K157"/>
+    <mergeCell ref="A157:K157"/>
+    <mergeCell ref="B158:K158"/>
+    <mergeCell ref="B159:K159"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -5874,12 +5963,20 @@
     <mergeCell ref="A83:K83"/>
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
-    <mergeCell ref="A99:K99"/>
-    <mergeCell ref="B142:K142"/>
-    <mergeCell ref="B143:K143"/>
-    <mergeCell ref="B100:K100"/>
+    <mergeCell ref="A101:K101"/>
+    <mergeCell ref="B144:K144"/>
+    <mergeCell ref="B145:K145"/>
+    <mergeCell ref="B102:K102"/>
+    <mergeCell ref="B130:K130"/>
+    <mergeCell ref="B131:K131"/>
+    <mergeCell ref="A143:K143"/>
+    <mergeCell ref="B103:K103"/>
+    <mergeCell ref="A115:K115"/>
+    <mergeCell ref="B116:K116"/>
+    <mergeCell ref="B117:K117"/>
+    <mergeCell ref="A129:K129"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B97 B102:B111 B116:B125 B130:B139 B144:B153">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B99 B104:B113 B118:B127 B132:B141 B146:B155">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5896,7 +5993,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B98 B100:B112 B114:B126 B128:B140 B142:B154 B156:B168">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B100 B102:B114 B116:B128 B130:B142 B144:B156 B158:B170">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5904,34 +6001,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B158:B167">
+  <conditionalFormatting sqref="B160:B169">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B158))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B160))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B158))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B160))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B158))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B160))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B158))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B160))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B158))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B160))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G98 G102:G112 G116:G126 G130:G140 G144:G154 G158:G168">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G100 G104:G114 G118:G128 G132:G142 G146:G156 G160:G170">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H168">
+  <conditionalFormatting sqref="H1:H170">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I98 I102:I112 I116:I126 I130:I140 I144:I154 I158:I168">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I100 I104:I114 I118:I128 I132:I142 I146:I156 I160:I170">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -5940,7 +6037,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F158:F167 F144:F153 F86:F97 F102:F111 F116:F125 F130:F139 F5:F45 F81 F50:F80" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F160:F169 F146:F155 F86:F99 F104:F113 F118:F127 F132:F141 F5:F45 F50:F81" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5956,13 +6053,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E97 E102:E111 E116:E125 E130:E139 E144:E153 E158:E167 E81 E50:E80</xm:sqref>
+          <xm:sqref>E5:E45 E86:E99 E104:E113 E118:E127 E132:E141 E146:E155 E160:E169 E50:E81</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B97 B102:B111 B116:B125 B130:B139 B144:B153 B158:B167 B81 B50:B80</xm:sqref>
+          <xm:sqref>B5:B45 B86:B99 B104:B113 B118:B127 B132:B141 B146:B155 B160:B169 B50:B81</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7603,6 +7700,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -7837,27 +7954,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7874,23 +7990,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W3 Datalab 1 Work III (can't concentrate)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E6DB97-A59D-4CE8-8310-0862A4DE3F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC6F2F09-EB6D-44C5-AF0E-444CC587EDB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$155</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$156</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="175">
   <si>
     <t>Date</t>
   </si>
@@ -618,6 +618,15 @@
   </si>
   <si>
     <t>Implement Decision Tree Regression</t>
+  </si>
+  <si>
+    <t>Follow the lecture</t>
+  </si>
+  <si>
+    <t>ILO 6.2</t>
+  </si>
+  <si>
+    <t>From 9:30 until end -2 hours</t>
   </si>
 </sst>
 </file>
@@ -1103,26 +1112,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1139,6 +1128,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1156,6 +1147,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1628,7 +1637,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K170"/>
+  <dimension ref="A1:K171"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1680,53 +1689,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3065,53 +3074,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="62"/>
+      <c r="K49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4164,53 +4173,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72" t="s">
+      <c r="A83" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="55"/>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="55"/>
-      <c r="I83" s="55"/>
-      <c r="J83" s="55"/>
-      <c r="K83" s="56"/>
+      <c r="B83" s="62"/>
+      <c r="C83" s="62"/>
+      <c r="D83" s="62"/>
+      <c r="E83" s="62"/>
+      <c r="F83" s="62"/>
+      <c r="G83" s="62"/>
+      <c r="H83" s="62"/>
+      <c r="I83" s="62"/>
+      <c r="J83" s="62"/>
+      <c r="K83" s="63"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="73" t="s">
+      <c r="B84" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="55"/>
-      <c r="D84" s="55"/>
-      <c r="E84" s="55"/>
-      <c r="F84" s="55"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="55"/>
-      <c r="I84" s="55"/>
-      <c r="J84" s="55"/>
-      <c r="K84" s="56"/>
+      <c r="C84" s="62"/>
+      <c r="D84" s="62"/>
+      <c r="E84" s="62"/>
+      <c r="F84" s="62"/>
+      <c r="G84" s="62"/>
+      <c r="H84" s="62"/>
+      <c r="I84" s="62"/>
+      <c r="J84" s="62"/>
+      <c r="K84" s="63"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="73" t="s">
+      <c r="B85" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="55"/>
-      <c r="D85" s="55"/>
-      <c r="E85" s="55"/>
-      <c r="F85" s="55"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="55"/>
-      <c r="I85" s="55"/>
-      <c r="J85" s="55"/>
-      <c r="K85" s="56"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="62"/>
+      <c r="G85" s="62"/>
+      <c r="H85" s="62"/>
+      <c r="I85" s="62"/>
+      <c r="J85" s="62"/>
+      <c r="K85" s="63"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -4238,7 +4247,7 @@
         <v>0.5</v>
       </c>
       <c r="I86" s="41">
-        <f t="shared" ref="I86:I100" si="2">H86-G86</f>
+        <f t="shared" ref="I86:I101" si="2">H86-G86</f>
         <v>0</v>
       </c>
       <c r="J86" s="45"/>
@@ -4395,11 +4404,11 @@
         <v>4</v>
       </c>
       <c r="H91" s="41">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I91" s="41">
         <f t="shared" si="2"/>
-        <v>-1.5</v>
+        <v>-1</v>
       </c>
       <c r="J91" s="45"/>
       <c r="K91" s="43"/>
@@ -4594,7 +4603,9 @@
         <v>-4</v>
       </c>
       <c r="J97" s="45"/>
-      <c r="K97" s="43"/>
+      <c r="K97" s="43" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="98" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A98" s="37">
@@ -4607,133 +4618,145 @@
         <v>17</v>
       </c>
       <c r="D98" s="38" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E98" s="40" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="F98" s="40" t="s">
-        <v>108</v>
+        <v>173</v>
       </c>
       <c r="G98" s="41">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="H98" s="41"/>
       <c r="I98" s="41">
         <f t="shared" si="2"/>
-        <v>-2.5</v>
+        <v>-1</v>
       </c>
       <c r="J98" s="45"/>
       <c r="K98" s="43"/>
     </row>
     <row r="99" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A99" s="37"/>
-      <c r="B99" s="38"/>
+      <c r="A99" s="37">
+        <v>45629</v>
+      </c>
+      <c r="B99" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C99" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D99" s="38"/>
-      <c r="E99" s="40"/>
-      <c r="F99" s="40"/>
-      <c r="G99" s="41"/>
+      <c r="D99" s="38" t="s">
+        <v>171</v>
+      </c>
+      <c r="E99" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F99" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G99" s="41">
+        <v>2.5</v>
+      </c>
       <c r="H99" s="41"/>
       <c r="I99" s="41">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-2.5</v>
       </c>
       <c r="J99" s="45"/>
       <c r="K99" s="43"/>
     </row>
     <row r="100" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A100" s="13"/>
-      <c r="B100" s="15"/>
-      <c r="C100" s="15"/>
-      <c r="D100" s="15"/>
-      <c r="E100" s="15" t="s">
+      <c r="A100" s="37"/>
+      <c r="B100" s="38"/>
+      <c r="C100" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D100" s="38"/>
+      <c r="E100" s="40"/>
+      <c r="F100" s="40"/>
+      <c r="G100" s="41"/>
+      <c r="H100" s="41"/>
+      <c r="I100" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J100" s="45"/>
+      <c r="K100" s="43"/>
+    </row>
+    <row r="101" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A101" s="13"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="15"/>
+      <c r="D101" s="15"/>
+      <c r="E101" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F100" s="15"/>
-      <c r="G100" s="18">
-        <f t="shared" ref="G100:H100" si="3">SUM(G86:G99)</f>
-        <v>16.5</v>
-      </c>
-      <c r="H100" s="18">
+      <c r="F101" s="15"/>
+      <c r="G101" s="18">
+        <f t="shared" ref="G101:H101" si="3">SUM(G86:G100)</f>
+        <v>17.5</v>
+      </c>
+      <c r="H101" s="18">
         <f t="shared" si="3"/>
-        <v>8.25</v>
-      </c>
-      <c r="I100" s="18">
+        <v>8.75</v>
+      </c>
+      <c r="I101" s="18">
         <f t="shared" si="2"/>
-        <v>-8.25</v>
-      </c>
-      <c r="J100" s="19"/>
-      <c r="K100" s="46"/>
-    </row>
-    <row r="101" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="74" t="s">
+        <v>-8.75</v>
+      </c>
+      <c r="J101" s="19"/>
+      <c r="K101" s="46"/>
+    </row>
+    <row r="102" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B101" s="55"/>
-      <c r="C101" s="55"/>
-      <c r="D101" s="55"/>
-      <c r="E101" s="55"/>
-      <c r="F101" s="55"/>
-      <c r="G101" s="55"/>
-      <c r="H101" s="55"/>
-      <c r="I101" s="55"/>
-      <c r="J101" s="55"/>
-      <c r="K101" s="56"/>
-    </row>
-    <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A102" s="23" t="s">
+      <c r="B102" s="62"/>
+      <c r="C102" s="62"/>
+      <c r="D102" s="62"/>
+      <c r="E102" s="62"/>
+      <c r="F102" s="62"/>
+      <c r="G102" s="62"/>
+      <c r="H102" s="62"/>
+      <c r="I102" s="62"/>
+      <c r="J102" s="62"/>
+      <c r="K102" s="63"/>
+    </row>
+    <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A103" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B102" s="58" t="s">
+      <c r="B103" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C102" s="55"/>
-      <c r="D102" s="55"/>
-      <c r="E102" s="55"/>
-      <c r="F102" s="55"/>
-      <c r="G102" s="55"/>
-      <c r="H102" s="55"/>
-      <c r="I102" s="55"/>
-      <c r="J102" s="55"/>
-      <c r="K102" s="56"/>
-    </row>
-    <row r="103" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="24" t="s">
+      <c r="C103" s="62"/>
+      <c r="D103" s="62"/>
+      <c r="E103" s="62"/>
+      <c r="F103" s="62"/>
+      <c r="G103" s="62"/>
+      <c r="H103" s="62"/>
+      <c r="I103" s="62"/>
+      <c r="J103" s="62"/>
+      <c r="K103" s="63"/>
+    </row>
+    <row r="104" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B103" s="58" t="s">
+      <c r="B104" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C103" s="55"/>
-      <c r="D103" s="55"/>
-      <c r="E103" s="55"/>
-      <c r="F103" s="55"/>
-      <c r="G103" s="55"/>
-      <c r="H103" s="55"/>
-      <c r="I103" s="55"/>
-      <c r="J103" s="55"/>
-      <c r="K103" s="56"/>
-    </row>
-    <row r="104" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A104" s="37"/>
-      <c r="B104" s="38"/>
-      <c r="C104" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D104" s="38"/>
-      <c r="E104" s="40"/>
-      <c r="F104" s="40"/>
-      <c r="G104" s="41"/>
-      <c r="H104" s="41"/>
-      <c r="I104" s="41">
-        <f t="shared" ref="I104:I114" si="4">H104-G104</f>
-        <v>0</v>
-      </c>
-      <c r="J104" s="45"/>
-      <c r="K104" s="43"/>
+      <c r="C104" s="62"/>
+      <c r="D104" s="62"/>
+      <c r="E104" s="62"/>
+      <c r="F104" s="62"/>
+      <c r="G104" s="62"/>
+      <c r="H104" s="62"/>
+      <c r="I104" s="62"/>
+      <c r="J104" s="62"/>
+      <c r="K104" s="63"/>
     </row>
     <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A105" s="37"/>
@@ -4747,7 +4770,7 @@
       <c r="G105" s="41"/>
       <c r="H105" s="41"/>
       <c r="I105" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I105:I115" si="4">H105-G105</f>
         <v>0</v>
       </c>
       <c r="J105" s="45"/>
@@ -4898,95 +4921,95 @@
       <c r="K113" s="43"/>
     </row>
     <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A114" s="13"/>
-      <c r="B114" s="15"/>
-      <c r="C114" s="15"/>
-      <c r="D114" s="15"/>
-      <c r="E114" s="15" t="s">
+      <c r="A114" s="37"/>
+      <c r="B114" s="38"/>
+      <c r="C114" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D114" s="38"/>
+      <c r="E114" s="40"/>
+      <c r="F114" s="40"/>
+      <c r="G114" s="41"/>
+      <c r="H114" s="41"/>
+      <c r="I114" s="41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J114" s="45"/>
+      <c r="K114" s="43"/>
+    </row>
+    <row r="115" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A115" s="13"/>
+      <c r="B115" s="15"/>
+      <c r="C115" s="15"/>
+      <c r="D115" s="15"/>
+      <c r="E115" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F114" s="15"/>
-      <c r="G114" s="18">
-        <f t="shared" ref="G114:H114" si="5">SUM(G104:G113)</f>
-        <v>0</v>
-      </c>
-      <c r="H114" s="18">
+      <c r="F115" s="15"/>
+      <c r="G115" s="18">
+        <f t="shared" ref="G115:H115" si="5">SUM(G105:G114)</f>
+        <v>0</v>
+      </c>
+      <c r="H115" s="18">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I114" s="18">
+      <c r="I115" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J114" s="19"/>
-      <c r="K114" s="46"/>
-    </row>
-    <row r="115" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="59" t="s">
+      <c r="J115" s="19"/>
+      <c r="K115" s="46"/>
+    </row>
+    <row r="116" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B115" s="55"/>
-      <c r="C115" s="55"/>
-      <c r="D115" s="55"/>
-      <c r="E115" s="55"/>
-      <c r="F115" s="55"/>
-      <c r="G115" s="55"/>
-      <c r="H115" s="55"/>
-      <c r="I115" s="55"/>
-      <c r="J115" s="55"/>
-      <c r="K115" s="56"/>
-    </row>
-    <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A116" s="25" t="s">
+      <c r="B116" s="62"/>
+      <c r="C116" s="62"/>
+      <c r="D116" s="62"/>
+      <c r="E116" s="62"/>
+      <c r="F116" s="62"/>
+      <c r="G116" s="62"/>
+      <c r="H116" s="62"/>
+      <c r="I116" s="62"/>
+      <c r="J116" s="62"/>
+      <c r="K116" s="63"/>
+    </row>
+    <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A117" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B116" s="60" t="s">
+      <c r="B117" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C116" s="55"/>
-      <c r="D116" s="55"/>
-      <c r="E116" s="55"/>
-      <c r="F116" s="55"/>
-      <c r="G116" s="55"/>
-      <c r="H116" s="55"/>
-      <c r="I116" s="55"/>
-      <c r="J116" s="55"/>
-      <c r="K116" s="56"/>
-    </row>
-    <row r="117" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="26" t="s">
+      <c r="C117" s="62"/>
+      <c r="D117" s="62"/>
+      <c r="E117" s="62"/>
+      <c r="F117" s="62"/>
+      <c r="G117" s="62"/>
+      <c r="H117" s="62"/>
+      <c r="I117" s="62"/>
+      <c r="J117" s="62"/>
+      <c r="K117" s="63"/>
+    </row>
+    <row r="118" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B117" s="60" t="s">
+      <c r="B118" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C117" s="55"/>
-      <c r="D117" s="55"/>
-      <c r="E117" s="55"/>
-      <c r="F117" s="55"/>
-      <c r="G117" s="55"/>
-      <c r="H117" s="55"/>
-      <c r="I117" s="55"/>
-      <c r="J117" s="55"/>
-      <c r="K117" s="56"/>
-    </row>
-    <row r="118" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A118" s="37"/>
-      <c r="B118" s="38"/>
-      <c r="C118" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D118" s="38"/>
-      <c r="E118" s="40"/>
-      <c r="F118" s="40"/>
-      <c r="G118" s="41"/>
-      <c r="H118" s="41"/>
-      <c r="I118" s="41">
-        <f t="shared" ref="I118:I128" si="6">H118-G118</f>
-        <v>0</v>
-      </c>
-      <c r="J118" s="45"/>
-      <c r="K118" s="43"/>
+      <c r="C118" s="62"/>
+      <c r="D118" s="62"/>
+      <c r="E118" s="62"/>
+      <c r="F118" s="62"/>
+      <c r="G118" s="62"/>
+      <c r="H118" s="62"/>
+      <c r="I118" s="62"/>
+      <c r="J118" s="62"/>
+      <c r="K118" s="63"/>
     </row>
     <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A119" s="37"/>
@@ -5000,7 +5023,7 @@
       <c r="G119" s="41"/>
       <c r="H119" s="41"/>
       <c r="I119" s="41">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="I119:I129" si="6">H119-G119</f>
         <v>0</v>
       </c>
       <c r="J119" s="45"/>
@@ -5151,95 +5174,95 @@
       <c r="K127" s="43"/>
     </row>
     <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A128" s="13"/>
-      <c r="B128" s="15"/>
-      <c r="C128" s="15"/>
-      <c r="D128" s="15"/>
-      <c r="E128" s="15" t="s">
+      <c r="A128" s="37"/>
+      <c r="B128" s="38"/>
+      <c r="C128" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D128" s="38"/>
+      <c r="E128" s="40"/>
+      <c r="F128" s="40"/>
+      <c r="G128" s="41"/>
+      <c r="H128" s="41"/>
+      <c r="I128" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J128" s="45"/>
+      <c r="K128" s="43"/>
+    </row>
+    <row r="129" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A129" s="13"/>
+      <c r="B129" s="15"/>
+      <c r="C129" s="15"/>
+      <c r="D129" s="15"/>
+      <c r="E129" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F128" s="15"/>
-      <c r="G128" s="18">
-        <f t="shared" ref="G128:H128" si="7">SUM(G118:G127)</f>
-        <v>0</v>
-      </c>
-      <c r="H128" s="18">
+      <c r="F129" s="15"/>
+      <c r="G129" s="18">
+        <f t="shared" ref="G129:H129" si="7">SUM(G119:G128)</f>
+        <v>0</v>
+      </c>
+      <c r="H129" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I128" s="18">
+      <c r="I129" s="18">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J128" s="19"/>
-      <c r="K128" s="46"/>
-    </row>
-    <row r="129" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="61" t="s">
+      <c r="J129" s="19"/>
+      <c r="K129" s="46"/>
+    </row>
+    <row r="130" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B129" s="55"/>
-      <c r="C129" s="55"/>
-      <c r="D129" s="55"/>
-      <c r="E129" s="55"/>
-      <c r="F129" s="55"/>
-      <c r="G129" s="55"/>
-      <c r="H129" s="55"/>
-      <c r="I129" s="55"/>
-      <c r="J129" s="55"/>
-      <c r="K129" s="56"/>
-    </row>
-    <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A130" s="27" t="s">
+      <c r="B130" s="62"/>
+      <c r="C130" s="62"/>
+      <c r="D130" s="62"/>
+      <c r="E130" s="62"/>
+      <c r="F130" s="62"/>
+      <c r="G130" s="62"/>
+      <c r="H130" s="62"/>
+      <c r="I130" s="62"/>
+      <c r="J130" s="62"/>
+      <c r="K130" s="63"/>
+    </row>
+    <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A131" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B130" s="54" t="s">
+      <c r="B131" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C130" s="55"/>
-      <c r="D130" s="55"/>
-      <c r="E130" s="55"/>
-      <c r="F130" s="55"/>
-      <c r="G130" s="55"/>
-      <c r="H130" s="55"/>
-      <c r="I130" s="55"/>
-      <c r="J130" s="55"/>
-      <c r="K130" s="56"/>
-    </row>
-    <row r="131" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="28" t="s">
+      <c r="C131" s="62"/>
+      <c r="D131" s="62"/>
+      <c r="E131" s="62"/>
+      <c r="F131" s="62"/>
+      <c r="G131" s="62"/>
+      <c r="H131" s="62"/>
+      <c r="I131" s="62"/>
+      <c r="J131" s="62"/>
+      <c r="K131" s="63"/>
+    </row>
+    <row r="132" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B131" s="54" t="s">
+      <c r="B132" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C131" s="55"/>
-      <c r="D131" s="55"/>
-      <c r="E131" s="55"/>
-      <c r="F131" s="55"/>
-      <c r="G131" s="55"/>
-      <c r="H131" s="55"/>
-      <c r="I131" s="55"/>
-      <c r="J131" s="55"/>
-      <c r="K131" s="56"/>
-    </row>
-    <row r="132" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A132" s="37"/>
-      <c r="B132" s="38"/>
-      <c r="C132" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D132" s="38"/>
-      <c r="E132" s="40"/>
-      <c r="F132" s="40"/>
-      <c r="G132" s="41"/>
-      <c r="H132" s="41"/>
-      <c r="I132" s="41">
-        <f t="shared" ref="I132:I142" si="8">H132-G132</f>
-        <v>0</v>
-      </c>
-      <c r="J132" s="45"/>
-      <c r="K132" s="43"/>
+      <c r="C132" s="62"/>
+      <c r="D132" s="62"/>
+      <c r="E132" s="62"/>
+      <c r="F132" s="62"/>
+      <c r="G132" s="62"/>
+      <c r="H132" s="62"/>
+      <c r="I132" s="62"/>
+      <c r="J132" s="62"/>
+      <c r="K132" s="63"/>
     </row>
     <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A133" s="37"/>
@@ -5253,7 +5276,7 @@
       <c r="G133" s="41"/>
       <c r="H133" s="41"/>
       <c r="I133" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I133:I143" si="8">H133-G133</f>
         <v>0</v>
       </c>
       <c r="J133" s="45"/>
@@ -5275,9 +5298,7 @@
         <v>0</v>
       </c>
       <c r="J134" s="45"/>
-      <c r="K134" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K134" s="43"/>
     </row>
     <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A135" s="37"/>
@@ -5295,7 +5316,9 @@
         <v>0</v>
       </c>
       <c r="J135" s="45"/>
-      <c r="K135" s="43"/>
+      <c r="K135" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="136" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A136" s="37"/>
@@ -5406,95 +5429,95 @@
       <c r="K141" s="43"/>
     </row>
     <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A142" s="13"/>
-      <c r="B142" s="15"/>
-      <c r="C142" s="15"/>
-      <c r="D142" s="15"/>
-      <c r="E142" s="15" t="s">
+      <c r="A142" s="37"/>
+      <c r="B142" s="38"/>
+      <c r="C142" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D142" s="38"/>
+      <c r="E142" s="40"/>
+      <c r="F142" s="40"/>
+      <c r="G142" s="41"/>
+      <c r="H142" s="41"/>
+      <c r="I142" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J142" s="45"/>
+      <c r="K142" s="43"/>
+    </row>
+    <row r="143" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A143" s="13"/>
+      <c r="B143" s="15"/>
+      <c r="C143" s="15"/>
+      <c r="D143" s="15"/>
+      <c r="E143" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F142" s="15"/>
-      <c r="G142" s="18">
-        <f t="shared" ref="G142:H142" si="9">SUM(G132:G141)</f>
-        <v>0</v>
-      </c>
-      <c r="H142" s="18">
+      <c r="F143" s="15"/>
+      <c r="G143" s="18">
+        <f t="shared" ref="G143:H143" si="9">SUM(G133:G142)</f>
+        <v>0</v>
+      </c>
+      <c r="H143" s="18">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="I142" s="18">
+      <c r="I143" s="18">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J142" s="19"/>
-      <c r="K142" s="46"/>
-    </row>
-    <row r="143" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="57" t="s">
+      <c r="J143" s="19"/>
+      <c r="K143" s="46"/>
+    </row>
+    <row r="144" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="B143" s="55"/>
-      <c r="C143" s="55"/>
-      <c r="D143" s="55"/>
-      <c r="E143" s="55"/>
-      <c r="F143" s="55"/>
-      <c r="G143" s="55"/>
-      <c r="H143" s="55"/>
-      <c r="I143" s="55"/>
-      <c r="J143" s="55"/>
-      <c r="K143" s="56"/>
-    </row>
-    <row r="144" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A144" s="29" t="s">
+      <c r="B144" s="62"/>
+      <c r="C144" s="62"/>
+      <c r="D144" s="62"/>
+      <c r="E144" s="62"/>
+      <c r="F144" s="62"/>
+      <c r="G144" s="62"/>
+      <c r="H144" s="62"/>
+      <c r="I144" s="62"/>
+      <c r="J144" s="62"/>
+      <c r="K144" s="63"/>
+    </row>
+    <row r="145" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A145" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B144" s="75" t="s">
+      <c r="B145" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C144" s="55"/>
-      <c r="D144" s="55"/>
-      <c r="E144" s="55"/>
-      <c r="F144" s="55"/>
-      <c r="G144" s="55"/>
-      <c r="H144" s="55"/>
-      <c r="I144" s="55"/>
-      <c r="J144" s="55"/>
-      <c r="K144" s="56"/>
-    </row>
-    <row r="145" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A145" s="30" t="s">
+      <c r="C145" s="62"/>
+      <c r="D145" s="62"/>
+      <c r="E145" s="62"/>
+      <c r="F145" s="62"/>
+      <c r="G145" s="62"/>
+      <c r="H145" s="62"/>
+      <c r="I145" s="62"/>
+      <c r="J145" s="62"/>
+      <c r="K145" s="63"/>
+    </row>
+    <row r="146" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B145" s="75" t="s">
+      <c r="B146" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C145" s="55"/>
-      <c r="D145" s="55"/>
-      <c r="E145" s="55"/>
-      <c r="F145" s="55"/>
-      <c r="G145" s="55"/>
-      <c r="H145" s="55"/>
-      <c r="I145" s="55"/>
-      <c r="J145" s="55"/>
-      <c r="K145" s="56"/>
-    </row>
-    <row r="146" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A146" s="37"/>
-      <c r="B146" s="38"/>
-      <c r="C146" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D146" s="38"/>
-      <c r="E146" s="40"/>
-      <c r="F146" s="40"/>
-      <c r="G146" s="41"/>
-      <c r="H146" s="41"/>
-      <c r="I146" s="41">
-        <f t="shared" ref="I146:I156" si="10">H146-G146</f>
-        <v>0</v>
-      </c>
-      <c r="J146" s="45"/>
-      <c r="K146" s="43"/>
+      <c r="C146" s="62"/>
+      <c r="D146" s="62"/>
+      <c r="E146" s="62"/>
+      <c r="F146" s="62"/>
+      <c r="G146" s="62"/>
+      <c r="H146" s="62"/>
+      <c r="I146" s="62"/>
+      <c r="J146" s="62"/>
+      <c r="K146" s="63"/>
     </row>
     <row r="147" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A147" s="37"/>
@@ -5508,7 +5531,7 @@
       <c r="G147" s="41"/>
       <c r="H147" s="41"/>
       <c r="I147" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I147:I157" si="10">H147-G147</f>
         <v>0</v>
       </c>
       <c r="J147" s="45"/>
@@ -5659,95 +5682,95 @@
       <c r="K155" s="43"/>
     </row>
     <row r="156" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A156" s="13"/>
-      <c r="B156" s="15"/>
-      <c r="C156" s="15"/>
-      <c r="D156" s="15"/>
-      <c r="E156" s="15" t="s">
+      <c r="A156" s="37"/>
+      <c r="B156" s="38"/>
+      <c r="C156" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D156" s="38"/>
+      <c r="E156" s="40"/>
+      <c r="F156" s="40"/>
+      <c r="G156" s="41"/>
+      <c r="H156" s="41"/>
+      <c r="I156" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J156" s="45"/>
+      <c r="K156" s="43"/>
+    </row>
+    <row r="157" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A157" s="13"/>
+      <c r="B157" s="15"/>
+      <c r="C157" s="15"/>
+      <c r="D157" s="15"/>
+      <c r="E157" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F156" s="15"/>
-      <c r="G156" s="18">
-        <f t="shared" ref="G156:H156" si="11">SUM(G146:G155)</f>
-        <v>0</v>
-      </c>
-      <c r="H156" s="18">
+      <c r="F157" s="15"/>
+      <c r="G157" s="18">
+        <f t="shared" ref="G157:H157" si="11">SUM(G147:G156)</f>
+        <v>0</v>
+      </c>
+      <c r="H157" s="18">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="I156" s="18">
+      <c r="I157" s="18">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J156" s="19"/>
-      <c r="K156" s="46"/>
-    </row>
-    <row r="157" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="62" t="s">
+      <c r="J157" s="19"/>
+      <c r="K157" s="46"/>
+    </row>
+    <row r="158" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B157" s="63"/>
-      <c r="C157" s="63"/>
-      <c r="D157" s="63"/>
-      <c r="E157" s="63"/>
-      <c r="F157" s="63"/>
-      <c r="G157" s="63"/>
-      <c r="H157" s="63"/>
-      <c r="I157" s="63"/>
-      <c r="J157" s="63"/>
-      <c r="K157" s="64"/>
-    </row>
-    <row r="158" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A158" s="32" t="s">
+      <c r="B158" s="55"/>
+      <c r="C158" s="55"/>
+      <c r="D158" s="55"/>
+      <c r="E158" s="55"/>
+      <c r="F158" s="55"/>
+      <c r="G158" s="55"/>
+      <c r="H158" s="55"/>
+      <c r="I158" s="55"/>
+      <c r="J158" s="55"/>
+      <c r="K158" s="56"/>
+    </row>
+    <row r="159" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A159" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B158" s="65" t="s">
+      <c r="B159" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C158" s="63"/>
-      <c r="D158" s="63"/>
-      <c r="E158" s="63"/>
-      <c r="F158" s="63"/>
-      <c r="G158" s="63"/>
-      <c r="H158" s="63"/>
-      <c r="I158" s="63"/>
-      <c r="J158" s="63"/>
-      <c r="K158" s="64"/>
-    </row>
-    <row r="159" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="33" t="s">
+      <c r="C159" s="55"/>
+      <c r="D159" s="55"/>
+      <c r="E159" s="55"/>
+      <c r="F159" s="55"/>
+      <c r="G159" s="55"/>
+      <c r="H159" s="55"/>
+      <c r="I159" s="55"/>
+      <c r="J159" s="55"/>
+      <c r="K159" s="56"/>
+    </row>
+    <row r="160" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B159" s="65" t="s">
+      <c r="B160" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C159" s="63"/>
-      <c r="D159" s="63"/>
-      <c r="E159" s="63"/>
-      <c r="F159" s="63"/>
-      <c r="G159" s="63"/>
-      <c r="H159" s="63"/>
-      <c r="I159" s="63"/>
-      <c r="J159" s="63"/>
-      <c r="K159" s="64"/>
-    </row>
-    <row r="160" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A160" s="37"/>
-      <c r="B160" s="38"/>
-      <c r="C160" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D160" s="38"/>
-      <c r="E160" s="40"/>
-      <c r="F160" s="40"/>
-      <c r="G160" s="41"/>
-      <c r="H160" s="41"/>
-      <c r="I160" s="41">
-        <f t="shared" ref="I160:I170" si="12">H160-G160</f>
-        <v>0</v>
-      </c>
-      <c r="J160" s="45"/>
-      <c r="K160" s="43"/>
+      <c r="C160" s="55"/>
+      <c r="D160" s="55"/>
+      <c r="E160" s="55"/>
+      <c r="F160" s="55"/>
+      <c r="G160" s="55"/>
+      <c r="H160" s="55"/>
+      <c r="I160" s="55"/>
+      <c r="J160" s="55"/>
+      <c r="K160" s="56"/>
     </row>
     <row r="161" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A161" s="37"/>
@@ -5761,7 +5784,7 @@
       <c r="G161" s="41"/>
       <c r="H161" s="41"/>
       <c r="I161" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="I161:I171" si="12">H161-G161</f>
         <v>0</v>
       </c>
       <c r="J161" s="45"/>
@@ -5912,35 +5935,53 @@
       <c r="K169" s="43"/>
     </row>
     <row r="170" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A170" s="48"/>
-      <c r="B170" s="49"/>
-      <c r="C170" s="49"/>
-      <c r="D170" s="49"/>
-      <c r="E170" s="49" t="s">
+      <c r="A170" s="37"/>
+      <c r="B170" s="38"/>
+      <c r="C170" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D170" s="38"/>
+      <c r="E170" s="40"/>
+      <c r="F170" s="40"/>
+      <c r="G170" s="41"/>
+      <c r="H170" s="41"/>
+      <c r="I170" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J170" s="45"/>
+      <c r="K170" s="43"/>
+    </row>
+    <row r="171" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A171" s="48"/>
+      <c r="B171" s="49"/>
+      <c r="C171" s="49"/>
+      <c r="D171" s="49"/>
+      <c r="E171" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F170" s="49"/>
-      <c r="G170" s="50">
-        <f t="shared" ref="G170:H170" si="13">SUM(G160:G169)</f>
-        <v>0</v>
-      </c>
-      <c r="H170" s="50">
+      <c r="F171" s="49"/>
+      <c r="G171" s="50">
+        <f t="shared" ref="G171:H171" si="13">SUM(G161:G170)</f>
+        <v>0</v>
+      </c>
+      <c r="H171" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="I170" s="50">
+      <c r="I171" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J170" s="51"/>
-      <c r="K170" s="52"/>
+      <c r="J171" s="51"/>
+      <c r="K171" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{148386E4-773C-4965-B2FA-BF62B2CF7AA1}">
+      <autoFilter ref="A1:K15" xr:uid="{548196C1-A0E0-42F3-A7F7-BA5BC9D0B2E2}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5951,9 +5992,17 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A157:K157"/>
-    <mergeCell ref="B158:K158"/>
+    <mergeCell ref="B131:K131"/>
+    <mergeCell ref="B132:K132"/>
+    <mergeCell ref="A144:K144"/>
+    <mergeCell ref="B104:K104"/>
+    <mergeCell ref="A116:K116"/>
+    <mergeCell ref="B117:K117"/>
+    <mergeCell ref="B118:K118"/>
+    <mergeCell ref="A130:K130"/>
+    <mergeCell ref="A158:K158"/>
     <mergeCell ref="B159:K159"/>
+    <mergeCell ref="B160:K160"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -5963,20 +6012,12 @@
     <mergeCell ref="A83:K83"/>
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
-    <mergeCell ref="A101:K101"/>
-    <mergeCell ref="B144:K144"/>
+    <mergeCell ref="A102:K102"/>
     <mergeCell ref="B145:K145"/>
-    <mergeCell ref="B102:K102"/>
-    <mergeCell ref="B130:K130"/>
-    <mergeCell ref="B131:K131"/>
-    <mergeCell ref="A143:K143"/>
+    <mergeCell ref="B146:K146"/>
     <mergeCell ref="B103:K103"/>
-    <mergeCell ref="A115:K115"/>
-    <mergeCell ref="B116:K116"/>
-    <mergeCell ref="B117:K117"/>
-    <mergeCell ref="A129:K129"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B99 B104:B113 B118:B127 B132:B141 B146:B155">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B100 B105:B114 B119:B128 B133:B142 B147:B156">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -5993,7 +6034,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B100 B102:B114 B116:B128 B130:B142 B144:B156 B158:B170">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B101 B103:B115 B117:B129 B131:B143 B145:B157 B159:B171">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -6001,34 +6042,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B160:B169">
+  <conditionalFormatting sqref="B161:B170">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B160))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B161))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B160))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B161))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B160))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B161))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B160))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B161))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B160))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B161))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G100 G104:G114 G118:G128 G132:G142 G146:G156 G160:G170">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G101 G105:G115 G119:G129 G133:G143 G147:G157 G161:G171">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H170">
+  <conditionalFormatting sqref="H1:H171">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I100 I104:I114 I118:I128 I132:I142 I146:I156 I160:I170">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I101 I105:I115 I119:I129 I133:I143 I147:I157 I161:I171">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -6037,7 +6078,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F160:F169 F146:F155 F86:F99 F104:F113 F118:F127 F132:F141 F5:F45 F50:F81" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F161:F170 F147:F156 F86:F100 F105:F114 F119:F128 F133:F142 F5:F45 F50:F81" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6053,13 +6094,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E99 E104:E113 E118:E127 E132:E141 E146:E155 E160:E169 E50:E81</xm:sqref>
+          <xm:sqref>E5:E45 E86:E100 E105:E114 E119:E128 E133:E142 E147:E156 E161:E170 E50:E81</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B99 B104:B113 B118:B127 B132:B141 B146:B155 B160:B169 B50:B81</xm:sqref>
+          <xm:sqref>B5:B45 B86:B100 B105:B114 B119:B128 B133:B142 B147:B156 B161:B170 B50:B81</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7700,26 +7741,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -7954,10 +7975,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7974,20 +8026,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W3 DataLab 1 Work IV (End of DataLab)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC6F2F09-EB6D-44C5-AF0E-444CC587EDB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8633915D-59D9-4213-B6FE-BA0807518E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -626,7 +626,7 @@
     <t>ILO 6.2</t>
   </si>
   <si>
-    <t>From 9:30 until end -2 hours</t>
+    <t>5,5 at 17:00</t>
   </si>
 </sst>
 </file>
@@ -1112,6 +1112,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1128,8 +1148,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1147,24 +1165,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1689,53 +1689,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3074,53 +3074,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4173,53 +4173,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -4612,7 +4612,7 @@
         <v>45629</v>
       </c>
       <c r="B98" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C98" s="39" t="s">
         <v>17</v>
@@ -4629,10 +4629,12 @@
       <c r="G98" s="41">
         <v>1</v>
       </c>
-      <c r="H98" s="41"/>
+      <c r="H98" s="41">
+        <v>1</v>
+      </c>
       <c r="I98" s="41">
         <f t="shared" si="2"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J98" s="45"/>
       <c r="K98" s="43"/>
@@ -4700,63 +4702,63 @@
       </c>
       <c r="H101" s="18">
         <f t="shared" si="3"/>
-        <v>8.75</v>
+        <v>9.75</v>
       </c>
       <c r="I101" s="18">
         <f t="shared" si="2"/>
-        <v>-8.75</v>
+        <v>-7.75</v>
       </c>
       <c r="J101" s="19"/>
       <c r="K101" s="46"/>
     </row>
     <row r="102" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="68" t="s">
+      <c r="A102" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B102" s="62"/>
-      <c r="C102" s="62"/>
-      <c r="D102" s="62"/>
-      <c r="E102" s="62"/>
-      <c r="F102" s="62"/>
-      <c r="G102" s="62"/>
-      <c r="H102" s="62"/>
-      <c r="I102" s="62"/>
-      <c r="J102" s="62"/>
-      <c r="K102" s="63"/>
+      <c r="B102" s="55"/>
+      <c r="C102" s="55"/>
+      <c r="D102" s="55"/>
+      <c r="E102" s="55"/>
+      <c r="F102" s="55"/>
+      <c r="G102" s="55"/>
+      <c r="H102" s="55"/>
+      <c r="I102" s="55"/>
+      <c r="J102" s="55"/>
+      <c r="K102" s="56"/>
     </row>
     <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A103" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B103" s="70" t="s">
+      <c r="B103" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C103" s="62"/>
-      <c r="D103" s="62"/>
-      <c r="E103" s="62"/>
-      <c r="F103" s="62"/>
-      <c r="G103" s="62"/>
-      <c r="H103" s="62"/>
-      <c r="I103" s="62"/>
-      <c r="J103" s="62"/>
-      <c r="K103" s="63"/>
+      <c r="C103" s="55"/>
+      <c r="D103" s="55"/>
+      <c r="E103" s="55"/>
+      <c r="F103" s="55"/>
+      <c r="G103" s="55"/>
+      <c r="H103" s="55"/>
+      <c r="I103" s="55"/>
+      <c r="J103" s="55"/>
+      <c r="K103" s="56"/>
     </row>
     <row r="104" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B104" s="70" t="s">
+      <c r="B104" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C104" s="62"/>
-      <c r="D104" s="62"/>
-      <c r="E104" s="62"/>
-      <c r="F104" s="62"/>
-      <c r="G104" s="62"/>
-      <c r="H104" s="62"/>
-      <c r="I104" s="62"/>
-      <c r="J104" s="62"/>
-      <c r="K104" s="63"/>
+      <c r="C104" s="55"/>
+      <c r="D104" s="55"/>
+      <c r="E104" s="55"/>
+      <c r="F104" s="55"/>
+      <c r="G104" s="55"/>
+      <c r="H104" s="55"/>
+      <c r="I104" s="55"/>
+      <c r="J104" s="55"/>
+      <c r="K104" s="56"/>
     </row>
     <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A105" s="37"/>
@@ -4963,53 +4965,53 @@
       <c r="K115" s="46"/>
     </row>
     <row r="116" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="73" t="s">
+      <c r="A116" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B116" s="62"/>
-      <c r="C116" s="62"/>
-      <c r="D116" s="62"/>
-      <c r="E116" s="62"/>
-      <c r="F116" s="62"/>
-      <c r="G116" s="62"/>
-      <c r="H116" s="62"/>
-      <c r="I116" s="62"/>
-      <c r="J116" s="62"/>
-      <c r="K116" s="63"/>
+      <c r="B116" s="55"/>
+      <c r="C116" s="55"/>
+      <c r="D116" s="55"/>
+      <c r="E116" s="55"/>
+      <c r="F116" s="55"/>
+      <c r="G116" s="55"/>
+      <c r="H116" s="55"/>
+      <c r="I116" s="55"/>
+      <c r="J116" s="55"/>
+      <c r="K116" s="56"/>
     </row>
     <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A117" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B117" s="74" t="s">
+      <c r="B117" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C117" s="62"/>
-      <c r="D117" s="62"/>
-      <c r="E117" s="62"/>
-      <c r="F117" s="62"/>
-      <c r="G117" s="62"/>
-      <c r="H117" s="62"/>
-      <c r="I117" s="62"/>
-      <c r="J117" s="62"/>
-      <c r="K117" s="63"/>
+      <c r="C117" s="55"/>
+      <c r="D117" s="55"/>
+      <c r="E117" s="55"/>
+      <c r="F117" s="55"/>
+      <c r="G117" s="55"/>
+      <c r="H117" s="55"/>
+      <c r="I117" s="55"/>
+      <c r="J117" s="55"/>
+      <c r="K117" s="56"/>
     </row>
     <row r="118" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B118" s="74" t="s">
+      <c r="B118" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
+      <c r="C118" s="55"/>
+      <c r="D118" s="55"/>
+      <c r="E118" s="55"/>
+      <c r="F118" s="55"/>
+      <c r="G118" s="55"/>
+      <c r="H118" s="55"/>
+      <c r="I118" s="55"/>
+      <c r="J118" s="55"/>
+      <c r="K118" s="56"/>
     </row>
     <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A119" s="37"/>
@@ -5216,53 +5218,53 @@
       <c r="K129" s="46"/>
     </row>
     <row r="130" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="75" t="s">
+      <c r="A130" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B130" s="62"/>
-      <c r="C130" s="62"/>
-      <c r="D130" s="62"/>
-      <c r="E130" s="62"/>
-      <c r="F130" s="62"/>
-      <c r="G130" s="62"/>
-      <c r="H130" s="62"/>
-      <c r="I130" s="62"/>
-      <c r="J130" s="62"/>
-      <c r="K130" s="63"/>
+      <c r="B130" s="55"/>
+      <c r="C130" s="55"/>
+      <c r="D130" s="55"/>
+      <c r="E130" s="55"/>
+      <c r="F130" s="55"/>
+      <c r="G130" s="55"/>
+      <c r="H130" s="55"/>
+      <c r="I130" s="55"/>
+      <c r="J130" s="55"/>
+      <c r="K130" s="56"/>
     </row>
     <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A131" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B131" s="71" t="s">
+      <c r="B131" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C131" s="62"/>
-      <c r="D131" s="62"/>
-      <c r="E131" s="62"/>
-      <c r="F131" s="62"/>
-      <c r="G131" s="62"/>
-      <c r="H131" s="62"/>
-      <c r="I131" s="62"/>
-      <c r="J131" s="62"/>
-      <c r="K131" s="63"/>
+      <c r="C131" s="55"/>
+      <c r="D131" s="55"/>
+      <c r="E131" s="55"/>
+      <c r="F131" s="55"/>
+      <c r="G131" s="55"/>
+      <c r="H131" s="55"/>
+      <c r="I131" s="55"/>
+      <c r="J131" s="55"/>
+      <c r="K131" s="56"/>
     </row>
     <row r="132" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B132" s="71" t="s">
+      <c r="B132" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C132" s="62"/>
-      <c r="D132" s="62"/>
-      <c r="E132" s="62"/>
-      <c r="F132" s="62"/>
-      <c r="G132" s="62"/>
-      <c r="H132" s="62"/>
-      <c r="I132" s="62"/>
-      <c r="J132" s="62"/>
-      <c r="K132" s="63"/>
+      <c r="C132" s="55"/>
+      <c r="D132" s="55"/>
+      <c r="E132" s="55"/>
+      <c r="F132" s="55"/>
+      <c r="G132" s="55"/>
+      <c r="H132" s="55"/>
+      <c r="I132" s="55"/>
+      <c r="J132" s="55"/>
+      <c r="K132" s="56"/>
     </row>
     <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A133" s="37"/>
@@ -5471,53 +5473,53 @@
       <c r="K143" s="46"/>
     </row>
     <row r="144" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="72" t="s">
+      <c r="A144" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B144" s="62"/>
-      <c r="C144" s="62"/>
-      <c r="D144" s="62"/>
-      <c r="E144" s="62"/>
-      <c r="F144" s="62"/>
-      <c r="G144" s="62"/>
-      <c r="H144" s="62"/>
-      <c r="I144" s="62"/>
-      <c r="J144" s="62"/>
-      <c r="K144" s="63"/>
+      <c r="B144" s="55"/>
+      <c r="C144" s="55"/>
+      <c r="D144" s="55"/>
+      <c r="E144" s="55"/>
+      <c r="F144" s="55"/>
+      <c r="G144" s="55"/>
+      <c r="H144" s="55"/>
+      <c r="I144" s="55"/>
+      <c r="J144" s="55"/>
+      <c r="K144" s="56"/>
     </row>
     <row r="145" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A145" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B145" s="69" t="s">
+      <c r="B145" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C145" s="62"/>
-      <c r="D145" s="62"/>
-      <c r="E145" s="62"/>
-      <c r="F145" s="62"/>
-      <c r="G145" s="62"/>
-      <c r="H145" s="62"/>
-      <c r="I145" s="62"/>
-      <c r="J145" s="62"/>
-      <c r="K145" s="63"/>
+      <c r="C145" s="55"/>
+      <c r="D145" s="55"/>
+      <c r="E145" s="55"/>
+      <c r="F145" s="55"/>
+      <c r="G145" s="55"/>
+      <c r="H145" s="55"/>
+      <c r="I145" s="55"/>
+      <c r="J145" s="55"/>
+      <c r="K145" s="56"/>
     </row>
     <row r="146" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B146" s="69" t="s">
+      <c r="B146" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C146" s="62"/>
-      <c r="D146" s="62"/>
-      <c r="E146" s="62"/>
-      <c r="F146" s="62"/>
-      <c r="G146" s="62"/>
-      <c r="H146" s="62"/>
-      <c r="I146" s="62"/>
-      <c r="J146" s="62"/>
-      <c r="K146" s="63"/>
+      <c r="C146" s="55"/>
+      <c r="D146" s="55"/>
+      <c r="E146" s="55"/>
+      <c r="F146" s="55"/>
+      <c r="G146" s="55"/>
+      <c r="H146" s="55"/>
+      <c r="I146" s="55"/>
+      <c r="J146" s="55"/>
+      <c r="K146" s="56"/>
     </row>
     <row r="147" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A147" s="37"/>
@@ -5724,53 +5726,53 @@
       <c r="K157" s="46"/>
     </row>
     <row r="158" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="54" t="s">
+      <c r="A158" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B158" s="55"/>
-      <c r="C158" s="55"/>
-      <c r="D158" s="55"/>
-      <c r="E158" s="55"/>
-      <c r="F158" s="55"/>
-      <c r="G158" s="55"/>
-      <c r="H158" s="55"/>
-      <c r="I158" s="55"/>
-      <c r="J158" s="55"/>
-      <c r="K158" s="56"/>
+      <c r="B158" s="63"/>
+      <c r="C158" s="63"/>
+      <c r="D158" s="63"/>
+      <c r="E158" s="63"/>
+      <c r="F158" s="63"/>
+      <c r="G158" s="63"/>
+      <c r="H158" s="63"/>
+      <c r="I158" s="63"/>
+      <c r="J158" s="63"/>
+      <c r="K158" s="64"/>
     </row>
     <row r="159" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A159" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B159" s="57" t="s">
+      <c r="B159" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C159" s="55"/>
-      <c r="D159" s="55"/>
-      <c r="E159" s="55"/>
-      <c r="F159" s="55"/>
-      <c r="G159" s="55"/>
-      <c r="H159" s="55"/>
-      <c r="I159" s="55"/>
-      <c r="J159" s="55"/>
-      <c r="K159" s="56"/>
+      <c r="C159" s="63"/>
+      <c r="D159" s="63"/>
+      <c r="E159" s="63"/>
+      <c r="F159" s="63"/>
+      <c r="G159" s="63"/>
+      <c r="H159" s="63"/>
+      <c r="I159" s="63"/>
+      <c r="J159" s="63"/>
+      <c r="K159" s="64"/>
     </row>
     <row r="160" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B160" s="57" t="s">
+      <c r="B160" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C160" s="55"/>
-      <c r="D160" s="55"/>
-      <c r="E160" s="55"/>
-      <c r="F160" s="55"/>
-      <c r="G160" s="55"/>
-      <c r="H160" s="55"/>
-      <c r="I160" s="55"/>
-      <c r="J160" s="55"/>
-      <c r="K160" s="56"/>
+      <c r="C160" s="63"/>
+      <c r="D160" s="63"/>
+      <c r="E160" s="63"/>
+      <c r="F160" s="63"/>
+      <c r="G160" s="63"/>
+      <c r="H160" s="63"/>
+      <c r="I160" s="63"/>
+      <c r="J160" s="63"/>
+      <c r="K160" s="64"/>
     </row>
     <row r="161" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A161" s="37"/>
@@ -5981,7 +5983,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{548196C1-A0E0-42F3-A7F7-BA5BC9D0B2E2}">
+      <autoFilter ref="A1:K15" xr:uid="{7C9185E5-A137-49DC-B738-85C392A73DBD}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5992,14 +5994,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B131:K131"/>
-    <mergeCell ref="B132:K132"/>
-    <mergeCell ref="A144:K144"/>
-    <mergeCell ref="B104:K104"/>
-    <mergeCell ref="A116:K116"/>
-    <mergeCell ref="B117:K117"/>
-    <mergeCell ref="B118:K118"/>
-    <mergeCell ref="A130:K130"/>
     <mergeCell ref="A158:K158"/>
     <mergeCell ref="B159:K159"/>
     <mergeCell ref="B160:K160"/>
@@ -6016,6 +6010,14 @@
     <mergeCell ref="B145:K145"/>
     <mergeCell ref="B146:K146"/>
     <mergeCell ref="B103:K103"/>
+    <mergeCell ref="B131:K131"/>
+    <mergeCell ref="B132:K132"/>
+    <mergeCell ref="A144:K144"/>
+    <mergeCell ref="B104:K104"/>
+    <mergeCell ref="A116:K116"/>
+    <mergeCell ref="B117:K117"/>
+    <mergeCell ref="B118:K118"/>
+    <mergeCell ref="A130:K130"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B100 B105:B114 B119:B128 B133:B142 B147:B156">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -7741,6 +7743,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -7975,27 +7997,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8012,23 +8033,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W4 DataLab 2 Work I (Beginning)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8633915D-59D9-4213-B6FE-BA0807518E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E60ABC6A-4F36-49B8-9EAB-F793030D2FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$156</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$190</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="214">
   <si>
     <t>Date</t>
   </si>
@@ -626,7 +626,124 @@
     <t>ILO 6.2</t>
   </si>
   <si>
-    <t>5,5 at 17:00</t>
+    <t>Took a bit longer than planned.</t>
+  </si>
+  <si>
+    <t>Learn about matrices</t>
+  </si>
+  <si>
+    <t>Application of matrices</t>
+  </si>
+  <si>
+    <t>Matrices Quiz</t>
+  </si>
+  <si>
+    <t>Introduction to Logistic Regression</t>
+  </si>
+  <si>
+    <t>Training and Cost Function</t>
+  </si>
+  <si>
+    <t>Decision Boundaries</t>
+  </si>
+  <si>
+    <t>Softmax Regression</t>
+  </si>
+  <si>
+    <t>Review the Chapter</t>
+  </si>
+  <si>
+    <t>Complete “ML-quiz-W3_3” in brightspace</t>
+  </si>
+  <si>
+    <t>Implement regression</t>
+  </si>
+  <si>
+    <t>Work in Creative Brief</t>
+  </si>
+  <si>
+    <t>Evidence Work Log Week 3</t>
+  </si>
+  <si>
+    <t>Evidence Learning Log Week 3</t>
+  </si>
+  <si>
+    <t>Regression Lecture</t>
+  </si>
+  <si>
+    <t>ILO 8.2</t>
+  </si>
+  <si>
+    <t>Complete “ML-quiz-W4_1” in brightspace</t>
+  </si>
+  <si>
+    <t>Training and visualizing decision trees</t>
+  </si>
+  <si>
+    <t>Making predictions and understanding purity</t>
+  </si>
+  <si>
+    <t>The CART training algorithm</t>
+  </si>
+  <si>
+    <t>Regularization Hyperparameters</t>
+  </si>
+  <si>
+    <t>Regression with decision trees</t>
+  </si>
+  <si>
+    <t>Implement a classification model</t>
+  </si>
+  <si>
+    <t>Practice Notebook</t>
+  </si>
+  <si>
+    <t>Do Calculus Quiz</t>
+  </si>
+  <si>
+    <t>Learn Calculus</t>
+  </si>
+  <si>
+    <t>Practice Calculus</t>
+  </si>
+  <si>
+    <t>2 hours so far</t>
+  </si>
+  <si>
+    <t>Complete “ML-quiz-W4_2” in brightspace</t>
+  </si>
+  <si>
+    <t>Stacking Ensembles</t>
+  </si>
+  <si>
+    <t>Boosting techniques, including AdaBoost, gradient boosting, and histogram-based gradient boosting.</t>
+  </si>
+  <si>
+    <t>Deep dive into random forests, extra-trees, and feature importance.</t>
+  </si>
+  <si>
+    <t>Bagging and pasting techniques, along with out-of-bag evaluation.</t>
+  </si>
+  <si>
+    <t>Introduction to ensemble learning and voting classifiers.</t>
+  </si>
+  <si>
+    <t>Read the chapter 7 summarization</t>
+  </si>
+  <si>
+    <t>Read the chapter 6 summarization</t>
+  </si>
+  <si>
+    <t>Start to implement classification model</t>
+  </si>
+  <si>
+    <t>1 on 1 meeting</t>
+  </si>
+  <si>
+    <t>Fill in Learning Log</t>
+  </si>
+  <si>
+    <t>I had done some overlapping work with the previous task so was shorter.</t>
   </si>
 </sst>
 </file>
@@ -1112,26 +1229,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1148,6 +1245,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1165,6 +1264,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1637,7 +1754,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K171"/>
+  <dimension ref="A1:K205"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1689,53 +1806,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3074,53 +3191,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="62"/>
+      <c r="K49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4173,53 +4290,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72" t="s">
+      <c r="A83" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="55"/>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="55"/>
-      <c r="I83" s="55"/>
-      <c r="J83" s="55"/>
-      <c r="K83" s="56"/>
+      <c r="B83" s="62"/>
+      <c r="C83" s="62"/>
+      <c r="D83" s="62"/>
+      <c r="E83" s="62"/>
+      <c r="F83" s="62"/>
+      <c r="G83" s="62"/>
+      <c r="H83" s="62"/>
+      <c r="I83" s="62"/>
+      <c r="J83" s="62"/>
+      <c r="K83" s="63"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="73" t="s">
+      <c r="B84" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="55"/>
-      <c r="D84" s="55"/>
-      <c r="E84" s="55"/>
-      <c r="F84" s="55"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="55"/>
-      <c r="I84" s="55"/>
-      <c r="J84" s="55"/>
-      <c r="K84" s="56"/>
+      <c r="C84" s="62"/>
+      <c r="D84" s="62"/>
+      <c r="E84" s="62"/>
+      <c r="F84" s="62"/>
+      <c r="G84" s="62"/>
+      <c r="H84" s="62"/>
+      <c r="I84" s="62"/>
+      <c r="J84" s="62"/>
+      <c r="K84" s="63"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="73" t="s">
+      <c r="B85" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="55"/>
-      <c r="D85" s="55"/>
-      <c r="E85" s="55"/>
-      <c r="F85" s="55"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="55"/>
-      <c r="I85" s="55"/>
-      <c r="J85" s="55"/>
-      <c r="K85" s="56"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="62"/>
+      <c r="G85" s="62"/>
+      <c r="H85" s="62"/>
+      <c r="I85" s="62"/>
+      <c r="J85" s="62"/>
+      <c r="K85" s="63"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -4247,7 +4364,7 @@
         <v>0.5</v>
       </c>
       <c r="I86" s="41">
-        <f t="shared" ref="I86:I101" si="2">H86-G86</f>
+        <f t="shared" ref="I86:I117" si="2">H86-G86</f>
         <v>0</v>
       </c>
       <c r="J86" s="45"/>
@@ -4580,7 +4697,7 @@
         <v>45629</v>
       </c>
       <c r="B97" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C97" s="39" t="s">
         <v>17</v>
@@ -4597,10 +4714,12 @@
       <c r="G97" s="41">
         <v>4</v>
       </c>
-      <c r="H97" s="41"/>
+      <c r="H97" s="41">
+        <v>5.5</v>
+      </c>
       <c r="I97" s="41">
         <f t="shared" si="2"/>
-        <v>-4</v>
+        <v>1.5</v>
       </c>
       <c r="J97" s="45"/>
       <c r="K97" s="43" t="s">
@@ -4644,7 +4763,7 @@
         <v>45629</v>
       </c>
       <c r="B99" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C99" s="39" t="s">
         <v>17</v>
@@ -4661,25 +4780,41 @@
       <c r="G99" s="41">
         <v>2.5</v>
       </c>
-      <c r="H99" s="41"/>
+      <c r="H99" s="41">
+        <v>2</v>
+      </c>
       <c r="I99" s="41">
         <f t="shared" si="2"/>
-        <v>-2.5</v>
+        <v>-0.5</v>
       </c>
       <c r="J99" s="45"/>
       <c r="K99" s="43"/>
     </row>
     <row r="100" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A100" s="37"/>
-      <c r="B100" s="38"/>
+      <c r="A100" s="37">
+        <v>45630</v>
+      </c>
+      <c r="B100" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C100" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D100" s="38"/>
-      <c r="E100" s="40"/>
-      <c r="F100" s="40"/>
-      <c r="G100" s="41"/>
-      <c r="H100" s="41"/>
+      <c r="D100" s="38" t="s">
+        <v>175</v>
+      </c>
+      <c r="E100" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F100" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G100" s="41">
+        <v>4</v>
+      </c>
+      <c r="H100" s="41">
+        <v>4</v>
+      </c>
       <c r="I100" s="41">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4688,838 +4823,1391 @@
       <c r="K100" s="43"/>
     </row>
     <row r="101" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A101" s="13"/>
-      <c r="B101" s="15"/>
-      <c r="C101" s="15"/>
-      <c r="D101" s="15"/>
-      <c r="E101" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F101" s="15"/>
-      <c r="G101" s="18">
-        <f t="shared" ref="G101:H101" si="3">SUM(G86:G100)</f>
-        <v>17.5</v>
-      </c>
-      <c r="H101" s="18">
-        <f t="shared" si="3"/>
-        <v>9.75</v>
-      </c>
-      <c r="I101" s="18">
+      <c r="A101" s="37">
+        <v>45630</v>
+      </c>
+      <c r="B101" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C101" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D101" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="E101" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F101" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G101" s="41">
+        <v>2</v>
+      </c>
+      <c r="H101" s="41">
+        <v>1</v>
+      </c>
+      <c r="I101" s="41">
         <f t="shared" si="2"/>
-        <v>-7.75</v>
-      </c>
-      <c r="J101" s="19"/>
-      <c r="K101" s="46"/>
-    </row>
-    <row r="102" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="74" t="s">
-        <v>22</v>
-      </c>
-      <c r="B102" s="55"/>
-      <c r="C102" s="55"/>
-      <c r="D102" s="55"/>
-      <c r="E102" s="55"/>
-      <c r="F102" s="55"/>
-      <c r="G102" s="55"/>
-      <c r="H102" s="55"/>
-      <c r="I102" s="55"/>
-      <c r="J102" s="55"/>
-      <c r="K102" s="56"/>
+        <v>-1</v>
+      </c>
+      <c r="J101" s="45"/>
+      <c r="K101" s="43"/>
+    </row>
+    <row r="102" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A102" s="37">
+        <v>45630</v>
+      </c>
+      <c r="B102" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C102" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D102" s="38" t="s">
+        <v>177</v>
+      </c>
+      <c r="E102" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F102" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G102" s="41">
+        <v>1</v>
+      </c>
+      <c r="H102" s="41"/>
+      <c r="I102" s="41">
+        <f t="shared" si="2"/>
+        <v>-1</v>
+      </c>
+      <c r="J102" s="45"/>
+      <c r="K102" s="43"/>
     </row>
     <row r="103" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A103" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B103" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="C103" s="55"/>
-      <c r="D103" s="55"/>
-      <c r="E103" s="55"/>
-      <c r="F103" s="55"/>
-      <c r="G103" s="55"/>
-      <c r="H103" s="55"/>
-      <c r="I103" s="55"/>
-      <c r="J103" s="55"/>
-      <c r="K103" s="56"/>
-    </row>
-    <row r="104" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B104" s="58" t="s">
-        <v>15</v>
-      </c>
-      <c r="C104" s="55"/>
-      <c r="D104" s="55"/>
-      <c r="E104" s="55"/>
-      <c r="F104" s="55"/>
-      <c r="G104" s="55"/>
-      <c r="H104" s="55"/>
-      <c r="I104" s="55"/>
-      <c r="J104" s="55"/>
-      <c r="K104" s="56"/>
+      <c r="A103" s="37">
+        <v>45631</v>
+      </c>
+      <c r="B103" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C103" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D103" s="38" t="s">
+        <v>178</v>
+      </c>
+      <c r="E103" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F103" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G103" s="41">
+        <v>1</v>
+      </c>
+      <c r="H103" s="41">
+        <v>1</v>
+      </c>
+      <c r="I103" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J103" s="45"/>
+      <c r="K103" s="43"/>
+    </row>
+    <row r="104" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A104" s="37">
+        <v>45631</v>
+      </c>
+      <c r="B104" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C104" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D104" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="E104" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F104" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G104" s="41">
+        <v>2</v>
+      </c>
+      <c r="H104" s="41">
+        <v>2</v>
+      </c>
+      <c r="I104" s="41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J104" s="45"/>
+      <c r="K104" s="43"/>
     </row>
     <row r="105" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A105" s="37"/>
-      <c r="B105" s="38"/>
+      <c r="A105" s="37">
+        <v>45631</v>
+      </c>
+      <c r="B105" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C105" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D105" s="38"/>
-      <c r="E105" s="40"/>
-      <c r="F105" s="40"/>
-      <c r="G105" s="41"/>
-      <c r="H105" s="41"/>
+      <c r="D105" s="38" t="s">
+        <v>180</v>
+      </c>
+      <c r="E105" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F105" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G105" s="41">
+        <v>1</v>
+      </c>
+      <c r="H105" s="41">
+        <v>1</v>
+      </c>
       <c r="I105" s="41">
-        <f t="shared" ref="I105:I115" si="4">H105-G105</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J105" s="45"/>
       <c r="K105" s="43"/>
     </row>
     <row r="106" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A106" s="37"/>
-      <c r="B106" s="38"/>
+      <c r="A106" s="37">
+        <v>45631</v>
+      </c>
+      <c r="B106" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C106" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D106" s="38"/>
-      <c r="E106" s="40"/>
-      <c r="F106" s="40"/>
-      <c r="G106" s="41"/>
-      <c r="H106" s="41"/>
+      <c r="D106" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="E106" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F106" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G106" s="41">
+        <v>2</v>
+      </c>
+      <c r="H106" s="41">
+        <v>2</v>
+      </c>
       <c r="I106" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J106" s="45"/>
       <c r="K106" s="43"/>
     </row>
     <row r="107" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A107" s="37"/>
-      <c r="B107" s="38"/>
+      <c r="A107" s="37">
+        <v>45631</v>
+      </c>
+      <c r="B107" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C107" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D107" s="38"/>
-      <c r="E107" s="40"/>
-      <c r="F107" s="40"/>
-      <c r="G107" s="41"/>
-      <c r="H107" s="41"/>
+      <c r="D107" s="38" t="s">
+        <v>182</v>
+      </c>
+      <c r="E107" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F107" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G107" s="41">
+        <v>1</v>
+      </c>
+      <c r="H107" s="41">
+        <v>1</v>
+      </c>
       <c r="I107" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J107" s="45"/>
       <c r="K107" s="43"/>
     </row>
     <row r="108" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A108" s="37"/>
-      <c r="B108" s="38"/>
+      <c r="A108" s="37">
+        <v>45631</v>
+      </c>
+      <c r="B108" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C108" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D108" s="38"/>
-      <c r="E108" s="40"/>
-      <c r="F108" s="40"/>
-      <c r="G108" s="41"/>
-      <c r="H108" s="41"/>
+      <c r="D108" s="38" t="s">
+        <v>183</v>
+      </c>
+      <c r="E108" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F108" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G108" s="41">
+        <v>1</v>
+      </c>
+      <c r="H108" s="41">
+        <v>1</v>
+      </c>
       <c r="I108" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J108" s="45"/>
       <c r="K108" s="43"/>
     </row>
     <row r="109" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A109" s="37"/>
-      <c r="B109" s="38"/>
+      <c r="A109" s="37">
+        <v>45632</v>
+      </c>
+      <c r="B109" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C109" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D109" s="38"/>
-      <c r="E109" s="40"/>
-      <c r="F109" s="40"/>
-      <c r="G109" s="41"/>
-      <c r="H109" s="41"/>
+      <c r="D109" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="E109" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F109" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G109" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H109" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I109" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J109" s="45"/>
       <c r="K109" s="43"/>
     </row>
     <row r="110" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A110" s="37"/>
-      <c r="B110" s="38"/>
+      <c r="A110" s="37">
+        <v>45632</v>
+      </c>
+      <c r="B110" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C110" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D110" s="38"/>
-      <c r="E110" s="40"/>
-      <c r="F110" s="40"/>
-      <c r="G110" s="41"/>
-      <c r="H110" s="41"/>
+      <c r="D110" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="E110" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F110" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="G110" s="41">
+        <v>4</v>
+      </c>
+      <c r="H110" s="41">
+        <v>4</v>
+      </c>
       <c r="I110" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J110" s="45"/>
       <c r="K110" s="43"/>
     </row>
     <row r="111" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A111" s="37"/>
-      <c r="B111" s="38"/>
+      <c r="A111" s="37">
+        <v>45632</v>
+      </c>
+      <c r="B111" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C111" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D111" s="38"/>
-      <c r="E111" s="40"/>
-      <c r="F111" s="40"/>
-      <c r="G111" s="41"/>
-      <c r="H111" s="41"/>
+      <c r="D111" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="E111" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F111" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G111" s="41">
+        <v>1</v>
+      </c>
+      <c r="H111" s="41">
+        <v>1</v>
+      </c>
       <c r="I111" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J111" s="45"/>
       <c r="K111" s="43"/>
     </row>
     <row r="112" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A112" s="37"/>
-      <c r="B112" s="38"/>
+      <c r="A112" s="37">
+        <v>45632</v>
+      </c>
+      <c r="B112" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C112" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D112" s="38"/>
-      <c r="E112" s="40"/>
-      <c r="F112" s="40"/>
-      <c r="G112" s="41"/>
-      <c r="H112" s="41"/>
+      <c r="D112" s="38" t="s">
+        <v>185</v>
+      </c>
+      <c r="E112" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F112" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="G112" s="41">
+        <v>2.5</v>
+      </c>
+      <c r="H112" s="41">
+        <v>1.5</v>
+      </c>
       <c r="I112" s="41">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>-1</v>
       </c>
       <c r="J112" s="45"/>
-      <c r="K112" s="43"/>
+      <c r="K112" s="43" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="113" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A113" s="37"/>
-      <c r="B113" s="38"/>
+      <c r="A113" s="37">
+        <v>45632</v>
+      </c>
+      <c r="B113" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C113" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D113" s="38"/>
-      <c r="E113" s="40"/>
-      <c r="F113" s="40"/>
-      <c r="G113" s="41"/>
-      <c r="H113" s="41"/>
+      <c r="D113" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="E113" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F113" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G113" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H113" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I113" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J113" s="45"/>
       <c r="K113" s="43"/>
     </row>
     <row r="114" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A114" s="37"/>
-      <c r="B114" s="38"/>
+      <c r="A114" s="37">
+        <v>45632</v>
+      </c>
+      <c r="B114" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C114" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D114" s="38"/>
-      <c r="E114" s="40"/>
-      <c r="F114" s="40"/>
-      <c r="G114" s="41"/>
-      <c r="H114" s="41"/>
+      <c r="D114" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="E114" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F114" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G114" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H114" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I114" s="41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J114" s="45"/>
       <c r="K114" s="43"/>
     </row>
     <row r="115" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A115" s="13"/>
-      <c r="B115" s="15"/>
-      <c r="C115" s="15"/>
-      <c r="D115" s="15"/>
-      <c r="E115" s="15" t="s">
+      <c r="A115" s="37"/>
+      <c r="B115" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C115" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D115" s="38" t="s">
+        <v>187</v>
+      </c>
+      <c r="E115" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F115" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G115" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H115" s="41"/>
+      <c r="I115" s="41">
+        <f t="shared" si="2"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J115" s="45"/>
+      <c r="K115" s="43"/>
+    </row>
+    <row r="116" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A116" s="37"/>
+      <c r="B116" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C116" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D116" s="38" t="s">
+        <v>186</v>
+      </c>
+      <c r="E116" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F116" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G116" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H116" s="41"/>
+      <c r="I116" s="41">
+        <f t="shared" si="2"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J116" s="45"/>
+      <c r="K116" s="43"/>
+    </row>
+    <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A117" s="13"/>
+      <c r="B117" s="15"/>
+      <c r="C117" s="15"/>
+      <c r="D117" s="15"/>
+      <c r="E117" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F115" s="15"/>
-      <c r="G115" s="18">
-        <f t="shared" ref="G115:H115" si="5">SUM(G105:G114)</f>
-        <v>0</v>
-      </c>
-      <c r="H115" s="18">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="I115" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="J115" s="19"/>
-      <c r="K115" s="46"/>
-    </row>
-    <row r="116" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="59" t="s">
-        <v>23</v>
-      </c>
-      <c r="B116" s="55"/>
-      <c r="C116" s="55"/>
-      <c r="D116" s="55"/>
-      <c r="E116" s="55"/>
-      <c r="F116" s="55"/>
-      <c r="G116" s="55"/>
-      <c r="H116" s="55"/>
-      <c r="I116" s="55"/>
-      <c r="J116" s="55"/>
-      <c r="K116" s="56"/>
-    </row>
-    <row r="117" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A117" s="25" t="s">
+      <c r="F117" s="15"/>
+      <c r="G117" s="18">
+        <f t="shared" ref="G117:H117" si="3">SUM(G86:G116)</f>
+        <v>42.25</v>
+      </c>
+      <c r="H117" s="18">
+        <f t="shared" si="3"/>
+        <v>38</v>
+      </c>
+      <c r="I117" s="18">
+        <f t="shared" si="2"/>
+        <v>-4.25</v>
+      </c>
+      <c r="J117" s="19"/>
+      <c r="K117" s="46"/>
+    </row>
+    <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="B118" s="62"/>
+      <c r="C118" s="62"/>
+      <c r="D118" s="62"/>
+      <c r="E118" s="62"/>
+      <c r="F118" s="62"/>
+      <c r="G118" s="62"/>
+      <c r="H118" s="62"/>
+      <c r="I118" s="62"/>
+      <c r="J118" s="62"/>
+      <c r="K118" s="63"/>
+    </row>
+    <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B117" s="60" t="s">
+      <c r="B119" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C117" s="55"/>
-      <c r="D117" s="55"/>
-      <c r="E117" s="55"/>
-      <c r="F117" s="55"/>
-      <c r="G117" s="55"/>
-      <c r="H117" s="55"/>
-      <c r="I117" s="55"/>
-      <c r="J117" s="55"/>
-      <c r="K117" s="56"/>
-    </row>
-    <row r="118" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="26" t="s">
+      <c r="C119" s="62"/>
+      <c r="D119" s="62"/>
+      <c r="E119" s="62"/>
+      <c r="F119" s="62"/>
+      <c r="G119" s="62"/>
+      <c r="H119" s="62"/>
+      <c r="I119" s="62"/>
+      <c r="J119" s="62"/>
+      <c r="K119" s="63"/>
+    </row>
+    <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B118" s="60" t="s">
+      <c r="B120" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C118" s="55"/>
-      <c r="D118" s="55"/>
-      <c r="E118" s="55"/>
-      <c r="F118" s="55"/>
-      <c r="G118" s="55"/>
-      <c r="H118" s="55"/>
-      <c r="I118" s="55"/>
-      <c r="J118" s="55"/>
-      <c r="K118" s="56"/>
-    </row>
-    <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A119" s="37"/>
-      <c r="B119" s="38"/>
-      <c r="C119" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D119" s="38"/>
-      <c r="E119" s="40"/>
-      <c r="F119" s="40"/>
-      <c r="G119" s="41"/>
-      <c r="H119" s="41"/>
-      <c r="I119" s="41">
-        <f t="shared" ref="I119:I129" si="6">H119-G119</f>
-        <v>0</v>
-      </c>
-      <c r="J119" s="45"/>
-      <c r="K119" s="43"/>
-    </row>
-    <row r="120" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A120" s="37"/>
-      <c r="B120" s="38"/>
-      <c r="C120" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D120" s="38"/>
-      <c r="E120" s="40"/>
-      <c r="F120" s="40"/>
-      <c r="G120" s="41"/>
-      <c r="H120" s="41"/>
-      <c r="I120" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J120" s="45"/>
-      <c r="K120" s="43"/>
+      <c r="C120" s="62"/>
+      <c r="D120" s="62"/>
+      <c r="E120" s="62"/>
+      <c r="F120" s="62"/>
+      <c r="G120" s="62"/>
+      <c r="H120" s="62"/>
+      <c r="I120" s="62"/>
+      <c r="J120" s="62"/>
+      <c r="K120" s="63"/>
     </row>
     <row r="121" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A121" s="37"/>
-      <c r="B121" s="38"/>
+      <c r="A121" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B121" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C121" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D121" s="38"/>
-      <c r="E121" s="40"/>
-      <c r="F121" s="40"/>
-      <c r="G121" s="41"/>
-      <c r="H121" s="41"/>
+      <c r="D121" s="38" t="s">
+        <v>212</v>
+      </c>
+      <c r="E121" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F121" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G121" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H121" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I121" s="41">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="I121:I122" si="4">H121-G121</f>
         <v>0</v>
       </c>
       <c r="J121" s="45"/>
       <c r="K121" s="43"/>
     </row>
     <row r="122" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A122" s="37"/>
-      <c r="B122" s="38"/>
+      <c r="A122" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B122" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C122" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D122" s="38"/>
-      <c r="E122" s="40"/>
-      <c r="F122" s="40"/>
-      <c r="G122" s="41"/>
-      <c r="H122" s="41"/>
+      <c r="D122" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="E122" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F122" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G122" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H122" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I122" s="41">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J122" s="45"/>
       <c r="K122" s="43"/>
     </row>
     <row r="123" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A123" s="37"/>
-      <c r="B123" s="38"/>
+      <c r="A123" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B123" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C123" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D123" s="38"/>
-      <c r="E123" s="40"/>
-      <c r="F123" s="40"/>
-      <c r="G123" s="41"/>
-      <c r="H123" s="41"/>
+      <c r="D123" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="E123" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F123" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G123" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H123" s="41">
+        <v>1.5</v>
+      </c>
       <c r="I123" s="41">
-        <f t="shared" si="6"/>
+        <f>H123-G123</f>
         <v>0</v>
       </c>
       <c r="J123" s="45"/>
       <c r="K123" s="43"/>
     </row>
     <row r="124" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A124" s="37"/>
-      <c r="B124" s="38"/>
+      <c r="A124" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B124" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C124" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D124" s="38"/>
-      <c r="E124" s="40"/>
-      <c r="F124" s="40"/>
-      <c r="G124" s="41"/>
-      <c r="H124" s="41"/>
+      <c r="D124" s="38" t="s">
+        <v>192</v>
+      </c>
+      <c r="E124" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F124" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G124" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H124" s="41">
+        <v>1</v>
+      </c>
       <c r="I124" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f t="shared" ref="I121:I149" si="5">H124-G124</f>
+        <v>-0.5</v>
       </c>
       <c r="J124" s="45"/>
       <c r="K124" s="43"/>
     </row>
     <row r="125" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A125" s="37"/>
-      <c r="B125" s="38"/>
+      <c r="A125" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B125" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C125" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D125" s="38"/>
-      <c r="E125" s="40"/>
-      <c r="F125" s="40"/>
-      <c r="G125" s="41"/>
-      <c r="H125" s="41"/>
+      <c r="D125" s="38" t="s">
+        <v>193</v>
+      </c>
+      <c r="E125" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F125" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G125" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H125" s="41">
+        <v>1</v>
+      </c>
       <c r="I125" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-0.5</v>
       </c>
       <c r="J125" s="45"/>
       <c r="K125" s="43"/>
     </row>
     <row r="126" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A126" s="37"/>
-      <c r="B126" s="38"/>
+      <c r="A126" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B126" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C126" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D126" s="38"/>
-      <c r="E126" s="40"/>
-      <c r="F126" s="40"/>
-      <c r="G126" s="41"/>
-      <c r="H126" s="41"/>
+      <c r="D126" s="38" t="s">
+        <v>194</v>
+      </c>
+      <c r="E126" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F126" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G126" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H126" s="41">
+        <v>1</v>
+      </c>
       <c r="I126" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-0.5</v>
       </c>
       <c r="J126" s="45"/>
       <c r="K126" s="43"/>
     </row>
     <row r="127" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A127" s="37"/>
-      <c r="B127" s="38"/>
+      <c r="A127" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B127" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C127" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D127" s="38"/>
-      <c r="E127" s="40"/>
-      <c r="F127" s="40"/>
-      <c r="G127" s="41"/>
-      <c r="H127" s="41"/>
+      <c r="D127" s="38" t="s">
+        <v>195</v>
+      </c>
+      <c r="E127" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F127" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G127" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H127" s="41">
+        <v>1</v>
+      </c>
       <c r="I127" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-0.5</v>
       </c>
       <c r="J127" s="45"/>
       <c r="K127" s="43"/>
     </row>
     <row r="128" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A128" s="37"/>
-      <c r="B128" s="38"/>
+      <c r="A128" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B128" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C128" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D128" s="38"/>
-      <c r="E128" s="40"/>
-      <c r="F128" s="40"/>
-      <c r="G128" s="41"/>
-      <c r="H128" s="41"/>
+      <c r="D128" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="E128" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F128" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G128" s="41">
+        <v>1</v>
+      </c>
+      <c r="H128" s="41">
+        <v>1.5</v>
+      </c>
       <c r="I128" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>0.5</v>
       </c>
       <c r="J128" s="45"/>
       <c r="K128" s="43"/>
     </row>
     <row r="129" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A129" s="13"/>
-      <c r="B129" s="15"/>
-      <c r="C129" s="15"/>
-      <c r="D129" s="15"/>
-      <c r="E129" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F129" s="15"/>
-      <c r="G129" s="18">
-        <f t="shared" ref="G129:H129" si="7">SUM(G119:G128)</f>
-        <v>0</v>
-      </c>
-      <c r="H129" s="18">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="I129" s="18">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J129" s="19"/>
-      <c r="K129" s="46"/>
-    </row>
-    <row r="130" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="61" t="s">
-        <v>24</v>
-      </c>
-      <c r="B130" s="55"/>
-      <c r="C130" s="55"/>
-      <c r="D130" s="55"/>
-      <c r="E130" s="55"/>
-      <c r="F130" s="55"/>
-      <c r="G130" s="55"/>
-      <c r="H130" s="55"/>
-      <c r="I130" s="55"/>
-      <c r="J130" s="55"/>
-      <c r="K130" s="56"/>
+      <c r="A129" s="37">
+        <v>45635</v>
+      </c>
+      <c r="B129" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C129" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D129" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="E129" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F129" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G129" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H129" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="I129" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J129" s="45"/>
+      <c r="K129" s="43"/>
+    </row>
+    <row r="130" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A130" s="37"/>
+      <c r="B130" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="C130" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D130" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="E130" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F130" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="G130" s="41">
+        <v>4</v>
+      </c>
+      <c r="H130" s="41"/>
+      <c r="I130" s="41">
+        <f t="shared" si="5"/>
+        <v>-4</v>
+      </c>
+      <c r="J130" s="45"/>
+      <c r="K130" s="43"/>
     </row>
     <row r="131" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A131" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B131" s="54" t="s">
-        <v>13</v>
-      </c>
-      <c r="C131" s="55"/>
-      <c r="D131" s="55"/>
-      <c r="E131" s="55"/>
-      <c r="F131" s="55"/>
-      <c r="G131" s="55"/>
-      <c r="H131" s="55"/>
-      <c r="I131" s="55"/>
-      <c r="J131" s="55"/>
-      <c r="K131" s="56"/>
-    </row>
-    <row r="132" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B132" s="54" t="s">
-        <v>15</v>
-      </c>
-      <c r="C132" s="55"/>
-      <c r="D132" s="55"/>
-      <c r="E132" s="55"/>
-      <c r="F132" s="55"/>
-      <c r="G132" s="55"/>
-      <c r="H132" s="55"/>
-      <c r="I132" s="55"/>
-      <c r="J132" s="55"/>
-      <c r="K132" s="56"/>
+      <c r="A131" s="37"/>
+      <c r="B131" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="C131" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D131" s="38" t="s">
+        <v>197</v>
+      </c>
+      <c r="E131" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F131" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="G131" s="41">
+        <v>2</v>
+      </c>
+      <c r="H131" s="41"/>
+      <c r="I131" s="41">
+        <f t="shared" si="5"/>
+        <v>-2</v>
+      </c>
+      <c r="J131" s="45"/>
+      <c r="K131" s="43"/>
+    </row>
+    <row r="132" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A132" s="37">
+        <v>45637</v>
+      </c>
+      <c r="B132" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C132" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D132" s="38" t="s">
+        <v>199</v>
+      </c>
+      <c r="E132" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F132" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G132" s="41">
+        <v>4</v>
+      </c>
+      <c r="H132" s="41"/>
+      <c r="I132" s="41">
+        <f t="shared" si="5"/>
+        <v>-4</v>
+      </c>
+      <c r="J132" s="45"/>
+      <c r="K132" s="43" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="133" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A133" s="37"/>
-      <c r="B133" s="38"/>
+      <c r="B133" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C133" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D133" s="38"/>
-      <c r="E133" s="40"/>
-      <c r="F133" s="40"/>
-      <c r="G133" s="41"/>
+      <c r="D133" s="38" t="s">
+        <v>200</v>
+      </c>
+      <c r="E133" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F133" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="G133" s="41">
+        <v>2</v>
+      </c>
       <c r="H133" s="41"/>
       <c r="I133" s="41">
-        <f t="shared" ref="I133:I143" si="8">H133-G133</f>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-2</v>
       </c>
       <c r="J133" s="45"/>
       <c r="K133" s="43"/>
     </row>
     <row r="134" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A134" s="37"/>
-      <c r="B134" s="38"/>
+      <c r="B134" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C134" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D134" s="38"/>
-      <c r="E134" s="40"/>
-      <c r="F134" s="40"/>
-      <c r="G134" s="41"/>
+      <c r="D134" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="E134" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F134" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G134" s="41">
+        <v>1</v>
+      </c>
       <c r="H134" s="41"/>
       <c r="I134" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-1</v>
       </c>
       <c r="J134" s="45"/>
       <c r="K134" s="43"/>
     </row>
     <row r="135" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A135" s="37"/>
-      <c r="B135" s="38"/>
+      <c r="A135" s="37">
+        <v>45638</v>
+      </c>
+      <c r="B135" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C135" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D135" s="38"/>
-      <c r="E135" s="40"/>
-      <c r="F135" s="40"/>
-      <c r="G135" s="41"/>
-      <c r="H135" s="41"/>
+      <c r="D135" s="38" t="s">
+        <v>207</v>
+      </c>
+      <c r="E135" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F135" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G135" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H135" s="41">
+        <v>1</v>
+      </c>
       <c r="I135" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-0.5</v>
       </c>
       <c r="J135" s="45"/>
-      <c r="K135" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K135" s="43"/>
     </row>
     <row r="136" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A136" s="37"/>
-      <c r="B136" s="38"/>
+      <c r="A136" s="37">
+        <v>45638</v>
+      </c>
+      <c r="B136" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C136" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D136" s="38"/>
-      <c r="E136" s="40"/>
-      <c r="F136" s="40"/>
-      <c r="G136" s="41"/>
-      <c r="H136" s="41"/>
+      <c r="D136" s="38" t="s">
+        <v>206</v>
+      </c>
+      <c r="E136" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F136" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G136" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H136" s="41">
+        <v>1</v>
+      </c>
       <c r="I136" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-0.5</v>
       </c>
       <c r="J136" s="45"/>
       <c r="K136" s="43"/>
     </row>
     <row r="137" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A137" s="37"/>
-      <c r="B137" s="38"/>
+      <c r="A137" s="37">
+        <v>45638</v>
+      </c>
+      <c r="B137" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C137" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D137" s="38"/>
-      <c r="E137" s="40"/>
-      <c r="F137" s="40"/>
-      <c r="G137" s="41"/>
-      <c r="H137" s="41"/>
+      <c r="D137" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="E137" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F137" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G137" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H137" s="41">
+        <v>1</v>
+      </c>
       <c r="I137" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-0.5</v>
       </c>
       <c r="J137" s="45"/>
       <c r="K137" s="43"/>
     </row>
     <row r="138" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A138" s="37"/>
-      <c r="B138" s="38"/>
+      <c r="A138" s="37">
+        <v>45638</v>
+      </c>
+      <c r="B138" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C138" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D138" s="38"/>
-      <c r="E138" s="40"/>
-      <c r="F138" s="40"/>
-      <c r="G138" s="41"/>
-      <c r="H138" s="41"/>
+      <c r="D138" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="E138" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F138" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G138" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H138" s="41">
+        <v>1</v>
+      </c>
       <c r="I138" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-0.5</v>
       </c>
       <c r="J138" s="45"/>
       <c r="K138" s="43"/>
     </row>
     <row r="139" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A139" s="37"/>
-      <c r="B139" s="38"/>
+      <c r="A139" s="37">
+        <v>45638</v>
+      </c>
+      <c r="B139" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C139" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D139" s="38"/>
-      <c r="E139" s="40"/>
-      <c r="F139" s="40"/>
-      <c r="G139" s="41"/>
-      <c r="H139" s="41"/>
+      <c r="D139" s="38" t="s">
+        <v>203</v>
+      </c>
+      <c r="E139" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F139" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G139" s="41">
+        <v>1.5</v>
+      </c>
+      <c r="H139" s="41">
+        <v>1</v>
+      </c>
       <c r="I139" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>-0.5</v>
       </c>
       <c r="J139" s="45"/>
       <c r="K139" s="43"/>
     </row>
     <row r="140" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A140" s="37"/>
-      <c r="B140" s="38"/>
+      <c r="A140" s="37">
+        <v>45638</v>
+      </c>
+      <c r="B140" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C140" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D140" s="38"/>
-      <c r="E140" s="40"/>
-      <c r="F140" s="40"/>
-      <c r="G140" s="41"/>
-      <c r="H140" s="41"/>
+      <c r="D140" s="38" t="s">
+        <v>208</v>
+      </c>
+      <c r="E140" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F140" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G140" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H140" s="41">
+        <v>1</v>
+      </c>
       <c r="I140" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>0.5</v>
       </c>
       <c r="J140" s="45"/>
       <c r="K140" s="43"/>
     </row>
     <row r="141" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A141" s="37"/>
-      <c r="B141" s="38"/>
+      <c r="A141" s="37">
+        <v>45638</v>
+      </c>
+      <c r="B141" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C141" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D141" s="38"/>
-      <c r="E141" s="40"/>
-      <c r="F141" s="40"/>
-      <c r="G141" s="41"/>
-      <c r="H141" s="41"/>
+      <c r="D141" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="E141" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F141" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G141" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H141" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I141" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J141" s="45"/>
       <c r="K141" s="43"/>
     </row>
     <row r="142" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A142" s="37"/>
-      <c r="B142" s="38"/>
+      <c r="A142" s="37">
+        <v>45639</v>
+      </c>
+      <c r="B142" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C142" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D142" s="38"/>
-      <c r="E142" s="40"/>
-      <c r="F142" s="40"/>
-      <c r="G142" s="41"/>
-      <c r="H142" s="41"/>
+      <c r="D142" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="E142" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F142" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G142" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H142" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I142" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J142" s="45"/>
       <c r="K142" s="43"/>
     </row>
     <row r="143" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A143" s="13"/>
-      <c r="B143" s="15"/>
-      <c r="C143" s="15"/>
-      <c r="D143" s="15"/>
-      <c r="E143" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F143" s="15"/>
-      <c r="G143" s="18">
-        <f t="shared" ref="G143:H143" si="9">SUM(G133:G142)</f>
-        <v>0</v>
-      </c>
-      <c r="H143" s="18">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="I143" s="18">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J143" s="19"/>
-      <c r="K143" s="46"/>
-    </row>
-    <row r="144" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="57" t="s">
-        <v>26</v>
-      </c>
-      <c r="B144" s="55"/>
-      <c r="C144" s="55"/>
-      <c r="D144" s="55"/>
-      <c r="E144" s="55"/>
-      <c r="F144" s="55"/>
-      <c r="G144" s="55"/>
-      <c r="H144" s="55"/>
-      <c r="I144" s="55"/>
-      <c r="J144" s="55"/>
-      <c r="K144" s="56"/>
+      <c r="A143" s="37">
+        <v>45639</v>
+      </c>
+      <c r="B143" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C143" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D143" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="E143" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F143" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="G143" s="41">
+        <v>4</v>
+      </c>
+      <c r="H143" s="41"/>
+      <c r="I143" s="41">
+        <f t="shared" si="5"/>
+        <v>-4</v>
+      </c>
+      <c r="J143" s="45"/>
+      <c r="K143" s="43"/>
+    </row>
+    <row r="144" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A144" s="37">
+        <v>45639</v>
+      </c>
+      <c r="B144" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C144" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D144" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="E144" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F144" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G144" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H144" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="I144" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J144" s="45"/>
+      <c r="K144" s="43"/>
     </row>
     <row r="145" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A145" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B145" s="75" t="s">
-        <v>13</v>
-      </c>
-      <c r="C145" s="55"/>
-      <c r="D145" s="55"/>
-      <c r="E145" s="55"/>
-      <c r="F145" s="55"/>
-      <c r="G145" s="55"/>
-      <c r="H145" s="55"/>
-      <c r="I145" s="55"/>
-      <c r="J145" s="55"/>
-      <c r="K145" s="56"/>
-    </row>
-    <row r="146" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B146" s="75" t="s">
-        <v>15</v>
-      </c>
-      <c r="C146" s="55"/>
-      <c r="D146" s="55"/>
-      <c r="E146" s="55"/>
-      <c r="F146" s="55"/>
-      <c r="G146" s="55"/>
-      <c r="H146" s="55"/>
-      <c r="I146" s="55"/>
-      <c r="J146" s="55"/>
-      <c r="K146" s="56"/>
+      <c r="A145" s="37">
+        <v>45639</v>
+      </c>
+      <c r="B145" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C145" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D145" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="E145" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F145" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="G145" s="41">
+        <v>1</v>
+      </c>
+      <c r="H145" s="41"/>
+      <c r="I145" s="41">
+        <f t="shared" si="5"/>
+        <v>-1</v>
+      </c>
+      <c r="J145" s="45"/>
+      <c r="K145" s="43"/>
+    </row>
+    <row r="146" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A146" s="37">
+        <v>45639</v>
+      </c>
+      <c r="B146" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C146" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D146" s="38" t="s">
+        <v>211</v>
+      </c>
+      <c r="E146" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F146" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G146" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H146" s="41"/>
+      <c r="I146" s="41">
+        <f t="shared" si="5"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J146" s="45"/>
+      <c r="K146" s="43"/>
     </row>
     <row r="147" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A147" s="37"/>
@@ -5533,7 +6221,7 @@
       <c r="G147" s="41"/>
       <c r="H147" s="41"/>
       <c r="I147" s="41">
-        <f t="shared" ref="I147:I157" si="10">H147-G147</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J147" s="45"/>
@@ -5551,83 +6239,84 @@
       <c r="G148" s="41"/>
       <c r="H148" s="41"/>
       <c r="I148" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J148" s="45"/>
       <c r="K148" s="43"/>
     </row>
     <row r="149" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A149" s="37"/>
-      <c r="B149" s="38"/>
-      <c r="C149" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D149" s="38"/>
-      <c r="E149" s="40"/>
-      <c r="F149" s="40"/>
-      <c r="G149" s="41"/>
-      <c r="H149" s="41"/>
-      <c r="I149" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J149" s="45"/>
-      <c r="K149" s="43"/>
-    </row>
-    <row r="150" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A150" s="37"/>
-      <c r="B150" s="38"/>
-      <c r="C150" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D150" s="38"/>
-      <c r="E150" s="40"/>
-      <c r="F150" s="40"/>
-      <c r="G150" s="41"/>
-      <c r="H150" s="41"/>
-      <c r="I150" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J150" s="45"/>
-      <c r="K150" s="43"/>
+      <c r="A149" s="13"/>
+      <c r="B149" s="15"/>
+      <c r="C149" s="15"/>
+      <c r="D149" s="15"/>
+      <c r="E149" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F149" s="15"/>
+      <c r="G149" s="18">
+        <f>SUM(G121:G148)</f>
+        <v>37</v>
+      </c>
+      <c r="H149" s="18">
+        <f>SUM(H121:H148)</f>
+        <v>15.25</v>
+      </c>
+      <c r="I149" s="18">
+        <f t="shared" si="5"/>
+        <v>-21.75</v>
+      </c>
+      <c r="J149" s="19"/>
+      <c r="K149" s="46"/>
+    </row>
+    <row r="150" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="73" t="s">
+        <v>23</v>
+      </c>
+      <c r="B150" s="62"/>
+      <c r="C150" s="62"/>
+      <c r="D150" s="62"/>
+      <c r="E150" s="62"/>
+      <c r="F150" s="62"/>
+      <c r="G150" s="62"/>
+      <c r="H150" s="62"/>
+      <c r="I150" s="62"/>
+      <c r="J150" s="62"/>
+      <c r="K150" s="63"/>
     </row>
     <row r="151" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A151" s="37"/>
-      <c r="B151" s="38"/>
-      <c r="C151" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D151" s="38"/>
-      <c r="E151" s="40"/>
-      <c r="F151" s="40"/>
-      <c r="G151" s="41"/>
-      <c r="H151" s="41"/>
-      <c r="I151" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J151" s="45"/>
-      <c r="K151" s="43"/>
-    </row>
-    <row r="152" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A152" s="37"/>
-      <c r="B152" s="38"/>
-      <c r="C152" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D152" s="38"/>
-      <c r="E152" s="40"/>
-      <c r="F152" s="40"/>
-      <c r="G152" s="41"/>
-      <c r="H152" s="41"/>
-      <c r="I152" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J152" s="45"/>
-      <c r="K152" s="43"/>
+      <c r="A151" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B151" s="74" t="s">
+        <v>13</v>
+      </c>
+      <c r="C151" s="62"/>
+      <c r="D151" s="62"/>
+      <c r="E151" s="62"/>
+      <c r="F151" s="62"/>
+      <c r="G151" s="62"/>
+      <c r="H151" s="62"/>
+      <c r="I151" s="62"/>
+      <c r="J151" s="62"/>
+      <c r="K151" s="63"/>
+    </row>
+    <row r="152" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B152" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="C152" s="62"/>
+      <c r="D152" s="62"/>
+      <c r="E152" s="62"/>
+      <c r="F152" s="62"/>
+      <c r="G152" s="62"/>
+      <c r="H152" s="62"/>
+      <c r="I152" s="62"/>
+      <c r="J152" s="62"/>
+      <c r="K152" s="63"/>
     </row>
     <row r="153" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A153" s="37"/>
@@ -5641,7 +6330,7 @@
       <c r="G153" s="41"/>
       <c r="H153" s="41"/>
       <c r="I153" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I153:I163" si="6">H153-G153</f>
         <v>0</v>
       </c>
       <c r="J153" s="45"/>
@@ -5659,7 +6348,7 @@
       <c r="G154" s="41"/>
       <c r="H154" s="41"/>
       <c r="I154" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J154" s="45"/>
@@ -5677,7 +6366,7 @@
       <c r="G155" s="41"/>
       <c r="H155" s="41"/>
       <c r="I155" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J155" s="45"/>
@@ -5695,84 +6384,83 @@
       <c r="G156" s="41"/>
       <c r="H156" s="41"/>
       <c r="I156" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J156" s="45"/>
       <c r="K156" s="43"/>
     </row>
     <row r="157" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A157" s="13"/>
-      <c r="B157" s="15"/>
-      <c r="C157" s="15"/>
-      <c r="D157" s="15"/>
-      <c r="E157" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F157" s="15"/>
-      <c r="G157" s="18">
-        <f t="shared" ref="G157:H157" si="11">SUM(G147:G156)</f>
-        <v>0</v>
-      </c>
-      <c r="H157" s="18">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I157" s="18">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J157" s="19"/>
-      <c r="K157" s="46"/>
-    </row>
-    <row r="158" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="62" t="s">
-        <v>27</v>
-      </c>
-      <c r="B158" s="63"/>
-      <c r="C158" s="63"/>
-      <c r="D158" s="63"/>
-      <c r="E158" s="63"/>
-      <c r="F158" s="63"/>
-      <c r="G158" s="63"/>
-      <c r="H158" s="63"/>
-      <c r="I158" s="63"/>
-      <c r="J158" s="63"/>
-      <c r="K158" s="64"/>
+      <c r="A157" s="37"/>
+      <c r="B157" s="38"/>
+      <c r="C157" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D157" s="38"/>
+      <c r="E157" s="40"/>
+      <c r="F157" s="40"/>
+      <c r="G157" s="41"/>
+      <c r="H157" s="41"/>
+      <c r="I157" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J157" s="45"/>
+      <c r="K157" s="43"/>
+    </row>
+    <row r="158" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A158" s="37"/>
+      <c r="B158" s="38"/>
+      <c r="C158" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D158" s="38"/>
+      <c r="E158" s="40"/>
+      <c r="F158" s="40"/>
+      <c r="G158" s="41"/>
+      <c r="H158" s="41"/>
+      <c r="I158" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J158" s="45"/>
+      <c r="K158" s="43"/>
     </row>
     <row r="159" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A159" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B159" s="65" t="s">
-        <v>13</v>
-      </c>
-      <c r="C159" s="63"/>
-      <c r="D159" s="63"/>
-      <c r="E159" s="63"/>
-      <c r="F159" s="63"/>
-      <c r="G159" s="63"/>
-      <c r="H159" s="63"/>
-      <c r="I159" s="63"/>
-      <c r="J159" s="63"/>
-      <c r="K159" s="64"/>
-    </row>
-    <row r="160" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A160" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B160" s="65" t="s">
-        <v>15</v>
-      </c>
-      <c r="C160" s="63"/>
-      <c r="D160" s="63"/>
-      <c r="E160" s="63"/>
-      <c r="F160" s="63"/>
-      <c r="G160" s="63"/>
-      <c r="H160" s="63"/>
-      <c r="I160" s="63"/>
-      <c r="J160" s="63"/>
-      <c r="K160" s="64"/>
+      <c r="A159" s="37"/>
+      <c r="B159" s="38"/>
+      <c r="C159" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D159" s="38"/>
+      <c r="E159" s="40"/>
+      <c r="F159" s="40"/>
+      <c r="G159" s="41"/>
+      <c r="H159" s="41"/>
+      <c r="I159" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J159" s="45"/>
+      <c r="K159" s="43"/>
+    </row>
+    <row r="160" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A160" s="37"/>
+      <c r="B160" s="38"/>
+      <c r="C160" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D160" s="38"/>
+      <c r="E160" s="40"/>
+      <c r="F160" s="40"/>
+      <c r="G160" s="41"/>
+      <c r="H160" s="41"/>
+      <c r="I160" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J160" s="45"/>
+      <c r="K160" s="43"/>
     </row>
     <row r="161" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A161" s="37"/>
@@ -5786,7 +6474,7 @@
       <c r="G161" s="41"/>
       <c r="H161" s="41"/>
       <c r="I161" s="41">
-        <f t="shared" ref="I161:I171" si="12">H161-G161</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J161" s="45"/>
@@ -5804,83 +6492,84 @@
       <c r="G162" s="41"/>
       <c r="H162" s="41"/>
       <c r="I162" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J162" s="45"/>
       <c r="K162" s="43"/>
     </row>
     <row r="163" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A163" s="37"/>
-      <c r="B163" s="38"/>
-      <c r="C163" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D163" s="38"/>
-      <c r="E163" s="40"/>
-      <c r="F163" s="40"/>
-      <c r="G163" s="41"/>
-      <c r="H163" s="41"/>
-      <c r="I163" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J163" s="45"/>
-      <c r="K163" s="43"/>
-    </row>
-    <row r="164" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A164" s="37"/>
-      <c r="B164" s="38"/>
-      <c r="C164" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D164" s="38"/>
-      <c r="E164" s="40"/>
-      <c r="F164" s="40"/>
-      <c r="G164" s="41"/>
-      <c r="H164" s="41"/>
-      <c r="I164" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J164" s="45"/>
-      <c r="K164" s="43"/>
+      <c r="A163" s="13"/>
+      <c r="B163" s="15"/>
+      <c r="C163" s="15"/>
+      <c r="D163" s="15"/>
+      <c r="E163" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F163" s="15"/>
+      <c r="G163" s="18">
+        <f t="shared" ref="G163:H163" si="7">SUM(G153:G162)</f>
+        <v>0</v>
+      </c>
+      <c r="H163" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="I163" s="18">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J163" s="19"/>
+      <c r="K163" s="46"/>
+    </row>
+    <row r="164" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="B164" s="62"/>
+      <c r="C164" s="62"/>
+      <c r="D164" s="62"/>
+      <c r="E164" s="62"/>
+      <c r="F164" s="62"/>
+      <c r="G164" s="62"/>
+      <c r="H164" s="62"/>
+      <c r="I164" s="62"/>
+      <c r="J164" s="62"/>
+      <c r="K164" s="63"/>
     </row>
     <row r="165" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A165" s="37"/>
-      <c r="B165" s="38"/>
-      <c r="C165" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D165" s="38"/>
-      <c r="E165" s="40"/>
-      <c r="F165" s="40"/>
-      <c r="G165" s="41"/>
-      <c r="H165" s="41"/>
-      <c r="I165" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J165" s="45"/>
-      <c r="K165" s="43"/>
-    </row>
-    <row r="166" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A166" s="37"/>
-      <c r="B166" s="38"/>
-      <c r="C166" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D166" s="38"/>
-      <c r="E166" s="40"/>
-      <c r="F166" s="40"/>
-      <c r="G166" s="41"/>
-      <c r="H166" s="41"/>
-      <c r="I166" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J166" s="45"/>
-      <c r="K166" s="43"/>
+      <c r="A165" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B165" s="71" t="s">
+        <v>13</v>
+      </c>
+      <c r="C165" s="62"/>
+      <c r="D165" s="62"/>
+      <c r="E165" s="62"/>
+      <c r="F165" s="62"/>
+      <c r="G165" s="62"/>
+      <c r="H165" s="62"/>
+      <c r="I165" s="62"/>
+      <c r="J165" s="62"/>
+      <c r="K165" s="63"/>
+    </row>
+    <row r="166" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B166" s="71" t="s">
+        <v>15</v>
+      </c>
+      <c r="C166" s="62"/>
+      <c r="D166" s="62"/>
+      <c r="E166" s="62"/>
+      <c r="F166" s="62"/>
+      <c r="G166" s="62"/>
+      <c r="H166" s="62"/>
+      <c r="I166" s="62"/>
+      <c r="J166" s="62"/>
+      <c r="K166" s="63"/>
     </row>
     <row r="167" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A167" s="37"/>
@@ -5894,7 +6583,7 @@
       <c r="G167" s="41"/>
       <c r="H167" s="41"/>
       <c r="I167" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="I167:I177" si="8">H167-G167</f>
         <v>0</v>
       </c>
       <c r="J167" s="45"/>
@@ -5912,7 +6601,7 @@
       <c r="G168" s="41"/>
       <c r="H168" s="41"/>
       <c r="I168" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J168" s="45"/>
@@ -5930,11 +6619,13 @@
       <c r="G169" s="41"/>
       <c r="H169" s="41"/>
       <c r="I169" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J169" s="45"/>
-      <c r="K169" s="43"/>
+      <c r="K169" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="170" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A170" s="37"/>
@@ -5948,42 +6639,656 @@
       <c r="G170" s="41"/>
       <c r="H170" s="41"/>
       <c r="I170" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J170" s="45"/>
       <c r="K170" s="43"/>
     </row>
     <row r="171" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A171" s="48"/>
-      <c r="B171" s="49"/>
-      <c r="C171" s="49"/>
-      <c r="D171" s="49"/>
-      <c r="E171" s="49" t="s">
+      <c r="A171" s="37"/>
+      <c r="B171" s="38"/>
+      <c r="C171" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D171" s="38"/>
+      <c r="E171" s="40"/>
+      <c r="F171" s="40"/>
+      <c r="G171" s="41"/>
+      <c r="H171" s="41"/>
+      <c r="I171" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J171" s="45"/>
+      <c r="K171" s="43"/>
+    </row>
+    <row r="172" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A172" s="37"/>
+      <c r="B172" s="38"/>
+      <c r="C172" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D172" s="38"/>
+      <c r="E172" s="40"/>
+      <c r="F172" s="40"/>
+      <c r="G172" s="41"/>
+      <c r="H172" s="41"/>
+      <c r="I172" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J172" s="45"/>
+      <c r="K172" s="43"/>
+    </row>
+    <row r="173" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A173" s="37"/>
+      <c r="B173" s="38"/>
+      <c r="C173" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D173" s="38"/>
+      <c r="E173" s="40"/>
+      <c r="F173" s="40"/>
+      <c r="G173" s="41"/>
+      <c r="H173" s="41"/>
+      <c r="I173" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J173" s="45"/>
+      <c r="K173" s="43"/>
+    </row>
+    <row r="174" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A174" s="37"/>
+      <c r="B174" s="38"/>
+      <c r="C174" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D174" s="38"/>
+      <c r="E174" s="40"/>
+      <c r="F174" s="40"/>
+      <c r="G174" s="41"/>
+      <c r="H174" s="41"/>
+      <c r="I174" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J174" s="45"/>
+      <c r="K174" s="43"/>
+    </row>
+    <row r="175" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A175" s="37"/>
+      <c r="B175" s="38"/>
+      <c r="C175" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D175" s="38"/>
+      <c r="E175" s="40"/>
+      <c r="F175" s="40"/>
+      <c r="G175" s="41"/>
+      <c r="H175" s="41"/>
+      <c r="I175" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J175" s="45"/>
+      <c r="K175" s="43"/>
+    </row>
+    <row r="176" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A176" s="37"/>
+      <c r="B176" s="38"/>
+      <c r="C176" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D176" s="38"/>
+      <c r="E176" s="40"/>
+      <c r="F176" s="40"/>
+      <c r="G176" s="41"/>
+      <c r="H176" s="41"/>
+      <c r="I176" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J176" s="45"/>
+      <c r="K176" s="43"/>
+    </row>
+    <row r="177" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A177" s="13"/>
+      <c r="B177" s="15"/>
+      <c r="C177" s="15"/>
+      <c r="D177" s="15"/>
+      <c r="E177" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F171" s="49"/>
-      <c r="G171" s="50">
-        <f t="shared" ref="G171:H171" si="13">SUM(G161:G170)</f>
-        <v>0</v>
-      </c>
-      <c r="H171" s="50">
+      <c r="F177" s="15"/>
+      <c r="G177" s="18">
+        <f t="shared" ref="G177:H177" si="9">SUM(G167:G176)</f>
+        <v>0</v>
+      </c>
+      <c r="H177" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="I177" s="18">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J177" s="19"/>
+      <c r="K177" s="46"/>
+    </row>
+    <row r="178" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="B178" s="62"/>
+      <c r="C178" s="62"/>
+      <c r="D178" s="62"/>
+      <c r="E178" s="62"/>
+      <c r="F178" s="62"/>
+      <c r="G178" s="62"/>
+      <c r="H178" s="62"/>
+      <c r="I178" s="62"/>
+      <c r="J178" s="62"/>
+      <c r="K178" s="63"/>
+    </row>
+    <row r="179" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A179" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B179" s="69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C179" s="62"/>
+      <c r="D179" s="62"/>
+      <c r="E179" s="62"/>
+      <c r="F179" s="62"/>
+      <c r="G179" s="62"/>
+      <c r="H179" s="62"/>
+      <c r="I179" s="62"/>
+      <c r="J179" s="62"/>
+      <c r="K179" s="63"/>
+    </row>
+    <row r="180" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B180" s="69" t="s">
+        <v>15</v>
+      </c>
+      <c r="C180" s="62"/>
+      <c r="D180" s="62"/>
+      <c r="E180" s="62"/>
+      <c r="F180" s="62"/>
+      <c r="G180" s="62"/>
+      <c r="H180" s="62"/>
+      <c r="I180" s="62"/>
+      <c r="J180" s="62"/>
+      <c r="K180" s="63"/>
+    </row>
+    <row r="181" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A181" s="37"/>
+      <c r="B181" s="38"/>
+      <c r="C181" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D181" s="38"/>
+      <c r="E181" s="40"/>
+      <c r="F181" s="40"/>
+      <c r="G181" s="41"/>
+      <c r="H181" s="41"/>
+      <c r="I181" s="41">
+        <f t="shared" ref="I181:I191" si="10">H181-G181</f>
+        <v>0</v>
+      </c>
+      <c r="J181" s="45"/>
+      <c r="K181" s="43"/>
+    </row>
+    <row r="182" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A182" s="37"/>
+      <c r="B182" s="38"/>
+      <c r="C182" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D182" s="38"/>
+      <c r="E182" s="40"/>
+      <c r="F182" s="40"/>
+      <c r="G182" s="41"/>
+      <c r="H182" s="41"/>
+      <c r="I182" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J182" s="45"/>
+      <c r="K182" s="43"/>
+    </row>
+    <row r="183" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A183" s="37"/>
+      <c r="B183" s="38"/>
+      <c r="C183" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D183" s="38"/>
+      <c r="E183" s="40"/>
+      <c r="F183" s="40"/>
+      <c r="G183" s="41"/>
+      <c r="H183" s="41"/>
+      <c r="I183" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J183" s="45"/>
+      <c r="K183" s="43"/>
+    </row>
+    <row r="184" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A184" s="37"/>
+      <c r="B184" s="38"/>
+      <c r="C184" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D184" s="38"/>
+      <c r="E184" s="40"/>
+      <c r="F184" s="40"/>
+      <c r="G184" s="41"/>
+      <c r="H184" s="41"/>
+      <c r="I184" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J184" s="45"/>
+      <c r="K184" s="43"/>
+    </row>
+    <row r="185" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A185" s="37"/>
+      <c r="B185" s="38"/>
+      <c r="C185" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D185" s="38"/>
+      <c r="E185" s="40"/>
+      <c r="F185" s="40"/>
+      <c r="G185" s="41"/>
+      <c r="H185" s="41"/>
+      <c r="I185" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J185" s="45"/>
+      <c r="K185" s="43"/>
+    </row>
+    <row r="186" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A186" s="37"/>
+      <c r="B186" s="38"/>
+      <c r="C186" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D186" s="38"/>
+      <c r="E186" s="40"/>
+      <c r="F186" s="40"/>
+      <c r="G186" s="41"/>
+      <c r="H186" s="41"/>
+      <c r="I186" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J186" s="45"/>
+      <c r="K186" s="43"/>
+    </row>
+    <row r="187" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A187" s="37"/>
+      <c r="B187" s="38"/>
+      <c r="C187" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D187" s="38"/>
+      <c r="E187" s="40"/>
+      <c r="F187" s="40"/>
+      <c r="G187" s="41"/>
+      <c r="H187" s="41"/>
+      <c r="I187" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J187" s="45"/>
+      <c r="K187" s="43"/>
+    </row>
+    <row r="188" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A188" s="37"/>
+      <c r="B188" s="38"/>
+      <c r="C188" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D188" s="38"/>
+      <c r="E188" s="40"/>
+      <c r="F188" s="40"/>
+      <c r="G188" s="41"/>
+      <c r="H188" s="41"/>
+      <c r="I188" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J188" s="45"/>
+      <c r="K188" s="43"/>
+    </row>
+    <row r="189" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A189" s="37"/>
+      <c r="B189" s="38"/>
+      <c r="C189" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D189" s="38"/>
+      <c r="E189" s="40"/>
+      <c r="F189" s="40"/>
+      <c r="G189" s="41"/>
+      <c r="H189" s="41"/>
+      <c r="I189" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J189" s="45"/>
+      <c r="K189" s="43"/>
+    </row>
+    <row r="190" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A190" s="37"/>
+      <c r="B190" s="38"/>
+      <c r="C190" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D190" s="38"/>
+      <c r="E190" s="40"/>
+      <c r="F190" s="40"/>
+      <c r="G190" s="41"/>
+      <c r="H190" s="41"/>
+      <c r="I190" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J190" s="45"/>
+      <c r="K190" s="43"/>
+    </row>
+    <row r="191" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A191" s="13"/>
+      <c r="B191" s="15"/>
+      <c r="C191" s="15"/>
+      <c r="D191" s="15"/>
+      <c r="E191" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F191" s="15"/>
+      <c r="G191" s="18">
+        <f t="shared" ref="G191:H191" si="11">SUM(G181:G190)</f>
+        <v>0</v>
+      </c>
+      <c r="H191" s="18">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="I191" s="18">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J191" s="19"/>
+      <c r="K191" s="46"/>
+    </row>
+    <row r="192" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="54" t="s">
+        <v>27</v>
+      </c>
+      <c r="B192" s="55"/>
+      <c r="C192" s="55"/>
+      <c r="D192" s="55"/>
+      <c r="E192" s="55"/>
+      <c r="F192" s="55"/>
+      <c r="G192" s="55"/>
+      <c r="H192" s="55"/>
+      <c r="I192" s="55"/>
+      <c r="J192" s="55"/>
+      <c r="K192" s="56"/>
+    </row>
+    <row r="193" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A193" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B193" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C193" s="55"/>
+      <c r="D193" s="55"/>
+      <c r="E193" s="55"/>
+      <c r="F193" s="55"/>
+      <c r="G193" s="55"/>
+      <c r="H193" s="55"/>
+      <c r="I193" s="55"/>
+      <c r="J193" s="55"/>
+      <c r="K193" s="56"/>
+    </row>
+    <row r="194" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B194" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C194" s="55"/>
+      <c r="D194" s="55"/>
+      <c r="E194" s="55"/>
+      <c r="F194" s="55"/>
+      <c r="G194" s="55"/>
+      <c r="H194" s="55"/>
+      <c r="I194" s="55"/>
+      <c r="J194" s="55"/>
+      <c r="K194" s="56"/>
+    </row>
+    <row r="195" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A195" s="37"/>
+      <c r="B195" s="38"/>
+      <c r="C195" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D195" s="38"/>
+      <c r="E195" s="40"/>
+      <c r="F195" s="40"/>
+      <c r="G195" s="41"/>
+      <c r="H195" s="41"/>
+      <c r="I195" s="41">
+        <f t="shared" ref="I195:I205" si="12">H195-G195</f>
+        <v>0</v>
+      </c>
+      <c r="J195" s="45"/>
+      <c r="K195" s="43"/>
+    </row>
+    <row r="196" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A196" s="37"/>
+      <c r="B196" s="38"/>
+      <c r="C196" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D196" s="38"/>
+      <c r="E196" s="40"/>
+      <c r="F196" s="40"/>
+      <c r="G196" s="41"/>
+      <c r="H196" s="41"/>
+      <c r="I196" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J196" s="45"/>
+      <c r="K196" s="43"/>
+    </row>
+    <row r="197" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A197" s="37"/>
+      <c r="B197" s="38"/>
+      <c r="C197" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D197" s="38"/>
+      <c r="E197" s="40"/>
+      <c r="F197" s="40"/>
+      <c r="G197" s="41"/>
+      <c r="H197" s="41"/>
+      <c r="I197" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J197" s="45"/>
+      <c r="K197" s="43"/>
+    </row>
+    <row r="198" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A198" s="37"/>
+      <c r="B198" s="38"/>
+      <c r="C198" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D198" s="38"/>
+      <c r="E198" s="40"/>
+      <c r="F198" s="40"/>
+      <c r="G198" s="41"/>
+      <c r="H198" s="41"/>
+      <c r="I198" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J198" s="45"/>
+      <c r="K198" s="43"/>
+    </row>
+    <row r="199" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A199" s="37"/>
+      <c r="B199" s="38"/>
+      <c r="C199" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D199" s="38"/>
+      <c r="E199" s="40"/>
+      <c r="F199" s="40"/>
+      <c r="G199" s="41"/>
+      <c r="H199" s="41"/>
+      <c r="I199" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J199" s="45"/>
+      <c r="K199" s="43"/>
+    </row>
+    <row r="200" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A200" s="37"/>
+      <c r="B200" s="38"/>
+      <c r="C200" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D200" s="38"/>
+      <c r="E200" s="40"/>
+      <c r="F200" s="40"/>
+      <c r="G200" s="41"/>
+      <c r="H200" s="41"/>
+      <c r="I200" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J200" s="45"/>
+      <c r="K200" s="43"/>
+    </row>
+    <row r="201" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A201" s="37"/>
+      <c r="B201" s="38"/>
+      <c r="C201" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D201" s="38"/>
+      <c r="E201" s="40"/>
+      <c r="F201" s="40"/>
+      <c r="G201" s="41"/>
+      <c r="H201" s="41"/>
+      <c r="I201" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J201" s="45"/>
+      <c r="K201" s="43"/>
+    </row>
+    <row r="202" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A202" s="37"/>
+      <c r="B202" s="38"/>
+      <c r="C202" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D202" s="38"/>
+      <c r="E202" s="40"/>
+      <c r="F202" s="40"/>
+      <c r="G202" s="41"/>
+      <c r="H202" s="41"/>
+      <c r="I202" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J202" s="45"/>
+      <c r="K202" s="43"/>
+    </row>
+    <row r="203" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A203" s="37"/>
+      <c r="B203" s="38"/>
+      <c r="C203" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D203" s="38"/>
+      <c r="E203" s="40"/>
+      <c r="F203" s="40"/>
+      <c r="G203" s="41"/>
+      <c r="H203" s="41"/>
+      <c r="I203" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J203" s="45"/>
+      <c r="K203" s="43"/>
+    </row>
+    <row r="204" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A204" s="37"/>
+      <c r="B204" s="38"/>
+      <c r="C204" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D204" s="38"/>
+      <c r="E204" s="40"/>
+      <c r="F204" s="40"/>
+      <c r="G204" s="41"/>
+      <c r="H204" s="41"/>
+      <c r="I204" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J204" s="45"/>
+      <c r="K204" s="43"/>
+    </row>
+    <row r="205" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A205" s="48"/>
+      <c r="B205" s="49"/>
+      <c r="C205" s="49"/>
+      <c r="D205" s="49"/>
+      <c r="E205" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="F205" s="49"/>
+      <c r="G205" s="50">
+        <f t="shared" ref="G205:H205" si="13">SUM(G195:G204)</f>
+        <v>0</v>
+      </c>
+      <c r="H205" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="I171" s="50">
+      <c r="I205" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J171" s="51"/>
-      <c r="K171" s="52"/>
+      <c r="J205" s="51"/>
+      <c r="K205" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{7C9185E5-A137-49DC-B738-85C392A73DBD}">
+      <autoFilter ref="A1:K15" xr:uid="{311AD4E8-C18A-4151-99EE-761FEC36C016}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -5994,9 +7299,17 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A158:K158"/>
-    <mergeCell ref="B159:K159"/>
-    <mergeCell ref="B160:K160"/>
+    <mergeCell ref="B165:K165"/>
+    <mergeCell ref="B166:K166"/>
+    <mergeCell ref="A178:K178"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A150:K150"/>
+    <mergeCell ref="B151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="A164:K164"/>
+    <mergeCell ref="A192:K192"/>
+    <mergeCell ref="B193:K193"/>
+    <mergeCell ref="B194:K194"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -6006,20 +7319,12 @@
     <mergeCell ref="A83:K83"/>
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
-    <mergeCell ref="A102:K102"/>
-    <mergeCell ref="B145:K145"/>
-    <mergeCell ref="B146:K146"/>
-    <mergeCell ref="B103:K103"/>
-    <mergeCell ref="B131:K131"/>
-    <mergeCell ref="B132:K132"/>
-    <mergeCell ref="A144:K144"/>
-    <mergeCell ref="B104:K104"/>
-    <mergeCell ref="A116:K116"/>
-    <mergeCell ref="B117:K117"/>
-    <mergeCell ref="B118:K118"/>
-    <mergeCell ref="A130:K130"/>
+    <mergeCell ref="A118:K118"/>
+    <mergeCell ref="B179:K179"/>
+    <mergeCell ref="B180:K180"/>
+    <mergeCell ref="B119:K119"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B100 B105:B114 B119:B128 B133:B142 B147:B156">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B153:B162 B167:B176 B181:B190 B121:B148">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -6036,7 +7341,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B101 B103:B115 B117:B129 B131:B143 B145:B157 B159:B171">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B151:B163 B165:B177 B179:B191 B193:B205 B119:B149">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -6044,34 +7349,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B161:B170">
+  <conditionalFormatting sqref="B195:B204">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B161))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B195))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B161))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B195))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B161))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B195))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B161))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B195))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B161))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B195))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G101 G105:G115 G119:G129 G133:G143 G147:G157 G161:G171">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G153:G163 G167:G177 G181:G191 G195:G205 G121:G149">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H171">
+  <conditionalFormatting sqref="H1:H205">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I101 I105:I115 I119:I129 I133:I143 I147:I157 I161:I171">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I153:I163 I167:I177 I181:I191 I195:I205 I86:I117 I121:I149">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -6080,7 +7385,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F161:F170 F147:F156 F86:F100 F105:F114 F119:F128 F133:F142 F5:F45 F50:F81" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F195:F204 F181:F190 F86:F116 F153:F162 F167:F176 F5:F45 F50:F81 F121:F148" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6096,13 +7401,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E100 E105:E114 E119:E128 E133:E142 E147:E156 E161:E170 E50:E81</xm:sqref>
+          <xm:sqref>E5:E45 E86:E116 E153:E162 E167:E176 E181:E190 E195:E204 E50:E81 E121:E148</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B100 B105:B114 B119:B128 B133:B142 B147:B156 B161:B170 B50:B81</xm:sqref>
+          <xm:sqref>B5:B45 B86:B116 B153:B162 B167:B176 B181:B190 B195:B204 B50:B81 B121:B148</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7743,26 +9048,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -7997,10 +9282,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8017,20 +9333,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W4 DataLab 2 Work II (End)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\OneDrive\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E60ABC6A-4F36-49B8-9EAB-F793030D2FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F191E3-AAD0-474C-8760-5359EE113EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="216">
   <si>
     <t>Date</t>
   </si>
@@ -744,6 +744,12 @@
   </si>
   <si>
     <t>I had done some overlapping work with the previous task so was shorter.</t>
+  </si>
+  <si>
+    <t>Add feedback to week 4 Learning Log</t>
+  </si>
+  <si>
+    <t>11&amp;13-12-2024</t>
   </si>
 </sst>
 </file>
@@ -1229,6 +1235,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1245,8 +1271,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1264,24 +1288,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1806,53 +1812,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3191,53 +3197,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4290,53 +4296,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5351,53 +5357,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="68" t="s">
+      <c r="A118" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="62"/>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
+      <c r="B118" s="55"/>
+      <c r="C118" s="55"/>
+      <c r="D118" s="55"/>
+      <c r="E118" s="55"/>
+      <c r="F118" s="55"/>
+      <c r="G118" s="55"/>
+      <c r="H118" s="55"/>
+      <c r="I118" s="55"/>
+      <c r="J118" s="55"/>
+      <c r="K118" s="56"/>
     </row>
     <row r="119" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="70" t="s">
+      <c r="B119" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="62"/>
-      <c r="D119" s="62"/>
-      <c r="E119" s="62"/>
-      <c r="F119" s="62"/>
-      <c r="G119" s="62"/>
-      <c r="H119" s="62"/>
-      <c r="I119" s="62"/>
-      <c r="J119" s="62"/>
-      <c r="K119" s="63"/>
+      <c r="C119" s="55"/>
+      <c r="D119" s="55"/>
+      <c r="E119" s="55"/>
+      <c r="F119" s="55"/>
+      <c r="G119" s="55"/>
+      <c r="H119" s="55"/>
+      <c r="I119" s="55"/>
+      <c r="J119" s="55"/>
+      <c r="K119" s="56"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="70" t="s">
+      <c r="B120" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="62"/>
-      <c r="D120" s="62"/>
-      <c r="E120" s="62"/>
-      <c r="F120" s="62"/>
-      <c r="G120" s="62"/>
-      <c r="H120" s="62"/>
-      <c r="I120" s="62"/>
-      <c r="J120" s="62"/>
-      <c r="K120" s="63"/>
+      <c r="C120" s="55"/>
+      <c r="D120" s="55"/>
+      <c r="E120" s="55"/>
+      <c r="F120" s="55"/>
+      <c r="G120" s="55"/>
+      <c r="H120" s="55"/>
+      <c r="I120" s="55"/>
+      <c r="J120" s="55"/>
+      <c r="K120" s="56"/>
     </row>
     <row r="121" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -5521,7 +5527,7 @@
         <v>1</v>
       </c>
       <c r="I124" s="41">
-        <f t="shared" ref="I121:I149" si="5">H124-G124</f>
+        <f t="shared" ref="I124:I149" si="5">H124-G124</f>
         <v>-0.5</v>
       </c>
       <c r="J124" s="45"/>
@@ -5744,8 +5750,8 @@
       <c r="K131" s="43"/>
     </row>
     <row r="132" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A132" s="37">
-        <v>45637</v>
+      <c r="A132" s="37" t="s">
+        <v>215</v>
       </c>
       <c r="B132" s="38" t="s">
         <v>52</v>
@@ -6171,10 +6177,12 @@
       <c r="G145" s="41">
         <v>1</v>
       </c>
-      <c r="H145" s="41"/>
+      <c r="H145" s="41">
+        <v>1.45</v>
+      </c>
       <c r="I145" s="41">
         <f t="shared" si="5"/>
-        <v>-1</v>
+        <v>0.44999999999999996</v>
       </c>
       <c r="J145" s="45"/>
       <c r="K145" s="43"/>
@@ -6184,7 +6192,7 @@
         <v>45639</v>
       </c>
       <c r="B146" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C146" s="39" t="s">
         <v>17</v>
@@ -6201,28 +6209,42 @@
       <c r="G146" s="41">
         <v>0.25</v>
       </c>
-      <c r="H146" s="41"/>
+      <c r="H146" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I146" s="41">
         <f t="shared" si="5"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J146" s="45"/>
       <c r="K146" s="43"/>
     </row>
     <row r="147" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A147" s="37"/>
-      <c r="B147" s="38"/>
+      <c r="A147" s="37">
+        <v>45639</v>
+      </c>
+      <c r="B147" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C147" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D147" s="38"/>
-      <c r="E147" s="40"/>
-      <c r="F147" s="40"/>
-      <c r="G147" s="41"/>
+      <c r="D147" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="E147" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F147" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G147" s="41">
+        <v>0.5</v>
+      </c>
       <c r="H147" s="41"/>
       <c r="I147" s="41">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="J147" s="45"/>
       <c r="K147" s="43"/>
@@ -6256,67 +6278,67 @@
       <c r="F149" s="15"/>
       <c r="G149" s="18">
         <f>SUM(G121:G148)</f>
-        <v>37</v>
+        <v>37.5</v>
       </c>
       <c r="H149" s="18">
         <f>SUM(H121:H148)</f>
-        <v>15.25</v>
+        <v>16.95</v>
       </c>
       <c r="I149" s="18">
         <f t="shared" si="5"/>
-        <v>-21.75</v>
+        <v>-20.55</v>
       </c>
       <c r="J149" s="19"/>
       <c r="K149" s="46"/>
     </row>
     <row r="150" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="73" t="s">
+      <c r="A150" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B150" s="62"/>
-      <c r="C150" s="62"/>
-      <c r="D150" s="62"/>
-      <c r="E150" s="62"/>
-      <c r="F150" s="62"/>
-      <c r="G150" s="62"/>
-      <c r="H150" s="62"/>
-      <c r="I150" s="62"/>
-      <c r="J150" s="62"/>
-      <c r="K150" s="63"/>
+      <c r="B150" s="55"/>
+      <c r="C150" s="55"/>
+      <c r="D150" s="55"/>
+      <c r="E150" s="55"/>
+      <c r="F150" s="55"/>
+      <c r="G150" s="55"/>
+      <c r="H150" s="55"/>
+      <c r="I150" s="55"/>
+      <c r="J150" s="55"/>
+      <c r="K150" s="56"/>
     </row>
     <row r="151" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A151" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B151" s="74" t="s">
+      <c r="B151" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C151" s="62"/>
-      <c r="D151" s="62"/>
-      <c r="E151" s="62"/>
-      <c r="F151" s="62"/>
-      <c r="G151" s="62"/>
-      <c r="H151" s="62"/>
-      <c r="I151" s="62"/>
-      <c r="J151" s="62"/>
-      <c r="K151" s="63"/>
+      <c r="C151" s="55"/>
+      <c r="D151" s="55"/>
+      <c r="E151" s="55"/>
+      <c r="F151" s="55"/>
+      <c r="G151" s="55"/>
+      <c r="H151" s="55"/>
+      <c r="I151" s="55"/>
+      <c r="J151" s="55"/>
+      <c r="K151" s="56"/>
     </row>
     <row r="152" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B152" s="74" t="s">
+      <c r="B152" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C152" s="62"/>
-      <c r="D152" s="62"/>
-      <c r="E152" s="62"/>
-      <c r="F152" s="62"/>
-      <c r="G152" s="62"/>
-      <c r="H152" s="62"/>
-      <c r="I152" s="62"/>
-      <c r="J152" s="62"/>
-      <c r="K152" s="63"/>
+      <c r="C152" s="55"/>
+      <c r="D152" s="55"/>
+      <c r="E152" s="55"/>
+      <c r="F152" s="55"/>
+      <c r="G152" s="55"/>
+      <c r="H152" s="55"/>
+      <c r="I152" s="55"/>
+      <c r="J152" s="55"/>
+      <c r="K152" s="56"/>
     </row>
     <row r="153" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A153" s="37"/>
@@ -6523,53 +6545,53 @@
       <c r="K163" s="46"/>
     </row>
     <row r="164" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="75" t="s">
+      <c r="A164" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B164" s="62"/>
-      <c r="C164" s="62"/>
-      <c r="D164" s="62"/>
-      <c r="E164" s="62"/>
-      <c r="F164" s="62"/>
-      <c r="G164" s="62"/>
-      <c r="H164" s="62"/>
-      <c r="I164" s="62"/>
-      <c r="J164" s="62"/>
-      <c r="K164" s="63"/>
+      <c r="B164" s="55"/>
+      <c r="C164" s="55"/>
+      <c r="D164" s="55"/>
+      <c r="E164" s="55"/>
+      <c r="F164" s="55"/>
+      <c r="G164" s="55"/>
+      <c r="H164" s="55"/>
+      <c r="I164" s="55"/>
+      <c r="J164" s="55"/>
+      <c r="K164" s="56"/>
     </row>
     <row r="165" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A165" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B165" s="71" t="s">
+      <c r="B165" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C165" s="62"/>
-      <c r="D165" s="62"/>
-      <c r="E165" s="62"/>
-      <c r="F165" s="62"/>
-      <c r="G165" s="62"/>
-      <c r="H165" s="62"/>
-      <c r="I165" s="62"/>
-      <c r="J165" s="62"/>
-      <c r="K165" s="63"/>
+      <c r="C165" s="55"/>
+      <c r="D165" s="55"/>
+      <c r="E165" s="55"/>
+      <c r="F165" s="55"/>
+      <c r="G165" s="55"/>
+      <c r="H165" s="55"/>
+      <c r="I165" s="55"/>
+      <c r="J165" s="55"/>
+      <c r="K165" s="56"/>
     </row>
     <row r="166" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B166" s="71" t="s">
+      <c r="B166" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C166" s="62"/>
-      <c r="D166" s="62"/>
-      <c r="E166" s="62"/>
-      <c r="F166" s="62"/>
-      <c r="G166" s="62"/>
-      <c r="H166" s="62"/>
-      <c r="I166" s="62"/>
-      <c r="J166" s="62"/>
-      <c r="K166" s="63"/>
+      <c r="C166" s="55"/>
+      <c r="D166" s="55"/>
+      <c r="E166" s="55"/>
+      <c r="F166" s="55"/>
+      <c r="G166" s="55"/>
+      <c r="H166" s="55"/>
+      <c r="I166" s="55"/>
+      <c r="J166" s="55"/>
+      <c r="K166" s="56"/>
     </row>
     <row r="167" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A167" s="37"/>
@@ -6778,53 +6800,53 @@
       <c r="K177" s="46"/>
     </row>
     <row r="178" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A178" s="72" t="s">
+      <c r="A178" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B178" s="62"/>
-      <c r="C178" s="62"/>
-      <c r="D178" s="62"/>
-      <c r="E178" s="62"/>
-      <c r="F178" s="62"/>
-      <c r="G178" s="62"/>
-      <c r="H178" s="62"/>
-      <c r="I178" s="62"/>
-      <c r="J178" s="62"/>
-      <c r="K178" s="63"/>
+      <c r="B178" s="55"/>
+      <c r="C178" s="55"/>
+      <c r="D178" s="55"/>
+      <c r="E178" s="55"/>
+      <c r="F178" s="55"/>
+      <c r="G178" s="55"/>
+      <c r="H178" s="55"/>
+      <c r="I178" s="55"/>
+      <c r="J178" s="55"/>
+      <c r="K178" s="56"/>
     </row>
     <row r="179" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A179" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B179" s="69" t="s">
+      <c r="B179" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C179" s="62"/>
-      <c r="D179" s="62"/>
-      <c r="E179" s="62"/>
-      <c r="F179" s="62"/>
-      <c r="G179" s="62"/>
-      <c r="H179" s="62"/>
-      <c r="I179" s="62"/>
-      <c r="J179" s="62"/>
-      <c r="K179" s="63"/>
+      <c r="C179" s="55"/>
+      <c r="D179" s="55"/>
+      <c r="E179" s="55"/>
+      <c r="F179" s="55"/>
+      <c r="G179" s="55"/>
+      <c r="H179" s="55"/>
+      <c r="I179" s="55"/>
+      <c r="J179" s="55"/>
+      <c r="K179" s="56"/>
     </row>
     <row r="180" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B180" s="69" t="s">
+      <c r="B180" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C180" s="62"/>
-      <c r="D180" s="62"/>
-      <c r="E180" s="62"/>
-      <c r="F180" s="62"/>
-      <c r="G180" s="62"/>
-      <c r="H180" s="62"/>
-      <c r="I180" s="62"/>
-      <c r="J180" s="62"/>
-      <c r="K180" s="63"/>
+      <c r="C180" s="55"/>
+      <c r="D180" s="55"/>
+      <c r="E180" s="55"/>
+      <c r="F180" s="55"/>
+      <c r="G180" s="55"/>
+      <c r="H180" s="55"/>
+      <c r="I180" s="55"/>
+      <c r="J180" s="55"/>
+      <c r="K180" s="56"/>
     </row>
     <row r="181" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A181" s="37"/>
@@ -7031,53 +7053,53 @@
       <c r="K191" s="46"/>
     </row>
     <row r="192" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A192" s="54" t="s">
+      <c r="A192" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B192" s="55"/>
-      <c r="C192" s="55"/>
-      <c r="D192" s="55"/>
-      <c r="E192" s="55"/>
-      <c r="F192" s="55"/>
-      <c r="G192" s="55"/>
-      <c r="H192" s="55"/>
-      <c r="I192" s="55"/>
-      <c r="J192" s="55"/>
-      <c r="K192" s="56"/>
+      <c r="B192" s="63"/>
+      <c r="C192" s="63"/>
+      <c r="D192" s="63"/>
+      <c r="E192" s="63"/>
+      <c r="F192" s="63"/>
+      <c r="G192" s="63"/>
+      <c r="H192" s="63"/>
+      <c r="I192" s="63"/>
+      <c r="J192" s="63"/>
+      <c r="K192" s="64"/>
     </row>
     <row r="193" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A193" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B193" s="57" t="s">
+      <c r="B193" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C193" s="55"/>
-      <c r="D193" s="55"/>
-      <c r="E193" s="55"/>
-      <c r="F193" s="55"/>
-      <c r="G193" s="55"/>
-      <c r="H193" s="55"/>
-      <c r="I193" s="55"/>
-      <c r="J193" s="55"/>
-      <c r="K193" s="56"/>
+      <c r="C193" s="63"/>
+      <c r="D193" s="63"/>
+      <c r="E193" s="63"/>
+      <c r="F193" s="63"/>
+      <c r="G193" s="63"/>
+      <c r="H193" s="63"/>
+      <c r="I193" s="63"/>
+      <c r="J193" s="63"/>
+      <c r="K193" s="64"/>
     </row>
     <row r="194" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B194" s="57" t="s">
+      <c r="B194" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C194" s="55"/>
-      <c r="D194" s="55"/>
-      <c r="E194" s="55"/>
-      <c r="F194" s="55"/>
-      <c r="G194" s="55"/>
-      <c r="H194" s="55"/>
-      <c r="I194" s="55"/>
-      <c r="J194" s="55"/>
-      <c r="K194" s="56"/>
+      <c r="C194" s="63"/>
+      <c r="D194" s="63"/>
+      <c r="E194" s="63"/>
+      <c r="F194" s="63"/>
+      <c r="G194" s="63"/>
+      <c r="H194" s="63"/>
+      <c r="I194" s="63"/>
+      <c r="J194" s="63"/>
+      <c r="K194" s="64"/>
     </row>
     <row r="195" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A195" s="37"/>
@@ -7288,7 +7310,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{311AD4E8-C18A-4151-99EE-761FEC36C016}">
+      <autoFilter ref="A1:K15" xr:uid="{47327E33-8D8B-49A0-88AB-625C74FC497C}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -7299,14 +7321,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B165:K165"/>
-    <mergeCell ref="B166:K166"/>
-    <mergeCell ref="A178:K178"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A150:K150"/>
-    <mergeCell ref="B151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="A164:K164"/>
     <mergeCell ref="A192:K192"/>
     <mergeCell ref="B193:K193"/>
     <mergeCell ref="B194:K194"/>
@@ -7323,8 +7337,16 @@
     <mergeCell ref="B179:K179"/>
     <mergeCell ref="B180:K180"/>
     <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B165:K165"/>
+    <mergeCell ref="B166:K166"/>
+    <mergeCell ref="A178:K178"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A150:K150"/>
+    <mergeCell ref="B151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="A164:K164"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B153:B162 B167:B176 B181:B190 B121:B148">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B148 B153:B162 B167:B176 B181:B190">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -7341,7 +7363,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B151:B163 B165:B177 B179:B191 B193:B205 B119:B149">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B149 B151:B163 B165:B177 B179:B191 B193:B205">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -7366,7 +7388,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B195))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G153:G163 G167:G177 G181:G191 G195:G205 G121:G149">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G149 G153:G163 G167:G177 G181:G191 G195:G205">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
@@ -7376,7 +7398,7 @@
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I153:I163 I167:I177 I181:I191 I195:I205 I86:I117 I121:I149">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I149 I153:I163 I167:I177 I181:I191 I195:I205">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -9048,6 +9070,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -9282,27 +9324,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9319,23 +9360,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W5 DataLab 1 Work II (Pre-Break)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA1A0852-4FB7-445A-8433-923C02F07E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4800F9A-E831-4758-BEA3-F9DED09CDD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$198</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$207</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="281">
   <si>
     <t>Date</t>
   </si>
@@ -380,9 +380,6 @@
     <t>Figure out the GitHub PDF problem</t>
   </si>
   <si>
-    <t>DataLab Task</t>
-  </si>
-  <si>
     <t>For some reason, GitHub refuses to show PDFs on my computer, but on other devices it does work. This is meant to try and fix that. POST-TASK EDIT: Seems to be  a problem with GitHub itself and not my device, and there does nto seem to be a solution.</t>
   </si>
   <si>
@@ -413,12 +410,6 @@
     <t>Install SQL</t>
   </si>
   <si>
-    <t>Stand Up Meeting</t>
-  </si>
-  <si>
-    <t>Plan in WorkLog</t>
-  </si>
-  <si>
     <t>Learn about basic SQL queries</t>
   </si>
   <si>
@@ -620,9 +611,6 @@
     <t>Implement Decision Tree Regression</t>
   </si>
   <si>
-    <t>Follow the lecture</t>
-  </si>
-  <si>
     <t>ILO 6.2</t>
   </si>
   <si>
@@ -816,6 +804,147 @@
   </si>
   <si>
     <t>Semi-supervised learning and label propagation techniques.</t>
+  </si>
+  <si>
+    <t>Do the stand-up meeting with mentor group</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog planning for Tuesday</t>
+  </si>
+  <si>
+    <t>Revising documents</t>
+  </si>
+  <si>
+    <t>Go through the WorkLog and fill in the "Task" column for previous weeks</t>
+  </si>
+  <si>
+    <t>Datalab tasks</t>
+  </si>
+  <si>
+    <t>Follow the k-means clustering tutorial</t>
+  </si>
+  <si>
+    <t>Practice k-means clustering with practice notebook</t>
+  </si>
+  <si>
+    <t>Implement k-means clustering in Python</t>
+  </si>
+  <si>
+    <t>Apply PCA for dimensionality reduction</t>
+  </si>
+  <si>
+    <t>Lecture on regression and classification</t>
+  </si>
+  <si>
+    <t>Prepare for Python retake on Saturday</t>
+  </si>
+  <si>
+    <t>Prepare for Python retake on Sunday</t>
+  </si>
+  <si>
+    <t>Block B Introduction</t>
+  </si>
+  <si>
+    <t>Packages basics</t>
+  </si>
+  <si>
+    <t>Do stand-up meeting with mentor group</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog for week 1</t>
+  </si>
+  <si>
+    <t>Fixing problem</t>
+  </si>
+  <si>
+    <t>Do the Monday datalab task</t>
+  </si>
+  <si>
+    <t>Read chapter 1</t>
+  </si>
+  <si>
+    <t>Plan in WorkLog for Friday</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog for Wednesday/Thursday</t>
+  </si>
+  <si>
+    <t>Stand Up Meeting On Friday With Mentor Group</t>
+  </si>
+  <si>
+    <t>Learning SQL</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog for Monday</t>
+  </si>
+  <si>
+    <t>Read chapter 2</t>
+  </si>
+  <si>
+    <t>Learning Vectors</t>
+  </si>
+  <si>
+    <t>Datalab preparation</t>
+  </si>
+  <si>
+    <t>Recieve Feedback</t>
+  </si>
+  <si>
+    <t>Datalab Tasks</t>
+  </si>
+  <si>
+    <t>Content Review</t>
+  </si>
+  <si>
+    <t>Retake application</t>
+  </si>
+  <si>
+    <t>Read Chapter 3</t>
+  </si>
+  <si>
+    <t>Read Chapter 4</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog for Tuesday</t>
+  </si>
+  <si>
+    <t>Follow the guest lecture</t>
+  </si>
+  <si>
+    <t>Learning Matrices</t>
+  </si>
+  <si>
+    <t>Read chapter 5</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog for Friday</t>
+  </si>
+  <si>
+    <t>Fill in Learning Log for week 4</t>
+  </si>
+  <si>
+    <t>Read chapter 6</t>
+  </si>
+  <si>
+    <t>Learning Calculus</t>
+  </si>
+  <si>
+    <t>Read chapter 7</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog for Fridat</t>
+  </si>
+  <si>
+    <t>Prepare for retake</t>
+  </si>
+  <si>
+    <t>Re-install all programs for Block B on new laptop</t>
+  </si>
+  <si>
+    <t>Installation</t>
+  </si>
+  <si>
+    <t>Had a bit of a problem with VSC not seeing the environment or some of the packages on my new laptop.</t>
   </si>
 </sst>
 </file>
@@ -1826,7 +1955,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K213"/>
+  <dimension ref="A1:K222"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -1934,7 +2063,7 @@
         <v>55</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D5" s="38" t="s">
         <v>70</v>
@@ -1966,7 +2095,7 @@
         <v>55</v>
       </c>
       <c r="C6" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D6" s="38" t="s">
         <v>71</v>
@@ -2000,7 +2129,7 @@
         <v>55</v>
       </c>
       <c r="C7" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D7" s="38" t="s">
         <v>72</v>
@@ -2032,7 +2161,7 @@
         <v>55</v>
       </c>
       <c r="C8" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D8" s="38" t="s">
         <v>73</v>
@@ -2064,7 +2193,7 @@
         <v>55</v>
       </c>
       <c r="C9" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D9" s="38" t="s">
         <v>74</v>
@@ -2096,7 +2225,7 @@
         <v>49</v>
       </c>
       <c r="C10" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D10" s="38" t="s">
         <v>75</v>
@@ -2130,7 +2259,7 @@
         <v>55</v>
       </c>
       <c r="C11" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D11" s="38" t="s">
         <v>76</v>
@@ -2164,7 +2293,7 @@
         <v>55</v>
       </c>
       <c r="C12" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D12" s="38" t="s">
         <v>77</v>
@@ -2196,10 +2325,10 @@
         <v>55</v>
       </c>
       <c r="C13" s="39" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>78</v>
+        <v>248</v>
       </c>
       <c r="E13" s="40" t="s">
         <v>47</v>
@@ -2228,7 +2357,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D14" s="38" t="s">
         <v>79</v>
@@ -2260,10 +2389,10 @@
         <v>55</v>
       </c>
       <c r="C15" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>80</v>
+        <v>249</v>
       </c>
       <c r="E15" s="40" t="s">
         <v>64</v>
@@ -2292,7 +2421,7 @@
         <v>55</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D16" s="38" t="s">
         <v>81</v>
@@ -2324,7 +2453,7 @@
         <v>58</v>
       </c>
       <c r="C17" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D17" s="38" t="s">
         <v>82</v>
@@ -2347,7 +2476,7 @@
       </c>
       <c r="J17" s="45"/>
       <c r="K17" s="44" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -2358,7 +2487,7 @@
         <v>55</v>
       </c>
       <c r="C18" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D18" s="38" t="s">
         <v>83</v>
@@ -2390,7 +2519,7 @@
         <v>55</v>
       </c>
       <c r="C19" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D19" s="38" t="s">
         <v>90</v>
@@ -2422,7 +2551,7 @@
         <v>49</v>
       </c>
       <c r="C20" s="39" t="s">
-        <v>17</v>
+        <v>250</v>
       </c>
       <c r="D20" s="38" t="s">
         <v>91</v>
@@ -2445,7 +2574,7 @@
       </c>
       <c r="J20" s="45"/>
       <c r="K20" s="44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -2456,10 +2585,10 @@
         <v>55</v>
       </c>
       <c r="C21" s="39" t="s">
-        <v>17</v>
+        <v>238</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>92</v>
+        <v>251</v>
       </c>
       <c r="E21" s="40" t="s">
         <v>50</v>
@@ -2488,10 +2617,10 @@
         <v>55</v>
       </c>
       <c r="C22" s="39" t="s">
-        <v>17</v>
+        <v>246</v>
       </c>
       <c r="D22" s="38" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E22" s="40" t="s">
         <v>64</v>
@@ -2520,10 +2649,10 @@
         <v>55</v>
       </c>
       <c r="C23" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D23" s="38" t="s">
-        <v>80</v>
+        <v>254</v>
       </c>
       <c r="E23" s="40" t="s">
         <v>62</v>
@@ -2552,16 +2681,16 @@
         <v>55</v>
       </c>
       <c r="C24" s="39" t="s">
-        <v>17</v>
+        <v>252</v>
       </c>
       <c r="D24" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E24" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F24" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G24" s="41">
         <v>1</v>
@@ -2584,16 +2713,16 @@
         <v>55</v>
       </c>
       <c r="C25" s="39" t="s">
-        <v>17</v>
+        <v>252</v>
       </c>
       <c r="D25" s="38" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E25" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F25" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G25" s="41">
         <v>1</v>
@@ -2616,16 +2745,16 @@
         <v>55</v>
       </c>
       <c r="C26" s="39" t="s">
-        <v>17</v>
+        <v>252</v>
       </c>
       <c r="D26" s="38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E26" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F26" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G26" s="41">
         <v>2</v>
@@ -2648,16 +2777,16 @@
         <v>55</v>
       </c>
       <c r="C27" s="39" t="s">
-        <v>17</v>
+        <v>252</v>
       </c>
       <c r="D27" s="38" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E27" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F27" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G27" s="41">
         <v>2</v>
@@ -2680,16 +2809,16 @@
         <v>55</v>
       </c>
       <c r="C28" s="39" t="s">
-        <v>17</v>
+        <v>252</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E28" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F28" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G28" s="41">
         <v>1</v>
@@ -2712,16 +2841,16 @@
         <v>55</v>
       </c>
       <c r="C29" s="39" t="s">
-        <v>17</v>
+        <v>252</v>
       </c>
       <c r="D29" s="38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E29" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F29" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G29" s="41">
         <v>1</v>
@@ -2734,7 +2863,7 @@
         <v>-0.5</v>
       </c>
       <c r="J29" s="53" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="K29" s="44"/>
     </row>
@@ -2746,10 +2875,10 @@
         <v>55</v>
       </c>
       <c r="C30" s="39" t="s">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="D30" s="38" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E30" s="40" t="s">
         <v>64</v>
@@ -2778,10 +2907,10 @@
         <v>55</v>
       </c>
       <c r="C31" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D31" s="38" t="s">
-        <v>104</v>
+        <v>253</v>
       </c>
       <c r="E31" s="40" t="s">
         <v>62</v>
@@ -2810,10 +2939,10 @@
         <v>55</v>
       </c>
       <c r="C32" s="39" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="D32" s="38" t="s">
-        <v>103</v>
+        <v>255</v>
       </c>
       <c r="E32" s="40" t="s">
         <v>47</v>
@@ -2842,16 +2971,16 @@
         <v>55</v>
       </c>
       <c r="C33" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E33" s="40" t="s">
         <v>47</v>
       </c>
       <c r="F33" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G33" s="41">
         <v>1</v>
@@ -2874,16 +3003,16 @@
         <v>55</v>
       </c>
       <c r="C34" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D34" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E34" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F34" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G34" s="41">
         <v>0.5</v>
@@ -2906,16 +3035,16 @@
         <v>55</v>
       </c>
       <c r="C35" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E35" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F35" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G35" s="41">
         <v>1</v>
@@ -2938,16 +3067,16 @@
         <v>49</v>
       </c>
       <c r="C36" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D36" s="38" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E36" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F36" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G36" s="41">
         <v>0.5</v>
@@ -2961,7 +3090,7 @@
       </c>
       <c r="J36" s="45"/>
       <c r="K36" s="44" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -2972,16 +3101,16 @@
         <v>55</v>
       </c>
       <c r="C37" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D37" s="38" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E37" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F37" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G37" s="41">
         <v>1</v>
@@ -3004,16 +3133,16 @@
         <v>55</v>
       </c>
       <c r="C38" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D38" s="38" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E38" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F38" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G38" s="41">
         <v>1</v>
@@ -3036,16 +3165,16 @@
         <v>61</v>
       </c>
       <c r="C39" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E39" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F39" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G39" s="41">
         <v>1</v>
@@ -3059,7 +3188,7 @@
       </c>
       <c r="J39" s="45"/>
       <c r="K39" s="44" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -3070,16 +3199,16 @@
         <v>55</v>
       </c>
       <c r="C40" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E40" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F40" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G40" s="41">
         <v>4</v>
@@ -3100,16 +3229,16 @@
         <v>43</v>
       </c>
       <c r="C41" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D41" s="38" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E41" s="40" t="s">
         <v>59</v>
       </c>
       <c r="F41" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G41" s="41">
         <v>4</v>
@@ -3128,16 +3257,16 @@
         <v>43</v>
       </c>
       <c r="C42" s="39" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="D42" s="38" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E42" s="40" t="s">
         <v>59</v>
       </c>
       <c r="F42" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G42" s="41">
         <v>4</v>
@@ -3156,10 +3285,10 @@
         <v>43</v>
       </c>
       <c r="C43" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D43" s="38" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E43" s="40" t="s">
         <v>64</v>
@@ -3186,10 +3315,10 @@
         <v>55</v>
       </c>
       <c r="C44" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D44" s="38" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E44" s="40" t="s">
         <v>64</v>
@@ -3216,10 +3345,10 @@
         <v>43</v>
       </c>
       <c r="C45" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D45" s="38" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E45" s="40" t="s">
         <v>64</v>
@@ -3319,10 +3448,10 @@
         <v>55</v>
       </c>
       <c r="C50" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D50" s="38" t="s">
-        <v>80</v>
+        <v>257</v>
       </c>
       <c r="E50" s="40" t="s">
         <v>64</v>
@@ -3351,16 +3480,16 @@
         <v>55</v>
       </c>
       <c r="C51" s="39" t="s">
-        <v>17</v>
+        <v>258</v>
       </c>
       <c r="D51" s="38" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E51" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F51" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G51" s="41">
         <v>1</v>
@@ -3383,16 +3512,16 @@
         <v>55</v>
       </c>
       <c r="C52" s="39" t="s">
-        <v>17</v>
+        <v>258</v>
       </c>
       <c r="D52" s="38" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E52" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F52" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G52" s="41">
         <v>2</v>
@@ -3415,16 +3544,16 @@
         <v>55</v>
       </c>
       <c r="C53" s="39" t="s">
-        <v>17</v>
+        <v>258</v>
       </c>
       <c r="D53" s="38" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E53" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F53" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G53" s="41">
         <v>2</v>
@@ -3447,16 +3576,16 @@
         <v>55</v>
       </c>
       <c r="C54" s="39" t="s">
-        <v>17</v>
+        <v>258</v>
       </c>
       <c r="D54" s="38" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E54" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F54" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G54" s="41">
         <v>1.5</v>
@@ -3479,16 +3608,16 @@
         <v>55</v>
       </c>
       <c r="C55" s="39" t="s">
-        <v>17</v>
+        <v>258</v>
       </c>
       <c r="D55" s="38" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E55" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F55" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G55" s="41">
         <v>1</v>
@@ -3511,16 +3640,16 @@
         <v>55</v>
       </c>
       <c r="C56" s="39" t="s">
-        <v>17</v>
+        <v>258</v>
       </c>
       <c r="D56" s="38" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E56" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F56" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G56" s="41">
         <v>0.5</v>
@@ -3543,10 +3672,10 @@
         <v>55</v>
       </c>
       <c r="C57" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D57" s="38" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E57" s="40" t="s">
         <v>62</v>
@@ -3575,10 +3704,10 @@
         <v>55</v>
       </c>
       <c r="C58" s="39" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="D58" s="38" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E58" s="40" t="s">
         <v>47</v>
@@ -3607,16 +3736,16 @@
         <v>55</v>
       </c>
       <c r="C59" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D59" s="38" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E59" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F59" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G59" s="41">
         <v>0.5</v>
@@ -3630,7 +3759,7 @@
       </c>
       <c r="J59" s="45"/>
       <c r="K59" s="43" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -3641,16 +3770,16 @@
         <v>55</v>
       </c>
       <c r="C60" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D60" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E60" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F60" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G60" s="41">
         <v>0.5</v>
@@ -3673,16 +3802,16 @@
         <v>55</v>
       </c>
       <c r="C61" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D61" s="38" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E61" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F61" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G61" s="41">
         <v>0.5</v>
@@ -3696,7 +3825,7 @@
       </c>
       <c r="J61" s="45"/>
       <c r="K61" s="43" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -3707,16 +3836,16 @@
         <v>55</v>
       </c>
       <c r="C62" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D62" s="38" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E62" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F62" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G62" s="41">
         <v>0.1</v>
@@ -3730,7 +3859,7 @@
       </c>
       <c r="J62" s="45"/>
       <c r="K62" s="43" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -3741,16 +3870,16 @@
         <v>46</v>
       </c>
       <c r="C63" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D63" s="38" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E63" s="40" t="s">
         <v>46</v>
       </c>
       <c r="F63" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G63" s="41">
         <v>0</v>
@@ -3764,7 +3893,7 @@
       </c>
       <c r="J63" s="45"/>
       <c r="K63" s="43" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -3775,16 +3904,16 @@
         <v>55</v>
       </c>
       <c r="C64" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D64" s="38" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E64" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F64" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G64" s="41">
         <v>4</v>
@@ -3807,16 +3936,16 @@
         <v>55</v>
       </c>
       <c r="C65" s="39" t="s">
-        <v>17</v>
+        <v>259</v>
       </c>
       <c r="D65" s="38" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E65" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F65" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G65" s="41">
         <v>3</v>
@@ -3839,16 +3968,16 @@
         <v>55</v>
       </c>
       <c r="C66" s="39" t="s">
-        <v>17</v>
+        <v>259</v>
       </c>
       <c r="D66" s="38" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E66" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F66" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G66" s="41">
         <v>2</v>
@@ -3871,16 +4000,16 @@
         <v>43</v>
       </c>
       <c r="C67" s="39" t="s">
-        <v>17</v>
+        <v>259</v>
       </c>
       <c r="D67" s="38" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E67" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F67" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G67" s="41">
         <v>1</v>
@@ -3901,16 +4030,16 @@
         <v>55</v>
       </c>
       <c r="C68" s="39" t="s">
-        <v>17</v>
+        <v>247</v>
       </c>
       <c r="D68" s="38" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E68" s="40" t="s">
         <v>59</v>
       </c>
       <c r="F68" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G68" s="41">
         <v>4</v>
@@ -3933,16 +4062,16 @@
         <v>55</v>
       </c>
       <c r="C69" s="39" t="s">
-        <v>17</v>
+        <v>260</v>
       </c>
       <c r="D69" s="38" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E69" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F69" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G69" s="41">
         <v>0.25</v>
@@ -3959,22 +4088,22 @@
     </row>
     <row r="70" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A70" s="47" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B70" s="38" t="s">
         <v>55</v>
       </c>
       <c r="C70" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D70" s="38" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E70" s="40" t="s">
         <v>64</v>
       </c>
       <c r="F70" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G70" s="41">
         <v>1</v>
@@ -3997,10 +4126,10 @@
         <v>55</v>
       </c>
       <c r="C71" s="39" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="D71" s="38" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E71" s="40" t="s">
         <v>47</v>
@@ -4029,16 +4158,16 @@
         <v>55</v>
       </c>
       <c r="C72" s="39" t="s">
-        <v>17</v>
+        <v>263</v>
       </c>
       <c r="D72" s="38" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E72" s="40" t="s">
         <v>47</v>
       </c>
       <c r="F72" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G72" s="41">
         <v>0.5</v>
@@ -4061,10 +4190,10 @@
         <v>55</v>
       </c>
       <c r="C73" s="39" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="D73" s="38" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E73" s="40" t="s">
         <v>66</v>
@@ -4093,10 +4222,10 @@
         <v>46</v>
       </c>
       <c r="C74" s="39" t="s">
-        <v>17</v>
+        <v>264</v>
       </c>
       <c r="D74" s="38" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E74" s="40" t="s">
         <v>46</v>
@@ -4125,16 +4254,16 @@
         <v>55</v>
       </c>
       <c r="C75" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D75" s="38" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E75" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F75" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G75" s="41">
         <v>4</v>
@@ -4148,7 +4277,7 @@
       </c>
       <c r="J75" s="45"/>
       <c r="K75" s="43" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="76" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -4159,10 +4288,10 @@
         <v>55</v>
       </c>
       <c r="C76" s="39" t="s">
-        <v>17</v>
+        <v>261</v>
       </c>
       <c r="D76" s="38" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E76" s="40" t="s">
         <v>47</v>
@@ -4191,10 +4320,10 @@
         <v>55</v>
       </c>
       <c r="C77" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D77" s="38" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E77" s="40" t="s">
         <v>64</v>
@@ -4223,10 +4352,10 @@
         <v>55</v>
       </c>
       <c r="C78" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D78" s="38" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E78" s="40" t="s">
         <v>62</v>
@@ -4246,7 +4375,7 @@
       </c>
       <c r="J78" s="45"/>
       <c r="K78" s="43" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="79" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -4257,10 +4386,10 @@
         <v>55</v>
       </c>
       <c r="C79" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D79" s="38" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E79" s="40" t="s">
         <v>62</v>
@@ -4287,10 +4416,10 @@
         <v>43</v>
       </c>
       <c r="C80" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D80" s="38" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E80" s="40" t="s">
         <v>64</v>
@@ -4315,10 +4444,10 @@
         <v>43</v>
       </c>
       <c r="C81" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D81" s="38" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E81" s="40" t="s">
         <v>64</v>
@@ -4418,10 +4547,10 @@
         <v>55</v>
       </c>
       <c r="C86" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D86" s="38" t="s">
-        <v>80</v>
+        <v>257</v>
       </c>
       <c r="E86" s="40" t="s">
         <v>62</v>
@@ -4450,10 +4579,10 @@
         <v>55</v>
       </c>
       <c r="C87" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D87" s="38" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E87" s="40" t="s">
         <v>62</v>
@@ -4482,16 +4611,16 @@
         <v>55</v>
       </c>
       <c r="C88" s="39" t="s">
-        <v>17</v>
+        <v>265</v>
       </c>
       <c r="D88" s="38" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E88" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F88" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G88" s="41">
         <v>2</v>
@@ -4514,16 +4643,16 @@
         <v>55</v>
       </c>
       <c r="C89" s="39" t="s">
-        <v>17</v>
+        <v>265</v>
       </c>
       <c r="D89" s="38" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E89" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F89" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G89" s="41">
         <v>0.5</v>
@@ -4546,16 +4675,16 @@
         <v>55</v>
       </c>
       <c r="C90" s="39" t="s">
-        <v>17</v>
+        <v>265</v>
       </c>
       <c r="D90" s="38" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E90" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F90" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G90" s="41">
         <v>0.5</v>
@@ -4578,16 +4707,16 @@
         <v>55</v>
       </c>
       <c r="C91" s="39" t="s">
-        <v>17</v>
+        <v>266</v>
       </c>
       <c r="D91" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E91" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F91" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G91" s="41">
         <v>4</v>
@@ -4610,16 +4739,16 @@
         <v>55</v>
       </c>
       <c r="C92" s="39" t="s">
-        <v>17</v>
+        <v>266</v>
       </c>
       <c r="D92" s="38" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E92" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F92" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G92" s="41">
         <v>0.5</v>
@@ -4642,16 +4771,16 @@
         <v>55</v>
       </c>
       <c r="C93" s="39" t="s">
-        <v>17</v>
+        <v>266</v>
       </c>
       <c r="D93" s="38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E93" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F93" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G93" s="41">
         <v>0.5</v>
@@ -4665,7 +4794,7 @@
       </c>
       <c r="J93" s="45"/>
       <c r="K93" s="43" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -4676,16 +4805,16 @@
         <v>55</v>
       </c>
       <c r="C94" s="39" t="s">
-        <v>17</v>
+        <v>260</v>
       </c>
       <c r="D94" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E94" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F94" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G94" s="41">
         <v>0.25</v>
@@ -4708,10 +4837,10 @@
         <v>55</v>
       </c>
       <c r="C95" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D95" s="38" t="s">
-        <v>80</v>
+        <v>267</v>
       </c>
       <c r="E95" s="40" t="s">
         <v>62</v>
@@ -4740,10 +4869,10 @@
         <v>55</v>
       </c>
       <c r="C96" s="39" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="D96" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E96" s="40" t="s">
         <v>47</v>
@@ -4772,16 +4901,16 @@
         <v>55</v>
       </c>
       <c r="C97" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D97" s="38" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E97" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F97" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G97" s="41">
         <v>4</v>
@@ -4795,7 +4924,7 @@
       </c>
       <c r="J97" s="45"/>
       <c r="K97" s="43" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -4806,16 +4935,16 @@
         <v>55</v>
       </c>
       <c r="C98" s="39" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="D98" s="38" t="s">
-        <v>172</v>
+        <v>268</v>
       </c>
       <c r="E98" s="40" t="s">
         <v>66</v>
       </c>
       <c r="F98" s="40" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="G98" s="41">
         <v>1</v>
@@ -4838,16 +4967,16 @@
         <v>55</v>
       </c>
       <c r="C99" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D99" s="38" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E99" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F99" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G99" s="41">
         <v>2.5</v>
@@ -4870,16 +4999,16 @@
         <v>55</v>
       </c>
       <c r="C100" s="39" t="s">
-        <v>17</v>
+        <v>269</v>
       </c>
       <c r="D100" s="38" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E100" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F100" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G100" s="41">
         <v>4</v>
@@ -4902,16 +5031,16 @@
         <v>55</v>
       </c>
       <c r="C101" s="39" t="s">
-        <v>17</v>
+        <v>269</v>
       </c>
       <c r="D101" s="38" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E101" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F101" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G101" s="41">
         <v>2</v>
@@ -4934,16 +5063,16 @@
         <v>43</v>
       </c>
       <c r="C102" s="39" t="s">
-        <v>17</v>
+        <v>269</v>
       </c>
       <c r="D102" s="38" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E102" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F102" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G102" s="41">
         <v>1</v>
@@ -4964,16 +5093,16 @@
         <v>55</v>
       </c>
       <c r="C103" s="39" t="s">
-        <v>17</v>
+        <v>270</v>
       </c>
       <c r="D103" s="38" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E103" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F103" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G103" s="41">
         <v>1</v>
@@ -4996,16 +5125,16 @@
         <v>55</v>
       </c>
       <c r="C104" s="39" t="s">
-        <v>17</v>
+        <v>270</v>
       </c>
       <c r="D104" s="38" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E104" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F104" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G104" s="41">
         <v>2</v>
@@ -5028,16 +5157,16 @@
         <v>55</v>
       </c>
       <c r="C105" s="39" t="s">
-        <v>17</v>
+        <v>270</v>
       </c>
       <c r="D105" s="38" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E105" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F105" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G105" s="41">
         <v>1</v>
@@ -5060,16 +5189,16 @@
         <v>55</v>
       </c>
       <c r="C106" s="39" t="s">
-        <v>17</v>
+        <v>270</v>
       </c>
       <c r="D106" s="38" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E106" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F106" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G106" s="41">
         <v>2</v>
@@ -5092,16 +5221,16 @@
         <v>55</v>
       </c>
       <c r="C107" s="39" t="s">
-        <v>17</v>
+        <v>270</v>
       </c>
       <c r="D107" s="38" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="E107" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F107" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G107" s="41">
         <v>1</v>
@@ -5124,16 +5253,16 @@
         <v>55</v>
       </c>
       <c r="C108" s="39" t="s">
-        <v>17</v>
+        <v>270</v>
       </c>
       <c r="D108" s="38" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E108" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F108" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G108" s="41">
         <v>1</v>
@@ -5156,7 +5285,7 @@
         <v>55</v>
       </c>
       <c r="C109" s="39" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="D109" s="38" t="s">
         <v>78</v>
@@ -5188,16 +5317,16 @@
         <v>55</v>
       </c>
       <c r="C110" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D110" s="38" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E110" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F110" s="40" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G110" s="41">
         <v>4</v>
@@ -5220,16 +5349,16 @@
         <v>55</v>
       </c>
       <c r="C111" s="39" t="s">
-        <v>17</v>
+        <v>263</v>
       </c>
       <c r="D111" s="38" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E111" s="40" t="s">
         <v>66</v>
       </c>
       <c r="F111" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G111" s="41">
         <v>1</v>
@@ -5252,16 +5381,16 @@
         <v>55</v>
       </c>
       <c r="C112" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D112" s="38" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E112" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F112" s="40" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G112" s="41">
         <v>2.5</v>
@@ -5275,7 +5404,7 @@
       </c>
       <c r="J112" s="45"/>
       <c r="K112" s="43" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -5286,10 +5415,10 @@
         <v>55</v>
       </c>
       <c r="C113" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D113" s="38" t="s">
-        <v>80</v>
+        <v>271</v>
       </c>
       <c r="E113" s="40" t="s">
         <v>62</v>
@@ -5318,10 +5447,10 @@
         <v>55</v>
       </c>
       <c r="C114" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D114" s="38" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E114" s="40" t="s">
         <v>62</v>
@@ -5348,10 +5477,10 @@
         <v>43</v>
       </c>
       <c r="C115" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D115" s="38" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E115" s="40" t="s">
         <v>64</v>
@@ -5376,10 +5505,10 @@
         <v>43</v>
       </c>
       <c r="C116" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D116" s="38" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="E116" s="40" t="s">
         <v>64</v>
@@ -5479,10 +5608,10 @@
         <v>55</v>
       </c>
       <c r="C121" s="39" t="s">
-        <v>17</v>
+        <v>208</v>
       </c>
       <c r="D121" s="38" t="s">
-        <v>212</v>
+        <v>272</v>
       </c>
       <c r="E121" s="40" t="s">
         <v>62</v>
@@ -5511,10 +5640,10 @@
         <v>55</v>
       </c>
       <c r="C122" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D122" s="38" t="s">
-        <v>80</v>
+        <v>257</v>
       </c>
       <c r="E122" s="40" t="s">
         <v>62</v>
@@ -5543,16 +5672,16 @@
         <v>55</v>
       </c>
       <c r="C123" s="39" t="s">
-        <v>17</v>
+        <v>273</v>
       </c>
       <c r="D123" s="38" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E123" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F123" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G123" s="41">
         <v>1.5</v>
@@ -5575,16 +5704,16 @@
         <v>55</v>
       </c>
       <c r="C124" s="39" t="s">
-        <v>17</v>
+        <v>273</v>
       </c>
       <c r="D124" s="38" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="E124" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F124" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G124" s="41">
         <v>1.5</v>
@@ -5593,7 +5722,7 @@
         <v>1</v>
       </c>
       <c r="I124" s="41">
-        <f t="shared" ref="I124:I149" si="5">H124-G124</f>
+        <f t="shared" ref="I124:I150" si="5">H124-G124</f>
         <v>-0.5</v>
       </c>
       <c r="J124" s="45"/>
@@ -5607,16 +5736,16 @@
         <v>55</v>
       </c>
       <c r="C125" s="39" t="s">
-        <v>17</v>
+        <v>273</v>
       </c>
       <c r="D125" s="38" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E125" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F125" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G125" s="41">
         <v>1.5</v>
@@ -5639,16 +5768,16 @@
         <v>55</v>
       </c>
       <c r="C126" s="39" t="s">
-        <v>17</v>
+        <v>273</v>
       </c>
       <c r="D126" s="38" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E126" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F126" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G126" s="41">
         <v>1.5</v>
@@ -5671,16 +5800,16 @@
         <v>55</v>
       </c>
       <c r="C127" s="39" t="s">
-        <v>17</v>
+        <v>273</v>
       </c>
       <c r="D127" s="38" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E127" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F127" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G127" s="41">
         <v>1.5</v>
@@ -5703,16 +5832,16 @@
         <v>55</v>
       </c>
       <c r="C128" s="39" t="s">
-        <v>17</v>
+        <v>273</v>
       </c>
       <c r="D128" s="38" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E128" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F128" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G128" s="41">
         <v>1</v>
@@ -5735,16 +5864,16 @@
         <v>55</v>
       </c>
       <c r="C129" s="39" t="s">
-        <v>17</v>
+        <v>273</v>
       </c>
       <c r="D129" s="38" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E129" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F129" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G129" s="41">
         <v>0.5</v>
@@ -5765,16 +5894,16 @@
         <v>58</v>
       </c>
       <c r="C130" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D130" s="38" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E130" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F130" s="40" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G130" s="41">
         <v>4</v>
@@ -5793,16 +5922,16 @@
         <v>58</v>
       </c>
       <c r="C131" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D131" s="38" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="E131" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F131" s="40" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G131" s="41">
         <v>2</v>
@@ -5817,22 +5946,22 @@
     </row>
     <row r="132" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A132" s="37" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B132" s="38" t="s">
         <v>52</v>
       </c>
       <c r="C132" s="39" t="s">
-        <v>17</v>
+        <v>274</v>
       </c>
       <c r="D132" s="38" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E132" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F132" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G132" s="41">
         <v>4</v>
@@ -5844,7 +5973,7 @@
       </c>
       <c r="J132" s="45"/>
       <c r="K132" s="43" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="133" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -5853,16 +5982,16 @@
         <v>43</v>
       </c>
       <c r="C133" s="39" t="s">
-        <v>17</v>
+        <v>274</v>
       </c>
       <c r="D133" s="38" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="E133" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F133" s="40" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G133" s="41">
         <v>2</v>
@@ -5881,16 +6010,16 @@
         <v>43</v>
       </c>
       <c r="C134" s="39" t="s">
-        <v>17</v>
+        <v>274</v>
       </c>
       <c r="D134" s="38" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="E134" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F134" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G134" s="41">
         <v>1</v>
@@ -5911,16 +6040,16 @@
         <v>55</v>
       </c>
       <c r="C135" s="39" t="s">
-        <v>17</v>
+        <v>275</v>
       </c>
       <c r="D135" s="38" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="E135" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F135" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G135" s="41">
         <v>1.5</v>
@@ -5943,16 +6072,16 @@
         <v>55</v>
       </c>
       <c r="C136" s="39" t="s">
-        <v>17</v>
+        <v>275</v>
       </c>
       <c r="D136" s="38" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E136" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F136" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G136" s="41">
         <v>1.5</v>
@@ -5975,16 +6104,16 @@
         <v>55</v>
       </c>
       <c r="C137" s="39" t="s">
-        <v>17</v>
+        <v>275</v>
       </c>
       <c r="D137" s="38" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="E137" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F137" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G137" s="41">
         <v>1.5</v>
@@ -6007,16 +6136,16 @@
         <v>55</v>
       </c>
       <c r="C138" s="39" t="s">
-        <v>17</v>
+        <v>275</v>
       </c>
       <c r="D138" s="38" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="E138" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F138" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G138" s="41">
         <v>1.5</v>
@@ -6039,16 +6168,16 @@
         <v>55</v>
       </c>
       <c r="C139" s="39" t="s">
-        <v>17</v>
+        <v>275</v>
       </c>
       <c r="D139" s="38" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="E139" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F139" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G139" s="41">
         <v>1.5</v>
@@ -6071,16 +6200,16 @@
         <v>55</v>
       </c>
       <c r="C140" s="39" t="s">
-        <v>17</v>
+        <v>275</v>
       </c>
       <c r="D140" s="38" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="E140" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F140" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G140" s="41">
         <v>0.5</v>
@@ -6103,16 +6232,16 @@
         <v>55</v>
       </c>
       <c r="C141" s="39" t="s">
-        <v>17</v>
+        <v>275</v>
       </c>
       <c r="D141" s="38" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E141" s="40" t="s">
         <v>56</v>
       </c>
       <c r="F141" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G141" s="41">
         <v>0.5</v>
@@ -6135,7 +6264,7 @@
         <v>55</v>
       </c>
       <c r="C142" s="39" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="D142" s="38" t="s">
         <v>78</v>
@@ -6144,7 +6273,7 @@
         <v>47</v>
       </c>
       <c r="F142" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G142" s="41">
         <v>0.25</v>
@@ -6167,16 +6296,16 @@
         <v>52</v>
       </c>
       <c r="C143" s="39" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="D143" s="38" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E143" s="40" t="s">
         <v>50</v>
       </c>
       <c r="F143" s="40" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G143" s="41">
         <v>4</v>
@@ -6197,10 +6326,10 @@
         <v>55</v>
       </c>
       <c r="C144" s="39" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="D144" s="38" t="s">
-        <v>80</v>
+        <v>276</v>
       </c>
       <c r="E144" s="40" t="s">
         <v>62</v>
@@ -6229,16 +6358,16 @@
         <v>55</v>
       </c>
       <c r="C145" s="39" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="D145" s="38" t="s">
-        <v>66</v>
+        <v>243</v>
       </c>
       <c r="E145" s="40" t="s">
         <v>66</v>
       </c>
       <c r="F145" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G145" s="41">
         <v>1</v>
@@ -6261,10 +6390,10 @@
         <v>55</v>
       </c>
       <c r="C146" s="39" t="s">
-        <v>17</v>
+        <v>261</v>
       </c>
       <c r="D146" s="38" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E146" s="40" t="s">
         <v>47</v>
@@ -6287,45 +6416,61 @@
     </row>
     <row r="147" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A147" s="37">
-        <v>45639</v>
+        <v>45640</v>
       </c>
       <c r="B147" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C147" s="39" t="s">
-        <v>17</v>
+        <v>277</v>
       </c>
       <c r="D147" s="38" t="s">
-        <v>214</v>
+        <v>244</v>
       </c>
       <c r="E147" s="40" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="F147" s="40" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G147" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="H147" s="41"/>
+        <v>2</v>
+      </c>
+      <c r="H147" s="41">
+        <v>2</v>
+      </c>
       <c r="I147" s="41">
         <f t="shared" si="5"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J147" s="45"/>
       <c r="K147" s="43"/>
     </row>
     <row r="148" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A148" s="37"/>
-      <c r="B148" s="38"/>
+      <c r="A148" s="37">
+        <v>45641</v>
+      </c>
+      <c r="B148" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C148" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D148" s="38"/>
-      <c r="E148" s="40"/>
-      <c r="F148" s="40"/>
-      <c r="G148" s="41"/>
-      <c r="H148" s="41"/>
+        <v>277</v>
+      </c>
+      <c r="D148" s="38" t="s">
+        <v>245</v>
+      </c>
+      <c r="E148" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F148" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="G148" s="41">
+        <v>3</v>
+      </c>
+      <c r="H148" s="41">
+        <v>3</v>
+      </c>
       <c r="I148" s="41">
         <f t="shared" si="5"/>
         <v>0</v>
@@ -6334,51 +6479,66 @@
       <c r="K148" s="43"/>
     </row>
     <row r="149" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A149" s="13"/>
-      <c r="B149" s="15"/>
-      <c r="C149" s="15"/>
-      <c r="D149" s="15"/>
-      <c r="E149" s="15" t="s">
+      <c r="A149" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B149" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C149" s="39" t="s">
+        <v>208</v>
+      </c>
+      <c r="D149" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="E149" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F149" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G149" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H149" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="I149" s="41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J149" s="45"/>
+      <c r="K149" s="43"/>
+    </row>
+    <row r="150" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A150" s="13"/>
+      <c r="B150" s="15"/>
+      <c r="C150" s="15"/>
+      <c r="D150" s="15"/>
+      <c r="E150" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F149" s="15"/>
-      <c r="G149" s="18">
-        <f>SUM(G121:G148)</f>
-        <v>37.5</v>
-      </c>
-      <c r="H149" s="18">
-        <f>SUM(H121:H148)</f>
-        <v>16.95</v>
-      </c>
-      <c r="I149" s="18">
+      <c r="F150" s="15"/>
+      <c r="G150" s="18">
+        <f>SUM(G121:G149)</f>
+        <v>42.5</v>
+      </c>
+      <c r="H150" s="18">
+        <f>SUM(H121:H149)</f>
+        <v>22.45</v>
+      </c>
+      <c r="I150" s="18">
         <f t="shared" si="5"/>
-        <v>-20.55</v>
-      </c>
-      <c r="J149" s="19"/>
-      <c r="K149" s="46"/>
-    </row>
-    <row r="150" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="73" t="s">
+        <v>-20.05</v>
+      </c>
+      <c r="J150" s="19"/>
+      <c r="K150" s="46"/>
+    </row>
+    <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B150" s="62"/>
-      <c r="C150" s="62"/>
-      <c r="D150" s="62"/>
-      <c r="E150" s="62"/>
-      <c r="F150" s="62"/>
-      <c r="G150" s="62"/>
-      <c r="H150" s="62"/>
-      <c r="I150" s="62"/>
-      <c r="J150" s="62"/>
-      <c r="K150" s="63"/>
-    </row>
-    <row r="151" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A151" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B151" s="74" t="s">
-        <v>13</v>
-      </c>
+      <c r="B151" s="62"/>
       <c r="C151" s="62"/>
       <c r="D151" s="62"/>
       <c r="E151" s="62"/>
@@ -6389,12 +6549,12 @@
       <c r="J151" s="62"/>
       <c r="K151" s="63"/>
     </row>
-    <row r="152" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="26" t="s">
-        <v>14</v>
+    <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A152" s="25" t="s">
+        <v>12</v>
       </c>
       <c r="B152" s="74" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C152" s="62"/>
       <c r="D152" s="62"/>
@@ -6406,37 +6566,22 @@
       <c r="J152" s="62"/>
       <c r="K152" s="63"/>
     </row>
-    <row r="153" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A153" s="37">
-        <v>45642</v>
-      </c>
-      <c r="B153" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="C153" s="39" t="s">
-        <v>80</v>
-      </c>
-      <c r="D153" s="38" t="s">
-        <v>216</v>
-      </c>
-      <c r="E153" s="40" t="s">
-        <v>62</v>
-      </c>
-      <c r="F153" s="40" t="s">
-        <v>87</v>
-      </c>
-      <c r="G153" s="41">
-        <v>0.25</v>
-      </c>
-      <c r="H153" s="41">
-        <v>0.25</v>
-      </c>
-      <c r="I153" s="41">
-        <f t="shared" ref="I153:I171" si="6">H153-G153</f>
-        <v>0</v>
-      </c>
-      <c r="J153" s="45"/>
-      <c r="K153" s="43"/>
+    <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B153" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="C153" s="62"/>
+      <c r="D153" s="62"/>
+      <c r="E153" s="62"/>
+      <c r="F153" s="62"/>
+      <c r="G153" s="62"/>
+      <c r="H153" s="62"/>
+      <c r="I153" s="62"/>
+      <c r="J153" s="62"/>
+      <c r="K153" s="63"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -6446,16 +6591,16 @@
         <v>55</v>
       </c>
       <c r="C154" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D154" s="38" t="s">
         <v>212</v>
-      </c>
-      <c r="D154" s="38" t="s">
-        <v>217</v>
       </c>
       <c r="E154" s="40" t="s">
         <v>62</v>
       </c>
       <c r="F154" s="40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G154" s="41">
         <v>0.25</v>
@@ -6464,7 +6609,7 @@
         <v>0.25</v>
       </c>
       <c r="I154" s="41">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="I154:I180" si="6">H154-G154</f>
         <v>0</v>
       </c>
       <c r="J154" s="45"/>
@@ -6478,22 +6623,22 @@
         <v>55</v>
       </c>
       <c r="C155" s="39" t="s">
-        <v>229</v>
+        <v>208</v>
       </c>
       <c r="D155" s="38" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E155" s="40" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F155" s="40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G155" s="41">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="H155" s="41">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="I155" s="41">
         <f t="shared" si="6"/>
@@ -6510,26 +6655,26 @@
         <v>55</v>
       </c>
       <c r="C156" s="39" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="D156" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="E156" s="40" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="F156" s="40" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="G156" s="41">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H156" s="41">
         <v>1</v>
       </c>
       <c r="I156" s="41">
         <f t="shared" si="6"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J156" s="45"/>
       <c r="K156" s="43"/>
@@ -6542,26 +6687,26 @@
         <v>55</v>
       </c>
       <c r="C157" s="39" t="s">
-        <v>219</v>
+        <v>279</v>
       </c>
       <c r="D157" s="38" t="s">
-        <v>221</v>
+        <v>278</v>
       </c>
       <c r="E157" s="40" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="F157" s="40" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="G157" s="41">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="H157" s="41">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="I157" s="41">
         <f t="shared" si="6"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J157" s="45"/>
       <c r="K157" s="43"/>
@@ -6574,22 +6719,22 @@
         <v>55</v>
       </c>
       <c r="C158" s="39" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D158" s="38" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="E158" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F158" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G158" s="41">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H158" s="41">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I158" s="41">
         <f t="shared" si="6"/>
@@ -6606,16 +6751,16 @@
         <v>55</v>
       </c>
       <c r="C159" s="39" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D159" s="38" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="E159" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F159" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G159" s="41">
         <v>2</v>
@@ -6638,26 +6783,26 @@
         <v>55</v>
       </c>
       <c r="C160" s="39" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="D160" s="38" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="E160" s="40" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="F160" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G160" s="41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H160" s="41">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I160" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="J160" s="45"/>
       <c r="K160" s="43"/>
@@ -6670,26 +6815,26 @@
         <v>55</v>
       </c>
       <c r="C161" s="39" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="D161" s="38" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="E161" s="40" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="F161" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G161" s="41">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="H161" s="41">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="I161" s="41">
         <f t="shared" si="6"/>
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="J161" s="45"/>
       <c r="K161" s="43"/>
@@ -6702,22 +6847,22 @@
         <v>55</v>
       </c>
       <c r="C162" s="39" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="D162" s="38" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="E162" s="40" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F162" s="40" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="G162" s="41">
-        <v>0.16</v>
+        <v>1</v>
       </c>
       <c r="H162" s="41">
-        <v>0.16</v>
+        <v>1</v>
       </c>
       <c r="I162" s="41">
         <f t="shared" si="6"/>
@@ -6734,26 +6879,26 @@
         <v>55</v>
       </c>
       <c r="C163" s="39" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="D163" s="38" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="E163" s="40" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="F163" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G163" s="41">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H163" s="41">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="I163" s="41">
         <f t="shared" si="6"/>
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="J163" s="45"/>
       <c r="K163" s="43"/>
@@ -6766,26 +6911,26 @@
         <v>55</v>
       </c>
       <c r="C164" s="39" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="D164" s="38" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="E164" s="40" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="F164" s="40" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="G164" s="41">
-        <v>2</v>
+        <v>0.16</v>
       </c>
       <c r="H164" s="41">
-        <v>1</v>
+        <v>0.16</v>
       </c>
       <c r="I164" s="41">
         <f t="shared" si="6"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J164" s="45"/>
       <c r="K164" s="43"/>
@@ -6798,26 +6943,26 @@
         <v>55</v>
       </c>
       <c r="C165" s="39" t="s">
+        <v>226</v>
+      </c>
+      <c r="D165" s="38" t="s">
         <v>230</v>
-      </c>
-      <c r="D165" s="38" t="s">
-        <v>236</v>
       </c>
       <c r="E165" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F165" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G165" s="41">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H165" s="41">
         <v>1</v>
       </c>
       <c r="I165" s="41">
         <f t="shared" si="6"/>
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="J165" s="45"/>
       <c r="K165" s="43"/>
@@ -6830,16 +6975,16 @@
         <v>55</v>
       </c>
       <c r="C166" s="39" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D166" s="38" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="E166" s="40" t="s">
         <v>67</v>
       </c>
       <c r="F166" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G166" s="41">
         <v>2</v>
@@ -6862,26 +7007,26 @@
         <v>55</v>
       </c>
       <c r="C167" s="39" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="D167" s="38" t="s">
         <v>232</v>
       </c>
       <c r="E167" s="40" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="F167" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G167" s="41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H167" s="41">
         <v>1</v>
       </c>
       <c r="I167" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J167" s="45"/>
       <c r="K167" s="43"/>
@@ -6894,39 +7039,55 @@
         <v>55</v>
       </c>
       <c r="C168" s="39" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="D168" s="38" t="s">
         <v>233</v>
       </c>
       <c r="E168" s="40" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="F168" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G168" s="41">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="H168" s="41">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I168" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J168" s="45"/>
       <c r="K168" s="43"/>
     </row>
     <row r="169" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A169" s="37"/>
-      <c r="B169" s="38"/>
-      <c r="C169" s="39"/>
-      <c r="D169" s="38"/>
-      <c r="E169" s="40"/>
-      <c r="F169" s="40"/>
-      <c r="G169" s="41"/>
-      <c r="H169" s="41"/>
+      <c r="A169" s="37">
+        <v>45642</v>
+      </c>
+      <c r="B169" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C169" s="39" t="s">
+        <v>227</v>
+      </c>
+      <c r="D169" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="E169" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F169" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="G169" s="41">
+        <v>1</v>
+      </c>
+      <c r="H169" s="41">
+        <v>1</v>
+      </c>
       <c r="I169" s="41">
         <f t="shared" si="6"/>
         <v>0</v>
@@ -6935,16 +7096,30 @@
       <c r="K169" s="43"/>
     </row>
     <row r="170" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A170" s="37"/>
-      <c r="B170" s="38"/>
+      <c r="A170" s="37">
+        <v>45642</v>
+      </c>
+      <c r="B170" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C170" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D170" s="38"/>
-      <c r="E170" s="40"/>
-      <c r="F170" s="40"/>
-      <c r="G170" s="41"/>
-      <c r="H170" s="41"/>
+        <v>227</v>
+      </c>
+      <c r="D170" s="38" t="s">
+        <v>229</v>
+      </c>
+      <c r="E170" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F170" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="G170" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H170" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I170" s="41">
         <f t="shared" si="6"/>
         <v>0</v>
@@ -6953,147 +7128,236 @@
       <c r="K170" s="43"/>
     </row>
     <row r="171" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A171" s="13"/>
-      <c r="B171" s="15"/>
-      <c r="C171" s="15"/>
-      <c r="D171" s="15"/>
-      <c r="E171" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F171" s="15"/>
-      <c r="G171" s="18">
-        <f t="shared" ref="G171:H171" si="7">SUM(G153:G170)</f>
-        <v>19.66</v>
-      </c>
-      <c r="H171" s="18">
-        <f t="shared" si="7"/>
-        <v>13.91</v>
-      </c>
-      <c r="I171" s="18">
+      <c r="A171" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B171" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C171" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D171" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="E171" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F171" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G171" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H171" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="I171" s="41">
         <f t="shared" si="6"/>
-        <v>-5.75</v>
-      </c>
-      <c r="J171" s="19"/>
-      <c r="K171" s="46"/>
-    </row>
-    <row r="172" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A172" s="75" t="s">
-        <v>24</v>
-      </c>
-      <c r="B172" s="62"/>
-      <c r="C172" s="62"/>
-      <c r="D172" s="62"/>
-      <c r="E172" s="62"/>
-      <c r="F172" s="62"/>
-      <c r="G172" s="62"/>
-      <c r="H172" s="62"/>
-      <c r="I172" s="62"/>
-      <c r="J172" s="62"/>
-      <c r="K172" s="63"/>
+        <v>0</v>
+      </c>
+      <c r="J171" s="45"/>
+      <c r="K171" s="43"/>
+    </row>
+    <row r="172" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A172" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B172" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C172" s="39" t="s">
+        <v>78</v>
+      </c>
+      <c r="D172" s="38" t="s">
+        <v>234</v>
+      </c>
+      <c r="E172" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F172" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G172" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H172" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="I172" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J172" s="45"/>
+      <c r="K172" s="43"/>
     </row>
     <row r="173" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A173" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B173" s="71" t="s">
-        <v>13</v>
-      </c>
-      <c r="C173" s="62"/>
-      <c r="D173" s="62"/>
-      <c r="E173" s="62"/>
-      <c r="F173" s="62"/>
-      <c r="G173" s="62"/>
-      <c r="H173" s="62"/>
-      <c r="I173" s="62"/>
-      <c r="J173" s="62"/>
-      <c r="K173" s="63"/>
-    </row>
-    <row r="174" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A174" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B174" s="71" t="s">
-        <v>15</v>
-      </c>
-      <c r="C174" s="62"/>
-      <c r="D174" s="62"/>
-      <c r="E174" s="62"/>
-      <c r="F174" s="62"/>
-      <c r="G174" s="62"/>
-      <c r="H174" s="62"/>
-      <c r="I174" s="62"/>
-      <c r="J174" s="62"/>
-      <c r="K174" s="63"/>
+      <c r="A173" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B173" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C173" s="39" t="s">
+        <v>236</v>
+      </c>
+      <c r="D173" s="38" t="s">
+        <v>237</v>
+      </c>
+      <c r="E173" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F173" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G173" s="41">
+        <v>1</v>
+      </c>
+      <c r="H173" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="I173" s="41">
+        <f t="shared" si="6"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J173" s="45"/>
+      <c r="K173" s="43"/>
+    </row>
+    <row r="174" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A174" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B174" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C174" s="39" t="s">
+        <v>238</v>
+      </c>
+      <c r="D174" s="38" t="s">
+        <v>239</v>
+      </c>
+      <c r="E174" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F174" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="G174" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H174" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="I174" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J174" s="45"/>
+      <c r="K174" s="43"/>
     </row>
     <row r="175" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A175" s="37"/>
-      <c r="B175" s="38"/>
+      <c r="A175" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B175" s="38" t="s">
+        <v>52</v>
+      </c>
       <c r="C175" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D175" s="38"/>
-      <c r="E175" s="40"/>
-      <c r="F175" s="40"/>
-      <c r="G175" s="41"/>
+        <v>238</v>
+      </c>
+      <c r="D175" s="38" t="s">
+        <v>240</v>
+      </c>
+      <c r="E175" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="F175" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G175" s="41">
+        <v>1</v>
+      </c>
       <c r="H175" s="41"/>
       <c r="I175" s="41">
-        <f t="shared" ref="I175:I185" si="8">H175-G175</f>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>-1</v>
       </c>
       <c r="J175" s="45"/>
-      <c r="K175" s="43"/>
+      <c r="K175" s="43" t="s">
+        <v>280</v>
+      </c>
     </row>
     <row r="176" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A176" s="37"/>
-      <c r="B176" s="38"/>
+      <c r="A176" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B176" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C176" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D176" s="38"/>
-      <c r="E176" s="40"/>
-      <c r="F176" s="40"/>
-      <c r="G176" s="41"/>
+        <v>238</v>
+      </c>
+      <c r="D176" s="38" t="s">
+        <v>241</v>
+      </c>
+      <c r="E176" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F176" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G176" s="41">
+        <v>2</v>
+      </c>
       <c r="H176" s="41"/>
       <c r="I176" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>-2</v>
       </c>
       <c r="J176" s="45"/>
       <c r="K176" s="43"/>
     </row>
     <row r="177" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A177" s="37"/>
-      <c r="B177" s="38"/>
+      <c r="A177" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B177" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C177" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D177" s="38"/>
-      <c r="E177" s="40"/>
-      <c r="F177" s="40"/>
-      <c r="G177" s="41"/>
+        <v>238</v>
+      </c>
+      <c r="D177" s="38" t="s">
+        <v>242</v>
+      </c>
+      <c r="E177" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F177" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G177" s="41">
+        <v>2</v>
+      </c>
       <c r="H177" s="41"/>
       <c r="I177" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>-2</v>
       </c>
       <c r="J177" s="45"/>
-      <c r="K177" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K177" s="43"/>
     </row>
     <row r="178" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A178" s="37"/>
       <c r="B178" s="38"/>
-      <c r="C178" s="39" t="s">
-        <v>17</v>
-      </c>
+      <c r="C178" s="39"/>
       <c r="D178" s="38"/>
       <c r="E178" s="40"/>
       <c r="F178" s="40"/>
       <c r="G178" s="41"/>
       <c r="H178" s="41"/>
       <c r="I178" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J178" s="45"/>
@@ -7111,83 +7375,84 @@
       <c r="G179" s="41"/>
       <c r="H179" s="41"/>
       <c r="I179" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J179" s="45"/>
       <c r="K179" s="43"/>
     </row>
     <row r="180" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A180" s="37"/>
-      <c r="B180" s="38"/>
-      <c r="C180" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D180" s="38"/>
-      <c r="E180" s="40"/>
-      <c r="F180" s="40"/>
-      <c r="G180" s="41"/>
-      <c r="H180" s="41"/>
-      <c r="I180" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J180" s="45"/>
-      <c r="K180" s="43"/>
-    </row>
-    <row r="181" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A181" s="37"/>
-      <c r="B181" s="38"/>
-      <c r="C181" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D181" s="38"/>
-      <c r="E181" s="40"/>
-      <c r="F181" s="40"/>
-      <c r="G181" s="41"/>
-      <c r="H181" s="41"/>
-      <c r="I181" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J181" s="45"/>
-      <c r="K181" s="43"/>
+      <c r="A180" s="13"/>
+      <c r="B180" s="15"/>
+      <c r="C180" s="15"/>
+      <c r="D180" s="15"/>
+      <c r="E180" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F180" s="15"/>
+      <c r="G180" s="18">
+        <f t="shared" ref="G180:H180" si="7">SUM(G154:G179)</f>
+        <v>27.16</v>
+      </c>
+      <c r="H180" s="18">
+        <f t="shared" si="7"/>
+        <v>15.91</v>
+      </c>
+      <c r="I180" s="18">
+        <f t="shared" si="6"/>
+        <v>-11.25</v>
+      </c>
+      <c r="J180" s="19"/>
+      <c r="K180" s="46"/>
+    </row>
+    <row r="181" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="B181" s="62"/>
+      <c r="C181" s="62"/>
+      <c r="D181" s="62"/>
+      <c r="E181" s="62"/>
+      <c r="F181" s="62"/>
+      <c r="G181" s="62"/>
+      <c r="H181" s="62"/>
+      <c r="I181" s="62"/>
+      <c r="J181" s="62"/>
+      <c r="K181" s="63"/>
     </row>
     <row r="182" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A182" s="37"/>
-      <c r="B182" s="38"/>
-      <c r="C182" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D182" s="38"/>
-      <c r="E182" s="40"/>
-      <c r="F182" s="40"/>
-      <c r="G182" s="41"/>
-      <c r="H182" s="41"/>
-      <c r="I182" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J182" s="45"/>
-      <c r="K182" s="43"/>
-    </row>
-    <row r="183" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A183" s="37"/>
-      <c r="B183" s="38"/>
-      <c r="C183" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D183" s="38"/>
-      <c r="E183" s="40"/>
-      <c r="F183" s="40"/>
-      <c r="G183" s="41"/>
-      <c r="H183" s="41"/>
-      <c r="I183" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J183" s="45"/>
-      <c r="K183" s="43"/>
+      <c r="A182" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B182" s="71" t="s">
+        <v>13</v>
+      </c>
+      <c r="C182" s="62"/>
+      <c r="D182" s="62"/>
+      <c r="E182" s="62"/>
+      <c r="F182" s="62"/>
+      <c r="G182" s="62"/>
+      <c r="H182" s="62"/>
+      <c r="I182" s="62"/>
+      <c r="J182" s="62"/>
+      <c r="K182" s="63"/>
+    </row>
+    <row r="183" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B183" s="71" t="s">
+        <v>15</v>
+      </c>
+      <c r="C183" s="62"/>
+      <c r="D183" s="62"/>
+      <c r="E183" s="62"/>
+      <c r="F183" s="62"/>
+      <c r="G183" s="62"/>
+      <c r="H183" s="62"/>
+      <c r="I183" s="62"/>
+      <c r="J183" s="62"/>
+      <c r="K183" s="63"/>
     </row>
     <row r="184" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A184" s="37"/>
@@ -7201,84 +7466,85 @@
       <c r="G184" s="41"/>
       <c r="H184" s="41"/>
       <c r="I184" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I184:I194" si="8">H184-G184</f>
         <v>0</v>
       </c>
       <c r="J184" s="45"/>
       <c r="K184" s="43"/>
     </row>
     <row r="185" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A185" s="13"/>
-      <c r="B185" s="15"/>
-      <c r="C185" s="15"/>
-      <c r="D185" s="15"/>
-      <c r="E185" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F185" s="15"/>
-      <c r="G185" s="18">
-        <f t="shared" ref="G185:H185" si="9">SUM(G175:G184)</f>
-        <v>0</v>
-      </c>
-      <c r="H185" s="18">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="I185" s="18">
+      <c r="A185" s="37"/>
+      <c r="B185" s="38"/>
+      <c r="C185" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D185" s="38"/>
+      <c r="E185" s="40"/>
+      <c r="F185" s="40"/>
+      <c r="G185" s="41"/>
+      <c r="H185" s="41"/>
+      <c r="I185" s="41">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J185" s="19"/>
-      <c r="K185" s="46"/>
-    </row>
-    <row r="186" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="72" t="s">
-        <v>26</v>
-      </c>
-      <c r="B186" s="62"/>
-      <c r="C186" s="62"/>
-      <c r="D186" s="62"/>
-      <c r="E186" s="62"/>
-      <c r="F186" s="62"/>
-      <c r="G186" s="62"/>
-      <c r="H186" s="62"/>
-      <c r="I186" s="62"/>
-      <c r="J186" s="62"/>
-      <c r="K186" s="63"/>
+      <c r="J185" s="45"/>
+      <c r="K185" s="43"/>
+    </row>
+    <row r="186" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A186" s="37"/>
+      <c r="B186" s="38"/>
+      <c r="C186" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D186" s="38"/>
+      <c r="E186" s="40"/>
+      <c r="F186" s="40"/>
+      <c r="G186" s="41"/>
+      <c r="H186" s="41"/>
+      <c r="I186" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J186" s="45"/>
+      <c r="K186" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="187" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A187" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B187" s="69" t="s">
-        <v>13</v>
-      </c>
-      <c r="C187" s="62"/>
-      <c r="D187" s="62"/>
-      <c r="E187" s="62"/>
-      <c r="F187" s="62"/>
-      <c r="G187" s="62"/>
-      <c r="H187" s="62"/>
-      <c r="I187" s="62"/>
-      <c r="J187" s="62"/>
-      <c r="K187" s="63"/>
-    </row>
-    <row r="188" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A188" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B188" s="69" t="s">
-        <v>15</v>
-      </c>
-      <c r="C188" s="62"/>
-      <c r="D188" s="62"/>
-      <c r="E188" s="62"/>
-      <c r="F188" s="62"/>
-      <c r="G188" s="62"/>
-      <c r="H188" s="62"/>
-      <c r="I188" s="62"/>
-      <c r="J188" s="62"/>
-      <c r="K188" s="63"/>
+      <c r="A187" s="37"/>
+      <c r="B187" s="38"/>
+      <c r="C187" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D187" s="38"/>
+      <c r="E187" s="40"/>
+      <c r="F187" s="40"/>
+      <c r="G187" s="41"/>
+      <c r="H187" s="41"/>
+      <c r="I187" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J187" s="45"/>
+      <c r="K187" s="43"/>
+    </row>
+    <row r="188" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A188" s="37"/>
+      <c r="B188" s="38"/>
+      <c r="C188" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D188" s="38"/>
+      <c r="E188" s="40"/>
+      <c r="F188" s="40"/>
+      <c r="G188" s="41"/>
+      <c r="H188" s="41"/>
+      <c r="I188" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J188" s="45"/>
+      <c r="K188" s="43"/>
     </row>
     <row r="189" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A189" s="37"/>
@@ -7292,7 +7558,7 @@
       <c r="G189" s="41"/>
       <c r="H189" s="41"/>
       <c r="I189" s="41">
-        <f t="shared" ref="I189:I199" si="10">H189-G189</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J189" s="45"/>
@@ -7310,7 +7576,7 @@
       <c r="G190" s="41"/>
       <c r="H190" s="41"/>
       <c r="I190" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J190" s="45"/>
@@ -7328,7 +7594,7 @@
       <c r="G191" s="41"/>
       <c r="H191" s="41"/>
       <c r="I191" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J191" s="45"/>
@@ -7346,7 +7612,7 @@
       <c r="G192" s="41"/>
       <c r="H192" s="41"/>
       <c r="I192" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J192" s="45"/>
@@ -7364,83 +7630,84 @@
       <c r="G193" s="41"/>
       <c r="H193" s="41"/>
       <c r="I193" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J193" s="45"/>
       <c r="K193" s="43"/>
     </row>
     <row r="194" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A194" s="37"/>
-      <c r="B194" s="38"/>
-      <c r="C194" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D194" s="38"/>
-      <c r="E194" s="40"/>
-      <c r="F194" s="40"/>
-      <c r="G194" s="41"/>
-      <c r="H194" s="41"/>
-      <c r="I194" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J194" s="45"/>
-      <c r="K194" s="43"/>
-    </row>
-    <row r="195" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A195" s="37"/>
-      <c r="B195" s="38"/>
-      <c r="C195" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D195" s="38"/>
-      <c r="E195" s="40"/>
-      <c r="F195" s="40"/>
-      <c r="G195" s="41"/>
-      <c r="H195" s="41"/>
-      <c r="I195" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J195" s="45"/>
-      <c r="K195" s="43"/>
+      <c r="A194" s="13"/>
+      <c r="B194" s="15"/>
+      <c r="C194" s="15"/>
+      <c r="D194" s="15"/>
+      <c r="E194" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F194" s="15"/>
+      <c r="G194" s="18">
+        <f t="shared" ref="G194:H194" si="9">SUM(G184:G193)</f>
+        <v>0</v>
+      </c>
+      <c r="H194" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="I194" s="18">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J194" s="19"/>
+      <c r="K194" s="46"/>
+    </row>
+    <row r="195" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="B195" s="62"/>
+      <c r="C195" s="62"/>
+      <c r="D195" s="62"/>
+      <c r="E195" s="62"/>
+      <c r="F195" s="62"/>
+      <c r="G195" s="62"/>
+      <c r="H195" s="62"/>
+      <c r="I195" s="62"/>
+      <c r="J195" s="62"/>
+      <c r="K195" s="63"/>
     </row>
     <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A196" s="37"/>
-      <c r="B196" s="38"/>
-      <c r="C196" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D196" s="38"/>
-      <c r="E196" s="40"/>
-      <c r="F196" s="40"/>
-      <c r="G196" s="41"/>
-      <c r="H196" s="41"/>
-      <c r="I196" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J196" s="45"/>
-      <c r="K196" s="43"/>
-    </row>
-    <row r="197" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A197" s="37"/>
-      <c r="B197" s="38"/>
-      <c r="C197" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D197" s="38"/>
-      <c r="E197" s="40"/>
-      <c r="F197" s="40"/>
-      <c r="G197" s="41"/>
-      <c r="H197" s="41"/>
-      <c r="I197" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J197" s="45"/>
-      <c r="K197" s="43"/>
+      <c r="A196" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B196" s="69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C196" s="62"/>
+      <c r="D196" s="62"/>
+      <c r="E196" s="62"/>
+      <c r="F196" s="62"/>
+      <c r="G196" s="62"/>
+      <c r="H196" s="62"/>
+      <c r="I196" s="62"/>
+      <c r="J196" s="62"/>
+      <c r="K196" s="63"/>
+    </row>
+    <row r="197" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B197" s="69" t="s">
+        <v>15</v>
+      </c>
+      <c r="C197" s="62"/>
+      <c r="D197" s="62"/>
+      <c r="E197" s="62"/>
+      <c r="F197" s="62"/>
+      <c r="G197" s="62"/>
+      <c r="H197" s="62"/>
+      <c r="I197" s="62"/>
+      <c r="J197" s="62"/>
+      <c r="K197" s="63"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="37"/>
@@ -7454,84 +7721,83 @@
       <c r="G198" s="41"/>
       <c r="H198" s="41"/>
       <c r="I198" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I198:I208" si="10">H198-G198</f>
         <v>0</v>
       </c>
       <c r="J198" s="45"/>
       <c r="K198" s="43"/>
     </row>
     <row r="199" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A199" s="13"/>
-      <c r="B199" s="15"/>
-      <c r="C199" s="15"/>
-      <c r="D199" s="15"/>
-      <c r="E199" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F199" s="15"/>
-      <c r="G199" s="18">
-        <f t="shared" ref="G199:H199" si="11">SUM(G189:G198)</f>
-        <v>0</v>
-      </c>
-      <c r="H199" s="18">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I199" s="18">
+      <c r="A199" s="37"/>
+      <c r="B199" s="38"/>
+      <c r="C199" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D199" s="38"/>
+      <c r="E199" s="40"/>
+      <c r="F199" s="40"/>
+      <c r="G199" s="41"/>
+      <c r="H199" s="41"/>
+      <c r="I199" s="41">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J199" s="19"/>
-      <c r="K199" s="46"/>
-    </row>
-    <row r="200" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A200" s="54" t="s">
-        <v>27</v>
-      </c>
-      <c r="B200" s="55"/>
-      <c r="C200" s="55"/>
-      <c r="D200" s="55"/>
-      <c r="E200" s="55"/>
-      <c r="F200" s="55"/>
-      <c r="G200" s="55"/>
-      <c r="H200" s="55"/>
-      <c r="I200" s="55"/>
-      <c r="J200" s="55"/>
-      <c r="K200" s="56"/>
+      <c r="J199" s="45"/>
+      <c r="K199" s="43"/>
+    </row>
+    <row r="200" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A200" s="37"/>
+      <c r="B200" s="38"/>
+      <c r="C200" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D200" s="38"/>
+      <c r="E200" s="40"/>
+      <c r="F200" s="40"/>
+      <c r="G200" s="41"/>
+      <c r="H200" s="41"/>
+      <c r="I200" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J200" s="45"/>
+      <c r="K200" s="43"/>
     </row>
     <row r="201" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A201" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B201" s="57" t="s">
-        <v>13</v>
-      </c>
-      <c r="C201" s="55"/>
-      <c r="D201" s="55"/>
-      <c r="E201" s="55"/>
-      <c r="F201" s="55"/>
-      <c r="G201" s="55"/>
-      <c r="H201" s="55"/>
-      <c r="I201" s="55"/>
-      <c r="J201" s="55"/>
-      <c r="K201" s="56"/>
-    </row>
-    <row r="202" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B202" s="57" t="s">
-        <v>15</v>
-      </c>
-      <c r="C202" s="55"/>
-      <c r="D202" s="55"/>
-      <c r="E202" s="55"/>
-      <c r="F202" s="55"/>
-      <c r="G202" s="55"/>
-      <c r="H202" s="55"/>
-      <c r="I202" s="55"/>
-      <c r="J202" s="55"/>
-      <c r="K202" s="56"/>
+      <c r="A201" s="37"/>
+      <c r="B201" s="38"/>
+      <c r="C201" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D201" s="38"/>
+      <c r="E201" s="40"/>
+      <c r="F201" s="40"/>
+      <c r="G201" s="41"/>
+      <c r="H201" s="41"/>
+      <c r="I201" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J201" s="45"/>
+      <c r="K201" s="43"/>
+    </row>
+    <row r="202" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A202" s="37"/>
+      <c r="B202" s="38"/>
+      <c r="C202" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D202" s="38"/>
+      <c r="E202" s="40"/>
+      <c r="F202" s="40"/>
+      <c r="G202" s="41"/>
+      <c r="H202" s="41"/>
+      <c r="I202" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J202" s="45"/>
+      <c r="K202" s="43"/>
     </row>
     <row r="203" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A203" s="37"/>
@@ -7545,7 +7811,7 @@
       <c r="G203" s="41"/>
       <c r="H203" s="41"/>
       <c r="I203" s="41">
-        <f t="shared" ref="I203:I213" si="12">H203-G203</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J203" s="45"/>
@@ -7563,7 +7829,7 @@
       <c r="G204" s="41"/>
       <c r="H204" s="41"/>
       <c r="I204" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J204" s="45"/>
@@ -7581,7 +7847,7 @@
       <c r="G205" s="41"/>
       <c r="H205" s="41"/>
       <c r="I205" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J205" s="45"/>
@@ -7599,7 +7865,7 @@
       <c r="G206" s="41"/>
       <c r="H206" s="41"/>
       <c r="I206" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J206" s="45"/>
@@ -7617,83 +7883,84 @@
       <c r="G207" s="41"/>
       <c r="H207" s="41"/>
       <c r="I207" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J207" s="45"/>
       <c r="K207" s="43"/>
     </row>
     <row r="208" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A208" s="37"/>
-      <c r="B208" s="38"/>
-      <c r="C208" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D208" s="38"/>
-      <c r="E208" s="40"/>
-      <c r="F208" s="40"/>
-      <c r="G208" s="41"/>
-      <c r="H208" s="41"/>
-      <c r="I208" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J208" s="45"/>
-      <c r="K208" s="43"/>
-    </row>
-    <row r="209" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A209" s="37"/>
-      <c r="B209" s="38"/>
-      <c r="C209" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D209" s="38"/>
-      <c r="E209" s="40"/>
-      <c r="F209" s="40"/>
-      <c r="G209" s="41"/>
-      <c r="H209" s="41"/>
-      <c r="I209" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J209" s="45"/>
-      <c r="K209" s="43"/>
+      <c r="A208" s="13"/>
+      <c r="B208" s="15"/>
+      <c r="C208" s="15"/>
+      <c r="D208" s="15"/>
+      <c r="E208" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F208" s="15"/>
+      <c r="G208" s="18">
+        <f t="shared" ref="G208:H208" si="11">SUM(G198:G207)</f>
+        <v>0</v>
+      </c>
+      <c r="H208" s="18">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="I208" s="18">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J208" s="19"/>
+      <c r="K208" s="46"/>
+    </row>
+    <row r="209" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="54" t="s">
+        <v>27</v>
+      </c>
+      <c r="B209" s="55"/>
+      <c r="C209" s="55"/>
+      <c r="D209" s="55"/>
+      <c r="E209" s="55"/>
+      <c r="F209" s="55"/>
+      <c r="G209" s="55"/>
+      <c r="H209" s="55"/>
+      <c r="I209" s="55"/>
+      <c r="J209" s="55"/>
+      <c r="K209" s="56"/>
     </row>
     <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A210" s="37"/>
-      <c r="B210" s="38"/>
-      <c r="C210" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D210" s="38"/>
-      <c r="E210" s="40"/>
-      <c r="F210" s="40"/>
-      <c r="G210" s="41"/>
-      <c r="H210" s="41"/>
-      <c r="I210" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J210" s="45"/>
-      <c r="K210" s="43"/>
-    </row>
-    <row r="211" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A211" s="37"/>
-      <c r="B211" s="38"/>
-      <c r="C211" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D211" s="38"/>
-      <c r="E211" s="40"/>
-      <c r="F211" s="40"/>
-      <c r="G211" s="41"/>
-      <c r="H211" s="41"/>
-      <c r="I211" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J211" s="45"/>
-      <c r="K211" s="43"/>
+      <c r="A210" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B210" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C210" s="55"/>
+      <c r="D210" s="55"/>
+      <c r="E210" s="55"/>
+      <c r="F210" s="55"/>
+      <c r="G210" s="55"/>
+      <c r="H210" s="55"/>
+      <c r="I210" s="55"/>
+      <c r="J210" s="55"/>
+      <c r="K210" s="56"/>
+    </row>
+    <row r="211" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B211" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C211" s="55"/>
+      <c r="D211" s="55"/>
+      <c r="E211" s="55"/>
+      <c r="F211" s="55"/>
+      <c r="G211" s="55"/>
+      <c r="H211" s="55"/>
+      <c r="I211" s="55"/>
+      <c r="J211" s="55"/>
+      <c r="K211" s="56"/>
     </row>
     <row r="212" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A212" s="37"/>
@@ -7707,42 +7974,204 @@
       <c r="G212" s="41"/>
       <c r="H212" s="41"/>
       <c r="I212" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="I212:I222" si="12">H212-G212</f>
         <v>0</v>
       </c>
       <c r="J212" s="45"/>
       <c r="K212" s="43"/>
     </row>
     <row r="213" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A213" s="48"/>
-      <c r="B213" s="49"/>
-      <c r="C213" s="49"/>
-      <c r="D213" s="49"/>
-      <c r="E213" s="49" t="s">
+      <c r="A213" s="37"/>
+      <c r="B213" s="38"/>
+      <c r="C213" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D213" s="38"/>
+      <c r="E213" s="40"/>
+      <c r="F213" s="40"/>
+      <c r="G213" s="41"/>
+      <c r="H213" s="41"/>
+      <c r="I213" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J213" s="45"/>
+      <c r="K213" s="43"/>
+    </row>
+    <row r="214" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A214" s="37"/>
+      <c r="B214" s="38"/>
+      <c r="C214" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D214" s="38"/>
+      <c r="E214" s="40"/>
+      <c r="F214" s="40"/>
+      <c r="G214" s="41"/>
+      <c r="H214" s="41"/>
+      <c r="I214" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J214" s="45"/>
+      <c r="K214" s="43"/>
+    </row>
+    <row r="215" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A215" s="37"/>
+      <c r="B215" s="38"/>
+      <c r="C215" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D215" s="38"/>
+      <c r="E215" s="40"/>
+      <c r="F215" s="40"/>
+      <c r="G215" s="41"/>
+      <c r="H215" s="41"/>
+      <c r="I215" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J215" s="45"/>
+      <c r="K215" s="43"/>
+    </row>
+    <row r="216" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A216" s="37"/>
+      <c r="B216" s="38"/>
+      <c r="C216" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D216" s="38"/>
+      <c r="E216" s="40"/>
+      <c r="F216" s="40"/>
+      <c r="G216" s="41"/>
+      <c r="H216" s="41"/>
+      <c r="I216" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J216" s="45"/>
+      <c r="K216" s="43"/>
+    </row>
+    <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A217" s="37"/>
+      <c r="B217" s="38"/>
+      <c r="C217" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D217" s="38"/>
+      <c r="E217" s="40"/>
+      <c r="F217" s="40"/>
+      <c r="G217" s="41"/>
+      <c r="H217" s="41"/>
+      <c r="I217" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J217" s="45"/>
+      <c r="K217" s="43"/>
+    </row>
+    <row r="218" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A218" s="37"/>
+      <c r="B218" s="38"/>
+      <c r="C218" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D218" s="38"/>
+      <c r="E218" s="40"/>
+      <c r="F218" s="40"/>
+      <c r="G218" s="41"/>
+      <c r="H218" s="41"/>
+      <c r="I218" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J218" s="45"/>
+      <c r="K218" s="43"/>
+    </row>
+    <row r="219" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A219" s="37"/>
+      <c r="B219" s="38"/>
+      <c r="C219" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D219" s="38"/>
+      <c r="E219" s="40"/>
+      <c r="F219" s="40"/>
+      <c r="G219" s="41"/>
+      <c r="H219" s="41"/>
+      <c r="I219" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J219" s="45"/>
+      <c r="K219" s="43"/>
+    </row>
+    <row r="220" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A220" s="37"/>
+      <c r="B220" s="38"/>
+      <c r="C220" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D220" s="38"/>
+      <c r="E220" s="40"/>
+      <c r="F220" s="40"/>
+      <c r="G220" s="41"/>
+      <c r="H220" s="41"/>
+      <c r="I220" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J220" s="45"/>
+      <c r="K220" s="43"/>
+    </row>
+    <row r="221" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A221" s="37"/>
+      <c r="B221" s="38"/>
+      <c r="C221" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D221" s="38"/>
+      <c r="E221" s="40"/>
+      <c r="F221" s="40"/>
+      <c r="G221" s="41"/>
+      <c r="H221" s="41"/>
+      <c r="I221" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J221" s="45"/>
+      <c r="K221" s="43"/>
+    </row>
+    <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A222" s="48"/>
+      <c r="B222" s="49"/>
+      <c r="C222" s="49"/>
+      <c r="D222" s="49"/>
+      <c r="E222" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F213" s="49"/>
-      <c r="G213" s="50">
-        <f t="shared" ref="G213:H213" si="13">SUM(G203:G212)</f>
-        <v>0</v>
-      </c>
-      <c r="H213" s="50">
+      <c r="F222" s="49"/>
+      <c r="G222" s="50">
+        <f t="shared" ref="G222:H222" si="13">SUM(G212:G221)</f>
+        <v>0</v>
+      </c>
+      <c r="H222" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="I213" s="50">
+      <c r="I222" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J213" s="51"/>
-      <c r="K213" s="52"/>
+      <c r="J222" s="51"/>
+      <c r="K222" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{E0E62371-B3FE-487E-A364-D1186735B483}">
+      <autoFilter ref="A1:K15" xr:uid="{8F2DE6E0-46DD-47D1-A4DA-AABA39C214A8}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -7753,17 +8182,17 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B173:K173"/>
-    <mergeCell ref="B174:K174"/>
-    <mergeCell ref="A186:K186"/>
+    <mergeCell ref="B182:K182"/>
+    <mergeCell ref="B183:K183"/>
+    <mergeCell ref="A195:K195"/>
     <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A150:K150"/>
-    <mergeCell ref="B151:K151"/>
+    <mergeCell ref="A151:K151"/>
     <mergeCell ref="B152:K152"/>
-    <mergeCell ref="A172:K172"/>
-    <mergeCell ref="A200:K200"/>
-    <mergeCell ref="B201:K201"/>
-    <mergeCell ref="B202:K202"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A181:K181"/>
+    <mergeCell ref="A209:K209"/>
+    <mergeCell ref="B210:K210"/>
+    <mergeCell ref="B211:K211"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -7774,11 +8203,11 @@
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
     <mergeCell ref="A118:K118"/>
-    <mergeCell ref="B187:K187"/>
-    <mergeCell ref="B188:K188"/>
+    <mergeCell ref="B196:K196"/>
+    <mergeCell ref="B197:K197"/>
     <mergeCell ref="B119:K119"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B148 B153:B170 B175:B184 B189:B198">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B179 B184:B193 B198:B207">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -7795,7 +8224,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B149 B151:B171 B173:B185 B187:B199 B201:B213">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B152:B180 B182:B194 B196:B208 B210:B222 B119:B150">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -7803,34 +8232,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B203:B212">
+  <conditionalFormatting sqref="B212:B221">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B203))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B212))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B203))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B212))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B203))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B212))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B203))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B212))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B203))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B212))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G149 G153:G171 G175:G185 G189:G199 G203:G213">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G154:G180 G184:G194 G198:G208 G212:G222 G121:G150">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H213">
+  <conditionalFormatting sqref="H1:H222">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I149 I175:I185 I189:I199 I203:I213 I153:I171">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I184:I194 I198:I208 I212:I222 I121:I150 I154:I180">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -7839,7 +8268,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F203:F212 F189:F198 F86:F116 F153:F170 F175:F184 F5:F45 F50:F81 F121:F148" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F212:F221 F198:F207 F86:F116 F154:F179 F184:F193 F5:F45 F50:F81 F121:F149" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7855,13 +8284,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E116 E153:E170 E175:E184 E189:E198 E203:E212 E50:E81 E121:E148</xm:sqref>
+          <xm:sqref>E5:E45 E86:E116 E154:E179 E184:E193 E198:E207 E212:E221 E50:E81 E121:E149</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B116 B153:B170 B175:B184 B189:B198 B203:B212 B50:B81 B121:B148</xm:sqref>
+          <xm:sqref>B5:B45 B86:B116 B154:B179 B184:B193 B198:B207 B212:B221 B50:B81 B121:B149</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
W5 DataLab 1 Work III (Break)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4800F9A-E831-4758-BEA3-F9DED09CDD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77673BE8-804C-4BDA-B1A9-8CFA33CE5ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1430,6 +1430,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1446,8 +1466,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1465,24 +1483,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2007,53 +2007,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3392,53 +3392,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4491,53 +4491,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5552,53 +5552,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="68" t="s">
+      <c r="A118" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="62"/>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
+      <c r="B118" s="55"/>
+      <c r="C118" s="55"/>
+      <c r="D118" s="55"/>
+      <c r="E118" s="55"/>
+      <c r="F118" s="55"/>
+      <c r="G118" s="55"/>
+      <c r="H118" s="55"/>
+      <c r="I118" s="55"/>
+      <c r="J118" s="55"/>
+      <c r="K118" s="56"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="70" t="s">
+      <c r="B119" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="62"/>
-      <c r="D119" s="62"/>
-      <c r="E119" s="62"/>
-      <c r="F119" s="62"/>
-      <c r="G119" s="62"/>
-      <c r="H119" s="62"/>
-      <c r="I119" s="62"/>
-      <c r="J119" s="62"/>
-      <c r="K119" s="63"/>
+      <c r="C119" s="55"/>
+      <c r="D119" s="55"/>
+      <c r="E119" s="55"/>
+      <c r="F119" s="55"/>
+      <c r="G119" s="55"/>
+      <c r="H119" s="55"/>
+      <c r="I119" s="55"/>
+      <c r="J119" s="55"/>
+      <c r="K119" s="56"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="70" t="s">
+      <c r="B120" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="62"/>
-      <c r="D120" s="62"/>
-      <c r="E120" s="62"/>
-      <c r="F120" s="62"/>
-      <c r="G120" s="62"/>
-      <c r="H120" s="62"/>
-      <c r="I120" s="62"/>
-      <c r="J120" s="62"/>
-      <c r="K120" s="63"/>
+      <c r="C120" s="55"/>
+      <c r="D120" s="55"/>
+      <c r="E120" s="55"/>
+      <c r="F120" s="55"/>
+      <c r="G120" s="55"/>
+      <c r="H120" s="55"/>
+      <c r="I120" s="55"/>
+      <c r="J120" s="55"/>
+      <c r="K120" s="56"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6535,53 +6535,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="73" t="s">
+      <c r="A151" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="62"/>
-      <c r="C151" s="62"/>
-      <c r="D151" s="62"/>
-      <c r="E151" s="62"/>
-      <c r="F151" s="62"/>
-      <c r="G151" s="62"/>
-      <c r="H151" s="62"/>
-      <c r="I151" s="62"/>
-      <c r="J151" s="62"/>
-      <c r="K151" s="63"/>
+      <c r="B151" s="55"/>
+      <c r="C151" s="55"/>
+      <c r="D151" s="55"/>
+      <c r="E151" s="55"/>
+      <c r="F151" s="55"/>
+      <c r="G151" s="55"/>
+      <c r="H151" s="55"/>
+      <c r="I151" s="55"/>
+      <c r="J151" s="55"/>
+      <c r="K151" s="56"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="74" t="s">
+      <c r="B152" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="62"/>
-      <c r="D152" s="62"/>
-      <c r="E152" s="62"/>
-      <c r="F152" s="62"/>
-      <c r="G152" s="62"/>
-      <c r="H152" s="62"/>
-      <c r="I152" s="62"/>
-      <c r="J152" s="62"/>
-      <c r="K152" s="63"/>
+      <c r="C152" s="55"/>
+      <c r="D152" s="55"/>
+      <c r="E152" s="55"/>
+      <c r="F152" s="55"/>
+      <c r="G152" s="55"/>
+      <c r="H152" s="55"/>
+      <c r="I152" s="55"/>
+      <c r="J152" s="55"/>
+      <c r="K152" s="56"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="74" t="s">
+      <c r="B153" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="62"/>
-      <c r="D153" s="62"/>
-      <c r="E153" s="62"/>
-      <c r="F153" s="62"/>
-      <c r="G153" s="62"/>
-      <c r="H153" s="62"/>
-      <c r="I153" s="62"/>
-      <c r="J153" s="62"/>
-      <c r="K153" s="63"/>
+      <c r="C153" s="55"/>
+      <c r="D153" s="55"/>
+      <c r="E153" s="55"/>
+      <c r="F153" s="55"/>
+      <c r="G153" s="55"/>
+      <c r="H153" s="55"/>
+      <c r="I153" s="55"/>
+      <c r="J153" s="55"/>
+      <c r="K153" s="56"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -7260,7 +7260,7 @@
         <v>45643</v>
       </c>
       <c r="B175" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C175" s="39" t="s">
         <v>238</v>
@@ -7277,10 +7277,12 @@
       <c r="G175" s="41">
         <v>1</v>
       </c>
-      <c r="H175" s="41"/>
+      <c r="H175" s="41">
+        <v>1.5</v>
+      </c>
       <c r="I175" s="41">
         <f t="shared" si="6"/>
-        <v>-1</v>
+        <v>0.5</v>
       </c>
       <c r="J175" s="45"/>
       <c r="K175" s="43" t="s">
@@ -7292,7 +7294,7 @@
         <v>45643</v>
       </c>
       <c r="B176" s="38" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="C176" s="39" t="s">
         <v>238</v>
@@ -7396,63 +7398,63 @@
       </c>
       <c r="H180" s="18">
         <f t="shared" si="7"/>
-        <v>15.91</v>
+        <v>17.41</v>
       </c>
       <c r="I180" s="18">
         <f t="shared" si="6"/>
-        <v>-11.25</v>
+        <v>-9.75</v>
       </c>
       <c r="J180" s="19"/>
       <c r="K180" s="46"/>
     </row>
     <row r="181" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A181" s="75" t="s">
+      <c r="A181" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B181" s="62"/>
-      <c r="C181" s="62"/>
-      <c r="D181" s="62"/>
-      <c r="E181" s="62"/>
-      <c r="F181" s="62"/>
-      <c r="G181" s="62"/>
-      <c r="H181" s="62"/>
-      <c r="I181" s="62"/>
-      <c r="J181" s="62"/>
-      <c r="K181" s="63"/>
+      <c r="B181" s="55"/>
+      <c r="C181" s="55"/>
+      <c r="D181" s="55"/>
+      <c r="E181" s="55"/>
+      <c r="F181" s="55"/>
+      <c r="G181" s="55"/>
+      <c r="H181" s="55"/>
+      <c r="I181" s="55"/>
+      <c r="J181" s="55"/>
+      <c r="K181" s="56"/>
     </row>
     <row r="182" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A182" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B182" s="71" t="s">
+      <c r="B182" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C182" s="62"/>
-      <c r="D182" s="62"/>
-      <c r="E182" s="62"/>
-      <c r="F182" s="62"/>
-      <c r="G182" s="62"/>
-      <c r="H182" s="62"/>
-      <c r="I182" s="62"/>
-      <c r="J182" s="62"/>
-      <c r="K182" s="63"/>
+      <c r="C182" s="55"/>
+      <c r="D182" s="55"/>
+      <c r="E182" s="55"/>
+      <c r="F182" s="55"/>
+      <c r="G182" s="55"/>
+      <c r="H182" s="55"/>
+      <c r="I182" s="55"/>
+      <c r="J182" s="55"/>
+      <c r="K182" s="56"/>
     </row>
     <row r="183" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B183" s="71" t="s">
+      <c r="B183" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C183" s="62"/>
-      <c r="D183" s="62"/>
-      <c r="E183" s="62"/>
-      <c r="F183" s="62"/>
-      <c r="G183" s="62"/>
-      <c r="H183" s="62"/>
-      <c r="I183" s="62"/>
-      <c r="J183" s="62"/>
-      <c r="K183" s="63"/>
+      <c r="C183" s="55"/>
+      <c r="D183" s="55"/>
+      <c r="E183" s="55"/>
+      <c r="F183" s="55"/>
+      <c r="G183" s="55"/>
+      <c r="H183" s="55"/>
+      <c r="I183" s="55"/>
+      <c r="J183" s="55"/>
+      <c r="K183" s="56"/>
     </row>
     <row r="184" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A184" s="37"/>
@@ -7661,53 +7663,53 @@
       <c r="K194" s="46"/>
     </row>
     <row r="195" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="72" t="s">
+      <c r="A195" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B195" s="62"/>
-      <c r="C195" s="62"/>
-      <c r="D195" s="62"/>
-      <c r="E195" s="62"/>
-      <c r="F195" s="62"/>
-      <c r="G195" s="62"/>
-      <c r="H195" s="62"/>
-      <c r="I195" s="62"/>
-      <c r="J195" s="62"/>
-      <c r="K195" s="63"/>
+      <c r="B195" s="55"/>
+      <c r="C195" s="55"/>
+      <c r="D195" s="55"/>
+      <c r="E195" s="55"/>
+      <c r="F195" s="55"/>
+      <c r="G195" s="55"/>
+      <c r="H195" s="55"/>
+      <c r="I195" s="55"/>
+      <c r="J195" s="55"/>
+      <c r="K195" s="56"/>
     </row>
     <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A196" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B196" s="69" t="s">
+      <c r="B196" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C196" s="62"/>
-      <c r="D196" s="62"/>
-      <c r="E196" s="62"/>
-      <c r="F196" s="62"/>
-      <c r="G196" s="62"/>
-      <c r="H196" s="62"/>
-      <c r="I196" s="62"/>
-      <c r="J196" s="62"/>
-      <c r="K196" s="63"/>
+      <c r="C196" s="55"/>
+      <c r="D196" s="55"/>
+      <c r="E196" s="55"/>
+      <c r="F196" s="55"/>
+      <c r="G196" s="55"/>
+      <c r="H196" s="55"/>
+      <c r="I196" s="55"/>
+      <c r="J196" s="55"/>
+      <c r="K196" s="56"/>
     </row>
     <row r="197" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B197" s="69" t="s">
+      <c r="B197" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C197" s="62"/>
-      <c r="D197" s="62"/>
-      <c r="E197" s="62"/>
-      <c r="F197" s="62"/>
-      <c r="G197" s="62"/>
-      <c r="H197" s="62"/>
-      <c r="I197" s="62"/>
-      <c r="J197" s="62"/>
-      <c r="K197" s="63"/>
+      <c r="C197" s="55"/>
+      <c r="D197" s="55"/>
+      <c r="E197" s="55"/>
+      <c r="F197" s="55"/>
+      <c r="G197" s="55"/>
+      <c r="H197" s="55"/>
+      <c r="I197" s="55"/>
+      <c r="J197" s="55"/>
+      <c r="K197" s="56"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="37"/>
@@ -7914,53 +7916,53 @@
       <c r="K208" s="46"/>
     </row>
     <row r="209" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A209" s="54" t="s">
+      <c r="A209" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B209" s="55"/>
-      <c r="C209" s="55"/>
-      <c r="D209" s="55"/>
-      <c r="E209" s="55"/>
-      <c r="F209" s="55"/>
-      <c r="G209" s="55"/>
-      <c r="H209" s="55"/>
-      <c r="I209" s="55"/>
-      <c r="J209" s="55"/>
-      <c r="K209" s="56"/>
+      <c r="B209" s="63"/>
+      <c r="C209" s="63"/>
+      <c r="D209" s="63"/>
+      <c r="E209" s="63"/>
+      <c r="F209" s="63"/>
+      <c r="G209" s="63"/>
+      <c r="H209" s="63"/>
+      <c r="I209" s="63"/>
+      <c r="J209" s="63"/>
+      <c r="K209" s="64"/>
     </row>
     <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A210" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B210" s="57" t="s">
+      <c r="B210" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C210" s="55"/>
-      <c r="D210" s="55"/>
-      <c r="E210" s="55"/>
-      <c r="F210" s="55"/>
-      <c r="G210" s="55"/>
-      <c r="H210" s="55"/>
-      <c r="I210" s="55"/>
-      <c r="J210" s="55"/>
-      <c r="K210" s="56"/>
+      <c r="C210" s="63"/>
+      <c r="D210" s="63"/>
+      <c r="E210" s="63"/>
+      <c r="F210" s="63"/>
+      <c r="G210" s="63"/>
+      <c r="H210" s="63"/>
+      <c r="I210" s="63"/>
+      <c r="J210" s="63"/>
+      <c r="K210" s="64"/>
     </row>
     <row r="211" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B211" s="57" t="s">
+      <c r="B211" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C211" s="55"/>
-      <c r="D211" s="55"/>
-      <c r="E211" s="55"/>
-      <c r="F211" s="55"/>
-      <c r="G211" s="55"/>
-      <c r="H211" s="55"/>
-      <c r="I211" s="55"/>
-      <c r="J211" s="55"/>
-      <c r="K211" s="56"/>
+      <c r="C211" s="63"/>
+      <c r="D211" s="63"/>
+      <c r="E211" s="63"/>
+      <c r="F211" s="63"/>
+      <c r="G211" s="63"/>
+      <c r="H211" s="63"/>
+      <c r="I211" s="63"/>
+      <c r="J211" s="63"/>
+      <c r="K211" s="64"/>
     </row>
     <row r="212" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A212" s="37"/>
@@ -8171,7 +8173,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{8F2DE6E0-46DD-47D1-A4DA-AABA39C214A8}">
+      <autoFilter ref="A1:K15" xr:uid="{746F7D6D-6DAD-4C2D-BC98-A9B5ADA04487}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -8182,14 +8184,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B182:K182"/>
-    <mergeCell ref="B183:K183"/>
-    <mergeCell ref="A195:K195"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A181:K181"/>
     <mergeCell ref="A209:K209"/>
     <mergeCell ref="B210:K210"/>
     <mergeCell ref="B211:K211"/>
@@ -8206,6 +8200,14 @@
     <mergeCell ref="B196:K196"/>
     <mergeCell ref="B197:K197"/>
     <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B182:K182"/>
+    <mergeCell ref="B183:K183"/>
+    <mergeCell ref="A195:K195"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A181:K181"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B179 B184:B193 B198:B207">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -8224,7 +8226,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B152:B180 B182:B194 B196:B208 B210:B222 B119:B150">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B152:B180 B182:B194 B196:B208 B210:B222">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -8249,7 +8251,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B212))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G154:G180 G184:G194 G198:G208 G212:G222 G121:G150">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G154:G180 G184:G194 G198:G208 G212:G222">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
@@ -8259,7 +8261,7 @@
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I184:I194 I198:I208 I212:I222 I121:I150 I154:I180">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I154:I180 I184:I194 I198:I208 I212:I222">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -9931,6 +9933,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -10165,27 +10187,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10202,23 +10223,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W5 DataLab 1 Work IV (Post break at 14:30)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77673BE8-804C-4BDA-B1A9-8CFA33CE5ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8028CE-5F24-4CA0-BF52-E158941D3939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$207</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$217</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="289">
   <si>
     <t>Date</t>
   </si>
@@ -945,6 +945,30 @@
   </si>
   <si>
     <t>Had a bit of a problem with VSC not seeing the environment or some of the packages on my new laptop.</t>
+  </si>
+  <si>
+    <t>Do the quiz about multivariable calculus</t>
+  </si>
+  <si>
+    <t>Do the quiz about python for symbolic calculus</t>
+  </si>
+  <si>
+    <t>Wednesday Math</t>
+  </si>
+  <si>
+    <t>Learn multivariable calculus</t>
+  </si>
+  <si>
+    <t>Learn python for Symbolic calculus</t>
+  </si>
+  <si>
+    <t>I understood the mathematical concept of multivariable calculus pretty quickly and so it didn't take as long as I predicted it to.</t>
+  </si>
+  <si>
+    <t>from 14:30</t>
+  </si>
+  <si>
+    <t>As stated above, I understood the concepts pretty quickly and did not have too much troubles with the quiz.</t>
   </si>
 </sst>
 </file>
@@ -1430,26 +1454,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1466,6 +1470,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1483,6 +1489,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1955,7 +1979,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K222"/>
+  <dimension ref="A1:K232"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -2007,53 +2031,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3392,53 +3416,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="62"/>
+      <c r="K49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4491,53 +4515,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72" t="s">
+      <c r="A83" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="55"/>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="55"/>
-      <c r="I83" s="55"/>
-      <c r="J83" s="55"/>
-      <c r="K83" s="56"/>
+      <c r="B83" s="62"/>
+      <c r="C83" s="62"/>
+      <c r="D83" s="62"/>
+      <c r="E83" s="62"/>
+      <c r="F83" s="62"/>
+      <c r="G83" s="62"/>
+      <c r="H83" s="62"/>
+      <c r="I83" s="62"/>
+      <c r="J83" s="62"/>
+      <c r="K83" s="63"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="73" t="s">
+      <c r="B84" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="55"/>
-      <c r="D84" s="55"/>
-      <c r="E84" s="55"/>
-      <c r="F84" s="55"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="55"/>
-      <c r="I84" s="55"/>
-      <c r="J84" s="55"/>
-      <c r="K84" s="56"/>
+      <c r="C84" s="62"/>
+      <c r="D84" s="62"/>
+      <c r="E84" s="62"/>
+      <c r="F84" s="62"/>
+      <c r="G84" s="62"/>
+      <c r="H84" s="62"/>
+      <c r="I84" s="62"/>
+      <c r="J84" s="62"/>
+      <c r="K84" s="63"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="73" t="s">
+      <c r="B85" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="55"/>
-      <c r="D85" s="55"/>
-      <c r="E85" s="55"/>
-      <c r="F85" s="55"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="55"/>
-      <c r="I85" s="55"/>
-      <c r="J85" s="55"/>
-      <c r="K85" s="56"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="62"/>
+      <c r="G85" s="62"/>
+      <c r="H85" s="62"/>
+      <c r="I85" s="62"/>
+      <c r="J85" s="62"/>
+      <c r="K85" s="63"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5552,53 +5576,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="74" t="s">
+      <c r="A118" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="55"/>
-      <c r="C118" s="55"/>
-      <c r="D118" s="55"/>
-      <c r="E118" s="55"/>
-      <c r="F118" s="55"/>
-      <c r="G118" s="55"/>
-      <c r="H118" s="55"/>
-      <c r="I118" s="55"/>
-      <c r="J118" s="55"/>
-      <c r="K118" s="56"/>
+      <c r="B118" s="62"/>
+      <c r="C118" s="62"/>
+      <c r="D118" s="62"/>
+      <c r="E118" s="62"/>
+      <c r="F118" s="62"/>
+      <c r="G118" s="62"/>
+      <c r="H118" s="62"/>
+      <c r="I118" s="62"/>
+      <c r="J118" s="62"/>
+      <c r="K118" s="63"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="58" t="s">
+      <c r="B119" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="55"/>
-      <c r="D119" s="55"/>
-      <c r="E119" s="55"/>
-      <c r="F119" s="55"/>
-      <c r="G119" s="55"/>
-      <c r="H119" s="55"/>
-      <c r="I119" s="55"/>
-      <c r="J119" s="55"/>
-      <c r="K119" s="56"/>
+      <c r="C119" s="62"/>
+      <c r="D119" s="62"/>
+      <c r="E119" s="62"/>
+      <c r="F119" s="62"/>
+      <c r="G119" s="62"/>
+      <c r="H119" s="62"/>
+      <c r="I119" s="62"/>
+      <c r="J119" s="62"/>
+      <c r="K119" s="63"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="58" t="s">
+      <c r="B120" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="55"/>
-      <c r="D120" s="55"/>
-      <c r="E120" s="55"/>
-      <c r="F120" s="55"/>
-      <c r="G120" s="55"/>
-      <c r="H120" s="55"/>
-      <c r="I120" s="55"/>
-      <c r="J120" s="55"/>
-      <c r="K120" s="56"/>
+      <c r="C120" s="62"/>
+      <c r="D120" s="62"/>
+      <c r="E120" s="62"/>
+      <c r="F120" s="62"/>
+      <c r="G120" s="62"/>
+      <c r="H120" s="62"/>
+      <c r="I120" s="62"/>
+      <c r="J120" s="62"/>
+      <c r="K120" s="63"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6535,53 +6559,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="59" t="s">
+      <c r="A151" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="55"/>
-      <c r="C151" s="55"/>
-      <c r="D151" s="55"/>
-      <c r="E151" s="55"/>
-      <c r="F151" s="55"/>
-      <c r="G151" s="55"/>
-      <c r="H151" s="55"/>
-      <c r="I151" s="55"/>
-      <c r="J151" s="55"/>
-      <c r="K151" s="56"/>
+      <c r="B151" s="62"/>
+      <c r="C151" s="62"/>
+      <c r="D151" s="62"/>
+      <c r="E151" s="62"/>
+      <c r="F151" s="62"/>
+      <c r="G151" s="62"/>
+      <c r="H151" s="62"/>
+      <c r="I151" s="62"/>
+      <c r="J151" s="62"/>
+      <c r="K151" s="63"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="60" t="s">
+      <c r="B152" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="55"/>
-      <c r="D152" s="55"/>
-      <c r="E152" s="55"/>
-      <c r="F152" s="55"/>
-      <c r="G152" s="55"/>
-      <c r="H152" s="55"/>
-      <c r="I152" s="55"/>
-      <c r="J152" s="55"/>
-      <c r="K152" s="56"/>
+      <c r="C152" s="62"/>
+      <c r="D152" s="62"/>
+      <c r="E152" s="62"/>
+      <c r="F152" s="62"/>
+      <c r="G152" s="62"/>
+      <c r="H152" s="62"/>
+      <c r="I152" s="62"/>
+      <c r="J152" s="62"/>
+      <c r="K152" s="63"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="60" t="s">
+      <c r="B153" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="55"/>
-      <c r="D153" s="55"/>
-      <c r="E153" s="55"/>
-      <c r="F153" s="55"/>
-      <c r="G153" s="55"/>
-      <c r="H153" s="55"/>
-      <c r="I153" s="55"/>
-      <c r="J153" s="55"/>
-      <c r="K153" s="56"/>
+      <c r="C153" s="62"/>
+      <c r="D153" s="62"/>
+      <c r="E153" s="62"/>
+      <c r="F153" s="62"/>
+      <c r="G153" s="62"/>
+      <c r="H153" s="62"/>
+      <c r="I153" s="62"/>
+      <c r="J153" s="62"/>
+      <c r="K153" s="63"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -6609,7 +6633,7 @@
         <v>0.25</v>
       </c>
       <c r="I154" s="41">
-        <f t="shared" ref="I154:I180" si="6">H154-G154</f>
+        <f t="shared" ref="I154:I190" si="6">H154-G154</f>
         <v>0</v>
       </c>
       <c r="J154" s="45"/>
@@ -7350,125 +7374,176 @@
       <c r="K177" s="43"/>
     </row>
     <row r="178" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A178" s="37"/>
-      <c r="B178" s="38"/>
-      <c r="C178" s="39"/>
-      <c r="D178" s="38"/>
-      <c r="E178" s="40"/>
-      <c r="F178" s="40"/>
-      <c r="G178" s="41"/>
-      <c r="H178" s="41"/>
+      <c r="A178" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B178" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C178" s="39" t="s">
+        <v>283</v>
+      </c>
+      <c r="D178" s="38" t="s">
+        <v>284</v>
+      </c>
+      <c r="E178" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F178" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="G178" s="41">
+        <v>3</v>
+      </c>
+      <c r="H178" s="41">
+        <v>1.5</v>
+      </c>
       <c r="I178" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-1.5</v>
       </c>
       <c r="J178" s="45"/>
-      <c r="K178" s="43"/>
+      <c r="K178" s="43" t="s">
+        <v>286</v>
+      </c>
     </row>
     <row r="179" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A179" s="37"/>
-      <c r="B179" s="38"/>
+      <c r="A179" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B179" s="38" t="s">
+        <v>55</v>
+      </c>
       <c r="C179" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D179" s="38"/>
-      <c r="E179" s="40"/>
-      <c r="F179" s="40"/>
-      <c r="G179" s="41"/>
-      <c r="H179" s="41"/>
+        <v>283</v>
+      </c>
+      <c r="D179" s="38" t="s">
+        <v>281</v>
+      </c>
+      <c r="E179" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F179" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G179" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H179" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I179" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-0.25</v>
       </c>
       <c r="J179" s="45"/>
-      <c r="K179" s="43"/>
+      <c r="K179" s="43" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="180" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A180" s="13"/>
-      <c r="B180" s="15"/>
-      <c r="C180" s="15"/>
-      <c r="D180" s="15"/>
-      <c r="E180" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F180" s="15"/>
-      <c r="G180" s="18">
-        <f t="shared" ref="G180:H180" si="7">SUM(G154:G179)</f>
-        <v>27.16</v>
-      </c>
-      <c r="H180" s="18">
-        <f t="shared" si="7"/>
-        <v>17.41</v>
-      </c>
-      <c r="I180" s="18">
+      <c r="A180" s="37">
+        <v>45643</v>
+      </c>
+      <c r="B180" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C180" s="39" t="s">
+        <v>283</v>
+      </c>
+      <c r="D180" s="38" t="s">
+        <v>285</v>
+      </c>
+      <c r="E180" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F180" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="G180" s="41">
+        <v>3</v>
+      </c>
+      <c r="H180" s="41"/>
+      <c r="I180" s="41">
         <f t="shared" si="6"/>
-        <v>-9.75</v>
-      </c>
-      <c r="J180" s="19"/>
-      <c r="K180" s="46"/>
-    </row>
-    <row r="181" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A181" s="61" t="s">
-        <v>24</v>
-      </c>
-      <c r="B181" s="55"/>
-      <c r="C181" s="55"/>
-      <c r="D181" s="55"/>
-      <c r="E181" s="55"/>
-      <c r="F181" s="55"/>
-      <c r="G181" s="55"/>
-      <c r="H181" s="55"/>
-      <c r="I181" s="55"/>
-      <c r="J181" s="55"/>
-      <c r="K181" s="56"/>
+        <v>-3</v>
+      </c>
+      <c r="J180" s="45"/>
+      <c r="K180" s="43" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="181" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A181" s="37"/>
+      <c r="B181" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C181" s="39" t="s">
+        <v>283</v>
+      </c>
+      <c r="D181" s="38" t="s">
+        <v>282</v>
+      </c>
+      <c r="E181" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F181" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G181" s="41">
+        <v>1</v>
+      </c>
+      <c r="H181" s="41"/>
+      <c r="I181" s="41">
+        <f t="shared" si="6"/>
+        <v>-1</v>
+      </c>
+      <c r="J181" s="45"/>
+      <c r="K181" s="43"/>
     </row>
     <row r="182" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A182" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B182" s="54" t="s">
-        <v>13</v>
-      </c>
-      <c r="C182" s="55"/>
-      <c r="D182" s="55"/>
-      <c r="E182" s="55"/>
-      <c r="F182" s="55"/>
-      <c r="G182" s="55"/>
-      <c r="H182" s="55"/>
-      <c r="I182" s="55"/>
-      <c r="J182" s="55"/>
-      <c r="K182" s="56"/>
-    </row>
-    <row r="183" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A183" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B183" s="54" t="s">
-        <v>15</v>
-      </c>
-      <c r="C183" s="55"/>
-      <c r="D183" s="55"/>
-      <c r="E183" s="55"/>
-      <c r="F183" s="55"/>
-      <c r="G183" s="55"/>
-      <c r="H183" s="55"/>
-      <c r="I183" s="55"/>
-      <c r="J183" s="55"/>
-      <c r="K183" s="56"/>
+      <c r="A182" s="37"/>
+      <c r="B182" s="38"/>
+      <c r="C182" s="39"/>
+      <c r="D182" s="38"/>
+      <c r="E182" s="40"/>
+      <c r="F182" s="40"/>
+      <c r="G182" s="41"/>
+      <c r="H182" s="41"/>
+      <c r="I182" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J182" s="45"/>
+      <c r="K182" s="43"/>
+    </row>
+    <row r="183" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A183" s="37"/>
+      <c r="B183" s="38"/>
+      <c r="C183" s="39"/>
+      <c r="D183" s="38"/>
+      <c r="E183" s="40"/>
+      <c r="F183" s="40"/>
+      <c r="G183" s="41"/>
+      <c r="H183" s="41"/>
+      <c r="I183" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J183" s="45"/>
+      <c r="K183" s="43"/>
     </row>
     <row r="184" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A184" s="37"/>
       <c r="B184" s="38"/>
-      <c r="C184" s="39" t="s">
-        <v>17</v>
-      </c>
+      <c r="C184" s="39"/>
       <c r="D184" s="38"/>
       <c r="E184" s="40"/>
       <c r="F184" s="40"/>
       <c r="G184" s="41"/>
       <c r="H184" s="41"/>
       <c r="I184" s="41">
-        <f t="shared" ref="I184:I194" si="8">H184-G184</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J184" s="45"/>
@@ -7477,16 +7552,14 @@
     <row r="185" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A185" s="37"/>
       <c r="B185" s="38"/>
-      <c r="C185" s="39" t="s">
-        <v>17</v>
-      </c>
+      <c r="C185" s="39"/>
       <c r="D185" s="38"/>
       <c r="E185" s="40"/>
       <c r="F185" s="40"/>
       <c r="G185" s="41"/>
       <c r="H185" s="41"/>
       <c r="I185" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J185" s="45"/>
@@ -7495,36 +7568,30 @@
     <row r="186" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A186" s="37"/>
       <c r="B186" s="38"/>
-      <c r="C186" s="39" t="s">
-        <v>17</v>
-      </c>
+      <c r="C186" s="39"/>
       <c r="D186" s="38"/>
       <c r="E186" s="40"/>
       <c r="F186" s="40"/>
       <c r="G186" s="41"/>
       <c r="H186" s="41"/>
       <c r="I186" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J186" s="45"/>
-      <c r="K186" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K186" s="43"/>
     </row>
     <row r="187" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A187" s="37"/>
       <c r="B187" s="38"/>
-      <c r="C187" s="39" t="s">
-        <v>17</v>
-      </c>
+      <c r="C187" s="39"/>
       <c r="D187" s="38"/>
       <c r="E187" s="40"/>
       <c r="F187" s="40"/>
       <c r="G187" s="41"/>
       <c r="H187" s="41"/>
       <c r="I187" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J187" s="45"/>
@@ -7533,16 +7600,14 @@
     <row r="188" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A188" s="37"/>
       <c r="B188" s="38"/>
-      <c r="C188" s="39" t="s">
-        <v>17</v>
-      </c>
+      <c r="C188" s="39"/>
       <c r="D188" s="38"/>
       <c r="E188" s="40"/>
       <c r="F188" s="40"/>
       <c r="G188" s="41"/>
       <c r="H188" s="41"/>
       <c r="I188" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J188" s="45"/>
@@ -7560,156 +7625,158 @@
       <c r="G189" s="41"/>
       <c r="H189" s="41"/>
       <c r="I189" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J189" s="45"/>
       <c r="K189" s="43"/>
     </row>
     <row r="190" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A190" s="37"/>
-      <c r="B190" s="38"/>
-      <c r="C190" s="39" t="s">
+      <c r="A190" s="13"/>
+      <c r="B190" s="15"/>
+      <c r="C190" s="15"/>
+      <c r="D190" s="15"/>
+      <c r="E190" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F190" s="15"/>
+      <c r="G190" s="18">
+        <f t="shared" ref="G190:H190" si="7">SUM(G154:G189)</f>
+        <v>34.659999999999997</v>
+      </c>
+      <c r="H190" s="18">
+        <f t="shared" si="7"/>
+        <v>19.16</v>
+      </c>
+      <c r="I190" s="18">
+        <f t="shared" si="6"/>
+        <v>-15.499999999999996</v>
+      </c>
+      <c r="J190" s="19"/>
+      <c r="K190" s="46"/>
+    </row>
+    <row r="191" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="B191" s="62"/>
+      <c r="C191" s="62"/>
+      <c r="D191" s="62"/>
+      <c r="E191" s="62"/>
+      <c r="F191" s="62"/>
+      <c r="G191" s="62"/>
+      <c r="H191" s="62"/>
+      <c r="I191" s="62"/>
+      <c r="J191" s="62"/>
+      <c r="K191" s="63"/>
+    </row>
+    <row r="192" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A192" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B192" s="71" t="s">
+        <v>13</v>
+      </c>
+      <c r="C192" s="62"/>
+      <c r="D192" s="62"/>
+      <c r="E192" s="62"/>
+      <c r="F192" s="62"/>
+      <c r="G192" s="62"/>
+      <c r="H192" s="62"/>
+      <c r="I192" s="62"/>
+      <c r="J192" s="62"/>
+      <c r="K192" s="63"/>
+    </row>
+    <row r="193" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B193" s="71" t="s">
+        <v>15</v>
+      </c>
+      <c r="C193" s="62"/>
+      <c r="D193" s="62"/>
+      <c r="E193" s="62"/>
+      <c r="F193" s="62"/>
+      <c r="G193" s="62"/>
+      <c r="H193" s="62"/>
+      <c r="I193" s="62"/>
+      <c r="J193" s="62"/>
+      <c r="K193" s="63"/>
+    </row>
+    <row r="194" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A194" s="37"/>
+      <c r="B194" s="38"/>
+      <c r="C194" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D190" s="38"/>
-      <c r="E190" s="40"/>
-      <c r="F190" s="40"/>
-      <c r="G190" s="41"/>
-      <c r="H190" s="41"/>
-      <c r="I190" s="41">
+      <c r="D194" s="38"/>
+      <c r="E194" s="40"/>
+      <c r="F194" s="40"/>
+      <c r="G194" s="41"/>
+      <c r="H194" s="41"/>
+      <c r="I194" s="41">
+        <f t="shared" ref="I194:I204" si="8">H194-G194</f>
+        <v>0</v>
+      </c>
+      <c r="J194" s="45"/>
+      <c r="K194" s="43"/>
+    </row>
+    <row r="195" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A195" s="37"/>
+      <c r="B195" s="38"/>
+      <c r="C195" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D195" s="38"/>
+      <c r="E195" s="40"/>
+      <c r="F195" s="40"/>
+      <c r="G195" s="41"/>
+      <c r="H195" s="41"/>
+      <c r="I195" s="41">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J190" s="45"/>
-      <c r="K190" s="43"/>
-    </row>
-    <row r="191" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A191" s="37"/>
-      <c r="B191" s="38"/>
-      <c r="C191" s="39" t="s">
+      <c r="J195" s="45"/>
+      <c r="K195" s="43"/>
+    </row>
+    <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A196" s="37"/>
+      <c r="B196" s="38"/>
+      <c r="C196" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D191" s="38"/>
-      <c r="E191" s="40"/>
-      <c r="F191" s="40"/>
-      <c r="G191" s="41"/>
-      <c r="H191" s="41"/>
-      <c r="I191" s="41">
+      <c r="D196" s="38"/>
+      <c r="E196" s="40"/>
+      <c r="F196" s="40"/>
+      <c r="G196" s="41"/>
+      <c r="H196" s="41"/>
+      <c r="I196" s="41">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J191" s="45"/>
-      <c r="K191" s="43"/>
-    </row>
-    <row r="192" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A192" s="37"/>
-      <c r="B192" s="38"/>
-      <c r="C192" s="39" t="s">
+      <c r="J196" s="45"/>
+      <c r="K196" s="43" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="197" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A197" s="37"/>
+      <c r="B197" s="38"/>
+      <c r="C197" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D192" s="38"/>
-      <c r="E192" s="40"/>
-      <c r="F192" s="40"/>
-      <c r="G192" s="41"/>
-      <c r="H192" s="41"/>
-      <c r="I192" s="41">
+      <c r="D197" s="38"/>
+      <c r="E197" s="40"/>
+      <c r="F197" s="40"/>
+      <c r="G197" s="41"/>
+      <c r="H197" s="41"/>
+      <c r="I197" s="41">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J192" s="45"/>
-      <c r="K192" s="43"/>
-    </row>
-    <row r="193" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A193" s="37"/>
-      <c r="B193" s="38"/>
-      <c r="C193" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D193" s="38"/>
-      <c r="E193" s="40"/>
-      <c r="F193" s="40"/>
-      <c r="G193" s="41"/>
-      <c r="H193" s="41"/>
-      <c r="I193" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J193" s="45"/>
-      <c r="K193" s="43"/>
-    </row>
-    <row r="194" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A194" s="13"/>
-      <c r="B194" s="15"/>
-      <c r="C194" s="15"/>
-      <c r="D194" s="15"/>
-      <c r="E194" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F194" s="15"/>
-      <c r="G194" s="18">
-        <f t="shared" ref="G194:H194" si="9">SUM(G184:G193)</f>
-        <v>0</v>
-      </c>
-      <c r="H194" s="18">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="I194" s="18">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J194" s="19"/>
-      <c r="K194" s="46"/>
-    </row>
-    <row r="195" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="57" t="s">
-        <v>26</v>
-      </c>
-      <c r="B195" s="55"/>
-      <c r="C195" s="55"/>
-      <c r="D195" s="55"/>
-      <c r="E195" s="55"/>
-      <c r="F195" s="55"/>
-      <c r="G195" s="55"/>
-      <c r="H195" s="55"/>
-      <c r="I195" s="55"/>
-      <c r="J195" s="55"/>
-      <c r="K195" s="56"/>
-    </row>
-    <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A196" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B196" s="75" t="s">
-        <v>13</v>
-      </c>
-      <c r="C196" s="55"/>
-      <c r="D196" s="55"/>
-      <c r="E196" s="55"/>
-      <c r="F196" s="55"/>
-      <c r="G196" s="55"/>
-      <c r="H196" s="55"/>
-      <c r="I196" s="55"/>
-      <c r="J196" s="55"/>
-      <c r="K196" s="56"/>
-    </row>
-    <row r="197" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A197" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B197" s="75" t="s">
-        <v>15</v>
-      </c>
-      <c r="C197" s="55"/>
-      <c r="D197" s="55"/>
-      <c r="E197" s="55"/>
-      <c r="F197" s="55"/>
-      <c r="G197" s="55"/>
-      <c r="H197" s="55"/>
-      <c r="I197" s="55"/>
-      <c r="J197" s="55"/>
-      <c r="K197" s="56"/>
+      <c r="J197" s="45"/>
+      <c r="K197" s="43"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="37"/>
@@ -7723,7 +7790,7 @@
       <c r="G198" s="41"/>
       <c r="H198" s="41"/>
       <c r="I198" s="41">
-        <f t="shared" ref="I198:I208" si="10">H198-G198</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J198" s="45"/>
@@ -7741,7 +7808,7 @@
       <c r="G199" s="41"/>
       <c r="H199" s="41"/>
       <c r="I199" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J199" s="45"/>
@@ -7759,7 +7826,7 @@
       <c r="G200" s="41"/>
       <c r="H200" s="41"/>
       <c r="I200" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J200" s="45"/>
@@ -7777,7 +7844,7 @@
       <c r="G201" s="41"/>
       <c r="H201" s="41"/>
       <c r="I201" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J201" s="45"/>
@@ -7795,7 +7862,7 @@
       <c r="G202" s="41"/>
       <c r="H202" s="41"/>
       <c r="I202" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J202" s="45"/>
@@ -7813,156 +7880,156 @@
       <c r="G203" s="41"/>
       <c r="H203" s="41"/>
       <c r="I203" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J203" s="45"/>
       <c r="K203" s="43"/>
     </row>
     <row r="204" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A204" s="37"/>
-      <c r="B204" s="38"/>
-      <c r="C204" s="39" t="s">
+      <c r="A204" s="13"/>
+      <c r="B204" s="15"/>
+      <c r="C204" s="15"/>
+      <c r="D204" s="15"/>
+      <c r="E204" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F204" s="15"/>
+      <c r="G204" s="18">
+        <f t="shared" ref="G204:H204" si="9">SUM(G194:G203)</f>
+        <v>0</v>
+      </c>
+      <c r="H204" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="I204" s="18">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J204" s="19"/>
+      <c r="K204" s="46"/>
+    </row>
+    <row r="205" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="B205" s="62"/>
+      <c r="C205" s="62"/>
+      <c r="D205" s="62"/>
+      <c r="E205" s="62"/>
+      <c r="F205" s="62"/>
+      <c r="G205" s="62"/>
+      <c r="H205" s="62"/>
+      <c r="I205" s="62"/>
+      <c r="J205" s="62"/>
+      <c r="K205" s="63"/>
+    </row>
+    <row r="206" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A206" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B206" s="69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C206" s="62"/>
+      <c r="D206" s="62"/>
+      <c r="E206" s="62"/>
+      <c r="F206" s="62"/>
+      <c r="G206" s="62"/>
+      <c r="H206" s="62"/>
+      <c r="I206" s="62"/>
+      <c r="J206" s="62"/>
+      <c r="K206" s="63"/>
+    </row>
+    <row r="207" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B207" s="69" t="s">
+        <v>15</v>
+      </c>
+      <c r="C207" s="62"/>
+      <c r="D207" s="62"/>
+      <c r="E207" s="62"/>
+      <c r="F207" s="62"/>
+      <c r="G207" s="62"/>
+      <c r="H207" s="62"/>
+      <c r="I207" s="62"/>
+      <c r="J207" s="62"/>
+      <c r="K207" s="63"/>
+    </row>
+    <row r="208" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A208" s="37"/>
+      <c r="B208" s="38"/>
+      <c r="C208" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D204" s="38"/>
-      <c r="E204" s="40"/>
-      <c r="F204" s="40"/>
-      <c r="G204" s="41"/>
-      <c r="H204" s="41"/>
-      <c r="I204" s="41">
+      <c r="D208" s="38"/>
+      <c r="E208" s="40"/>
+      <c r="F208" s="40"/>
+      <c r="G208" s="41"/>
+      <c r="H208" s="41"/>
+      <c r="I208" s="41">
+        <f t="shared" ref="I208:I218" si="10">H208-G208</f>
+        <v>0</v>
+      </c>
+      <c r="J208" s="45"/>
+      <c r="K208" s="43"/>
+    </row>
+    <row r="209" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A209" s="37"/>
+      <c r="B209" s="38"/>
+      <c r="C209" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D209" s="38"/>
+      <c r="E209" s="40"/>
+      <c r="F209" s="40"/>
+      <c r="G209" s="41"/>
+      <c r="H209" s="41"/>
+      <c r="I209" s="41">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J204" s="45"/>
-      <c r="K204" s="43"/>
-    </row>
-    <row r="205" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A205" s="37"/>
-      <c r="B205" s="38"/>
-      <c r="C205" s="39" t="s">
+      <c r="J209" s="45"/>
+      <c r="K209" s="43"/>
+    </row>
+    <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A210" s="37"/>
+      <c r="B210" s="38"/>
+      <c r="C210" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D205" s="38"/>
-      <c r="E205" s="40"/>
-      <c r="F205" s="40"/>
-      <c r="G205" s="41"/>
-      <c r="H205" s="41"/>
-      <c r="I205" s="41">
+      <c r="D210" s="38"/>
+      <c r="E210" s="40"/>
+      <c r="F210" s="40"/>
+      <c r="G210" s="41"/>
+      <c r="H210" s="41"/>
+      <c r="I210" s="41">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J205" s="45"/>
-      <c r="K205" s="43"/>
-    </row>
-    <row r="206" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A206" s="37"/>
-      <c r="B206" s="38"/>
-      <c r="C206" s="39" t="s">
+      <c r="J210" s="45"/>
+      <c r="K210" s="43"/>
+    </row>
+    <row r="211" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A211" s="37"/>
+      <c r="B211" s="38"/>
+      <c r="C211" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D206" s="38"/>
-      <c r="E206" s="40"/>
-      <c r="F206" s="40"/>
-      <c r="G206" s="41"/>
-      <c r="H206" s="41"/>
-      <c r="I206" s="41">
+      <c r="D211" s="38"/>
+      <c r="E211" s="40"/>
+      <c r="F211" s="40"/>
+      <c r="G211" s="41"/>
+      <c r="H211" s="41"/>
+      <c r="I211" s="41">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J206" s="45"/>
-      <c r="K206" s="43"/>
-    </row>
-    <row r="207" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A207" s="37"/>
-      <c r="B207" s="38"/>
-      <c r="C207" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D207" s="38"/>
-      <c r="E207" s="40"/>
-      <c r="F207" s="40"/>
-      <c r="G207" s="41"/>
-      <c r="H207" s="41"/>
-      <c r="I207" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J207" s="45"/>
-      <c r="K207" s="43"/>
-    </row>
-    <row r="208" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A208" s="13"/>
-      <c r="B208" s="15"/>
-      <c r="C208" s="15"/>
-      <c r="D208" s="15"/>
-      <c r="E208" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F208" s="15"/>
-      <c r="G208" s="18">
-        <f t="shared" ref="G208:H208" si="11">SUM(G198:G207)</f>
-        <v>0</v>
-      </c>
-      <c r="H208" s="18">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I208" s="18">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J208" s="19"/>
-      <c r="K208" s="46"/>
-    </row>
-    <row r="209" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A209" s="62" t="s">
-        <v>27</v>
-      </c>
-      <c r="B209" s="63"/>
-      <c r="C209" s="63"/>
-      <c r="D209" s="63"/>
-      <c r="E209" s="63"/>
-      <c r="F209" s="63"/>
-      <c r="G209" s="63"/>
-      <c r="H209" s="63"/>
-      <c r="I209" s="63"/>
-      <c r="J209" s="63"/>
-      <c r="K209" s="64"/>
-    </row>
-    <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A210" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B210" s="65" t="s">
-        <v>13</v>
-      </c>
-      <c r="C210" s="63"/>
-      <c r="D210" s="63"/>
-      <c r="E210" s="63"/>
-      <c r="F210" s="63"/>
-      <c r="G210" s="63"/>
-      <c r="H210" s="63"/>
-      <c r="I210" s="63"/>
-      <c r="J210" s="63"/>
-      <c r="K210" s="64"/>
-    </row>
-    <row r="211" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A211" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B211" s="65" t="s">
-        <v>15</v>
-      </c>
-      <c r="C211" s="63"/>
-      <c r="D211" s="63"/>
-      <c r="E211" s="63"/>
-      <c r="F211" s="63"/>
-      <c r="G211" s="63"/>
-      <c r="H211" s="63"/>
-      <c r="I211" s="63"/>
-      <c r="J211" s="63"/>
-      <c r="K211" s="64"/>
+      <c r="J211" s="45"/>
+      <c r="K211" s="43"/>
     </row>
     <row r="212" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A212" s="37"/>
@@ -7976,7 +8043,7 @@
       <c r="G212" s="41"/>
       <c r="H212" s="41"/>
       <c r="I212" s="41">
-        <f t="shared" ref="I212:I222" si="12">H212-G212</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J212" s="45"/>
@@ -7994,7 +8061,7 @@
       <c r="G213" s="41"/>
       <c r="H213" s="41"/>
       <c r="I213" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J213" s="45"/>
@@ -8012,7 +8079,7 @@
       <c r="G214" s="41"/>
       <c r="H214" s="41"/>
       <c r="I214" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J214" s="45"/>
@@ -8030,7 +8097,7 @@
       <c r="G215" s="41"/>
       <c r="H215" s="41"/>
       <c r="I215" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J215" s="45"/>
@@ -8048,7 +8115,7 @@
       <c r="G216" s="41"/>
       <c r="H216" s="41"/>
       <c r="I216" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J216" s="45"/>
@@ -8066,114 +8133,295 @@
       <c r="G217" s="41"/>
       <c r="H217" s="41"/>
       <c r="I217" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J217" s="45"/>
       <c r="K217" s="43"/>
     </row>
     <row r="218" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A218" s="37"/>
-      <c r="B218" s="38"/>
-      <c r="C218" s="39" t="s">
+      <c r="A218" s="13"/>
+      <c r="B218" s="15"/>
+      <c r="C218" s="15"/>
+      <c r="D218" s="15"/>
+      <c r="E218" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F218" s="15"/>
+      <c r="G218" s="18">
+        <f t="shared" ref="G218:H218" si="11">SUM(G208:G217)</f>
+        <v>0</v>
+      </c>
+      <c r="H218" s="18">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="I218" s="18">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J218" s="19"/>
+      <c r="K218" s="46"/>
+    </row>
+    <row r="219" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="54" t="s">
+        <v>27</v>
+      </c>
+      <c r="B219" s="55"/>
+      <c r="C219" s="55"/>
+      <c r="D219" s="55"/>
+      <c r="E219" s="55"/>
+      <c r="F219" s="55"/>
+      <c r="G219" s="55"/>
+      <c r="H219" s="55"/>
+      <c r="I219" s="55"/>
+      <c r="J219" s="55"/>
+      <c r="K219" s="56"/>
+    </row>
+    <row r="220" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A220" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B220" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C220" s="55"/>
+      <c r="D220" s="55"/>
+      <c r="E220" s="55"/>
+      <c r="F220" s="55"/>
+      <c r="G220" s="55"/>
+      <c r="H220" s="55"/>
+      <c r="I220" s="55"/>
+      <c r="J220" s="55"/>
+      <c r="K220" s="56"/>
+    </row>
+    <row r="221" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A221" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B221" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C221" s="55"/>
+      <c r="D221" s="55"/>
+      <c r="E221" s="55"/>
+      <c r="F221" s="55"/>
+      <c r="G221" s="55"/>
+      <c r="H221" s="55"/>
+      <c r="I221" s="55"/>
+      <c r="J221" s="55"/>
+      <c r="K221" s="56"/>
+    </row>
+    <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A222" s="37"/>
+      <c r="B222" s="38"/>
+      <c r="C222" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D218" s="38"/>
-      <c r="E218" s="40"/>
-      <c r="F218" s="40"/>
-      <c r="G218" s="41"/>
-      <c r="H218" s="41"/>
-      <c r="I218" s="41">
+      <c r="D222" s="38"/>
+      <c r="E222" s="40"/>
+      <c r="F222" s="40"/>
+      <c r="G222" s="41"/>
+      <c r="H222" s="41"/>
+      <c r="I222" s="41">
+        <f t="shared" ref="I222:I232" si="12">H222-G222</f>
+        <v>0</v>
+      </c>
+      <c r="J222" s="45"/>
+      <c r="K222" s="43"/>
+    </row>
+    <row r="223" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A223" s="37"/>
+      <c r="B223" s="38"/>
+      <c r="C223" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D223" s="38"/>
+      <c r="E223" s="40"/>
+      <c r="F223" s="40"/>
+      <c r="G223" s="41"/>
+      <c r="H223" s="41"/>
+      <c r="I223" s="41">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J218" s="45"/>
-      <c r="K218" s="43"/>
-    </row>
-    <row r="219" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A219" s="37"/>
-      <c r="B219" s="38"/>
-      <c r="C219" s="39" t="s">
+      <c r="J223" s="45"/>
+      <c r="K223" s="43"/>
+    </row>
+    <row r="224" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A224" s="37"/>
+      <c r="B224" s="38"/>
+      <c r="C224" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D219" s="38"/>
-      <c r="E219" s="40"/>
-      <c r="F219" s="40"/>
-      <c r="G219" s="41"/>
-      <c r="H219" s="41"/>
-      <c r="I219" s="41">
+      <c r="D224" s="38"/>
+      <c r="E224" s="40"/>
+      <c r="F224" s="40"/>
+      <c r="G224" s="41"/>
+      <c r="H224" s="41"/>
+      <c r="I224" s="41">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J219" s="45"/>
-      <c r="K219" s="43"/>
-    </row>
-    <row r="220" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A220" s="37"/>
-      <c r="B220" s="38"/>
-      <c r="C220" s="39" t="s">
+      <c r="J224" s="45"/>
+      <c r="K224" s="43"/>
+    </row>
+    <row r="225" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A225" s="37"/>
+      <c r="B225" s="38"/>
+      <c r="C225" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D220" s="38"/>
-      <c r="E220" s="40"/>
-      <c r="F220" s="40"/>
-      <c r="G220" s="41"/>
-      <c r="H220" s="41"/>
-      <c r="I220" s="41">
+      <c r="D225" s="38"/>
+      <c r="E225" s="40"/>
+      <c r="F225" s="40"/>
+      <c r="G225" s="41"/>
+      <c r="H225" s="41"/>
+      <c r="I225" s="41">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J220" s="45"/>
-      <c r="K220" s="43"/>
-    </row>
-    <row r="221" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A221" s="37"/>
-      <c r="B221" s="38"/>
-      <c r="C221" s="39" t="s">
+      <c r="J225" s="45"/>
+      <c r="K225" s="43"/>
+    </row>
+    <row r="226" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A226" s="37"/>
+      <c r="B226" s="38"/>
+      <c r="C226" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D221" s="38"/>
-      <c r="E221" s="40"/>
-      <c r="F221" s="40"/>
-      <c r="G221" s="41"/>
-      <c r="H221" s="41"/>
-      <c r="I221" s="41">
+      <c r="D226" s="38"/>
+      <c r="E226" s="40"/>
+      <c r="F226" s="40"/>
+      <c r="G226" s="41"/>
+      <c r="H226" s="41"/>
+      <c r="I226" s="41">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J221" s="45"/>
-      <c r="K221" s="43"/>
-    </row>
-    <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A222" s="48"/>
-      <c r="B222" s="49"/>
-      <c r="C222" s="49"/>
-      <c r="D222" s="49"/>
-      <c r="E222" s="49" t="s">
+      <c r="J226" s="45"/>
+      <c r="K226" s="43"/>
+    </row>
+    <row r="227" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A227" s="37"/>
+      <c r="B227" s="38"/>
+      <c r="C227" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D227" s="38"/>
+      <c r="E227" s="40"/>
+      <c r="F227" s="40"/>
+      <c r="G227" s="41"/>
+      <c r="H227" s="41"/>
+      <c r="I227" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J227" s="45"/>
+      <c r="K227" s="43"/>
+    </row>
+    <row r="228" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A228" s="37"/>
+      <c r="B228" s="38"/>
+      <c r="C228" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D228" s="38"/>
+      <c r="E228" s="40"/>
+      <c r="F228" s="40"/>
+      <c r="G228" s="41"/>
+      <c r="H228" s="41"/>
+      <c r="I228" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J228" s="45"/>
+      <c r="K228" s="43"/>
+    </row>
+    <row r="229" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A229" s="37"/>
+      <c r="B229" s="38"/>
+      <c r="C229" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D229" s="38"/>
+      <c r="E229" s="40"/>
+      <c r="F229" s="40"/>
+      <c r="G229" s="41"/>
+      <c r="H229" s="41"/>
+      <c r="I229" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J229" s="45"/>
+      <c r="K229" s="43"/>
+    </row>
+    <row r="230" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A230" s="37"/>
+      <c r="B230" s="38"/>
+      <c r="C230" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D230" s="38"/>
+      <c r="E230" s="40"/>
+      <c r="F230" s="40"/>
+      <c r="G230" s="41"/>
+      <c r="H230" s="41"/>
+      <c r="I230" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J230" s="45"/>
+      <c r="K230" s="43"/>
+    </row>
+    <row r="231" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A231" s="37"/>
+      <c r="B231" s="38"/>
+      <c r="C231" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D231" s="38"/>
+      <c r="E231" s="40"/>
+      <c r="F231" s="40"/>
+      <c r="G231" s="41"/>
+      <c r="H231" s="41"/>
+      <c r="I231" s="41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J231" s="45"/>
+      <c r="K231" s="43"/>
+    </row>
+    <row r="232" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A232" s="48"/>
+      <c r="B232" s="49"/>
+      <c r="C232" s="49"/>
+      <c r="D232" s="49"/>
+      <c r="E232" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F222" s="49"/>
-      <c r="G222" s="50">
-        <f t="shared" ref="G222:H222" si="13">SUM(G212:G221)</f>
-        <v>0</v>
-      </c>
-      <c r="H222" s="50">
+      <c r="F232" s="49"/>
+      <c r="G232" s="50">
+        <f t="shared" ref="G232:H232" si="13">SUM(G222:G231)</f>
+        <v>0</v>
+      </c>
+      <c r="H232" s="50">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="I222" s="50">
+      <c r="I232" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J222" s="51"/>
-      <c r="K222" s="52"/>
+      <c r="J232" s="51"/>
+      <c r="K232" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{746F7D6D-6DAD-4C2D-BC98-A9B5ADA04487}">
+      <autoFilter ref="A1:K15" xr:uid="{C6B22F4D-F1D6-44A9-B873-E0C60B5C503D}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -8184,9 +8432,17 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A209:K209"/>
-    <mergeCell ref="B210:K210"/>
-    <mergeCell ref="B211:K211"/>
+    <mergeCell ref="B192:K192"/>
+    <mergeCell ref="B193:K193"/>
+    <mergeCell ref="A205:K205"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A191:K191"/>
+    <mergeCell ref="A219:K219"/>
+    <mergeCell ref="B220:K220"/>
+    <mergeCell ref="B221:K221"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -8197,19 +8453,11 @@
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
     <mergeCell ref="A118:K118"/>
-    <mergeCell ref="B196:K196"/>
-    <mergeCell ref="B197:K197"/>
+    <mergeCell ref="B206:K206"/>
+    <mergeCell ref="B207:K207"/>
     <mergeCell ref="B119:K119"/>
-    <mergeCell ref="B182:K182"/>
-    <mergeCell ref="B183:K183"/>
-    <mergeCell ref="A195:K195"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A181:K181"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B179 B184:B193 B198:B207">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B189 B194:B203 B208:B217">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -8226,7 +8474,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B152:B180 B182:B194 B196:B208 B210:B222">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B152:B190 B192:B204 B206:B218 B220:B232">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -8234,34 +8482,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B212:B221">
+  <conditionalFormatting sqref="B222:B231">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B212))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B222))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B212))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B222))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B212))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B222))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B212))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B222))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B212))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B222))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G154:G180 G184:G194 G198:G208 G212:G222">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G154:G190 G194:G204 G208:G218 G222:G232">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H222">
+  <conditionalFormatting sqref="H1:H232">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I154:I180 I184:I194 I198:I208 I212:I222">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I194:I204 I208:I218 I222:I232 I154:I190">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -8270,7 +8518,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F212:F221 F198:F207 F86:F116 F154:F179 F184:F193 F5:F45 F50:F81 F121:F149" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F222:F231 F208:F217 F86:F116 F154:F189 F194:F203 F5:F45 F50:F81 F121:F149" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8286,13 +8534,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E116 E154:E179 E184:E193 E198:E207 E212:E221 E50:E81 E121:E149</xm:sqref>
+          <xm:sqref>E5:E45 E86:E116 E154:E189 E194:E203 E208:E217 E222:E231 E50:E81 E121:E149</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B116 B154:B179 B184:B193 B198:B207 B212:B221 B50:B81 B121:B149</xm:sqref>
+          <xm:sqref>B5:B45 B86:B116 B154:B189 B194:B203 B208:B217 B222:B231 B50:B81 B121:B149</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -9933,26 +10181,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -10187,10 +10415,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10207,20 +10466,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W5 DataLab 1 Work V (End of DataLab)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8028CE-5F24-4CA0-BF52-E158941D3939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BB232EB-8AB6-4425-968F-7285EA28ADFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="288">
   <si>
     <t>Date</t>
   </si>
@@ -963,9 +963,6 @@
   </si>
   <si>
     <t>I understood the mathematical concept of multivariable calculus pretty quickly and so it didn't take as long as I predicted it to.</t>
-  </si>
-  <si>
-    <t>from 14:30</t>
   </si>
   <si>
     <t>As stated above, I understood the concepts pretty quickly and did not have too much troubles with the quiz.</t>
@@ -1454,6 +1451,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1470,8 +1487,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1489,24 +1504,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2031,53 +2028,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3416,53 +3413,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4515,53 +4512,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5576,53 +5573,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="68" t="s">
+      <c r="A118" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="62"/>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
+      <c r="B118" s="55"/>
+      <c r="C118" s="55"/>
+      <c r="D118" s="55"/>
+      <c r="E118" s="55"/>
+      <c r="F118" s="55"/>
+      <c r="G118" s="55"/>
+      <c r="H118" s="55"/>
+      <c r="I118" s="55"/>
+      <c r="J118" s="55"/>
+      <c r="K118" s="56"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="70" t="s">
+      <c r="B119" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="62"/>
-      <c r="D119" s="62"/>
-      <c r="E119" s="62"/>
-      <c r="F119" s="62"/>
-      <c r="G119" s="62"/>
-      <c r="H119" s="62"/>
-      <c r="I119" s="62"/>
-      <c r="J119" s="62"/>
-      <c r="K119" s="63"/>
+      <c r="C119" s="55"/>
+      <c r="D119" s="55"/>
+      <c r="E119" s="55"/>
+      <c r="F119" s="55"/>
+      <c r="G119" s="55"/>
+      <c r="H119" s="55"/>
+      <c r="I119" s="55"/>
+      <c r="J119" s="55"/>
+      <c r="K119" s="56"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="70" t="s">
+      <c r="B120" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="62"/>
-      <c r="D120" s="62"/>
-      <c r="E120" s="62"/>
-      <c r="F120" s="62"/>
-      <c r="G120" s="62"/>
-      <c r="H120" s="62"/>
-      <c r="I120" s="62"/>
-      <c r="J120" s="62"/>
-      <c r="K120" s="63"/>
+      <c r="C120" s="55"/>
+      <c r="D120" s="55"/>
+      <c r="E120" s="55"/>
+      <c r="F120" s="55"/>
+      <c r="G120" s="55"/>
+      <c r="H120" s="55"/>
+      <c r="I120" s="55"/>
+      <c r="J120" s="55"/>
+      <c r="K120" s="56"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6559,53 +6556,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="73" t="s">
+      <c r="A151" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="62"/>
-      <c r="C151" s="62"/>
-      <c r="D151" s="62"/>
-      <c r="E151" s="62"/>
-      <c r="F151" s="62"/>
-      <c r="G151" s="62"/>
-      <c r="H151" s="62"/>
-      <c r="I151" s="62"/>
-      <c r="J151" s="62"/>
-      <c r="K151" s="63"/>
+      <c r="B151" s="55"/>
+      <c r="C151" s="55"/>
+      <c r="D151" s="55"/>
+      <c r="E151" s="55"/>
+      <c r="F151" s="55"/>
+      <c r="G151" s="55"/>
+      <c r="H151" s="55"/>
+      <c r="I151" s="55"/>
+      <c r="J151" s="55"/>
+      <c r="K151" s="56"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="74" t="s">
+      <c r="B152" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="62"/>
-      <c r="D152" s="62"/>
-      <c r="E152" s="62"/>
-      <c r="F152" s="62"/>
-      <c r="G152" s="62"/>
-      <c r="H152" s="62"/>
-      <c r="I152" s="62"/>
-      <c r="J152" s="62"/>
-      <c r="K152" s="63"/>
+      <c r="C152" s="55"/>
+      <c r="D152" s="55"/>
+      <c r="E152" s="55"/>
+      <c r="F152" s="55"/>
+      <c r="G152" s="55"/>
+      <c r="H152" s="55"/>
+      <c r="I152" s="55"/>
+      <c r="J152" s="55"/>
+      <c r="K152" s="56"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="74" t="s">
+      <c r="B153" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="62"/>
-      <c r="D153" s="62"/>
-      <c r="E153" s="62"/>
-      <c r="F153" s="62"/>
-      <c r="G153" s="62"/>
-      <c r="H153" s="62"/>
-      <c r="I153" s="62"/>
-      <c r="J153" s="62"/>
-      <c r="K153" s="63"/>
+      <c r="C153" s="55"/>
+      <c r="D153" s="55"/>
+      <c r="E153" s="55"/>
+      <c r="F153" s="55"/>
+      <c r="G153" s="55"/>
+      <c r="H153" s="55"/>
+      <c r="I153" s="55"/>
+      <c r="J153" s="55"/>
+      <c r="K153" s="56"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -7438,7 +7435,7 @@
       </c>
       <c r="J179" s="45"/>
       <c r="K179" s="43" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="180" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -7446,7 +7443,7 @@
         <v>45643</v>
       </c>
       <c r="B180" s="38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C180" s="39" t="s">
         <v>283</v>
@@ -7463,15 +7460,15 @@
       <c r="G180" s="41">
         <v>3</v>
       </c>
-      <c r="H180" s="41"/>
+      <c r="H180" s="41">
+        <v>2.5</v>
+      </c>
       <c r="I180" s="41">
         <f t="shared" si="6"/>
-        <v>-3</v>
+        <v>-0.5</v>
       </c>
       <c r="J180" s="45"/>
-      <c r="K180" s="43" t="s">
-        <v>287</v>
-      </c>
+      <c r="K180" s="43"/>
     </row>
     <row r="181" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A181" s="37"/>
@@ -7646,63 +7643,63 @@
       </c>
       <c r="H190" s="18">
         <f t="shared" si="7"/>
-        <v>19.16</v>
+        <v>21.66</v>
       </c>
       <c r="I190" s="18">
         <f t="shared" si="6"/>
-        <v>-15.499999999999996</v>
+        <v>-12.999999999999996</v>
       </c>
       <c r="J190" s="19"/>
       <c r="K190" s="46"/>
     </row>
     <row r="191" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A191" s="75" t="s">
+      <c r="A191" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B191" s="62"/>
-      <c r="C191" s="62"/>
-      <c r="D191" s="62"/>
-      <c r="E191" s="62"/>
-      <c r="F191" s="62"/>
-      <c r="G191" s="62"/>
-      <c r="H191" s="62"/>
-      <c r="I191" s="62"/>
-      <c r="J191" s="62"/>
-      <c r="K191" s="63"/>
+      <c r="B191" s="55"/>
+      <c r="C191" s="55"/>
+      <c r="D191" s="55"/>
+      <c r="E191" s="55"/>
+      <c r="F191" s="55"/>
+      <c r="G191" s="55"/>
+      <c r="H191" s="55"/>
+      <c r="I191" s="55"/>
+      <c r="J191" s="55"/>
+      <c r="K191" s="56"/>
     </row>
     <row r="192" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A192" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B192" s="71" t="s">
+      <c r="B192" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C192" s="62"/>
-      <c r="D192" s="62"/>
-      <c r="E192" s="62"/>
-      <c r="F192" s="62"/>
-      <c r="G192" s="62"/>
-      <c r="H192" s="62"/>
-      <c r="I192" s="62"/>
-      <c r="J192" s="62"/>
-      <c r="K192" s="63"/>
+      <c r="C192" s="55"/>
+      <c r="D192" s="55"/>
+      <c r="E192" s="55"/>
+      <c r="F192" s="55"/>
+      <c r="G192" s="55"/>
+      <c r="H192" s="55"/>
+      <c r="I192" s="55"/>
+      <c r="J192" s="55"/>
+      <c r="K192" s="56"/>
     </row>
     <row r="193" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B193" s="71" t="s">
+      <c r="B193" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C193" s="62"/>
-      <c r="D193" s="62"/>
-      <c r="E193" s="62"/>
-      <c r="F193" s="62"/>
-      <c r="G193" s="62"/>
-      <c r="H193" s="62"/>
-      <c r="I193" s="62"/>
-      <c r="J193" s="62"/>
-      <c r="K193" s="63"/>
+      <c r="C193" s="55"/>
+      <c r="D193" s="55"/>
+      <c r="E193" s="55"/>
+      <c r="F193" s="55"/>
+      <c r="G193" s="55"/>
+      <c r="H193" s="55"/>
+      <c r="I193" s="55"/>
+      <c r="J193" s="55"/>
+      <c r="K193" s="56"/>
     </row>
     <row r="194" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A194" s="37"/>
@@ -7911,53 +7908,53 @@
       <c r="K204" s="46"/>
     </row>
     <row r="205" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A205" s="72" t="s">
+      <c r="A205" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B205" s="62"/>
-      <c r="C205" s="62"/>
-      <c r="D205" s="62"/>
-      <c r="E205" s="62"/>
-      <c r="F205" s="62"/>
-      <c r="G205" s="62"/>
-      <c r="H205" s="62"/>
-      <c r="I205" s="62"/>
-      <c r="J205" s="62"/>
-      <c r="K205" s="63"/>
+      <c r="B205" s="55"/>
+      <c r="C205" s="55"/>
+      <c r="D205" s="55"/>
+      <c r="E205" s="55"/>
+      <c r="F205" s="55"/>
+      <c r="G205" s="55"/>
+      <c r="H205" s="55"/>
+      <c r="I205" s="55"/>
+      <c r="J205" s="55"/>
+      <c r="K205" s="56"/>
     </row>
     <row r="206" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A206" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B206" s="69" t="s">
+      <c r="B206" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C206" s="62"/>
-      <c r="D206" s="62"/>
-      <c r="E206" s="62"/>
-      <c r="F206" s="62"/>
-      <c r="G206" s="62"/>
-      <c r="H206" s="62"/>
-      <c r="I206" s="62"/>
-      <c r="J206" s="62"/>
-      <c r="K206" s="63"/>
+      <c r="C206" s="55"/>
+      <c r="D206" s="55"/>
+      <c r="E206" s="55"/>
+      <c r="F206" s="55"/>
+      <c r="G206" s="55"/>
+      <c r="H206" s="55"/>
+      <c r="I206" s="55"/>
+      <c r="J206" s="55"/>
+      <c r="K206" s="56"/>
     </row>
     <row r="207" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B207" s="69" t="s">
+      <c r="B207" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C207" s="62"/>
-      <c r="D207" s="62"/>
-      <c r="E207" s="62"/>
-      <c r="F207" s="62"/>
-      <c r="G207" s="62"/>
-      <c r="H207" s="62"/>
-      <c r="I207" s="62"/>
-      <c r="J207" s="62"/>
-      <c r="K207" s="63"/>
+      <c r="C207" s="55"/>
+      <c r="D207" s="55"/>
+      <c r="E207" s="55"/>
+      <c r="F207" s="55"/>
+      <c r="G207" s="55"/>
+      <c r="H207" s="55"/>
+      <c r="I207" s="55"/>
+      <c r="J207" s="55"/>
+      <c r="K207" s="56"/>
     </row>
     <row r="208" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A208" s="37"/>
@@ -8164,53 +8161,53 @@
       <c r="K218" s="46"/>
     </row>
     <row r="219" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="54" t="s">
+      <c r="A219" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B219" s="55"/>
-      <c r="C219" s="55"/>
-      <c r="D219" s="55"/>
-      <c r="E219" s="55"/>
-      <c r="F219" s="55"/>
-      <c r="G219" s="55"/>
-      <c r="H219" s="55"/>
-      <c r="I219" s="55"/>
-      <c r="J219" s="55"/>
-      <c r="K219" s="56"/>
+      <c r="B219" s="63"/>
+      <c r="C219" s="63"/>
+      <c r="D219" s="63"/>
+      <c r="E219" s="63"/>
+      <c r="F219" s="63"/>
+      <c r="G219" s="63"/>
+      <c r="H219" s="63"/>
+      <c r="I219" s="63"/>
+      <c r="J219" s="63"/>
+      <c r="K219" s="64"/>
     </row>
     <row r="220" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A220" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B220" s="57" t="s">
+      <c r="B220" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C220" s="55"/>
-      <c r="D220" s="55"/>
-      <c r="E220" s="55"/>
-      <c r="F220" s="55"/>
-      <c r="G220" s="55"/>
-      <c r="H220" s="55"/>
-      <c r="I220" s="55"/>
-      <c r="J220" s="55"/>
-      <c r="K220" s="56"/>
+      <c r="C220" s="63"/>
+      <c r="D220" s="63"/>
+      <c r="E220" s="63"/>
+      <c r="F220" s="63"/>
+      <c r="G220" s="63"/>
+      <c r="H220" s="63"/>
+      <c r="I220" s="63"/>
+      <c r="J220" s="63"/>
+      <c r="K220" s="64"/>
     </row>
     <row r="221" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B221" s="57" t="s">
+      <c r="B221" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C221" s="55"/>
-      <c r="D221" s="55"/>
-      <c r="E221" s="55"/>
-      <c r="F221" s="55"/>
-      <c r="G221" s="55"/>
-      <c r="H221" s="55"/>
-      <c r="I221" s="55"/>
-      <c r="J221" s="55"/>
-      <c r="K221" s="56"/>
+      <c r="C221" s="63"/>
+      <c r="D221" s="63"/>
+      <c r="E221" s="63"/>
+      <c r="F221" s="63"/>
+      <c r="G221" s="63"/>
+      <c r="H221" s="63"/>
+      <c r="I221" s="63"/>
+      <c r="J221" s="63"/>
+      <c r="K221" s="64"/>
     </row>
     <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A222" s="37"/>
@@ -8421,7 +8418,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{C6B22F4D-F1D6-44A9-B873-E0C60B5C503D}">
+      <autoFilter ref="A1:K15" xr:uid="{C341563A-5BC5-4F1E-BC72-B4C1ADE699F2}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -8432,14 +8429,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B192:K192"/>
-    <mergeCell ref="B193:K193"/>
-    <mergeCell ref="A205:K205"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A191:K191"/>
     <mergeCell ref="A219:K219"/>
     <mergeCell ref="B220:K220"/>
     <mergeCell ref="B221:K221"/>
@@ -8456,6 +8445,14 @@
     <mergeCell ref="B206:K206"/>
     <mergeCell ref="B207:K207"/>
     <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B192:K192"/>
+    <mergeCell ref="B193:K193"/>
+    <mergeCell ref="A205:K205"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A191:K191"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B189 B194:B203 B208:B217">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -8509,7 +8506,7 @@
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I194:I204 I208:I218 I222:I232 I154:I190">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I154:I190 I194:I204 I208:I218 I222:I232">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -10181,6 +10178,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -10415,27 +10432,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10452,23 +10468,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W5 DataLab 2 Work I
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BB232EB-8AB6-4425-968F-7285EA28ADFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24790124-BCC0-4623-BC8B-2D7D393573E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$217</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$220</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="300">
   <si>
     <t>Date</t>
   </si>
@@ -966,6 +966,42 @@
   </si>
   <si>
     <t>As stated above, I understood the concepts pretty quickly and did not have too much troubles with the quiz.</t>
+  </si>
+  <si>
+    <t>Stand-up meeting with mentor group</t>
+  </si>
+  <si>
+    <t>Datalab Practice</t>
+  </si>
+  <si>
+    <t>Do the DBSCAN Jupyter notebook</t>
+  </si>
+  <si>
+    <t>Implement Random Hierarchical Clustering</t>
+  </si>
+  <si>
+    <t>Implement DBSCAN for Density-Based Clustering</t>
+  </si>
+  <si>
+    <t>Evaluation and Model Comparison</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog actual hours</t>
+  </si>
+  <si>
+    <t>Fill in Learning Log for week 5</t>
+  </si>
+  <si>
+    <t>Evidence in Learning Log week 5</t>
+  </si>
+  <si>
+    <t>Evidence in WorkLog week 5</t>
+  </si>
+  <si>
+    <t>Read the DataCamp tutorials</t>
+  </si>
+  <si>
+    <t>0,1 so far</t>
   </si>
 </sst>
 </file>
@@ -1451,26 +1487,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1487,6 +1503,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1504,6 +1522,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1976,7 +2012,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K232"/>
+  <dimension ref="A1:K235"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -2028,53 +2064,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3413,53 +3449,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="62"/>
+      <c r="K49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4512,53 +4548,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72" t="s">
+      <c r="A83" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="55"/>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="55"/>
-      <c r="I83" s="55"/>
-      <c r="J83" s="55"/>
-      <c r="K83" s="56"/>
+      <c r="B83" s="62"/>
+      <c r="C83" s="62"/>
+      <c r="D83" s="62"/>
+      <c r="E83" s="62"/>
+      <c r="F83" s="62"/>
+      <c r="G83" s="62"/>
+      <c r="H83" s="62"/>
+      <c r="I83" s="62"/>
+      <c r="J83" s="62"/>
+      <c r="K83" s="63"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="73" t="s">
+      <c r="B84" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="55"/>
-      <c r="D84" s="55"/>
-      <c r="E84" s="55"/>
-      <c r="F84" s="55"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="55"/>
-      <c r="I84" s="55"/>
-      <c r="J84" s="55"/>
-      <c r="K84" s="56"/>
+      <c r="C84" s="62"/>
+      <c r="D84" s="62"/>
+      <c r="E84" s="62"/>
+      <c r="F84" s="62"/>
+      <c r="G84" s="62"/>
+      <c r="H84" s="62"/>
+      <c r="I84" s="62"/>
+      <c r="J84" s="62"/>
+      <c r="K84" s="63"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="73" t="s">
+      <c r="B85" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="55"/>
-      <c r="D85" s="55"/>
-      <c r="E85" s="55"/>
-      <c r="F85" s="55"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="55"/>
-      <c r="I85" s="55"/>
-      <c r="J85" s="55"/>
-      <c r="K85" s="56"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="62"/>
+      <c r="G85" s="62"/>
+      <c r="H85" s="62"/>
+      <c r="I85" s="62"/>
+      <c r="J85" s="62"/>
+      <c r="K85" s="63"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5573,53 +5609,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="74" t="s">
+      <c r="A118" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="55"/>
-      <c r="C118" s="55"/>
-      <c r="D118" s="55"/>
-      <c r="E118" s="55"/>
-      <c r="F118" s="55"/>
-      <c r="G118" s="55"/>
-      <c r="H118" s="55"/>
-      <c r="I118" s="55"/>
-      <c r="J118" s="55"/>
-      <c r="K118" s="56"/>
+      <c r="B118" s="62"/>
+      <c r="C118" s="62"/>
+      <c r="D118" s="62"/>
+      <c r="E118" s="62"/>
+      <c r="F118" s="62"/>
+      <c r="G118" s="62"/>
+      <c r="H118" s="62"/>
+      <c r="I118" s="62"/>
+      <c r="J118" s="62"/>
+      <c r="K118" s="63"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="58" t="s">
+      <c r="B119" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="55"/>
-      <c r="D119" s="55"/>
-      <c r="E119" s="55"/>
-      <c r="F119" s="55"/>
-      <c r="G119" s="55"/>
-      <c r="H119" s="55"/>
-      <c r="I119" s="55"/>
-      <c r="J119" s="55"/>
-      <c r="K119" s="56"/>
+      <c r="C119" s="62"/>
+      <c r="D119" s="62"/>
+      <c r="E119" s="62"/>
+      <c r="F119" s="62"/>
+      <c r="G119" s="62"/>
+      <c r="H119" s="62"/>
+      <c r="I119" s="62"/>
+      <c r="J119" s="62"/>
+      <c r="K119" s="63"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="58" t="s">
+      <c r="B120" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="55"/>
-      <c r="D120" s="55"/>
-      <c r="E120" s="55"/>
-      <c r="F120" s="55"/>
-      <c r="G120" s="55"/>
-      <c r="H120" s="55"/>
-      <c r="I120" s="55"/>
-      <c r="J120" s="55"/>
-      <c r="K120" s="56"/>
+      <c r="C120" s="62"/>
+      <c r="D120" s="62"/>
+      <c r="E120" s="62"/>
+      <c r="F120" s="62"/>
+      <c r="G120" s="62"/>
+      <c r="H120" s="62"/>
+      <c r="I120" s="62"/>
+      <c r="J120" s="62"/>
+      <c r="K120" s="63"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6556,53 +6592,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="59" t="s">
+      <c r="A151" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="55"/>
-      <c r="C151" s="55"/>
-      <c r="D151" s="55"/>
-      <c r="E151" s="55"/>
-      <c r="F151" s="55"/>
-      <c r="G151" s="55"/>
-      <c r="H151" s="55"/>
-      <c r="I151" s="55"/>
-      <c r="J151" s="55"/>
-      <c r="K151" s="56"/>
+      <c r="B151" s="62"/>
+      <c r="C151" s="62"/>
+      <c r="D151" s="62"/>
+      <c r="E151" s="62"/>
+      <c r="F151" s="62"/>
+      <c r="G151" s="62"/>
+      <c r="H151" s="62"/>
+      <c r="I151" s="62"/>
+      <c r="J151" s="62"/>
+      <c r="K151" s="63"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="60" t="s">
+      <c r="B152" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="55"/>
-      <c r="D152" s="55"/>
-      <c r="E152" s="55"/>
-      <c r="F152" s="55"/>
-      <c r="G152" s="55"/>
-      <c r="H152" s="55"/>
-      <c r="I152" s="55"/>
-      <c r="J152" s="55"/>
-      <c r="K152" s="56"/>
+      <c r="C152" s="62"/>
+      <c r="D152" s="62"/>
+      <c r="E152" s="62"/>
+      <c r="F152" s="62"/>
+      <c r="G152" s="62"/>
+      <c r="H152" s="62"/>
+      <c r="I152" s="62"/>
+      <c r="J152" s="62"/>
+      <c r="K152" s="63"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="60" t="s">
+      <c r="B153" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="55"/>
-      <c r="D153" s="55"/>
-      <c r="E153" s="55"/>
-      <c r="F153" s="55"/>
-      <c r="G153" s="55"/>
-      <c r="H153" s="55"/>
-      <c r="I153" s="55"/>
-      <c r="J153" s="55"/>
-      <c r="K153" s="56"/>
+      <c r="C153" s="62"/>
+      <c r="D153" s="62"/>
+      <c r="E153" s="62"/>
+      <c r="F153" s="62"/>
+      <c r="G153" s="62"/>
+      <c r="H153" s="62"/>
+      <c r="I153" s="62"/>
+      <c r="J153" s="62"/>
+      <c r="K153" s="63"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -6630,7 +6666,7 @@
         <v>0.25</v>
       </c>
       <c r="I154" s="41">
-        <f t="shared" ref="I154:I190" si="6">H154-G154</f>
+        <f t="shared" ref="I154:I193" si="6">H154-G154</f>
         <v>0</v>
       </c>
       <c r="J154" s="45"/>
@@ -7471,9 +7507,11 @@
       <c r="K180" s="43"/>
     </row>
     <row r="181" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A181" s="37"/>
+      <c r="A181" s="37">
+        <v>45645</v>
+      </c>
       <c r="B181" s="38" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="C181" s="39" t="s">
         <v>283</v>
@@ -7496,17 +7534,35 @@
         <v>-1</v>
       </c>
       <c r="J181" s="45"/>
-      <c r="K181" s="43"/>
+      <c r="K181" s="43" t="s">
+        <v>299</v>
+      </c>
     </row>
     <row r="182" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A182" s="37"/>
-      <c r="B182" s="38"/>
-      <c r="C182" s="39"/>
-      <c r="D182" s="38"/>
-      <c r="E182" s="40"/>
-      <c r="F182" s="40"/>
-      <c r="G182" s="41"/>
-      <c r="H182" s="41"/>
+      <c r="A182" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B182" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C182" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D182" s="38" t="s">
+        <v>271</v>
+      </c>
+      <c r="E182" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F182" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G182" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H182" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I182" s="41">
         <f t="shared" si="6"/>
         <v>0</v>
@@ -7515,247 +7571,377 @@
       <c r="K182" s="43"/>
     </row>
     <row r="183" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A183" s="37"/>
-      <c r="B183" s="38"/>
-      <c r="C183" s="39"/>
-      <c r="D183" s="38"/>
-      <c r="E183" s="40"/>
-      <c r="F183" s="40"/>
-      <c r="G183" s="41"/>
+      <c r="A183" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B183" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C183" s="39" t="s">
+        <v>78</v>
+      </c>
+      <c r="D183" s="38" t="s">
+        <v>288</v>
+      </c>
+      <c r="E183" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F183" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="G183" s="41">
+        <v>0.25</v>
+      </c>
       <c r="H183" s="41"/>
       <c r="I183" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-0.25</v>
       </c>
       <c r="J183" s="45"/>
       <c r="K183" s="43"/>
     </row>
     <row r="184" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A184" s="37"/>
-      <c r="B184" s="38"/>
-      <c r="C184" s="39"/>
-      <c r="D184" s="38"/>
-      <c r="E184" s="40"/>
-      <c r="F184" s="40"/>
-      <c r="G184" s="41"/>
+      <c r="A184" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B184" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C184" s="39" t="s">
+        <v>289</v>
+      </c>
+      <c r="D184" s="38" t="s">
+        <v>290</v>
+      </c>
+      <c r="E184" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F184" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="G184" s="41">
+        <v>1</v>
+      </c>
       <c r="H184" s="41"/>
       <c r="I184" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J184" s="45"/>
       <c r="K184" s="43"/>
     </row>
     <row r="185" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A185" s="37"/>
-      <c r="B185" s="38"/>
-      <c r="C185" s="39"/>
-      <c r="D185" s="38"/>
-      <c r="E185" s="40"/>
-      <c r="F185" s="40"/>
-      <c r="G185" s="41"/>
+      <c r="A185" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B185" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C185" s="39" t="s">
+        <v>289</v>
+      </c>
+      <c r="D185" s="38" t="s">
+        <v>298</v>
+      </c>
+      <c r="E185" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F185" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="G185" s="41">
+        <v>1</v>
+      </c>
       <c r="H185" s="41"/>
       <c r="I185" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J185" s="45"/>
       <c r="K185" s="43"/>
     </row>
     <row r="186" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A186" s="37"/>
-      <c r="B186" s="38"/>
-      <c r="C186" s="39"/>
-      <c r="D186" s="38"/>
-      <c r="E186" s="40"/>
-      <c r="F186" s="40"/>
-      <c r="G186" s="41"/>
+      <c r="A186" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B186" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C186" s="39" t="s">
+        <v>262</v>
+      </c>
+      <c r="D186" s="38" t="s">
+        <v>291</v>
+      </c>
+      <c r="E186" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F186" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G186" s="41">
+        <v>1</v>
+      </c>
       <c r="H186" s="41"/>
       <c r="I186" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J186" s="45"/>
       <c r="K186" s="43"/>
     </row>
     <row r="187" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A187" s="37"/>
-      <c r="B187" s="38"/>
-      <c r="C187" s="39"/>
-      <c r="D187" s="38"/>
-      <c r="E187" s="40"/>
-      <c r="F187" s="40"/>
-      <c r="G187" s="41"/>
+      <c r="A187" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B187" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C187" s="39" t="s">
+        <v>262</v>
+      </c>
+      <c r="D187" s="38" t="s">
+        <v>292</v>
+      </c>
+      <c r="E187" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F187" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G187" s="41">
+        <v>1</v>
+      </c>
       <c r="H187" s="41"/>
       <c r="I187" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J187" s="45"/>
       <c r="K187" s="43"/>
     </row>
     <row r="188" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A188" s="37"/>
-      <c r="B188" s="38"/>
-      <c r="C188" s="39"/>
-      <c r="D188" s="38"/>
-      <c r="E188" s="40"/>
-      <c r="F188" s="40"/>
-      <c r="G188" s="41"/>
+      <c r="A188" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B188" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C188" s="39" t="s">
+        <v>262</v>
+      </c>
+      <c r="D188" s="38" t="s">
+        <v>293</v>
+      </c>
+      <c r="E188" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F188" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G188" s="41">
+        <v>1</v>
+      </c>
       <c r="H188" s="41"/>
       <c r="I188" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J188" s="45"/>
       <c r="K188" s="43"/>
     </row>
     <row r="189" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A189" s="37"/>
-      <c r="B189" s="38"/>
+      <c r="A189" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B189" s="38" t="s">
+        <v>43</v>
+      </c>
       <c r="C189" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D189" s="38"/>
-      <c r="E189" s="40"/>
-      <c r="F189" s="40"/>
-      <c r="G189" s="41"/>
+        <v>80</v>
+      </c>
+      <c r="D189" s="38" t="s">
+        <v>294</v>
+      </c>
+      <c r="E189" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F189" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G189" s="41">
+        <v>0.25</v>
+      </c>
       <c r="H189" s="41"/>
       <c r="I189" s="41">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-0.25</v>
       </c>
       <c r="J189" s="45"/>
       <c r="K189" s="43"/>
     </row>
     <row r="190" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A190" s="13"/>
-      <c r="B190" s="15"/>
-      <c r="C190" s="15"/>
-      <c r="D190" s="15"/>
-      <c r="E190" s="15" t="s">
+      <c r="A190" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B190" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C190" s="39" t="s">
+        <v>208</v>
+      </c>
+      <c r="D190" s="38" t="s">
+        <v>295</v>
+      </c>
+      <c r="E190" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F190" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G190" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H190" s="41"/>
+      <c r="I190" s="41">
+        <f t="shared" si="6"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J190" s="45"/>
+      <c r="K190" s="43"/>
+    </row>
+    <row r="191" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A191" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B191" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C191" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D191" s="38" t="s">
+        <v>297</v>
+      </c>
+      <c r="E191" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F191" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G191" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H191" s="41"/>
+      <c r="I191" s="41">
+        <f t="shared" si="6"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J191" s="45"/>
+      <c r="K191" s="43"/>
+    </row>
+    <row r="192" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A192" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B192" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C192" s="39" t="s">
+        <v>208</v>
+      </c>
+      <c r="D192" s="38" t="s">
+        <v>296</v>
+      </c>
+      <c r="E192" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F192" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G192" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H192" s="41"/>
+      <c r="I192" s="41">
+        <f t="shared" si="6"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J192" s="45"/>
+      <c r="K192" s="43"/>
+    </row>
+    <row r="193" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A193" s="13"/>
+      <c r="B193" s="15"/>
+      <c r="C193" s="15"/>
+      <c r="D193" s="15"/>
+      <c r="E193" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F190" s="15"/>
-      <c r="G190" s="18">
-        <f t="shared" ref="G190:H190" si="7">SUM(G154:G189)</f>
-        <v>34.659999999999997</v>
-      </c>
-      <c r="H190" s="18">
-        <f t="shared" si="7"/>
-        <v>21.66</v>
-      </c>
-      <c r="I190" s="18">
+      <c r="F193" s="15"/>
+      <c r="G193" s="18">
+        <f>SUM(G154:G192)</f>
+        <v>41.16</v>
+      </c>
+      <c r="H193" s="18">
+        <f>SUM(H154:H192)</f>
+        <v>21.91</v>
+      </c>
+      <c r="I193" s="18">
         <f t="shared" si="6"/>
-        <v>-12.999999999999996</v>
-      </c>
-      <c r="J190" s="19"/>
-      <c r="K190" s="46"/>
-    </row>
-    <row r="191" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A191" s="61" t="s">
+        <v>-19.249999999999996</v>
+      </c>
+      <c r="J193" s="19"/>
+      <c r="K193" s="46"/>
+    </row>
+    <row r="194" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B191" s="55"/>
-      <c r="C191" s="55"/>
-      <c r="D191" s="55"/>
-      <c r="E191" s="55"/>
-      <c r="F191" s="55"/>
-      <c r="G191" s="55"/>
-      <c r="H191" s="55"/>
-      <c r="I191" s="55"/>
-      <c r="J191" s="55"/>
-      <c r="K191" s="56"/>
-    </row>
-    <row r="192" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A192" s="27" t="s">
+      <c r="B194" s="62"/>
+      <c r="C194" s="62"/>
+      <c r="D194" s="62"/>
+      <c r="E194" s="62"/>
+      <c r="F194" s="62"/>
+      <c r="G194" s="62"/>
+      <c r="H194" s="62"/>
+      <c r="I194" s="62"/>
+      <c r="J194" s="62"/>
+      <c r="K194" s="63"/>
+    </row>
+    <row r="195" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A195" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B192" s="54" t="s">
+      <c r="B195" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C192" s="55"/>
-      <c r="D192" s="55"/>
-      <c r="E192" s="55"/>
-      <c r="F192" s="55"/>
-      <c r="G192" s="55"/>
-      <c r="H192" s="55"/>
-      <c r="I192" s="55"/>
-      <c r="J192" s="55"/>
-      <c r="K192" s="56"/>
-    </row>
-    <row r="193" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A193" s="28" t="s">
+      <c r="C195" s="62"/>
+      <c r="D195" s="62"/>
+      <c r="E195" s="62"/>
+      <c r="F195" s="62"/>
+      <c r="G195" s="62"/>
+      <c r="H195" s="62"/>
+      <c r="I195" s="62"/>
+      <c r="J195" s="62"/>
+      <c r="K195" s="63"/>
+    </row>
+    <row r="196" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B193" s="54" t="s">
+      <c r="B196" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C193" s="55"/>
-      <c r="D193" s="55"/>
-      <c r="E193" s="55"/>
-      <c r="F193" s="55"/>
-      <c r="G193" s="55"/>
-      <c r="H193" s="55"/>
-      <c r="I193" s="55"/>
-      <c r="J193" s="55"/>
-      <c r="K193" s="56"/>
-    </row>
-    <row r="194" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A194" s="37"/>
-      <c r="B194" s="38"/>
-      <c r="C194" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D194" s="38"/>
-      <c r="E194" s="40"/>
-      <c r="F194" s="40"/>
-      <c r="G194" s="41"/>
-      <c r="H194" s="41"/>
-      <c r="I194" s="41">
-        <f t="shared" ref="I194:I204" si="8">H194-G194</f>
-        <v>0</v>
-      </c>
-      <c r="J194" s="45"/>
-      <c r="K194" s="43"/>
-    </row>
-    <row r="195" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A195" s="37"/>
-      <c r="B195" s="38"/>
-      <c r="C195" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D195" s="38"/>
-      <c r="E195" s="40"/>
-      <c r="F195" s="40"/>
-      <c r="G195" s="41"/>
-      <c r="H195" s="41"/>
-      <c r="I195" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J195" s="45"/>
-      <c r="K195" s="43"/>
-    </row>
-    <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A196" s="37"/>
-      <c r="B196" s="38"/>
-      <c r="C196" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D196" s="38"/>
-      <c r="E196" s="40"/>
-      <c r="F196" s="40"/>
-      <c r="G196" s="41"/>
-      <c r="H196" s="41"/>
-      <c r="I196" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J196" s="45"/>
-      <c r="K196" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="C196" s="62"/>
+      <c r="D196" s="62"/>
+      <c r="E196" s="62"/>
+      <c r="F196" s="62"/>
+      <c r="G196" s="62"/>
+      <c r="H196" s="62"/>
+      <c r="I196" s="62"/>
+      <c r="J196" s="62"/>
+      <c r="K196" s="63"/>
     </row>
     <row r="197" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A197" s="37"/>
@@ -7769,7 +7955,7 @@
       <c r="G197" s="41"/>
       <c r="H197" s="41"/>
       <c r="I197" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I197:I207" si="7">H197-G197</f>
         <v>0</v>
       </c>
       <c r="J197" s="45"/>
@@ -7787,7 +7973,7 @@
       <c r="G198" s="41"/>
       <c r="H198" s="41"/>
       <c r="I198" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J198" s="45"/>
@@ -7805,11 +7991,13 @@
       <c r="G199" s="41"/>
       <c r="H199" s="41"/>
       <c r="I199" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J199" s="45"/>
-      <c r="K199" s="43"/>
+      <c r="K199" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="200" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A200" s="37"/>
@@ -7823,7 +8011,7 @@
       <c r="G200" s="41"/>
       <c r="H200" s="41"/>
       <c r="I200" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J200" s="45"/>
@@ -7841,7 +8029,7 @@
       <c r="G201" s="41"/>
       <c r="H201" s="41"/>
       <c r="I201" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J201" s="45"/>
@@ -7859,7 +8047,7 @@
       <c r="G202" s="41"/>
       <c r="H202" s="41"/>
       <c r="I202" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J202" s="45"/>
@@ -7877,138 +8065,138 @@
       <c r="G203" s="41"/>
       <c r="H203" s="41"/>
       <c r="I203" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J203" s="45"/>
       <c r="K203" s="43"/>
     </row>
     <row r="204" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A204" s="13"/>
-      <c r="B204" s="15"/>
-      <c r="C204" s="15"/>
-      <c r="D204" s="15"/>
-      <c r="E204" s="15" t="s">
+      <c r="A204" s="37"/>
+      <c r="B204" s="38"/>
+      <c r="C204" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D204" s="38"/>
+      <c r="E204" s="40"/>
+      <c r="F204" s="40"/>
+      <c r="G204" s="41"/>
+      <c r="H204" s="41"/>
+      <c r="I204" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J204" s="45"/>
+      <c r="K204" s="43"/>
+    </row>
+    <row r="205" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A205" s="37"/>
+      <c r="B205" s="38"/>
+      <c r="C205" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D205" s="38"/>
+      <c r="E205" s="40"/>
+      <c r="F205" s="40"/>
+      <c r="G205" s="41"/>
+      <c r="H205" s="41"/>
+      <c r="I205" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J205" s="45"/>
+      <c r="K205" s="43"/>
+    </row>
+    <row r="206" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A206" s="37"/>
+      <c r="B206" s="38"/>
+      <c r="C206" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D206" s="38"/>
+      <c r="E206" s="40"/>
+      <c r="F206" s="40"/>
+      <c r="G206" s="41"/>
+      <c r="H206" s="41"/>
+      <c r="I206" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J206" s="45"/>
+      <c r="K206" s="43"/>
+    </row>
+    <row r="207" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A207" s="13"/>
+      <c r="B207" s="15"/>
+      <c r="C207" s="15"/>
+      <c r="D207" s="15"/>
+      <c r="E207" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F204" s="15"/>
-      <c r="G204" s="18">
-        <f t="shared" ref="G204:H204" si="9">SUM(G194:G203)</f>
-        <v>0</v>
-      </c>
-      <c r="H204" s="18">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="I204" s="18">
+      <c r="F207" s="15"/>
+      <c r="G207" s="18">
+        <f t="shared" ref="G207:H207" si="8">SUM(G197:G206)</f>
+        <v>0</v>
+      </c>
+      <c r="H207" s="18">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J204" s="19"/>
-      <c r="K204" s="46"/>
-    </row>
-    <row r="205" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A205" s="57" t="s">
+      <c r="I207" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J207" s="19"/>
+      <c r="K207" s="46"/>
+    </row>
+    <row r="208" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A208" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="B205" s="55"/>
-      <c r="C205" s="55"/>
-      <c r="D205" s="55"/>
-      <c r="E205" s="55"/>
-      <c r="F205" s="55"/>
-      <c r="G205" s="55"/>
-      <c r="H205" s="55"/>
-      <c r="I205" s="55"/>
-      <c r="J205" s="55"/>
-      <c r="K205" s="56"/>
-    </row>
-    <row r="206" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A206" s="29" t="s">
+      <c r="B208" s="62"/>
+      <c r="C208" s="62"/>
+      <c r="D208" s="62"/>
+      <c r="E208" s="62"/>
+      <c r="F208" s="62"/>
+      <c r="G208" s="62"/>
+      <c r="H208" s="62"/>
+      <c r="I208" s="62"/>
+      <c r="J208" s="62"/>
+      <c r="K208" s="63"/>
+    </row>
+    <row r="209" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A209" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B206" s="75" t="s">
+      <c r="B209" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C206" s="55"/>
-      <c r="D206" s="55"/>
-      <c r="E206" s="55"/>
-      <c r="F206" s="55"/>
-      <c r="G206" s="55"/>
-      <c r="H206" s="55"/>
-      <c r="I206" s="55"/>
-      <c r="J206" s="55"/>
-      <c r="K206" s="56"/>
-    </row>
-    <row r="207" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A207" s="30" t="s">
+      <c r="C209" s="62"/>
+      <c r="D209" s="62"/>
+      <c r="E209" s="62"/>
+      <c r="F209" s="62"/>
+      <c r="G209" s="62"/>
+      <c r="H209" s="62"/>
+      <c r="I209" s="62"/>
+      <c r="J209" s="62"/>
+      <c r="K209" s="63"/>
+    </row>
+    <row r="210" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A210" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B207" s="75" t="s">
+      <c r="B210" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C207" s="55"/>
-      <c r="D207" s="55"/>
-      <c r="E207" s="55"/>
-      <c r="F207" s="55"/>
-      <c r="G207" s="55"/>
-      <c r="H207" s="55"/>
-      <c r="I207" s="55"/>
-      <c r="J207" s="55"/>
-      <c r="K207" s="56"/>
-    </row>
-    <row r="208" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A208" s="37"/>
-      <c r="B208" s="38"/>
-      <c r="C208" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D208" s="38"/>
-      <c r="E208" s="40"/>
-      <c r="F208" s="40"/>
-      <c r="G208" s="41"/>
-      <c r="H208" s="41"/>
-      <c r="I208" s="41">
-        <f t="shared" ref="I208:I218" si="10">H208-G208</f>
-        <v>0</v>
-      </c>
-      <c r="J208" s="45"/>
-      <c r="K208" s="43"/>
-    </row>
-    <row r="209" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A209" s="37"/>
-      <c r="B209" s="38"/>
-      <c r="C209" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D209" s="38"/>
-      <c r="E209" s="40"/>
-      <c r="F209" s="40"/>
-      <c r="G209" s="41"/>
-      <c r="H209" s="41"/>
-      <c r="I209" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J209" s="45"/>
-      <c r="K209" s="43"/>
-    </row>
-    <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A210" s="37"/>
-      <c r="B210" s="38"/>
-      <c r="C210" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D210" s="38"/>
-      <c r="E210" s="40"/>
-      <c r="F210" s="40"/>
-      <c r="G210" s="41"/>
-      <c r="H210" s="41"/>
-      <c r="I210" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J210" s="45"/>
-      <c r="K210" s="43"/>
+      <c r="C210" s="62"/>
+      <c r="D210" s="62"/>
+      <c r="E210" s="62"/>
+      <c r="F210" s="62"/>
+      <c r="G210" s="62"/>
+      <c r="H210" s="62"/>
+      <c r="I210" s="62"/>
+      <c r="J210" s="62"/>
+      <c r="K210" s="63"/>
     </row>
     <row r="211" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A211" s="37"/>
@@ -8022,7 +8210,7 @@
       <c r="G211" s="41"/>
       <c r="H211" s="41"/>
       <c r="I211" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I211:I221" si="9">H211-G211</f>
         <v>0</v>
       </c>
       <c r="J211" s="45"/>
@@ -8040,7 +8228,7 @@
       <c r="G212" s="41"/>
       <c r="H212" s="41"/>
       <c r="I212" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J212" s="45"/>
@@ -8058,7 +8246,7 @@
       <c r="G213" s="41"/>
       <c r="H213" s="41"/>
       <c r="I213" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J213" s="45"/>
@@ -8076,7 +8264,7 @@
       <c r="G214" s="41"/>
       <c r="H214" s="41"/>
       <c r="I214" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J214" s="45"/>
@@ -8094,7 +8282,7 @@
       <c r="G215" s="41"/>
       <c r="H215" s="41"/>
       <c r="I215" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J215" s="45"/>
@@ -8112,7 +8300,7 @@
       <c r="G216" s="41"/>
       <c r="H216" s="41"/>
       <c r="I216" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J216" s="45"/>
@@ -8130,138 +8318,138 @@
       <c r="G217" s="41"/>
       <c r="H217" s="41"/>
       <c r="I217" s="41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J217" s="45"/>
       <c r="K217" s="43"/>
     </row>
     <row r="218" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A218" s="13"/>
-      <c r="B218" s="15"/>
-      <c r="C218" s="15"/>
-      <c r="D218" s="15"/>
-      <c r="E218" s="15" t="s">
+      <c r="A218" s="37"/>
+      <c r="B218" s="38"/>
+      <c r="C218" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D218" s="38"/>
+      <c r="E218" s="40"/>
+      <c r="F218" s="40"/>
+      <c r="G218" s="41"/>
+      <c r="H218" s="41"/>
+      <c r="I218" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J218" s="45"/>
+      <c r="K218" s="43"/>
+    </row>
+    <row r="219" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A219" s="37"/>
+      <c r="B219" s="38"/>
+      <c r="C219" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D219" s="38"/>
+      <c r="E219" s="40"/>
+      <c r="F219" s="40"/>
+      <c r="G219" s="41"/>
+      <c r="H219" s="41"/>
+      <c r="I219" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J219" s="45"/>
+      <c r="K219" s="43"/>
+    </row>
+    <row r="220" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A220" s="37"/>
+      <c r="B220" s="38"/>
+      <c r="C220" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D220" s="38"/>
+      <c r="E220" s="40"/>
+      <c r="F220" s="40"/>
+      <c r="G220" s="41"/>
+      <c r="H220" s="41"/>
+      <c r="I220" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J220" s="45"/>
+      <c r="K220" s="43"/>
+    </row>
+    <row r="221" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A221" s="13"/>
+      <c r="B221" s="15"/>
+      <c r="C221" s="15"/>
+      <c r="D221" s="15"/>
+      <c r="E221" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F218" s="15"/>
-      <c r="G218" s="18">
-        <f t="shared" ref="G218:H218" si="11">SUM(G208:G217)</f>
-        <v>0</v>
-      </c>
-      <c r="H218" s="18">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I218" s="18">
+      <c r="F221" s="15"/>
+      <c r="G221" s="18">
+        <f t="shared" ref="G221:H221" si="10">SUM(G211:G220)</f>
+        <v>0</v>
+      </c>
+      <c r="H221" s="18">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J218" s="19"/>
-      <c r="K218" s="46"/>
-    </row>
-    <row r="219" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="62" t="s">
+      <c r="I221" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J221" s="19"/>
+      <c r="K221" s="46"/>
+    </row>
+    <row r="222" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B219" s="63"/>
-      <c r="C219" s="63"/>
-      <c r="D219" s="63"/>
-      <c r="E219" s="63"/>
-      <c r="F219" s="63"/>
-      <c r="G219" s="63"/>
-      <c r="H219" s="63"/>
-      <c r="I219" s="63"/>
-      <c r="J219" s="63"/>
-      <c r="K219" s="64"/>
-    </row>
-    <row r="220" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A220" s="32" t="s">
+      <c r="B222" s="55"/>
+      <c r="C222" s="55"/>
+      <c r="D222" s="55"/>
+      <c r="E222" s="55"/>
+      <c r="F222" s="55"/>
+      <c r="G222" s="55"/>
+      <c r="H222" s="55"/>
+      <c r="I222" s="55"/>
+      <c r="J222" s="55"/>
+      <c r="K222" s="56"/>
+    </row>
+    <row r="223" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A223" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B220" s="65" t="s">
+      <c r="B223" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C220" s="63"/>
-      <c r="D220" s="63"/>
-      <c r="E220" s="63"/>
-      <c r="F220" s="63"/>
-      <c r="G220" s="63"/>
-      <c r="H220" s="63"/>
-      <c r="I220" s="63"/>
-      <c r="J220" s="63"/>
-      <c r="K220" s="64"/>
-    </row>
-    <row r="221" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A221" s="33" t="s">
+      <c r="C223" s="55"/>
+      <c r="D223" s="55"/>
+      <c r="E223" s="55"/>
+      <c r="F223" s="55"/>
+      <c r="G223" s="55"/>
+      <c r="H223" s="55"/>
+      <c r="I223" s="55"/>
+      <c r="J223" s="55"/>
+      <c r="K223" s="56"/>
+    </row>
+    <row r="224" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A224" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B221" s="65" t="s">
+      <c r="B224" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C221" s="63"/>
-      <c r="D221" s="63"/>
-      <c r="E221" s="63"/>
-      <c r="F221" s="63"/>
-      <c r="G221" s="63"/>
-      <c r="H221" s="63"/>
-      <c r="I221" s="63"/>
-      <c r="J221" s="63"/>
-      <c r="K221" s="64"/>
-    </row>
-    <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A222" s="37"/>
-      <c r="B222" s="38"/>
-      <c r="C222" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D222" s="38"/>
-      <c r="E222" s="40"/>
-      <c r="F222" s="40"/>
-      <c r="G222" s="41"/>
-      <c r="H222" s="41"/>
-      <c r="I222" s="41">
-        <f t="shared" ref="I222:I232" si="12">H222-G222</f>
-        <v>0</v>
-      </c>
-      <c r="J222" s="45"/>
-      <c r="K222" s="43"/>
-    </row>
-    <row r="223" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A223" s="37"/>
-      <c r="B223" s="38"/>
-      <c r="C223" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D223" s="38"/>
-      <c r="E223" s="40"/>
-      <c r="F223" s="40"/>
-      <c r="G223" s="41"/>
-      <c r="H223" s="41"/>
-      <c r="I223" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J223" s="45"/>
-      <c r="K223" s="43"/>
-    </row>
-    <row r="224" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A224" s="37"/>
-      <c r="B224" s="38"/>
-      <c r="C224" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D224" s="38"/>
-      <c r="E224" s="40"/>
-      <c r="F224" s="40"/>
-      <c r="G224" s="41"/>
-      <c r="H224" s="41"/>
-      <c r="I224" s="41">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="J224" s="45"/>
-      <c r="K224" s="43"/>
+      <c r="C224" s="55"/>
+      <c r="D224" s="55"/>
+      <c r="E224" s="55"/>
+      <c r="F224" s="55"/>
+      <c r="G224" s="55"/>
+      <c r="H224" s="55"/>
+      <c r="I224" s="55"/>
+      <c r="J224" s="55"/>
+      <c r="K224" s="56"/>
     </row>
     <row r="225" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A225" s="37"/>
@@ -8275,7 +8463,7 @@
       <c r="G225" s="41"/>
       <c r="H225" s="41"/>
       <c r="I225" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="I225:I235" si="11">H225-G225</f>
         <v>0</v>
       </c>
       <c r="J225" s="45"/>
@@ -8293,7 +8481,7 @@
       <c r="G226" s="41"/>
       <c r="H226" s="41"/>
       <c r="I226" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J226" s="45"/>
@@ -8311,7 +8499,7 @@
       <c r="G227" s="41"/>
       <c r="H227" s="41"/>
       <c r="I227" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J227" s="45"/>
@@ -8329,7 +8517,7 @@
       <c r="G228" s="41"/>
       <c r="H228" s="41"/>
       <c r="I228" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J228" s="45"/>
@@ -8347,7 +8535,7 @@
       <c r="G229" s="41"/>
       <c r="H229" s="41"/>
       <c r="I229" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J229" s="45"/>
@@ -8365,7 +8553,7 @@
       <c r="G230" s="41"/>
       <c r="H230" s="41"/>
       <c r="I230" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J230" s="45"/>
@@ -8383,42 +8571,96 @@
       <c r="G231" s="41"/>
       <c r="H231" s="41"/>
       <c r="I231" s="41">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J231" s="45"/>
       <c r="K231" s="43"/>
     </row>
     <row r="232" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A232" s="48"/>
-      <c r="B232" s="49"/>
-      <c r="C232" s="49"/>
-      <c r="D232" s="49"/>
-      <c r="E232" s="49" t="s">
+      <c r="A232" s="37"/>
+      <c r="B232" s="38"/>
+      <c r="C232" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D232" s="38"/>
+      <c r="E232" s="40"/>
+      <c r="F232" s="40"/>
+      <c r="G232" s="41"/>
+      <c r="H232" s="41"/>
+      <c r="I232" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J232" s="45"/>
+      <c r="K232" s="43"/>
+    </row>
+    <row r="233" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A233" s="37"/>
+      <c r="B233" s="38"/>
+      <c r="C233" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D233" s="38"/>
+      <c r="E233" s="40"/>
+      <c r="F233" s="40"/>
+      <c r="G233" s="41"/>
+      <c r="H233" s="41"/>
+      <c r="I233" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J233" s="45"/>
+      <c r="K233" s="43"/>
+    </row>
+    <row r="234" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A234" s="37"/>
+      <c r="B234" s="38"/>
+      <c r="C234" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D234" s="38"/>
+      <c r="E234" s="40"/>
+      <c r="F234" s="40"/>
+      <c r="G234" s="41"/>
+      <c r="H234" s="41"/>
+      <c r="I234" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J234" s="45"/>
+      <c r="K234" s="43"/>
+    </row>
+    <row r="235" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A235" s="48"/>
+      <c r="B235" s="49"/>
+      <c r="C235" s="49"/>
+      <c r="D235" s="49"/>
+      <c r="E235" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F232" s="49"/>
-      <c r="G232" s="50">
-        <f t="shared" ref="G232:H232" si="13">SUM(G222:G231)</f>
-        <v>0</v>
-      </c>
-      <c r="H232" s="50">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="I232" s="50">
+      <c r="F235" s="49"/>
+      <c r="G235" s="50">
+        <f t="shared" ref="G235:H235" si="12">SUM(G225:G234)</f>
+        <v>0</v>
+      </c>
+      <c r="H235" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J232" s="51"/>
-      <c r="K232" s="52"/>
+      <c r="I235" s="50">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J235" s="51"/>
+      <c r="K235" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{C341563A-5BC5-4F1E-BC72-B4C1ADE699F2}">
+      <autoFilter ref="A1:K15" xr:uid="{B1F15A25-4CDC-43AE-BA01-97157FD3ABCF}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -8429,9 +8671,17 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A219:K219"/>
-    <mergeCell ref="B220:K220"/>
-    <mergeCell ref="B221:K221"/>
+    <mergeCell ref="B195:K195"/>
+    <mergeCell ref="B196:K196"/>
+    <mergeCell ref="A208:K208"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A194:K194"/>
+    <mergeCell ref="A222:K222"/>
+    <mergeCell ref="B223:K223"/>
+    <mergeCell ref="B224:K224"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -8442,19 +8692,11 @@
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
     <mergeCell ref="A118:K118"/>
-    <mergeCell ref="B206:K206"/>
-    <mergeCell ref="B207:K207"/>
+    <mergeCell ref="B209:K209"/>
+    <mergeCell ref="B210:K210"/>
     <mergeCell ref="B119:K119"/>
-    <mergeCell ref="B192:K192"/>
-    <mergeCell ref="B193:K193"/>
-    <mergeCell ref="A205:K205"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A191:K191"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B189 B194:B203 B208:B217">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B197:B206 B211:B220 B154:B192">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -8471,7 +8713,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B152:B190 B192:B204 B206:B218 B220:B232">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B195:B207 B209:B221 B223:B235 B152:B193">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -8479,34 +8721,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B222:B231">
+  <conditionalFormatting sqref="B225:B234">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B222))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B225))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B222))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B225))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B222))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B225))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B222))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B225))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B222))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B225))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G154:G190 G194:G204 G208:G218 G222:G232">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G197:G207 G211:G221 G225:G235 G154:G193">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H232">
+  <conditionalFormatting sqref="H1:H235">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I154:I190 I194:I204 I208:I218 I222:I232">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I197:I207 I211:I221 I225:I235 I154:I193">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -8515,7 +8757,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F222:F231 F208:F217 F86:F116 F154:F189 F194:F203 F5:F45 F50:F81 F121:F149" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F225:F234 F211:F220 F86:F116 F197:F206 F5:F45 F50:F81 F121:F149 F154:F192" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8531,13 +8773,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E116 E154:E189 E194:E203 E208:E217 E222:E231 E50:E81 E121:E149</xm:sqref>
+          <xm:sqref>E5:E45 E86:E116 E197:E206 E211:E220 E225:E234 E50:E81 E121:E149 E154:E192</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B116 B154:B189 B194:B203 B208:B217 B222:B231 B50:B81 B121:B149</xm:sqref>
+          <xm:sqref>B5:B45 B86:B116 B197:B206 B211:B220 B225:B234 B50:B81 B121:B149 B154:B192</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -10178,26 +10420,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -10432,10 +10654,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10452,20 +10705,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W5 DataLab 2 Work III
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24790124-BCC0-4623-BC8B-2D7D393573E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DFB966D-60F6-4EBD-9B3F-8BAF2DACF9B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$220</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$221</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="303">
   <si>
     <t>Date</t>
   </si>
@@ -1002,6 +1002,15 @@
   </si>
   <si>
     <t>0,1 so far</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Informal DBSCAN Lecture</t>
+  </si>
+  <si>
+    <t>Had torubles with dependencies % packages</t>
   </si>
 </sst>
 </file>
@@ -1487,6 +1496,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1503,8 +1532,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1522,24 +1549,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2012,7 +2021,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K235"/>
+  <dimension ref="A1:K236"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -2064,53 +2073,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3449,53 +3458,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4548,53 +4557,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5609,53 +5618,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="68" t="s">
+      <c r="A118" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="62"/>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
+      <c r="B118" s="55"/>
+      <c r="C118" s="55"/>
+      <c r="D118" s="55"/>
+      <c r="E118" s="55"/>
+      <c r="F118" s="55"/>
+      <c r="G118" s="55"/>
+      <c r="H118" s="55"/>
+      <c r="I118" s="55"/>
+      <c r="J118" s="55"/>
+      <c r="K118" s="56"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="70" t="s">
+      <c r="B119" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="62"/>
-      <c r="D119" s="62"/>
-      <c r="E119" s="62"/>
-      <c r="F119" s="62"/>
-      <c r="G119" s="62"/>
-      <c r="H119" s="62"/>
-      <c r="I119" s="62"/>
-      <c r="J119" s="62"/>
-      <c r="K119" s="63"/>
+      <c r="C119" s="55"/>
+      <c r="D119" s="55"/>
+      <c r="E119" s="55"/>
+      <c r="F119" s="55"/>
+      <c r="G119" s="55"/>
+      <c r="H119" s="55"/>
+      <c r="I119" s="55"/>
+      <c r="J119" s="55"/>
+      <c r="K119" s="56"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="70" t="s">
+      <c r="B120" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="62"/>
-      <c r="D120" s="62"/>
-      <c r="E120" s="62"/>
-      <c r="F120" s="62"/>
-      <c r="G120" s="62"/>
-      <c r="H120" s="62"/>
-      <c r="I120" s="62"/>
-      <c r="J120" s="62"/>
-      <c r="K120" s="63"/>
+      <c r="C120" s="55"/>
+      <c r="D120" s="55"/>
+      <c r="E120" s="55"/>
+      <c r="F120" s="55"/>
+      <c r="G120" s="55"/>
+      <c r="H120" s="55"/>
+      <c r="I120" s="55"/>
+      <c r="J120" s="55"/>
+      <c r="K120" s="56"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6592,53 +6601,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="73" t="s">
+      <c r="A151" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="62"/>
-      <c r="C151" s="62"/>
-      <c r="D151" s="62"/>
-      <c r="E151" s="62"/>
-      <c r="F151" s="62"/>
-      <c r="G151" s="62"/>
-      <c r="H151" s="62"/>
-      <c r="I151" s="62"/>
-      <c r="J151" s="62"/>
-      <c r="K151" s="63"/>
+      <c r="B151" s="55"/>
+      <c r="C151" s="55"/>
+      <c r="D151" s="55"/>
+      <c r="E151" s="55"/>
+      <c r="F151" s="55"/>
+      <c r="G151" s="55"/>
+      <c r="H151" s="55"/>
+      <c r="I151" s="55"/>
+      <c r="J151" s="55"/>
+      <c r="K151" s="56"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="74" t="s">
+      <c r="B152" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="62"/>
-      <c r="D152" s="62"/>
-      <c r="E152" s="62"/>
-      <c r="F152" s="62"/>
-      <c r="G152" s="62"/>
-      <c r="H152" s="62"/>
-      <c r="I152" s="62"/>
-      <c r="J152" s="62"/>
-      <c r="K152" s="63"/>
+      <c r="C152" s="55"/>
+      <c r="D152" s="55"/>
+      <c r="E152" s="55"/>
+      <c r="F152" s="55"/>
+      <c r="G152" s="55"/>
+      <c r="H152" s="55"/>
+      <c r="I152" s="55"/>
+      <c r="J152" s="55"/>
+      <c r="K152" s="56"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="74" t="s">
+      <c r="B153" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="62"/>
-      <c r="D153" s="62"/>
-      <c r="E153" s="62"/>
-      <c r="F153" s="62"/>
-      <c r="G153" s="62"/>
-      <c r="H153" s="62"/>
-      <c r="I153" s="62"/>
-      <c r="J153" s="62"/>
-      <c r="K153" s="63"/>
+      <c r="C153" s="55"/>
+      <c r="D153" s="55"/>
+      <c r="E153" s="55"/>
+      <c r="F153" s="55"/>
+      <c r="G153" s="55"/>
+      <c r="H153" s="55"/>
+      <c r="I153" s="55"/>
+      <c r="J153" s="55"/>
+      <c r="K153" s="56"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -6666,7 +6675,7 @@
         <v>0.25</v>
       </c>
       <c r="I154" s="41">
-        <f t="shared" ref="I154:I193" si="6">H154-G154</f>
+        <f t="shared" ref="I154:I194" si="6">H154-G154</f>
         <v>0</v>
       </c>
       <c r="J154" s="45"/>
@@ -7575,7 +7584,7 @@
         <v>45646</v>
       </c>
       <c r="B183" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C183" s="39" t="s">
         <v>78</v>
@@ -7592,10 +7601,12 @@
       <c r="G183" s="41">
         <v>0.25</v>
       </c>
-      <c r="H183" s="41"/>
+      <c r="H183" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I183" s="41">
         <f t="shared" si="6"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J183" s="45"/>
       <c r="K183" s="43"/>
@@ -7605,7 +7616,7 @@
         <v>45646</v>
       </c>
       <c r="B184" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C184" s="39" t="s">
         <v>289</v>
@@ -7622,40 +7633,46 @@
       <c r="G184" s="41">
         <v>1</v>
       </c>
-      <c r="H184" s="41"/>
+      <c r="H184" s="41">
+        <v>3.25</v>
+      </c>
       <c r="I184" s="41">
         <f t="shared" si="6"/>
-        <v>-1</v>
+        <v>2.25</v>
       </c>
       <c r="J184" s="45"/>
-      <c r="K184" s="43"/>
+      <c r="K184" s="43" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="185" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A185" s="37">
         <v>45646</v>
       </c>
       <c r="B185" s="38" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C185" s="39" t="s">
-        <v>289</v>
+        <v>66</v>
       </c>
       <c r="D185" s="38" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E185" s="40" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="F185" s="40" t="s">
         <v>105</v>
       </c>
       <c r="G185" s="41">
-        <v>1</v>
-      </c>
-      <c r="H185" s="41"/>
+        <v>0.25</v>
+      </c>
+      <c r="H185" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I185" s="41">
         <f t="shared" si="6"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J185" s="45"/>
       <c r="K185" s="43"/>
@@ -7665,19 +7682,19 @@
         <v>45646</v>
       </c>
       <c r="B186" s="38" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="C186" s="39" t="s">
-        <v>262</v>
+        <v>289</v>
       </c>
       <c r="D186" s="38" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="E186" s="40" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F186" s="40" t="s">
-        <v>185</v>
+        <v>105</v>
       </c>
       <c r="G186" s="41">
         <v>1</v>
@@ -7701,7 +7718,7 @@
         <v>262</v>
       </c>
       <c r="D187" s="38" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E187" s="40" t="s">
         <v>50</v>
@@ -7731,7 +7748,7 @@
         <v>262</v>
       </c>
       <c r="D188" s="38" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E188" s="40" t="s">
         <v>50</v>
@@ -7758,24 +7775,24 @@
         <v>43</v>
       </c>
       <c r="C189" s="39" t="s">
-        <v>80</v>
+        <v>262</v>
       </c>
       <c r="D189" s="38" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E189" s="40" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="F189" s="40" t="s">
-        <v>87</v>
+        <v>185</v>
       </c>
       <c r="G189" s="41">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="H189" s="41"/>
       <c r="I189" s="41">
         <f t="shared" si="6"/>
-        <v>-0.25</v>
+        <v>-1</v>
       </c>
       <c r="J189" s="45"/>
       <c r="K189" s="43"/>
@@ -7788,16 +7805,16 @@
         <v>43</v>
       </c>
       <c r="C190" s="39" t="s">
-        <v>208</v>
+        <v>80</v>
       </c>
       <c r="D190" s="38" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E190" s="40" t="s">
         <v>64</v>
       </c>
       <c r="F190" s="40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G190" s="41">
         <v>0.25</v>
@@ -7818,16 +7835,16 @@
         <v>43</v>
       </c>
       <c r="C191" s="39" t="s">
-        <v>80</v>
+        <v>208</v>
       </c>
       <c r="D191" s="38" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E191" s="40" t="s">
         <v>64</v>
       </c>
       <c r="F191" s="40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G191" s="41">
         <v>0.25</v>
@@ -7838,7 +7855,9 @@
         <v>-0.25</v>
       </c>
       <c r="J191" s="45"/>
-      <c r="K191" s="43"/>
+      <c r="K191" s="43" t="s">
+        <v>300</v>
+      </c>
     </row>
     <row r="192" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A192" s="37">
@@ -7848,16 +7867,16 @@
         <v>43</v>
       </c>
       <c r="C192" s="39" t="s">
-        <v>208</v>
+        <v>80</v>
       </c>
       <c r="D192" s="38" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E192" s="40" t="s">
         <v>64</v>
       </c>
       <c r="F192" s="40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G192" s="41">
         <v>0.25</v>
@@ -7871,95 +7890,107 @@
       <c r="K192" s="43"/>
     </row>
     <row r="193" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A193" s="13"/>
-      <c r="B193" s="15"/>
-      <c r="C193" s="15"/>
-      <c r="D193" s="15"/>
-      <c r="E193" s="15" t="s">
+      <c r="A193" s="37">
+        <v>45646</v>
+      </c>
+      <c r="B193" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C193" s="39" t="s">
+        <v>208</v>
+      </c>
+      <c r="D193" s="38" t="s">
+        <v>296</v>
+      </c>
+      <c r="E193" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F193" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G193" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H193" s="41"/>
+      <c r="I193" s="41">
+        <f t="shared" si="6"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J193" s="45"/>
+      <c r="K193" s="43"/>
+    </row>
+    <row r="194" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A194" s="13"/>
+      <c r="B194" s="15"/>
+      <c r="C194" s="15"/>
+      <c r="D194" s="15"/>
+      <c r="E194" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F193" s="15"/>
-      <c r="G193" s="18">
-        <f>SUM(G154:G192)</f>
-        <v>41.16</v>
-      </c>
-      <c r="H193" s="18">
-        <f>SUM(H154:H192)</f>
-        <v>21.91</v>
-      </c>
-      <c r="I193" s="18">
+      <c r="F194" s="15"/>
+      <c r="G194" s="18">
+        <f>SUM(G154:G193)</f>
+        <v>41.41</v>
+      </c>
+      <c r="H194" s="18">
+        <f>SUM(H154:H193)</f>
+        <v>25.66</v>
+      </c>
+      <c r="I194" s="18">
         <f t="shared" si="6"/>
-        <v>-19.249999999999996</v>
-      </c>
-      <c r="J193" s="19"/>
-      <c r="K193" s="46"/>
-    </row>
-    <row r="194" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A194" s="75" t="s">
+        <v>-15.749999999999996</v>
+      </c>
+      <c r="J194" s="19"/>
+      <c r="K194" s="46"/>
+    </row>
+    <row r="195" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B194" s="62"/>
-      <c r="C194" s="62"/>
-      <c r="D194" s="62"/>
-      <c r="E194" s="62"/>
-      <c r="F194" s="62"/>
-      <c r="G194" s="62"/>
-      <c r="H194" s="62"/>
-      <c r="I194" s="62"/>
-      <c r="J194" s="62"/>
-      <c r="K194" s="63"/>
-    </row>
-    <row r="195" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A195" s="27" t="s">
+      <c r="B195" s="55"/>
+      <c r="C195" s="55"/>
+      <c r="D195" s="55"/>
+      <c r="E195" s="55"/>
+      <c r="F195" s="55"/>
+      <c r="G195" s="55"/>
+      <c r="H195" s="55"/>
+      <c r="I195" s="55"/>
+      <c r="J195" s="55"/>
+      <c r="K195" s="56"/>
+    </row>
+    <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A196" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B195" s="71" t="s">
+      <c r="B196" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C195" s="62"/>
-      <c r="D195" s="62"/>
-      <c r="E195" s="62"/>
-      <c r="F195" s="62"/>
-      <c r="G195" s="62"/>
-      <c r="H195" s="62"/>
-      <c r="I195" s="62"/>
-      <c r="J195" s="62"/>
-      <c r="K195" s="63"/>
-    </row>
-    <row r="196" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A196" s="28" t="s">
+      <c r="C196" s="55"/>
+      <c r="D196" s="55"/>
+      <c r="E196" s="55"/>
+      <c r="F196" s="55"/>
+      <c r="G196" s="55"/>
+      <c r="H196" s="55"/>
+      <c r="I196" s="55"/>
+      <c r="J196" s="55"/>
+      <c r="K196" s="56"/>
+    </row>
+    <row r="197" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B196" s="71" t="s">
+      <c r="B197" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C196" s="62"/>
-      <c r="D196" s="62"/>
-      <c r="E196" s="62"/>
-      <c r="F196" s="62"/>
-      <c r="G196" s="62"/>
-      <c r="H196" s="62"/>
-      <c r="I196" s="62"/>
-      <c r="J196" s="62"/>
-      <c r="K196" s="63"/>
-    </row>
-    <row r="197" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A197" s="37"/>
-      <c r="B197" s="38"/>
-      <c r="C197" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D197" s="38"/>
-      <c r="E197" s="40"/>
-      <c r="F197" s="40"/>
-      <c r="G197" s="41"/>
-      <c r="H197" s="41"/>
-      <c r="I197" s="41">
-        <f t="shared" ref="I197:I207" si="7">H197-G197</f>
-        <v>0</v>
-      </c>
-      <c r="J197" s="45"/>
-      <c r="K197" s="43"/>
+      <c r="C197" s="55"/>
+      <c r="D197" s="55"/>
+      <c r="E197" s="55"/>
+      <c r="F197" s="55"/>
+      <c r="G197" s="55"/>
+      <c r="H197" s="55"/>
+      <c r="I197" s="55"/>
+      <c r="J197" s="55"/>
+      <c r="K197" s="56"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="37"/>
@@ -7973,7 +8004,7 @@
       <c r="G198" s="41"/>
       <c r="H198" s="41"/>
       <c r="I198" s="41">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="I198:I208" si="7">H198-G198</f>
         <v>0</v>
       </c>
       <c r="J198" s="45"/>
@@ -7995,9 +8026,7 @@
         <v>0</v>
       </c>
       <c r="J199" s="45"/>
-      <c r="K199" s="43" t="s">
-        <v>25</v>
-      </c>
+      <c r="K199" s="43"/>
     </row>
     <row r="200" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A200" s="37"/>
@@ -8015,7 +8044,9 @@
         <v>0</v>
       </c>
       <c r="J200" s="45"/>
-      <c r="K200" s="43"/>
+      <c r="K200" s="43" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="201" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A201" s="37"/>
@@ -8126,95 +8157,95 @@
       <c r="K206" s="43"/>
     </row>
     <row r="207" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A207" s="13"/>
-      <c r="B207" s="15"/>
-      <c r="C207" s="15"/>
-      <c r="D207" s="15"/>
-      <c r="E207" s="15" t="s">
+      <c r="A207" s="37"/>
+      <c r="B207" s="38"/>
+      <c r="C207" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D207" s="38"/>
+      <c r="E207" s="40"/>
+      <c r="F207" s="40"/>
+      <c r="G207" s="41"/>
+      <c r="H207" s="41"/>
+      <c r="I207" s="41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="J207" s="45"/>
+      <c r="K207" s="43"/>
+    </row>
+    <row r="208" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A208" s="13"/>
+      <c r="B208" s="15"/>
+      <c r="C208" s="15"/>
+      <c r="D208" s="15"/>
+      <c r="E208" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F207" s="15"/>
-      <c r="G207" s="18">
-        <f t="shared" ref="G207:H207" si="8">SUM(G197:G206)</f>
-        <v>0</v>
-      </c>
-      <c r="H207" s="18">
+      <c r="F208" s="15"/>
+      <c r="G208" s="18">
+        <f t="shared" ref="G208:H208" si="8">SUM(G198:G207)</f>
+        <v>0</v>
+      </c>
+      <c r="H208" s="18">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="I207" s="18">
+      <c r="I208" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J207" s="19"/>
-      <c r="K207" s="46"/>
-    </row>
-    <row r="208" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A208" s="72" t="s">
+      <c r="J208" s="19"/>
+      <c r="K208" s="46"/>
+    </row>
+    <row r="209" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B208" s="62"/>
-      <c r="C208" s="62"/>
-      <c r="D208" s="62"/>
-      <c r="E208" s="62"/>
-      <c r="F208" s="62"/>
-      <c r="G208" s="62"/>
-      <c r="H208" s="62"/>
-      <c r="I208" s="62"/>
-      <c r="J208" s="62"/>
-      <c r="K208" s="63"/>
-    </row>
-    <row r="209" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A209" s="29" t="s">
+      <c r="B209" s="55"/>
+      <c r="C209" s="55"/>
+      <c r="D209" s="55"/>
+      <c r="E209" s="55"/>
+      <c r="F209" s="55"/>
+      <c r="G209" s="55"/>
+      <c r="H209" s="55"/>
+      <c r="I209" s="55"/>
+      <c r="J209" s="55"/>
+      <c r="K209" s="56"/>
+    </row>
+    <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A210" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B209" s="69" t="s">
+      <c r="B210" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C209" s="62"/>
-      <c r="D209" s="62"/>
-      <c r="E209" s="62"/>
-      <c r="F209" s="62"/>
-      <c r="G209" s="62"/>
-      <c r="H209" s="62"/>
-      <c r="I209" s="62"/>
-      <c r="J209" s="62"/>
-      <c r="K209" s="63"/>
-    </row>
-    <row r="210" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A210" s="30" t="s">
+      <c r="C210" s="55"/>
+      <c r="D210" s="55"/>
+      <c r="E210" s="55"/>
+      <c r="F210" s="55"/>
+      <c r="G210" s="55"/>
+      <c r="H210" s="55"/>
+      <c r="I210" s="55"/>
+      <c r="J210" s="55"/>
+      <c r="K210" s="56"/>
+    </row>
+    <row r="211" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B210" s="69" t="s">
+      <c r="B211" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C210" s="62"/>
-      <c r="D210" s="62"/>
-      <c r="E210" s="62"/>
-      <c r="F210" s="62"/>
-      <c r="G210" s="62"/>
-      <c r="H210" s="62"/>
-      <c r="I210" s="62"/>
-      <c r="J210" s="62"/>
-      <c r="K210" s="63"/>
-    </row>
-    <row r="211" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A211" s="37"/>
-      <c r="B211" s="38"/>
-      <c r="C211" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D211" s="38"/>
-      <c r="E211" s="40"/>
-      <c r="F211" s="40"/>
-      <c r="G211" s="41"/>
-      <c r="H211" s="41"/>
-      <c r="I211" s="41">
-        <f t="shared" ref="I211:I221" si="9">H211-G211</f>
-        <v>0</v>
-      </c>
-      <c r="J211" s="45"/>
-      <c r="K211" s="43"/>
+      <c r="C211" s="55"/>
+      <c r="D211" s="55"/>
+      <c r="E211" s="55"/>
+      <c r="F211" s="55"/>
+      <c r="G211" s="55"/>
+      <c r="H211" s="55"/>
+      <c r="I211" s="55"/>
+      <c r="J211" s="55"/>
+      <c r="K211" s="56"/>
     </row>
     <row r="212" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A212" s="37"/>
@@ -8228,7 +8259,7 @@
       <c r="G212" s="41"/>
       <c r="H212" s="41"/>
       <c r="I212" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I212:I222" si="9">H212-G212</f>
         <v>0</v>
       </c>
       <c r="J212" s="45"/>
@@ -8379,95 +8410,95 @@
       <c r="K220" s="43"/>
     </row>
     <row r="221" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A221" s="13"/>
-      <c r="B221" s="15"/>
-      <c r="C221" s="15"/>
-      <c r="D221" s="15"/>
-      <c r="E221" s="15" t="s">
+      <c r="A221" s="37"/>
+      <c r="B221" s="38"/>
+      <c r="C221" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D221" s="38"/>
+      <c r="E221" s="40"/>
+      <c r="F221" s="40"/>
+      <c r="G221" s="41"/>
+      <c r="H221" s="41"/>
+      <c r="I221" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J221" s="45"/>
+      <c r="K221" s="43"/>
+    </row>
+    <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A222" s="13"/>
+      <c r="B222" s="15"/>
+      <c r="C222" s="15"/>
+      <c r="D222" s="15"/>
+      <c r="E222" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F221" s="15"/>
-      <c r="G221" s="18">
-        <f t="shared" ref="G221:H221" si="10">SUM(G211:G220)</f>
-        <v>0</v>
-      </c>
-      <c r="H221" s="18">
+      <c r="F222" s="15"/>
+      <c r="G222" s="18">
+        <f t="shared" ref="G222:H222" si="10">SUM(G212:G221)</f>
+        <v>0</v>
+      </c>
+      <c r="H222" s="18">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="I221" s="18">
+      <c r="I222" s="18">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J221" s="19"/>
-      <c r="K221" s="46"/>
-    </row>
-    <row r="222" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A222" s="54" t="s">
+      <c r="J222" s="19"/>
+      <c r="K222" s="46"/>
+    </row>
+    <row r="223" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A223" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B222" s="55"/>
-      <c r="C222" s="55"/>
-      <c r="D222" s="55"/>
-      <c r="E222" s="55"/>
-      <c r="F222" s="55"/>
-      <c r="G222" s="55"/>
-      <c r="H222" s="55"/>
-      <c r="I222" s="55"/>
-      <c r="J222" s="55"/>
-      <c r="K222" s="56"/>
-    </row>
-    <row r="223" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A223" s="32" t="s">
+      <c r="B223" s="63"/>
+      <c r="C223" s="63"/>
+      <c r="D223" s="63"/>
+      <c r="E223" s="63"/>
+      <c r="F223" s="63"/>
+      <c r="G223" s="63"/>
+      <c r="H223" s="63"/>
+      <c r="I223" s="63"/>
+      <c r="J223" s="63"/>
+      <c r="K223" s="64"/>
+    </row>
+    <row r="224" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A224" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B223" s="57" t="s">
+      <c r="B224" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C223" s="55"/>
-      <c r="D223" s="55"/>
-      <c r="E223" s="55"/>
-      <c r="F223" s="55"/>
-      <c r="G223" s="55"/>
-      <c r="H223" s="55"/>
-      <c r="I223" s="55"/>
-      <c r="J223" s="55"/>
-      <c r="K223" s="56"/>
-    </row>
-    <row r="224" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A224" s="33" t="s">
+      <c r="C224" s="63"/>
+      <c r="D224" s="63"/>
+      <c r="E224" s="63"/>
+      <c r="F224" s="63"/>
+      <c r="G224" s="63"/>
+      <c r="H224" s="63"/>
+      <c r="I224" s="63"/>
+      <c r="J224" s="63"/>
+      <c r="K224" s="64"/>
+    </row>
+    <row r="225" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A225" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B224" s="57" t="s">
+      <c r="B225" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C224" s="55"/>
-      <c r="D224" s="55"/>
-      <c r="E224" s="55"/>
-      <c r="F224" s="55"/>
-      <c r="G224" s="55"/>
-      <c r="H224" s="55"/>
-      <c r="I224" s="55"/>
-      <c r="J224" s="55"/>
-      <c r="K224" s="56"/>
-    </row>
-    <row r="225" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A225" s="37"/>
-      <c r="B225" s="38"/>
-      <c r="C225" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D225" s="38"/>
-      <c r="E225" s="40"/>
-      <c r="F225" s="40"/>
-      <c r="G225" s="41"/>
-      <c r="H225" s="41"/>
-      <c r="I225" s="41">
-        <f t="shared" ref="I225:I235" si="11">H225-G225</f>
-        <v>0</v>
-      </c>
-      <c r="J225" s="45"/>
-      <c r="K225" s="43"/>
+      <c r="C225" s="63"/>
+      <c r="D225" s="63"/>
+      <c r="E225" s="63"/>
+      <c r="F225" s="63"/>
+      <c r="G225" s="63"/>
+      <c r="H225" s="63"/>
+      <c r="I225" s="63"/>
+      <c r="J225" s="63"/>
+      <c r="K225" s="64"/>
     </row>
     <row r="226" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A226" s="37"/>
@@ -8481,7 +8512,7 @@
       <c r="G226" s="41"/>
       <c r="H226" s="41"/>
       <c r="I226" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="I226:I236" si="11">H226-G226</f>
         <v>0</v>
       </c>
       <c r="J226" s="45"/>
@@ -8632,35 +8663,53 @@
       <c r="K234" s="43"/>
     </row>
     <row r="235" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A235" s="48"/>
-      <c r="B235" s="49"/>
-      <c r="C235" s="49"/>
-      <c r="D235" s="49"/>
-      <c r="E235" s="49" t="s">
+      <c r="A235" s="37"/>
+      <c r="B235" s="38"/>
+      <c r="C235" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D235" s="38"/>
+      <c r="E235" s="40"/>
+      <c r="F235" s="40"/>
+      <c r="G235" s="41"/>
+      <c r="H235" s="41"/>
+      <c r="I235" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J235" s="45"/>
+      <c r="K235" s="43"/>
+    </row>
+    <row r="236" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A236" s="48"/>
+      <c r="B236" s="49"/>
+      <c r="C236" s="49"/>
+      <c r="D236" s="49"/>
+      <c r="E236" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F235" s="49"/>
-      <c r="G235" s="50">
-        <f t="shared" ref="G235:H235" si="12">SUM(G225:G234)</f>
-        <v>0</v>
-      </c>
-      <c r="H235" s="50">
+      <c r="F236" s="49"/>
+      <c r="G236" s="50">
+        <f t="shared" ref="G236:H236" si="12">SUM(G226:G235)</f>
+        <v>0</v>
+      </c>
+      <c r="H236" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="I235" s="50">
+      <c r="I236" s="50">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J235" s="51"/>
-      <c r="K235" s="52"/>
+      <c r="J236" s="51"/>
+      <c r="K236" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{B1F15A25-4CDC-43AE-BA01-97157FD3ABCF}">
+      <autoFilter ref="A1:K15" xr:uid="{EAE1109F-3B36-43D3-915C-2BC1CA012B0B}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -8671,17 +8720,9 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B195:K195"/>
-    <mergeCell ref="B196:K196"/>
-    <mergeCell ref="A208:K208"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A194:K194"/>
-    <mergeCell ref="A222:K222"/>
-    <mergeCell ref="B223:K223"/>
+    <mergeCell ref="A223:K223"/>
     <mergeCell ref="B224:K224"/>
+    <mergeCell ref="B225:K225"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -8692,11 +8733,19 @@
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
     <mergeCell ref="A118:K118"/>
-    <mergeCell ref="B209:K209"/>
     <mergeCell ref="B210:K210"/>
+    <mergeCell ref="B211:K211"/>
     <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B196:K196"/>
+    <mergeCell ref="B197:K197"/>
+    <mergeCell ref="A209:K209"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A195:K195"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B197:B206 B211:B220 B154:B192">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B193 B198:B207 B212:B221">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -8713,7 +8762,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B195:B207 B209:B221 B223:B235 B152:B193">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B152:B194 B196:B208 B210:B222 B224:B236">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -8721,34 +8770,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B225:B234">
+  <conditionalFormatting sqref="B226:B235">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B225))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B226))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B225))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B226))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B225))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B226))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B225))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B226))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B225))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B226))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G197:G207 G211:G221 G225:G235 G154:G193">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G154:G194 G198:G208 G212:G222 G226:G236">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H235">
+  <conditionalFormatting sqref="H1:H236">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I197:I207 I211:I221 I225:I235 I154:I193">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I198:I208 I212:I222 I226:I236 I154:I194">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -8757,7 +8806,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F225:F234 F211:F220 F86:F116 F197:F206 F5:F45 F50:F81 F121:F149 F154:F192" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F226:F235 F212:F221 F86:F116 F198:F207 F5:F45 F50:F81 F121:F149 F154:F193" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8773,13 +8822,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E116 E197:E206 E211:E220 E225:E234 E50:E81 E121:E149 E154:E192</xm:sqref>
+          <xm:sqref>E5:E45 E86:E116 E198:E207 E212:E221 E226:E235 E50:E81 E121:E149 E154:E193</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B116 B197:B206 B211:B220 B225:B234 B50:B81 B121:B149 B154:B192</xm:sqref>
+          <xm:sqref>B5:B45 B86:B116 B198:B207 B212:B221 B226:B235 B50:B81 B121:B149 B154:B193</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -10420,6 +10469,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -10654,27 +10723,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10691,23 +10759,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Catch up last week
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37B1FE2-DB25-45D7-88C5-D085FEE3D72C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81ED3363-ADE9-4926-8DBC-9C31D6801C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worklog_Tasks&amp;Times" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="325">
   <si>
     <t>Date</t>
   </si>
@@ -1037,9 +1037,6 @@
     <t xml:space="preserve">Due to sickness, combined with a few breaks due to me being busy, and this being done over 2 days, this took quite some time more than planned. </t>
   </si>
   <si>
-    <t>2 at 17:00</t>
-  </si>
-  <si>
     <t>Fill in WorkLog planning for Monday</t>
   </si>
   <si>
@@ -1073,7 +1070,13 @@
     <t>Learn Cross-Validation</t>
   </si>
   <si>
-    <t>Learn how to evaluate using Cross-Validation &amp; ist variants</t>
+    <t>Learn how to evaluate using Cross-Validation &amp; its variants</t>
+  </si>
+  <si>
+    <t>07&amp;13.01.2025</t>
+  </si>
+  <si>
+    <t>Do DataCamp course "Model Validation in Python"</t>
   </si>
 </sst>
 </file>
@@ -8066,7 +8069,7 @@
         <v>79</v>
       </c>
       <c r="D198" s="38" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E198" s="40" t="s">
         <v>61</v>
@@ -8098,7 +8101,7 @@
         <v>207</v>
       </c>
       <c r="D199" s="38" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E199" s="40" t="s">
         <v>61</v>
@@ -8186,11 +8189,11 @@
       </c>
     </row>
     <row r="202" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A202" s="37">
-        <v>45664</v>
+      <c r="A202" s="37" t="s">
+        <v>323</v>
       </c>
       <c r="B202" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C202" s="39" t="s">
         <v>305</v>
@@ -8207,15 +8210,15 @@
       <c r="G202" s="41">
         <v>4</v>
       </c>
-      <c r="H202" s="41"/>
+      <c r="H202" s="41">
+        <v>5</v>
+      </c>
       <c r="I202" s="41">
         <f t="shared" si="7"/>
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="J202" s="45"/>
-      <c r="K202" s="43" t="s">
-        <v>311</v>
-      </c>
+      <c r="K202" s="43"/>
     </row>
     <row r="203" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A203" s="37">
@@ -8314,13 +8317,13 @@
         <v>45670</v>
       </c>
       <c r="B206" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C206" s="39" t="s">
+        <v>321</v>
+      </c>
+      <c r="D206" s="38" t="s">
         <v>322</v>
-      </c>
-      <c r="D206" s="38" t="s">
-        <v>323</v>
       </c>
       <c r="E206" s="40" t="s">
         <v>66</v>
@@ -8331,28 +8334,40 @@
       <c r="G206" s="41">
         <v>2</v>
       </c>
-      <c r="H206" s="41"/>
+      <c r="H206" s="41">
+        <v>1.5</v>
+      </c>
       <c r="I206" s="41">
         <f t="shared" si="7"/>
-        <v>-2</v>
+        <v>-0.5</v>
       </c>
       <c r="J206" s="45"/>
       <c r="K206" s="43"/>
     </row>
     <row r="207" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A207" s="37"/>
-      <c r="B207" s="38"/>
+      <c r="B207" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C207" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D207" s="38"/>
-      <c r="E207" s="40"/>
-      <c r="F207" s="40"/>
-      <c r="G207" s="41"/>
+        <v>321</v>
+      </c>
+      <c r="D207" s="38" t="s">
+        <v>324</v>
+      </c>
+      <c r="E207" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="F207" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="G207" s="41">
+        <v>4</v>
+      </c>
       <c r="H207" s="41"/>
       <c r="I207" s="41">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="J207" s="45"/>
       <c r="K207" s="43"/>
@@ -8386,15 +8401,15 @@
       <c r="F209" s="15"/>
       <c r="G209" s="18">
         <f t="shared" ref="G209:H209" si="8">SUM(G198:G208)</f>
-        <v>18.75</v>
+        <v>22.75</v>
       </c>
       <c r="H209" s="18">
         <f t="shared" si="8"/>
-        <v>8</v>
+        <v>14.5</v>
       </c>
       <c r="I209" s="18">
         <f t="shared" si="7"/>
-        <v>-10.75</v>
+        <v>-8.25</v>
       </c>
       <c r="J209" s="19"/>
       <c r="K209" s="46"/>
@@ -8459,7 +8474,7 @@
         <v>79</v>
       </c>
       <c r="D213" s="38" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E213" s="40" t="s">
         <v>61</v>
@@ -8491,7 +8506,7 @@
         <v>207</v>
       </c>
       <c r="D214" s="38" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E214" s="40" t="s">
         <v>61</v>
@@ -8520,10 +8535,10 @@
         <v>54</v>
       </c>
       <c r="C215" s="39" t="s">
+        <v>314</v>
+      </c>
+      <c r="D215" s="38" t="s">
         <v>315</v>
-      </c>
-      <c r="D215" s="38" t="s">
-        <v>316</v>
       </c>
       <c r="E215" s="40" t="s">
         <v>66</v>
@@ -8552,10 +8567,10 @@
         <v>54</v>
       </c>
       <c r="C216" s="39" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D216" s="38" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E216" s="40" t="s">
         <v>66</v>
@@ -8581,13 +8596,13 @@
         <v>45670</v>
       </c>
       <c r="B217" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C217" s="39" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D217" s="38" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E217" s="40" t="s">
         <v>63</v>
@@ -8598,10 +8613,12 @@
       <c r="G217" s="41">
         <v>0.5</v>
       </c>
-      <c r="H217" s="41"/>
+      <c r="H217" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I217" s="41">
         <f t="shared" si="9"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J217" s="45"/>
       <c r="K217" s="43"/>
@@ -8614,10 +8631,10 @@
         <v>45</v>
       </c>
       <c r="C218" s="39" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D218" s="38" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E218" s="40" t="s">
         <v>67</v>
@@ -8725,11 +8742,11 @@
       </c>
       <c r="H223" s="18">
         <f t="shared" si="10"/>
-        <v>1.85</v>
+        <v>2.35</v>
       </c>
       <c r="I223" s="18">
         <f t="shared" si="9"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J223" s="19"/>
       <c r="K223" s="46"/>
@@ -8992,7 +9009,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{1419A995-DC1D-44CF-8D40-CAC1F2997D1E}">
+      <autoFilter ref="A1:K15" xr:uid="{EFD0DA2C-85A2-41CD-9897-E6AD670C26ED}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>

</xml_diff>

<commit_message>
W7 DataLab 1 Work III (Gradient Descent Article))
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81ED3363-ADE9-4926-8DBC-9C31D6801C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57EB2914-3E63-49CC-A556-B91CA4402C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$222</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Worklog_Tasks&amp;Times'!$A$1:$K$228</definedName>
     <definedName name="Z_8BAC9A6B_5D32_4E8D_967D_E17D357516F8_.wvu.FilterData" localSheetId="0" hidden="1">'Worklog_Tasks&amp;Times'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="334">
   <si>
     <t>Date</t>
   </si>
@@ -1077,6 +1077,33 @@
   </si>
   <si>
     <t>Do DataCamp course "Model Validation in Python"</t>
+  </si>
+  <si>
+    <t>Learn Optimization Algorithms</t>
+  </si>
+  <si>
+    <t>Learn Gradient Descent Optimization Algorithm</t>
+  </si>
+  <si>
+    <t>Learn Gradient Descent with Momentum</t>
+  </si>
+  <si>
+    <t>Learn how to implement Regression Model</t>
+  </si>
+  <si>
+    <t>Learn how to Train the Model with Gradient Descent</t>
+  </si>
+  <si>
+    <t>Do Assignment 1</t>
+  </si>
+  <si>
+    <t>Do Assignment 2</t>
+  </si>
+  <si>
+    <t>Fill out Block A WorkLog regarding Python Exam retake</t>
+  </si>
+  <si>
+    <t>Block A Evidencing</t>
   </si>
 </sst>
 </file>
@@ -1562,26 +1589,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1598,6 +1605,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1615,6 +1624,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2087,7 +2114,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K237"/>
+  <dimension ref="A1:K243"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -2139,53 +2166,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3524,53 +3551,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="62"/>
+      <c r="K49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4623,53 +4650,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72" t="s">
+      <c r="A83" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="55"/>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="55"/>
-      <c r="I83" s="55"/>
-      <c r="J83" s="55"/>
-      <c r="K83" s="56"/>
+      <c r="B83" s="62"/>
+      <c r="C83" s="62"/>
+      <c r="D83" s="62"/>
+      <c r="E83" s="62"/>
+      <c r="F83" s="62"/>
+      <c r="G83" s="62"/>
+      <c r="H83" s="62"/>
+      <c r="I83" s="62"/>
+      <c r="J83" s="62"/>
+      <c r="K83" s="63"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="73" t="s">
+      <c r="B84" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="55"/>
-      <c r="D84" s="55"/>
-      <c r="E84" s="55"/>
-      <c r="F84" s="55"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="55"/>
-      <c r="I84" s="55"/>
-      <c r="J84" s="55"/>
-      <c r="K84" s="56"/>
+      <c r="C84" s="62"/>
+      <c r="D84" s="62"/>
+      <c r="E84" s="62"/>
+      <c r="F84" s="62"/>
+      <c r="G84" s="62"/>
+      <c r="H84" s="62"/>
+      <c r="I84" s="62"/>
+      <c r="J84" s="62"/>
+      <c r="K84" s="63"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="73" t="s">
+      <c r="B85" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="55"/>
-      <c r="D85" s="55"/>
-      <c r="E85" s="55"/>
-      <c r="F85" s="55"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="55"/>
-      <c r="I85" s="55"/>
-      <c r="J85" s="55"/>
-      <c r="K85" s="56"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="62"/>
+      <c r="G85" s="62"/>
+      <c r="H85" s="62"/>
+      <c r="I85" s="62"/>
+      <c r="J85" s="62"/>
+      <c r="K85" s="63"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5684,53 +5711,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="74" t="s">
+      <c r="A118" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="55"/>
-      <c r="C118" s="55"/>
-      <c r="D118" s="55"/>
-      <c r="E118" s="55"/>
-      <c r="F118" s="55"/>
-      <c r="G118" s="55"/>
-      <c r="H118" s="55"/>
-      <c r="I118" s="55"/>
-      <c r="J118" s="55"/>
-      <c r="K118" s="56"/>
+      <c r="B118" s="62"/>
+      <c r="C118" s="62"/>
+      <c r="D118" s="62"/>
+      <c r="E118" s="62"/>
+      <c r="F118" s="62"/>
+      <c r="G118" s="62"/>
+      <c r="H118" s="62"/>
+      <c r="I118" s="62"/>
+      <c r="J118" s="62"/>
+      <c r="K118" s="63"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="58" t="s">
+      <c r="B119" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="55"/>
-      <c r="D119" s="55"/>
-      <c r="E119" s="55"/>
-      <c r="F119" s="55"/>
-      <c r="G119" s="55"/>
-      <c r="H119" s="55"/>
-      <c r="I119" s="55"/>
-      <c r="J119" s="55"/>
-      <c r="K119" s="56"/>
+      <c r="C119" s="62"/>
+      <c r="D119" s="62"/>
+      <c r="E119" s="62"/>
+      <c r="F119" s="62"/>
+      <c r="G119" s="62"/>
+      <c r="H119" s="62"/>
+      <c r="I119" s="62"/>
+      <c r="J119" s="62"/>
+      <c r="K119" s="63"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="58" t="s">
+      <c r="B120" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="55"/>
-      <c r="D120" s="55"/>
-      <c r="E120" s="55"/>
-      <c r="F120" s="55"/>
-      <c r="G120" s="55"/>
-      <c r="H120" s="55"/>
-      <c r="I120" s="55"/>
-      <c r="J120" s="55"/>
-      <c r="K120" s="56"/>
+      <c r="C120" s="62"/>
+      <c r="D120" s="62"/>
+      <c r="E120" s="62"/>
+      <c r="F120" s="62"/>
+      <c r="G120" s="62"/>
+      <c r="H120" s="62"/>
+      <c r="I120" s="62"/>
+      <c r="J120" s="62"/>
+      <c r="K120" s="63"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6667,53 +6694,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="59" t="s">
+      <c r="A151" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="55"/>
-      <c r="C151" s="55"/>
-      <c r="D151" s="55"/>
-      <c r="E151" s="55"/>
-      <c r="F151" s="55"/>
-      <c r="G151" s="55"/>
-      <c r="H151" s="55"/>
-      <c r="I151" s="55"/>
-      <c r="J151" s="55"/>
-      <c r="K151" s="56"/>
+      <c r="B151" s="62"/>
+      <c r="C151" s="62"/>
+      <c r="D151" s="62"/>
+      <c r="E151" s="62"/>
+      <c r="F151" s="62"/>
+      <c r="G151" s="62"/>
+      <c r="H151" s="62"/>
+      <c r="I151" s="62"/>
+      <c r="J151" s="62"/>
+      <c r="K151" s="63"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="60" t="s">
+      <c r="B152" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="55"/>
-      <c r="D152" s="55"/>
-      <c r="E152" s="55"/>
-      <c r="F152" s="55"/>
-      <c r="G152" s="55"/>
-      <c r="H152" s="55"/>
-      <c r="I152" s="55"/>
-      <c r="J152" s="55"/>
-      <c r="K152" s="56"/>
+      <c r="C152" s="62"/>
+      <c r="D152" s="62"/>
+      <c r="E152" s="62"/>
+      <c r="F152" s="62"/>
+      <c r="G152" s="62"/>
+      <c r="H152" s="62"/>
+      <c r="I152" s="62"/>
+      <c r="J152" s="62"/>
+      <c r="K152" s="63"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="60" t="s">
+      <c r="B153" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="55"/>
-      <c r="D153" s="55"/>
-      <c r="E153" s="55"/>
-      <c r="F153" s="55"/>
-      <c r="G153" s="55"/>
-      <c r="H153" s="55"/>
-      <c r="I153" s="55"/>
-      <c r="J153" s="55"/>
-      <c r="K153" s="56"/>
+      <c r="C153" s="62"/>
+      <c r="D153" s="62"/>
+      <c r="E153" s="62"/>
+      <c r="F153" s="62"/>
+      <c r="G153" s="62"/>
+      <c r="H153" s="62"/>
+      <c r="I153" s="62"/>
+      <c r="J153" s="62"/>
+      <c r="K153" s="63"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -8010,53 +8037,53 @@
       <c r="K194" s="46"/>
     </row>
     <row r="195" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="61" t="s">
+      <c r="A195" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B195" s="55"/>
-      <c r="C195" s="55"/>
-      <c r="D195" s="55"/>
-      <c r="E195" s="55"/>
-      <c r="F195" s="55"/>
-      <c r="G195" s="55"/>
-      <c r="H195" s="55"/>
-      <c r="I195" s="55"/>
-      <c r="J195" s="55"/>
-      <c r="K195" s="56"/>
+      <c r="B195" s="62"/>
+      <c r="C195" s="62"/>
+      <c r="D195" s="62"/>
+      <c r="E195" s="62"/>
+      <c r="F195" s="62"/>
+      <c r="G195" s="62"/>
+      <c r="H195" s="62"/>
+      <c r="I195" s="62"/>
+      <c r="J195" s="62"/>
+      <c r="K195" s="63"/>
     </row>
     <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A196" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B196" s="54" t="s">
+      <c r="B196" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C196" s="55"/>
-      <c r="D196" s="55"/>
-      <c r="E196" s="55"/>
-      <c r="F196" s="55"/>
-      <c r="G196" s="55"/>
-      <c r="H196" s="55"/>
-      <c r="I196" s="55"/>
-      <c r="J196" s="55"/>
-      <c r="K196" s="56"/>
+      <c r="C196" s="62"/>
+      <c r="D196" s="62"/>
+      <c r="E196" s="62"/>
+      <c r="F196" s="62"/>
+      <c r="G196" s="62"/>
+      <c r="H196" s="62"/>
+      <c r="I196" s="62"/>
+      <c r="J196" s="62"/>
+      <c r="K196" s="63"/>
     </row>
     <row r="197" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B197" s="54" t="s">
+      <c r="B197" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C197" s="55"/>
-      <c r="D197" s="55"/>
-      <c r="E197" s="55"/>
-      <c r="F197" s="55"/>
-      <c r="G197" s="55"/>
-      <c r="H197" s="55"/>
-      <c r="I197" s="55"/>
-      <c r="J197" s="55"/>
-      <c r="K197" s="56"/>
+      <c r="C197" s="62"/>
+      <c r="D197" s="62"/>
+      <c r="E197" s="62"/>
+      <c r="F197" s="62"/>
+      <c r="G197" s="62"/>
+      <c r="H197" s="62"/>
+      <c r="I197" s="62"/>
+      <c r="J197" s="62"/>
+      <c r="K197" s="63"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="37">
@@ -8084,7 +8111,7 @@
         <v>0.25</v>
       </c>
       <c r="I198" s="41">
-        <f t="shared" ref="I198:I209" si="7">H198-G198</f>
+        <f t="shared" ref="I198:I215" si="7">H198-G198</f>
         <v>0</v>
       </c>
       <c r="J198" s="45"/>
@@ -8373,16 +8400,30 @@
       <c r="K207" s="43"/>
     </row>
     <row r="208" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A208" s="37"/>
-      <c r="B208" s="38"/>
+      <c r="A208" s="37">
+        <v>45671</v>
+      </c>
+      <c r="B208" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C208" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D208" s="38"/>
-      <c r="E208" s="40"/>
-      <c r="F208" s="40"/>
-      <c r="G208" s="41"/>
-      <c r="H208" s="41"/>
+        <v>325</v>
+      </c>
+      <c r="D208" s="38" t="s">
+        <v>326</v>
+      </c>
+      <c r="E208" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F208" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="G208" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H208" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I208" s="41">
         <f t="shared" si="7"/>
         <v>0</v>
@@ -8391,299 +8432,303 @@
       <c r="K208" s="43"/>
     </row>
     <row r="209" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A209" s="13"/>
-      <c r="B209" s="15"/>
-      <c r="C209" s="15"/>
-      <c r="D209" s="15"/>
-      <c r="E209" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F209" s="15"/>
-      <c r="G209" s="18">
-        <f t="shared" ref="G209:H209" si="8">SUM(G198:G208)</f>
-        <v>22.75</v>
-      </c>
-      <c r="H209" s="18">
-        <f t="shared" si="8"/>
-        <v>14.5</v>
-      </c>
-      <c r="I209" s="18">
+      <c r="A209" s="37">
+        <v>45671</v>
+      </c>
+      <c r="B209" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C209" s="39" t="s">
+        <v>325</v>
+      </c>
+      <c r="D209" s="38" t="s">
+        <v>327</v>
+      </c>
+      <c r="E209" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F209" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="G209" s="41">
+        <v>1</v>
+      </c>
+      <c r="H209" s="41"/>
+      <c r="I209" s="41">
         <f t="shared" si="7"/>
-        <v>-8.25</v>
-      </c>
-      <c r="J209" s="19"/>
-      <c r="K209" s="46"/>
-    </row>
-    <row r="210" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A210" s="57" t="s">
-        <v>25</v>
-      </c>
-      <c r="B210" s="55"/>
-      <c r="C210" s="55"/>
-      <c r="D210" s="55"/>
-      <c r="E210" s="55"/>
-      <c r="F210" s="55"/>
-      <c r="G210" s="55"/>
-      <c r="H210" s="55"/>
-      <c r="I210" s="55"/>
-      <c r="J210" s="55"/>
-      <c r="K210" s="56"/>
+        <v>-1</v>
+      </c>
+      <c r="J209" s="45"/>
+      <c r="K209" s="43"/>
+    </row>
+    <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A210" s="37">
+        <v>45671</v>
+      </c>
+      <c r="B210" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C210" s="39" t="s">
+        <v>325</v>
+      </c>
+      <c r="D210" s="38" t="s">
+        <v>328</v>
+      </c>
+      <c r="E210" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F210" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="G210" s="41">
+        <v>1</v>
+      </c>
+      <c r="H210" s="41"/>
+      <c r="I210" s="41">
+        <f t="shared" si="7"/>
+        <v>-1</v>
+      </c>
+      <c r="J210" s="45"/>
+      <c r="K210" s="43"/>
     </row>
     <row r="211" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A211" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B211" s="75" t="s">
-        <v>13</v>
-      </c>
-      <c r="C211" s="55"/>
-      <c r="D211" s="55"/>
-      <c r="E211" s="55"/>
-      <c r="F211" s="55"/>
-      <c r="G211" s="55"/>
-      <c r="H211" s="55"/>
-      <c r="I211" s="55"/>
-      <c r="J211" s="55"/>
-      <c r="K211" s="56"/>
-    </row>
-    <row r="212" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A212" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B212" s="75" t="s">
-        <v>15</v>
-      </c>
-      <c r="C212" s="55"/>
-      <c r="D212" s="55"/>
-      <c r="E212" s="55"/>
-      <c r="F212" s="55"/>
-      <c r="G212" s="55"/>
-      <c r="H212" s="55"/>
-      <c r="I212" s="55"/>
-      <c r="J212" s="55"/>
-      <c r="K212" s="56"/>
+      <c r="A211" s="37">
+        <v>45671</v>
+      </c>
+      <c r="B211" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C211" s="39" t="s">
+        <v>325</v>
+      </c>
+      <c r="D211" s="38" t="s">
+        <v>329</v>
+      </c>
+      <c r="E211" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F211" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="G211" s="41">
+        <v>1</v>
+      </c>
+      <c r="H211" s="41"/>
+      <c r="I211" s="41">
+        <f t="shared" si="7"/>
+        <v>-1</v>
+      </c>
+      <c r="J211" s="45"/>
+      <c r="K211" s="43"/>
+    </row>
+    <row r="212" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A212" s="37">
+        <v>45671</v>
+      </c>
+      <c r="B212" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C212" s="39" t="s">
+        <v>325</v>
+      </c>
+      <c r="D212" s="38" t="s">
+        <v>330</v>
+      </c>
+      <c r="E212" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="F212" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="G212" s="41">
+        <v>2</v>
+      </c>
+      <c r="H212" s="41"/>
+      <c r="I212" s="41">
+        <f t="shared" si="7"/>
+        <v>-2</v>
+      </c>
+      <c r="J212" s="45"/>
+      <c r="K212" s="43"/>
     </row>
     <row r="213" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A213" s="37">
-        <v>45670</v>
+        <v>45671</v>
       </c>
       <c r="B213" s="38" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="C213" s="39" t="s">
-        <v>79</v>
+        <v>325</v>
       </c>
       <c r="D213" s="38" t="s">
-        <v>311</v>
+        <v>331</v>
       </c>
       <c r="E213" s="40" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="F213" s="40" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="G213" s="41">
-        <v>0.25</v>
-      </c>
-      <c r="H213" s="41">
-        <v>0.25</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="H213" s="41"/>
       <c r="I213" s="41">
-        <f t="shared" ref="I213:I223" si="9">H213-G213</f>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>-2</v>
       </c>
       <c r="J213" s="45"/>
       <c r="K213" s="43"/>
     </row>
     <row r="214" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A214" s="37">
-        <v>45670</v>
-      </c>
-      <c r="B214" s="38" t="s">
-        <v>54</v>
-      </c>
+      <c r="A214" s="37"/>
+      <c r="B214" s="38"/>
       <c r="C214" s="39" t="s">
-        <v>207</v>
-      </c>
-      <c r="D214" s="38" t="s">
-        <v>312</v>
-      </c>
-      <c r="E214" s="40" t="s">
-        <v>61</v>
-      </c>
-      <c r="F214" s="40" t="s">
-        <v>87</v>
-      </c>
-      <c r="G214" s="41">
-        <v>0.25</v>
-      </c>
-      <c r="H214" s="41">
-        <v>0.25</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="D214" s="38"/>
+      <c r="E214" s="40"/>
+      <c r="F214" s="40"/>
+      <c r="G214" s="41"/>
+      <c r="H214" s="41"/>
       <c r="I214" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J214" s="45"/>
       <c r="K214" s="43"/>
     </row>
     <row r="215" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A215" s="37">
+      <c r="A215" s="13"/>
+      <c r="B215" s="15"/>
+      <c r="C215" s="15"/>
+      <c r="D215" s="15"/>
+      <c r="E215" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F215" s="15"/>
+      <c r="G215" s="18">
+        <f t="shared" ref="G215:H215" si="8">SUM(G198:G214)</f>
+        <v>30.25</v>
+      </c>
+      <c r="H215" s="18">
+        <f t="shared" si="8"/>
+        <v>15</v>
+      </c>
+      <c r="I215" s="18">
+        <f t="shared" si="7"/>
+        <v>-15.25</v>
+      </c>
+      <c r="J215" s="19"/>
+      <c r="K215" s="46"/>
+    </row>
+    <row r="216" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="B216" s="62"/>
+      <c r="C216" s="62"/>
+      <c r="D216" s="62"/>
+      <c r="E216" s="62"/>
+      <c r="F216" s="62"/>
+      <c r="G216" s="62"/>
+      <c r="H216" s="62"/>
+      <c r="I216" s="62"/>
+      <c r="J216" s="62"/>
+      <c r="K216" s="63"/>
+    </row>
+    <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A217" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B217" s="69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C217" s="62"/>
+      <c r="D217" s="62"/>
+      <c r="E217" s="62"/>
+      <c r="F217" s="62"/>
+      <c r="G217" s="62"/>
+      <c r="H217" s="62"/>
+      <c r="I217" s="62"/>
+      <c r="J217" s="62"/>
+      <c r="K217" s="63"/>
+    </row>
+    <row r="218" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B218" s="69" t="s">
+        <v>15</v>
+      </c>
+      <c r="C218" s="62"/>
+      <c r="D218" s="62"/>
+      <c r="E218" s="62"/>
+      <c r="F218" s="62"/>
+      <c r="G218" s="62"/>
+      <c r="H218" s="62"/>
+      <c r="I218" s="62"/>
+      <c r="J218" s="62"/>
+      <c r="K218" s="63"/>
+    </row>
+    <row r="219" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A219" s="37">
         <v>45670</v>
       </c>
-      <c r="B215" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="C215" s="39" t="s">
-        <v>314</v>
-      </c>
-      <c r="D215" s="38" t="s">
-        <v>315</v>
-      </c>
-      <c r="E215" s="40" t="s">
-        <v>66</v>
-      </c>
-      <c r="F215" s="40" t="s">
-        <v>184</v>
-      </c>
-      <c r="G215" s="41">
-        <v>0.75</v>
-      </c>
-      <c r="H215" s="41">
-        <v>0.75</v>
-      </c>
-      <c r="I215" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J215" s="45"/>
-      <c r="K215" s="43"/>
-    </row>
-    <row r="216" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A216" s="37">
-        <v>45670</v>
-      </c>
-      <c r="B216" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="C216" s="39" t="s">
-        <v>314</v>
-      </c>
-      <c r="D216" s="38" t="s">
-        <v>316</v>
-      </c>
-      <c r="E216" s="40" t="s">
-        <v>66</v>
-      </c>
-      <c r="F216" s="40" t="s">
-        <v>184</v>
-      </c>
-      <c r="G216" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="H216" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="I216" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J216" s="45"/>
-      <c r="K216" s="43"/>
-    </row>
-    <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A217" s="37">
-        <v>45670</v>
-      </c>
-      <c r="B217" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="C217" s="39" t="s">
-        <v>318</v>
-      </c>
-      <c r="D217" s="38" t="s">
-        <v>317</v>
-      </c>
-      <c r="E217" s="40" t="s">
-        <v>63</v>
-      </c>
-      <c r="F217" s="40" t="s">
+      <c r="B219" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="C219" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="D219" s="38" t="s">
+        <v>311</v>
+      </c>
+      <c r="E219" s="40" t="s">
+        <v>61</v>
+      </c>
+      <c r="F219" s="40" t="s">
         <v>86</v>
       </c>
-      <c r="G217" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="H217" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="I217" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J217" s="45"/>
-      <c r="K217" s="43"/>
-    </row>
-    <row r="218" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A218" s="37">
-        <v>45670</v>
-      </c>
-      <c r="B218" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="C218" s="39" t="s">
-        <v>320</v>
-      </c>
-      <c r="D218" s="38" t="s">
-        <v>319</v>
-      </c>
-      <c r="E218" s="40" t="s">
-        <v>67</v>
-      </c>
-      <c r="F218" s="40" t="s">
-        <v>86</v>
-      </c>
-      <c r="G218" s="41">
-        <v>0.1</v>
-      </c>
-      <c r="H218" s="41">
-        <v>0.1</v>
-      </c>
-      <c r="I218" s="41">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J218" s="45"/>
-      <c r="K218" s="43"/>
-    </row>
-    <row r="219" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A219" s="37"/>
-      <c r="B219" s="38"/>
-      <c r="C219" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D219" s="38"/>
-      <c r="E219" s="40"/>
-      <c r="F219" s="40"/>
-      <c r="G219" s="41"/>
-      <c r="H219" s="41"/>
+      <c r="G219" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H219" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I219" s="41">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I219:I229" si="9">H219-G219</f>
         <v>0</v>
       </c>
       <c r="J219" s="45"/>
       <c r="K219" s="43"/>
     </row>
     <row r="220" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A220" s="37"/>
-      <c r="B220" s="38"/>
+      <c r="A220" s="37">
+        <v>45670</v>
+      </c>
+      <c r="B220" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C220" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D220" s="38"/>
-      <c r="E220" s="40"/>
-      <c r="F220" s="40"/>
-      <c r="G220" s="41"/>
-      <c r="H220" s="41"/>
+        <v>207</v>
+      </c>
+      <c r="D220" s="38" t="s">
+        <v>312</v>
+      </c>
+      <c r="E220" s="40" t="s">
+        <v>61</v>
+      </c>
+      <c r="F220" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G220" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H220" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I220" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -8692,16 +8737,30 @@
       <c r="K220" s="43"/>
     </row>
     <row r="221" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A221" s="37"/>
-      <c r="B221" s="38"/>
+      <c r="A221" s="37">
+        <v>45670</v>
+      </c>
+      <c r="B221" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C221" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D221" s="38"/>
-      <c r="E221" s="40"/>
-      <c r="F221" s="40"/>
-      <c r="G221" s="41"/>
-      <c r="H221" s="41"/>
+        <v>314</v>
+      </c>
+      <c r="D221" s="38" t="s">
+        <v>315</v>
+      </c>
+      <c r="E221" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F221" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="G221" s="41">
+        <v>0.75</v>
+      </c>
+      <c r="H221" s="41">
+        <v>0.75</v>
+      </c>
       <c r="I221" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -8710,16 +8769,30 @@
       <c r="K221" s="43"/>
     </row>
     <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A222" s="37"/>
-      <c r="B222" s="38"/>
+      <c r="A222" s="37">
+        <v>45670</v>
+      </c>
+      <c r="B222" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C222" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D222" s="38"/>
-      <c r="E222" s="40"/>
-      <c r="F222" s="40"/>
-      <c r="G222" s="41"/>
-      <c r="H222" s="41"/>
+        <v>314</v>
+      </c>
+      <c r="D222" s="38" t="s">
+        <v>316</v>
+      </c>
+      <c r="E222" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="F222" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="G222" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H222" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I222" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -8728,91 +8801,160 @@
       <c r="K222" s="43"/>
     </row>
     <row r="223" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A223" s="13"/>
-      <c r="B223" s="15"/>
-      <c r="C223" s="15"/>
-      <c r="D223" s="15"/>
-      <c r="E223" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F223" s="15"/>
-      <c r="G223" s="18">
-        <f t="shared" ref="G223:H223" si="10">SUM(G213:G222)</f>
-        <v>2.35</v>
-      </c>
-      <c r="H223" s="18">
-        <f t="shared" si="10"/>
-        <v>2.35</v>
-      </c>
-      <c r="I223" s="18">
+      <c r="A223" s="37">
+        <v>45670</v>
+      </c>
+      <c r="B223" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="C223" s="39" t="s">
+        <v>318</v>
+      </c>
+      <c r="D223" s="38" t="s">
+        <v>317</v>
+      </c>
+      <c r="E223" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F223" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="G223" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H223" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="I223" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J223" s="19"/>
-      <c r="K223" s="46"/>
-    </row>
-    <row r="224" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A224" s="62" t="s">
-        <v>26</v>
-      </c>
-      <c r="B224" s="63"/>
-      <c r="C224" s="63"/>
-      <c r="D224" s="63"/>
-      <c r="E224" s="63"/>
-      <c r="F224" s="63"/>
-      <c r="G224" s="63"/>
-      <c r="H224" s="63"/>
-      <c r="I224" s="63"/>
-      <c r="J224" s="63"/>
-      <c r="K224" s="64"/>
+      <c r="J223" s="45"/>
+      <c r="K223" s="43"/>
+    </row>
+    <row r="224" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A224" s="37">
+        <v>45670</v>
+      </c>
+      <c r="B224" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="C224" s="39" t="s">
+        <v>320</v>
+      </c>
+      <c r="D224" s="38" t="s">
+        <v>319</v>
+      </c>
+      <c r="E224" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="F224" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="G224" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="H224" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="I224" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J224" s="45"/>
+      <c r="K224" s="43"/>
     </row>
     <row r="225" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A225" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B225" s="65" t="s">
-        <v>13</v>
-      </c>
-      <c r="C225" s="63"/>
-      <c r="D225" s="63"/>
-      <c r="E225" s="63"/>
-      <c r="F225" s="63"/>
-      <c r="G225" s="63"/>
-      <c r="H225" s="63"/>
-      <c r="I225" s="63"/>
-      <c r="J225" s="63"/>
-      <c r="K225" s="64"/>
-    </row>
-    <row r="226" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A226" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B226" s="65" t="s">
-        <v>15</v>
-      </c>
-      <c r="C226" s="63"/>
-      <c r="D226" s="63"/>
-      <c r="E226" s="63"/>
-      <c r="F226" s="63"/>
-      <c r="G226" s="63"/>
-      <c r="H226" s="63"/>
-      <c r="I226" s="63"/>
-      <c r="J226" s="63"/>
-      <c r="K226" s="64"/>
+      <c r="A225" s="37">
+        <v>45671</v>
+      </c>
+      <c r="B225" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="C225" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="D225" s="38" t="s">
+        <v>266</v>
+      </c>
+      <c r="E225" s="40" t="s">
+        <v>61</v>
+      </c>
+      <c r="F225" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="G225" s="41">
+        <v>0.15</v>
+      </c>
+      <c r="H225" s="41">
+        <v>0.15</v>
+      </c>
+      <c r="I225" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J225" s="45"/>
+      <c r="K225" s="43"/>
+    </row>
+    <row r="226" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A226" s="37">
+        <v>45671</v>
+      </c>
+      <c r="B226" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="C226" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="D226" s="38" t="s">
+        <v>287</v>
+      </c>
+      <c r="E226" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="F226" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="G226" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H226" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="I226" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J226" s="45"/>
+      <c r="K226" s="43"/>
     </row>
     <row r="227" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A227" s="37"/>
-      <c r="B227" s="38"/>
+      <c r="A227" s="37">
+        <v>45671</v>
+      </c>
+      <c r="B227" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C227" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D227" s="38"/>
-      <c r="E227" s="40"/>
-      <c r="F227" s="40"/>
-      <c r="G227" s="41"/>
-      <c r="H227" s="41"/>
+        <v>333</v>
+      </c>
+      <c r="D227" s="38" t="s">
+        <v>332</v>
+      </c>
+      <c r="E227" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F227" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="G227" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H227" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I227" s="41">
-        <f t="shared" ref="I227:I237" si="11">H227-G227</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J227" s="45"/>
@@ -8830,83 +8972,84 @@
       <c r="G228" s="41"/>
       <c r="H228" s="41"/>
       <c r="I228" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J228" s="45"/>
       <c r="K228" s="43"/>
     </row>
     <row r="229" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A229" s="37"/>
-      <c r="B229" s="38"/>
-      <c r="C229" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D229" s="38"/>
-      <c r="E229" s="40"/>
-      <c r="F229" s="40"/>
-      <c r="G229" s="41"/>
-      <c r="H229" s="41"/>
-      <c r="I229" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J229" s="45"/>
-      <c r="K229" s="43"/>
-    </row>
-    <row r="230" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A230" s="37"/>
-      <c r="B230" s="38"/>
-      <c r="C230" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D230" s="38"/>
-      <c r="E230" s="40"/>
-      <c r="F230" s="40"/>
-      <c r="G230" s="41"/>
-      <c r="H230" s="41"/>
-      <c r="I230" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J230" s="45"/>
-      <c r="K230" s="43"/>
+      <c r="A229" s="13"/>
+      <c r="B229" s="15"/>
+      <c r="C229" s="15"/>
+      <c r="D229" s="15"/>
+      <c r="E229" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F229" s="15"/>
+      <c r="G229" s="18">
+        <f t="shared" ref="G229:H229" si="10">SUM(G219:G228)</f>
+        <v>3</v>
+      </c>
+      <c r="H229" s="18">
+        <f t="shared" si="10"/>
+        <v>3</v>
+      </c>
+      <c r="I229" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J229" s="19"/>
+      <c r="K229" s="46"/>
+    </row>
+    <row r="230" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A230" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="B230" s="55"/>
+      <c r="C230" s="55"/>
+      <c r="D230" s="55"/>
+      <c r="E230" s="55"/>
+      <c r="F230" s="55"/>
+      <c r="G230" s="55"/>
+      <c r="H230" s="55"/>
+      <c r="I230" s="55"/>
+      <c r="J230" s="55"/>
+      <c r="K230" s="56"/>
     </row>
     <row r="231" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A231" s="37"/>
-      <c r="B231" s="38"/>
-      <c r="C231" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D231" s="38"/>
-      <c r="E231" s="40"/>
-      <c r="F231" s="40"/>
-      <c r="G231" s="41"/>
-      <c r="H231" s="41"/>
-      <c r="I231" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J231" s="45"/>
-      <c r="K231" s="43"/>
-    </row>
-    <row r="232" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A232" s="37"/>
-      <c r="B232" s="38"/>
-      <c r="C232" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D232" s="38"/>
-      <c r="E232" s="40"/>
-      <c r="F232" s="40"/>
-      <c r="G232" s="41"/>
-      <c r="H232" s="41"/>
-      <c r="I232" s="41">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J232" s="45"/>
-      <c r="K232" s="43"/>
+      <c r="A231" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B231" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C231" s="55"/>
+      <c r="D231" s="55"/>
+      <c r="E231" s="55"/>
+      <c r="F231" s="55"/>
+      <c r="G231" s="55"/>
+      <c r="H231" s="55"/>
+      <c r="I231" s="55"/>
+      <c r="J231" s="55"/>
+      <c r="K231" s="56"/>
+    </row>
+    <row r="232" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A232" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B232" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C232" s="55"/>
+      <c r="D232" s="55"/>
+      <c r="E232" s="55"/>
+      <c r="F232" s="55"/>
+      <c r="G232" s="55"/>
+      <c r="H232" s="55"/>
+      <c r="I232" s="55"/>
+      <c r="J232" s="55"/>
+      <c r="K232" s="56"/>
     </row>
     <row r="233" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A233" s="37"/>
@@ -8920,7 +9063,7 @@
       <c r="G233" s="41"/>
       <c r="H233" s="41"/>
       <c r="I233" s="41">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="I233:I243" si="11">H233-G233</f>
         <v>0</v>
       </c>
       <c r="J233" s="45"/>
@@ -8981,35 +9124,143 @@
       <c r="K236" s="43"/>
     </row>
     <row r="237" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A237" s="48"/>
-      <c r="B237" s="49"/>
-      <c r="C237" s="49"/>
-      <c r="D237" s="49"/>
-      <c r="E237" s="49" t="s">
+      <c r="A237" s="37"/>
+      <c r="B237" s="38"/>
+      <c r="C237" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D237" s="38"/>
+      <c r="E237" s="40"/>
+      <c r="F237" s="40"/>
+      <c r="G237" s="41"/>
+      <c r="H237" s="41"/>
+      <c r="I237" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J237" s="45"/>
+      <c r="K237" s="43"/>
+    </row>
+    <row r="238" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A238" s="37"/>
+      <c r="B238" s="38"/>
+      <c r="C238" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D238" s="38"/>
+      <c r="E238" s="40"/>
+      <c r="F238" s="40"/>
+      <c r="G238" s="41"/>
+      <c r="H238" s="41"/>
+      <c r="I238" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J238" s="45"/>
+      <c r="K238" s="43"/>
+    </row>
+    <row r="239" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A239" s="37"/>
+      <c r="B239" s="38"/>
+      <c r="C239" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D239" s="38"/>
+      <c r="E239" s="40"/>
+      <c r="F239" s="40"/>
+      <c r="G239" s="41"/>
+      <c r="H239" s="41"/>
+      <c r="I239" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J239" s="45"/>
+      <c r="K239" s="43"/>
+    </row>
+    <row r="240" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A240" s="37"/>
+      <c r="B240" s="38"/>
+      <c r="C240" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D240" s="38"/>
+      <c r="E240" s="40"/>
+      <c r="F240" s="40"/>
+      <c r="G240" s="41"/>
+      <c r="H240" s="41"/>
+      <c r="I240" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J240" s="45"/>
+      <c r="K240" s="43"/>
+    </row>
+    <row r="241" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A241" s="37"/>
+      <c r="B241" s="38"/>
+      <c r="C241" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D241" s="38"/>
+      <c r="E241" s="40"/>
+      <c r="F241" s="40"/>
+      <c r="G241" s="41"/>
+      <c r="H241" s="41"/>
+      <c r="I241" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J241" s="45"/>
+      <c r="K241" s="43"/>
+    </row>
+    <row r="242" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A242" s="37"/>
+      <c r="B242" s="38"/>
+      <c r="C242" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D242" s="38"/>
+      <c r="E242" s="40"/>
+      <c r="F242" s="40"/>
+      <c r="G242" s="41"/>
+      <c r="H242" s="41"/>
+      <c r="I242" s="41">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J242" s="45"/>
+      <c r="K242" s="43"/>
+    </row>
+    <row r="243" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A243" s="48"/>
+      <c r="B243" s="49"/>
+      <c r="C243" s="49"/>
+      <c r="D243" s="49"/>
+      <c r="E243" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F237" s="49"/>
-      <c r="G237" s="50">
-        <f t="shared" ref="G237:H237" si="12">SUM(G227:G236)</f>
-        <v>0</v>
-      </c>
-      <c r="H237" s="50">
+      <c r="F243" s="49"/>
+      <c r="G243" s="50">
+        <f t="shared" ref="G243:H243" si="12">SUM(G233:G242)</f>
+        <v>0</v>
+      </c>
+      <c r="H243" s="50">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="I237" s="50">
+      <c r="I243" s="50">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J237" s="51"/>
-      <c r="K237" s="52"/>
+      <c r="J243" s="51"/>
+      <c r="K243" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{EFD0DA2C-85A2-41CD-9897-E6AD670C26ED}">
+      <autoFilter ref="A1:K15" xr:uid="{DD83653E-2878-4270-B2F3-7C093852FF55}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -9020,9 +9271,17 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="A224:K224"/>
-    <mergeCell ref="B225:K225"/>
-    <mergeCell ref="B226:K226"/>
+    <mergeCell ref="B196:K196"/>
+    <mergeCell ref="B197:K197"/>
+    <mergeCell ref="A216:K216"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A195:K195"/>
+    <mergeCell ref="A230:K230"/>
+    <mergeCell ref="B231:K231"/>
+    <mergeCell ref="B232:K232"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B4:K4"/>
@@ -9033,19 +9292,11 @@
     <mergeCell ref="B84:K84"/>
     <mergeCell ref="B85:K85"/>
     <mergeCell ref="A118:K118"/>
-    <mergeCell ref="B211:K211"/>
-    <mergeCell ref="B212:K212"/>
+    <mergeCell ref="B217:K217"/>
+    <mergeCell ref="B218:K218"/>
     <mergeCell ref="B119:K119"/>
-    <mergeCell ref="B196:K196"/>
-    <mergeCell ref="B197:K197"/>
-    <mergeCell ref="A210:K210"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A195:K195"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B193 B198:B208 B213:B222">
+  <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B193 B198:B214 B219:B228">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -9062,7 +9313,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B152:B194 B196:B209 B211:B223 B225:B237">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B150 B152:B194 B196:B215 B217:B229 B231:B243">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -9070,34 +9321,34 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B227:B236">
+  <conditionalFormatting sqref="B233:B242">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
-      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B227))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B233))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH(("Planned"),(B227))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Planned"),(B233))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B227))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("In-Progress"),(B233))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B227))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Blocked"),(B233))))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Done">
-      <formula>NOT(ISERROR(SEARCH(("Done"),(B227))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("Done"),(B233))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G154:G194 G198:G209 G213:G223 G227:G237">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G150 G154:G194 G198:G215 G219:G229 G233:G243">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H237">
+  <conditionalFormatting sqref="H1:H243">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I154:I194 I198:I209 I213:I223 I227:I237">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I150 I154:I194 I198:I215 I219:I229 I233:I243">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -9106,7 +9357,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F227:F236 F213:F222 F86:F116 F198:F208 F5:F45 F50:F81 F121:F149 F154:F193" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F233:F242 F219:F228 F86:F116 F198:F214 F5:F45 F50:F81 F121:F149 F154:F193" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9122,13 +9373,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E116 E198:E208 E213:E222 E227:E236 E50:E81 E121:E149 E154:E193</xm:sqref>
+          <xm:sqref>E5:E45 E86:E116 E198:E214 E219:E228 E233:E242 E50:E81 E121:E149 E154:E193</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B116 B198:B208 B213:B222 B227:B236 B50:B81 B121:B149 B154:B193</xm:sqref>
+          <xm:sqref>B5:B45 B86:B116 B198:B214 B219:B228 B233:B242 B50:B81 B121:B149 B154:B193</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -10769,26 +11020,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -11023,10 +11254,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11043,20 +11305,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W7 DataLab 1 Work IV (Post-Break)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57EB2914-3E63-49CC-A556-B91CA4402C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8D10EE-9CD4-4E21-A9DB-AEDEB4349A9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1139" uniqueCount="336">
   <si>
     <t>Date</t>
   </si>
@@ -1104,6 +1104,12 @@
   </si>
   <si>
     <t>Block A Evidencing</t>
+  </si>
+  <si>
+    <t>https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/dbf52b5262095348a7b3b20dff20823b21fc03fb/Block%20B/Gradient%20Descent%20With%20Momentum%20from%20Scratch%20Program.ipynb</t>
+  </si>
+  <si>
+    <t>start at 13:00</t>
   </si>
 </sst>
 </file>
@@ -1589,6 +1595,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1605,8 +1631,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1624,24 +1648,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2166,53 +2172,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3551,53 +3557,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4650,53 +4656,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5711,53 +5717,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="68" t="s">
+      <c r="A118" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="62"/>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
+      <c r="B118" s="55"/>
+      <c r="C118" s="55"/>
+      <c r="D118" s="55"/>
+      <c r="E118" s="55"/>
+      <c r="F118" s="55"/>
+      <c r="G118" s="55"/>
+      <c r="H118" s="55"/>
+      <c r="I118" s="55"/>
+      <c r="J118" s="55"/>
+      <c r="K118" s="56"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="70" t="s">
+      <c r="B119" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="62"/>
-      <c r="D119" s="62"/>
-      <c r="E119" s="62"/>
-      <c r="F119" s="62"/>
-      <c r="G119" s="62"/>
-      <c r="H119" s="62"/>
-      <c r="I119" s="62"/>
-      <c r="J119" s="62"/>
-      <c r="K119" s="63"/>
+      <c r="C119" s="55"/>
+      <c r="D119" s="55"/>
+      <c r="E119" s="55"/>
+      <c r="F119" s="55"/>
+      <c r="G119" s="55"/>
+      <c r="H119" s="55"/>
+      <c r="I119" s="55"/>
+      <c r="J119" s="55"/>
+      <c r="K119" s="56"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="70" t="s">
+      <c r="B120" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="62"/>
-      <c r="D120" s="62"/>
-      <c r="E120" s="62"/>
-      <c r="F120" s="62"/>
-      <c r="G120" s="62"/>
-      <c r="H120" s="62"/>
-      <c r="I120" s="62"/>
-      <c r="J120" s="62"/>
-      <c r="K120" s="63"/>
+      <c r="C120" s="55"/>
+      <c r="D120" s="55"/>
+      <c r="E120" s="55"/>
+      <c r="F120" s="55"/>
+      <c r="G120" s="55"/>
+      <c r="H120" s="55"/>
+      <c r="I120" s="55"/>
+      <c r="J120" s="55"/>
+      <c r="K120" s="56"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6694,53 +6700,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="73" t="s">
+      <c r="A151" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="62"/>
-      <c r="C151" s="62"/>
-      <c r="D151" s="62"/>
-      <c r="E151" s="62"/>
-      <c r="F151" s="62"/>
-      <c r="G151" s="62"/>
-      <c r="H151" s="62"/>
-      <c r="I151" s="62"/>
-      <c r="J151" s="62"/>
-      <c r="K151" s="63"/>
+      <c r="B151" s="55"/>
+      <c r="C151" s="55"/>
+      <c r="D151" s="55"/>
+      <c r="E151" s="55"/>
+      <c r="F151" s="55"/>
+      <c r="G151" s="55"/>
+      <c r="H151" s="55"/>
+      <c r="I151" s="55"/>
+      <c r="J151" s="55"/>
+      <c r="K151" s="56"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="74" t="s">
+      <c r="B152" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="62"/>
-      <c r="D152" s="62"/>
-      <c r="E152" s="62"/>
-      <c r="F152" s="62"/>
-      <c r="G152" s="62"/>
-      <c r="H152" s="62"/>
-      <c r="I152" s="62"/>
-      <c r="J152" s="62"/>
-      <c r="K152" s="63"/>
+      <c r="C152" s="55"/>
+      <c r="D152" s="55"/>
+      <c r="E152" s="55"/>
+      <c r="F152" s="55"/>
+      <c r="G152" s="55"/>
+      <c r="H152" s="55"/>
+      <c r="I152" s="55"/>
+      <c r="J152" s="55"/>
+      <c r="K152" s="56"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="74" t="s">
+      <c r="B153" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="62"/>
-      <c r="D153" s="62"/>
-      <c r="E153" s="62"/>
-      <c r="F153" s="62"/>
-      <c r="G153" s="62"/>
-      <c r="H153" s="62"/>
-      <c r="I153" s="62"/>
-      <c r="J153" s="62"/>
-      <c r="K153" s="63"/>
+      <c r="C153" s="55"/>
+      <c r="D153" s="55"/>
+      <c r="E153" s="55"/>
+      <c r="F153" s="55"/>
+      <c r="G153" s="55"/>
+      <c r="H153" s="55"/>
+      <c r="I153" s="55"/>
+      <c r="J153" s="55"/>
+      <c r="K153" s="56"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -8037,53 +8043,53 @@
       <c r="K194" s="46"/>
     </row>
     <row r="195" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="75" t="s">
+      <c r="A195" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B195" s="62"/>
-      <c r="C195" s="62"/>
-      <c r="D195" s="62"/>
-      <c r="E195" s="62"/>
-      <c r="F195" s="62"/>
-      <c r="G195" s="62"/>
-      <c r="H195" s="62"/>
-      <c r="I195" s="62"/>
-      <c r="J195" s="62"/>
-      <c r="K195" s="63"/>
+      <c r="B195" s="55"/>
+      <c r="C195" s="55"/>
+      <c r="D195" s="55"/>
+      <c r="E195" s="55"/>
+      <c r="F195" s="55"/>
+      <c r="G195" s="55"/>
+      <c r="H195" s="55"/>
+      <c r="I195" s="55"/>
+      <c r="J195" s="55"/>
+      <c r="K195" s="56"/>
     </row>
     <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A196" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B196" s="71" t="s">
+      <c r="B196" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C196" s="62"/>
-      <c r="D196" s="62"/>
-      <c r="E196" s="62"/>
-      <c r="F196" s="62"/>
-      <c r="G196" s="62"/>
-      <c r="H196" s="62"/>
-      <c r="I196" s="62"/>
-      <c r="J196" s="62"/>
-      <c r="K196" s="63"/>
+      <c r="C196" s="55"/>
+      <c r="D196" s="55"/>
+      <c r="E196" s="55"/>
+      <c r="F196" s="55"/>
+      <c r="G196" s="55"/>
+      <c r="H196" s="55"/>
+      <c r="I196" s="55"/>
+      <c r="J196" s="55"/>
+      <c r="K196" s="56"/>
     </row>
     <row r="197" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B197" s="71" t="s">
+      <c r="B197" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C197" s="62"/>
-      <c r="D197" s="62"/>
-      <c r="E197" s="62"/>
-      <c r="F197" s="62"/>
-      <c r="G197" s="62"/>
-      <c r="H197" s="62"/>
-      <c r="I197" s="62"/>
-      <c r="J197" s="62"/>
-      <c r="K197" s="63"/>
+      <c r="C197" s="55"/>
+      <c r="D197" s="55"/>
+      <c r="E197" s="55"/>
+      <c r="F197" s="55"/>
+      <c r="G197" s="55"/>
+      <c r="H197" s="55"/>
+      <c r="I197" s="55"/>
+      <c r="J197" s="55"/>
+      <c r="K197" s="56"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="37">
@@ -8428,7 +8434,9 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J208" s="45"/>
+      <c r="J208" s="53" t="s">
+        <v>334</v>
+      </c>
       <c r="K208" s="43"/>
     </row>
     <row r="209" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -8436,7 +8444,7 @@
         <v>45671</v>
       </c>
       <c r="B209" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C209" s="39" t="s">
         <v>325</v>
@@ -8453,10 +8461,12 @@
       <c r="G209" s="41">
         <v>1</v>
       </c>
-      <c r="H209" s="41"/>
+      <c r="H209" s="41">
+        <v>1</v>
+      </c>
       <c r="I209" s="41">
         <f t="shared" si="7"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J209" s="45"/>
       <c r="K209" s="43"/>
@@ -8466,7 +8476,7 @@
         <v>45671</v>
       </c>
       <c r="B210" s="38" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C210" s="39" t="s">
         <v>325</v>
@@ -8483,10 +8493,12 @@
       <c r="G210" s="41">
         <v>1</v>
       </c>
-      <c r="H210" s="41"/>
+      <c r="H210" s="41">
+        <v>1</v>
+      </c>
       <c r="I210" s="41">
         <f t="shared" si="7"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J210" s="45"/>
       <c r="K210" s="43"/>
@@ -8496,7 +8508,7 @@
         <v>45671</v>
       </c>
       <c r="B211" s="38" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C211" s="39" t="s">
         <v>325</v>
@@ -8519,7 +8531,9 @@
         <v>-1</v>
       </c>
       <c r="J211" s="45"/>
-      <c r="K211" s="43"/>
+      <c r="K211" s="43" t="s">
+        <v>335</v>
+      </c>
     </row>
     <row r="212" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A212" s="37">
@@ -8614,63 +8628,63 @@
       </c>
       <c r="H215" s="18">
         <f t="shared" si="8"/>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I215" s="18">
         <f t="shared" si="7"/>
-        <v>-15.25</v>
+        <v>-13.25</v>
       </c>
       <c r="J215" s="19"/>
       <c r="K215" s="46"/>
     </row>
     <row r="216" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A216" s="72" t="s">
+      <c r="A216" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="B216" s="62"/>
-      <c r="C216" s="62"/>
-      <c r="D216" s="62"/>
-      <c r="E216" s="62"/>
-      <c r="F216" s="62"/>
-      <c r="G216" s="62"/>
-      <c r="H216" s="62"/>
-      <c r="I216" s="62"/>
-      <c r="J216" s="62"/>
-      <c r="K216" s="63"/>
+      <c r="B216" s="55"/>
+      <c r="C216" s="55"/>
+      <c r="D216" s="55"/>
+      <c r="E216" s="55"/>
+      <c r="F216" s="55"/>
+      <c r="G216" s="55"/>
+      <c r="H216" s="55"/>
+      <c r="I216" s="55"/>
+      <c r="J216" s="55"/>
+      <c r="K216" s="56"/>
     </row>
     <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A217" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B217" s="69" t="s">
+      <c r="B217" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C217" s="62"/>
-      <c r="D217" s="62"/>
-      <c r="E217" s="62"/>
-      <c r="F217" s="62"/>
-      <c r="G217" s="62"/>
-      <c r="H217" s="62"/>
-      <c r="I217" s="62"/>
-      <c r="J217" s="62"/>
-      <c r="K217" s="63"/>
+      <c r="C217" s="55"/>
+      <c r="D217" s="55"/>
+      <c r="E217" s="55"/>
+      <c r="F217" s="55"/>
+      <c r="G217" s="55"/>
+      <c r="H217" s="55"/>
+      <c r="I217" s="55"/>
+      <c r="J217" s="55"/>
+      <c r="K217" s="56"/>
     </row>
     <row r="218" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B218" s="69" t="s">
+      <c r="B218" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C218" s="62"/>
-      <c r="D218" s="62"/>
-      <c r="E218" s="62"/>
-      <c r="F218" s="62"/>
-      <c r="G218" s="62"/>
-      <c r="H218" s="62"/>
-      <c r="I218" s="62"/>
-      <c r="J218" s="62"/>
-      <c r="K218" s="63"/>
+      <c r="C218" s="55"/>
+      <c r="D218" s="55"/>
+      <c r="E218" s="55"/>
+      <c r="F218" s="55"/>
+      <c r="G218" s="55"/>
+      <c r="H218" s="55"/>
+      <c r="I218" s="55"/>
+      <c r="J218" s="55"/>
+      <c r="K218" s="56"/>
     </row>
     <row r="219" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A219" s="37">
@@ -9003,53 +9017,53 @@
       <c r="K229" s="46"/>
     </row>
     <row r="230" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A230" s="54" t="s">
+      <c r="A230" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="B230" s="55"/>
-      <c r="C230" s="55"/>
-      <c r="D230" s="55"/>
-      <c r="E230" s="55"/>
-      <c r="F230" s="55"/>
-      <c r="G230" s="55"/>
-      <c r="H230" s="55"/>
-      <c r="I230" s="55"/>
-      <c r="J230" s="55"/>
-      <c r="K230" s="56"/>
+      <c r="B230" s="63"/>
+      <c r="C230" s="63"/>
+      <c r="D230" s="63"/>
+      <c r="E230" s="63"/>
+      <c r="F230" s="63"/>
+      <c r="G230" s="63"/>
+      <c r="H230" s="63"/>
+      <c r="I230" s="63"/>
+      <c r="J230" s="63"/>
+      <c r="K230" s="64"/>
     </row>
     <row r="231" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A231" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B231" s="57" t="s">
+      <c r="B231" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C231" s="55"/>
-      <c r="D231" s="55"/>
-      <c r="E231" s="55"/>
-      <c r="F231" s="55"/>
-      <c r="G231" s="55"/>
-      <c r="H231" s="55"/>
-      <c r="I231" s="55"/>
-      <c r="J231" s="55"/>
-      <c r="K231" s="56"/>
+      <c r="C231" s="63"/>
+      <c r="D231" s="63"/>
+      <c r="E231" s="63"/>
+      <c r="F231" s="63"/>
+      <c r="G231" s="63"/>
+      <c r="H231" s="63"/>
+      <c r="I231" s="63"/>
+      <c r="J231" s="63"/>
+      <c r="K231" s="64"/>
     </row>
     <row r="232" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B232" s="57" t="s">
+      <c r="B232" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C232" s="55"/>
-      <c r="D232" s="55"/>
-      <c r="E232" s="55"/>
-      <c r="F232" s="55"/>
-      <c r="G232" s="55"/>
-      <c r="H232" s="55"/>
-      <c r="I232" s="55"/>
-      <c r="J232" s="55"/>
-      <c r="K232" s="56"/>
+      <c r="C232" s="63"/>
+      <c r="D232" s="63"/>
+      <c r="E232" s="63"/>
+      <c r="F232" s="63"/>
+      <c r="G232" s="63"/>
+      <c r="H232" s="63"/>
+      <c r="I232" s="63"/>
+      <c r="J232" s="63"/>
+      <c r="K232" s="64"/>
     </row>
     <row r="233" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A233" s="37"/>
@@ -9260,7 +9274,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{DD83653E-2878-4270-B2F3-7C093852FF55}">
+      <autoFilter ref="A1:K15" xr:uid="{31E37D5F-FC0E-474C-A508-4E46DF4C8456}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -9271,14 +9285,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B196:K196"/>
-    <mergeCell ref="B197:K197"/>
-    <mergeCell ref="A216:K216"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A195:K195"/>
     <mergeCell ref="A230:K230"/>
     <mergeCell ref="B231:K231"/>
     <mergeCell ref="B232:K232"/>
@@ -9295,6 +9301,14 @@
     <mergeCell ref="B217:K217"/>
     <mergeCell ref="B218:K218"/>
     <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B196:K196"/>
+    <mergeCell ref="B197:K197"/>
+    <mergeCell ref="A216:K216"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A195:K195"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B193 B198:B214 B219:B228">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -9363,9 +9377,10 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="J29" r:id="rId1" xr:uid="{0999D960-5356-4EE8-BA28-70F36BB764AC}"/>
+    <hyperlink ref="J208" r:id="rId2" xr:uid="{6C2E871F-AE23-4B7F-AE67-E54AFFFB2865}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -11020,6 +11035,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -11254,27 +11289,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11291,23 +11325,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W7 DataLab 1 Work V (Post Assignment 1)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8D10EE-9CD4-4E21-A9DB-AEDEB4349A9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01921536-D2D0-402E-B0AE-F067CF12A8AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1139" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="338">
   <si>
     <t>Date</t>
   </si>
@@ -1109,7 +1109,13 @@
     <t>https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/dbf52b5262095348a7b3b20dff20823b21fc03fb/Block%20B/Gradient%20Descent%20With%20Momentum%20from%20Scratch%20Program.ipynb</t>
   </si>
   <si>
-    <t>start at 13:00</t>
+    <t>Slow work after a break during the datalab.</t>
+  </si>
+  <si>
+    <t>I had the material fresh in my head so I did it quite quickly.</t>
+  </si>
+  <si>
+    <t>start at 15:30</t>
   </si>
 </sst>
 </file>
@@ -1595,26 +1601,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1631,6 +1617,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1648,6 +1636,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2172,53 +2178,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3557,53 +3563,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="62"/>
+      <c r="K49" s="63"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4656,53 +4662,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72" t="s">
+      <c r="A83" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="55"/>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="55"/>
-      <c r="I83" s="55"/>
-      <c r="J83" s="55"/>
-      <c r="K83" s="56"/>
+      <c r="B83" s="62"/>
+      <c r="C83" s="62"/>
+      <c r="D83" s="62"/>
+      <c r="E83" s="62"/>
+      <c r="F83" s="62"/>
+      <c r="G83" s="62"/>
+      <c r="H83" s="62"/>
+      <c r="I83" s="62"/>
+      <c r="J83" s="62"/>
+      <c r="K83" s="63"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="73" t="s">
+      <c r="B84" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="55"/>
-      <c r="D84" s="55"/>
-      <c r="E84" s="55"/>
-      <c r="F84" s="55"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="55"/>
-      <c r="I84" s="55"/>
-      <c r="J84" s="55"/>
-      <c r="K84" s="56"/>
+      <c r="C84" s="62"/>
+      <c r="D84" s="62"/>
+      <c r="E84" s="62"/>
+      <c r="F84" s="62"/>
+      <c r="G84" s="62"/>
+      <c r="H84" s="62"/>
+      <c r="I84" s="62"/>
+      <c r="J84" s="62"/>
+      <c r="K84" s="63"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="73" t="s">
+      <c r="B85" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="55"/>
-      <c r="D85" s="55"/>
-      <c r="E85" s="55"/>
-      <c r="F85" s="55"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="55"/>
-      <c r="I85" s="55"/>
-      <c r="J85" s="55"/>
-      <c r="K85" s="56"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="62"/>
+      <c r="G85" s="62"/>
+      <c r="H85" s="62"/>
+      <c r="I85" s="62"/>
+      <c r="J85" s="62"/>
+      <c r="K85" s="63"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5717,53 +5723,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="74" t="s">
+      <c r="A118" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="55"/>
-      <c r="C118" s="55"/>
-      <c r="D118" s="55"/>
-      <c r="E118" s="55"/>
-      <c r="F118" s="55"/>
-      <c r="G118" s="55"/>
-      <c r="H118" s="55"/>
-      <c r="I118" s="55"/>
-      <c r="J118" s="55"/>
-      <c r="K118" s="56"/>
+      <c r="B118" s="62"/>
+      <c r="C118" s="62"/>
+      <c r="D118" s="62"/>
+      <c r="E118" s="62"/>
+      <c r="F118" s="62"/>
+      <c r="G118" s="62"/>
+      <c r="H118" s="62"/>
+      <c r="I118" s="62"/>
+      <c r="J118" s="62"/>
+      <c r="K118" s="63"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="58" t="s">
+      <c r="B119" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="55"/>
-      <c r="D119" s="55"/>
-      <c r="E119" s="55"/>
-      <c r="F119" s="55"/>
-      <c r="G119" s="55"/>
-      <c r="H119" s="55"/>
-      <c r="I119" s="55"/>
-      <c r="J119" s="55"/>
-      <c r="K119" s="56"/>
+      <c r="C119" s="62"/>
+      <c r="D119" s="62"/>
+      <c r="E119" s="62"/>
+      <c r="F119" s="62"/>
+      <c r="G119" s="62"/>
+      <c r="H119" s="62"/>
+      <c r="I119" s="62"/>
+      <c r="J119" s="62"/>
+      <c r="K119" s="63"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="58" t="s">
+      <c r="B120" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="55"/>
-      <c r="D120" s="55"/>
-      <c r="E120" s="55"/>
-      <c r="F120" s="55"/>
-      <c r="G120" s="55"/>
-      <c r="H120" s="55"/>
-      <c r="I120" s="55"/>
-      <c r="J120" s="55"/>
-      <c r="K120" s="56"/>
+      <c r="C120" s="62"/>
+      <c r="D120" s="62"/>
+      <c r="E120" s="62"/>
+      <c r="F120" s="62"/>
+      <c r="G120" s="62"/>
+      <c r="H120" s="62"/>
+      <c r="I120" s="62"/>
+      <c r="J120" s="62"/>
+      <c r="K120" s="63"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6700,53 +6706,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="59" t="s">
+      <c r="A151" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="55"/>
-      <c r="C151" s="55"/>
-      <c r="D151" s="55"/>
-      <c r="E151" s="55"/>
-      <c r="F151" s="55"/>
-      <c r="G151" s="55"/>
-      <c r="H151" s="55"/>
-      <c r="I151" s="55"/>
-      <c r="J151" s="55"/>
-      <c r="K151" s="56"/>
+      <c r="B151" s="62"/>
+      <c r="C151" s="62"/>
+      <c r="D151" s="62"/>
+      <c r="E151" s="62"/>
+      <c r="F151" s="62"/>
+      <c r="G151" s="62"/>
+      <c r="H151" s="62"/>
+      <c r="I151" s="62"/>
+      <c r="J151" s="62"/>
+      <c r="K151" s="63"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="60" t="s">
+      <c r="B152" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="55"/>
-      <c r="D152" s="55"/>
-      <c r="E152" s="55"/>
-      <c r="F152" s="55"/>
-      <c r="G152" s="55"/>
-      <c r="H152" s="55"/>
-      <c r="I152" s="55"/>
-      <c r="J152" s="55"/>
-      <c r="K152" s="56"/>
+      <c r="C152" s="62"/>
+      <c r="D152" s="62"/>
+      <c r="E152" s="62"/>
+      <c r="F152" s="62"/>
+      <c r="G152" s="62"/>
+      <c r="H152" s="62"/>
+      <c r="I152" s="62"/>
+      <c r="J152" s="62"/>
+      <c r="K152" s="63"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="60" t="s">
+      <c r="B153" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="55"/>
-      <c r="D153" s="55"/>
-      <c r="E153" s="55"/>
-      <c r="F153" s="55"/>
-      <c r="G153" s="55"/>
-      <c r="H153" s="55"/>
-      <c r="I153" s="55"/>
-      <c r="J153" s="55"/>
-      <c r="K153" s="56"/>
+      <c r="C153" s="62"/>
+      <c r="D153" s="62"/>
+      <c r="E153" s="62"/>
+      <c r="F153" s="62"/>
+      <c r="G153" s="62"/>
+      <c r="H153" s="62"/>
+      <c r="I153" s="62"/>
+      <c r="J153" s="62"/>
+      <c r="K153" s="63"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -8043,53 +8049,53 @@
       <c r="K194" s="46"/>
     </row>
     <row r="195" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="61" t="s">
+      <c r="A195" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B195" s="55"/>
-      <c r="C195" s="55"/>
-      <c r="D195" s="55"/>
-      <c r="E195" s="55"/>
-      <c r="F195" s="55"/>
-      <c r="G195" s="55"/>
-      <c r="H195" s="55"/>
-      <c r="I195" s="55"/>
-      <c r="J195" s="55"/>
-      <c r="K195" s="56"/>
+      <c r="B195" s="62"/>
+      <c r="C195" s="62"/>
+      <c r="D195" s="62"/>
+      <c r="E195" s="62"/>
+      <c r="F195" s="62"/>
+      <c r="G195" s="62"/>
+      <c r="H195" s="62"/>
+      <c r="I195" s="62"/>
+      <c r="J195" s="62"/>
+      <c r="K195" s="63"/>
     </row>
     <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A196" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B196" s="54" t="s">
+      <c r="B196" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C196" s="55"/>
-      <c r="D196" s="55"/>
-      <c r="E196" s="55"/>
-      <c r="F196" s="55"/>
-      <c r="G196" s="55"/>
-      <c r="H196" s="55"/>
-      <c r="I196" s="55"/>
-      <c r="J196" s="55"/>
-      <c r="K196" s="56"/>
+      <c r="C196" s="62"/>
+      <c r="D196" s="62"/>
+      <c r="E196" s="62"/>
+      <c r="F196" s="62"/>
+      <c r="G196" s="62"/>
+      <c r="H196" s="62"/>
+      <c r="I196" s="62"/>
+      <c r="J196" s="62"/>
+      <c r="K196" s="63"/>
     </row>
     <row r="197" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B197" s="54" t="s">
+      <c r="B197" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C197" s="55"/>
-      <c r="D197" s="55"/>
-      <c r="E197" s="55"/>
-      <c r="F197" s="55"/>
-      <c r="G197" s="55"/>
-      <c r="H197" s="55"/>
-      <c r="I197" s="55"/>
-      <c r="J197" s="55"/>
-      <c r="K197" s="56"/>
+      <c r="C197" s="62"/>
+      <c r="D197" s="62"/>
+      <c r="E197" s="62"/>
+      <c r="F197" s="62"/>
+      <c r="G197" s="62"/>
+      <c r="H197" s="62"/>
+      <c r="I197" s="62"/>
+      <c r="J197" s="62"/>
+      <c r="K197" s="63"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="37">
@@ -8508,7 +8514,7 @@
         <v>45671</v>
       </c>
       <c r="B211" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C211" s="39" t="s">
         <v>325</v>
@@ -8525,10 +8531,12 @@
       <c r="G211" s="41">
         <v>1</v>
       </c>
-      <c r="H211" s="41"/>
+      <c r="H211" s="41">
+        <v>2</v>
+      </c>
       <c r="I211" s="41">
         <f t="shared" si="7"/>
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="J211" s="45"/>
       <c r="K211" s="43" t="s">
@@ -8540,7 +8548,7 @@
         <v>45671</v>
       </c>
       <c r="B212" s="38" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C212" s="39" t="s">
         <v>325</v>
@@ -8555,22 +8563,26 @@
         <v>104</v>
       </c>
       <c r="G212" s="41">
-        <v>2</v>
-      </c>
-      <c r="H212" s="41"/>
+        <v>1</v>
+      </c>
+      <c r="H212" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I212" s="41">
         <f t="shared" si="7"/>
-        <v>-2</v>
+        <v>-0.5</v>
       </c>
       <c r="J212" s="45"/>
-      <c r="K212" s="43"/>
+      <c r="K212" s="43" t="s">
+        <v>336</v>
+      </c>
     </row>
     <row r="213" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A213" s="37">
         <v>45671</v>
       </c>
       <c r="B213" s="38" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C213" s="39" t="s">
         <v>325</v>
@@ -8593,7 +8605,9 @@
         <v>-2</v>
       </c>
       <c r="J213" s="45"/>
-      <c r="K213" s="43"/>
+      <c r="K213" s="43" t="s">
+        <v>337</v>
+      </c>
     </row>
     <row r="214" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A214" s="37"/>
@@ -8624,67 +8638,67 @@
       <c r="F215" s="15"/>
       <c r="G215" s="18">
         <f t="shared" ref="G215:H215" si="8">SUM(G198:G214)</f>
-        <v>30.25</v>
+        <v>29.25</v>
       </c>
       <c r="H215" s="18">
         <f t="shared" si="8"/>
-        <v>17</v>
+        <v>19.5</v>
       </c>
       <c r="I215" s="18">
         <f t="shared" si="7"/>
-        <v>-13.25</v>
+        <v>-9.75</v>
       </c>
       <c r="J215" s="19"/>
       <c r="K215" s="46"/>
     </row>
     <row r="216" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A216" s="57" t="s">
+      <c r="A216" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="B216" s="55"/>
-      <c r="C216" s="55"/>
-      <c r="D216" s="55"/>
-      <c r="E216" s="55"/>
-      <c r="F216" s="55"/>
-      <c r="G216" s="55"/>
-      <c r="H216" s="55"/>
-      <c r="I216" s="55"/>
-      <c r="J216" s="55"/>
-      <c r="K216" s="56"/>
+      <c r="B216" s="62"/>
+      <c r="C216" s="62"/>
+      <c r="D216" s="62"/>
+      <c r="E216" s="62"/>
+      <c r="F216" s="62"/>
+      <c r="G216" s="62"/>
+      <c r="H216" s="62"/>
+      <c r="I216" s="62"/>
+      <c r="J216" s="62"/>
+      <c r="K216" s="63"/>
     </row>
     <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A217" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B217" s="75" t="s">
+      <c r="B217" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C217" s="55"/>
-      <c r="D217" s="55"/>
-      <c r="E217" s="55"/>
-      <c r="F217" s="55"/>
-      <c r="G217" s="55"/>
-      <c r="H217" s="55"/>
-      <c r="I217" s="55"/>
-      <c r="J217" s="55"/>
-      <c r="K217" s="56"/>
+      <c r="C217" s="62"/>
+      <c r="D217" s="62"/>
+      <c r="E217" s="62"/>
+      <c r="F217" s="62"/>
+      <c r="G217" s="62"/>
+      <c r="H217" s="62"/>
+      <c r="I217" s="62"/>
+      <c r="J217" s="62"/>
+      <c r="K217" s="63"/>
     </row>
     <row r="218" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B218" s="75" t="s">
+      <c r="B218" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C218" s="55"/>
-      <c r="D218" s="55"/>
-      <c r="E218" s="55"/>
-      <c r="F218" s="55"/>
-      <c r="G218" s="55"/>
-      <c r="H218" s="55"/>
-      <c r="I218" s="55"/>
-      <c r="J218" s="55"/>
-      <c r="K218" s="56"/>
+      <c r="C218" s="62"/>
+      <c r="D218" s="62"/>
+      <c r="E218" s="62"/>
+      <c r="F218" s="62"/>
+      <c r="G218" s="62"/>
+      <c r="H218" s="62"/>
+      <c r="I218" s="62"/>
+      <c r="J218" s="62"/>
+      <c r="K218" s="63"/>
     </row>
     <row r="219" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A219" s="37">
@@ -9017,53 +9031,53 @@
       <c r="K229" s="46"/>
     </row>
     <row r="230" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A230" s="62" t="s">
+      <c r="A230" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="B230" s="63"/>
-      <c r="C230" s="63"/>
-      <c r="D230" s="63"/>
-      <c r="E230" s="63"/>
-      <c r="F230" s="63"/>
-      <c r="G230" s="63"/>
-      <c r="H230" s="63"/>
-      <c r="I230" s="63"/>
-      <c r="J230" s="63"/>
-      <c r="K230" s="64"/>
+      <c r="B230" s="55"/>
+      <c r="C230" s="55"/>
+      <c r="D230" s="55"/>
+      <c r="E230" s="55"/>
+      <c r="F230" s="55"/>
+      <c r="G230" s="55"/>
+      <c r="H230" s="55"/>
+      <c r="I230" s="55"/>
+      <c r="J230" s="55"/>
+      <c r="K230" s="56"/>
     </row>
     <row r="231" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A231" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B231" s="65" t="s">
+      <c r="B231" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C231" s="63"/>
-      <c r="D231" s="63"/>
-      <c r="E231" s="63"/>
-      <c r="F231" s="63"/>
-      <c r="G231" s="63"/>
-      <c r="H231" s="63"/>
-      <c r="I231" s="63"/>
-      <c r="J231" s="63"/>
-      <c r="K231" s="64"/>
+      <c r="C231" s="55"/>
+      <c r="D231" s="55"/>
+      <c r="E231" s="55"/>
+      <c r="F231" s="55"/>
+      <c r="G231" s="55"/>
+      <c r="H231" s="55"/>
+      <c r="I231" s="55"/>
+      <c r="J231" s="55"/>
+      <c r="K231" s="56"/>
     </row>
     <row r="232" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B232" s="65" t="s">
+      <c r="B232" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C232" s="63"/>
-      <c r="D232" s="63"/>
-      <c r="E232" s="63"/>
-      <c r="F232" s="63"/>
-      <c r="G232" s="63"/>
-      <c r="H232" s="63"/>
-      <c r="I232" s="63"/>
-      <c r="J232" s="63"/>
-      <c r="K232" s="64"/>
+      <c r="C232" s="55"/>
+      <c r="D232" s="55"/>
+      <c r="E232" s="55"/>
+      <c r="F232" s="55"/>
+      <c r="G232" s="55"/>
+      <c r="H232" s="55"/>
+      <c r="I232" s="55"/>
+      <c r="J232" s="55"/>
+      <c r="K232" s="56"/>
     </row>
     <row r="233" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A233" s="37"/>
@@ -9274,7 +9288,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{31E37D5F-FC0E-474C-A508-4E46DF4C8456}">
+      <autoFilter ref="A1:K15" xr:uid="{2E277F2C-D3D1-4F1B-98F1-00ADF10F2A5F}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -9285,6 +9299,14 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
+    <mergeCell ref="B196:K196"/>
+    <mergeCell ref="B197:K197"/>
+    <mergeCell ref="A216:K216"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A195:K195"/>
     <mergeCell ref="A230:K230"/>
     <mergeCell ref="B231:K231"/>
     <mergeCell ref="B232:K232"/>
@@ -9301,14 +9323,6 @@
     <mergeCell ref="B217:K217"/>
     <mergeCell ref="B218:K218"/>
     <mergeCell ref="B119:K119"/>
-    <mergeCell ref="B196:K196"/>
-    <mergeCell ref="B197:K197"/>
-    <mergeCell ref="A216:K216"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A195:K195"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B193 B198:B214 B219:B228">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -11035,26 +11049,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -11289,10 +11283,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11309,20 +11334,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W7 DataLab 1 Work VI (END)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01921536-D2D0-402E-B0AE-F067CF12A8AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2266E3E3-79D0-411A-B9A8-3BB11A1F9C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1115,7 +1115,7 @@
     <t>I had the material fresh in my head so I did it quite quickly.</t>
   </si>
   <si>
-    <t>start at 15:30</t>
+    <t>1,5 at 17:00</t>
   </si>
 </sst>
 </file>
@@ -1601,6 +1601,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1617,8 +1637,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1636,24 +1654,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2178,53 +2178,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3563,53 +3563,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4662,53 +4662,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5723,53 +5723,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="68" t="s">
+      <c r="A118" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="62"/>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
+      <c r="B118" s="55"/>
+      <c r="C118" s="55"/>
+      <c r="D118" s="55"/>
+      <c r="E118" s="55"/>
+      <c r="F118" s="55"/>
+      <c r="G118" s="55"/>
+      <c r="H118" s="55"/>
+      <c r="I118" s="55"/>
+      <c r="J118" s="55"/>
+      <c r="K118" s="56"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="70" t="s">
+      <c r="B119" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="62"/>
-      <c r="D119" s="62"/>
-      <c r="E119" s="62"/>
-      <c r="F119" s="62"/>
-      <c r="G119" s="62"/>
-      <c r="H119" s="62"/>
-      <c r="I119" s="62"/>
-      <c r="J119" s="62"/>
-      <c r="K119" s="63"/>
+      <c r="C119" s="55"/>
+      <c r="D119" s="55"/>
+      <c r="E119" s="55"/>
+      <c r="F119" s="55"/>
+      <c r="G119" s="55"/>
+      <c r="H119" s="55"/>
+      <c r="I119" s="55"/>
+      <c r="J119" s="55"/>
+      <c r="K119" s="56"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="70" t="s">
+      <c r="B120" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="62"/>
-      <c r="D120" s="62"/>
-      <c r="E120" s="62"/>
-      <c r="F120" s="62"/>
-      <c r="G120" s="62"/>
-      <c r="H120" s="62"/>
-      <c r="I120" s="62"/>
-      <c r="J120" s="62"/>
-      <c r="K120" s="63"/>
+      <c r="C120" s="55"/>
+      <c r="D120" s="55"/>
+      <c r="E120" s="55"/>
+      <c r="F120" s="55"/>
+      <c r="G120" s="55"/>
+      <c r="H120" s="55"/>
+      <c r="I120" s="55"/>
+      <c r="J120" s="55"/>
+      <c r="K120" s="56"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6706,53 +6706,53 @@
       <c r="K150" s="46"/>
     </row>
     <row r="151" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="73" t="s">
+      <c r="A151" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B151" s="62"/>
-      <c r="C151" s="62"/>
-      <c r="D151" s="62"/>
-      <c r="E151" s="62"/>
-      <c r="F151" s="62"/>
-      <c r="G151" s="62"/>
-      <c r="H151" s="62"/>
-      <c r="I151" s="62"/>
-      <c r="J151" s="62"/>
-      <c r="K151" s="63"/>
+      <c r="B151" s="55"/>
+      <c r="C151" s="55"/>
+      <c r="D151" s="55"/>
+      <c r="E151" s="55"/>
+      <c r="F151" s="55"/>
+      <c r="G151" s="55"/>
+      <c r="H151" s="55"/>
+      <c r="I151" s="55"/>
+      <c r="J151" s="55"/>
+      <c r="K151" s="56"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B152" s="74" t="s">
+      <c r="B152" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C152" s="62"/>
-      <c r="D152" s="62"/>
-      <c r="E152" s="62"/>
-      <c r="F152" s="62"/>
-      <c r="G152" s="62"/>
-      <c r="H152" s="62"/>
-      <c r="I152" s="62"/>
-      <c r="J152" s="62"/>
-      <c r="K152" s="63"/>
+      <c r="C152" s="55"/>
+      <c r="D152" s="55"/>
+      <c r="E152" s="55"/>
+      <c r="F152" s="55"/>
+      <c r="G152" s="55"/>
+      <c r="H152" s="55"/>
+      <c r="I152" s="55"/>
+      <c r="J152" s="55"/>
+      <c r="K152" s="56"/>
     </row>
     <row r="153" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B153" s="74" t="s">
+      <c r="B153" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="62"/>
-      <c r="D153" s="62"/>
-      <c r="E153" s="62"/>
-      <c r="F153" s="62"/>
-      <c r="G153" s="62"/>
-      <c r="H153" s="62"/>
-      <c r="I153" s="62"/>
-      <c r="J153" s="62"/>
-      <c r="K153" s="63"/>
+      <c r="C153" s="55"/>
+      <c r="D153" s="55"/>
+      <c r="E153" s="55"/>
+      <c r="F153" s="55"/>
+      <c r="G153" s="55"/>
+      <c r="H153" s="55"/>
+      <c r="I153" s="55"/>
+      <c r="J153" s="55"/>
+      <c r="K153" s="56"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="37">
@@ -8049,53 +8049,53 @@
       <c r="K194" s="46"/>
     </row>
     <row r="195" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="75" t="s">
+      <c r="A195" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B195" s="62"/>
-      <c r="C195" s="62"/>
-      <c r="D195" s="62"/>
-      <c r="E195" s="62"/>
-      <c r="F195" s="62"/>
-      <c r="G195" s="62"/>
-      <c r="H195" s="62"/>
-      <c r="I195" s="62"/>
-      <c r="J195" s="62"/>
-      <c r="K195" s="63"/>
+      <c r="B195" s="55"/>
+      <c r="C195" s="55"/>
+      <c r="D195" s="55"/>
+      <c r="E195" s="55"/>
+      <c r="F195" s="55"/>
+      <c r="G195" s="55"/>
+      <c r="H195" s="55"/>
+      <c r="I195" s="55"/>
+      <c r="J195" s="55"/>
+      <c r="K195" s="56"/>
     </row>
     <row r="196" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A196" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B196" s="71" t="s">
+      <c r="B196" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C196" s="62"/>
-      <c r="D196" s="62"/>
-      <c r="E196" s="62"/>
-      <c r="F196" s="62"/>
-      <c r="G196" s="62"/>
-      <c r="H196" s="62"/>
-      <c r="I196" s="62"/>
-      <c r="J196" s="62"/>
-      <c r="K196" s="63"/>
+      <c r="C196" s="55"/>
+      <c r="D196" s="55"/>
+      <c r="E196" s="55"/>
+      <c r="F196" s="55"/>
+      <c r="G196" s="55"/>
+      <c r="H196" s="55"/>
+      <c r="I196" s="55"/>
+      <c r="J196" s="55"/>
+      <c r="K196" s="56"/>
     </row>
     <row r="197" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B197" s="71" t="s">
+      <c r="B197" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C197" s="62"/>
-      <c r="D197" s="62"/>
-      <c r="E197" s="62"/>
-      <c r="F197" s="62"/>
-      <c r="G197" s="62"/>
-      <c r="H197" s="62"/>
-      <c r="I197" s="62"/>
-      <c r="J197" s="62"/>
-      <c r="K197" s="63"/>
+      <c r="C197" s="55"/>
+      <c r="D197" s="55"/>
+      <c r="E197" s="55"/>
+      <c r="F197" s="55"/>
+      <c r="G197" s="55"/>
+      <c r="H197" s="55"/>
+      <c r="I197" s="55"/>
+      <c r="J197" s="55"/>
+      <c r="K197" s="56"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="37">
@@ -8652,53 +8652,53 @@
       <c r="K215" s="46"/>
     </row>
     <row r="216" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A216" s="72" t="s">
+      <c r="A216" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="B216" s="62"/>
-      <c r="C216" s="62"/>
-      <c r="D216" s="62"/>
-      <c r="E216" s="62"/>
-      <c r="F216" s="62"/>
-      <c r="G216" s="62"/>
-      <c r="H216" s="62"/>
-      <c r="I216" s="62"/>
-      <c r="J216" s="62"/>
-      <c r="K216" s="63"/>
+      <c r="B216" s="55"/>
+      <c r="C216" s="55"/>
+      <c r="D216" s="55"/>
+      <c r="E216" s="55"/>
+      <c r="F216" s="55"/>
+      <c r="G216" s="55"/>
+      <c r="H216" s="55"/>
+      <c r="I216" s="55"/>
+      <c r="J216" s="55"/>
+      <c r="K216" s="56"/>
     </row>
     <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A217" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B217" s="69" t="s">
+      <c r="B217" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C217" s="62"/>
-      <c r="D217" s="62"/>
-      <c r="E217" s="62"/>
-      <c r="F217" s="62"/>
-      <c r="G217" s="62"/>
-      <c r="H217" s="62"/>
-      <c r="I217" s="62"/>
-      <c r="J217" s="62"/>
-      <c r="K217" s="63"/>
+      <c r="C217" s="55"/>
+      <c r="D217" s="55"/>
+      <c r="E217" s="55"/>
+      <c r="F217" s="55"/>
+      <c r="G217" s="55"/>
+      <c r="H217" s="55"/>
+      <c r="I217" s="55"/>
+      <c r="J217" s="55"/>
+      <c r="K217" s="56"/>
     </row>
     <row r="218" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B218" s="69" t="s">
+      <c r="B218" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C218" s="62"/>
-      <c r="D218" s="62"/>
-      <c r="E218" s="62"/>
-      <c r="F218" s="62"/>
-      <c r="G218" s="62"/>
-      <c r="H218" s="62"/>
-      <c r="I218" s="62"/>
-      <c r="J218" s="62"/>
-      <c r="K218" s="63"/>
+      <c r="C218" s="55"/>
+      <c r="D218" s="55"/>
+      <c r="E218" s="55"/>
+      <c r="F218" s="55"/>
+      <c r="G218" s="55"/>
+      <c r="H218" s="55"/>
+      <c r="I218" s="55"/>
+      <c r="J218" s="55"/>
+      <c r="K218" s="56"/>
     </row>
     <row r="219" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A219" s="37">
@@ -9031,53 +9031,53 @@
       <c r="K229" s="46"/>
     </row>
     <row r="230" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A230" s="54" t="s">
+      <c r="A230" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="B230" s="55"/>
-      <c r="C230" s="55"/>
-      <c r="D230" s="55"/>
-      <c r="E230" s="55"/>
-      <c r="F230" s="55"/>
-      <c r="G230" s="55"/>
-      <c r="H230" s="55"/>
-      <c r="I230" s="55"/>
-      <c r="J230" s="55"/>
-      <c r="K230" s="56"/>
+      <c r="B230" s="63"/>
+      <c r="C230" s="63"/>
+      <c r="D230" s="63"/>
+      <c r="E230" s="63"/>
+      <c r="F230" s="63"/>
+      <c r="G230" s="63"/>
+      <c r="H230" s="63"/>
+      <c r="I230" s="63"/>
+      <c r="J230" s="63"/>
+      <c r="K230" s="64"/>
     </row>
     <row r="231" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A231" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B231" s="57" t="s">
+      <c r="B231" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C231" s="55"/>
-      <c r="D231" s="55"/>
-      <c r="E231" s="55"/>
-      <c r="F231" s="55"/>
-      <c r="G231" s="55"/>
-      <c r="H231" s="55"/>
-      <c r="I231" s="55"/>
-      <c r="J231" s="55"/>
-      <c r="K231" s="56"/>
+      <c r="C231" s="63"/>
+      <c r="D231" s="63"/>
+      <c r="E231" s="63"/>
+      <c r="F231" s="63"/>
+      <c r="G231" s="63"/>
+      <c r="H231" s="63"/>
+      <c r="I231" s="63"/>
+      <c r="J231" s="63"/>
+      <c r="K231" s="64"/>
     </row>
     <row r="232" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B232" s="57" t="s">
+      <c r="B232" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C232" s="55"/>
-      <c r="D232" s="55"/>
-      <c r="E232" s="55"/>
-      <c r="F232" s="55"/>
-      <c r="G232" s="55"/>
-      <c r="H232" s="55"/>
-      <c r="I232" s="55"/>
-      <c r="J232" s="55"/>
-      <c r="K232" s="56"/>
+      <c r="C232" s="63"/>
+      <c r="D232" s="63"/>
+      <c r="E232" s="63"/>
+      <c r="F232" s="63"/>
+      <c r="G232" s="63"/>
+      <c r="H232" s="63"/>
+      <c r="I232" s="63"/>
+      <c r="J232" s="63"/>
+      <c r="K232" s="64"/>
     </row>
     <row r="233" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A233" s="37"/>
@@ -9288,7 +9288,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{2E277F2C-D3D1-4F1B-98F1-00ADF10F2A5F}">
+      <autoFilter ref="A1:K15" xr:uid="{6B0E91C2-4BB1-40A1-9A34-C7496E3ACB01}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -9299,14 +9299,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B196:K196"/>
-    <mergeCell ref="B197:K197"/>
-    <mergeCell ref="A216:K216"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A151:K151"/>
-    <mergeCell ref="B152:K152"/>
-    <mergeCell ref="B153:K153"/>
-    <mergeCell ref="A195:K195"/>
     <mergeCell ref="A230:K230"/>
     <mergeCell ref="B231:K231"/>
     <mergeCell ref="B232:K232"/>
@@ -9323,6 +9315,14 @@
     <mergeCell ref="B217:K217"/>
     <mergeCell ref="B218:K218"/>
     <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B196:K196"/>
+    <mergeCell ref="B197:K197"/>
+    <mergeCell ref="A216:K216"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A151:K151"/>
+    <mergeCell ref="B152:K152"/>
+    <mergeCell ref="B153:K153"/>
+    <mergeCell ref="A195:K195"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B149 B154:B193 B198:B214 B219:B228">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -11049,6 +11049,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -11283,27 +11303,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11320,23 +11339,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W8 DataLab 1 Work I (Start)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D7737C4-7F45-4895-AF18-E22EEE5E9DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388BE7D2-C6B0-43CF-B7DE-F128F8BD0CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="369">
   <si>
     <t>Date</t>
   </si>
@@ -1177,6 +1177,39 @@
   <si>
     <t>I somehow missed this when catching up in week 7, so I did it later.</t>
   </si>
+  <si>
+    <t>Finish Learning Log Block A</t>
+  </si>
+  <si>
+    <t>Hand in Block A retake</t>
+  </si>
+  <si>
+    <t>Begin work on presentation</t>
+  </si>
+  <si>
+    <t>Fill in WorkLog for Monday &amp; Tuesday</t>
+  </si>
+  <si>
+    <t>Work on Creative Brief</t>
+  </si>
+  <si>
+    <t>Final Presentation</t>
+  </si>
+  <si>
+    <t>Send e-mail regarding errors</t>
+  </si>
+  <si>
+    <t>Finish Jupyter notebooks Logistical &amp; Linear Regression</t>
+  </si>
+  <si>
+    <t>Continue work on presentation</t>
+  </si>
+  <si>
+    <t>ILO 11.1</t>
+  </si>
+  <si>
+    <t>Finishing touches to SMARTER-goals</t>
+  </si>
 </sst>
 </file>
 
@@ -1187,7 +1220,7 @@
     <numFmt numFmtId="165" formatCode="d&quot;-&quot;mmm&quot;-&quot;yyyy"/>
     <numFmt numFmtId="166" formatCode="d/m/yy"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1273,6 +1306,12 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="15">
@@ -1510,7 +1549,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1661,6 +1700,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1677,8 +1736,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1697,24 +1754,6 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1722,6 +1761,10 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2186,7 +2229,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K257"/>
+  <dimension ref="A1:K261"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -2238,53 +2281,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="60"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="63"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3623,53 +3666,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="59"/>
-      <c r="J47" s="59"/>
-      <c r="K47" s="60"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="67"/>
+      <c r="F47" s="67"/>
+      <c r="G47" s="67"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="67"/>
+      <c r="J47" s="67"/>
+      <c r="K47" s="68"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="63"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="65" t="s">
+      <c r="B49" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="63"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="55"/>
+      <c r="J49" s="55"/>
+      <c r="K49" s="56"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4720,53 +4763,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="66" t="s">
+      <c r="A83" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="62"/>
-      <c r="C83" s="62"/>
-      <c r="D83" s="62"/>
-      <c r="E83" s="62"/>
-      <c r="F83" s="62"/>
-      <c r="G83" s="62"/>
-      <c r="H83" s="62"/>
-      <c r="I83" s="62"/>
-      <c r="J83" s="62"/>
-      <c r="K83" s="63"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="55"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="55"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="55"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="55"/>
+      <c r="J83" s="55"/>
+      <c r="K83" s="56"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="67" t="s">
+      <c r="B84" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="62"/>
-      <c r="D84" s="62"/>
-      <c r="E84" s="62"/>
-      <c r="F84" s="62"/>
-      <c r="G84" s="62"/>
-      <c r="H84" s="62"/>
-      <c r="I84" s="62"/>
-      <c r="J84" s="62"/>
-      <c r="K84" s="63"/>
+      <c r="C84" s="55"/>
+      <c r="D84" s="55"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="55"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="55"/>
+      <c r="J84" s="55"/>
+      <c r="K84" s="56"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="67" t="s">
+      <c r="B85" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="62"/>
-      <c r="D85" s="62"/>
-      <c r="E85" s="62"/>
-      <c r="F85" s="62"/>
-      <c r="G85" s="62"/>
-      <c r="H85" s="62"/>
-      <c r="I85" s="62"/>
-      <c r="J85" s="62"/>
-      <c r="K85" s="63"/>
+      <c r="C85" s="55"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="55"/>
+      <c r="F85" s="55"/>
+      <c r="G85" s="55"/>
+      <c r="H85" s="55"/>
+      <c r="I85" s="55"/>
+      <c r="J85" s="55"/>
+      <c r="K85" s="56"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5781,53 +5824,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="68" t="s">
+      <c r="A118" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="62"/>
-      <c r="C118" s="62"/>
-      <c r="D118" s="62"/>
-      <c r="E118" s="62"/>
-      <c r="F118" s="62"/>
-      <c r="G118" s="62"/>
-      <c r="H118" s="62"/>
-      <c r="I118" s="62"/>
-      <c r="J118" s="62"/>
-      <c r="K118" s="63"/>
+      <c r="B118" s="55"/>
+      <c r="C118" s="55"/>
+      <c r="D118" s="55"/>
+      <c r="E118" s="55"/>
+      <c r="F118" s="55"/>
+      <c r="G118" s="55"/>
+      <c r="H118" s="55"/>
+      <c r="I118" s="55"/>
+      <c r="J118" s="55"/>
+      <c r="K118" s="56"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="70" t="s">
+      <c r="B119" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="62"/>
-      <c r="D119" s="62"/>
-      <c r="E119" s="62"/>
-      <c r="F119" s="62"/>
-      <c r="G119" s="62"/>
-      <c r="H119" s="62"/>
-      <c r="I119" s="62"/>
-      <c r="J119" s="62"/>
-      <c r="K119" s="63"/>
+      <c r="C119" s="55"/>
+      <c r="D119" s="55"/>
+      <c r="E119" s="55"/>
+      <c r="F119" s="55"/>
+      <c r="G119" s="55"/>
+      <c r="H119" s="55"/>
+      <c r="I119" s="55"/>
+      <c r="J119" s="55"/>
+      <c r="K119" s="56"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="70" t="s">
+      <c r="B120" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="62"/>
-      <c r="D120" s="62"/>
-      <c r="E120" s="62"/>
-      <c r="F120" s="62"/>
-      <c r="G120" s="62"/>
-      <c r="H120" s="62"/>
-      <c r="I120" s="62"/>
-      <c r="J120" s="62"/>
-      <c r="K120" s="63"/>
+      <c r="C120" s="55"/>
+      <c r="D120" s="55"/>
+      <c r="E120" s="55"/>
+      <c r="F120" s="55"/>
+      <c r="G120" s="55"/>
+      <c r="H120" s="55"/>
+      <c r="I120" s="55"/>
+      <c r="J120" s="55"/>
+      <c r="K120" s="56"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6820,53 +6863,53 @@
       <c r="K152" s="46"/>
     </row>
     <row r="153" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="73" t="s">
+      <c r="A153" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B153" s="62"/>
-      <c r="C153" s="62"/>
-      <c r="D153" s="62"/>
-      <c r="E153" s="62"/>
-      <c r="F153" s="62"/>
-      <c r="G153" s="62"/>
-      <c r="H153" s="62"/>
-      <c r="I153" s="62"/>
-      <c r="J153" s="62"/>
-      <c r="K153" s="63"/>
+      <c r="B153" s="55"/>
+      <c r="C153" s="55"/>
+      <c r="D153" s="55"/>
+      <c r="E153" s="55"/>
+      <c r="F153" s="55"/>
+      <c r="G153" s="55"/>
+      <c r="H153" s="55"/>
+      <c r="I153" s="55"/>
+      <c r="J153" s="55"/>
+      <c r="K153" s="56"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B154" s="74" t="s">
+      <c r="B154" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C154" s="62"/>
-      <c r="D154" s="62"/>
-      <c r="E154" s="62"/>
-      <c r="F154" s="62"/>
-      <c r="G154" s="62"/>
-      <c r="H154" s="62"/>
-      <c r="I154" s="62"/>
-      <c r="J154" s="62"/>
-      <c r="K154" s="63"/>
+      <c r="C154" s="55"/>
+      <c r="D154" s="55"/>
+      <c r="E154" s="55"/>
+      <c r="F154" s="55"/>
+      <c r="G154" s="55"/>
+      <c r="H154" s="55"/>
+      <c r="I154" s="55"/>
+      <c r="J154" s="55"/>
+      <c r="K154" s="56"/>
     </row>
     <row r="155" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B155" s="74" t="s">
+      <c r="B155" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C155" s="62"/>
-      <c r="D155" s="62"/>
-      <c r="E155" s="62"/>
-      <c r="F155" s="62"/>
-      <c r="G155" s="62"/>
-      <c r="H155" s="62"/>
-      <c r="I155" s="62"/>
-      <c r="J155" s="62"/>
-      <c r="K155" s="63"/>
+      <c r="C155" s="55"/>
+      <c r="D155" s="55"/>
+      <c r="E155" s="55"/>
+      <c r="F155" s="55"/>
+      <c r="G155" s="55"/>
+      <c r="H155" s="55"/>
+      <c r="I155" s="55"/>
+      <c r="J155" s="55"/>
+      <c r="K155" s="56"/>
     </row>
     <row r="156" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A156" s="37">
@@ -8163,53 +8206,53 @@
       <c r="K196" s="46"/>
     </row>
     <row r="197" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A197" s="75" t="s">
+      <c r="A197" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="B197" s="62"/>
-      <c r="C197" s="62"/>
-      <c r="D197" s="62"/>
-      <c r="E197" s="62"/>
-      <c r="F197" s="62"/>
-      <c r="G197" s="62"/>
-      <c r="H197" s="62"/>
-      <c r="I197" s="62"/>
-      <c r="J197" s="62"/>
-      <c r="K197" s="63"/>
+      <c r="B197" s="55"/>
+      <c r="C197" s="55"/>
+      <c r="D197" s="55"/>
+      <c r="E197" s="55"/>
+      <c r="F197" s="55"/>
+      <c r="G197" s="55"/>
+      <c r="H197" s="55"/>
+      <c r="I197" s="55"/>
+      <c r="J197" s="55"/>
+      <c r="K197" s="56"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B198" s="71" t="s">
+      <c r="B198" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="C198" s="62"/>
-      <c r="D198" s="62"/>
-      <c r="E198" s="62"/>
-      <c r="F198" s="62"/>
-      <c r="G198" s="62"/>
-      <c r="H198" s="62"/>
-      <c r="I198" s="62"/>
-      <c r="J198" s="62"/>
-      <c r="K198" s="63"/>
+      <c r="C198" s="55"/>
+      <c r="D198" s="55"/>
+      <c r="E198" s="55"/>
+      <c r="F198" s="55"/>
+      <c r="G198" s="55"/>
+      <c r="H198" s="55"/>
+      <c r="I198" s="55"/>
+      <c r="J198" s="55"/>
+      <c r="K198" s="56"/>
     </row>
     <row r="199" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B199" s="71" t="s">
+      <c r="B199" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C199" s="62"/>
-      <c r="D199" s="62"/>
-      <c r="E199" s="62"/>
-      <c r="F199" s="62"/>
-      <c r="G199" s="62"/>
-      <c r="H199" s="62"/>
-      <c r="I199" s="62"/>
-      <c r="J199" s="62"/>
-      <c r="K199" s="63"/>
+      <c r="C199" s="55"/>
+      <c r="D199" s="55"/>
+      <c r="E199" s="55"/>
+      <c r="F199" s="55"/>
+      <c r="G199" s="55"/>
+      <c r="H199" s="55"/>
+      <c r="I199" s="55"/>
+      <c r="J199" s="55"/>
+      <c r="K199" s="56"/>
     </row>
     <row r="200" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A200" s="37">
@@ -8835,53 +8878,53 @@
       <c r="K219" s="46"/>
     </row>
     <row r="220" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A220" s="72" t="s">
+      <c r="A220" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="B220" s="62"/>
-      <c r="C220" s="62"/>
-      <c r="D220" s="62"/>
-      <c r="E220" s="62"/>
-      <c r="F220" s="62"/>
-      <c r="G220" s="62"/>
-      <c r="H220" s="62"/>
-      <c r="I220" s="62"/>
-      <c r="J220" s="62"/>
-      <c r="K220" s="63"/>
+      <c r="B220" s="55"/>
+      <c r="C220" s="55"/>
+      <c r="D220" s="55"/>
+      <c r="E220" s="55"/>
+      <c r="F220" s="55"/>
+      <c r="G220" s="55"/>
+      <c r="H220" s="55"/>
+      <c r="I220" s="55"/>
+      <c r="J220" s="55"/>
+      <c r="K220" s="56"/>
     </row>
     <row r="221" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A221" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B221" s="69" t="s">
+      <c r="B221" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C221" s="62"/>
-      <c r="D221" s="62"/>
-      <c r="E221" s="62"/>
-      <c r="F221" s="62"/>
-      <c r="G221" s="62"/>
-      <c r="H221" s="62"/>
-      <c r="I221" s="62"/>
-      <c r="J221" s="62"/>
-      <c r="K221" s="63"/>
+      <c r="C221" s="55"/>
+      <c r="D221" s="55"/>
+      <c r="E221" s="55"/>
+      <c r="F221" s="55"/>
+      <c r="G221" s="55"/>
+      <c r="H221" s="55"/>
+      <c r="I221" s="55"/>
+      <c r="J221" s="55"/>
+      <c r="K221" s="56"/>
     </row>
     <row r="222" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B222" s="69" t="s">
+      <c r="B222" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C222" s="62"/>
-      <c r="D222" s="62"/>
-      <c r="E222" s="62"/>
-      <c r="F222" s="62"/>
-      <c r="G222" s="62"/>
-      <c r="H222" s="62"/>
-      <c r="I222" s="62"/>
-      <c r="J222" s="62"/>
-      <c r="K222" s="63"/>
+      <c r="C222" s="55"/>
+      <c r="D222" s="55"/>
+      <c r="E222" s="55"/>
+      <c r="F222" s="55"/>
+      <c r="G222" s="55"/>
+      <c r="H222" s="55"/>
+      <c r="I222" s="55"/>
+      <c r="J222" s="55"/>
+      <c r="K222" s="56"/>
     </row>
     <row r="223" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A223" s="37">
@@ -9253,10 +9296,12 @@
       <c r="G234" s="41">
         <v>0.25</v>
       </c>
-      <c r="H234" s="41"/>
+      <c r="H234" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I234" s="41">
         <f t="shared" si="8"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J234" s="45"/>
       <c r="K234" s="43"/>
@@ -9283,10 +9328,12 @@
       <c r="G235" s="41">
         <v>0.25</v>
       </c>
-      <c r="H235" s="41"/>
+      <c r="H235" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I235" s="41">
         <f t="shared" si="8"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J235" s="45"/>
       <c r="K235" s="43"/>
@@ -9313,10 +9360,12 @@
       <c r="G236" s="41">
         <v>0.5</v>
       </c>
-      <c r="H236" s="41"/>
+      <c r="H236" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I236" s="41">
         <f t="shared" si="8"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="J236" s="45"/>
       <c r="K236" s="43"/>
@@ -9343,10 +9392,12 @@
       <c r="G237" s="41">
         <v>1</v>
       </c>
-      <c r="H237" s="41"/>
+      <c r="H237" s="41">
+        <v>1</v>
+      </c>
       <c r="I237" s="41">
         <f t="shared" si="8"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J237" s="45"/>
       <c r="K237" s="43"/>
@@ -9422,7 +9473,7 @@
         <v>45676</v>
       </c>
       <c r="B240" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C240" s="39" t="s">
         <v>206</v>
@@ -9439,10 +9490,12 @@
       <c r="G240" s="41">
         <v>1</v>
       </c>
-      <c r="H240" s="41"/>
+      <c r="H240" s="41">
+        <v>1</v>
+      </c>
       <c r="I240" s="41">
         <f t="shared" si="8"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J240" s="45"/>
       <c r="K240" s="43"/>
@@ -9518,93 +9571,121 @@
       </c>
       <c r="H243" s="18">
         <f>SUM(H223:H242)</f>
-        <v>7.5</v>
+        <v>10.5</v>
       </c>
       <c r="I243" s="18">
         <f t="shared" si="8"/>
-        <v>-13</v>
+        <v>-10</v>
       </c>
       <c r="J243" s="19"/>
       <c r="K243" s="46"/>
     </row>
     <row r="244" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A244" s="54" t="s">
+      <c r="A244" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="B244" s="55"/>
-      <c r="C244" s="55"/>
-      <c r="D244" s="55"/>
-      <c r="E244" s="55"/>
-      <c r="F244" s="55"/>
-      <c r="G244" s="55"/>
-      <c r="H244" s="55"/>
-      <c r="I244" s="55"/>
-      <c r="J244" s="55"/>
-      <c r="K244" s="56"/>
+      <c r="B244" s="63"/>
+      <c r="C244" s="63"/>
+      <c r="D244" s="63"/>
+      <c r="E244" s="63"/>
+      <c r="F244" s="63"/>
+      <c r="G244" s="63"/>
+      <c r="H244" s="63"/>
+      <c r="I244" s="63"/>
+      <c r="J244" s="63"/>
+      <c r="K244" s="64"/>
     </row>
     <row r="245" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A245" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B245" s="57" t="s">
+      <c r="B245" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C245" s="55"/>
-      <c r="D245" s="55"/>
-      <c r="E245" s="55"/>
-      <c r="F245" s="55"/>
-      <c r="G245" s="55"/>
-      <c r="H245" s="55"/>
-      <c r="I245" s="55"/>
-      <c r="J245" s="55"/>
-      <c r="K245" s="56"/>
+      <c r="C245" s="63"/>
+      <c r="D245" s="63"/>
+      <c r="E245" s="63"/>
+      <c r="F245" s="63"/>
+      <c r="G245" s="63"/>
+      <c r="H245" s="63"/>
+      <c r="I245" s="63"/>
+      <c r="J245" s="63"/>
+      <c r="K245" s="64"/>
     </row>
     <row r="246" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A246" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B246" s="57" t="s">
+      <c r="B246" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C246" s="55"/>
-      <c r="D246" s="55"/>
-      <c r="E246" s="55"/>
-      <c r="F246" s="55"/>
-      <c r="G246" s="55"/>
-      <c r="H246" s="55"/>
-      <c r="I246" s="55"/>
-      <c r="J246" s="55"/>
-      <c r="K246" s="56"/>
+      <c r="C246" s="63"/>
+      <c r="D246" s="63"/>
+      <c r="E246" s="63"/>
+      <c r="F246" s="63"/>
+      <c r="G246" s="63"/>
+      <c r="H246" s="63"/>
+      <c r="I246" s="63"/>
+      <c r="J246" s="63"/>
+      <c r="K246" s="64"/>
     </row>
     <row r="247" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A247" s="37"/>
-      <c r="B247" s="38"/>
+      <c r="A247" s="37">
+        <v>45677</v>
+      </c>
+      <c r="B247" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C247" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D247" s="38"/>
-      <c r="E247" s="40"/>
-      <c r="F247" s="40"/>
-      <c r="G247" s="41"/>
-      <c r="H247" s="41"/>
+        <v>331</v>
+      </c>
+      <c r="D247" s="38" t="s">
+        <v>358</v>
+      </c>
+      <c r="E247" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F247" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="G247" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H247" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I247" s="41">
-        <f t="shared" ref="I247:I257" si="9">H247-G247</f>
+        <f t="shared" ref="I247:I259" si="9">H247-G247</f>
         <v>0</v>
       </c>
       <c r="J247" s="45"/>
       <c r="K247" s="43"/>
     </row>
     <row r="248" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A248" s="37"/>
-      <c r="B248" s="38"/>
+      <c r="A248" s="37">
+        <v>45677</v>
+      </c>
+      <c r="B248" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C248" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D248" s="38"/>
-      <c r="E248" s="40"/>
-      <c r="F248" s="40"/>
-      <c r="G248" s="41"/>
-      <c r="H248" s="41"/>
+        <v>331</v>
+      </c>
+      <c r="D248" s="38" t="s">
+        <v>359</v>
+      </c>
+      <c r="E248" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F248" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="G248" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="H248" s="41">
+        <v>0.1</v>
+      </c>
       <c r="I248" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -9613,16 +9694,30 @@
       <c r="K248" s="43"/>
     </row>
     <row r="249" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A249" s="37"/>
-      <c r="B249" s="38"/>
+      <c r="A249" s="37">
+        <v>45677</v>
+      </c>
+      <c r="B249" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C249" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D249" s="38"/>
-      <c r="E249" s="40"/>
-      <c r="F249" s="40"/>
-      <c r="G249" s="41"/>
-      <c r="H249" s="41"/>
+        <v>363</v>
+      </c>
+      <c r="D249" s="38" t="s">
+        <v>360</v>
+      </c>
+      <c r="E249" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="F249" s="40" t="s">
+        <v>367</v>
+      </c>
+      <c r="G249" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H249" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I249" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -9631,16 +9726,30 @@
       <c r="K249" s="43"/>
     </row>
     <row r="250" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A250" s="37"/>
-      <c r="B250" s="38"/>
+      <c r="A250" s="37">
+        <v>45677</v>
+      </c>
+      <c r="B250" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C250" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D250" s="38"/>
-      <c r="E250" s="40"/>
-      <c r="F250" s="40"/>
-      <c r="G250" s="41"/>
-      <c r="H250" s="41"/>
+        <v>236</v>
+      </c>
+      <c r="D250" s="38" t="s">
+        <v>364</v>
+      </c>
+      <c r="E250" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="F250" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="G250" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H250" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I250" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -9649,16 +9758,30 @@
       <c r="K250" s="43"/>
     </row>
     <row r="251" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A251" s="37"/>
-      <c r="B251" s="38"/>
+      <c r="A251" s="37">
+        <v>45677</v>
+      </c>
+      <c r="B251" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C251" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D251" s="38"/>
-      <c r="E251" s="40"/>
-      <c r="F251" s="40"/>
-      <c r="G251" s="41"/>
-      <c r="H251" s="41"/>
+        <v>349</v>
+      </c>
+      <c r="D251" s="38" t="s">
+        <v>362</v>
+      </c>
+      <c r="E251" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="F251" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="G251" s="41">
+        <v>4</v>
+      </c>
+      <c r="H251" s="41">
+        <v>4</v>
+      </c>
       <c r="I251" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -9667,16 +9790,30 @@
       <c r="K251" s="43"/>
     </row>
     <row r="252" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A252" s="37"/>
-      <c r="B252" s="38"/>
+      <c r="A252" s="37">
+        <v>45678</v>
+      </c>
+      <c r="B252" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C252" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D252" s="38"/>
-      <c r="E252" s="40"/>
-      <c r="F252" s="40"/>
-      <c r="G252" s="41"/>
-      <c r="H252" s="41"/>
+        <v>79</v>
+      </c>
+      <c r="D252" s="38" t="s">
+        <v>361</v>
+      </c>
+      <c r="E252" s="40" t="s">
+        <v>61</v>
+      </c>
+      <c r="F252" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="G252" s="41">
+        <v>0.15</v>
+      </c>
+      <c r="H252" s="41">
+        <v>0.15</v>
+      </c>
       <c r="I252" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -9685,16 +9822,30 @@
       <c r="K252" s="43"/>
     </row>
     <row r="253" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A253" s="37"/>
-      <c r="B253" s="38"/>
+      <c r="A253" s="37">
+        <v>45678</v>
+      </c>
+      <c r="B253" s="38" t="s">
+        <v>54</v>
+      </c>
       <c r="C253" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D253" s="38"/>
-      <c r="E253" s="40"/>
-      <c r="F253" s="40"/>
-      <c r="G253" s="41"/>
-      <c r="H253" s="41"/>
+        <v>77</v>
+      </c>
+      <c r="D253" s="38" t="s">
+        <v>286</v>
+      </c>
+      <c r="E253" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="F253" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G253" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="H253" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I253" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -9703,50 +9854,82 @@
       <c r="K253" s="43"/>
     </row>
     <row r="254" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A254" s="37"/>
-      <c r="B254" s="38"/>
+      <c r="A254" s="37">
+        <v>45678</v>
+      </c>
+      <c r="B254" s="38" t="s">
+        <v>51</v>
+      </c>
       <c r="C254" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D254" s="38"/>
-      <c r="E254" s="40"/>
-      <c r="F254" s="40"/>
-      <c r="G254" s="41"/>
+        <v>206</v>
+      </c>
+      <c r="D254" s="38" t="s">
+        <v>368</v>
+      </c>
+      <c r="E254" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F254" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G254" s="41">
+        <v>0.25</v>
+      </c>
       <c r="H254" s="41"/>
       <c r="I254" s="41">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-0.25</v>
       </c>
       <c r="J254" s="45"/>
       <c r="K254" s="43"/>
     </row>
     <row r="255" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A255" s="37"/>
-      <c r="B255" s="38"/>
+      <c r="A255" s="37">
+        <v>45678</v>
+      </c>
+      <c r="B255" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C255" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D255" s="38"/>
-      <c r="E255" s="40"/>
-      <c r="F255" s="40"/>
-      <c r="G255" s="41"/>
+        <v>236</v>
+      </c>
+      <c r="D255" s="38" t="s">
+        <v>365</v>
+      </c>
+      <c r="E255" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="F255" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="G255" s="41">
+        <v>4</v>
+      </c>
       <c r="H255" s="41"/>
       <c r="I255" s="41">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="J255" s="45"/>
       <c r="K255" s="43"/>
     </row>
     <row r="256" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A256" s="37"/>
-      <c r="B256" s="38"/>
+      <c r="B256" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C256" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D256" s="38"/>
-      <c r="E256" s="40"/>
-      <c r="F256" s="40"/>
+        <v>363</v>
+      </c>
+      <c r="D256" s="38" t="s">
+        <v>366</v>
+      </c>
+      <c r="E256" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="F256" s="40" t="s">
+        <v>367</v>
+      </c>
       <c r="G256" s="41"/>
       <c r="H256" s="41"/>
       <c r="I256" s="41">
@@ -9757,35 +9940,83 @@
       <c r="K256" s="43"/>
     </row>
     <row r="257" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A257" s="48"/>
-      <c r="B257" s="49"/>
-      <c r="C257" s="49"/>
-      <c r="D257" s="49"/>
-      <c r="E257" s="49" t="s">
+      <c r="A257" s="37"/>
+      <c r="B257" s="38"/>
+      <c r="C257" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D257" s="38"/>
+      <c r="E257" s="40"/>
+      <c r="F257" s="40"/>
+      <c r="G257" s="41"/>
+      <c r="H257" s="41"/>
+      <c r="I257" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J257" s="45"/>
+      <c r="K257" s="43"/>
+    </row>
+    <row r="258" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A258" s="37"/>
+      <c r="B258" s="38"/>
+      <c r="C258" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D258" s="38"/>
+      <c r="E258" s="40"/>
+      <c r="F258" s="40"/>
+      <c r="G258" s="41"/>
+      <c r="H258" s="41"/>
+      <c r="I258" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J258" s="45"/>
+      <c r="K258" s="43"/>
+    </row>
+    <row r="259" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A259" s="48"/>
+      <c r="B259" s="49"/>
+      <c r="C259" s="49"/>
+      <c r="D259" s="49"/>
+      <c r="E259" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F257" s="49"/>
-      <c r="G257" s="50">
-        <f t="shared" ref="G257:H257" si="10">SUM(G247:G256)</f>
-        <v>0</v>
-      </c>
-      <c r="H257" s="50">
+      <c r="F259" s="49"/>
+      <c r="G259" s="50">
+        <f t="shared" ref="G259:H259" si="10">SUM(G247:G258)</f>
+        <v>10</v>
+      </c>
+      <c r="H259" s="50">
         <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="I257" s="50">
+        <v>5.75</v>
+      </c>
+      <c r="I259" s="50">
         <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J257" s="51"/>
-      <c r="K257" s="52"/>
+        <v>-4.25</v>
+      </c>
+      <c r="J259" s="51"/>
+      <c r="K259" s="52"/>
+    </row>
+    <row r="260" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E260" s="40"/>
+    </row>
+    <row r="261" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G261" s="79" t="s">
+        <v>18</v>
+      </c>
+      <c r="H261" s="80">
+        <f>H46+H82+H117+H152+H196+H219+H243+H259</f>
+        <v>192.54</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{7FAA7E16-50E7-4532-BC99-31DB9966F18E}">
+      <autoFilter ref="A1:K15" xr:uid="{9D3D98CF-DB4D-4810-AECB-DDB35F09E772}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -9796,14 +10027,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B198:K198"/>
-    <mergeCell ref="B199:K199"/>
-    <mergeCell ref="A220:K220"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A153:K153"/>
-    <mergeCell ref="B154:K154"/>
-    <mergeCell ref="B155:K155"/>
-    <mergeCell ref="A197:K197"/>
     <mergeCell ref="A244:K244"/>
     <mergeCell ref="B245:K245"/>
     <mergeCell ref="B246:K246"/>
@@ -9820,6 +10043,14 @@
     <mergeCell ref="B221:K221"/>
     <mergeCell ref="B222:K222"/>
     <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B198:K198"/>
+    <mergeCell ref="B199:K199"/>
+    <mergeCell ref="A220:K220"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A153:K153"/>
+    <mergeCell ref="B154:K154"/>
+    <mergeCell ref="B155:K155"/>
+    <mergeCell ref="A197:K197"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B151 B156:B195 B200:B218 B223:B242">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -9838,7 +10069,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B152 B154:B196 B198:B219 B221:B243 B245:B257">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B152 B154:B196 B198:B219 B221:B243 B245:B259">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -9846,7 +10077,7 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B247:B256">
+  <conditionalFormatting sqref="B247:B258">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B247))))</formula>
     </cfRule>
@@ -9863,17 +10094,17 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B247))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G152 G156:G196 G200:G219 G223:G243 G247:G257">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G152 G156:G196 G200:G219 G223:G243 G247:G259">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H257">
+  <conditionalFormatting sqref="H1:H259">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I152 I156:I196 I200:I219 I223:I243 I247:I257">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I152 I156:I196 I200:I219 I223:I243 I247:I259">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -9882,7 +10113,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F247:F256 F86:F116 F5:F45 F50:F81 F121:F151 F156:F195 F200:F218 F223:F242" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F247:F258 F86:F116 F5:F45 F50:F81 F121:F151 F156:F195 F200:F218 F223:F242" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9899,13 +10130,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E116 E247:E256 E50:E81 E121:E151 E156:E195 E200:E218 E223:E242</xm:sqref>
+          <xm:sqref>E5:E45 E86:E116 E247:E258 E50:E81 E121:E151 E156:E195 E200:E218 E223:E242</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B116 B247:B256 B50:B81 B121:B151 B156:B195 B200:B218 B223:B242</xm:sqref>
+          <xm:sqref>B5:B45 B86:B116 B247:B258 B50:B81 B121:B151 B156:B195 B200:B218 B223:B242</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -11546,6 +11777,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -11780,27 +12031,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11817,23 +12067,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W8 DataLab 1 Work II (Notebooks Finish)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388BE7D2-C6B0-43CF-B7DE-F128F8BD0CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB545EE4-E8A4-471F-8C78-A18B96978E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1266" uniqueCount="370">
   <si>
     <t>Date</t>
   </si>
@@ -1154,9 +1154,6 @@
     <t>Creative Brief Work</t>
   </si>
   <si>
-    <t>5,5 so far</t>
-  </si>
-  <si>
     <t>Evidence in Learning Log week 7</t>
   </si>
   <si>
@@ -1175,9 +1172,6 @@
     <t>Do the Linear Regression from Scratch</t>
   </si>
   <si>
-    <t>I somehow missed this when catching up in week 7, so I did it later.</t>
-  </si>
-  <si>
     <t>Finish Learning Log Block A</t>
   </si>
   <si>
@@ -1209,6 +1203,15 @@
   </si>
   <si>
     <t>Finishing touches to SMARTER-goals</t>
+  </si>
+  <si>
+    <t>I somehow missed this when catching up in week 7, so I did it later. Had a couple errors so the task took longer than expected.</t>
+  </si>
+  <si>
+    <t>Had a bunch of errors that took me some time to fix.</t>
+  </si>
+  <si>
+    <t>Had a couple of errors that I had to fix, which took time.</t>
   </si>
 </sst>
 </file>
@@ -1549,7 +1552,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1700,26 +1703,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1736,6 +1720,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1754,6 +1740,24 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1761,10 +1765,6 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2281,53 +2281,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="61"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="64"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="56"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="64"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3666,53 +3666,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="65" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="67"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="67"/>
-      <c r="H47" s="67"/>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="68"/>
+      <c r="B47" s="60"/>
+      <c r="C47" s="60"/>
+      <c r="D47" s="60"/>
+      <c r="E47" s="60"/>
+      <c r="F47" s="60"/>
+      <c r="G47" s="60"/>
+      <c r="H47" s="60"/>
+      <c r="I47" s="60"/>
+      <c r="J47" s="60"/>
+      <c r="K47" s="61"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="55"/>
-      <c r="K48" s="56"/>
+      <c r="C48" s="63"/>
+      <c r="D48" s="63"/>
+      <c r="E48" s="63"/>
+      <c r="F48" s="63"/>
+      <c r="G48" s="63"/>
+      <c r="H48" s="63"/>
+      <c r="I48" s="63"/>
+      <c r="J48" s="63"/>
+      <c r="K48" s="64"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="56"/>
+      <c r="C49" s="63"/>
+      <c r="D49" s="63"/>
+      <c r="E49" s="63"/>
+      <c r="F49" s="63"/>
+      <c r="G49" s="63"/>
+      <c r="H49" s="63"/>
+      <c r="I49" s="63"/>
+      <c r="J49" s="63"/>
+      <c r="K49" s="64"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4763,53 +4763,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72" t="s">
+      <c r="A83" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="55"/>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="55"/>
-      <c r="I83" s="55"/>
-      <c r="J83" s="55"/>
-      <c r="K83" s="56"/>
+      <c r="B83" s="63"/>
+      <c r="C83" s="63"/>
+      <c r="D83" s="63"/>
+      <c r="E83" s="63"/>
+      <c r="F83" s="63"/>
+      <c r="G83" s="63"/>
+      <c r="H83" s="63"/>
+      <c r="I83" s="63"/>
+      <c r="J83" s="63"/>
+      <c r="K83" s="64"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="73" t="s">
+      <c r="B84" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="55"/>
-      <c r="D84" s="55"/>
-      <c r="E84" s="55"/>
-      <c r="F84" s="55"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="55"/>
-      <c r="I84" s="55"/>
-      <c r="J84" s="55"/>
-      <c r="K84" s="56"/>
+      <c r="C84" s="63"/>
+      <c r="D84" s="63"/>
+      <c r="E84" s="63"/>
+      <c r="F84" s="63"/>
+      <c r="G84" s="63"/>
+      <c r="H84" s="63"/>
+      <c r="I84" s="63"/>
+      <c r="J84" s="63"/>
+      <c r="K84" s="64"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="73" t="s">
+      <c r="B85" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="55"/>
-      <c r="D85" s="55"/>
-      <c r="E85" s="55"/>
-      <c r="F85" s="55"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="55"/>
-      <c r="I85" s="55"/>
-      <c r="J85" s="55"/>
-      <c r="K85" s="56"/>
+      <c r="C85" s="63"/>
+      <c r="D85" s="63"/>
+      <c r="E85" s="63"/>
+      <c r="F85" s="63"/>
+      <c r="G85" s="63"/>
+      <c r="H85" s="63"/>
+      <c r="I85" s="63"/>
+      <c r="J85" s="63"/>
+      <c r="K85" s="64"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5824,53 +5824,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="74" t="s">
+      <c r="A118" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="55"/>
-      <c r="C118" s="55"/>
-      <c r="D118" s="55"/>
-      <c r="E118" s="55"/>
-      <c r="F118" s="55"/>
-      <c r="G118" s="55"/>
-      <c r="H118" s="55"/>
-      <c r="I118" s="55"/>
-      <c r="J118" s="55"/>
-      <c r="K118" s="56"/>
+      <c r="B118" s="63"/>
+      <c r="C118" s="63"/>
+      <c r="D118" s="63"/>
+      <c r="E118" s="63"/>
+      <c r="F118" s="63"/>
+      <c r="G118" s="63"/>
+      <c r="H118" s="63"/>
+      <c r="I118" s="63"/>
+      <c r="J118" s="63"/>
+      <c r="K118" s="64"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="58" t="s">
+      <c r="B119" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="55"/>
-      <c r="D119" s="55"/>
-      <c r="E119" s="55"/>
-      <c r="F119" s="55"/>
-      <c r="G119" s="55"/>
-      <c r="H119" s="55"/>
-      <c r="I119" s="55"/>
-      <c r="J119" s="55"/>
-      <c r="K119" s="56"/>
+      <c r="C119" s="63"/>
+      <c r="D119" s="63"/>
+      <c r="E119" s="63"/>
+      <c r="F119" s="63"/>
+      <c r="G119" s="63"/>
+      <c r="H119" s="63"/>
+      <c r="I119" s="63"/>
+      <c r="J119" s="63"/>
+      <c r="K119" s="64"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="58" t="s">
+      <c r="B120" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="55"/>
-      <c r="D120" s="55"/>
-      <c r="E120" s="55"/>
-      <c r="F120" s="55"/>
-      <c r="G120" s="55"/>
-      <c r="H120" s="55"/>
-      <c r="I120" s="55"/>
-      <c r="J120" s="55"/>
-      <c r="K120" s="56"/>
+      <c r="C120" s="63"/>
+      <c r="D120" s="63"/>
+      <c r="E120" s="63"/>
+      <c r="F120" s="63"/>
+      <c r="G120" s="63"/>
+      <c r="H120" s="63"/>
+      <c r="I120" s="63"/>
+      <c r="J120" s="63"/>
+      <c r="K120" s="64"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6863,53 +6863,53 @@
       <c r="K152" s="46"/>
     </row>
     <row r="153" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="59" t="s">
+      <c r="A153" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="B153" s="55"/>
-      <c r="C153" s="55"/>
-      <c r="D153" s="55"/>
-      <c r="E153" s="55"/>
-      <c r="F153" s="55"/>
-      <c r="G153" s="55"/>
-      <c r="H153" s="55"/>
-      <c r="I153" s="55"/>
-      <c r="J153" s="55"/>
-      <c r="K153" s="56"/>
+      <c r="B153" s="63"/>
+      <c r="C153" s="63"/>
+      <c r="D153" s="63"/>
+      <c r="E153" s="63"/>
+      <c r="F153" s="63"/>
+      <c r="G153" s="63"/>
+      <c r="H153" s="63"/>
+      <c r="I153" s="63"/>
+      <c r="J153" s="63"/>
+      <c r="K153" s="64"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B154" s="60" t="s">
+      <c r="B154" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C154" s="55"/>
-      <c r="D154" s="55"/>
-      <c r="E154" s="55"/>
-      <c r="F154" s="55"/>
-      <c r="G154" s="55"/>
-      <c r="H154" s="55"/>
-      <c r="I154" s="55"/>
-      <c r="J154" s="55"/>
-      <c r="K154" s="56"/>
+      <c r="C154" s="63"/>
+      <c r="D154" s="63"/>
+      <c r="E154" s="63"/>
+      <c r="F154" s="63"/>
+      <c r="G154" s="63"/>
+      <c r="H154" s="63"/>
+      <c r="I154" s="63"/>
+      <c r="J154" s="63"/>
+      <c r="K154" s="64"/>
     </row>
     <row r="155" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B155" s="60" t="s">
+      <c r="B155" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C155" s="55"/>
-      <c r="D155" s="55"/>
-      <c r="E155" s="55"/>
-      <c r="F155" s="55"/>
-      <c r="G155" s="55"/>
-      <c r="H155" s="55"/>
-      <c r="I155" s="55"/>
-      <c r="J155" s="55"/>
-      <c r="K155" s="56"/>
+      <c r="C155" s="63"/>
+      <c r="D155" s="63"/>
+      <c r="E155" s="63"/>
+      <c r="F155" s="63"/>
+      <c r="G155" s="63"/>
+      <c r="H155" s="63"/>
+      <c r="I155" s="63"/>
+      <c r="J155" s="63"/>
+      <c r="K155" s="64"/>
     </row>
     <row r="156" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A156" s="37">
@@ -8206,53 +8206,53 @@
       <c r="K196" s="46"/>
     </row>
     <row r="197" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A197" s="61" t="s">
+      <c r="A197" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="B197" s="55"/>
-      <c r="C197" s="55"/>
-      <c r="D197" s="55"/>
-      <c r="E197" s="55"/>
-      <c r="F197" s="55"/>
-      <c r="G197" s="55"/>
-      <c r="H197" s="55"/>
-      <c r="I197" s="55"/>
-      <c r="J197" s="55"/>
-      <c r="K197" s="56"/>
+      <c r="B197" s="63"/>
+      <c r="C197" s="63"/>
+      <c r="D197" s="63"/>
+      <c r="E197" s="63"/>
+      <c r="F197" s="63"/>
+      <c r="G197" s="63"/>
+      <c r="H197" s="63"/>
+      <c r="I197" s="63"/>
+      <c r="J197" s="63"/>
+      <c r="K197" s="64"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B198" s="54" t="s">
+      <c r="B198" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C198" s="55"/>
-      <c r="D198" s="55"/>
-      <c r="E198" s="55"/>
-      <c r="F198" s="55"/>
-      <c r="G198" s="55"/>
-      <c r="H198" s="55"/>
-      <c r="I198" s="55"/>
-      <c r="J198" s="55"/>
-      <c r="K198" s="56"/>
+      <c r="C198" s="63"/>
+      <c r="D198" s="63"/>
+      <c r="E198" s="63"/>
+      <c r="F198" s="63"/>
+      <c r="G198" s="63"/>
+      <c r="H198" s="63"/>
+      <c r="I198" s="63"/>
+      <c r="J198" s="63"/>
+      <c r="K198" s="64"/>
     </row>
     <row r="199" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B199" s="54" t="s">
+      <c r="B199" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="C199" s="55"/>
-      <c r="D199" s="55"/>
-      <c r="E199" s="55"/>
-      <c r="F199" s="55"/>
-      <c r="G199" s="55"/>
-      <c r="H199" s="55"/>
-      <c r="I199" s="55"/>
-      <c r="J199" s="55"/>
-      <c r="K199" s="56"/>
+      <c r="C199" s="63"/>
+      <c r="D199" s="63"/>
+      <c r="E199" s="63"/>
+      <c r="F199" s="63"/>
+      <c r="G199" s="63"/>
+      <c r="H199" s="63"/>
+      <c r="I199" s="63"/>
+      <c r="J199" s="63"/>
+      <c r="K199" s="64"/>
     </row>
     <row r="200" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A200" s="37">
@@ -8773,13 +8773,13 @@
         <v>45676</v>
       </c>
       <c r="B216" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C216" s="39" t="s">
         <v>236</v>
       </c>
       <c r="D216" s="38" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E216" s="40" t="s">
         <v>49</v>
@@ -8790,14 +8790,16 @@
       <c r="G216" s="41">
         <v>2</v>
       </c>
-      <c r="H216" s="41"/>
+      <c r="H216" s="41">
+        <v>4</v>
+      </c>
       <c r="I216" s="41">
         <f t="shared" si="7"/>
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="J216" s="45"/>
       <c r="K216" s="43" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
     </row>
     <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -8868,63 +8870,63 @@
       </c>
       <c r="H219" s="18">
         <f>SUM(H200:H218)</f>
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I219" s="18">
         <f t="shared" si="7"/>
-        <v>-9.75</v>
+        <v>-5.75</v>
       </c>
       <c r="J219" s="19"/>
       <c r="K219" s="46"/>
     </row>
     <row r="220" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A220" s="57" t="s">
+      <c r="A220" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="B220" s="55"/>
-      <c r="C220" s="55"/>
-      <c r="D220" s="55"/>
-      <c r="E220" s="55"/>
-      <c r="F220" s="55"/>
-      <c r="G220" s="55"/>
-      <c r="H220" s="55"/>
-      <c r="I220" s="55"/>
-      <c r="J220" s="55"/>
-      <c r="K220" s="56"/>
+      <c r="B220" s="63"/>
+      <c r="C220" s="63"/>
+      <c r="D220" s="63"/>
+      <c r="E220" s="63"/>
+      <c r="F220" s="63"/>
+      <c r="G220" s="63"/>
+      <c r="H220" s="63"/>
+      <c r="I220" s="63"/>
+      <c r="J220" s="63"/>
+      <c r="K220" s="64"/>
     </row>
     <row r="221" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A221" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B221" s="75" t="s">
+      <c r="B221" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C221" s="55"/>
-      <c r="D221" s="55"/>
-      <c r="E221" s="55"/>
-      <c r="F221" s="55"/>
-      <c r="G221" s="55"/>
-      <c r="H221" s="55"/>
-      <c r="I221" s="55"/>
-      <c r="J221" s="55"/>
-      <c r="K221" s="56"/>
+      <c r="C221" s="63"/>
+      <c r="D221" s="63"/>
+      <c r="E221" s="63"/>
+      <c r="F221" s="63"/>
+      <c r="G221" s="63"/>
+      <c r="H221" s="63"/>
+      <c r="I221" s="63"/>
+      <c r="J221" s="63"/>
+      <c r="K221" s="64"/>
     </row>
     <row r="222" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B222" s="75" t="s">
+      <c r="B222" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C222" s="55"/>
-      <c r="D222" s="55"/>
-      <c r="E222" s="55"/>
-      <c r="F222" s="55"/>
-      <c r="G222" s="55"/>
-      <c r="H222" s="55"/>
-      <c r="I222" s="55"/>
-      <c r="J222" s="55"/>
-      <c r="K222" s="56"/>
+      <c r="C222" s="63"/>
+      <c r="D222" s="63"/>
+      <c r="E222" s="63"/>
+      <c r="F222" s="63"/>
+      <c r="G222" s="63"/>
+      <c r="H222" s="63"/>
+      <c r="I222" s="63"/>
+      <c r="J222" s="63"/>
+      <c r="K222" s="64"/>
     </row>
     <row r="223" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A223" s="37">
@@ -9349,7 +9351,7 @@
         <v>348</v>
       </c>
       <c r="D236" s="38" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E236" s="40" t="s">
         <v>63</v>
@@ -9407,7 +9409,7 @@
         <v>45674</v>
       </c>
       <c r="B238" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C238" s="39" t="s">
         <v>236</v>
@@ -9424,14 +9426,16 @@
       <c r="G238" s="41">
         <v>4</v>
       </c>
-      <c r="H238" s="41"/>
+      <c r="H238" s="41">
+        <v>5.75</v>
+      </c>
       <c r="I238" s="41">
         <f t="shared" si="8"/>
-        <v>-4</v>
+        <v>1.75</v>
       </c>
       <c r="J238" s="45"/>
       <c r="K238" s="43" t="s">
-        <v>350</v>
+        <v>368</v>
       </c>
     </row>
     <row r="239" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9465,7 +9469,7 @@
       </c>
       <c r="J239" s="45"/>
       <c r="K239" s="43" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="240" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9479,7 +9483,7 @@
         <v>206</v>
       </c>
       <c r="D240" s="38" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E240" s="40" t="s">
         <v>63</v>
@@ -9509,7 +9513,7 @@
         <v>206</v>
       </c>
       <c r="D241" s="38" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E241" s="40" t="s">
         <v>63</v>
@@ -9537,7 +9541,7 @@
         <v>79</v>
       </c>
       <c r="D242" s="38" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E242" s="40" t="s">
         <v>63</v>
@@ -9571,63 +9575,63 @@
       </c>
       <c r="H243" s="18">
         <f>SUM(H223:H242)</f>
-        <v>10.5</v>
+        <v>16.25</v>
       </c>
       <c r="I243" s="18">
         <f t="shared" si="8"/>
-        <v>-10</v>
+        <v>-4.25</v>
       </c>
       <c r="J243" s="19"/>
       <c r="K243" s="46"/>
     </row>
     <row r="244" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A244" s="62" t="s">
+      <c r="A244" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="B244" s="63"/>
-      <c r="C244" s="63"/>
-      <c r="D244" s="63"/>
-      <c r="E244" s="63"/>
-      <c r="F244" s="63"/>
-      <c r="G244" s="63"/>
-      <c r="H244" s="63"/>
-      <c r="I244" s="63"/>
-      <c r="J244" s="63"/>
-      <c r="K244" s="64"/>
+      <c r="B244" s="56"/>
+      <c r="C244" s="56"/>
+      <c r="D244" s="56"/>
+      <c r="E244" s="56"/>
+      <c r="F244" s="56"/>
+      <c r="G244" s="56"/>
+      <c r="H244" s="56"/>
+      <c r="I244" s="56"/>
+      <c r="J244" s="56"/>
+      <c r="K244" s="57"/>
     </row>
     <row r="245" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A245" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B245" s="65" t="s">
+      <c r="B245" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C245" s="63"/>
-      <c r="D245" s="63"/>
-      <c r="E245" s="63"/>
-      <c r="F245" s="63"/>
-      <c r="G245" s="63"/>
-      <c r="H245" s="63"/>
-      <c r="I245" s="63"/>
-      <c r="J245" s="63"/>
-      <c r="K245" s="64"/>
+      <c r="C245" s="56"/>
+      <c r="D245" s="56"/>
+      <c r="E245" s="56"/>
+      <c r="F245" s="56"/>
+      <c r="G245" s="56"/>
+      <c r="H245" s="56"/>
+      <c r="I245" s="56"/>
+      <c r="J245" s="56"/>
+      <c r="K245" s="57"/>
     </row>
     <row r="246" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A246" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B246" s="65" t="s">
+      <c r="B246" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C246" s="63"/>
-      <c r="D246" s="63"/>
-      <c r="E246" s="63"/>
-      <c r="F246" s="63"/>
-      <c r="G246" s="63"/>
-      <c r="H246" s="63"/>
-      <c r="I246" s="63"/>
-      <c r="J246" s="63"/>
-      <c r="K246" s="64"/>
+      <c r="C246" s="56"/>
+      <c r="D246" s="56"/>
+      <c r="E246" s="56"/>
+      <c r="F246" s="56"/>
+      <c r="G246" s="56"/>
+      <c r="H246" s="56"/>
+      <c r="I246" s="56"/>
+      <c r="J246" s="56"/>
+      <c r="K246" s="57"/>
     </row>
     <row r="247" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A247" s="37">
@@ -9640,7 +9644,7 @@
         <v>331</v>
       </c>
       <c r="D247" s="38" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E247" s="40" t="s">
         <v>63</v>
@@ -9672,7 +9676,7 @@
         <v>331</v>
       </c>
       <c r="D248" s="38" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E248" s="40" t="s">
         <v>63</v>
@@ -9701,16 +9705,16 @@
         <v>54</v>
       </c>
       <c r="C249" s="39" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D249" s="38" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="E249" s="40" t="s">
         <v>43</v>
       </c>
       <c r="F249" s="40" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="G249" s="41">
         <v>0.5</v>
@@ -9736,7 +9740,7 @@
         <v>236</v>
       </c>
       <c r="D250" s="38" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E250" s="40" t="s">
         <v>64</v>
@@ -9768,7 +9772,7 @@
         <v>349</v>
       </c>
       <c r="D251" s="38" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E251" s="40" t="s">
         <v>49</v>
@@ -9800,7 +9804,7 @@
         <v>79</v>
       </c>
       <c r="D252" s="38" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E252" s="40" t="s">
         <v>61</v>
@@ -9858,13 +9862,13 @@
         <v>45678</v>
       </c>
       <c r="B254" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C254" s="39" t="s">
         <v>206</v>
       </c>
       <c r="D254" s="38" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E254" s="40" t="s">
         <v>63</v>
@@ -9875,10 +9879,12 @@
       <c r="G254" s="41">
         <v>0.25</v>
       </c>
-      <c r="H254" s="41"/>
+      <c r="H254" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I254" s="41">
         <f t="shared" si="9"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J254" s="45"/>
       <c r="K254" s="43"/>
@@ -9888,13 +9894,13 @@
         <v>45678</v>
       </c>
       <c r="B255" s="38" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C255" s="39" t="s">
         <v>236</v>
       </c>
       <c r="D255" s="38" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="E255" s="40" t="s">
         <v>49</v>
@@ -9905,13 +9911,17 @@
       <c r="G255" s="41">
         <v>4</v>
       </c>
-      <c r="H255" s="41"/>
+      <c r="H255" s="41">
+        <v>4.25</v>
+      </c>
       <c r="I255" s="41">
         <f t="shared" si="9"/>
-        <v>-4</v>
+        <v>0.25</v>
       </c>
       <c r="J255" s="45"/>
-      <c r="K255" s="43"/>
+      <c r="K255" s="43" t="s">
+        <v>369</v>
+      </c>
     </row>
     <row r="256" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A256" s="37"/>
@@ -9919,16 +9929,16 @@
         <v>42</v>
       </c>
       <c r="C256" s="39" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D256" s="38" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="E256" s="40" t="s">
         <v>43</v>
       </c>
       <c r="F256" s="40" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="G256" s="41"/>
       <c r="H256" s="41"/>
@@ -9990,11 +10000,11 @@
       </c>
       <c r="H259" s="50">
         <f t="shared" si="10"/>
-        <v>5.75</v>
+        <v>10.25</v>
       </c>
       <c r="I259" s="50">
         <f t="shared" si="9"/>
-        <v>-4.25</v>
+        <v>0.25</v>
       </c>
       <c r="J259" s="51"/>
       <c r="K259" s="52"/>
@@ -10003,12 +10013,12 @@
       <c r="E260" s="40"/>
     </row>
     <row r="261" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G261" s="79" t="s">
+      <c r="G261" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="H261" s="80">
+      <c r="H261" s="54">
         <f>H46+H82+H117+H152+H196+H219+H243+H259</f>
-        <v>192.54</v>
+        <v>206.79</v>
       </c>
     </row>
   </sheetData>
@@ -10016,7 +10026,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{9D3D98CF-DB4D-4810-AECB-DDB35F09E772}">
+      <autoFilter ref="A1:K15" xr:uid="{A64F5071-78C5-46B1-9F42-0443704A2C92}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -10027,6 +10037,14 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
+    <mergeCell ref="B198:K198"/>
+    <mergeCell ref="B199:K199"/>
+    <mergeCell ref="A220:K220"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A153:K153"/>
+    <mergeCell ref="B154:K154"/>
+    <mergeCell ref="B155:K155"/>
+    <mergeCell ref="A197:K197"/>
     <mergeCell ref="A244:K244"/>
     <mergeCell ref="B245:K245"/>
     <mergeCell ref="B246:K246"/>
@@ -10043,14 +10061,6 @@
     <mergeCell ref="B221:K221"/>
     <mergeCell ref="B222:K222"/>
     <mergeCell ref="B119:K119"/>
-    <mergeCell ref="B198:K198"/>
-    <mergeCell ref="B199:K199"/>
-    <mergeCell ref="A220:K220"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A153:K153"/>
-    <mergeCell ref="B154:K154"/>
-    <mergeCell ref="B155:K155"/>
-    <mergeCell ref="A197:K197"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B151 B156:B195 B200:B218 B223:B242">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -10569,58 +10579,58 @@
       <c r="K13" s="17"/>
     </row>
     <row r="14" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="76" t="s">
+      <c r="B14" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="77"/>
-      <c r="D14" s="77"/>
-      <c r="E14" s="77"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="77"/>
-      <c r="H14" s="77"/>
-      <c r="I14" s="77"/>
-      <c r="J14" s="77"/>
-      <c r="K14" s="77"/>
+      <c r="C14" s="78"/>
+      <c r="D14" s="78"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="78"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="78"/>
+      <c r="I14" s="78"/>
+      <c r="J14" s="78"/>
+      <c r="K14" s="78"/>
     </row>
     <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="9"/>
     </row>
     <row r="19" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="78" t="s">
+      <c r="B19" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="78"/>
-      <c r="D19" s="78"/>
-      <c r="E19" s="78"/>
-      <c r="F19" s="78"/>
+      <c r="C19" s="79"/>
+      <c r="D19" s="79"/>
+      <c r="E19" s="79"/>
+      <c r="F19" s="79"/>
     </row>
     <row r="20" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="78"/>
-      <c r="C20" s="78"/>
-      <c r="D20" s="78"/>
-      <c r="E20" s="78"/>
-      <c r="F20" s="78"/>
+      <c r="B20" s="79"/>
+      <c r="C20" s="79"/>
+      <c r="D20" s="79"/>
+      <c r="E20" s="79"/>
+      <c r="F20" s="79"/>
     </row>
     <row r="21" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="78"/>
-      <c r="C21" s="78"/>
-      <c r="D21" s="78"/>
-      <c r="E21" s="78"/>
-      <c r="F21" s="78"/>
+      <c r="B21" s="79"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="79"/>
+      <c r="F21" s="79"/>
     </row>
     <row r="22" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="78"/>
-      <c r="C22" s="78"/>
-      <c r="D22" s="78"/>
-      <c r="E22" s="78"/>
-      <c r="F22" s="78"/>
+      <c r="B22" s="79"/>
+      <c r="C22" s="79"/>
+      <c r="D22" s="79"/>
+      <c r="E22" s="79"/>
+      <c r="F22" s="79"/>
     </row>
     <row r="23" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="78"/>
-      <c r="C23" s="78"/>
-      <c r="D23" s="78"/>
-      <c r="E23" s="78"/>
-      <c r="F23" s="78"/>
+      <c r="B23" s="79"/>
+      <c r="C23" s="79"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="79"/>
+      <c r="F23" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -11777,26 +11787,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -12031,10 +12021,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -12051,20 +12072,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W8 DataLab 1 Work III (End of day)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB545EE4-E8A4-471F-8C78-A18B96978E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7589D462-AA72-4E08-9F4C-EFEE2E3F1067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1266" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="371">
   <si>
     <t>Date</t>
   </si>
@@ -1212,6 +1212,9 @@
   </si>
   <si>
     <t>Had a couple of errors that I had to fix, which took time.</t>
+  </si>
+  <si>
+    <t>Finish the Algebraic Example notebook</t>
   </si>
 </sst>
 </file>
@@ -1704,6 +1707,26 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1720,8 +1743,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1739,24 +1760,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2229,7 +2232,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K261"/>
+  <dimension ref="A1:K263"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -2281,53 +2284,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
-      <c r="K2" s="61"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="69"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="62" t="s">
+      <c r="B3" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="57"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="64"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="57"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3666,53 +3669,53 @@
       <c r="K46" s="46"/>
     </row>
     <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="65" t="s">
+      <c r="A47" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="60"/>
-      <c r="C47" s="60"/>
-      <c r="D47" s="60"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="60"/>
-      <c r="G47" s="60"/>
-      <c r="H47" s="60"/>
-      <c r="I47" s="60"/>
-      <c r="J47" s="60"/>
-      <c r="K47" s="61"/>
+      <c r="B47" s="68"/>
+      <c r="C47" s="68"/>
+      <c r="D47" s="68"/>
+      <c r="E47" s="68"/>
+      <c r="F47" s="68"/>
+      <c r="G47" s="68"/>
+      <c r="H47" s="68"/>
+      <c r="I47" s="68"/>
+      <c r="J47" s="68"/>
+      <c r="K47" s="69"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="66" t="s">
+      <c r="B48" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="63"/>
-      <c r="D48" s="63"/>
-      <c r="E48" s="63"/>
-      <c r="F48" s="63"/>
-      <c r="G48" s="63"/>
-      <c r="H48" s="63"/>
-      <c r="I48" s="63"/>
-      <c r="J48" s="63"/>
-      <c r="K48" s="64"/>
+      <c r="C48" s="56"/>
+      <c r="D48" s="56"/>
+      <c r="E48" s="56"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="56"/>
+      <c r="H48" s="56"/>
+      <c r="I48" s="56"/>
+      <c r="J48" s="56"/>
+      <c r="K48" s="57"/>
     </row>
     <row r="49" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="66" t="s">
+      <c r="B49" s="72" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="63"/>
-      <c r="D49" s="63"/>
-      <c r="E49" s="63"/>
-      <c r="F49" s="63"/>
-      <c r="G49" s="63"/>
-      <c r="H49" s="63"/>
-      <c r="I49" s="63"/>
-      <c r="J49" s="63"/>
-      <c r="K49" s="64"/>
+      <c r="C49" s="56"/>
+      <c r="D49" s="56"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="56"/>
+      <c r="I49" s="56"/>
+      <c r="J49" s="56"/>
+      <c r="K49" s="57"/>
     </row>
     <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="47">
@@ -4763,53 +4766,53 @@
       <c r="K82" s="46"/>
     </row>
     <row r="83" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="67" t="s">
+      <c r="A83" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="B83" s="63"/>
-      <c r="C83" s="63"/>
-      <c r="D83" s="63"/>
-      <c r="E83" s="63"/>
-      <c r="F83" s="63"/>
-      <c r="G83" s="63"/>
-      <c r="H83" s="63"/>
-      <c r="I83" s="63"/>
-      <c r="J83" s="63"/>
-      <c r="K83" s="64"/>
+      <c r="B83" s="56"/>
+      <c r="C83" s="56"/>
+      <c r="D83" s="56"/>
+      <c r="E83" s="56"/>
+      <c r="F83" s="56"/>
+      <c r="G83" s="56"/>
+      <c r="H83" s="56"/>
+      <c r="I83" s="56"/>
+      <c r="J83" s="56"/>
+      <c r="K83" s="57"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="68" t="s">
+      <c r="B84" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C84" s="63"/>
-      <c r="D84" s="63"/>
-      <c r="E84" s="63"/>
-      <c r="F84" s="63"/>
-      <c r="G84" s="63"/>
-      <c r="H84" s="63"/>
-      <c r="I84" s="63"/>
-      <c r="J84" s="63"/>
-      <c r="K84" s="64"/>
+      <c r="C84" s="56"/>
+      <c r="D84" s="56"/>
+      <c r="E84" s="56"/>
+      <c r="F84" s="56"/>
+      <c r="G84" s="56"/>
+      <c r="H84" s="56"/>
+      <c r="I84" s="56"/>
+      <c r="J84" s="56"/>
+      <c r="K84" s="57"/>
     </row>
     <row r="85" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="68" t="s">
+      <c r="B85" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C85" s="63"/>
-      <c r="D85" s="63"/>
-      <c r="E85" s="63"/>
-      <c r="F85" s="63"/>
-      <c r="G85" s="63"/>
-      <c r="H85" s="63"/>
-      <c r="I85" s="63"/>
-      <c r="J85" s="63"/>
-      <c r="K85" s="64"/>
+      <c r="C85" s="56"/>
+      <c r="D85" s="56"/>
+      <c r="E85" s="56"/>
+      <c r="F85" s="56"/>
+      <c r="G85" s="56"/>
+      <c r="H85" s="56"/>
+      <c r="I85" s="56"/>
+      <c r="J85" s="56"/>
+      <c r="K85" s="57"/>
     </row>
     <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="37">
@@ -5824,53 +5827,53 @@
       <c r="K117" s="46"/>
     </row>
     <row r="118" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="69" t="s">
+      <c r="A118" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="B118" s="63"/>
-      <c r="C118" s="63"/>
-      <c r="D118" s="63"/>
-      <c r="E118" s="63"/>
-      <c r="F118" s="63"/>
-      <c r="G118" s="63"/>
-      <c r="H118" s="63"/>
-      <c r="I118" s="63"/>
-      <c r="J118" s="63"/>
-      <c r="K118" s="64"/>
+      <c r="B118" s="56"/>
+      <c r="C118" s="56"/>
+      <c r="D118" s="56"/>
+      <c r="E118" s="56"/>
+      <c r="F118" s="56"/>
+      <c r="G118" s="56"/>
+      <c r="H118" s="56"/>
+      <c r="I118" s="56"/>
+      <c r="J118" s="56"/>
+      <c r="K118" s="57"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B119" s="71" t="s">
+      <c r="B119" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="C119" s="63"/>
-      <c r="D119" s="63"/>
-      <c r="E119" s="63"/>
-      <c r="F119" s="63"/>
-      <c r="G119" s="63"/>
-      <c r="H119" s="63"/>
-      <c r="I119" s="63"/>
-      <c r="J119" s="63"/>
-      <c r="K119" s="64"/>
+      <c r="C119" s="56"/>
+      <c r="D119" s="56"/>
+      <c r="E119" s="56"/>
+      <c r="F119" s="56"/>
+      <c r="G119" s="56"/>
+      <c r="H119" s="56"/>
+      <c r="I119" s="56"/>
+      <c r="J119" s="56"/>
+      <c r="K119" s="57"/>
     </row>
     <row r="120" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B120" s="71" t="s">
+      <c r="B120" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="63"/>
-      <c r="D120" s="63"/>
-      <c r="E120" s="63"/>
-      <c r="F120" s="63"/>
-      <c r="G120" s="63"/>
-      <c r="H120" s="63"/>
-      <c r="I120" s="63"/>
-      <c r="J120" s="63"/>
-      <c r="K120" s="64"/>
+      <c r="C120" s="56"/>
+      <c r="D120" s="56"/>
+      <c r="E120" s="56"/>
+      <c r="F120" s="56"/>
+      <c r="G120" s="56"/>
+      <c r="H120" s="56"/>
+      <c r="I120" s="56"/>
+      <c r="J120" s="56"/>
+      <c r="K120" s="57"/>
     </row>
     <row r="121" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A121" s="37">
@@ -6863,53 +6866,53 @@
       <c r="K152" s="46"/>
     </row>
     <row r="153" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="74" t="s">
+      <c r="A153" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B153" s="63"/>
-      <c r="C153" s="63"/>
-      <c r="D153" s="63"/>
-      <c r="E153" s="63"/>
-      <c r="F153" s="63"/>
-      <c r="G153" s="63"/>
-      <c r="H153" s="63"/>
-      <c r="I153" s="63"/>
-      <c r="J153" s="63"/>
-      <c r="K153" s="64"/>
+      <c r="B153" s="56"/>
+      <c r="C153" s="56"/>
+      <c r="D153" s="56"/>
+      <c r="E153" s="56"/>
+      <c r="F153" s="56"/>
+      <c r="G153" s="56"/>
+      <c r="H153" s="56"/>
+      <c r="I153" s="56"/>
+      <c r="J153" s="56"/>
+      <c r="K153" s="57"/>
     </row>
     <row r="154" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A154" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B154" s="75" t="s">
+      <c r="B154" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="C154" s="63"/>
-      <c r="D154" s="63"/>
-      <c r="E154" s="63"/>
-      <c r="F154" s="63"/>
-      <c r="G154" s="63"/>
-      <c r="H154" s="63"/>
-      <c r="I154" s="63"/>
-      <c r="J154" s="63"/>
-      <c r="K154" s="64"/>
+      <c r="C154" s="56"/>
+      <c r="D154" s="56"/>
+      <c r="E154" s="56"/>
+      <c r="F154" s="56"/>
+      <c r="G154" s="56"/>
+      <c r="H154" s="56"/>
+      <c r="I154" s="56"/>
+      <c r="J154" s="56"/>
+      <c r="K154" s="57"/>
     </row>
     <row r="155" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B155" s="75" t="s">
+      <c r="B155" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C155" s="63"/>
-      <c r="D155" s="63"/>
-      <c r="E155" s="63"/>
-      <c r="F155" s="63"/>
-      <c r="G155" s="63"/>
-      <c r="H155" s="63"/>
-      <c r="I155" s="63"/>
-      <c r="J155" s="63"/>
-      <c r="K155" s="64"/>
+      <c r="C155" s="56"/>
+      <c r="D155" s="56"/>
+      <c r="E155" s="56"/>
+      <c r="F155" s="56"/>
+      <c r="G155" s="56"/>
+      <c r="H155" s="56"/>
+      <c r="I155" s="56"/>
+      <c r="J155" s="56"/>
+      <c r="K155" s="57"/>
     </row>
     <row r="156" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A156" s="37">
@@ -8206,53 +8209,53 @@
       <c r="K196" s="46"/>
     </row>
     <row r="197" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A197" s="76" t="s">
+      <c r="A197" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="B197" s="63"/>
-      <c r="C197" s="63"/>
-      <c r="D197" s="63"/>
-      <c r="E197" s="63"/>
-      <c r="F197" s="63"/>
-      <c r="G197" s="63"/>
-      <c r="H197" s="63"/>
-      <c r="I197" s="63"/>
-      <c r="J197" s="63"/>
-      <c r="K197" s="64"/>
+      <c r="B197" s="56"/>
+      <c r="C197" s="56"/>
+      <c r="D197" s="56"/>
+      <c r="E197" s="56"/>
+      <c r="F197" s="56"/>
+      <c r="G197" s="56"/>
+      <c r="H197" s="56"/>
+      <c r="I197" s="56"/>
+      <c r="J197" s="56"/>
+      <c r="K197" s="57"/>
     </row>
     <row r="198" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A198" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B198" s="72" t="s">
+      <c r="B198" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C198" s="63"/>
-      <c r="D198" s="63"/>
-      <c r="E198" s="63"/>
-      <c r="F198" s="63"/>
-      <c r="G198" s="63"/>
-      <c r="H198" s="63"/>
-      <c r="I198" s="63"/>
-      <c r="J198" s="63"/>
-      <c r="K198" s="64"/>
+      <c r="C198" s="56"/>
+      <c r="D198" s="56"/>
+      <c r="E198" s="56"/>
+      <c r="F198" s="56"/>
+      <c r="G198" s="56"/>
+      <c r="H198" s="56"/>
+      <c r="I198" s="56"/>
+      <c r="J198" s="56"/>
+      <c r="K198" s="57"/>
     </row>
     <row r="199" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B199" s="72" t="s">
+      <c r="B199" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="C199" s="63"/>
-      <c r="D199" s="63"/>
-      <c r="E199" s="63"/>
-      <c r="F199" s="63"/>
-      <c r="G199" s="63"/>
-      <c r="H199" s="63"/>
-      <c r="I199" s="63"/>
-      <c r="J199" s="63"/>
-      <c r="K199" s="64"/>
+      <c r="C199" s="56"/>
+      <c r="D199" s="56"/>
+      <c r="E199" s="56"/>
+      <c r="F199" s="56"/>
+      <c r="G199" s="56"/>
+      <c r="H199" s="56"/>
+      <c r="I199" s="56"/>
+      <c r="J199" s="56"/>
+      <c r="K199" s="57"/>
     </row>
     <row r="200" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A200" s="37">
@@ -8880,53 +8883,53 @@
       <c r="K219" s="46"/>
     </row>
     <row r="220" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A220" s="73" t="s">
+      <c r="A220" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="B220" s="63"/>
-      <c r="C220" s="63"/>
-      <c r="D220" s="63"/>
-      <c r="E220" s="63"/>
-      <c r="F220" s="63"/>
-      <c r="G220" s="63"/>
-      <c r="H220" s="63"/>
-      <c r="I220" s="63"/>
-      <c r="J220" s="63"/>
-      <c r="K220" s="64"/>
+      <c r="B220" s="56"/>
+      <c r="C220" s="56"/>
+      <c r="D220" s="56"/>
+      <c r="E220" s="56"/>
+      <c r="F220" s="56"/>
+      <c r="G220" s="56"/>
+      <c r="H220" s="56"/>
+      <c r="I220" s="56"/>
+      <c r="J220" s="56"/>
+      <c r="K220" s="57"/>
     </row>
     <row r="221" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A221" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B221" s="70" t="s">
+      <c r="B221" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="C221" s="63"/>
-      <c r="D221" s="63"/>
-      <c r="E221" s="63"/>
-      <c r="F221" s="63"/>
-      <c r="G221" s="63"/>
-      <c r="H221" s="63"/>
-      <c r="I221" s="63"/>
-      <c r="J221" s="63"/>
-      <c r="K221" s="64"/>
+      <c r="C221" s="56"/>
+      <c r="D221" s="56"/>
+      <c r="E221" s="56"/>
+      <c r="F221" s="56"/>
+      <c r="G221" s="56"/>
+      <c r="H221" s="56"/>
+      <c r="I221" s="56"/>
+      <c r="J221" s="56"/>
+      <c r="K221" s="57"/>
     </row>
     <row r="222" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B222" s="70" t="s">
+      <c r="B222" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="C222" s="63"/>
-      <c r="D222" s="63"/>
-      <c r="E222" s="63"/>
-      <c r="F222" s="63"/>
-      <c r="G222" s="63"/>
-      <c r="H222" s="63"/>
-      <c r="I222" s="63"/>
-      <c r="J222" s="63"/>
-      <c r="K222" s="64"/>
+      <c r="C222" s="56"/>
+      <c r="D222" s="56"/>
+      <c r="E222" s="56"/>
+      <c r="F222" s="56"/>
+      <c r="G222" s="56"/>
+      <c r="H222" s="56"/>
+      <c r="I222" s="56"/>
+      <c r="J222" s="56"/>
+      <c r="K222" s="57"/>
     </row>
     <row r="223" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A223" s="37">
@@ -9585,53 +9588,53 @@
       <c r="K243" s="46"/>
     </row>
     <row r="244" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A244" s="55" t="s">
+      <c r="A244" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B244" s="56"/>
-      <c r="C244" s="56"/>
-      <c r="D244" s="56"/>
-      <c r="E244" s="56"/>
-      <c r="F244" s="56"/>
-      <c r="G244" s="56"/>
-      <c r="H244" s="56"/>
-      <c r="I244" s="56"/>
-      <c r="J244" s="56"/>
-      <c r="K244" s="57"/>
+      <c r="B244" s="64"/>
+      <c r="C244" s="64"/>
+      <c r="D244" s="64"/>
+      <c r="E244" s="64"/>
+      <c r="F244" s="64"/>
+      <c r="G244" s="64"/>
+      <c r="H244" s="64"/>
+      <c r="I244" s="64"/>
+      <c r="J244" s="64"/>
+      <c r="K244" s="65"/>
     </row>
     <row r="245" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A245" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B245" s="58" t="s">
+      <c r="B245" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="C245" s="56"/>
-      <c r="D245" s="56"/>
-      <c r="E245" s="56"/>
-      <c r="F245" s="56"/>
-      <c r="G245" s="56"/>
-      <c r="H245" s="56"/>
-      <c r="I245" s="56"/>
-      <c r="J245" s="56"/>
-      <c r="K245" s="57"/>
+      <c r="C245" s="64"/>
+      <c r="D245" s="64"/>
+      <c r="E245" s="64"/>
+      <c r="F245" s="64"/>
+      <c r="G245" s="64"/>
+      <c r="H245" s="64"/>
+      <c r="I245" s="64"/>
+      <c r="J245" s="64"/>
+      <c r="K245" s="65"/>
     </row>
     <row r="246" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A246" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B246" s="58" t="s">
+      <c r="B246" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="C246" s="56"/>
-      <c r="D246" s="56"/>
-      <c r="E246" s="56"/>
-      <c r="F246" s="56"/>
-      <c r="G246" s="56"/>
-      <c r="H246" s="56"/>
-      <c r="I246" s="56"/>
-      <c r="J246" s="56"/>
-      <c r="K246" s="57"/>
+      <c r="C246" s="64"/>
+      <c r="D246" s="64"/>
+      <c r="E246" s="64"/>
+      <c r="F246" s="64"/>
+      <c r="G246" s="64"/>
+      <c r="H246" s="64"/>
+      <c r="I246" s="64"/>
+      <c r="J246" s="64"/>
+      <c r="K246" s="65"/>
     </row>
     <row r="247" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A247" s="37">
@@ -9659,7 +9662,7 @@
         <v>0.5</v>
       </c>
       <c r="I247" s="41">
-        <f t="shared" ref="I247:I259" si="9">H247-G247</f>
+        <f t="shared" ref="I247:I261" si="9">H247-G247</f>
         <v>0</v>
       </c>
       <c r="J247" s="45"/>
@@ -9924,24 +9927,30 @@
       </c>
     </row>
     <row r="256" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A256" s="37"/>
+      <c r="A256" s="37">
+        <v>45678</v>
+      </c>
       <c r="B256" s="38" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C256" s="39" t="s">
-        <v>361</v>
+        <v>236</v>
       </c>
       <c r="D256" s="38" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="E256" s="40" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F256" s="40" t="s">
-        <v>365</v>
-      </c>
-      <c r="G256" s="41"/>
-      <c r="H256" s="41"/>
+        <v>104</v>
+      </c>
+      <c r="G256" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="H256" s="41">
+        <v>0.5</v>
+      </c>
       <c r="I256" s="41">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -9951,13 +9960,19 @@
     </row>
     <row r="257" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A257" s="37"/>
-      <c r="B257" s="38"/>
+      <c r="B257" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C257" s="39" t="s">
-        <v>17</v>
+        <v>236</v>
       </c>
       <c r="D257" s="38"/>
-      <c r="E257" s="40"/>
-      <c r="F257" s="40"/>
+      <c r="E257" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="F257" s="40" t="s">
+        <v>88</v>
+      </c>
       <c r="G257" s="41"/>
       <c r="H257" s="41"/>
       <c r="I257" s="41">
@@ -9969,13 +9984,21 @@
     </row>
     <row r="258" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A258" s="37"/>
-      <c r="B258" s="38"/>
+      <c r="B258" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C258" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D258" s="38"/>
-      <c r="E258" s="40"/>
-      <c r="F258" s="40"/>
+        <v>361</v>
+      </c>
+      <c r="D258" s="38" t="s">
+        <v>364</v>
+      </c>
+      <c r="E258" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="F258" s="40" t="s">
+        <v>365</v>
+      </c>
       <c r="G258" s="41"/>
       <c r="H258" s="41"/>
       <c r="I258" s="41">
@@ -9986,39 +10009,75 @@
       <c r="K258" s="43"/>
     </row>
     <row r="259" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A259" s="48"/>
-      <c r="B259" s="49"/>
-      <c r="C259" s="49"/>
-      <c r="D259" s="49"/>
-      <c r="E259" s="49" t="s">
+      <c r="A259" s="37"/>
+      <c r="B259" s="38"/>
+      <c r="C259" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D259" s="38"/>
+      <c r="E259" s="40"/>
+      <c r="F259" s="40"/>
+      <c r="G259" s="41"/>
+      <c r="H259" s="41"/>
+      <c r="I259" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J259" s="45"/>
+      <c r="K259" s="43"/>
+    </row>
+    <row r="260" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A260" s="37"/>
+      <c r="B260" s="38"/>
+      <c r="C260" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D260" s="38"/>
+      <c r="E260" s="40"/>
+      <c r="F260" s="40"/>
+      <c r="G260" s="41"/>
+      <c r="H260" s="41"/>
+      <c r="I260" s="41">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J260" s="45"/>
+      <c r="K260" s="43"/>
+    </row>
+    <row r="261" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A261" s="48"/>
+      <c r="B261" s="49"/>
+      <c r="C261" s="49"/>
+      <c r="D261" s="49"/>
+      <c r="E261" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F259" s="49"/>
-      <c r="G259" s="50">
-        <f t="shared" ref="G259:H259" si="10">SUM(G247:G258)</f>
-        <v>10</v>
-      </c>
-      <c r="H259" s="50">
+      <c r="F261" s="49"/>
+      <c r="G261" s="50">
+        <f t="shared" ref="G261:H261" si="10">SUM(G247:G260)</f>
+        <v>10.5</v>
+      </c>
+      <c r="H261" s="50">
         <f t="shared" si="10"/>
-        <v>10.25</v>
-      </c>
-      <c r="I259" s="50">
+        <v>10.75</v>
+      </c>
+      <c r="I261" s="50">
         <f t="shared" si="9"/>
         <v>0.25</v>
       </c>
-      <c r="J259" s="51"/>
-      <c r="K259" s="52"/>
-    </row>
-    <row r="260" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E260" s="40"/>
-    </row>
-    <row r="261" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G261" s="38" t="s">
+      <c r="J261" s="51"/>
+      <c r="K261" s="52"/>
+    </row>
+    <row r="262" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E262" s="40"/>
+    </row>
+    <row r="263" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G263" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="H261" s="54">
-        <f>H46+H82+H117+H152+H196+H219+H243+H259</f>
-        <v>206.79</v>
+      <c r="H263" s="54">
+        <f>H46+H82+H117+H152+H196+H219+H243+H261</f>
+        <v>207.29</v>
       </c>
     </row>
   </sheetData>
@@ -10026,7 +10085,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{A64F5071-78C5-46B1-9F42-0443704A2C92}">
+      <autoFilter ref="A1:K15" xr:uid="{76B1C689-22FA-402A-8A1F-50A615E4699E}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -10037,14 +10096,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B198:K198"/>
-    <mergeCell ref="B199:K199"/>
-    <mergeCell ref="A220:K220"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="A153:K153"/>
-    <mergeCell ref="B154:K154"/>
-    <mergeCell ref="B155:K155"/>
-    <mergeCell ref="A197:K197"/>
     <mergeCell ref="A244:K244"/>
     <mergeCell ref="B245:K245"/>
     <mergeCell ref="B246:K246"/>
@@ -10061,6 +10112,14 @@
     <mergeCell ref="B221:K221"/>
     <mergeCell ref="B222:K222"/>
     <mergeCell ref="B119:K119"/>
+    <mergeCell ref="B198:K198"/>
+    <mergeCell ref="B199:K199"/>
+    <mergeCell ref="A220:K220"/>
+    <mergeCell ref="B120:K120"/>
+    <mergeCell ref="A153:K153"/>
+    <mergeCell ref="B154:K154"/>
+    <mergeCell ref="B155:K155"/>
+    <mergeCell ref="A197:K197"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B45 B48:B81 B86:B116 B121:B151 B156:B195 B200:B218 B223:B242">
     <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Unplanned">
@@ -10079,7 +10138,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B152 B154:B196 B198:B219 B221:B243 B245:B259">
+  <conditionalFormatting sqref="B5:B46 B48:B82 B84:B117 B119:B152 B154:B196 B198:B219 B221:B243 B245:B261">
     <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -10087,7 +10146,7 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B247:B258">
+  <conditionalFormatting sqref="B247:B260">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B247))))</formula>
     </cfRule>
@@ -10104,17 +10163,17 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B247))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G152 G156:G196 G200:G219 G223:G243 G247:G259">
+  <conditionalFormatting sqref="G1 G3:G46 G50:G82 G86:G117 G121:G152 G156:G196 G200:G219 G223:G243 G247:G261">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H259">
+  <conditionalFormatting sqref="H1:H261">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I152 I156:I196 I200:I219 I223:I243 I247:I259">
+  <conditionalFormatting sqref="I5:I46 I50:I82 I86:I117 I121:I152 I156:I196 I200:I219 I223:I243 I247:I261">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -10123,7 +10182,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F247:F258 F86:F116 F5:F45 F50:F81 F121:F151 F156:F195 F200:F218 F223:F242" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F247:F260 F86:F116 F5:F45 F50:F81 F121:F151 F156:F195 F200:F218 F223:F242" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10140,13 +10199,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:E45 E86:E116 E247:E258 E50:E81 E121:E151 E156:E195 E200:E218 E223:E242</xm:sqref>
+          <xm:sqref>E5:E45 E86:E116 E247:E260 E50:E81 E121:E151 E156:E195 E200:E218 E223:E242</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B45 B86:B116 B247:B258 B50:B81 B121:B151 B156:B195 B200:B218 B223:B242</xm:sqref>
+          <xm:sqref>B5:B45 B86:B116 B247:B260 B50:B81 B121:B151 B156:B195 B200:B218 B223:B242</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -11787,6 +11846,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -12021,27 +12100,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12058,23 +12136,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Block A retake evidencing
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1FB65E-3215-48CB-9C09-1C1847BE51A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42A55F4-E33A-468A-9572-2CCF911F1307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1821,6 +1821,29 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1837,8 +1860,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1857,33 +1878,12 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2353,53 +2353,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
-      <c r="K2" s="61"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="70"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="62" t="s">
+      <c r="B3" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="64"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="58"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3734,53 +3734,53 @@
       <c r="K44" s="46"/>
     </row>
     <row r="45" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="65" t="s">
+      <c r="A45" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="B45" s="60"/>
-      <c r="C45" s="60"/>
-      <c r="D45" s="60"/>
-      <c r="E45" s="60"/>
-      <c r="F45" s="60"/>
-      <c r="G45" s="60"/>
-      <c r="H45" s="60"/>
-      <c r="I45" s="60"/>
-      <c r="J45" s="60"/>
-      <c r="K45" s="61"/>
+      <c r="B45" s="69"/>
+      <c r="C45" s="69"/>
+      <c r="D45" s="69"/>
+      <c r="E45" s="69"/>
+      <c r="F45" s="69"/>
+      <c r="G45" s="69"/>
+      <c r="H45" s="69"/>
+      <c r="I45" s="69"/>
+      <c r="J45" s="69"/>
+      <c r="K45" s="70"/>
     </row>
     <row r="46" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A46" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="66" t="s">
+      <c r="B46" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C46" s="63"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="63"/>
-      <c r="F46" s="63"/>
-      <c r="G46" s="63"/>
-      <c r="H46" s="63"/>
-      <c r="I46" s="63"/>
-      <c r="J46" s="63"/>
-      <c r="K46" s="64"/>
+      <c r="C46" s="57"/>
+      <c r="D46" s="57"/>
+      <c r="E46" s="57"/>
+      <c r="F46" s="57"/>
+      <c r="G46" s="57"/>
+      <c r="H46" s="57"/>
+      <c r="I46" s="57"/>
+      <c r="J46" s="57"/>
+      <c r="K46" s="58"/>
     </row>
     <row r="47" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B47" s="66" t="s">
+      <c r="B47" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="C47" s="63"/>
-      <c r="D47" s="63"/>
-      <c r="E47" s="63"/>
-      <c r="F47" s="63"/>
-      <c r="G47" s="63"/>
-      <c r="H47" s="63"/>
-      <c r="I47" s="63"/>
-      <c r="J47" s="63"/>
-      <c r="K47" s="64"/>
+      <c r="C47" s="57"/>
+      <c r="D47" s="57"/>
+      <c r="E47" s="57"/>
+      <c r="F47" s="57"/>
+      <c r="G47" s="57"/>
+      <c r="H47" s="57"/>
+      <c r="I47" s="57"/>
+      <c r="J47" s="57"/>
+      <c r="K47" s="58"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="47">
@@ -4843,53 +4843,53 @@
       <c r="K79" s="46"/>
     </row>
     <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="67" t="s">
+      <c r="A80" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="B80" s="63"/>
-      <c r="C80" s="63"/>
-      <c r="D80" s="63"/>
-      <c r="E80" s="63"/>
-      <c r="F80" s="63"/>
-      <c r="G80" s="63"/>
-      <c r="H80" s="63"/>
-      <c r="I80" s="63"/>
-      <c r="J80" s="63"/>
-      <c r="K80" s="64"/>
+      <c r="B80" s="57"/>
+      <c r="C80" s="57"/>
+      <c r="D80" s="57"/>
+      <c r="E80" s="57"/>
+      <c r="F80" s="57"/>
+      <c r="G80" s="57"/>
+      <c r="H80" s="57"/>
+      <c r="I80" s="57"/>
+      <c r="J80" s="57"/>
+      <c r="K80" s="58"/>
     </row>
     <row r="81" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A81" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B81" s="68" t="s">
+      <c r="B81" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C81" s="63"/>
-      <c r="D81" s="63"/>
-      <c r="E81" s="63"/>
-      <c r="F81" s="63"/>
-      <c r="G81" s="63"/>
-      <c r="H81" s="63"/>
-      <c r="I81" s="63"/>
-      <c r="J81" s="63"/>
-      <c r="K81" s="64"/>
+      <c r="C81" s="57"/>
+      <c r="D81" s="57"/>
+      <c r="E81" s="57"/>
+      <c r="F81" s="57"/>
+      <c r="G81" s="57"/>
+      <c r="H81" s="57"/>
+      <c r="I81" s="57"/>
+      <c r="J81" s="57"/>
+      <c r="K81" s="58"/>
     </row>
     <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="68" t="s">
+      <c r="B82" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C82" s="63"/>
-      <c r="D82" s="63"/>
-      <c r="E82" s="63"/>
-      <c r="F82" s="63"/>
-      <c r="G82" s="63"/>
-      <c r="H82" s="63"/>
-      <c r="I82" s="63"/>
-      <c r="J82" s="63"/>
-      <c r="K82" s="64"/>
+      <c r="C82" s="57"/>
+      <c r="D82" s="57"/>
+      <c r="E82" s="57"/>
+      <c r="F82" s="57"/>
+      <c r="G82" s="57"/>
+      <c r="H82" s="57"/>
+      <c r="I82" s="57"/>
+      <c r="J82" s="57"/>
+      <c r="K82" s="58"/>
     </row>
     <row r="83" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A83" s="37">
@@ -5926,53 +5926,53 @@
       <c r="K113" s="46"/>
     </row>
     <row r="114" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="69" t="s">
+      <c r="A114" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="B114" s="63"/>
-      <c r="C114" s="63"/>
-      <c r="D114" s="63"/>
-      <c r="E114" s="63"/>
-      <c r="F114" s="63"/>
-      <c r="G114" s="63"/>
-      <c r="H114" s="63"/>
-      <c r="I114" s="63"/>
-      <c r="J114" s="63"/>
-      <c r="K114" s="64"/>
+      <c r="B114" s="57"/>
+      <c r="C114" s="57"/>
+      <c r="D114" s="57"/>
+      <c r="E114" s="57"/>
+      <c r="F114" s="57"/>
+      <c r="G114" s="57"/>
+      <c r="H114" s="57"/>
+      <c r="I114" s="57"/>
+      <c r="J114" s="57"/>
+      <c r="K114" s="58"/>
     </row>
     <row r="115" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A115" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B115" s="71" t="s">
+      <c r="B115" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C115" s="63"/>
-      <c r="D115" s="63"/>
-      <c r="E115" s="63"/>
-      <c r="F115" s="63"/>
-      <c r="G115" s="63"/>
-      <c r="H115" s="63"/>
-      <c r="I115" s="63"/>
-      <c r="J115" s="63"/>
-      <c r="K115" s="64"/>
+      <c r="C115" s="57"/>
+      <c r="D115" s="57"/>
+      <c r="E115" s="57"/>
+      <c r="F115" s="57"/>
+      <c r="G115" s="57"/>
+      <c r="H115" s="57"/>
+      <c r="I115" s="57"/>
+      <c r="J115" s="57"/>
+      <c r="K115" s="58"/>
     </row>
     <row r="116" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B116" s="71" t="s">
+      <c r="B116" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C116" s="63"/>
-      <c r="D116" s="63"/>
-      <c r="E116" s="63"/>
-      <c r="F116" s="63"/>
-      <c r="G116" s="63"/>
-      <c r="H116" s="63"/>
-      <c r="I116" s="63"/>
-      <c r="J116" s="63"/>
-      <c r="K116" s="64"/>
+      <c r="C116" s="57"/>
+      <c r="D116" s="57"/>
+      <c r="E116" s="57"/>
+      <c r="F116" s="57"/>
+      <c r="G116" s="57"/>
+      <c r="H116" s="57"/>
+      <c r="I116" s="57"/>
+      <c r="J116" s="57"/>
+      <c r="K116" s="58"/>
     </row>
     <row r="117" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A117" s="37">
@@ -6975,53 +6975,53 @@
       <c r="K146" s="46"/>
     </row>
     <row r="147" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="74" t="s">
+      <c r="A147" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="B147" s="63"/>
-      <c r="C147" s="63"/>
-      <c r="D147" s="63"/>
-      <c r="E147" s="63"/>
-      <c r="F147" s="63"/>
-      <c r="G147" s="63"/>
-      <c r="H147" s="63"/>
-      <c r="I147" s="63"/>
-      <c r="J147" s="63"/>
-      <c r="K147" s="64"/>
+      <c r="B147" s="57"/>
+      <c r="C147" s="57"/>
+      <c r="D147" s="57"/>
+      <c r="E147" s="57"/>
+      <c r="F147" s="57"/>
+      <c r="G147" s="57"/>
+      <c r="H147" s="57"/>
+      <c r="I147" s="57"/>
+      <c r="J147" s="57"/>
+      <c r="K147" s="58"/>
     </row>
     <row r="148" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A148" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B148" s="75" t="s">
+      <c r="B148" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C148" s="63"/>
-      <c r="D148" s="63"/>
-      <c r="E148" s="63"/>
-      <c r="F148" s="63"/>
-      <c r="G148" s="63"/>
-      <c r="H148" s="63"/>
-      <c r="I148" s="63"/>
-      <c r="J148" s="63"/>
-      <c r="K148" s="64"/>
+      <c r="C148" s="57"/>
+      <c r="D148" s="57"/>
+      <c r="E148" s="57"/>
+      <c r="F148" s="57"/>
+      <c r="G148" s="57"/>
+      <c r="H148" s="57"/>
+      <c r="I148" s="57"/>
+      <c r="J148" s="57"/>
+      <c r="K148" s="58"/>
     </row>
     <row r="149" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B149" s="75" t="s">
+      <c r="B149" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="C149" s="63"/>
-      <c r="D149" s="63"/>
-      <c r="E149" s="63"/>
-      <c r="F149" s="63"/>
-      <c r="G149" s="63"/>
-      <c r="H149" s="63"/>
-      <c r="I149" s="63"/>
-      <c r="J149" s="63"/>
-      <c r="K149" s="64"/>
+      <c r="C149" s="57"/>
+      <c r="D149" s="57"/>
+      <c r="E149" s="57"/>
+      <c r="F149" s="57"/>
+      <c r="G149" s="57"/>
+      <c r="H149" s="57"/>
+      <c r="I149" s="57"/>
+      <c r="J149" s="57"/>
+      <c r="K149" s="58"/>
     </row>
     <row r="150" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A150" s="37">
@@ -8364,53 +8364,53 @@
       <c r="K189" s="46"/>
     </row>
     <row r="190" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="76" t="s">
+      <c r="A190" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="B190" s="63"/>
-      <c r="C190" s="63"/>
-      <c r="D190" s="63"/>
-      <c r="E190" s="63"/>
-      <c r="F190" s="63"/>
-      <c r="G190" s="63"/>
-      <c r="H190" s="63"/>
-      <c r="I190" s="63"/>
-      <c r="J190" s="63"/>
-      <c r="K190" s="64"/>
+      <c r="B190" s="57"/>
+      <c r="C190" s="57"/>
+      <c r="D190" s="57"/>
+      <c r="E190" s="57"/>
+      <c r="F190" s="57"/>
+      <c r="G190" s="57"/>
+      <c r="H190" s="57"/>
+      <c r="I190" s="57"/>
+      <c r="J190" s="57"/>
+      <c r="K190" s="58"/>
     </row>
     <row r="191" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A191" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B191" s="72" t="s">
+      <c r="B191" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="C191" s="63"/>
-      <c r="D191" s="63"/>
-      <c r="E191" s="63"/>
-      <c r="F191" s="63"/>
-      <c r="G191" s="63"/>
-      <c r="H191" s="63"/>
-      <c r="I191" s="63"/>
-      <c r="J191" s="63"/>
-      <c r="K191" s="64"/>
+      <c r="C191" s="57"/>
+      <c r="D191" s="57"/>
+      <c r="E191" s="57"/>
+      <c r="F191" s="57"/>
+      <c r="G191" s="57"/>
+      <c r="H191" s="57"/>
+      <c r="I191" s="57"/>
+      <c r="J191" s="57"/>
+      <c r="K191" s="58"/>
     </row>
     <row r="192" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B192" s="72" t="s">
+      <c r="B192" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C192" s="63"/>
-      <c r="D192" s="63"/>
-      <c r="E192" s="63"/>
-      <c r="F192" s="63"/>
-      <c r="G192" s="63"/>
-      <c r="H192" s="63"/>
-      <c r="I192" s="63"/>
-      <c r="J192" s="63"/>
-      <c r="K192" s="64"/>
+      <c r="C192" s="57"/>
+      <c r="D192" s="57"/>
+      <c r="E192" s="57"/>
+      <c r="F192" s="57"/>
+      <c r="G192" s="57"/>
+      <c r="H192" s="57"/>
+      <c r="I192" s="57"/>
+      <c r="J192" s="57"/>
+      <c r="K192" s="58"/>
     </row>
     <row r="193" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A193" s="37">
@@ -9048,53 +9048,53 @@
       <c r="K211" s="46"/>
     </row>
     <row r="212" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A212" s="73" t="s">
+      <c r="A212" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="B212" s="63"/>
-      <c r="C212" s="63"/>
-      <c r="D212" s="63"/>
-      <c r="E212" s="63"/>
-      <c r="F212" s="63"/>
-      <c r="G212" s="63"/>
-      <c r="H212" s="63"/>
-      <c r="I212" s="63"/>
-      <c r="J212" s="63"/>
-      <c r="K212" s="64"/>
+      <c r="B212" s="57"/>
+      <c r="C212" s="57"/>
+      <c r="D212" s="57"/>
+      <c r="E212" s="57"/>
+      <c r="F212" s="57"/>
+      <c r="G212" s="57"/>
+      <c r="H212" s="57"/>
+      <c r="I212" s="57"/>
+      <c r="J212" s="57"/>
+      <c r="K212" s="58"/>
     </row>
     <row r="213" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A213" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B213" s="70" t="s">
+      <c r="B213" s="77" t="s">
         <v>13</v>
       </c>
-      <c r="C213" s="63"/>
-      <c r="D213" s="63"/>
-      <c r="E213" s="63"/>
-      <c r="F213" s="63"/>
-      <c r="G213" s="63"/>
-      <c r="H213" s="63"/>
-      <c r="I213" s="63"/>
-      <c r="J213" s="63"/>
-      <c r="K213" s="64"/>
+      <c r="C213" s="57"/>
+      <c r="D213" s="57"/>
+      <c r="E213" s="57"/>
+      <c r="F213" s="57"/>
+      <c r="G213" s="57"/>
+      <c r="H213" s="57"/>
+      <c r="I213" s="57"/>
+      <c r="J213" s="57"/>
+      <c r="K213" s="58"/>
     </row>
     <row r="214" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B214" s="70" t="s">
+      <c r="B214" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="C214" s="63"/>
-      <c r="D214" s="63"/>
-      <c r="E214" s="63"/>
-      <c r="F214" s="63"/>
-      <c r="G214" s="63"/>
-      <c r="H214" s="63"/>
-      <c r="I214" s="63"/>
-      <c r="J214" s="63"/>
-      <c r="K214" s="64"/>
+      <c r="C214" s="57"/>
+      <c r="D214" s="57"/>
+      <c r="E214" s="57"/>
+      <c r="F214" s="57"/>
+      <c r="G214" s="57"/>
+      <c r="H214" s="57"/>
+      <c r="I214" s="57"/>
+      <c r="J214" s="57"/>
+      <c r="K214" s="58"/>
     </row>
     <row r="215" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A215" s="37">
@@ -9387,7 +9387,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J223" s="80" t="s">
+      <c r="J223" s="55" t="s">
         <v>405</v>
       </c>
     </row>
@@ -9420,7 +9420,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J224" s="80" t="s">
+      <c r="J224" s="55" t="s">
         <v>372</v>
       </c>
     </row>
@@ -9453,7 +9453,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J225" s="80" t="s">
+      <c r="J225" s="55" t="s">
         <v>372</v>
       </c>
     </row>
@@ -9552,7 +9552,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J228" s="80" t="s">
+      <c r="J228" s="55" t="s">
         <v>405</v>
       </c>
     </row>
@@ -9787,53 +9787,53 @@
       <c r="K235" s="46"/>
     </row>
     <row r="236" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A236" s="55" t="s">
+      <c r="A236" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="B236" s="56"/>
-      <c r="C236" s="56"/>
-      <c r="D236" s="56"/>
-      <c r="E236" s="56"/>
-      <c r="F236" s="56"/>
-      <c r="G236" s="56"/>
-      <c r="H236" s="56"/>
-      <c r="I236" s="56"/>
-      <c r="J236" s="56"/>
-      <c r="K236" s="57"/>
+      <c r="B236" s="65"/>
+      <c r="C236" s="65"/>
+      <c r="D236" s="65"/>
+      <c r="E236" s="65"/>
+      <c r="F236" s="65"/>
+      <c r="G236" s="65"/>
+      <c r="H236" s="65"/>
+      <c r="I236" s="65"/>
+      <c r="J236" s="65"/>
+      <c r="K236" s="66"/>
     </row>
     <row r="237" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A237" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B237" s="58" t="s">
+      <c r="B237" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C237" s="56"/>
-      <c r="D237" s="56"/>
-      <c r="E237" s="56"/>
-      <c r="F237" s="56"/>
-      <c r="G237" s="56"/>
-      <c r="H237" s="56"/>
-      <c r="I237" s="56"/>
-      <c r="J237" s="56"/>
-      <c r="K237" s="57"/>
+      <c r="C237" s="65"/>
+      <c r="D237" s="65"/>
+      <c r="E237" s="65"/>
+      <c r="F237" s="65"/>
+      <c r="G237" s="65"/>
+      <c r="H237" s="65"/>
+      <c r="I237" s="65"/>
+      <c r="J237" s="65"/>
+      <c r="K237" s="66"/>
     </row>
     <row r="238" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B238" s="58" t="s">
+      <c r="B238" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C238" s="56"/>
-      <c r="D238" s="56"/>
-      <c r="E238" s="56"/>
-      <c r="F238" s="56"/>
-      <c r="G238" s="56"/>
-      <c r="H238" s="56"/>
-      <c r="I238" s="56"/>
-      <c r="J238" s="56"/>
-      <c r="K238" s="57"/>
+      <c r="C238" s="65"/>
+      <c r="D238" s="65"/>
+      <c r="E238" s="65"/>
+      <c r="F238" s="65"/>
+      <c r="G238" s="65"/>
+      <c r="H238" s="65"/>
+      <c r="I238" s="65"/>
+      <c r="J238" s="65"/>
+      <c r="K238" s="66"/>
     </row>
     <row r="239" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A239" s="37">
@@ -9864,7 +9864,7 @@
         <f t="shared" ref="I239:I261" si="8">H239-G239</f>
         <v>0</v>
       </c>
-      <c r="J239" s="80" t="s">
+      <c r="J239" s="55" t="s">
         <v>405</v>
       </c>
       <c r="K239" s="43"/>
@@ -10324,7 +10324,7 @@
         <v>45680</v>
       </c>
       <c r="B254" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C254" s="39" t="s">
         <v>315</v>
@@ -10341,10 +10341,12 @@
       <c r="G254" s="41">
         <v>0.25</v>
       </c>
-      <c r="H254" s="41"/>
+      <c r="H254" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I254" s="41">
         <f t="shared" si="8"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J254" s="45"/>
       <c r="K254" s="43"/>
@@ -10520,11 +10522,11 @@
       </c>
       <c r="H261" s="50">
         <f t="shared" si="9"/>
-        <v>21.75</v>
+        <v>22</v>
       </c>
       <c r="I261" s="50">
         <f t="shared" si="8"/>
-        <v>-4.5</v>
+        <v>-4.25</v>
       </c>
       <c r="J261" s="51"/>
       <c r="K261" s="52"/>
@@ -10538,7 +10540,7 @@
       </c>
       <c r="H263" s="54">
         <f>H44+H79+H113+H146+H189+H211+H235+H261</f>
-        <v>249.33999999999997</v>
+        <v>249.58999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -10546,7 +10548,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{4EFFB633-5705-4017-A0AB-5A9CD769A4BF}">
+      <autoFilter ref="A1:K15" xr:uid="{9D9A2EF4-6DF7-4017-B6F7-BC8B2F6AC336}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -10557,14 +10559,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B191:K191"/>
-    <mergeCell ref="B192:K192"/>
-    <mergeCell ref="A212:K212"/>
-    <mergeCell ref="B116:K116"/>
-    <mergeCell ref="A147:K147"/>
-    <mergeCell ref="B148:K148"/>
-    <mergeCell ref="B149:K149"/>
-    <mergeCell ref="A190:K190"/>
     <mergeCell ref="A236:K236"/>
     <mergeCell ref="B237:K237"/>
     <mergeCell ref="B238:K238"/>
@@ -10581,8 +10575,16 @@
     <mergeCell ref="B213:K213"/>
     <mergeCell ref="B214:K214"/>
     <mergeCell ref="B115:K115"/>
+    <mergeCell ref="B191:K191"/>
+    <mergeCell ref="B192:K192"/>
+    <mergeCell ref="A212:K212"/>
+    <mergeCell ref="B116:K116"/>
+    <mergeCell ref="A147:K147"/>
+    <mergeCell ref="B148:K148"/>
+    <mergeCell ref="B149:K149"/>
+    <mergeCell ref="A190:K190"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B43 B46:B78 B83:B112 B117:B145 B215:B234 B150:B188 B193:B210 B239:B260">
+  <conditionalFormatting sqref="B5:B43 B46:B78 B83:B112 B117:B145 B150:B188 B193:B210 B215:B234 B239:B260">
     <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -10599,7 +10601,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B44 B46:B79 B81:B113 B115:B146 B213:B235 B148:B189 B191:B211 B237:B261">
+  <conditionalFormatting sqref="B5:B44 B46:B79 B81:B113 B115:B146 B148:B189 B191:B211 B213:B235 B237:B261">
     <cfRule type="containsText" dxfId="5" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -10607,7 +10609,7 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G44 G48:G79 G83:G113 G117:G146 G215:G235 G150:G189 G193:G211 G239:G261">
+  <conditionalFormatting sqref="G1 G3:G44 G48:G79 G83:G113 G117:G146 G150:G189 G193:G211 G215:G235 G239:G261">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
@@ -10617,7 +10619,7 @@
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I44 I48:I79 I83:I113 I117:I146 I215:I235 I150:I189 I193:I211 I239:I261">
+  <conditionalFormatting sqref="I5:I44 I48:I79 I83:I113 I117:I146 I150:I189 I193:I211 I215:I235 I239:I261">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -11174,58 +11176,58 @@
       <c r="K13" s="17"/>
     </row>
     <row r="14" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="77" t="s">
+      <c r="B14" s="78" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="78"/>
-      <c r="D14" s="78"/>
-      <c r="E14" s="78"/>
-      <c r="F14" s="78"/>
-      <c r="G14" s="78"/>
-      <c r="H14" s="78"/>
-      <c r="I14" s="78"/>
-      <c r="J14" s="78"/>
-      <c r="K14" s="78"/>
+      <c r="C14" s="79"/>
+      <c r="D14" s="79"/>
+      <c r="E14" s="79"/>
+      <c r="F14" s="79"/>
+      <c r="G14" s="79"/>
+      <c r="H14" s="79"/>
+      <c r="I14" s="79"/>
+      <c r="J14" s="79"/>
+      <c r="K14" s="79"/>
     </row>
     <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="9"/>
     </row>
     <row r="19" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="79" t="s">
+      <c r="B19" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="79"/>
-      <c r="D19" s="79"/>
-      <c r="E19" s="79"/>
-      <c r="F19" s="79"/>
+      <c r="C19" s="80"/>
+      <c r="D19" s="80"/>
+      <c r="E19" s="80"/>
+      <c r="F19" s="80"/>
     </row>
     <row r="20" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="79"/>
-      <c r="C20" s="79"/>
-      <c r="D20" s="79"/>
-      <c r="E20" s="79"/>
-      <c r="F20" s="79"/>
+      <c r="B20" s="80"/>
+      <c r="C20" s="80"/>
+      <c r="D20" s="80"/>
+      <c r="E20" s="80"/>
+      <c r="F20" s="80"/>
     </row>
     <row r="21" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="79"/>
-      <c r="C21" s="79"/>
-      <c r="D21" s="79"/>
-      <c r="E21" s="79"/>
-      <c r="F21" s="79"/>
+      <c r="B21" s="80"/>
+      <c r="C21" s="80"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="80"/>
     </row>
     <row r="22" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="79"/>
-      <c r="C22" s="79"/>
-      <c r="D22" s="79"/>
-      <c r="E22" s="79"/>
-      <c r="F22" s="79"/>
+      <c r="B22" s="80"/>
+      <c r="C22" s="80"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="80"/>
+      <c r="F22" s="80"/>
     </row>
     <row r="23" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="79"/>
-      <c r="C23" s="79"/>
-      <c r="D23" s="79"/>
-      <c r="E23" s="79"/>
-      <c r="F23" s="79"/>
+      <c r="B23" s="80"/>
+      <c r="C23" s="80"/>
+      <c r="D23" s="80"/>
+      <c r="E23" s="80"/>
+      <c r="F23" s="80"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -12382,6 +12384,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -12616,27 +12638,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12653,23 +12674,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
WorkLog & Learning Log complete
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42A55F4-E33A-468A-9572-2CCF911F1307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2AA9278-1F75-4DAA-A66F-6F2B1B008347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1390" uniqueCount="416">
   <si>
     <t>Date</t>
   </si>
@@ -1181,9 +1181,6 @@
     <t>Finish WorkLog</t>
   </si>
   <si>
-    <t>Finish Learning Log</t>
-  </si>
-  <si>
     <t>Finish Self-assesment rubric</t>
   </si>
   <si>
@@ -1202,9 +1199,6 @@
     <t>https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/tree/0e7620868343501c8dfcfa39189c1d60ae3a3b5e/Old%20Python%20Files</t>
   </si>
   <si>
-    <t>AAA</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894 </t>
   </si>
   <si>
@@ -1226,9 +1220,6 @@
     <t>I had the content fresh in my mind so I did this quicker than expected.</t>
   </si>
   <si>
-    <t>I'm still not too sure about the SMATER goals. AAA</t>
-  </si>
-  <si>
     <t>https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/0e7620868343501c8dfcfa39189c1d60ae3a3b5e/Block%20B/2024-11-25.png</t>
   </si>
   <si>
@@ -1329,6 +1320,36 @@
   </si>
   <si>
     <t>Hand in Block A retake again with all documents, just to be sure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/641210492f586c7e7048ca3999cc3dd4c452cfa2/Block%20B/Submission%20History%20-%20Project%201A%202024-2025%20-%20Breda%20University%20of%20Applied%20Sciences%20(1).pdf </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/641210492f586c7e7048ca3999cc3dd4c452cfa2/Block%20B/Final%20Presentation.pptx </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/641210492f586c7e7048ca3999cc3dd4c452cfa2/Deliverables/CreativeBrief_MaksBurchard_240894.ipynb </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/641210492f586c7e7048ca3999cc3dd4c452cfa2/Deliverables/FinalReport_Maks_Burchard_240894.docx </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/641210492f586c7e7048ca3999cc3dd4c452cfa2/Block%20B/AlgebraicExample_Final.ipynb </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/641210492f586c7e7048ca3999cc3dd4c452cfa2/Block%20B/LogisticRegression_Final.ipynb </t>
+  </si>
+  <si>
+    <t>Finish Learning Log section A and B</t>
+  </si>
+  <si>
+    <t>Finish Learning Log section C</t>
+  </si>
+  <si>
+    <t>I'm still not too sure about the SMATER goals.</t>
+  </si>
+  <si>
+    <t>Finish Learning Log section D</t>
   </si>
 </sst>
 </file>
@@ -2301,7 +2322,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K263"/>
+  <dimension ref="A1:K265"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -2529,7 +2550,7 @@
         <v>-0.5</v>
       </c>
       <c r="J8" s="53" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="K8" s="44"/>
     </row>
@@ -2663,7 +2684,7 @@
         <v>-0.25</v>
       </c>
       <c r="J12" s="53" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="K12" s="44"/>
     </row>
@@ -2729,7 +2750,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="53" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="K14" s="44"/>
     </row>
@@ -2763,9 +2784,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="45"/>
-      <c r="K15" s="44" t="s">
-        <v>366</v>
-      </c>
+      <c r="K15" s="44"/>
     </row>
     <row r="16" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A16" s="37">
@@ -2797,7 +2816,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="53" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K16" s="44"/>
     </row>
@@ -2832,7 +2851,7 @@
       </c>
       <c r="J17" s="45"/>
       <c r="K17" s="44" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -2865,9 +2884,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="45"/>
-      <c r="K18" s="44" t="s">
-        <v>366</v>
-      </c>
+      <c r="K18" s="44"/>
     </row>
     <row r="19" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A19" s="37">
@@ -2899,7 +2916,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="53" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K19" s="44"/>
     </row>
@@ -2948,7 +2965,7 @@
         <v>227</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="E21" s="40" t="s">
         <v>49</v>
@@ -2967,7 +2984,7 @@
         <v>0</v>
       </c>
       <c r="J21" s="53" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="K21" s="44"/>
     </row>
@@ -3033,9 +3050,7 @@
         <v>0</v>
       </c>
       <c r="J23" s="45"/>
-      <c r="K23" s="44" t="s">
-        <v>366</v>
-      </c>
+      <c r="K23" s="44"/>
     </row>
     <row r="24" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A24" s="37">
@@ -3067,7 +3082,7 @@
         <v>0</v>
       </c>
       <c r="J24" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K24" s="44"/>
     </row>
@@ -3101,7 +3116,7 @@
         <v>0</v>
       </c>
       <c r="J25" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K25" s="44"/>
     </row>
@@ -3135,7 +3150,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K26" s="44"/>
     </row>
@@ -3169,7 +3184,7 @@
         <v>0</v>
       </c>
       <c r="J27" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K27" s="44"/>
     </row>
@@ -3203,7 +3218,7 @@
         <v>0</v>
       </c>
       <c r="J28" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K28" s="44"/>
     </row>
@@ -3240,7 +3255,7 @@
         <v>105</v>
       </c>
       <c r="K29" s="44" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -3273,7 +3288,7 @@
         <v>0</v>
       </c>
       <c r="J30" s="53" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K30" s="44"/>
     </row>
@@ -3307,9 +3322,7 @@
         <v>0</v>
       </c>
       <c r="J31" s="45"/>
-      <c r="K31" s="44" t="s">
-        <v>366</v>
-      </c>
+      <c r="K31" s="44"/>
     </row>
     <row r="32" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A32" s="37">
@@ -3535,7 +3548,7 @@
         <v>0</v>
       </c>
       <c r="J38" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K38" s="44"/>
     </row>
@@ -3569,7 +3582,7 @@
         <v>0</v>
       </c>
       <c r="J39" s="53" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="K39" s="44" t="s">
         <v>139</v>
@@ -3605,7 +3618,7 @@
         <v>0</v>
       </c>
       <c r="J40" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K40" s="44"/>
     </row>
@@ -3639,9 +3652,7 @@
         <v>0</v>
       </c>
       <c r="J41" s="45"/>
-      <c r="K41" s="44" t="s">
-        <v>366</v>
-      </c>
+      <c r="K41" s="44"/>
     </row>
     <row r="42" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A42" s="37">
@@ -3705,9 +3716,7 @@
         <v>-0.35</v>
       </c>
       <c r="J43" s="45"/>
-      <c r="K43" s="44" t="s">
-        <v>366</v>
-      </c>
+      <c r="K43" s="44"/>
     </row>
     <row r="44" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A44" s="13"/>
@@ -3812,9 +3821,7 @@
         <v>0</v>
       </c>
       <c r="J48" s="45"/>
-      <c r="K48" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K48" s="43"/>
     </row>
     <row r="49" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A49" s="47">
@@ -3846,7 +3853,7 @@
         <v>0</v>
       </c>
       <c r="J49" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K49" s="43"/>
     </row>
@@ -3880,7 +3887,7 @@
         <v>0</v>
       </c>
       <c r="J50" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K50" s="43"/>
     </row>
@@ -3914,7 +3921,7 @@
         <v>0</v>
       </c>
       <c r="J51" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K51" s="43"/>
     </row>
@@ -3948,7 +3955,7 @@
         <v>0</v>
       </c>
       <c r="J52" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K52" s="43"/>
     </row>
@@ -3982,7 +3989,7 @@
         <v>0</v>
       </c>
       <c r="J53" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K53" s="43"/>
     </row>
@@ -4016,7 +4023,7 @@
         <v>0</v>
       </c>
       <c r="J54" s="53" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="K54" s="43"/>
     </row>
@@ -4050,9 +4057,7 @@
         <v>0</v>
       </c>
       <c r="J55" s="45"/>
-      <c r="K55" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K55" s="43"/>
     </row>
     <row r="56" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A56" s="47">
@@ -4150,7 +4155,7 @@
         <v>0</v>
       </c>
       <c r="J58" s="53" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="K58" s="43"/>
     </row>
@@ -4286,7 +4291,7 @@
         <v>-0.45000000000000018</v>
       </c>
       <c r="J62" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K62" s="43"/>
     </row>
@@ -4384,7 +4389,7 @@
         <v>0</v>
       </c>
       <c r="J65" s="53" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="K65" s="43"/>
     </row>
@@ -4450,7 +4455,7 @@
         <v>-0.25</v>
       </c>
       <c r="J67" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K67" s="43"/>
     </row>
@@ -4612,7 +4617,7 @@
         <v>-0.5</v>
       </c>
       <c r="J72" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K72" s="43"/>
     </row>
@@ -4678,9 +4683,7 @@
         <v>0</v>
       </c>
       <c r="J74" s="45"/>
-      <c r="K74" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K74" s="43"/>
     </row>
     <row r="75" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A75" s="47">
@@ -4713,7 +4716,7 @@
       </c>
       <c r="J75" s="45"/>
       <c r="K75" s="43" t="s">
-        <v>374</v>
+        <v>414</v>
       </c>
     </row>
     <row r="76" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -4746,9 +4749,7 @@
         <v>0</v>
       </c>
       <c r="J76" s="45"/>
-      <c r="K76" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K76" s="43"/>
     </row>
     <row r="77" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A77" s="47">
@@ -4780,9 +4781,7 @@
         <v>0</v>
       </c>
       <c r="J77" s="45"/>
-      <c r="K77" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K77" s="43"/>
     </row>
     <row r="78" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A78" s="47">
@@ -4814,9 +4813,7 @@
         <v>-0.1</v>
       </c>
       <c r="J78" s="45"/>
-      <c r="K78" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K78" s="43"/>
     </row>
     <row r="79" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A79" s="13"/>
@@ -4921,9 +4918,7 @@
         <v>0</v>
       </c>
       <c r="J83" s="45"/>
-      <c r="K83" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K83" s="43"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="37">
@@ -4955,9 +4950,7 @@
         <v>0</v>
       </c>
       <c r="J84" s="45"/>
-      <c r="K84" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K84" s="43"/>
     </row>
     <row r="85" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A85" s="37">
@@ -4989,7 +4982,7 @@
         <v>-0.5</v>
       </c>
       <c r="J85" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K85" s="43"/>
     </row>
@@ -5055,7 +5048,7 @@
         <v>-0.25</v>
       </c>
       <c r="J87" s="53" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="K87" s="43"/>
     </row>
@@ -5089,7 +5082,7 @@
         <v>-1</v>
       </c>
       <c r="J88" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K88" s="43"/>
     </row>
@@ -5155,7 +5148,7 @@
         <v>0.5</v>
       </c>
       <c r="J90" s="53" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="K90" s="43" t="s">
         <v>156</v>
@@ -5223,9 +5216,7 @@
         <v>0</v>
       </c>
       <c r="J92" s="45"/>
-      <c r="K92" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K92" s="43"/>
     </row>
     <row r="93" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A93" s="37">
@@ -5289,7 +5280,7 @@
         <v>1.5</v>
       </c>
       <c r="J94" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K94" s="43" t="s">
         <v>163</v>
@@ -5325,7 +5316,7 @@
         <v>0</v>
       </c>
       <c r="J95" s="53" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="K95" s="43"/>
     </row>
@@ -5359,7 +5350,7 @@
         <v>-0.5</v>
       </c>
       <c r="J96" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K96" s="43"/>
     </row>
@@ -5426,7 +5417,7 @@
       </c>
       <c r="J98" s="45"/>
       <c r="K98" s="43" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -5459,7 +5450,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K99" s="43"/>
     </row>
@@ -5493,7 +5484,7 @@
         <v>0</v>
       </c>
       <c r="J100" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K100" s="43"/>
     </row>
@@ -5527,7 +5518,7 @@
         <v>0</v>
       </c>
       <c r="J101" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K101" s="43"/>
     </row>
@@ -5561,7 +5552,7 @@
         <v>0</v>
       </c>
       <c r="J102" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K102" s="43"/>
     </row>
@@ -5595,7 +5586,7 @@
         <v>0</v>
       </c>
       <c r="J103" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K103" s="43"/>
     </row>
@@ -5693,7 +5684,7 @@
         <v>0</v>
       </c>
       <c r="J106" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K106" s="43"/>
     </row>
@@ -5759,7 +5750,7 @@
         <v>-1</v>
       </c>
       <c r="J108" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K108" s="43" t="s">
         <v>198</v>
@@ -5795,9 +5786,7 @@
         <v>0</v>
       </c>
       <c r="J109" s="45"/>
-      <c r="K109" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K109" s="43"/>
     </row>
     <row r="110" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A110" s="37">
@@ -5829,9 +5818,7 @@
         <v>0</v>
       </c>
       <c r="J110" s="45"/>
-      <c r="K110" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K110" s="43"/>
     </row>
     <row r="111" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A111" s="37">
@@ -5863,9 +5850,7 @@
         <v>-0.25</v>
       </c>
       <c r="J111" s="45"/>
-      <c r="K111" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K111" s="43"/>
     </row>
     <row r="112" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A112" s="37">
@@ -5897,9 +5882,7 @@
         <v>-0.25</v>
       </c>
       <c r="J112" s="45"/>
-      <c r="K112" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K112" s="43"/>
     </row>
     <row r="113" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A113" s="13"/>
@@ -6004,9 +5987,7 @@
         <v>0</v>
       </c>
       <c r="J117" s="45"/>
-      <c r="K117" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K117" s="43"/>
     </row>
     <row r="118" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A118" s="37">
@@ -6038,9 +6019,7 @@
         <v>0</v>
       </c>
       <c r="J118" s="45"/>
-      <c r="K118" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K118" s="43"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="37">
@@ -6072,7 +6051,7 @@
         <v>0</v>
       </c>
       <c r="J119" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K119" s="43"/>
     </row>
@@ -6106,7 +6085,7 @@
         <v>-0.5</v>
       </c>
       <c r="J120" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K120" s="43"/>
     </row>
@@ -6140,7 +6119,7 @@
         <v>-0.5</v>
       </c>
       <c r="J121" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K121" s="43"/>
     </row>
@@ -6174,7 +6153,7 @@
         <v>-0.5</v>
       </c>
       <c r="J122" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K122" s="43"/>
     </row>
@@ -6208,7 +6187,7 @@
         <v>-0.5</v>
       </c>
       <c r="J123" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K123" s="43"/>
     </row>
@@ -6274,7 +6253,7 @@
         <v>0</v>
       </c>
       <c r="J125" s="53" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="K125" s="43"/>
     </row>
@@ -6309,7 +6288,7 @@
       </c>
       <c r="J126" s="45"/>
       <c r="K126" s="43" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -6342,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="J127" s="53" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="K127" s="43"/>
     </row>
@@ -6408,7 +6387,7 @@
         <v>-0.5</v>
       </c>
       <c r="J129" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K129" s="43"/>
     </row>
@@ -6442,7 +6421,7 @@
         <v>-0.5</v>
       </c>
       <c r="J130" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K130" s="43"/>
     </row>
@@ -6476,7 +6455,7 @@
         <v>-0.5</v>
       </c>
       <c r="J131" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K131" s="43"/>
     </row>
@@ -6510,7 +6489,7 @@
         <v>-0.5</v>
       </c>
       <c r="J132" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K132" s="43"/>
     </row>
@@ -6544,7 +6523,7 @@
         <v>-0.5</v>
       </c>
       <c r="J133" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K133" s="43"/>
     </row>
@@ -6610,7 +6589,7 @@
         <v>0</v>
       </c>
       <c r="J135" s="53" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="K135" s="43"/>
     </row>
@@ -6676,10 +6655,10 @@
         <v>-1</v>
       </c>
       <c r="J137" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K137" s="43" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="138" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -6712,9 +6691,7 @@
         <v>0</v>
       </c>
       <c r="J138" s="45"/>
-      <c r="K138" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K138" s="43"/>
     </row>
     <row r="139" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A139" s="37">
@@ -6810,7 +6787,7 @@
         <v>0</v>
       </c>
       <c r="J141" s="53" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="K141" s="43"/>
     </row>
@@ -6844,7 +6821,7 @@
         <v>0</v>
       </c>
       <c r="J142" s="53" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="K142" s="43"/>
     </row>
@@ -6878,9 +6855,7 @@
         <v>0</v>
       </c>
       <c r="J143" s="45"/>
-      <c r="K143" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K143" s="43"/>
     </row>
     <row r="144" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A144" s="37">
@@ -6912,9 +6887,7 @@
         <v>-0.25</v>
       </c>
       <c r="J144" s="45"/>
-      <c r="K144" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K144" s="43"/>
     </row>
     <row r="145" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A145" s="37">
@@ -6946,9 +6919,7 @@
         <v>-0.25</v>
       </c>
       <c r="J145" s="45"/>
-      <c r="K145" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K145" s="43"/>
     </row>
     <row r="146" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A146" s="13"/>
@@ -7053,9 +7024,7 @@
         <v>0</v>
       </c>
       <c r="J150" s="45"/>
-      <c r="K150" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K150" s="43"/>
     </row>
     <row r="151" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A151" s="37">
@@ -7087,9 +7056,7 @@
         <v>0</v>
       </c>
       <c r="J151" s="45"/>
-      <c r="K151" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K151" s="43"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="37">
@@ -7121,7 +7088,7 @@
         <v>0</v>
       </c>
       <c r="J152" s="53" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="K152" s="43"/>
     </row>
@@ -7187,7 +7154,7 @@
         <v>-0.5</v>
       </c>
       <c r="J154" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K154" s="43"/>
     </row>
@@ -7221,7 +7188,7 @@
         <v>-0.5</v>
       </c>
       <c r="J155" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K155" s="43"/>
     </row>
@@ -7255,7 +7222,7 @@
         <v>-0.5</v>
       </c>
       <c r="J156" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K156" s="43"/>
     </row>
@@ -7289,7 +7256,7 @@
         <v>-0.5</v>
       </c>
       <c r="J157" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K157" s="43"/>
     </row>
@@ -7355,7 +7322,7 @@
         <v>-0.25</v>
       </c>
       <c r="J159" s="53" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="K159" s="43"/>
     </row>
@@ -7421,7 +7388,7 @@
         <v>-0.5</v>
       </c>
       <c r="J161" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K161" s="43"/>
     </row>
@@ -7455,7 +7422,7 @@
         <v>-1</v>
       </c>
       <c r="J162" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K162" s="43"/>
     </row>
@@ -7489,7 +7456,7 @@
         <v>-1</v>
       </c>
       <c r="J163" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K163" s="43"/>
     </row>
@@ -7523,7 +7490,7 @@
         <v>-1</v>
       </c>
       <c r="J164" s="53" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K164" s="43"/>
     </row>
@@ -7589,7 +7556,7 @@
         <v>0</v>
       </c>
       <c r="J166" s="53" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="K166" s="43"/>
     </row>
@@ -7623,9 +7590,7 @@
         <v>0</v>
       </c>
       <c r="J167" s="45"/>
-      <c r="K167" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K167" s="43"/>
     </row>
     <row r="168" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A168" s="37">
@@ -7689,9 +7654,7 @@
         <v>-0.5</v>
       </c>
       <c r="J169" s="45"/>
-      <c r="K169" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K169" s="43"/>
     </row>
     <row r="170" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A170" s="37">
@@ -7723,7 +7686,7 @@
         <v>0</v>
       </c>
       <c r="J170" s="53" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="K170" s="43"/>
     </row>
@@ -7757,7 +7720,7 @@
         <v>0.5</v>
       </c>
       <c r="J171" s="53" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="K171" s="43" t="s">
         <v>267</v>
@@ -7793,7 +7756,7 @@
         <v>0</v>
       </c>
       <c r="J172" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K172" s="43"/>
     </row>
@@ -7827,7 +7790,7 @@
         <v>0</v>
       </c>
       <c r="J173" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K173" s="43"/>
     </row>
@@ -7895,7 +7858,7 @@
         <v>-0.25</v>
       </c>
       <c r="J175" s="53" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="K175" s="43" t="s">
         <v>273</v>
@@ -7963,9 +7926,7 @@
         <v>0</v>
       </c>
       <c r="J177" s="45"/>
-      <c r="K177" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K177" s="43"/>
     </row>
     <row r="178" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A178" s="37">
@@ -8029,7 +7990,7 @@
         <v>2.25</v>
       </c>
       <c r="J179" s="53" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="K179" s="43" t="s">
         <v>325</v>
@@ -8097,7 +8058,7 @@
         <v>0</v>
       </c>
       <c r="J181" s="53" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="K181" s="43"/>
     </row>
@@ -8131,7 +8092,7 @@
         <v>0</v>
       </c>
       <c r="J182" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K182" s="43"/>
     </row>
@@ -8165,7 +8126,7 @@
         <v>0</v>
       </c>
       <c r="J183" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K183" s="43"/>
     </row>
@@ -8199,7 +8160,7 @@
         <v>0</v>
       </c>
       <c r="J184" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K184" s="43"/>
     </row>
@@ -8233,9 +8194,7 @@
         <v>-0.1</v>
       </c>
       <c r="J185" s="45"/>
-      <c r="K185" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K185" s="43"/>
     </row>
     <row r="186" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A186" s="37">
@@ -8267,9 +8226,7 @@
         <v>0</v>
       </c>
       <c r="J186" s="45"/>
-      <c r="K186" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K186" s="43"/>
     </row>
     <row r="187" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A187" s="37">
@@ -8301,9 +8258,7 @@
         <v>0</v>
       </c>
       <c r="J187" s="45"/>
-      <c r="K187" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K187" s="43"/>
     </row>
     <row r="188" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A188" s="37">
@@ -8335,9 +8290,7 @@
         <v>0</v>
       </c>
       <c r="J188" s="45"/>
-      <c r="K188" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K188" s="43"/>
     </row>
     <row r="189" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A189" s="13"/>
@@ -8442,9 +8395,7 @@
         <v>0</v>
       </c>
       <c r="J193" s="45"/>
-      <c r="K193" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K193" s="43"/>
     </row>
     <row r="194" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A194" s="37">
@@ -8476,9 +8427,7 @@
         <v>0</v>
       </c>
       <c r="J194" s="45"/>
-      <c r="K194" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K194" s="43"/>
     </row>
     <row r="195" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A195" s="37">
@@ -8541,7 +8490,7 @@
         <v>1.25</v>
       </c>
       <c r="J196" s="53" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="K196" s="43" t="s">
         <v>294</v>
@@ -8577,7 +8526,7 @@
         <v>1</v>
       </c>
       <c r="J197" s="53" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="K197" s="43"/>
     </row>
@@ -8643,7 +8592,7 @@
         <v>0</v>
       </c>
       <c r="J199" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K199" s="43"/>
     </row>
@@ -8677,7 +8626,7 @@
         <v>0</v>
       </c>
       <c r="J200" s="53" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K200" s="43"/>
     </row>
@@ -8711,7 +8660,7 @@
         <v>-0.5</v>
       </c>
       <c r="J201" s="53" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="K201" s="43"/>
     </row>
@@ -8877,7 +8826,7 @@
         <v>-0.5</v>
       </c>
       <c r="J206" s="53" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="K206" s="43" t="s">
         <v>318</v>
@@ -8913,7 +8862,7 @@
         <v>0.5</v>
       </c>
       <c r="J207" s="53" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="K207" s="43" t="s">
         <v>319</v>
@@ -8949,7 +8898,7 @@
         <v>2</v>
       </c>
       <c r="J208" s="53" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="K208" s="43" t="s">
         <v>350</v>
@@ -8985,9 +8934,7 @@
         <v>0</v>
       </c>
       <c r="J209" s="45"/>
-      <c r="K209" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K209" s="43"/>
     </row>
     <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A210" s="37">
@@ -9019,9 +8966,7 @@
         <v>0</v>
       </c>
       <c r="J210" s="45"/>
-      <c r="K210" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K210" s="43"/>
     </row>
     <row r="211" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A211" s="13"/>
@@ -9126,9 +9071,7 @@
         <v>0</v>
       </c>
       <c r="J215" s="45"/>
-      <c r="K215" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K215" s="43"/>
     </row>
     <row r="216" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A216" s="37">
@@ -9160,9 +9103,7 @@
         <v>0</v>
       </c>
       <c r="J216" s="45"/>
-      <c r="K216" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K216" s="43"/>
     </row>
     <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A217" s="37">
@@ -9322,9 +9263,7 @@
         <v>0</v>
       </c>
       <c r="J221" s="45"/>
-      <c r="K221" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K221" s="43"/>
     </row>
     <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A222" s="37">
@@ -9369,7 +9308,7 @@
         <v>315</v>
       </c>
       <c r="D223" s="38" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E223" s="40" t="s">
         <v>63</v>
@@ -9388,7 +9327,7 @@
         <v>0</v>
       </c>
       <c r="J223" s="55" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="224" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9421,7 +9360,7 @@
         <v>0</v>
       </c>
       <c r="J224" s="55" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="225" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9454,7 +9393,7 @@
         <v>0</v>
       </c>
       <c r="J225" s="55" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="226" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9487,9 +9426,7 @@
         <v>0</v>
       </c>
       <c r="J226" s="45"/>
-      <c r="K226" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K226" s="43"/>
     </row>
     <row r="227" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A227" s="37">
@@ -9553,7 +9490,7 @@
         <v>0</v>
       </c>
       <c r="J228" s="55" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="229" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9618,7 +9555,7 @@
         <v>1.75</v>
       </c>
       <c r="J230" s="53" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="K230" s="43" t="s">
         <v>351</v>
@@ -9654,7 +9591,7 @@
         <v>0.5</v>
       </c>
       <c r="J231" s="53" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="K231" s="43" t="s">
         <v>337</v>
@@ -9690,9 +9627,7 @@
         <v>0</v>
       </c>
       <c r="J232" s="45"/>
-      <c r="K232" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K232" s="43"/>
     </row>
     <row r="233" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A233" s="37">
@@ -9724,9 +9659,7 @@
         <v>0</v>
       </c>
       <c r="J233" s="45"/>
-      <c r="K233" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K233" s="43"/>
     </row>
     <row r="234" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A234" s="37">
@@ -9758,9 +9691,7 @@
         <v>-0.15</v>
       </c>
       <c r="J234" s="45"/>
-      <c r="K234" s="43" t="s">
-        <v>366</v>
-      </c>
+      <c r="K234" s="43"/>
     </row>
     <row r="235" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A235" s="13"/>
@@ -9861,11 +9792,11 @@
         <v>0.5</v>
       </c>
       <c r="I239" s="41">
-        <f t="shared" ref="I239:I261" si="8">H239-G239</f>
+        <f t="shared" ref="I239:I263" si="8">H239-G239</f>
         <v>0</v>
       </c>
       <c r="J239" s="55" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="K239" s="43"/>
     </row>
@@ -9898,7 +9829,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J240" s="45"/>
+      <c r="J240" s="53" t="s">
+        <v>406</v>
+      </c>
       <c r="K240" s="43"/>
     </row>
     <row r="241" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9930,7 +9863,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J241" s="45"/>
+      <c r="J241" s="53" t="s">
+        <v>407</v>
+      </c>
       <c r="K241" s="43"/>
     </row>
     <row r="242" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9994,7 +9929,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J243" s="45"/>
+      <c r="J243" s="53" t="s">
+        <v>408</v>
+      </c>
       <c r="K243" s="43"/>
     </row>
     <row r="244" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10122,7 +10059,9 @@
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
-      <c r="J247" s="45"/>
+      <c r="J247" s="53" t="s">
+        <v>411</v>
+      </c>
       <c r="K247" s="43" t="s">
         <v>352</v>
       </c>
@@ -10156,7 +10095,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J248" s="45"/>
+      <c r="J248" s="53" t="s">
+        <v>410</v>
+      </c>
       <c r="K248" s="43"/>
     </row>
     <row r="249" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10170,7 +10111,7 @@
         <v>333</v>
       </c>
       <c r="D249" s="38" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E249" s="40" t="s">
         <v>49</v>
@@ -10188,7 +10129,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J249" s="45"/>
+      <c r="J249" s="53" t="s">
+        <v>408</v>
+      </c>
       <c r="K249" s="43"/>
     </row>
     <row r="250" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10202,7 +10145,7 @@
         <v>227</v>
       </c>
       <c r="D250" s="38" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E250" s="40" t="s">
         <v>63</v>
@@ -10220,7 +10163,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J250" s="45"/>
+      <c r="J250" s="53" t="s">
+        <v>409</v>
+      </c>
       <c r="K250" s="43"/>
     </row>
     <row r="251" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10252,7 +10197,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J251" s="45"/>
+      <c r="J251" s="53" t="s">
+        <v>408</v>
+      </c>
       <c r="K251" s="43"/>
     </row>
     <row r="252" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10284,7 +10231,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J252" s="45"/>
+      <c r="J252" s="53" t="s">
+        <v>408</v>
+      </c>
       <c r="K252" s="43"/>
     </row>
     <row r="253" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10316,7 +10265,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J253" s="45"/>
+      <c r="J253" s="53" t="s">
+        <v>409</v>
+      </c>
       <c r="K253" s="43"/>
     </row>
     <row r="254" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10330,7 +10281,7 @@
         <v>315</v>
       </c>
       <c r="D254" s="38" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E254" s="40" t="s">
         <v>63</v>
@@ -10348,7 +10299,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J254" s="45"/>
+      <c r="J254" s="53" t="s">
+        <v>406</v>
+      </c>
       <c r="K254" s="43"/>
     </row>
     <row r="255" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10356,7 +10309,7 @@
         <v>45680</v>
       </c>
       <c r="B255" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C255" s="39" t="s">
         <v>79</v>
@@ -10373,10 +10326,12 @@
       <c r="G255" s="41">
         <v>1</v>
       </c>
-      <c r="H255" s="41"/>
+      <c r="H255" s="41">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="I255" s="41">
         <f t="shared" si="8"/>
-        <v>-1</v>
+        <v>0.10000000000000009</v>
       </c>
       <c r="J255" s="45"/>
       <c r="K255" s="43"/>
@@ -10386,13 +10341,13 @@
         <v>45680</v>
       </c>
       <c r="B256" s="38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C256" s="39" t="s">
         <v>197</v>
       </c>
       <c r="D256" s="38" t="s">
-        <v>359</v>
+        <v>412</v>
       </c>
       <c r="E256" s="40" t="s">
         <v>63</v>
@@ -10403,10 +10358,12 @@
       <c r="G256" s="41">
         <v>1</v>
       </c>
-      <c r="H256" s="41"/>
+      <c r="H256" s="41">
+        <v>1</v>
+      </c>
       <c r="I256" s="41">
         <f t="shared" si="8"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J256" s="45"/>
       <c r="K256" s="43"/>
@@ -10419,10 +10376,10 @@
         <v>42</v>
       </c>
       <c r="C257" s="39" t="s">
-        <v>361</v>
+        <v>197</v>
       </c>
       <c r="D257" s="38" t="s">
-        <v>360</v>
+        <v>413</v>
       </c>
       <c r="E257" s="40" t="s">
         <v>63</v>
@@ -10431,12 +10388,12 @@
         <v>87</v>
       </c>
       <c r="G257" s="41">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H257" s="41"/>
       <c r="I257" s="41">
         <f t="shared" si="8"/>
-        <v>-0.5</v>
+        <v>-1</v>
       </c>
       <c r="J257" s="45"/>
       <c r="K257" s="43"/>
@@ -10449,98 +10406,158 @@
         <v>42</v>
       </c>
       <c r="C258" s="39" t="s">
-        <v>345</v>
+        <v>197</v>
       </c>
       <c r="D258" s="38" t="s">
-        <v>354</v>
+        <v>415</v>
       </c>
       <c r="E258" s="40" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="F258" s="40" t="s">
-        <v>348</v>
+        <v>87</v>
       </c>
       <c r="G258" s="41">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="H258" s="41"/>
       <c r="I258" s="41">
         <f t="shared" si="8"/>
-        <v>-2</v>
+        <v>-0.5</v>
       </c>
       <c r="J258" s="45"/>
       <c r="K258" s="43"/>
     </row>
     <row r="259" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A259" s="37"/>
-      <c r="B259" s="38"/>
+      <c r="A259" s="37">
+        <v>45680</v>
+      </c>
+      <c r="B259" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C259" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D259" s="38"/>
-      <c r="E259" s="40"/>
-      <c r="F259" s="40"/>
-      <c r="G259" s="41"/>
+        <v>360</v>
+      </c>
+      <c r="D259" s="38" t="s">
+        <v>359</v>
+      </c>
+      <c r="E259" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F259" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G259" s="41">
+        <v>0.5</v>
+      </c>
       <c r="H259" s="41"/>
       <c r="I259" s="41">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="J259" s="45"/>
       <c r="K259" s="43"/>
     </row>
     <row r="260" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A260" s="37"/>
-      <c r="B260" s="38"/>
+      <c r="A260" s="37">
+        <v>45680</v>
+      </c>
+      <c r="B260" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C260" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D260" s="38"/>
-      <c r="E260" s="40"/>
-      <c r="F260" s="40"/>
-      <c r="G260" s="41"/>
+        <v>345</v>
+      </c>
+      <c r="D260" s="38" t="s">
+        <v>354</v>
+      </c>
+      <c r="E260" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="F260" s="40" t="s">
+        <v>348</v>
+      </c>
+      <c r="G260" s="41">
+        <v>2</v>
+      </c>
       <c r="H260" s="41"/>
       <c r="I260" s="41">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="J260" s="45"/>
       <c r="K260" s="43"/>
     </row>
     <row r="261" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A261" s="48"/>
-      <c r="B261" s="49"/>
-      <c r="C261" s="49"/>
-      <c r="D261" s="49"/>
-      <c r="E261" s="49" t="s">
+      <c r="A261" s="37"/>
+      <c r="B261" s="38"/>
+      <c r="C261" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D261" s="38"/>
+      <c r="E261" s="40"/>
+      <c r="F261" s="40"/>
+      <c r="G261" s="41"/>
+      <c r="H261" s="41"/>
+      <c r="I261" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J261" s="45"/>
+      <c r="K261" s="43"/>
+    </row>
+    <row r="262" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A262" s="37"/>
+      <c r="B262" s="38"/>
+      <c r="C262" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D262" s="38"/>
+      <c r="E262" s="40"/>
+      <c r="F262" s="40"/>
+      <c r="G262" s="41"/>
+      <c r="H262" s="41"/>
+      <c r="I262" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J262" s="45"/>
+      <c r="K262" s="43"/>
+    </row>
+    <row r="263" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A263" s="48"/>
+      <c r="B263" s="49"/>
+      <c r="C263" s="49"/>
+      <c r="D263" s="49"/>
+      <c r="E263" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F261" s="49"/>
-      <c r="G261" s="50">
-        <f t="shared" ref="G261:H261" si="9">SUM(G239:G260)</f>
-        <v>26.25</v>
-      </c>
-      <c r="H261" s="50">
+      <c r="F263" s="49"/>
+      <c r="G263" s="50">
+        <f t="shared" ref="G263:H263" si="9">SUM(G239:G262)</f>
+        <v>27.75</v>
+      </c>
+      <c r="H263" s="50">
         <f t="shared" si="9"/>
-        <v>22</v>
-      </c>
-      <c r="I261" s="50">
+        <v>24.1</v>
+      </c>
+      <c r="I263" s="50">
         <f t="shared" si="8"/>
-        <v>-4.25</v>
-      </c>
-      <c r="J261" s="51"/>
-      <c r="K261" s="52"/>
-    </row>
-    <row r="262" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E262" s="40"/>
-    </row>
-    <row r="263" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G263" s="38" t="s">
+        <v>-3.6499999999999986</v>
+      </c>
+      <c r="J263" s="51"/>
+      <c r="K263" s="52"/>
+    </row>
+    <row r="264" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E264" s="40"/>
+    </row>
+    <row r="265" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G265" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="H263" s="54">
-        <f>H44+H79+H113+H146+H189+H211+H235+H261</f>
-        <v>249.58999999999997</v>
+      <c r="H265" s="54">
+        <f>H44+H79+H113+H146+H189+H211+H235+H263</f>
+        <v>251.68999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -10548,7 +10565,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{9D9A2EF4-6DF7-4017-B6F7-BC8B2F6AC336}">
+      <autoFilter ref="A1:K15" xr:uid="{E9824AA5-EB70-4DCB-A5C2-78FA16A67488}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -10584,7 +10601,7 @@
     <mergeCell ref="B149:K149"/>
     <mergeCell ref="A190:K190"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B43 B46:B78 B83:B112 B117:B145 B150:B188 B193:B210 B215:B234 B239:B260">
+  <conditionalFormatting sqref="B5:B43 B46:B78 B83:B112 B117:B145 B150:B188 B193:B210 B215:B234 B239:B262">
     <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -10601,7 +10618,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B44 B46:B79 B81:B113 B115:B146 B148:B189 B191:B211 B213:B235 B237:B261">
+  <conditionalFormatting sqref="B5:B44 B46:B79 B81:B113 B115:B146 B148:B189 B191:B211 B213:B235 B237:B263">
     <cfRule type="containsText" dxfId="5" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -10609,17 +10626,17 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G44 G48:G79 G83:G113 G117:G146 G150:G189 G193:G211 G215:G235 G239:G261">
+  <conditionalFormatting sqref="G1 G3:G44 G48:G79 G83:G113 G117:G146 G150:G189 G193:G211 G215:G235 G239:G263">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H261">
+  <conditionalFormatting sqref="H1:H263">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I44 I48:I79 I83:I113 I117:I146 I150:I189 I193:I211 I215:I235 I239:I261">
+  <conditionalFormatting sqref="I5:I44 I48:I79 I83:I113 I117:I146 I150:I189 I193:I211 I215:I235 I239:I263">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -10628,7 +10645,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F215:F234 F5:F43 F48:F78 F83:F112 F117:F145 F150:F188 F193:F210 F239:F260" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F215:F234 F5:F43 F48:F78 F83:F112 F117:F145 F150:F188 F193:F210 F239:F262" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10727,9 +10744,20 @@
     <hyperlink ref="J230" r:id="rId92" xr:uid="{E183232F-EA5A-4B6E-8CFF-DA9B9914B627}"/>
     <hyperlink ref="J231" r:id="rId93" xr:uid="{EFCF5C0A-E154-4514-9E30-5E20FF6EDA00}"/>
     <hyperlink ref="J239" r:id="rId94" xr:uid="{5BAE8CCE-DAC0-4B75-8943-53DD6F6B2BF6}"/>
+    <hyperlink ref="J254" r:id="rId95" xr:uid="{0E91B18A-45EB-4F50-9AAE-FF4D618BC908}"/>
+    <hyperlink ref="J240" r:id="rId96" xr:uid="{441BEB57-2195-436B-BCB3-8CE24964BFBD}"/>
+    <hyperlink ref="J241" r:id="rId97" xr:uid="{11A4B9A5-86F6-4EAC-B17C-222A33BCBB78}"/>
+    <hyperlink ref="J243" r:id="rId98" xr:uid="{6661CD06-A836-47F1-8B27-3662E66C6F94}"/>
+    <hyperlink ref="J249" r:id="rId99" xr:uid="{C1180E4D-13B6-4B8E-963C-F99496D4E6E3}"/>
+    <hyperlink ref="J252" r:id="rId100" xr:uid="{E2AE8D27-FF41-4578-8366-83BB63CE6F29}"/>
+    <hyperlink ref="J253" r:id="rId101" xr:uid="{1A45F8B2-47F8-4971-A6E6-1FF0E5AAC481}"/>
+    <hyperlink ref="J250" r:id="rId102" xr:uid="{1BE0AAD3-6C80-4D51-AD77-D4D4E4578DBF}"/>
+    <hyperlink ref="J251" r:id="rId103" xr:uid="{16CA5873-1B08-42B1-8CFB-B21C99D3DA09}"/>
+    <hyperlink ref="J248" r:id="rId104" xr:uid="{5579EECA-7B58-48DE-95CC-8A44F9E9CF3D}"/>
+    <hyperlink ref="J247" r:id="rId105" xr:uid="{17750EDF-0632-423C-A63E-900EA839D2C0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId95"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId106"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -10737,13 +10765,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E215:E234 E5:E43 E48:E78 E83:E112 E117:E145 E150:E188 E193:E210 E239:E260</xm:sqref>
+          <xm:sqref>E215:E234 E5:E43 E48:E78 E83:E112 E117:E145 E150:E188 E193:E210 E239:E262</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B215:B234 B5:B43 B48:B78 B83:B112 B117:B145 B150:B188 B193:B210 B239:B260</xm:sqref>
+          <xm:sqref>B215:B234 B5:B43 B48:B78 B83:B112 B117:B145 B150:B188 B193:B210 B239:B262</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
W8 Datalab II work II (post-presentation)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2794DAD-FBF2-4197-B917-1259E232B55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9189F31-AD8F-4D2F-A4C2-603A8E283166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1878,6 +1878,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1894,8 +1914,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1913,24 +1931,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2407,53 +2407,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="62"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="70"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="63" t="s">
+      <c r="B3" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="65"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="63" t="s">
+      <c r="B4" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="65"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="58"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3790,53 +3790,53 @@
       <c r="K44" s="46"/>
     </row>
     <row r="45" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="66" t="s">
+      <c r="A45" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="B45" s="61"/>
-      <c r="C45" s="61"/>
-      <c r="D45" s="61"/>
-      <c r="E45" s="61"/>
-      <c r="F45" s="61"/>
-      <c r="G45" s="61"/>
-      <c r="H45" s="61"/>
-      <c r="I45" s="61"/>
-      <c r="J45" s="61"/>
-      <c r="K45" s="62"/>
+      <c r="B45" s="69"/>
+      <c r="C45" s="69"/>
+      <c r="D45" s="69"/>
+      <c r="E45" s="69"/>
+      <c r="F45" s="69"/>
+      <c r="G45" s="69"/>
+      <c r="H45" s="69"/>
+      <c r="I45" s="69"/>
+      <c r="J45" s="69"/>
+      <c r="K45" s="70"/>
     </row>
     <row r="46" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A46" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="67" t="s">
+      <c r="B46" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C46" s="64"/>
-      <c r="D46" s="64"/>
-      <c r="E46" s="64"/>
-      <c r="F46" s="64"/>
-      <c r="G46" s="64"/>
-      <c r="H46" s="64"/>
-      <c r="I46" s="64"/>
-      <c r="J46" s="64"/>
-      <c r="K46" s="65"/>
+      <c r="C46" s="57"/>
+      <c r="D46" s="57"/>
+      <c r="E46" s="57"/>
+      <c r="F46" s="57"/>
+      <c r="G46" s="57"/>
+      <c r="H46" s="57"/>
+      <c r="I46" s="57"/>
+      <c r="J46" s="57"/>
+      <c r="K46" s="58"/>
     </row>
     <row r="47" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B47" s="67" t="s">
+      <c r="B47" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="C47" s="64"/>
-      <c r="D47" s="64"/>
-      <c r="E47" s="64"/>
-      <c r="F47" s="64"/>
-      <c r="G47" s="64"/>
-      <c r="H47" s="64"/>
-      <c r="I47" s="64"/>
-      <c r="J47" s="64"/>
-      <c r="K47" s="65"/>
+      <c r="C47" s="57"/>
+      <c r="D47" s="57"/>
+      <c r="E47" s="57"/>
+      <c r="F47" s="57"/>
+      <c r="G47" s="57"/>
+      <c r="H47" s="57"/>
+      <c r="I47" s="57"/>
+      <c r="J47" s="57"/>
+      <c r="K47" s="58"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="47">
@@ -4901,53 +4901,53 @@
       <c r="K79" s="46"/>
     </row>
     <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="68" t="s">
+      <c r="A80" s="74" t="s">
         <v>20</v>
       </c>
-      <c r="B80" s="64"/>
-      <c r="C80" s="64"/>
-      <c r="D80" s="64"/>
-      <c r="E80" s="64"/>
-      <c r="F80" s="64"/>
-      <c r="G80" s="64"/>
-      <c r="H80" s="64"/>
-      <c r="I80" s="64"/>
-      <c r="J80" s="64"/>
-      <c r="K80" s="65"/>
+      <c r="B80" s="57"/>
+      <c r="C80" s="57"/>
+      <c r="D80" s="57"/>
+      <c r="E80" s="57"/>
+      <c r="F80" s="57"/>
+      <c r="G80" s="57"/>
+      <c r="H80" s="57"/>
+      <c r="I80" s="57"/>
+      <c r="J80" s="57"/>
+      <c r="K80" s="58"/>
     </row>
     <row r="81" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A81" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B81" s="69" t="s">
+      <c r="B81" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C81" s="64"/>
-      <c r="D81" s="64"/>
-      <c r="E81" s="64"/>
-      <c r="F81" s="64"/>
-      <c r="G81" s="64"/>
-      <c r="H81" s="64"/>
-      <c r="I81" s="64"/>
-      <c r="J81" s="64"/>
-      <c r="K81" s="65"/>
+      <c r="C81" s="57"/>
+      <c r="D81" s="57"/>
+      <c r="E81" s="57"/>
+      <c r="F81" s="57"/>
+      <c r="G81" s="57"/>
+      <c r="H81" s="57"/>
+      <c r="I81" s="57"/>
+      <c r="J81" s="57"/>
+      <c r="K81" s="58"/>
     </row>
     <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="69" t="s">
+      <c r="B82" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C82" s="64"/>
-      <c r="D82" s="64"/>
-      <c r="E82" s="64"/>
-      <c r="F82" s="64"/>
-      <c r="G82" s="64"/>
-      <c r="H82" s="64"/>
-      <c r="I82" s="64"/>
-      <c r="J82" s="64"/>
-      <c r="K82" s="65"/>
+      <c r="C82" s="57"/>
+      <c r="D82" s="57"/>
+      <c r="E82" s="57"/>
+      <c r="F82" s="57"/>
+      <c r="G82" s="57"/>
+      <c r="H82" s="57"/>
+      <c r="I82" s="57"/>
+      <c r="J82" s="57"/>
+      <c r="K82" s="58"/>
     </row>
     <row r="83" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A83" s="37">
@@ -5984,53 +5984,53 @@
       <c r="K113" s="46"/>
     </row>
     <row r="114" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="70" t="s">
+      <c r="A114" s="76" t="s">
         <v>21</v>
       </c>
-      <c r="B114" s="64"/>
-      <c r="C114" s="64"/>
-      <c r="D114" s="64"/>
-      <c r="E114" s="64"/>
-      <c r="F114" s="64"/>
-      <c r="G114" s="64"/>
-      <c r="H114" s="64"/>
-      <c r="I114" s="64"/>
-      <c r="J114" s="64"/>
-      <c r="K114" s="65"/>
+      <c r="B114" s="57"/>
+      <c r="C114" s="57"/>
+      <c r="D114" s="57"/>
+      <c r="E114" s="57"/>
+      <c r="F114" s="57"/>
+      <c r="G114" s="57"/>
+      <c r="H114" s="57"/>
+      <c r="I114" s="57"/>
+      <c r="J114" s="57"/>
+      <c r="K114" s="58"/>
     </row>
     <row r="115" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A115" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B115" s="72" t="s">
+      <c r="B115" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C115" s="64"/>
-      <c r="D115" s="64"/>
-      <c r="E115" s="64"/>
-      <c r="F115" s="64"/>
-      <c r="G115" s="64"/>
-      <c r="H115" s="64"/>
-      <c r="I115" s="64"/>
-      <c r="J115" s="64"/>
-      <c r="K115" s="65"/>
+      <c r="C115" s="57"/>
+      <c r="D115" s="57"/>
+      <c r="E115" s="57"/>
+      <c r="F115" s="57"/>
+      <c r="G115" s="57"/>
+      <c r="H115" s="57"/>
+      <c r="I115" s="57"/>
+      <c r="J115" s="57"/>
+      <c r="K115" s="58"/>
     </row>
     <row r="116" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B116" s="72" t="s">
+      <c r="B116" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C116" s="64"/>
-      <c r="D116" s="64"/>
-      <c r="E116" s="64"/>
-      <c r="F116" s="64"/>
-      <c r="G116" s="64"/>
-      <c r="H116" s="64"/>
-      <c r="I116" s="64"/>
-      <c r="J116" s="64"/>
-      <c r="K116" s="65"/>
+      <c r="C116" s="57"/>
+      <c r="D116" s="57"/>
+      <c r="E116" s="57"/>
+      <c r="F116" s="57"/>
+      <c r="G116" s="57"/>
+      <c r="H116" s="57"/>
+      <c r="I116" s="57"/>
+      <c r="J116" s="57"/>
+      <c r="K116" s="58"/>
     </row>
     <row r="117" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A117" s="37">
@@ -7033,53 +7033,53 @@
       <c r="K146" s="46"/>
     </row>
     <row r="147" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="75" t="s">
+      <c r="A147" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="B147" s="64"/>
-      <c r="C147" s="64"/>
-      <c r="D147" s="64"/>
-      <c r="E147" s="64"/>
-      <c r="F147" s="64"/>
-      <c r="G147" s="64"/>
-      <c r="H147" s="64"/>
-      <c r="I147" s="64"/>
-      <c r="J147" s="64"/>
-      <c r="K147" s="65"/>
+      <c r="B147" s="57"/>
+      <c r="C147" s="57"/>
+      <c r="D147" s="57"/>
+      <c r="E147" s="57"/>
+      <c r="F147" s="57"/>
+      <c r="G147" s="57"/>
+      <c r="H147" s="57"/>
+      <c r="I147" s="57"/>
+      <c r="J147" s="57"/>
+      <c r="K147" s="58"/>
     </row>
     <row r="148" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A148" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B148" s="76" t="s">
+      <c r="B148" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C148" s="64"/>
-      <c r="D148" s="64"/>
-      <c r="E148" s="64"/>
-      <c r="F148" s="64"/>
-      <c r="G148" s="64"/>
-      <c r="H148" s="64"/>
-      <c r="I148" s="64"/>
-      <c r="J148" s="64"/>
-      <c r="K148" s="65"/>
+      <c r="C148" s="57"/>
+      <c r="D148" s="57"/>
+      <c r="E148" s="57"/>
+      <c r="F148" s="57"/>
+      <c r="G148" s="57"/>
+      <c r="H148" s="57"/>
+      <c r="I148" s="57"/>
+      <c r="J148" s="57"/>
+      <c r="K148" s="58"/>
     </row>
     <row r="149" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B149" s="76" t="s">
+      <c r="B149" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="C149" s="64"/>
-      <c r="D149" s="64"/>
-      <c r="E149" s="64"/>
-      <c r="F149" s="64"/>
-      <c r="G149" s="64"/>
-      <c r="H149" s="64"/>
-      <c r="I149" s="64"/>
-      <c r="J149" s="64"/>
-      <c r="K149" s="65"/>
+      <c r="C149" s="57"/>
+      <c r="D149" s="57"/>
+      <c r="E149" s="57"/>
+      <c r="F149" s="57"/>
+      <c r="G149" s="57"/>
+      <c r="H149" s="57"/>
+      <c r="I149" s="57"/>
+      <c r="J149" s="57"/>
+      <c r="K149" s="58"/>
     </row>
     <row r="150" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A150" s="37">
@@ -8422,53 +8422,53 @@
       <c r="K189" s="46"/>
     </row>
     <row r="190" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="77" t="s">
+      <c r="A190" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B190" s="64"/>
-      <c r="C190" s="64"/>
-      <c r="D190" s="64"/>
-      <c r="E190" s="64"/>
-      <c r="F190" s="64"/>
-      <c r="G190" s="64"/>
-      <c r="H190" s="64"/>
-      <c r="I190" s="64"/>
-      <c r="J190" s="64"/>
-      <c r="K190" s="65"/>
+      <c r="B190" s="57"/>
+      <c r="C190" s="57"/>
+      <c r="D190" s="57"/>
+      <c r="E190" s="57"/>
+      <c r="F190" s="57"/>
+      <c r="G190" s="57"/>
+      <c r="H190" s="57"/>
+      <c r="I190" s="57"/>
+      <c r="J190" s="57"/>
+      <c r="K190" s="58"/>
     </row>
     <row r="191" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A191" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B191" s="73" t="s">
+      <c r="B191" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="C191" s="64"/>
-      <c r="D191" s="64"/>
-      <c r="E191" s="64"/>
-      <c r="F191" s="64"/>
-      <c r="G191" s="64"/>
-      <c r="H191" s="64"/>
-      <c r="I191" s="64"/>
-      <c r="J191" s="64"/>
-      <c r="K191" s="65"/>
+      <c r="C191" s="57"/>
+      <c r="D191" s="57"/>
+      <c r="E191" s="57"/>
+      <c r="F191" s="57"/>
+      <c r="G191" s="57"/>
+      <c r="H191" s="57"/>
+      <c r="I191" s="57"/>
+      <c r="J191" s="57"/>
+      <c r="K191" s="58"/>
     </row>
     <row r="192" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B192" s="73" t="s">
+      <c r="B192" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C192" s="64"/>
-      <c r="D192" s="64"/>
-      <c r="E192" s="64"/>
-      <c r="F192" s="64"/>
-      <c r="G192" s="64"/>
-      <c r="H192" s="64"/>
-      <c r="I192" s="64"/>
-      <c r="J192" s="64"/>
-      <c r="K192" s="65"/>
+      <c r="C192" s="57"/>
+      <c r="D192" s="57"/>
+      <c r="E192" s="57"/>
+      <c r="F192" s="57"/>
+      <c r="G192" s="57"/>
+      <c r="H192" s="57"/>
+      <c r="I192" s="57"/>
+      <c r="J192" s="57"/>
+      <c r="K192" s="58"/>
     </row>
     <row r="193" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A193" s="37">
@@ -9106,53 +9106,53 @@
       <c r="K211" s="46"/>
     </row>
     <row r="212" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A212" s="74" t="s">
+      <c r="A212" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="B212" s="64"/>
-      <c r="C212" s="64"/>
-      <c r="D212" s="64"/>
-      <c r="E212" s="64"/>
-      <c r="F212" s="64"/>
-      <c r="G212" s="64"/>
-      <c r="H212" s="64"/>
-      <c r="I212" s="64"/>
-      <c r="J212" s="64"/>
-      <c r="K212" s="65"/>
+      <c r="B212" s="57"/>
+      <c r="C212" s="57"/>
+      <c r="D212" s="57"/>
+      <c r="E212" s="57"/>
+      <c r="F212" s="57"/>
+      <c r="G212" s="57"/>
+      <c r="H212" s="57"/>
+      <c r="I212" s="57"/>
+      <c r="J212" s="57"/>
+      <c r="K212" s="58"/>
     </row>
     <row r="213" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A213" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B213" s="71" t="s">
+      <c r="B213" s="77" t="s">
         <v>13</v>
       </c>
-      <c r="C213" s="64"/>
-      <c r="D213" s="64"/>
-      <c r="E213" s="64"/>
-      <c r="F213" s="64"/>
-      <c r="G213" s="64"/>
-      <c r="H213" s="64"/>
-      <c r="I213" s="64"/>
-      <c r="J213" s="64"/>
-      <c r="K213" s="65"/>
+      <c r="C213" s="57"/>
+      <c r="D213" s="57"/>
+      <c r="E213" s="57"/>
+      <c r="F213" s="57"/>
+      <c r="G213" s="57"/>
+      <c r="H213" s="57"/>
+      <c r="I213" s="57"/>
+      <c r="J213" s="57"/>
+      <c r="K213" s="58"/>
     </row>
     <row r="214" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B214" s="71" t="s">
+      <c r="B214" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="C214" s="64"/>
-      <c r="D214" s="64"/>
-      <c r="E214" s="64"/>
-      <c r="F214" s="64"/>
-      <c r="G214" s="64"/>
-      <c r="H214" s="64"/>
-      <c r="I214" s="64"/>
-      <c r="J214" s="64"/>
-      <c r="K214" s="65"/>
+      <c r="C214" s="57"/>
+      <c r="D214" s="57"/>
+      <c r="E214" s="57"/>
+      <c r="F214" s="57"/>
+      <c r="G214" s="57"/>
+      <c r="H214" s="57"/>
+      <c r="I214" s="57"/>
+      <c r="J214" s="57"/>
+      <c r="K214" s="58"/>
     </row>
     <row r="215" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A215" s="37">
@@ -9845,53 +9845,53 @@
       <c r="K235" s="46"/>
     </row>
     <row r="236" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A236" s="56" t="s">
+      <c r="A236" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="B236" s="57"/>
-      <c r="C236" s="57"/>
-      <c r="D236" s="57"/>
-      <c r="E236" s="57"/>
-      <c r="F236" s="57"/>
-      <c r="G236" s="57"/>
-      <c r="H236" s="57"/>
-      <c r="I236" s="57"/>
-      <c r="J236" s="57"/>
-      <c r="K236" s="58"/>
+      <c r="B236" s="65"/>
+      <c r="C236" s="65"/>
+      <c r="D236" s="65"/>
+      <c r="E236" s="65"/>
+      <c r="F236" s="65"/>
+      <c r="G236" s="65"/>
+      <c r="H236" s="65"/>
+      <c r="I236" s="65"/>
+      <c r="J236" s="65"/>
+      <c r="K236" s="66"/>
     </row>
     <row r="237" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A237" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B237" s="59" t="s">
+      <c r="B237" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C237" s="57"/>
-      <c r="D237" s="57"/>
-      <c r="E237" s="57"/>
-      <c r="F237" s="57"/>
-      <c r="G237" s="57"/>
-      <c r="H237" s="57"/>
-      <c r="I237" s="57"/>
-      <c r="J237" s="57"/>
-      <c r="K237" s="58"/>
+      <c r="C237" s="65"/>
+      <c r="D237" s="65"/>
+      <c r="E237" s="65"/>
+      <c r="F237" s="65"/>
+      <c r="G237" s="65"/>
+      <c r="H237" s="65"/>
+      <c r="I237" s="65"/>
+      <c r="J237" s="65"/>
+      <c r="K237" s="66"/>
     </row>
     <row r="238" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B238" s="59" t="s">
+      <c r="B238" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C238" s="57"/>
-      <c r="D238" s="57"/>
-      <c r="E238" s="57"/>
-      <c r="F238" s="57"/>
-      <c r="G238" s="57"/>
-      <c r="H238" s="57"/>
-      <c r="I238" s="57"/>
-      <c r="J238" s="57"/>
-      <c r="K238" s="58"/>
+      <c r="C238" s="65"/>
+      <c r="D238" s="65"/>
+      <c r="E238" s="65"/>
+      <c r="F238" s="65"/>
+      <c r="G238" s="65"/>
+      <c r="H238" s="65"/>
+      <c r="I238" s="65"/>
+      <c r="J238" s="65"/>
+      <c r="K238" s="66"/>
     </row>
     <row r="239" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A239" s="37">
@@ -10746,7 +10746,7 @@
         <v>45681</v>
       </c>
       <c r="B264" s="38" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C264" s="39" t="s">
         <v>76</v>
@@ -10763,10 +10763,12 @@
       <c r="G264" s="41">
         <v>0.25</v>
       </c>
-      <c r="H264" s="41"/>
+      <c r="H264" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I264" s="41">
         <f t="shared" si="8"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J264" s="45"/>
       <c r="K264" s="43"/>
@@ -10776,7 +10778,7 @@
         <v>45681</v>
       </c>
       <c r="B265" s="38" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C265" s="39" t="s">
         <v>344</v>
@@ -10793,10 +10795,12 @@
       <c r="G265" s="41">
         <v>0.25</v>
       </c>
-      <c r="H265" s="41"/>
+      <c r="H265" s="41">
+        <v>0.25</v>
+      </c>
       <c r="I265" s="41">
         <f t="shared" si="8"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="J265" s="45"/>
       <c r="K265" s="43"/>
@@ -10806,7 +10810,7 @@
         <v>45681</v>
       </c>
       <c r="B266" s="38" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C266" s="39" t="s">
         <v>344</v>
@@ -10823,10 +10827,12 @@
       <c r="G266" s="41">
         <v>3.75</v>
       </c>
-      <c r="H266" s="41"/>
+      <c r="H266" s="41">
+        <v>1.75</v>
+      </c>
       <c r="I266" s="41">
         <f t="shared" si="8"/>
-        <v>-3.75</v>
+        <v>-2</v>
       </c>
       <c r="J266" s="45"/>
       <c r="K266" s="43"/>
@@ -10846,11 +10852,11 @@
       </c>
       <c r="H267" s="50">
         <f t="shared" si="9"/>
-        <v>28.75</v>
+        <v>31</v>
       </c>
       <c r="I267" s="50">
         <f t="shared" si="8"/>
-        <v>-4.1499999999999986</v>
+        <v>-1.8999999999999986</v>
       </c>
       <c r="J267" s="51"/>
       <c r="K267" s="52"/>
@@ -10864,7 +10870,7 @@
       </c>
       <c r="H269" s="54">
         <f>H44+H79+H113+H146+H189+H211+H235+H267</f>
-        <v>256.33999999999997</v>
+        <v>258.58999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -10872,7 +10878,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{B74141F6-2621-4D41-BEFA-BA4CC02DEC69}">
+      <autoFilter ref="A1:K15" xr:uid="{4156E376-828C-4BE6-9122-475CF5BFDDAA}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -10883,14 +10889,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B191:K191"/>
-    <mergeCell ref="B192:K192"/>
-    <mergeCell ref="A212:K212"/>
-    <mergeCell ref="B116:K116"/>
-    <mergeCell ref="A147:K147"/>
-    <mergeCell ref="B148:K148"/>
-    <mergeCell ref="B149:K149"/>
-    <mergeCell ref="A190:K190"/>
     <mergeCell ref="A236:K236"/>
     <mergeCell ref="B237:K237"/>
     <mergeCell ref="B238:K238"/>
@@ -10907,6 +10905,14 @@
     <mergeCell ref="B213:K213"/>
     <mergeCell ref="B214:K214"/>
     <mergeCell ref="B115:K115"/>
+    <mergeCell ref="B191:K191"/>
+    <mergeCell ref="B192:K192"/>
+    <mergeCell ref="A212:K212"/>
+    <mergeCell ref="B116:K116"/>
+    <mergeCell ref="A147:K147"/>
+    <mergeCell ref="B148:K148"/>
+    <mergeCell ref="B149:K149"/>
+    <mergeCell ref="A190:K190"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B43 B46:B78 B83:B112 B117:B145 B150:B188 B193:B210 B215:B234 B239:B266">
     <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="Unplanned">
@@ -12774,6 +12780,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -13008,27 +13034,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13045,23 +13070,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
W8 Datalab II work III (W8 LL Feedback)
</commit_message>
<xml_diff>
--- a/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Deliverables/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9189F31-AD8F-4D2F-A4C2-603A8E283166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45CA6644-7692-478A-8483-DF76BB1E9311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1479" uniqueCount="430">
   <si>
     <t>Date</t>
   </si>
@@ -1383,6 +1383,15 @@
   </si>
   <si>
     <t>Add link to final report in creative brief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/d5abdbda997298c5edfd9312bbeacd84588db915/Block%20B/Final%20Presentation.pptx </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/d5abdbda997298c5edfd9312bbeacd84588db915/Deliverables/CreativeBrief_MaksBurchard_240894.ipynb </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/d5abdbda997298c5edfd9312bbeacd84588db915/Deliverables/Worklog%20-%20Y1B-2024-25_ADSAI.xlsx </t>
   </si>
 </sst>
 </file>
@@ -1878,26 +1887,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1914,6 +1903,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1931,6 +1922,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2407,53 +2416,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="70"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="62"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="65"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="71" t="s">
+      <c r="B4" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="58"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="65"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -3790,53 +3799,53 @@
       <c r="K44" s="46"/>
     </row>
     <row r="45" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="72" t="s">
+      <c r="A45" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="B45" s="69"/>
-      <c r="C45" s="69"/>
-      <c r="D45" s="69"/>
-      <c r="E45" s="69"/>
-      <c r="F45" s="69"/>
-      <c r="G45" s="69"/>
-      <c r="H45" s="69"/>
-      <c r="I45" s="69"/>
-      <c r="J45" s="69"/>
-      <c r="K45" s="70"/>
+      <c r="B45" s="61"/>
+      <c r="C45" s="61"/>
+      <c r="D45" s="61"/>
+      <c r="E45" s="61"/>
+      <c r="F45" s="61"/>
+      <c r="G45" s="61"/>
+      <c r="H45" s="61"/>
+      <c r="I45" s="61"/>
+      <c r="J45" s="61"/>
+      <c r="K45" s="62"/>
     </row>
     <row r="46" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A46" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="73" t="s">
+      <c r="B46" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C46" s="57"/>
-      <c r="D46" s="57"/>
-      <c r="E46" s="57"/>
-      <c r="F46" s="57"/>
-      <c r="G46" s="57"/>
-      <c r="H46" s="57"/>
-      <c r="I46" s="57"/>
-      <c r="J46" s="57"/>
-      <c r="K46" s="58"/>
+      <c r="C46" s="64"/>
+      <c r="D46" s="64"/>
+      <c r="E46" s="64"/>
+      <c r="F46" s="64"/>
+      <c r="G46" s="64"/>
+      <c r="H46" s="64"/>
+      <c r="I46" s="64"/>
+      <c r="J46" s="64"/>
+      <c r="K46" s="65"/>
     </row>
     <row r="47" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B47" s="73" t="s">
+      <c r="B47" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="C47" s="57"/>
-      <c r="D47" s="57"/>
-      <c r="E47" s="57"/>
-      <c r="F47" s="57"/>
-      <c r="G47" s="57"/>
-      <c r="H47" s="57"/>
-      <c r="I47" s="57"/>
-      <c r="J47" s="57"/>
-      <c r="K47" s="58"/>
+      <c r="C47" s="64"/>
+      <c r="D47" s="64"/>
+      <c r="E47" s="64"/>
+      <c r="F47" s="64"/>
+      <c r="G47" s="64"/>
+      <c r="H47" s="64"/>
+      <c r="I47" s="64"/>
+      <c r="J47" s="64"/>
+      <c r="K47" s="65"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="47">
@@ -4901,53 +4910,53 @@
       <c r="K79" s="46"/>
     </row>
     <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="74" t="s">
+      <c r="A80" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="B80" s="57"/>
-      <c r="C80" s="57"/>
-      <c r="D80" s="57"/>
-      <c r="E80" s="57"/>
-      <c r="F80" s="57"/>
-      <c r="G80" s="57"/>
-      <c r="H80" s="57"/>
-      <c r="I80" s="57"/>
-      <c r="J80" s="57"/>
-      <c r="K80" s="58"/>
+      <c r="B80" s="64"/>
+      <c r="C80" s="64"/>
+      <c r="D80" s="64"/>
+      <c r="E80" s="64"/>
+      <c r="F80" s="64"/>
+      <c r="G80" s="64"/>
+      <c r="H80" s="64"/>
+      <c r="I80" s="64"/>
+      <c r="J80" s="64"/>
+      <c r="K80" s="65"/>
     </row>
     <row r="81" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A81" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B81" s="75" t="s">
+      <c r="B81" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C81" s="57"/>
-      <c r="D81" s="57"/>
-      <c r="E81" s="57"/>
-      <c r="F81" s="57"/>
-      <c r="G81" s="57"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="57"/>
-      <c r="J81" s="57"/>
-      <c r="K81" s="58"/>
+      <c r="C81" s="64"/>
+      <c r="D81" s="64"/>
+      <c r="E81" s="64"/>
+      <c r="F81" s="64"/>
+      <c r="G81" s="64"/>
+      <c r="H81" s="64"/>
+      <c r="I81" s="64"/>
+      <c r="J81" s="64"/>
+      <c r="K81" s="65"/>
     </row>
     <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="75" t="s">
+      <c r="B82" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C82" s="57"/>
-      <c r="D82" s="57"/>
-      <c r="E82" s="57"/>
-      <c r="F82" s="57"/>
-      <c r="G82" s="57"/>
-      <c r="H82" s="57"/>
-      <c r="I82" s="57"/>
-      <c r="J82" s="57"/>
-      <c r="K82" s="58"/>
+      <c r="C82" s="64"/>
+      <c r="D82" s="64"/>
+      <c r="E82" s="64"/>
+      <c r="F82" s="64"/>
+      <c r="G82" s="64"/>
+      <c r="H82" s="64"/>
+      <c r="I82" s="64"/>
+      <c r="J82" s="64"/>
+      <c r="K82" s="65"/>
     </row>
     <row r="83" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A83" s="37">
@@ -5984,53 +5993,53 @@
       <c r="K113" s="46"/>
     </row>
     <row r="114" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="76" t="s">
+      <c r="A114" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="B114" s="57"/>
-      <c r="C114" s="57"/>
-      <c r="D114" s="57"/>
-      <c r="E114" s="57"/>
-      <c r="F114" s="57"/>
-      <c r="G114" s="57"/>
-      <c r="H114" s="57"/>
-      <c r="I114" s="57"/>
-      <c r="J114" s="57"/>
-      <c r="K114" s="58"/>
+      <c r="B114" s="64"/>
+      <c r="C114" s="64"/>
+      <c r="D114" s="64"/>
+      <c r="E114" s="64"/>
+      <c r="F114" s="64"/>
+      <c r="G114" s="64"/>
+      <c r="H114" s="64"/>
+      <c r="I114" s="64"/>
+      <c r="J114" s="64"/>
+      <c r="K114" s="65"/>
     </row>
     <row r="115" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A115" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B115" s="60" t="s">
+      <c r="B115" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C115" s="57"/>
-      <c r="D115" s="57"/>
-      <c r="E115" s="57"/>
-      <c r="F115" s="57"/>
-      <c r="G115" s="57"/>
-      <c r="H115" s="57"/>
-      <c r="I115" s="57"/>
-      <c r="J115" s="57"/>
-      <c r="K115" s="58"/>
+      <c r="C115" s="64"/>
+      <c r="D115" s="64"/>
+      <c r="E115" s="64"/>
+      <c r="F115" s="64"/>
+      <c r="G115" s="64"/>
+      <c r="H115" s="64"/>
+      <c r="I115" s="64"/>
+      <c r="J115" s="64"/>
+      <c r="K115" s="65"/>
     </row>
     <row r="116" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B116" s="60" t="s">
+      <c r="B116" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="C116" s="57"/>
-      <c r="D116" s="57"/>
-      <c r="E116" s="57"/>
-      <c r="F116" s="57"/>
-      <c r="G116" s="57"/>
-      <c r="H116" s="57"/>
-      <c r="I116" s="57"/>
-      <c r="J116" s="57"/>
-      <c r="K116" s="58"/>
+      <c r="C116" s="64"/>
+      <c r="D116" s="64"/>
+      <c r="E116" s="64"/>
+      <c r="F116" s="64"/>
+      <c r="G116" s="64"/>
+      <c r="H116" s="64"/>
+      <c r="I116" s="64"/>
+      <c r="J116" s="64"/>
+      <c r="K116" s="65"/>
     </row>
     <row r="117" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A117" s="37">
@@ -7033,53 +7042,53 @@
       <c r="K146" s="46"/>
     </row>
     <row r="147" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="61" t="s">
+      <c r="A147" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="B147" s="57"/>
-      <c r="C147" s="57"/>
-      <c r="D147" s="57"/>
-      <c r="E147" s="57"/>
-      <c r="F147" s="57"/>
-      <c r="G147" s="57"/>
-      <c r="H147" s="57"/>
-      <c r="I147" s="57"/>
-      <c r="J147" s="57"/>
-      <c r="K147" s="58"/>
+      <c r="B147" s="64"/>
+      <c r="C147" s="64"/>
+      <c r="D147" s="64"/>
+      <c r="E147" s="64"/>
+      <c r="F147" s="64"/>
+      <c r="G147" s="64"/>
+      <c r="H147" s="64"/>
+      <c r="I147" s="64"/>
+      <c r="J147" s="64"/>
+      <c r="K147" s="65"/>
     </row>
     <row r="148" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A148" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B148" s="62" t="s">
+      <c r="B148" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="C148" s="57"/>
-      <c r="D148" s="57"/>
-      <c r="E148" s="57"/>
-      <c r="F148" s="57"/>
-      <c r="G148" s="57"/>
-      <c r="H148" s="57"/>
-      <c r="I148" s="57"/>
-      <c r="J148" s="57"/>
-      <c r="K148" s="58"/>
+      <c r="C148" s="64"/>
+      <c r="D148" s="64"/>
+      <c r="E148" s="64"/>
+      <c r="F148" s="64"/>
+      <c r="G148" s="64"/>
+      <c r="H148" s="64"/>
+      <c r="I148" s="64"/>
+      <c r="J148" s="64"/>
+      <c r="K148" s="65"/>
     </row>
     <row r="149" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B149" s="62" t="s">
+      <c r="B149" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="C149" s="57"/>
-      <c r="D149" s="57"/>
-      <c r="E149" s="57"/>
-      <c r="F149" s="57"/>
-      <c r="G149" s="57"/>
-      <c r="H149" s="57"/>
-      <c r="I149" s="57"/>
-      <c r="J149" s="57"/>
-      <c r="K149" s="58"/>
+      <c r="C149" s="64"/>
+      <c r="D149" s="64"/>
+      <c r="E149" s="64"/>
+      <c r="F149" s="64"/>
+      <c r="G149" s="64"/>
+      <c r="H149" s="64"/>
+      <c r="I149" s="64"/>
+      <c r="J149" s="64"/>
+      <c r="K149" s="65"/>
     </row>
     <row r="150" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A150" s="37">
@@ -8422,53 +8431,53 @@
       <c r="K189" s="46"/>
     </row>
     <row r="190" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="63" t="s">
+      <c r="A190" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="B190" s="57"/>
-      <c r="C190" s="57"/>
-      <c r="D190" s="57"/>
-      <c r="E190" s="57"/>
-      <c r="F190" s="57"/>
-      <c r="G190" s="57"/>
-      <c r="H190" s="57"/>
-      <c r="I190" s="57"/>
-      <c r="J190" s="57"/>
-      <c r="K190" s="58"/>
+      <c r="B190" s="64"/>
+      <c r="C190" s="64"/>
+      <c r="D190" s="64"/>
+      <c r="E190" s="64"/>
+      <c r="F190" s="64"/>
+      <c r="G190" s="64"/>
+      <c r="H190" s="64"/>
+      <c r="I190" s="64"/>
+      <c r="J190" s="64"/>
+      <c r="K190" s="65"/>
     </row>
     <row r="191" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A191" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B191" s="56" t="s">
+      <c r="B191" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C191" s="57"/>
-      <c r="D191" s="57"/>
-      <c r="E191" s="57"/>
-      <c r="F191" s="57"/>
-      <c r="G191" s="57"/>
-      <c r="H191" s="57"/>
-      <c r="I191" s="57"/>
-      <c r="J191" s="57"/>
-      <c r="K191" s="58"/>
+      <c r="C191" s="64"/>
+      <c r="D191" s="64"/>
+      <c r="E191" s="64"/>
+      <c r="F191" s="64"/>
+      <c r="G191" s="64"/>
+      <c r="H191" s="64"/>
+      <c r="I191" s="64"/>
+      <c r="J191" s="64"/>
+      <c r="K191" s="65"/>
     </row>
     <row r="192" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B192" s="56" t="s">
+      <c r="B192" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C192" s="57"/>
-      <c r="D192" s="57"/>
-      <c r="E192" s="57"/>
-      <c r="F192" s="57"/>
-      <c r="G192" s="57"/>
-      <c r="H192" s="57"/>
-      <c r="I192" s="57"/>
-      <c r="J192" s="57"/>
-      <c r="K192" s="58"/>
+      <c r="C192" s="64"/>
+      <c r="D192" s="64"/>
+      <c r="E192" s="64"/>
+      <c r="F192" s="64"/>
+      <c r="G192" s="64"/>
+      <c r="H192" s="64"/>
+      <c r="I192" s="64"/>
+      <c r="J192" s="64"/>
+      <c r="K192" s="65"/>
     </row>
     <row r="193" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A193" s="37">
@@ -9106,53 +9115,53 @@
       <c r="K211" s="46"/>
     </row>
     <row r="212" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A212" s="59" t="s">
+      <c r="A212" s="74" t="s">
         <v>24</v>
       </c>
-      <c r="B212" s="57"/>
-      <c r="C212" s="57"/>
-      <c r="D212" s="57"/>
-      <c r="E212" s="57"/>
-      <c r="F212" s="57"/>
-      <c r="G212" s="57"/>
-      <c r="H212" s="57"/>
-      <c r="I212" s="57"/>
-      <c r="J212" s="57"/>
-      <c r="K212" s="58"/>
+      <c r="B212" s="64"/>
+      <c r="C212" s="64"/>
+      <c r="D212" s="64"/>
+      <c r="E212" s="64"/>
+      <c r="F212" s="64"/>
+      <c r="G212" s="64"/>
+      <c r="H212" s="64"/>
+      <c r="I212" s="64"/>
+      <c r="J212" s="64"/>
+      <c r="K212" s="65"/>
     </row>
     <row r="213" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A213" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B213" s="77" t="s">
+      <c r="B213" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C213" s="57"/>
-      <c r="D213" s="57"/>
-      <c r="E213" s="57"/>
-      <c r="F213" s="57"/>
-      <c r="G213" s="57"/>
-      <c r="H213" s="57"/>
-      <c r="I213" s="57"/>
-      <c r="J213" s="57"/>
-      <c r="K213" s="58"/>
+      <c r="C213" s="64"/>
+      <c r="D213" s="64"/>
+      <c r="E213" s="64"/>
+      <c r="F213" s="64"/>
+      <c r="G213" s="64"/>
+      <c r="H213" s="64"/>
+      <c r="I213" s="64"/>
+      <c r="J213" s="64"/>
+      <c r="K213" s="65"/>
     </row>
     <row r="214" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B214" s="77" t="s">
+      <c r="B214" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C214" s="57"/>
-      <c r="D214" s="57"/>
-      <c r="E214" s="57"/>
-      <c r="F214" s="57"/>
-      <c r="G214" s="57"/>
-      <c r="H214" s="57"/>
-      <c r="I214" s="57"/>
-      <c r="J214" s="57"/>
-      <c r="K214" s="58"/>
+      <c r="C214" s="64"/>
+      <c r="D214" s="64"/>
+      <c r="E214" s="64"/>
+      <c r="F214" s="64"/>
+      <c r="G214" s="64"/>
+      <c r="H214" s="64"/>
+      <c r="I214" s="64"/>
+      <c r="J214" s="64"/>
+      <c r="K214" s="65"/>
     </row>
     <row r="215" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A215" s="37">
@@ -9845,53 +9854,53 @@
       <c r="K235" s="46"/>
     </row>
     <row r="236" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A236" s="64" t="s">
+      <c r="A236" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="B236" s="65"/>
-      <c r="C236" s="65"/>
-      <c r="D236" s="65"/>
-      <c r="E236" s="65"/>
-      <c r="F236" s="65"/>
-      <c r="G236" s="65"/>
-      <c r="H236" s="65"/>
-      <c r="I236" s="65"/>
-      <c r="J236" s="65"/>
-      <c r="K236" s="66"/>
+      <c r="B236" s="57"/>
+      <c r="C236" s="57"/>
+      <c r="D236" s="57"/>
+      <c r="E236" s="57"/>
+      <c r="F236" s="57"/>
+      <c r="G236" s="57"/>
+      <c r="H236" s="57"/>
+      <c r="I236" s="57"/>
+      <c r="J236" s="57"/>
+      <c r="K236" s="58"/>
     </row>
     <row r="237" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A237" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B237" s="67" t="s">
+      <c r="B237" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="C237" s="65"/>
-      <c r="D237" s="65"/>
-      <c r="E237" s="65"/>
-      <c r="F237" s="65"/>
-      <c r="G237" s="65"/>
-      <c r="H237" s="65"/>
-      <c r="I237" s="65"/>
-      <c r="J237" s="65"/>
-      <c r="K237" s="66"/>
+      <c r="C237" s="57"/>
+      <c r="D237" s="57"/>
+      <c r="E237" s="57"/>
+      <c r="F237" s="57"/>
+      <c r="G237" s="57"/>
+      <c r="H237" s="57"/>
+      <c r="I237" s="57"/>
+      <c r="J237" s="57"/>
+      <c r="K237" s="58"/>
     </row>
     <row r="238" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B238" s="67" t="s">
+      <c r="B238" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="C238" s="65"/>
-      <c r="D238" s="65"/>
-      <c r="E238" s="65"/>
-      <c r="F238" s="65"/>
-      <c r="G238" s="65"/>
-      <c r="H238" s="65"/>
-      <c r="I238" s="65"/>
-      <c r="J238" s="65"/>
-      <c r="K238" s="66"/>
+      <c r="C238" s="57"/>
+      <c r="D238" s="57"/>
+      <c r="E238" s="57"/>
+      <c r="F238" s="57"/>
+      <c r="G238" s="57"/>
+      <c r="H238" s="57"/>
+      <c r="I238" s="57"/>
+      <c r="J238" s="57"/>
+      <c r="K238" s="58"/>
     </row>
     <row r="239" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A239" s="37">
@@ -10706,7 +10715,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J262" s="45"/>
+      <c r="J262" s="53" t="s">
+        <v>429</v>
+      </c>
       <c r="K262" s="43"/>
     </row>
     <row r="263" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10738,7 +10749,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J263" s="45"/>
+      <c r="J263" s="53" t="s">
+        <v>428</v>
+      </c>
       <c r="K263" s="43"/>
     </row>
     <row r="264" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10802,7 +10815,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J265" s="45"/>
+      <c r="J265" s="53" t="s">
+        <v>427</v>
+      </c>
       <c r="K265" s="43"/>
     </row>
     <row r="266" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10878,7 +10893,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{4156E376-828C-4BE6-9122-475CF5BFDDAA}">
+      <autoFilter ref="A1:K15" xr:uid="{017496B0-259A-4A30-86DD-B1A31A784FA1}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -10889,6 +10904,14 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
+    <mergeCell ref="B191:K191"/>
+    <mergeCell ref="B192:K192"/>
+    <mergeCell ref="A212:K212"/>
+    <mergeCell ref="B116:K116"/>
+    <mergeCell ref="A147:K147"/>
+    <mergeCell ref="B148:K148"/>
+    <mergeCell ref="B149:K149"/>
+    <mergeCell ref="A190:K190"/>
     <mergeCell ref="A236:K236"/>
     <mergeCell ref="B237:K237"/>
     <mergeCell ref="B238:K238"/>
@@ -10905,14 +10928,6 @@
     <mergeCell ref="B213:K213"/>
     <mergeCell ref="B214:K214"/>
     <mergeCell ref="B115:K115"/>
-    <mergeCell ref="B191:K191"/>
-    <mergeCell ref="B192:K192"/>
-    <mergeCell ref="A212:K212"/>
-    <mergeCell ref="B116:K116"/>
-    <mergeCell ref="A147:K147"/>
-    <mergeCell ref="B148:K148"/>
-    <mergeCell ref="B149:K149"/>
-    <mergeCell ref="A190:K190"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B43 B46:B78 B83:B112 B117:B145 B150:B188 B193:B210 B215:B234 B239:B266">
     <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="Unplanned">
@@ -11123,9 +11138,12 @@
     <hyperlink ref="J259" r:id="rId158" xr:uid="{D5D09BF0-FE64-4BBE-85F5-43D9FFB93CCF}"/>
     <hyperlink ref="J260" r:id="rId159" xr:uid="{993D6CEC-0D78-4F0A-A657-93188AFE2C21}"/>
     <hyperlink ref="J261" r:id="rId160" xr:uid="{510DBEE4-0A09-44A7-9D14-5A6A15E020AC}"/>
+    <hyperlink ref="J265" r:id="rId161" xr:uid="{A4875ED5-FA8C-41E6-8CC1-75054128D52D}"/>
+    <hyperlink ref="J263" r:id="rId162" xr:uid="{3B7ECD0E-DDEF-483D-8F11-E9E05596E2F4}"/>
+    <hyperlink ref="J262" r:id="rId163" xr:uid="{17824D2F-1BB7-4EFB-A1B0-095D943E93E7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId161"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId164"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -12780,26 +12798,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -13034,10 +13032,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -13054,20 +13083,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>